<commit_message>
Modeles recherche - 2026-09-14
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -96,30 +96,31 @@
     <sheet name="regression_multifeatures" sheetId="87" state="visible" r:id="rId87"/>
     <sheet name="rotation_risk_on_off" sheetId="88" state="visible" r:id="rId88"/>
     <sheet name="rotation_sectorielle" sheetId="89" state="visible" r:id="rId89"/>
-    <sheet name="sahm_rule" sheetId="90" state="visible" r:id="rId90"/>
-    <sheet name="saisonnalite" sheetId="91" state="visible" r:id="rId91"/>
-    <sheet name="screening_features" sheetId="92" state="visible" r:id="rId92"/>
-    <sheet name="similarite_vocabulaire_minutes" sheetId="93" state="visible" r:id="rId93"/>
-    <sheet name="sizing_robuste" sheetId="94" state="visible" r:id="rId94"/>
-    <sheet name="skew_kurtosis" sheetId="95" state="visible" r:id="rId95"/>
-    <sheet name="soutenabilite_dette" sheetId="96" state="visible" r:id="rId96"/>
-    <sheet name="stacking" sheetId="97" state="visible" r:id="rId97"/>
-    <sheet name="stationnarite_taux" sheetId="98" state="visible" r:id="rId98"/>
-    <sheet name="stress_test_historique" sheetId="99" state="visible" r:id="rId99"/>
-    <sheet name="surprise_inflation" sheetId="100" state="visible" r:id="rId100"/>
-    <sheet name="surprise_macro_composite" sheetId="101" state="visible" r:id="rId101"/>
-    <sheet name="taux_reel_us" sheetId="102" state="visible" r:id="rId102"/>
-    <sheet name="test_chow" sheetId="103" state="visible" r:id="rId103"/>
-    <sheet name="test_overfitting_momentum" sheetId="104" state="visible" r:id="rId104"/>
-    <sheet name="ton_banques_centrales" sheetId="105" state="visible" r:id="rId105"/>
-    <sheet name="ton_fomc" sheetId="106" state="visible" r:id="rId106"/>
-    <sheet name="ton_minutes_fomc" sheetId="107" state="visible" r:id="rId107"/>
-    <sheet name="var_conditionnelle_regime" sheetId="108" state="visible" r:id="rId108"/>
-    <sheet name="var_drawdown" sheetId="109" state="visible" r:id="rId109"/>
-    <sheet name="var_sp500_vix" sheetId="110" state="visible" r:id="rId110"/>
-    <sheet name="vol_cross_asset" sheetId="111" state="visible" r:id="rId111"/>
-    <sheet name="volatilite_ewma" sheetId="112" state="visible" r:id="rId112"/>
-    <sheet name="walkforward_direction_sp500" sheetId="113" state="visible" r:id="rId113"/>
+    <sheet name="ruptures_perimetre" sheetId="90" state="visible" r:id="rId90"/>
+    <sheet name="sahm_rule" sheetId="91" state="visible" r:id="rId91"/>
+    <sheet name="saisonnalite" sheetId="92" state="visible" r:id="rId92"/>
+    <sheet name="screening_features" sheetId="93" state="visible" r:id="rId93"/>
+    <sheet name="similarite_vocabulaire_minutes" sheetId="94" state="visible" r:id="rId94"/>
+    <sheet name="sizing_robuste" sheetId="95" state="visible" r:id="rId95"/>
+    <sheet name="skew_kurtosis" sheetId="96" state="visible" r:id="rId96"/>
+    <sheet name="soutenabilite_dette" sheetId="97" state="visible" r:id="rId97"/>
+    <sheet name="stacking" sheetId="98" state="visible" r:id="rId98"/>
+    <sheet name="stationnarite_taux" sheetId="99" state="visible" r:id="rId99"/>
+    <sheet name="stress_test_historique" sheetId="100" state="visible" r:id="rId100"/>
+    <sheet name="surprise_inflation" sheetId="101" state="visible" r:id="rId101"/>
+    <sheet name="surprise_macro_composite" sheetId="102" state="visible" r:id="rId102"/>
+    <sheet name="taux_reel_us" sheetId="103" state="visible" r:id="rId103"/>
+    <sheet name="test_chow" sheetId="104" state="visible" r:id="rId104"/>
+    <sheet name="test_overfitting_momentum" sheetId="105" state="visible" r:id="rId105"/>
+    <sheet name="ton_banques_centrales" sheetId="106" state="visible" r:id="rId106"/>
+    <sheet name="ton_fomc" sheetId="107" state="visible" r:id="rId107"/>
+    <sheet name="ton_minutes_fomc" sheetId="108" state="visible" r:id="rId108"/>
+    <sheet name="var_conditionnelle_regime" sheetId="109" state="visible" r:id="rId109"/>
+    <sheet name="var_drawdown" sheetId="110" state="visible" r:id="rId110"/>
+    <sheet name="var_sp500_vix" sheetId="111" state="visible" r:id="rId111"/>
+    <sheet name="vol_cross_asset" sheetId="112" state="visible" r:id="rId112"/>
+    <sheet name="volatilite_ewma" sheetId="113" state="visible" r:id="rId113"/>
+    <sheet name="walkforward_direction_sp500" sheetId="114" state="visible" r:id="rId114"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -550,21 +551,21 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-14 13:47 UTC</t>
+          <t>Genere le 2026-09-14 14:10 UTC</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>112 fichiers d'etat</t>
+          <t>113 fichiers d'etat</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Lecture du jour -- 2026-09-14 13:47 UTC</t>
+          <t>Lecture du jour -- 2026-09-14 14:09 UTC</t>
         </is>
       </c>
     </row>
@@ -928,7 +929,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>**ton_banques_centrales** -- ton (pour mille, meme lexique) : Fed +13.42, BCE +7.28, Banque d'Angleterre -15.34. Plus positive : Fed, plus negative : Banque d'Angleterre -- les tons DIVERGENT -- BCE se detend pendant que Fed, Banque d'Angleterre se durcit</t>
+          <t>**ton_banques_centrales** -- variation du ton depuis la publication precedente, par institution (pour mille, meme lexique) : Fed -4.28, BCE +12.50, Banque d'Angleterre -4.90 -- les tons DIVERGENT -- BCE se detend pendant que Fed, Banque d'Angleterre se durcit. Les niveaux ne sont PAS comparables entre institutions : un seul mot de ton les deplace de Fed 6.7, BCE 0.6, Banque d'Angleterre 0.3 pour mille respectivement, selon la longueur du document</t>
         </is>
       </c>
     </row>
@@ -1285,7 +1286,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>**var_sp500_vix** -- VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.4264235235490972 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.05236097746923429 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser)</t>
+          <t>**var_sp500_vix** -- VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.42642352354906876 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.052360977469234446 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser)</t>
         </is>
       </c>
     </row>
@@ -1810,6 +1811,284 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>scenario</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>date_pic</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>date_creux</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>chute_pct</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>niveau_sp500_rejoue</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>GFC_2008</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2007-10-09</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2009-03-09</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>-56.78</v>
+      </c>
+      <c r="F2" t="n">
+        <v>3316.85</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>COVID_2020</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2020-02-19</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2020-03-23</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>-33.92</v>
+      </c>
+      <c r="F3" t="n">
+        <v>5070.28</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>GFC_2008</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2007-10-09</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2009-03-09</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>-56.78</v>
+      </c>
+      <c r="F4" t="n">
+        <v>3300.79</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>COVID_2020</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2020-02-19</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2020-03-23</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>-33.92</v>
+      </c>
+      <c r="F5" t="n">
+        <v>5045.73</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>GFC_2008</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2007-10-09</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2009-03-09</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>-56.78</v>
+      </c>
+      <c r="F6" t="n">
+        <v>3281.48</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>COVID_2020</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2020-02-19</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2020-03-23</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>-33.92</v>
+      </c>
+      <c r="F7" t="n">
+        <v>5016.22</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>GFC_2008</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2007-10-09</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2009-03-09</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>-56.78</v>
+      </c>
+      <c r="F8" t="n">
+        <v>3309.7</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>COVID_2020</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2020-02-19</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2020-03-23</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>-33.92</v>
+      </c>
+      <c r="F9" t="n">
+        <v>5059.35</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet101.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1878,7 +2157,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet101.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet102.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1976,7 +2255,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet102.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet103.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2082,7 +2361,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet103.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet104.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2196,7 +2475,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet104.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet105.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2320,13 +2599,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet105.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet106.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -2335,6 +2614,7 @@
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="48" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2368,6 +2648,7 @@
           <t>lecture</t>
         </is>
       </c>
+      <c r="G1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2443,6 +2724,91 @@
         <is>
           <t>ton plus negatif que la publication precedente</t>
         </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Fed</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>20260729</v>
+      </c>
+      <c r="C5" t="n">
+        <v>13.423</v>
+      </c>
+      <c r="D5" t="n">
+        <v>149</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-4.276</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>ton plus negatif que la publication precedente</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>6.71</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>BCE</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>declaration_2026-09-10</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>7.283</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1785</v>
+      </c>
+      <c r="E6" t="n">
+        <v>12.502</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>ton plus positif que la publication precedente</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Banque d'Angleterre</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>resume_2026-07-30</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>-15.337</v>
+      </c>
+      <c r="D7" t="n">
+        <v>3912</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-4.897</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>ton plus negatif que la publication precedente</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>0.26</v>
       </c>
     </row>
   </sheetData>
@@ -2450,7 +2816,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet106.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet107.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2557,7 +2923,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet107.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet108.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2640,7 +3006,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet108.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet109.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2801,148 +3167,6 @@
       </c>
       <c r="G5" t="n">
         <v>-1.141</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet109.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="23" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>date</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>var_95_pct</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>cvar_95_pct</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>var_99_pct</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>cvar_99_pct</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>drawdown_max_252j_pct</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-09-08</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>-1.447</v>
-      </c>
-      <c r="C2" t="n">
-        <v>-1.803</v>
-      </c>
-      <c r="D2" t="n">
-        <v>-2.084</v>
-      </c>
-      <c r="E2" t="n">
-        <v>-2.504</v>
-      </c>
-      <c r="F2" t="n">
-        <v>-9.098000000000001</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>-1.447</v>
-      </c>
-      <c r="C3" t="n">
-        <v>-1.803</v>
-      </c>
-      <c r="D3" t="n">
-        <v>-2.084</v>
-      </c>
-      <c r="E3" t="n">
-        <v>-2.504</v>
-      </c>
-      <c r="F3" t="n">
-        <v>-9.098000000000001</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-09-10</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>-1.447</v>
-      </c>
-      <c r="C4" t="n">
-        <v>-1.803</v>
-      </c>
-      <c r="D4" t="n">
-        <v>-2.084</v>
-      </c>
-      <c r="E4" t="n">
-        <v>-2.504</v>
-      </c>
-      <c r="F4" t="n">
-        <v>-9.098000000000001</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>-1.447</v>
-      </c>
-      <c r="C5" t="n">
-        <v>-1.803</v>
-      </c>
-      <c r="D5" t="n">
-        <v>-2.084</v>
-      </c>
-      <c r="E5" t="n">
-        <v>-2.504</v>
-      </c>
-      <c r="F5" t="n">
-        <v>-9.098000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -3062,6 +3286,148 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>date</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>var_95_pct</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>cvar_95_pct</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>var_99_pct</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>cvar_99_pct</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>drawdown_max_252j_pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>-1.447</v>
+      </c>
+      <c r="C2" t="n">
+        <v>-1.803</v>
+      </c>
+      <c r="D2" t="n">
+        <v>-2.084</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-2.504</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-9.098000000000001</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>-1.447</v>
+      </c>
+      <c r="C3" t="n">
+        <v>-1.803</v>
+      </c>
+      <c r="D3" t="n">
+        <v>-2.084</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-2.504</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-9.098000000000001</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>-1.447</v>
+      </c>
+      <c r="C4" t="n">
+        <v>-1.803</v>
+      </c>
+      <c r="D4" t="n">
+        <v>-2.084</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-2.504</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-9.098000000000001</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>-1.447</v>
+      </c>
+      <c r="C5" t="n">
+        <v>-1.803</v>
+      </c>
+      <c r="D5" t="n">
+        <v>-2.084</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-2.504</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-9.098000000000001</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet111.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3162,7 +3528,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet111.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet112.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3372,7 +3738,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet112.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet113.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3515,7 +3881,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet113.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet114.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -47013,6 +47379,252 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="23" customWidth="1" min="1" max="1"/>
+    <col width="27" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>serie</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>colonne</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>date_avant</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>taille_avant</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>date_apres</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>taille_apres</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>variation_pct</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>nature</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>crowding_cross_asset</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>n_marches_tendus</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>15</v>
+      </c>
+      <c r="G2" t="n">
+        <v>400</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>a verifier (peut etre un resultat)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>crowding_cross_asset</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>n_marches_total</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>15</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>32</v>
+      </c>
+      <c r="G3" t="n">
+        <v>113.3</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>perimetre</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>dollar_smile</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>n_devises_non_usd_courtes</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G4" t="n">
+        <v>33.3</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>perimetre</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>nombre_effectif_paris</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>n_marches</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>15</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>32</v>
+      </c>
+      <c r="G5" t="n">
+        <v>113.3</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>perimetre</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>nombre_effectif_paris</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>nombre_effectif_paris</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>8.539999999999999</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>13.39</v>
+      </c>
+      <c r="G6" t="n">
+        <v>56.8</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>a verifier (peut etre un resultat)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet91.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -47085,7 +47697,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet91.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet92.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -47271,7 +47883,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet92.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet93.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -47687,7 +48299,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet93.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet94.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -47770,7 +48382,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet94.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet95.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -47894,7 +48506,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet95.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet96.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -47982,7 +48594,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet96.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet97.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -48173,7 +48785,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet97.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet98.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -48351,7 +48963,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet98.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet99.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -48963,282 +49575,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet99.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="21" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>date</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>scenario</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>date_pic</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>date_creux</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>chute_pct</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>niveau_sp500_rejoue</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-09-08</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>GFC_2008</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2007-10-09</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2009-03-09</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>-56.78</v>
-      </c>
-      <c r="F2" t="n">
-        <v>3316.85</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2026-09-08</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>COVID_2020</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>2020-02-19</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>2020-03-23</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>-33.92</v>
-      </c>
-      <c r="F3" t="n">
-        <v>5070.28</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>GFC_2008</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>2007-10-09</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>2009-03-09</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>-56.78</v>
-      </c>
-      <c r="F4" t="n">
-        <v>3300.79</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>COVID_2020</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>2020-02-19</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>2020-03-23</t>
-        </is>
-      </c>
-      <c r="E5" t="n">
-        <v>-33.92</v>
-      </c>
-      <c r="F5" t="n">
-        <v>5045.73</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-09-10</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>GFC_2008</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>2007-10-09</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>2009-03-09</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>-56.78</v>
-      </c>
-      <c r="F6" t="n">
-        <v>3281.48</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2026-09-10</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>COVID_2020</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>2020-02-19</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>2020-03-23</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>-33.92</v>
-      </c>
-      <c r="F7" t="n">
-        <v>5016.22</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>GFC_2008</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>2007-10-09</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>2009-03-09</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>-56.78</v>
-      </c>
-      <c r="F8" t="n">
-        <v>3309.7</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>COVID_2020</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>2020-02-19</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>2020-03-23</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>-33.92</v>
-      </c>
-      <c r="F9" t="n">
-        <v>5059.35</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
fix: align freshness with source publication cadence
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -1,129 +1,129 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Lecture du jour" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="activite_zone_euro" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="analyse_spectrale" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="anomalie_multivariee" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="arima" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="balance_commerciale" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="beta_facteur_macro" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="beta_vol" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="bilans_banques_centrales" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="carry_proxy" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="causalite_granger" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="changepoint_volatilite" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="chemin_taux_fed" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="choc_taux" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="choc_vol_parametrique" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="clustering_marches" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="coherence_fed" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="cointegration_secteurs" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="cointegration_taux" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="complexite_texte_fomc" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="complexite_texte_minutes" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="concentration_traders" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="conditions_financieres" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="correlation_cot_prix" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="correlation_facteurs" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="correlation_glissante" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="correlations_positionnement" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="courbe_taux_us" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="couts_transaction" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet name="covar" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet name="crowding_cross_asset" sheetId="31" state="visible" r:id="rId31"/>
-    <sheet name="cycle_credit" sheetId="32" state="visible" r:id="rId32"/>
-    <sheet name="cycle_immobilier" sheetId="33" state="visible" r:id="rId33"/>
-    <sheet name="decision_stump" sheetId="34" state="visible" r:id="rId34"/>
-    <sheet name="decomposition_stl" sheetId="35" state="visible" r:id="rId35"/>
-    <sheet name="decomposition_variance" sheetId="36" state="visible" r:id="rId36"/>
-    <sheet name="dependance_queue" sheetId="37" state="visible" r:id="rId37"/>
-    <sheet name="detection_saut" sheetId="38" state="visible" r:id="rId38"/>
-    <sheet name="differentiel_taux_change" sheetId="39" state="visible" r:id="rId39"/>
-    <sheet name="dispersion_sectorielle" sheetId="40" state="visible" r:id="rId40"/>
-    <sheet name="divergence_cot_prix" sheetId="41" state="visible" r:id="rId41"/>
-    <sheet name="divergence_taux_directeurs" sheetId="42" state="visible" r:id="rId42"/>
-    <sheet name="dollar_smile" sheetId="43" state="visible" r:id="rId43"/>
-    <sheet name="ecart_communique_minutes" sheetId="44" state="visible" r:id="rId44"/>
-    <sheet name="emission_tresor_us" sheetId="45" state="visible" r:id="rId45"/>
-    <sheet name="ensemble_signaux" sheetId="46" state="visible" r:id="rId46"/>
-    <sheet name="entites_geographiques_minutes" sheetId="47" state="visible" r:id="rId47"/>
-    <sheet name="extremes_historiques" sheetId="48" state="visible" r:id="rId48"/>
-    <sheet name="facteur_qualite_credit" sheetId="49" state="visible" r:id="rId49"/>
-    <sheet name="fraicheur" sheetId="50" state="visible" r:id="rId50"/>
-    <sheet name="frequence_mots_cles_fomc" sheetId="51" state="visible" r:id="rId51"/>
-    <sheet name="frequence_mots_cles_minutes" sheetId="52" state="visible" r:id="rId52"/>
-    <sheet name="garch" sheetId="53" state="visible" r:id="rId53"/>
-    <sheet name="hp_filter_taux" sheetId="54" state="visible" r:id="rId54"/>
-    <sheet name="hurst" sheetId="55" state="visible" r:id="rId55"/>
-    <sheet name="importance_permutation" sheetId="56" state="visible" r:id="rId56"/>
-    <sheet name="indices_mondiaux" sheetId="57" state="visible" r:id="rId57"/>
-    <sheet name="inflation_comparee" sheetId="58" state="visible" r:id="rId58"/>
-    <sheet name="intensite_desaccord" sheetId="59" state="visible" r:id="rId59"/>
-    <sheet name="kalman_niveau_local" sheetId="60" state="visible" r:id="rId60"/>
-    <sheet name="kmeans_regimes" sheetId="61" state="visible" r:id="rId61"/>
-    <sheet name="langage_prudence" sheetId="62" state="visible" r:id="rId62"/>
-    <sheet name="liquidite_nette_fed" sheetId="63" state="visible" r:id="rId63"/>
-    <sheet name="lisibilite_flesch_kincaid" sheetId="64" state="visible" r:id="rId64"/>
-    <sheet name="low_volatility" sheetId="65" state="visible" r:id="rId65"/>
-    <sheet name="matieres_premieres_macro" sheetId="66" state="visible" r:id="rId66"/>
-    <sheet name="metaux_precieux" sheetId="67" state="visible" r:id="rId67"/>
-    <sheet name="momentum_credit" sheetId="68" state="visible" r:id="rId68"/>
-    <sheet name="momentum_cross_sectional" sheetId="69" state="visible" r:id="rId69"/>
-    <sheet name="momentum_positionnement" sheetId="70" state="visible" r:id="rId70"/>
-    <sheet name="momentum_prix" sheetId="71" state="visible" r:id="rId71"/>
-    <sheet name="nombre_effectif_paris" sheetId="72" state="visible" r:id="rId72"/>
-    <sheet name="ornstein_uhlenbeck_credit" sheetId="73" state="visible" r:id="rId73"/>
-    <sheet name="ornstein_uhlenbeck_vix" sheetId="74" state="visible" r:id="rId74"/>
-    <sheet name="pca_taux" sheetId="75" state="visible" r:id="rId75"/>
-    <sheet name="pentes_courbes" sheetId="76" state="visible" r:id="rId76"/>
-    <sheet name="persistance_extremes" sheetId="77" state="visible" r:id="rId77"/>
-    <sheet name="positionnement_cot" sheetId="78" state="visible" r:id="rId78"/>
-    <sheet name="positionnement_courbe_taux" sheetId="79" state="visible" r:id="rId79"/>
-    <sheet name="positionnement_devises" sheetId="80" state="visible" r:id="rId80"/>
-    <sheet name="prevision_vol_regression" sheetId="81" state="visible" r:id="rId81"/>
-    <sheet name="qualite_regime_macro" sheetId="82" state="visible" r:id="rId82"/>
-    <sheet name="ratio_commercial_speculatif" sheetId="83" state="visible" r:id="rId83"/>
-    <sheet name="ratios_conditionnels_regime" sheetId="84" state="visible" r:id="rId84"/>
-    <sheet name="ratios_performance" sheetId="85" state="visible" r:id="rId85"/>
-    <sheet name="reer_us" sheetId="86" state="visible" r:id="rId86"/>
-    <sheet name="regime_monetaire_emploi" sheetId="87" state="visible" r:id="rId87"/>
-    <sheet name="regle_taylor" sheetId="88" state="visible" r:id="rId88"/>
-    <sheet name="regression_multifeatures" sheetId="89" state="visible" r:id="rId89"/>
-    <sheet name="rotation_risk_on_off" sheetId="90" state="visible" r:id="rId90"/>
-    <sheet name="rotation_sectorielle" sheetId="91" state="visible" r:id="rId91"/>
-    <sheet name="ruptures_perimetre" sheetId="92" state="visible" r:id="rId92"/>
-    <sheet name="sahm_rule" sheetId="93" state="visible" r:id="rId93"/>
-    <sheet name="saisonnalite" sheetId="94" state="visible" r:id="rId94"/>
-    <sheet name="screening_features" sheetId="95" state="visible" r:id="rId95"/>
-    <sheet name="similarite_vocabulaire_minutes" sheetId="96" state="visible" r:id="rId96"/>
-    <sheet name="sizing_robuste" sheetId="97" state="visible" r:id="rId97"/>
-    <sheet name="skew_kurtosis" sheetId="98" state="visible" r:id="rId98"/>
-    <sheet name="soutenabilite_dette" sheetId="99" state="visible" r:id="rId99"/>
-    <sheet name="stacking" sheetId="100" state="visible" r:id="rId100"/>
-    <sheet name="stationnarite_taux" sheetId="101" state="visible" r:id="rId101"/>
-    <sheet name="stress_test_historique" sheetId="102" state="visible" r:id="rId102"/>
-    <sheet name="surprise_inflation" sheetId="103" state="visible" r:id="rId103"/>
-    <sheet name="surprise_macro_composite" sheetId="104" state="visible" r:id="rId104"/>
-    <sheet name="taux_reel_us" sheetId="105" state="visible" r:id="rId105"/>
-    <sheet name="test_chow" sheetId="106" state="visible" r:id="rId106"/>
-    <sheet name="test_overfitting_momentum" sheetId="107" state="visible" r:id="rId107"/>
-    <sheet name="ton_banques_centrales" sheetId="108" state="visible" r:id="rId108"/>
-    <sheet name="ton_fomc" sheetId="109" state="visible" r:id="rId109"/>
-    <sheet name="ton_minutes_fomc" sheetId="110" state="visible" r:id="rId110"/>
-    <sheet name="univers_sources" sheetId="111" state="visible" r:id="rId111"/>
-    <sheet name="var_conditionnelle_regime" sheetId="112" state="visible" r:id="rId112"/>
-    <sheet name="var_drawdown" sheetId="113" state="visible" r:id="rId113"/>
-    <sheet name="var_sp500_vix" sheetId="114" state="visible" r:id="rId114"/>
-    <sheet name="vol_cross_asset" sheetId="115" state="visible" r:id="rId115"/>
-    <sheet name="volatilite_ewma" sheetId="116" state="visible" r:id="rId116"/>
-    <sheet name="walkforward_direction_sp500" sheetId="117" state="visible" r:id="rId117"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lecture du jour" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="activite_zone_euro" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="analyse_spectrale" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="anomalie_multivariee" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="arima" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="balance_commerciale" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="beta_facteur_macro" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="beta_vol" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="bilans_banques_centrales" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="carry_proxy" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="causalite_granger" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="changepoint_volatilite" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="chemin_taux_fed" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choc_taux" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choc_vol_parametrique" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="clustering_marches" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="coherence_fed" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cointegration_secteurs" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cointegration_taux" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="complexite_texte_fomc" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="complexite_texte_minutes" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="concentration_traders" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="conditions_financieres" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="correlation_cot_prix" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="correlation_facteurs" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="correlation_glissante" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="correlations_positionnement" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="courbe_taux_us" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="couts_transaction" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="covar" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="crowding_cross_asset" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cycle_credit" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cycle_immobilier" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="decision_stump" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="decomposition_stl" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="decomposition_variance" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="dependance_queue" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="detection_saut" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="differentiel_taux_change" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="dispersion_sectorielle" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="divergence_cot_prix" sheetId="41" state="visible" r:id="rId41"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="divergence_taux_directeurs" sheetId="42" state="visible" r:id="rId42"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="dollar_smile" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ecart_communique_minutes" sheetId="44" state="visible" r:id="rId44"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="emission_tresor_us" sheetId="45" state="visible" r:id="rId45"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ensemble_signaux" sheetId="46" state="visible" r:id="rId46"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="entites_geographiques_minutes" sheetId="47" state="visible" r:id="rId47"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extremes_historiques" sheetId="48" state="visible" r:id="rId48"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="facteur_qualite_credit" sheetId="49" state="visible" r:id="rId49"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="fraicheur" sheetId="50" state="visible" r:id="rId50"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="frequence_mots_cles_fomc" sheetId="51" state="visible" r:id="rId51"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="frequence_mots_cles_minutes" sheetId="52" state="visible" r:id="rId52"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="garch" sheetId="53" state="visible" r:id="rId53"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hp_filter_taux" sheetId="54" state="visible" r:id="rId54"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hurst" sheetId="55" state="visible" r:id="rId55"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="importance_permutation" sheetId="56" state="visible" r:id="rId56"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="indices_mondiaux" sheetId="57" state="visible" r:id="rId57"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="inflation_comparee" sheetId="58" state="visible" r:id="rId58"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="intensite_desaccord" sheetId="59" state="visible" r:id="rId59"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="kalman_niveau_local" sheetId="60" state="visible" r:id="rId60"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="kmeans_regimes" sheetId="61" state="visible" r:id="rId61"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="langage_prudence" sheetId="62" state="visible" r:id="rId62"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="liquidite_nette_fed" sheetId="63" state="visible" r:id="rId63"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="lisibilite_flesch_kincaid" sheetId="64" state="visible" r:id="rId64"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="low_volatility" sheetId="65" state="visible" r:id="rId65"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="matieres_premieres_macro" sheetId="66" state="visible" r:id="rId66"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="metaux_precieux" sheetId="67" state="visible" r:id="rId67"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="momentum_credit" sheetId="68" state="visible" r:id="rId68"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="momentum_cross_sectional" sheetId="69" state="visible" r:id="rId69"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="momentum_positionnement" sheetId="70" state="visible" r:id="rId70"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="momentum_prix" sheetId="71" state="visible" r:id="rId71"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="nombre_effectif_paris" sheetId="72" state="visible" r:id="rId72"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ornstein_uhlenbeck_credit" sheetId="73" state="visible" r:id="rId73"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ornstein_uhlenbeck_vix" sheetId="74" state="visible" r:id="rId74"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pca_taux" sheetId="75" state="visible" r:id="rId75"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pentes_courbes" sheetId="76" state="visible" r:id="rId76"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="persistance_extremes" sheetId="77" state="visible" r:id="rId77"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="positionnement_cot" sheetId="78" state="visible" r:id="rId78"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="positionnement_courbe_taux" sheetId="79" state="visible" r:id="rId79"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="positionnement_devises" sheetId="80" state="visible" r:id="rId80"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="prevision_vol_regression" sheetId="81" state="visible" r:id="rId81"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="qualite_regime_macro" sheetId="82" state="visible" r:id="rId82"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ratio_commercial_speculatif" sheetId="83" state="visible" r:id="rId83"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ratios_conditionnels_regime" sheetId="84" state="visible" r:id="rId84"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ratios_performance" sheetId="85" state="visible" r:id="rId85"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="reer_us" sheetId="86" state="visible" r:id="rId86"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="regime_monetaire_emploi" sheetId="87" state="visible" r:id="rId87"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="regle_taylor" sheetId="88" state="visible" r:id="rId88"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="regression_multifeatures" sheetId="89" state="visible" r:id="rId89"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="rotation_risk_on_off" sheetId="90" state="visible" r:id="rId90"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="rotation_sectorielle" sheetId="91" state="visible" r:id="rId91"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ruptures_perimetre" sheetId="92" state="visible" r:id="rId92"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sahm_rule" sheetId="93" state="visible" r:id="rId93"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="saisonnalite" sheetId="94" state="visible" r:id="rId94"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="screening_features" sheetId="95" state="visible" r:id="rId95"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="similarite_vocabulaire_minutes" sheetId="96" state="visible" r:id="rId96"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sizing_robuste" sheetId="97" state="visible" r:id="rId97"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="skew_kurtosis" sheetId="98" state="visible" r:id="rId98"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="soutenabilite_dette" sheetId="99" state="visible" r:id="rId99"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="stacking" sheetId="100" state="visible" r:id="rId100"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="stationnarite_taux" sheetId="101" state="visible" r:id="rId101"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="stress_test_historique" sheetId="102" state="visible" r:id="rId102"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="surprise_inflation" sheetId="103" state="visible" r:id="rId103"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="surprise_macro_composite" sheetId="104" state="visible" r:id="rId104"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="taux_reel_us" sheetId="105" state="visible" r:id="rId105"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="test_chow" sheetId="106" state="visible" r:id="rId106"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="test_overfitting_momentum" sheetId="107" state="visible" r:id="rId107"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ton_banques_centrales" sheetId="108" state="visible" r:id="rId108"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ton_fomc" sheetId="109" state="visible" r:id="rId109"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ton_minutes_fomc" sheetId="110" state="visible" r:id="rId110"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="univers_sources" sheetId="111" state="visible" r:id="rId111"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="var_conditionnelle_regime" sheetId="112" state="visible" r:id="rId112"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="var_drawdown" sheetId="113" state="visible" r:id="rId113"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="var_sp500_vix" sheetId="114" state="visible" r:id="rId114"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="vol_cross_asset" sheetId="115" state="visible" r:id="rId115"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="volatilite_ewma" sheetId="116" state="visible" r:id="rId116"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="walkforward_direction_sp500" sheetId="117" state="visible" r:id="rId117"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-25 08:04 UTC</t>
+          <t>Genere le 2026-09-25 08:06 UTC</t>
         </is>
       </c>
     </row>
@@ -568,14 +568,14 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-25 08:04 UTC</t>
+          <t>Rapport global — 2026-09-25 08:06 UTC</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>**Etat global : ATTENTION** · 112/112 modeles reussis · 5 source(s) suspecte(s) · 0 source(s) gelee(s).</t>
+          <t>**Etat global : OK** · 112/112 modeles reussis · 0 source(s) suspecte(s) · 0 source(s) gelee(s).</t>
         </is>
       </c>
     </row>
@@ -41998,14 +41998,14 @@
         <v>1</v>
       </c>
       <c r="E95" t="n">
-        <v>42</v>
+        <v>70</v>
       </c>
       <c r="F95" t="n">
         <v>6815</v>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>SUSPECTE</t>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -42027,14 +42027,14 @@
         <v>1</v>
       </c>
       <c r="E96" t="n">
-        <v>42</v>
+        <v>90</v>
       </c>
       <c r="F96" t="n">
         <v>9929</v>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>SUSPECTE</t>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -42056,14 +42056,14 @@
         <v>1</v>
       </c>
       <c r="E97" t="n">
-        <v>42</v>
+        <v>90</v>
       </c>
       <c r="F97" t="n">
         <v>12929</v>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>SUSPECTE</t>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -42085,14 +42085,14 @@
         <v>1</v>
       </c>
       <c r="E98" t="n">
-        <v>42</v>
+        <v>90</v>
       </c>
       <c r="F98" t="n">
         <v>6613</v>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>SUSPECTE</t>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -42114,14 +42114,14 @@
         <v>1</v>
       </c>
       <c r="E99" t="n">
-        <v>42</v>
+        <v>90</v>
       </c>
       <c r="F99" t="n">
         <v>13290</v>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>SUSPECTE</t>
+          <t>OK</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Recherche - publication 2026-09-25T08:11Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -1,129 +1,129 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lecture du jour" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="activite_zone_euro" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="analyse_spectrale" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="anomalie_multivariee" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="arima" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="balance_commerciale" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="beta_facteur_macro" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="beta_vol" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="bilans_banques_centrales" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="carry_proxy" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="causalite_granger" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="changepoint_volatilite" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="chemin_taux_fed" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choc_taux" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choc_vol_parametrique" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="clustering_marches" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="coherence_fed" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cointegration_secteurs" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cointegration_taux" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="complexite_texte_fomc" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="complexite_texte_minutes" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="concentration_traders" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="conditions_financieres" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="correlation_cot_prix" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="correlation_facteurs" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="correlation_glissante" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="correlations_positionnement" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="courbe_taux_us" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="couts_transaction" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="covar" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="crowding_cross_asset" sheetId="31" state="visible" r:id="rId31"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cycle_credit" sheetId="32" state="visible" r:id="rId32"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cycle_immobilier" sheetId="33" state="visible" r:id="rId33"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="decision_stump" sheetId="34" state="visible" r:id="rId34"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="decomposition_stl" sheetId="35" state="visible" r:id="rId35"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="decomposition_variance" sheetId="36" state="visible" r:id="rId36"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="dependance_queue" sheetId="37" state="visible" r:id="rId37"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="detection_saut" sheetId="38" state="visible" r:id="rId38"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="differentiel_taux_change" sheetId="39" state="visible" r:id="rId39"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="dispersion_sectorielle" sheetId="40" state="visible" r:id="rId40"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="divergence_cot_prix" sheetId="41" state="visible" r:id="rId41"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="divergence_taux_directeurs" sheetId="42" state="visible" r:id="rId42"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="dollar_smile" sheetId="43" state="visible" r:id="rId43"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ecart_communique_minutes" sheetId="44" state="visible" r:id="rId44"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="emission_tresor_us" sheetId="45" state="visible" r:id="rId45"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ensemble_signaux" sheetId="46" state="visible" r:id="rId46"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="entites_geographiques_minutes" sheetId="47" state="visible" r:id="rId47"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extremes_historiques" sheetId="48" state="visible" r:id="rId48"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="facteur_qualite_credit" sheetId="49" state="visible" r:id="rId49"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="fraicheur" sheetId="50" state="visible" r:id="rId50"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="frequence_mots_cles_fomc" sheetId="51" state="visible" r:id="rId51"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="frequence_mots_cles_minutes" sheetId="52" state="visible" r:id="rId52"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="garch" sheetId="53" state="visible" r:id="rId53"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hp_filter_taux" sheetId="54" state="visible" r:id="rId54"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hurst" sheetId="55" state="visible" r:id="rId55"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="importance_permutation" sheetId="56" state="visible" r:id="rId56"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="indices_mondiaux" sheetId="57" state="visible" r:id="rId57"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="inflation_comparee" sheetId="58" state="visible" r:id="rId58"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="intensite_desaccord" sheetId="59" state="visible" r:id="rId59"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="kalman_niveau_local" sheetId="60" state="visible" r:id="rId60"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="kmeans_regimes" sheetId="61" state="visible" r:id="rId61"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="langage_prudence" sheetId="62" state="visible" r:id="rId62"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="liquidite_nette_fed" sheetId="63" state="visible" r:id="rId63"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="lisibilite_flesch_kincaid" sheetId="64" state="visible" r:id="rId64"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="low_volatility" sheetId="65" state="visible" r:id="rId65"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="matieres_premieres_macro" sheetId="66" state="visible" r:id="rId66"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="metaux_precieux" sheetId="67" state="visible" r:id="rId67"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="momentum_credit" sheetId="68" state="visible" r:id="rId68"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="momentum_cross_sectional" sheetId="69" state="visible" r:id="rId69"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="momentum_positionnement" sheetId="70" state="visible" r:id="rId70"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="momentum_prix" sheetId="71" state="visible" r:id="rId71"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="nombre_effectif_paris" sheetId="72" state="visible" r:id="rId72"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ornstein_uhlenbeck_credit" sheetId="73" state="visible" r:id="rId73"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ornstein_uhlenbeck_vix" sheetId="74" state="visible" r:id="rId74"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pca_taux" sheetId="75" state="visible" r:id="rId75"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pentes_courbes" sheetId="76" state="visible" r:id="rId76"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="persistance_extremes" sheetId="77" state="visible" r:id="rId77"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="positionnement_cot" sheetId="78" state="visible" r:id="rId78"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="positionnement_courbe_taux" sheetId="79" state="visible" r:id="rId79"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="positionnement_devises" sheetId="80" state="visible" r:id="rId80"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="prevision_vol_regression" sheetId="81" state="visible" r:id="rId81"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="qualite_regime_macro" sheetId="82" state="visible" r:id="rId82"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ratio_commercial_speculatif" sheetId="83" state="visible" r:id="rId83"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ratios_conditionnels_regime" sheetId="84" state="visible" r:id="rId84"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ratios_performance" sheetId="85" state="visible" r:id="rId85"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="reer_us" sheetId="86" state="visible" r:id="rId86"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="regime_monetaire_emploi" sheetId="87" state="visible" r:id="rId87"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="regle_taylor" sheetId="88" state="visible" r:id="rId88"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="regression_multifeatures" sheetId="89" state="visible" r:id="rId89"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="rotation_risk_on_off" sheetId="90" state="visible" r:id="rId90"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="rotation_sectorielle" sheetId="91" state="visible" r:id="rId91"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ruptures_perimetre" sheetId="92" state="visible" r:id="rId92"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sahm_rule" sheetId="93" state="visible" r:id="rId93"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="saisonnalite" sheetId="94" state="visible" r:id="rId94"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="screening_features" sheetId="95" state="visible" r:id="rId95"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="similarite_vocabulaire_minutes" sheetId="96" state="visible" r:id="rId96"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sizing_robuste" sheetId="97" state="visible" r:id="rId97"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="skew_kurtosis" sheetId="98" state="visible" r:id="rId98"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="soutenabilite_dette" sheetId="99" state="visible" r:id="rId99"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="stacking" sheetId="100" state="visible" r:id="rId100"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="stationnarite_taux" sheetId="101" state="visible" r:id="rId101"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="stress_test_historique" sheetId="102" state="visible" r:id="rId102"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="surprise_inflation" sheetId="103" state="visible" r:id="rId103"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="surprise_macro_composite" sheetId="104" state="visible" r:id="rId104"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="taux_reel_us" sheetId="105" state="visible" r:id="rId105"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="test_chow" sheetId="106" state="visible" r:id="rId106"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="test_overfitting_momentum" sheetId="107" state="visible" r:id="rId107"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ton_banques_centrales" sheetId="108" state="visible" r:id="rId108"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ton_fomc" sheetId="109" state="visible" r:id="rId109"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ton_minutes_fomc" sheetId="110" state="visible" r:id="rId110"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="univers_sources" sheetId="111" state="visible" r:id="rId111"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="var_conditionnelle_regime" sheetId="112" state="visible" r:id="rId112"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="var_drawdown" sheetId="113" state="visible" r:id="rId113"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="var_sp500_vix" sheetId="114" state="visible" r:id="rId114"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="vol_cross_asset" sheetId="115" state="visible" r:id="rId115"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="volatilite_ewma" sheetId="116" state="visible" r:id="rId116"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="walkforward_direction_sp500" sheetId="117" state="visible" r:id="rId117"/>
+    <sheet name="Lecture du jour" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="activite_zone_euro" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="analyse_spectrale" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="anomalie_multivariee" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="arima" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="balance_commerciale" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="beta_facteur_macro" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="beta_vol" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="bilans_banques_centrales" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="carry_proxy" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="causalite_granger" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="changepoint_volatilite" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="chemin_taux_fed" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="choc_taux" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="choc_vol_parametrique" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="clustering_marches" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="coherence_fed" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="cointegration_secteurs" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="cointegration_taux" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="complexite_texte_fomc" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="complexite_texte_minutes" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="concentration_traders" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="conditions_financieres" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="correlation_cot_prix" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="correlation_facteurs" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="correlation_glissante" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="correlations_positionnement" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="courbe_taux_us" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="couts_transaction" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="covar" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="crowding_cross_asset" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet name="cycle_credit" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="cycle_immobilier" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet name="decision_stump" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="decomposition_stl" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet name="decomposition_variance" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet name="dependance_queue" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet name="detection_saut" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet name="differentiel_taux_change" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet name="dispersion_sectorielle" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet name="divergence_cot_prix" sheetId="41" state="visible" r:id="rId41"/>
+    <sheet name="divergence_taux_directeurs" sheetId="42" state="visible" r:id="rId42"/>
+    <sheet name="dollar_smile" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet name="ecart_communique_minutes" sheetId="44" state="visible" r:id="rId44"/>
+    <sheet name="emission_tresor_us" sheetId="45" state="visible" r:id="rId45"/>
+    <sheet name="ensemble_signaux" sheetId="46" state="visible" r:id="rId46"/>
+    <sheet name="entites_geographiques_minutes" sheetId="47" state="visible" r:id="rId47"/>
+    <sheet name="extremes_historiques" sheetId="48" state="visible" r:id="rId48"/>
+    <sheet name="facteur_qualite_credit" sheetId="49" state="visible" r:id="rId49"/>
+    <sheet name="fraicheur" sheetId="50" state="visible" r:id="rId50"/>
+    <sheet name="frequence_mots_cles_fomc" sheetId="51" state="visible" r:id="rId51"/>
+    <sheet name="frequence_mots_cles_minutes" sheetId="52" state="visible" r:id="rId52"/>
+    <sheet name="garch" sheetId="53" state="visible" r:id="rId53"/>
+    <sheet name="hp_filter_taux" sheetId="54" state="visible" r:id="rId54"/>
+    <sheet name="hurst" sheetId="55" state="visible" r:id="rId55"/>
+    <sheet name="importance_permutation" sheetId="56" state="visible" r:id="rId56"/>
+    <sheet name="indices_mondiaux" sheetId="57" state="visible" r:id="rId57"/>
+    <sheet name="inflation_comparee" sheetId="58" state="visible" r:id="rId58"/>
+    <sheet name="intensite_desaccord" sheetId="59" state="visible" r:id="rId59"/>
+    <sheet name="kalman_niveau_local" sheetId="60" state="visible" r:id="rId60"/>
+    <sheet name="kmeans_regimes" sheetId="61" state="visible" r:id="rId61"/>
+    <sheet name="langage_prudence" sheetId="62" state="visible" r:id="rId62"/>
+    <sheet name="liquidite_nette_fed" sheetId="63" state="visible" r:id="rId63"/>
+    <sheet name="lisibilite_flesch_kincaid" sheetId="64" state="visible" r:id="rId64"/>
+    <sheet name="low_volatility" sheetId="65" state="visible" r:id="rId65"/>
+    <sheet name="matieres_premieres_macro" sheetId="66" state="visible" r:id="rId66"/>
+    <sheet name="metaux_precieux" sheetId="67" state="visible" r:id="rId67"/>
+    <sheet name="momentum_credit" sheetId="68" state="visible" r:id="rId68"/>
+    <sheet name="momentum_cross_sectional" sheetId="69" state="visible" r:id="rId69"/>
+    <sheet name="momentum_positionnement" sheetId="70" state="visible" r:id="rId70"/>
+    <sheet name="momentum_prix" sheetId="71" state="visible" r:id="rId71"/>
+    <sheet name="nombre_effectif_paris" sheetId="72" state="visible" r:id="rId72"/>
+    <sheet name="ornstein_uhlenbeck_credit" sheetId="73" state="visible" r:id="rId73"/>
+    <sheet name="ornstein_uhlenbeck_vix" sheetId="74" state="visible" r:id="rId74"/>
+    <sheet name="pca_taux" sheetId="75" state="visible" r:id="rId75"/>
+    <sheet name="pentes_courbes" sheetId="76" state="visible" r:id="rId76"/>
+    <sheet name="persistance_extremes" sheetId="77" state="visible" r:id="rId77"/>
+    <sheet name="positionnement_cot" sheetId="78" state="visible" r:id="rId78"/>
+    <sheet name="positionnement_courbe_taux" sheetId="79" state="visible" r:id="rId79"/>
+    <sheet name="positionnement_devises" sheetId="80" state="visible" r:id="rId80"/>
+    <sheet name="prevision_vol_regression" sheetId="81" state="visible" r:id="rId81"/>
+    <sheet name="qualite_regime_macro" sheetId="82" state="visible" r:id="rId82"/>
+    <sheet name="ratio_commercial_speculatif" sheetId="83" state="visible" r:id="rId83"/>
+    <sheet name="ratios_conditionnels_regime" sheetId="84" state="visible" r:id="rId84"/>
+    <sheet name="ratios_performance" sheetId="85" state="visible" r:id="rId85"/>
+    <sheet name="reer_us" sheetId="86" state="visible" r:id="rId86"/>
+    <sheet name="regime_monetaire_emploi" sheetId="87" state="visible" r:id="rId87"/>
+    <sheet name="regle_taylor" sheetId="88" state="visible" r:id="rId88"/>
+    <sheet name="regression_multifeatures" sheetId="89" state="visible" r:id="rId89"/>
+    <sheet name="rotation_risk_on_off" sheetId="90" state="visible" r:id="rId90"/>
+    <sheet name="rotation_sectorielle" sheetId="91" state="visible" r:id="rId91"/>
+    <sheet name="ruptures_perimetre" sheetId="92" state="visible" r:id="rId92"/>
+    <sheet name="sahm_rule" sheetId="93" state="visible" r:id="rId93"/>
+    <sheet name="saisonnalite" sheetId="94" state="visible" r:id="rId94"/>
+    <sheet name="screening_features" sheetId="95" state="visible" r:id="rId95"/>
+    <sheet name="similarite_vocabulaire_minutes" sheetId="96" state="visible" r:id="rId96"/>
+    <sheet name="sizing_robuste" sheetId="97" state="visible" r:id="rId97"/>
+    <sheet name="skew_kurtosis" sheetId="98" state="visible" r:id="rId98"/>
+    <sheet name="soutenabilite_dette" sheetId="99" state="visible" r:id="rId99"/>
+    <sheet name="stacking" sheetId="100" state="visible" r:id="rId100"/>
+    <sheet name="stationnarite_taux" sheetId="101" state="visible" r:id="rId101"/>
+    <sheet name="stress_test_historique" sheetId="102" state="visible" r:id="rId102"/>
+    <sheet name="surprise_inflation" sheetId="103" state="visible" r:id="rId103"/>
+    <sheet name="surprise_macro_composite" sheetId="104" state="visible" r:id="rId104"/>
+    <sheet name="taux_reel_us" sheetId="105" state="visible" r:id="rId105"/>
+    <sheet name="test_chow" sheetId="106" state="visible" r:id="rId106"/>
+    <sheet name="test_overfitting_momentum" sheetId="107" state="visible" r:id="rId107"/>
+    <sheet name="ton_banques_centrales" sheetId="108" state="visible" r:id="rId108"/>
+    <sheet name="ton_fomc" sheetId="109" state="visible" r:id="rId109"/>
+    <sheet name="ton_minutes_fomc" sheetId="110" state="visible" r:id="rId110"/>
+    <sheet name="univers_sources" sheetId="111" state="visible" r:id="rId111"/>
+    <sheet name="var_conditionnelle_regime" sheetId="112" state="visible" r:id="rId112"/>
+    <sheet name="var_drawdown" sheetId="113" state="visible" r:id="rId113"/>
+    <sheet name="var_sp500_vix" sheetId="114" state="visible" r:id="rId114"/>
+    <sheet name="vol_cross_asset" sheetId="115" state="visible" r:id="rId115"/>
+    <sheet name="volatilite_ewma" sheetId="116" state="visible" r:id="rId116"/>
+    <sheet name="walkforward_direction_sp500" sheetId="117" state="visible" r:id="rId117"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-25 08:06 UTC</t>
+          <t>Genere le 2026-09-25 08:10 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-25 08:06 UTC</t>
+          <t>Rapport global — 2026-09-25 08:10 UTC</t>
         </is>
       </c>
     </row>
@@ -1240,7 +1240,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.4230376399790394 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.05274682750137143 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-24)_</t>
+          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.42303763997892396 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.0527468275013714 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-24)_</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rationalise la structure des rapports
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -1,129 +1,129 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Lecture du jour" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="activite_zone_euro" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="analyse_spectrale" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="anomalie_multivariee" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="arima" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="balance_commerciale" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="beta_facteur_macro" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="beta_vol" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="bilans_banques_centrales" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="carry_proxy" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="causalite_granger" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="changepoint_volatilite" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="chemin_taux_fed" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="choc_taux" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="choc_vol_parametrique" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="clustering_marches" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="coherence_fed" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="cointegration_secteurs" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="cointegration_taux" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="complexite_texte_fomc" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="complexite_texte_minutes" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="concentration_traders" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="conditions_financieres" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="correlation_cot_prix" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="correlation_facteurs" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="correlation_glissante" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="correlations_positionnement" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="courbe_taux_us" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="couts_transaction" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet name="covar" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet name="crowding_cross_asset" sheetId="31" state="visible" r:id="rId31"/>
-    <sheet name="cycle_credit" sheetId="32" state="visible" r:id="rId32"/>
-    <sheet name="cycle_immobilier" sheetId="33" state="visible" r:id="rId33"/>
-    <sheet name="decision_stump" sheetId="34" state="visible" r:id="rId34"/>
-    <sheet name="decomposition_stl" sheetId="35" state="visible" r:id="rId35"/>
-    <sheet name="decomposition_variance" sheetId="36" state="visible" r:id="rId36"/>
-    <sheet name="dependance_queue" sheetId="37" state="visible" r:id="rId37"/>
-    <sheet name="detection_saut" sheetId="38" state="visible" r:id="rId38"/>
-    <sheet name="differentiel_taux_change" sheetId="39" state="visible" r:id="rId39"/>
-    <sheet name="dispersion_sectorielle" sheetId="40" state="visible" r:id="rId40"/>
-    <sheet name="divergence_cot_prix" sheetId="41" state="visible" r:id="rId41"/>
-    <sheet name="divergence_taux_directeurs" sheetId="42" state="visible" r:id="rId42"/>
-    <sheet name="dollar_smile" sheetId="43" state="visible" r:id="rId43"/>
-    <sheet name="ecart_communique_minutes" sheetId="44" state="visible" r:id="rId44"/>
-    <sheet name="emission_tresor_us" sheetId="45" state="visible" r:id="rId45"/>
-    <sheet name="ensemble_signaux" sheetId="46" state="visible" r:id="rId46"/>
-    <sheet name="entites_geographiques_minutes" sheetId="47" state="visible" r:id="rId47"/>
-    <sheet name="extremes_historiques" sheetId="48" state="visible" r:id="rId48"/>
-    <sheet name="facteur_qualite_credit" sheetId="49" state="visible" r:id="rId49"/>
-    <sheet name="fraicheur" sheetId="50" state="visible" r:id="rId50"/>
-    <sheet name="frequence_mots_cles_fomc" sheetId="51" state="visible" r:id="rId51"/>
-    <sheet name="frequence_mots_cles_minutes" sheetId="52" state="visible" r:id="rId52"/>
-    <sheet name="garch" sheetId="53" state="visible" r:id="rId53"/>
-    <sheet name="hp_filter_taux" sheetId="54" state="visible" r:id="rId54"/>
-    <sheet name="hurst" sheetId="55" state="visible" r:id="rId55"/>
-    <sheet name="importance_permutation" sheetId="56" state="visible" r:id="rId56"/>
-    <sheet name="indices_mondiaux" sheetId="57" state="visible" r:id="rId57"/>
-    <sheet name="inflation_comparee" sheetId="58" state="visible" r:id="rId58"/>
-    <sheet name="intensite_desaccord" sheetId="59" state="visible" r:id="rId59"/>
-    <sheet name="kalman_niveau_local" sheetId="60" state="visible" r:id="rId60"/>
-    <sheet name="kmeans_regimes" sheetId="61" state="visible" r:id="rId61"/>
-    <sheet name="langage_prudence" sheetId="62" state="visible" r:id="rId62"/>
-    <sheet name="liquidite_nette_fed" sheetId="63" state="visible" r:id="rId63"/>
-    <sheet name="lisibilite_flesch_kincaid" sheetId="64" state="visible" r:id="rId64"/>
-    <sheet name="low_volatility" sheetId="65" state="visible" r:id="rId65"/>
-    <sheet name="matieres_premieres_macro" sheetId="66" state="visible" r:id="rId66"/>
-    <sheet name="metaux_precieux" sheetId="67" state="visible" r:id="rId67"/>
-    <sheet name="momentum_credit" sheetId="68" state="visible" r:id="rId68"/>
-    <sheet name="momentum_cross_sectional" sheetId="69" state="visible" r:id="rId69"/>
-    <sheet name="momentum_positionnement" sheetId="70" state="visible" r:id="rId70"/>
-    <sheet name="momentum_prix" sheetId="71" state="visible" r:id="rId71"/>
-    <sheet name="nombre_effectif_paris" sheetId="72" state="visible" r:id="rId72"/>
-    <sheet name="ornstein_uhlenbeck_credit" sheetId="73" state="visible" r:id="rId73"/>
-    <sheet name="ornstein_uhlenbeck_vix" sheetId="74" state="visible" r:id="rId74"/>
-    <sheet name="pca_taux" sheetId="75" state="visible" r:id="rId75"/>
-    <sheet name="pentes_courbes" sheetId="76" state="visible" r:id="rId76"/>
-    <sheet name="persistance_extremes" sheetId="77" state="visible" r:id="rId77"/>
-    <sheet name="positionnement_cot" sheetId="78" state="visible" r:id="rId78"/>
-    <sheet name="positionnement_courbe_taux" sheetId="79" state="visible" r:id="rId79"/>
-    <sheet name="positionnement_devises" sheetId="80" state="visible" r:id="rId80"/>
-    <sheet name="prevision_vol_regression" sheetId="81" state="visible" r:id="rId81"/>
-    <sheet name="qualite_regime_macro" sheetId="82" state="visible" r:id="rId82"/>
-    <sheet name="ratio_commercial_speculatif" sheetId="83" state="visible" r:id="rId83"/>
-    <sheet name="ratios_conditionnels_regime" sheetId="84" state="visible" r:id="rId84"/>
-    <sheet name="ratios_performance" sheetId="85" state="visible" r:id="rId85"/>
-    <sheet name="reer_us" sheetId="86" state="visible" r:id="rId86"/>
-    <sheet name="regime_monetaire_emploi" sheetId="87" state="visible" r:id="rId87"/>
-    <sheet name="regle_taylor" sheetId="88" state="visible" r:id="rId88"/>
-    <sheet name="regression_multifeatures" sheetId="89" state="visible" r:id="rId89"/>
-    <sheet name="rotation_risk_on_off" sheetId="90" state="visible" r:id="rId90"/>
-    <sheet name="rotation_sectorielle" sheetId="91" state="visible" r:id="rId91"/>
-    <sheet name="ruptures_perimetre" sheetId="92" state="visible" r:id="rId92"/>
-    <sheet name="sahm_rule" sheetId="93" state="visible" r:id="rId93"/>
-    <sheet name="saisonnalite" sheetId="94" state="visible" r:id="rId94"/>
-    <sheet name="screening_features" sheetId="95" state="visible" r:id="rId95"/>
-    <sheet name="similarite_vocabulaire_minutes" sheetId="96" state="visible" r:id="rId96"/>
-    <sheet name="sizing_robuste" sheetId="97" state="visible" r:id="rId97"/>
-    <sheet name="skew_kurtosis" sheetId="98" state="visible" r:id="rId98"/>
-    <sheet name="soutenabilite_dette" sheetId="99" state="visible" r:id="rId99"/>
-    <sheet name="stacking" sheetId="100" state="visible" r:id="rId100"/>
-    <sheet name="stationnarite_taux" sheetId="101" state="visible" r:id="rId101"/>
-    <sheet name="stress_test_historique" sheetId="102" state="visible" r:id="rId102"/>
-    <sheet name="surprise_inflation" sheetId="103" state="visible" r:id="rId103"/>
-    <sheet name="surprise_macro_composite" sheetId="104" state="visible" r:id="rId104"/>
-    <sheet name="taux_reel_us" sheetId="105" state="visible" r:id="rId105"/>
-    <sheet name="test_chow" sheetId="106" state="visible" r:id="rId106"/>
-    <sheet name="test_overfitting_momentum" sheetId="107" state="visible" r:id="rId107"/>
-    <sheet name="ton_banques_centrales" sheetId="108" state="visible" r:id="rId108"/>
-    <sheet name="ton_fomc" sheetId="109" state="visible" r:id="rId109"/>
-    <sheet name="ton_minutes_fomc" sheetId="110" state="visible" r:id="rId110"/>
-    <sheet name="univers_sources" sheetId="111" state="visible" r:id="rId111"/>
-    <sheet name="var_conditionnelle_regime" sheetId="112" state="visible" r:id="rId112"/>
-    <sheet name="var_drawdown" sheetId="113" state="visible" r:id="rId113"/>
-    <sheet name="var_sp500_vix" sheetId="114" state="visible" r:id="rId114"/>
-    <sheet name="vol_cross_asset" sheetId="115" state="visible" r:id="rId115"/>
-    <sheet name="volatilite_ewma" sheetId="116" state="visible" r:id="rId116"/>
-    <sheet name="walkforward_direction_sp500" sheetId="117" state="visible" r:id="rId117"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lecture du jour" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="activite_zone_euro" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="analyse_spectrale" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="anomalie_multivariee" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="arima" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="balance_commerciale" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="beta_facteur_macro" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="beta_vol" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="bilans_banques_centrales" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="carry_proxy" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="causalite_granger" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="changepoint_volatilite" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="chemin_taux_fed" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choc_taux" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choc_vol_parametrique" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="clustering_marches" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="coherence_fed" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cointegration_secteurs" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cointegration_taux" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="complexite_texte_fomc" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="complexite_texte_minutes" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="concentration_traders" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="conditions_financieres" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="correlation_cot_prix" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="correlation_facteurs" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="correlation_glissante" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="correlations_positionnement" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="courbe_taux_us" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="couts_transaction" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="covar" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="crowding_cross_asset" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cycle_credit" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cycle_immobilier" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="decision_stump" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="decomposition_stl" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="decomposition_variance" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="dependance_queue" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="detection_saut" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="differentiel_taux_change" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="dispersion_sectorielle" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="divergence_cot_prix" sheetId="41" state="visible" r:id="rId41"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="divergence_taux_directeurs" sheetId="42" state="visible" r:id="rId42"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="dollar_smile" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ecart_communique_minutes" sheetId="44" state="visible" r:id="rId44"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="emission_tresor_us" sheetId="45" state="visible" r:id="rId45"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ensemble_signaux" sheetId="46" state="visible" r:id="rId46"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="entites_geographiques_minutes" sheetId="47" state="visible" r:id="rId47"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extremes_historiques" sheetId="48" state="visible" r:id="rId48"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="facteur_qualite_credit" sheetId="49" state="visible" r:id="rId49"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="fraicheur" sheetId="50" state="visible" r:id="rId50"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="frequence_mots_cles_fomc" sheetId="51" state="visible" r:id="rId51"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="frequence_mots_cles_minutes" sheetId="52" state="visible" r:id="rId52"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="garch" sheetId="53" state="visible" r:id="rId53"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hp_filter_taux" sheetId="54" state="visible" r:id="rId54"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hurst" sheetId="55" state="visible" r:id="rId55"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="importance_permutation" sheetId="56" state="visible" r:id="rId56"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="indices_mondiaux" sheetId="57" state="visible" r:id="rId57"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="inflation_comparee" sheetId="58" state="visible" r:id="rId58"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="intensite_desaccord" sheetId="59" state="visible" r:id="rId59"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="kalman_niveau_local" sheetId="60" state="visible" r:id="rId60"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="kmeans_regimes" sheetId="61" state="visible" r:id="rId61"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="langage_prudence" sheetId="62" state="visible" r:id="rId62"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="liquidite_nette_fed" sheetId="63" state="visible" r:id="rId63"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="lisibilite_flesch_kincaid" sheetId="64" state="visible" r:id="rId64"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="low_volatility" sheetId="65" state="visible" r:id="rId65"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="matieres_premieres_macro" sheetId="66" state="visible" r:id="rId66"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="metaux_precieux" sheetId="67" state="visible" r:id="rId67"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="momentum_credit" sheetId="68" state="visible" r:id="rId68"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="momentum_cross_sectional" sheetId="69" state="visible" r:id="rId69"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="momentum_positionnement" sheetId="70" state="visible" r:id="rId70"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="momentum_prix" sheetId="71" state="visible" r:id="rId71"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="nombre_effectif_paris" sheetId="72" state="visible" r:id="rId72"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ornstein_uhlenbeck_credit" sheetId="73" state="visible" r:id="rId73"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ornstein_uhlenbeck_vix" sheetId="74" state="visible" r:id="rId74"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pca_taux" sheetId="75" state="visible" r:id="rId75"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pentes_courbes" sheetId="76" state="visible" r:id="rId76"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="persistance_extremes" sheetId="77" state="visible" r:id="rId77"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="positionnement_cot" sheetId="78" state="visible" r:id="rId78"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="positionnement_courbe_taux" sheetId="79" state="visible" r:id="rId79"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="positionnement_devises" sheetId="80" state="visible" r:id="rId80"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="prevision_vol_regression" sheetId="81" state="visible" r:id="rId81"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="qualite_regime_macro" sheetId="82" state="visible" r:id="rId82"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ratio_commercial_speculatif" sheetId="83" state="visible" r:id="rId83"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ratios_conditionnels_regime" sheetId="84" state="visible" r:id="rId84"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ratios_performance" sheetId="85" state="visible" r:id="rId85"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="reer_us" sheetId="86" state="visible" r:id="rId86"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="regime_monetaire_emploi" sheetId="87" state="visible" r:id="rId87"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="regle_taylor" sheetId="88" state="visible" r:id="rId88"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="regression_multifeatures" sheetId="89" state="visible" r:id="rId89"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="rotation_risk_on_off" sheetId="90" state="visible" r:id="rId90"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="rotation_sectorielle" sheetId="91" state="visible" r:id="rId91"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ruptures_perimetre" sheetId="92" state="visible" r:id="rId92"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sahm_rule" sheetId="93" state="visible" r:id="rId93"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="saisonnalite" sheetId="94" state="visible" r:id="rId94"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="screening_features" sheetId="95" state="visible" r:id="rId95"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="similarite_vocabulaire_minutes" sheetId="96" state="visible" r:id="rId96"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sizing_robuste" sheetId="97" state="visible" r:id="rId97"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="skew_kurtosis" sheetId="98" state="visible" r:id="rId98"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="soutenabilite_dette" sheetId="99" state="visible" r:id="rId99"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="stacking" sheetId="100" state="visible" r:id="rId100"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="stationnarite_taux" sheetId="101" state="visible" r:id="rId101"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="stress_test_historique" sheetId="102" state="visible" r:id="rId102"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="surprise_inflation" sheetId="103" state="visible" r:id="rId103"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="surprise_macro_composite" sheetId="104" state="visible" r:id="rId104"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="taux_reel_us" sheetId="105" state="visible" r:id="rId105"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="test_chow" sheetId="106" state="visible" r:id="rId106"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="test_overfitting_momentum" sheetId="107" state="visible" r:id="rId107"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ton_banques_centrales" sheetId="108" state="visible" r:id="rId108"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ton_fomc" sheetId="109" state="visible" r:id="rId109"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ton_minutes_fomc" sheetId="110" state="visible" r:id="rId110"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="univers_sources" sheetId="111" state="visible" r:id="rId111"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="var_conditionnelle_regime" sheetId="112" state="visible" r:id="rId112"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="var_drawdown" sheetId="113" state="visible" r:id="rId113"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="var_sp500_vix" sheetId="114" state="visible" r:id="rId114"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="vol_cross_asset" sheetId="115" state="visible" r:id="rId115"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="volatilite_ewma" sheetId="116" state="visible" r:id="rId116"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="walkforward_direction_sp500" sheetId="117" state="visible" r:id="rId117"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-25 08:10 UTC</t>
+          <t>Genere le 2026-09-25 08:20 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-25 08:10 UTC</t>
+          <t>Rapport global — 2026-09-25 08:20 UTC</t>
         </is>
       </c>
     </row>
@@ -1240,7 +1240,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.42303763997892396 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.0527468275013714 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-24)_</t>
+          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.42303763997917443 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.052746827501372995 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-24)_</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Recherche - publication 2026-09-25T08:26Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -1,129 +1,129 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lecture du jour" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="activite_zone_euro" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="analyse_spectrale" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="anomalie_multivariee" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="arima" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="balance_commerciale" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="beta_facteur_macro" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="beta_vol" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="bilans_banques_centrales" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="carry_proxy" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="causalite_granger" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="changepoint_volatilite" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="chemin_taux_fed" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choc_taux" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choc_vol_parametrique" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="clustering_marches" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="coherence_fed" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cointegration_secteurs" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cointegration_taux" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="complexite_texte_fomc" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="complexite_texte_minutes" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="concentration_traders" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="conditions_financieres" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="correlation_cot_prix" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="correlation_facteurs" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="correlation_glissante" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="correlations_positionnement" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="courbe_taux_us" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="couts_transaction" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="covar" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="crowding_cross_asset" sheetId="31" state="visible" r:id="rId31"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cycle_credit" sheetId="32" state="visible" r:id="rId32"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cycle_immobilier" sheetId="33" state="visible" r:id="rId33"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="decision_stump" sheetId="34" state="visible" r:id="rId34"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="decomposition_stl" sheetId="35" state="visible" r:id="rId35"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="decomposition_variance" sheetId="36" state="visible" r:id="rId36"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="dependance_queue" sheetId="37" state="visible" r:id="rId37"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="detection_saut" sheetId="38" state="visible" r:id="rId38"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="differentiel_taux_change" sheetId="39" state="visible" r:id="rId39"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="dispersion_sectorielle" sheetId="40" state="visible" r:id="rId40"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="divergence_cot_prix" sheetId="41" state="visible" r:id="rId41"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="divergence_taux_directeurs" sheetId="42" state="visible" r:id="rId42"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="dollar_smile" sheetId="43" state="visible" r:id="rId43"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ecart_communique_minutes" sheetId="44" state="visible" r:id="rId44"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="emission_tresor_us" sheetId="45" state="visible" r:id="rId45"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ensemble_signaux" sheetId="46" state="visible" r:id="rId46"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="entites_geographiques_minutes" sheetId="47" state="visible" r:id="rId47"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="extremes_historiques" sheetId="48" state="visible" r:id="rId48"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="facteur_qualite_credit" sheetId="49" state="visible" r:id="rId49"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="fraicheur" sheetId="50" state="visible" r:id="rId50"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="frequence_mots_cles_fomc" sheetId="51" state="visible" r:id="rId51"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="frequence_mots_cles_minutes" sheetId="52" state="visible" r:id="rId52"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="garch" sheetId="53" state="visible" r:id="rId53"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hp_filter_taux" sheetId="54" state="visible" r:id="rId54"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="hurst" sheetId="55" state="visible" r:id="rId55"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="importance_permutation" sheetId="56" state="visible" r:id="rId56"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="indices_mondiaux" sheetId="57" state="visible" r:id="rId57"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="inflation_comparee" sheetId="58" state="visible" r:id="rId58"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="intensite_desaccord" sheetId="59" state="visible" r:id="rId59"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="kalman_niveau_local" sheetId="60" state="visible" r:id="rId60"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="kmeans_regimes" sheetId="61" state="visible" r:id="rId61"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="langage_prudence" sheetId="62" state="visible" r:id="rId62"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="liquidite_nette_fed" sheetId="63" state="visible" r:id="rId63"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="lisibilite_flesch_kincaid" sheetId="64" state="visible" r:id="rId64"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="low_volatility" sheetId="65" state="visible" r:id="rId65"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="matieres_premieres_macro" sheetId="66" state="visible" r:id="rId66"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="metaux_precieux" sheetId="67" state="visible" r:id="rId67"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="momentum_credit" sheetId="68" state="visible" r:id="rId68"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="momentum_cross_sectional" sheetId="69" state="visible" r:id="rId69"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="momentum_positionnement" sheetId="70" state="visible" r:id="rId70"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="momentum_prix" sheetId="71" state="visible" r:id="rId71"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="nombre_effectif_paris" sheetId="72" state="visible" r:id="rId72"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ornstein_uhlenbeck_credit" sheetId="73" state="visible" r:id="rId73"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ornstein_uhlenbeck_vix" sheetId="74" state="visible" r:id="rId74"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pca_taux" sheetId="75" state="visible" r:id="rId75"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pentes_courbes" sheetId="76" state="visible" r:id="rId76"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="persistance_extremes" sheetId="77" state="visible" r:id="rId77"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="positionnement_cot" sheetId="78" state="visible" r:id="rId78"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="positionnement_courbe_taux" sheetId="79" state="visible" r:id="rId79"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="positionnement_devises" sheetId="80" state="visible" r:id="rId80"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="prevision_vol_regression" sheetId="81" state="visible" r:id="rId81"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="qualite_regime_macro" sheetId="82" state="visible" r:id="rId82"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ratio_commercial_speculatif" sheetId="83" state="visible" r:id="rId83"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ratios_conditionnels_regime" sheetId="84" state="visible" r:id="rId84"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ratios_performance" sheetId="85" state="visible" r:id="rId85"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="reer_us" sheetId="86" state="visible" r:id="rId86"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="regime_monetaire_emploi" sheetId="87" state="visible" r:id="rId87"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="regle_taylor" sheetId="88" state="visible" r:id="rId88"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="regression_multifeatures" sheetId="89" state="visible" r:id="rId89"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="rotation_risk_on_off" sheetId="90" state="visible" r:id="rId90"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="rotation_sectorielle" sheetId="91" state="visible" r:id="rId91"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ruptures_perimetre" sheetId="92" state="visible" r:id="rId92"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sahm_rule" sheetId="93" state="visible" r:id="rId93"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="saisonnalite" sheetId="94" state="visible" r:id="rId94"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="screening_features" sheetId="95" state="visible" r:id="rId95"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="similarite_vocabulaire_minutes" sheetId="96" state="visible" r:id="rId96"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sizing_robuste" sheetId="97" state="visible" r:id="rId97"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="skew_kurtosis" sheetId="98" state="visible" r:id="rId98"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="soutenabilite_dette" sheetId="99" state="visible" r:id="rId99"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="stacking" sheetId="100" state="visible" r:id="rId100"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="stationnarite_taux" sheetId="101" state="visible" r:id="rId101"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="stress_test_historique" sheetId="102" state="visible" r:id="rId102"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="surprise_inflation" sheetId="103" state="visible" r:id="rId103"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="surprise_macro_composite" sheetId="104" state="visible" r:id="rId104"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="taux_reel_us" sheetId="105" state="visible" r:id="rId105"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="test_chow" sheetId="106" state="visible" r:id="rId106"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="test_overfitting_momentum" sheetId="107" state="visible" r:id="rId107"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ton_banques_centrales" sheetId="108" state="visible" r:id="rId108"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ton_fomc" sheetId="109" state="visible" r:id="rId109"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ton_minutes_fomc" sheetId="110" state="visible" r:id="rId110"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="univers_sources" sheetId="111" state="visible" r:id="rId111"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="var_conditionnelle_regime" sheetId="112" state="visible" r:id="rId112"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="var_drawdown" sheetId="113" state="visible" r:id="rId113"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="var_sp500_vix" sheetId="114" state="visible" r:id="rId114"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="vol_cross_asset" sheetId="115" state="visible" r:id="rId115"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="volatilite_ewma" sheetId="116" state="visible" r:id="rId116"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="walkforward_direction_sp500" sheetId="117" state="visible" r:id="rId117"/>
+    <sheet name="Lecture du jour" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="activite_zone_euro" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="analyse_spectrale" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="anomalie_multivariee" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="arima" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="balance_commerciale" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="beta_facteur_macro" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="beta_vol" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="bilans_banques_centrales" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="carry_proxy" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="causalite_granger" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="changepoint_volatilite" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="chemin_taux_fed" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="choc_taux" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="choc_vol_parametrique" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="clustering_marches" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="coherence_fed" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="cointegration_secteurs" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="cointegration_taux" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="complexite_texte_fomc" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="complexite_texte_minutes" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="concentration_traders" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="conditions_financieres" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="correlation_cot_prix" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="correlation_facteurs" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="correlation_glissante" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="correlations_positionnement" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="courbe_taux_us" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="couts_transaction" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="covar" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="crowding_cross_asset" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet name="cycle_credit" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="cycle_immobilier" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet name="decision_stump" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="decomposition_stl" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet name="decomposition_variance" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet name="dependance_queue" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet name="detection_saut" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet name="differentiel_taux_change" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet name="dispersion_sectorielle" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet name="divergence_cot_prix" sheetId="41" state="visible" r:id="rId41"/>
+    <sheet name="divergence_taux_directeurs" sheetId="42" state="visible" r:id="rId42"/>
+    <sheet name="dollar_smile" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet name="ecart_communique_minutes" sheetId="44" state="visible" r:id="rId44"/>
+    <sheet name="emission_tresor_us" sheetId="45" state="visible" r:id="rId45"/>
+    <sheet name="ensemble_signaux" sheetId="46" state="visible" r:id="rId46"/>
+    <sheet name="entites_geographiques_minutes" sheetId="47" state="visible" r:id="rId47"/>
+    <sheet name="extremes_historiques" sheetId="48" state="visible" r:id="rId48"/>
+    <sheet name="facteur_qualite_credit" sheetId="49" state="visible" r:id="rId49"/>
+    <sheet name="fraicheur" sheetId="50" state="visible" r:id="rId50"/>
+    <sheet name="frequence_mots_cles_fomc" sheetId="51" state="visible" r:id="rId51"/>
+    <sheet name="frequence_mots_cles_minutes" sheetId="52" state="visible" r:id="rId52"/>
+    <sheet name="garch" sheetId="53" state="visible" r:id="rId53"/>
+    <sheet name="hp_filter_taux" sheetId="54" state="visible" r:id="rId54"/>
+    <sheet name="hurst" sheetId="55" state="visible" r:id="rId55"/>
+    <sheet name="importance_permutation" sheetId="56" state="visible" r:id="rId56"/>
+    <sheet name="indices_mondiaux" sheetId="57" state="visible" r:id="rId57"/>
+    <sheet name="inflation_comparee" sheetId="58" state="visible" r:id="rId58"/>
+    <sheet name="intensite_desaccord" sheetId="59" state="visible" r:id="rId59"/>
+    <sheet name="kalman_niveau_local" sheetId="60" state="visible" r:id="rId60"/>
+    <sheet name="kmeans_regimes" sheetId="61" state="visible" r:id="rId61"/>
+    <sheet name="langage_prudence" sheetId="62" state="visible" r:id="rId62"/>
+    <sheet name="liquidite_nette_fed" sheetId="63" state="visible" r:id="rId63"/>
+    <sheet name="lisibilite_flesch_kincaid" sheetId="64" state="visible" r:id="rId64"/>
+    <sheet name="low_volatility" sheetId="65" state="visible" r:id="rId65"/>
+    <sheet name="matieres_premieres_macro" sheetId="66" state="visible" r:id="rId66"/>
+    <sheet name="metaux_precieux" sheetId="67" state="visible" r:id="rId67"/>
+    <sheet name="momentum_credit" sheetId="68" state="visible" r:id="rId68"/>
+    <sheet name="momentum_cross_sectional" sheetId="69" state="visible" r:id="rId69"/>
+    <sheet name="momentum_positionnement" sheetId="70" state="visible" r:id="rId70"/>
+    <sheet name="momentum_prix" sheetId="71" state="visible" r:id="rId71"/>
+    <sheet name="nombre_effectif_paris" sheetId="72" state="visible" r:id="rId72"/>
+    <sheet name="ornstein_uhlenbeck_credit" sheetId="73" state="visible" r:id="rId73"/>
+    <sheet name="ornstein_uhlenbeck_vix" sheetId="74" state="visible" r:id="rId74"/>
+    <sheet name="pca_taux" sheetId="75" state="visible" r:id="rId75"/>
+    <sheet name="pentes_courbes" sheetId="76" state="visible" r:id="rId76"/>
+    <sheet name="persistance_extremes" sheetId="77" state="visible" r:id="rId77"/>
+    <sheet name="positionnement_cot" sheetId="78" state="visible" r:id="rId78"/>
+    <sheet name="positionnement_courbe_taux" sheetId="79" state="visible" r:id="rId79"/>
+    <sheet name="positionnement_devises" sheetId="80" state="visible" r:id="rId80"/>
+    <sheet name="prevision_vol_regression" sheetId="81" state="visible" r:id="rId81"/>
+    <sheet name="qualite_regime_macro" sheetId="82" state="visible" r:id="rId82"/>
+    <sheet name="ratio_commercial_speculatif" sheetId="83" state="visible" r:id="rId83"/>
+    <sheet name="ratios_conditionnels_regime" sheetId="84" state="visible" r:id="rId84"/>
+    <sheet name="ratios_performance" sheetId="85" state="visible" r:id="rId85"/>
+    <sheet name="reer_us" sheetId="86" state="visible" r:id="rId86"/>
+    <sheet name="regime_monetaire_emploi" sheetId="87" state="visible" r:id="rId87"/>
+    <sheet name="regle_taylor" sheetId="88" state="visible" r:id="rId88"/>
+    <sheet name="regression_multifeatures" sheetId="89" state="visible" r:id="rId89"/>
+    <sheet name="rotation_risk_on_off" sheetId="90" state="visible" r:id="rId90"/>
+    <sheet name="rotation_sectorielle" sheetId="91" state="visible" r:id="rId91"/>
+    <sheet name="ruptures_perimetre" sheetId="92" state="visible" r:id="rId92"/>
+    <sheet name="sahm_rule" sheetId="93" state="visible" r:id="rId93"/>
+    <sheet name="saisonnalite" sheetId="94" state="visible" r:id="rId94"/>
+    <sheet name="screening_features" sheetId="95" state="visible" r:id="rId95"/>
+    <sheet name="similarite_vocabulaire_minutes" sheetId="96" state="visible" r:id="rId96"/>
+    <sheet name="sizing_robuste" sheetId="97" state="visible" r:id="rId97"/>
+    <sheet name="skew_kurtosis" sheetId="98" state="visible" r:id="rId98"/>
+    <sheet name="soutenabilite_dette" sheetId="99" state="visible" r:id="rId99"/>
+    <sheet name="stacking" sheetId="100" state="visible" r:id="rId100"/>
+    <sheet name="stationnarite_taux" sheetId="101" state="visible" r:id="rId101"/>
+    <sheet name="stress_test_historique" sheetId="102" state="visible" r:id="rId102"/>
+    <sheet name="surprise_inflation" sheetId="103" state="visible" r:id="rId103"/>
+    <sheet name="surprise_macro_composite" sheetId="104" state="visible" r:id="rId104"/>
+    <sheet name="taux_reel_us" sheetId="105" state="visible" r:id="rId105"/>
+    <sheet name="test_chow" sheetId="106" state="visible" r:id="rId106"/>
+    <sheet name="test_overfitting_momentum" sheetId="107" state="visible" r:id="rId107"/>
+    <sheet name="ton_banques_centrales" sheetId="108" state="visible" r:id="rId108"/>
+    <sheet name="ton_fomc" sheetId="109" state="visible" r:id="rId109"/>
+    <sheet name="ton_minutes_fomc" sheetId="110" state="visible" r:id="rId110"/>
+    <sheet name="univers_sources" sheetId="111" state="visible" r:id="rId111"/>
+    <sheet name="var_conditionnelle_regime" sheetId="112" state="visible" r:id="rId112"/>
+    <sheet name="var_drawdown" sheetId="113" state="visible" r:id="rId113"/>
+    <sheet name="var_sp500_vix" sheetId="114" state="visible" r:id="rId114"/>
+    <sheet name="vol_cross_asset" sheetId="115" state="visible" r:id="rId115"/>
+    <sheet name="volatilite_ewma" sheetId="116" state="visible" r:id="rId116"/>
+    <sheet name="walkforward_direction_sp500" sheetId="117" state="visible" r:id="rId117"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-25 08:20 UTC</t>
+          <t>Genere le 2026-09-25 08:26 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-25 08:20 UTC</t>
+          <t>Rapport global — 2026-09-25 08:26 UTC</t>
         </is>
       </c>
     </row>
@@ -1240,7 +1240,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.42303763997917443 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.052746827501372995 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-24)_</t>
+          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.42303763997892396 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.0527468275013714 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-24)_</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Recherche - publication 2026-09-25T14:10Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-25 08:26 UTC</t>
+          <t>Genere le 2026-09-25 14:10 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-25 08:26 UTC</t>
+          <t>Rapport global — 2026-09-25 14:10 UTC</t>
         </is>
       </c>
     </row>
@@ -792,14 +792,14 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>**Soutenabilite dette** — 8 pays. charge la plus lourde : Canada a 25.5% du revenu. taux 10 ans AU-DESSUS de l'inflation dans 5 pays -- Royaume-Uni (+2.1pt), Etats-Unis (+1.7pt), Japon (+1.0pt), Canada (+0.9pt), Zone euro (+0.8pt). Configuration ou le ratio d'endettement monte meme a budget primaire equilibre (approximation : croissance nominale reduite a l'inflation) _(observation : date non exposee)_</t>
+          <t>**Soutenabilite dette** — 8 pays. charge la plus lourde : Canada a 25.5% du revenu. taux 10 ans AU-DESSUS de l'inflation dans 5 pays -- Royaume-Uni (+2.2pt), Etats-Unis (+1.7pt), Japon (+1.0pt), Canada (+0.9pt), Zone euro (+0.8pt). Configuration ou le ratio d'endettement monte meme a budget primaire equilibre (approximation : croissance nominale reduite a l'inflation) _(observation : date non exposee)_</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>**Matieres premieres macro** — ratio cuivre/or stable -- pas de signal net sur la croissance (+4.2% sur 3 mois). Brent 99.2$ (+37.9% sur 3 mois, +43.0% sur 12 mois), gaz +1.2% sur 3 mois, ecart Brent-WTI +5.7$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-25)_</t>
+          <t>**Matieres premieres macro** — ratio cuivre/or stable -- pas de signal net sur la croissance (+4.0% sur 3 mois). Brent 98.8$ (+37.2% sur 3 mois, +42.3% sur 12 mois), gaz +0.7% sur 3 mois, ecart Brent-WTI +5.9$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
@@ -862,7 +862,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>**Conditions financieres** — indice conditions financieres=+0.121 (3 composantes: {'taux_directeur': 0.5989298167517355, 'courbe_inversee': 0.3359699129001652, 'vix': -0.5733149066357414}) -- conditions proches de la normale _(observation : 2026-09-23)_</t>
+          <t>**Conditions financieres** — indice conditions financieres=+0.102 (3 composantes: {'taux_directeur': 0.5989298167517355, 'courbe_inversee': 0.3359699129001652, 'vix': -0.6289631025613203}) -- conditions proches de la normale _(observation : 2026-09-23)_</t>
         </is>
       </c>
     </row>
@@ -960,7 +960,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>**Indices mondiaux** — 7 indices (devise locale) : Coree (KOSPI) +103.1% en tete sur 12 mois, Hong Kong (Hang Seng) -7.6% en queue -- ecart tres large entre blocs sur 12 mois (111pt) -- les cycles economiques ou les flux divergent nettement. ROTATION en cours : Coree (KOSPI) mene sur 12 mois mais Hong Kong (Hang Seng) a repris la tete sur 3 mois _(observation : 2026-09-25)_</t>
+          <t>**Indices mondiaux** — 7 indices (devise locale) : Coree (KOSPI) +103.1% en tete sur 12 mois, Hong Kong (Hang Seng) -7.5% en queue -- ecart tres large entre blocs sur 12 mois (111pt) -- les cycles economiques ou les flux divergent nettement. ROTATION en cours : Coree (KOSPI) mene sur 12 mois mais Hong Kong (Hang Seng) a repris la tete sur 3 mois _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
@@ -1191,7 +1191,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>**Vol cross asset** — 6 mesures de volatilite : Petrole (OVX) 87e pct, Or (GVZ) 81e pct, Taux US (MOVE) 55e pct, Nasdaq (VXN) 40e pct, Vol de la vol (VVIX) 36e pct, Actions US (VIX) 27e pct -- stress LOCALISE sur Petrole (OVX), Or (GVZ) pendant que le reste ne l'est pas -- episode propre a cette classe d'actifs, pas une aversion au risque d'ensemble _(observation : 2026-09-25)_</t>
+          <t>**Vol cross asset** — 6 mesures de volatilite : Petrole (OVX) 87e pct, Or (GVZ) 81e pct, Taux US (MOVE) 55e pct, Nasdaq (VXN) 40e pct, Vol de la vol (VVIX) 36e pct, Actions US (VIX) 23e pct -- stress LOCALISE sur Petrole (OVX), Or (GVZ) pendant que le reste ne l'est pas -- episode propre a cette classe d'actifs, pas une aversion au risque d'ensemble _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
@@ -1219,7 +1219,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>**Ornstein uhlenbeck vix** — VIX actuel=15.57, niveau moyen estime (mu)=20.20, demi-vie=28.8j, ecart actuel=-4.63 -- VIX actuel en-dessous de son niveau moyen de long terme _(observation : 2026-09-25)_</t>
+          <t>**Ornstein uhlenbeck vix** — VIX actuel=15.12, niveau moyen estime (mu)=20.20, demi-vie=28.8j, ecart actuel=-5.08 -- VIX actuel en-dessous de son niveau moyen de long terme _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
@@ -1233,21 +1233,21 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>**Kalman niveau local** — VIX observe=15.57, filtre Kalman=15.57 (ecart-type=0.62), ratio signal/bruit=0.2051 -- le filtre lisse fortement le bruit, reagit lentement (ecart obs.-filtre=-0.00) _(observation : 2026-09-25)_</t>
+          <t>**Kalman niveau local** — VIX observe=15.12, filtre Kalman=15.19 (ecart-type=0.62), ratio signal/bruit=0.2051 -- le filtre lisse fortement le bruit, reagit lentement (ecart obs.-filtre=-0.07) _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.42303763997892396 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.0527468275013714 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-24)_</t>
+          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.4230376399790394 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.05274682750137143 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-24)_</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>**Analyse spectrale** — 3 periodes dominantes (jours de bourse) : [2.2, 4.0, 5.4] -- cycle(s) connu(s) qui ressortent : 4.0j~hebdomadaire, 5.4j~hebdomadaire _(observation : 2026-09-25)_</t>
+          <t>**Analyse spectrale** — 3 periodes dominantes (jours de bourse) : [2.2, 5.4, 4.0] -- cycle(s) connu(s) qui ressortent : 5.4j~hebdomadaire, 4.0j~hebdomadaire _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
@@ -1317,7 +1317,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>**Qualite regime macro** — instabilite taux=0.0088, instabilite VIX=0.0669 -- score qualite du regime=-0.0379 (plus haut = regime plus stable/previsible) _(observation : 2026-09-23)_</t>
+          <t>**Qualite regime macro** — instabilite taux=0.0088, instabilite VIX=0.0671 -- score qualite du regime=-0.0379 (plus haut = regime plus stable/previsible) _(observation : 2026-09-23)_</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1331,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>**Decomposition stl** — VIX : tendance=15.57, composante saisonniere (periode 5j)=-0.375, residu=+0.372 -- la saisonnalite explique 0.71% de la variance totale (negligeable) _(observation : 2026-09-25)_</t>
+          <t>**Decomposition stl** — VIX : tendance=15.52, composante saisonniere (periode 5j)=-0.484, residu=+0.088 -- la saisonnalite explique 0.71% de la variance totale (negligeable) _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
@@ -4355,10 +4355,10 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>-0.1567</v>
+        <v>-0.159</v>
       </c>
       <c r="E54" t="n">
-        <v>0.9435</v>
+        <v>0.9432</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
@@ -7823,10 +7823,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>15.57</v>
+        <v>15.12</v>
       </c>
       <c r="D7" t="n">
-        <v>27.1</v>
+        <v>23.1</v>
       </c>
       <c r="E7" t="n">
         <v>1260</v>
@@ -17230,10 +17230,10 @@
         </is>
       </c>
       <c r="D109" t="n">
-        <v>-1.9657</v>
+        <v>-1.9682</v>
       </c>
       <c r="E109" t="n">
-        <v>0.5464</v>
+        <v>0.545</v>
       </c>
       <c r="F109" t="inlineStr">
         <is>
@@ -17258,10 +17258,10 @@
         </is>
       </c>
       <c r="D110" t="n">
-        <v>-2.2164</v>
+        <v>-2.2149</v>
       </c>
       <c r="E110" t="n">
-        <v>0.4159</v>
+        <v>0.4167</v>
       </c>
       <c r="F110" t="inlineStr">
         <is>
@@ -19803,7 +19803,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.1205</v>
+        <v>0.102</v>
       </c>
       <c r="C12" t="n">
         <v>3</v>
@@ -19815,7 +19815,7 @@
         <v>0.336</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.5733</v>
+        <v>-0.629</v>
       </c>
     </row>
   </sheetData>
@@ -32548,19 +32548,19 @@
         <v>2.2</v>
       </c>
       <c r="C12" t="n">
-        <v>433.22</v>
+        <v>432.96</v>
       </c>
       <c r="D12" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="E12" t="n">
+        <v>353.18</v>
+      </c>
+      <c r="F12" t="n">
         <v>4</v>
       </c>
-      <c r="E12" t="n">
-        <v>353.64</v>
-      </c>
-      <c r="F12" t="n">
-        <v>5.4</v>
-      </c>
       <c r="G12" t="n">
-        <v>352.39</v>
+        <v>352.55</v>
       </c>
     </row>
   </sheetData>
@@ -33784,13 +33784,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>15.573</v>
+        <v>15.516</v>
       </c>
       <c r="C12" t="n">
-        <v>-0.375</v>
+        <v>-0.484</v>
       </c>
       <c r="D12" t="n">
-        <v>0.372</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="E12" t="n">
         <v>0.71</v>
@@ -34637,11 +34637,11 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>-0.05</v>
+        <v>-0.112</v>
       </c>
       <c r="D4" t="n">
         <v>-0.022</v>
@@ -34782,11 +34782,11 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>-1.563</v>
+        <v>-1.549</v>
       </c>
       <c r="D9" t="n">
         <v>0.343</v>
@@ -44216,25 +44216,25 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>fred/IUDSOIA.csv</t>
+          <t>bilans/RBA_BILAN_TOTAL.csv</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="C172" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D172" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E172" t="n">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="F172" t="n">
-        <v>3000</v>
+        <v>691</v>
       </c>
       <c r="G172" t="inlineStr">
         <is>
@@ -44245,25 +44245,25 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>souverains/UK_10A.csv</t>
+          <t>bilans/RBA_OR_ET_DEVISES.csv</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="C173" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D173" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E173" t="n">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="F173" t="n">
-        <v>9281</v>
+        <v>691</v>
       </c>
       <c r="G173" t="inlineStr">
         <is>
@@ -44274,25 +44274,25 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>souverains/UK_20A.csv</t>
+          <t>bilans/RBA_TITRES_LOCAUX.csv</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="C174" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D174" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E174" t="n">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="F174" t="n">
-        <v>6752</v>
+        <v>691</v>
       </c>
       <c r="G174" t="inlineStr">
         <is>
@@ -44303,16 +44303,16 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>souverains/UK_5A.csv</t>
+          <t>fred/BAMLC0A0CM.csv</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="C175" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D175" t="n">
         <v>1</v>
@@ -44321,7 +44321,7 @@
         <v>42</v>
       </c>
       <c r="F175" t="n">
-        <v>8289</v>
+        <v>795</v>
       </c>
       <c r="G175" t="inlineStr">
         <is>
@@ -44332,7 +44332,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>bilans/RBA_BILAN_TOTAL.csv</t>
+          <t>fred/BAMLC0A0CMEY.csv</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -44344,13 +44344,13 @@
         <v>2</v>
       </c>
       <c r="D176" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E176" t="n">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="F176" t="n">
-        <v>691</v>
+        <v>795</v>
       </c>
       <c r="G176" t="inlineStr">
         <is>
@@ -44361,7 +44361,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>bilans/RBA_OR_ET_DEVISES.csv</t>
+          <t>fred/BAMLEMCBPIOAS.csv</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
@@ -44373,13 +44373,13 @@
         <v>2</v>
       </c>
       <c r="D177" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E177" t="n">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="F177" t="n">
-        <v>691</v>
+        <v>795</v>
       </c>
       <c r="G177" t="inlineStr">
         <is>
@@ -44390,7 +44390,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>bilans/RBA_TITRES_LOCAUX.csv</t>
+          <t>fred/BAMLEMFSFCRPIOAS.csv</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -44402,13 +44402,13 @@
         <v>2</v>
       </c>
       <c r="D178" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E178" t="n">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="F178" t="n">
-        <v>691</v>
+        <v>795</v>
       </c>
       <c r="G178" t="inlineStr">
         <is>
@@ -44419,7 +44419,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>fred/BAMLC0A0CM.csv</t>
+          <t>fred/BAMLEMHBHYCRPIOAS.csv</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -44448,7 +44448,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>fred/BAMLC0A0CMEY.csv</t>
+          <t>fred/BAMLEMPBPUBSICRPIOAS.csv</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -44477,7 +44477,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>fred/BAMLEMCBPIOAS.csv</t>
+          <t>fred/BAMLH0A0HYM2.csv</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -44506,7 +44506,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>fred/BAMLEMFSFCRPIOAS.csv</t>
+          <t>fred/BAMLHE00EHYIEY.csv</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
@@ -44535,7 +44535,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>fred/BAMLEMHBHYCRPIOAS.csv</t>
+          <t>fred/BAMLHE00EHYIOAS.csv</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -44564,7 +44564,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>fred/BAMLEMPBPUBSICRPIOAS.csv</t>
+          <t>fred/DFF.csv</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -44582,7 +44582,7 @@
         <v>42</v>
       </c>
       <c r="F184" t="n">
-        <v>795</v>
+        <v>3000</v>
       </c>
       <c r="G184" t="inlineStr">
         <is>
@@ -44593,7 +44593,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>fred/BAMLH0A0HYM2.csv</t>
+          <t>fred/DFII10.csv</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -44611,7 +44611,7 @@
         <v>42</v>
       </c>
       <c r="F185" t="n">
-        <v>795</v>
+        <v>3000</v>
       </c>
       <c r="G185" t="inlineStr">
         <is>
@@ -44622,7 +44622,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>fred/BAMLHE00EHYIEY.csv</t>
+          <t>fred/DFII5.csv</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -44640,7 +44640,7 @@
         <v>42</v>
       </c>
       <c r="F186" t="n">
-        <v>795</v>
+        <v>3000</v>
       </c>
       <c r="G186" t="inlineStr">
         <is>
@@ -44651,7 +44651,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>fred/BAMLHE00EHYIOAS.csv</t>
+          <t>fred/DGS1.csv</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -44669,7 +44669,7 @@
         <v>42</v>
       </c>
       <c r="F187" t="n">
-        <v>795</v>
+        <v>3000</v>
       </c>
       <c r="G187" t="inlineStr">
         <is>
@@ -44680,7 +44680,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>fred/DFF.csv</t>
+          <t>fred/DGS10.csv</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -44709,7 +44709,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>fred/DFII10.csv</t>
+          <t>fred/DGS1MO.csv</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -44738,7 +44738,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>fred/DFII5.csv</t>
+          <t>fred/DGS2.csv</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -44767,7 +44767,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>fred/DGS1.csv</t>
+          <t>fred/DGS30.csv</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -44796,7 +44796,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>fred/DGS10.csv</t>
+          <t>fred/DGS3MO.csv</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -44825,7 +44825,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>fred/DGS1MO.csv</t>
+          <t>fred/DGS5.csv</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -44854,7 +44854,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>fred/DGS2.csv</t>
+          <t>fred/DGS6MO.csv</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -44883,7 +44883,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>fred/DGS30.csv</t>
+          <t>fred/IUDSOIA.csv</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -44912,7 +44912,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>fred/DGS3MO.csv</t>
+          <t>fred/RESPPLLOPNWW.csv</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -44924,13 +44924,13 @@
         <v>2</v>
       </c>
       <c r="D196" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E196" t="n">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="F196" t="n">
-        <v>3000</v>
+        <v>1241</v>
       </c>
       <c r="G196" t="inlineStr">
         <is>
@@ -44941,7 +44941,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>fred/DGS5.csv</t>
+          <t>fred/TREAST.csv</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -44953,13 +44953,13 @@
         <v>2</v>
       </c>
       <c r="D197" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E197" t="n">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="F197" t="n">
-        <v>3000</v>
+        <v>1241</v>
       </c>
       <c r="G197" t="inlineStr">
         <is>
@@ -44970,7 +44970,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>fred/DGS6MO.csv</t>
+          <t>fred/WALCL.csv</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -44982,13 +44982,13 @@
         <v>2</v>
       </c>
       <c r="D198" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E198" t="n">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="F198" t="n">
-        <v>3000</v>
+        <v>1241</v>
       </c>
       <c r="G198" t="inlineStr">
         <is>
@@ -44999,7 +44999,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>fred/RESPPLLOPNWW.csv</t>
+          <t>fred/WLRRAL.csv</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -45028,7 +45028,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>fred/TREAST.csv</t>
+          <t>fred/WRESBAL.csv</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -45046,7 +45046,7 @@
         <v>63</v>
       </c>
       <c r="F200" t="n">
-        <v>1241</v>
+        <v>2230</v>
       </c>
       <c r="G200" t="inlineStr">
         <is>
@@ -45057,7 +45057,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>fred/WALCL.csv</t>
+          <t>fred/WSHOMCB.csv</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -45086,7 +45086,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>fred/WLRRAL.csv</t>
+          <t>fred/WSHOSHO.csv</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -45115,7 +45115,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>fred/WRESBAL.csv</t>
+          <t>fred/WTREGEN.csv</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -45133,7 +45133,7 @@
         <v>63</v>
       </c>
       <c r="F203" t="n">
-        <v>2230</v>
+        <v>2125</v>
       </c>
       <c r="G203" t="inlineStr">
         <is>
@@ -45144,7 +45144,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>fred/WSHOMCB.csv</t>
+          <t>marches/indices/KOSPI.csv</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
@@ -45156,13 +45156,13 @@
         <v>2</v>
       </c>
       <c r="D204" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E204" t="n">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="F204" t="n">
-        <v>1241</v>
+        <v>3682</v>
       </c>
       <c r="G204" t="inlineStr">
         <is>
@@ -45173,7 +45173,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>fred/WSHOSHO.csv</t>
+          <t>souverains/AUSTRALIE_10A.csv</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -45185,13 +45185,13 @@
         <v>2</v>
       </c>
       <c r="D205" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E205" t="n">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="F205" t="n">
-        <v>1241</v>
+        <v>3361</v>
       </c>
       <c r="G205" t="inlineStr">
         <is>
@@ -45202,7 +45202,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>fred/WTREGEN.csv</t>
+          <t>souverains/AUSTRALIE_2A.csv</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -45214,13 +45214,13 @@
         <v>2</v>
       </c>
       <c r="D206" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E206" t="n">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="F206" t="n">
-        <v>2125</v>
+        <v>3283</v>
       </c>
       <c r="G206" t="inlineStr">
         <is>
@@ -45231,7 +45231,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>marches/indices/KOSPI.csv</t>
+          <t>souverains/AUSTRALIE_5A.csv</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -45249,7 +45249,7 @@
         <v>42</v>
       </c>
       <c r="F207" t="n">
-        <v>3682</v>
+        <v>3283</v>
       </c>
       <c r="G207" t="inlineStr">
         <is>
@@ -45260,7 +45260,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>souverains/AUSTRALIE_10A.csv</t>
+          <t>souverains/CANADA_10A.csv</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -45278,7 +45278,7 @@
         <v>42</v>
       </c>
       <c r="F208" t="n">
-        <v>3361</v>
+        <v>6434</v>
       </c>
       <c r="G208" t="inlineStr">
         <is>
@@ -45289,7 +45289,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>souverains/AUSTRALIE_2A.csv</t>
+          <t>souverains/CANADA_2A.csv</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -45307,7 +45307,7 @@
         <v>42</v>
       </c>
       <c r="F209" t="n">
-        <v>3283</v>
+        <v>6433</v>
       </c>
       <c r="G209" t="inlineStr">
         <is>
@@ -45318,7 +45318,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>souverains/AUSTRALIE_5A.csv</t>
+          <t>souverains/CANADA_5A.csv</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -45336,7 +45336,7 @@
         <v>42</v>
       </c>
       <c r="F210" t="n">
-        <v>3283</v>
+        <v>6433</v>
       </c>
       <c r="G210" t="inlineStr">
         <is>
@@ -45347,7 +45347,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>souverains/CANADA_10A.csv</t>
+          <t>souverains/CANADA_LONG.csv</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
@@ -45365,7 +45365,7 @@
         <v>42</v>
       </c>
       <c r="F211" t="n">
-        <v>6434</v>
+        <v>6433</v>
       </c>
       <c r="G211" t="inlineStr">
         <is>
@@ -45376,7 +45376,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>souverains/CANADA_2A.csv</t>
+          <t>souverains/UK_10A.csv</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -45394,7 +45394,7 @@
         <v>42</v>
       </c>
       <c r="F212" t="n">
-        <v>6433</v>
+        <v>9282</v>
       </c>
       <c r="G212" t="inlineStr">
         <is>
@@ -45405,7 +45405,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>souverains/CANADA_5A.csv</t>
+          <t>souverains/UK_20A.csv</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -45423,7 +45423,7 @@
         <v>42</v>
       </c>
       <c r="F213" t="n">
-        <v>6433</v>
+        <v>6753</v>
       </c>
       <c r="G213" t="inlineStr">
         <is>
@@ -45434,7 +45434,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>souverains/CANADA_LONG.csv</t>
+          <t>souverains/UK_5A.csv</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -45452,7 +45452,7 @@
         <v>42</v>
       </c>
       <c r="F214" t="n">
-        <v>6433</v>
+        <v>8290</v>
       </c>
       <c r="G214" t="inlineStr">
         <is>
@@ -45463,7 +45463,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
+          <t>tresor_us/dette_quotidienne.csv</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -45481,7 +45481,7 @@
         <v>42</v>
       </c>
       <c r="F215" t="n">
-        <v>5637</v>
+        <v>2000</v>
       </c>
       <c r="G215" t="inlineStr">
         <is>
@@ -45492,7 +45492,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
+          <t>tresor_us/solde_tresorerie.csv</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -45510,7 +45510,7 @@
         <v>42</v>
       </c>
       <c r="F216" t="n">
-        <v>5637</v>
+        <v>500</v>
       </c>
       <c r="G216" t="inlineStr">
         <is>
@@ -45521,16 +45521,16 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
+          <t>fred/ECBDFR.csv</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C217" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D217" t="n">
         <v>1</v>
@@ -45539,7 +45539,7 @@
         <v>42</v>
       </c>
       <c r="F217" t="n">
-        <v>5637</v>
+        <v>3000</v>
       </c>
       <c r="G217" t="inlineStr">
         <is>
@@ -45550,25 +45550,25 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
+          <t>fred/MORTGAGE30US.csv</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C218" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D218" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E218" t="n">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="F218" t="n">
-        <v>5637</v>
+        <v>2896</v>
       </c>
       <c r="G218" t="inlineStr">
         <is>
@@ -45579,16 +45579,16 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
+          <t>fred/RRPONTSYD.csv</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C219" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D219" t="n">
         <v>1</v>
@@ -45597,7 +45597,7 @@
         <v>42</v>
       </c>
       <c r="F219" t="n">
-        <v>5637</v>
+        <v>3000</v>
       </c>
       <c r="G219" t="inlineStr">
         <is>
@@ -45608,16 +45608,16 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
+          <t>fred/T10YIE.csv</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C220" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D220" t="n">
         <v>1</v>
@@ -45626,7 +45626,7 @@
         <v>42</v>
       </c>
       <c r="F220" t="n">
-        <v>5637</v>
+        <v>3000</v>
       </c>
       <c r="G220" t="inlineStr">
         <is>
@@ -45637,16 +45637,16 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
+          <t>marches/volatilite/GVZ.csv</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C221" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D221" t="n">
         <v>1</v>
@@ -45655,7 +45655,7 @@
         <v>42</v>
       </c>
       <c r="F221" t="n">
-        <v>5637</v>
+        <v>3770</v>
       </c>
       <c r="G221" t="inlineStr">
         <is>
@@ -45666,16 +45666,16 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
+          <t>marches/volatilite/MOVE.csv</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C222" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D222" t="n">
         <v>1</v>
@@ -45684,7 +45684,7 @@
         <v>42</v>
       </c>
       <c r="F222" t="n">
-        <v>5637</v>
+        <v>3689</v>
       </c>
       <c r="G222" t="inlineStr">
         <is>
@@ -45695,16 +45695,16 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
+          <t>marches/volatilite/OVX.csv</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C223" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D223" t="n">
         <v>1</v>
@@ -45713,7 +45713,7 @@
         <v>42</v>
       </c>
       <c r="F223" t="n">
-        <v>5637</v>
+        <v>3770</v>
       </c>
       <c r="G223" t="inlineStr">
         <is>
@@ -45724,16 +45724,16 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>tresor_us/dette_quotidienne.csv</t>
+          <t>marches/volatilite/VVIX.csv</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C224" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D224" t="n">
         <v>1</v>
@@ -45742,7 +45742,7 @@
         <v>42</v>
       </c>
       <c r="F224" t="n">
-        <v>2000</v>
+        <v>3762</v>
       </c>
       <c r="G224" t="inlineStr">
         <is>
@@ -45753,16 +45753,16 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>tresor_us/solde_tresorerie.csv</t>
+          <t>marches/volatilite/VXN.csv</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C225" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D225" t="n">
         <v>1</v>
@@ -45771,7 +45771,7 @@
         <v>42</v>
       </c>
       <c r="F225" t="n">
-        <v>500</v>
+        <v>3770</v>
       </c>
       <c r="G225" t="inlineStr">
         <is>
@@ -45782,7 +45782,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>fred/ECBDFR.csv</t>
+          <t>souverains/SUEDE_10A.csv</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -45800,7 +45800,7 @@
         <v>42</v>
       </c>
       <c r="F226" t="n">
-        <v>3000</v>
+        <v>9201</v>
       </c>
       <c r="G226" t="inlineStr">
         <is>
@@ -45811,7 +45811,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>fred/MORTGAGE30US.csv</t>
+          <t>souverains/SUEDE_2A.csv</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -45823,13 +45823,13 @@
         <v>1</v>
       </c>
       <c r="D227" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E227" t="n">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="F227" t="n">
-        <v>2896</v>
+        <v>9201</v>
       </c>
       <c r="G227" t="inlineStr">
         <is>
@@ -45840,7 +45840,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>fred/RRPONTSYD.csv</t>
+          <t>souverains/SUEDE_5A.csv</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -45858,7 +45858,7 @@
         <v>42</v>
       </c>
       <c r="F228" t="n">
-        <v>3000</v>
+        <v>9203</v>
       </c>
       <c r="G228" t="inlineStr">
         <is>
@@ -45869,7 +45869,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>fred/T10YIE.csv</t>
+          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -45887,7 +45887,7 @@
         <v>42</v>
       </c>
       <c r="F229" t="n">
-        <v>3000</v>
+        <v>5638</v>
       </c>
       <c r="G229" t="inlineStr">
         <is>
@@ -45898,7 +45898,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>marches/volatilite/GVZ.csv</t>
+          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -45916,7 +45916,7 @@
         <v>42</v>
       </c>
       <c r="F230" t="n">
-        <v>3770</v>
+        <v>5638</v>
       </c>
       <c r="G230" t="inlineStr">
         <is>
@@ -45927,7 +45927,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>marches/volatilite/MOVE.csv</t>
+          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -45945,7 +45945,7 @@
         <v>42</v>
       </c>
       <c r="F231" t="n">
-        <v>3689</v>
+        <v>5638</v>
       </c>
       <c r="G231" t="inlineStr">
         <is>
@@ -45956,7 +45956,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>marches/volatilite/OVX.csv</t>
+          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -45974,7 +45974,7 @@
         <v>42</v>
       </c>
       <c r="F232" t="n">
-        <v>3770</v>
+        <v>5638</v>
       </c>
       <c r="G232" t="inlineStr">
         <is>
@@ -45985,7 +45985,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>marches/volatilite/VVIX.csv</t>
+          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -46003,7 +46003,7 @@
         <v>42</v>
       </c>
       <c r="F233" t="n">
-        <v>3762</v>
+        <v>5638</v>
       </c>
       <c r="G233" t="inlineStr">
         <is>
@@ -46014,7 +46014,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>marches/volatilite/VXN.csv</t>
+          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -46032,7 +46032,7 @@
         <v>42</v>
       </c>
       <c r="F234" t="n">
-        <v>3770</v>
+        <v>5638</v>
       </c>
       <c r="G234" t="inlineStr">
         <is>
@@ -46043,7 +46043,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_10A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -46061,7 +46061,7 @@
         <v>42</v>
       </c>
       <c r="F235" t="n">
-        <v>9201</v>
+        <v>5638</v>
       </c>
       <c r="G235" t="inlineStr">
         <is>
@@ -46072,7 +46072,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_2A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -46090,7 +46090,7 @@
         <v>42</v>
       </c>
       <c r="F236" t="n">
-        <v>9201</v>
+        <v>5638</v>
       </c>
       <c r="G236" t="inlineStr">
         <is>
@@ -46101,7 +46101,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_5A.csv</t>
+          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
@@ -46119,7 +46119,7 @@
         <v>42</v>
       </c>
       <c r="F237" t="n">
-        <v>9203</v>
+        <v>5638</v>
       </c>
       <c r="G237" t="inlineStr">
         <is>
@@ -48687,55 +48687,55 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>10722.49</v>
+        <v>10704.25</v>
       </c>
       <c r="D4" t="n">
-        <v>2.04</v>
+        <v>1.87</v>
       </c>
       <c r="E4" t="n">
-        <v>16.37</v>
+        <v>16.17</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Zone euro (Euro Stoxx 50)</t>
+          <t>Etats-Unis (S&amp;P 500)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>6320.54</v>
+        <v>7704.13</v>
       </c>
       <c r="D5" t="n">
-        <v>1.59</v>
+        <v>4.71</v>
       </c>
       <c r="E5" t="n">
-        <v>16.08</v>
+        <v>16.06</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Etats-Unis (S&amp;P 500)</t>
+          <t>Zone euro (Euro Stoxx 50)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>7704.13</v>
+        <v>6315.25</v>
       </c>
       <c r="D6" t="n">
-        <v>4.71</v>
+        <v>1.51</v>
       </c>
       <c r="E6" t="n">
-        <v>16.06</v>
+        <v>15.98</v>
       </c>
     </row>
     <row r="7">
@@ -48750,13 +48750,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>25423.13</v>
+        <v>25433.95</v>
       </c>
       <c r="D7" t="n">
-        <v>3.05</v>
+        <v>3.09</v>
       </c>
       <c r="E7" t="n">
-        <v>8.02</v>
+        <v>8.07</v>
       </c>
     </row>
     <row r="8">
@@ -48771,13 +48771,13 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>24483.59</v>
+        <v>24510.09</v>
       </c>
       <c r="D8" t="n">
-        <v>7.99</v>
+        <v>8.109999999999999</v>
       </c>
       <c r="E8" t="n">
-        <v>-7.56</v>
+        <v>-7.46</v>
       </c>
     </row>
   </sheetData>
@@ -49434,16 +49434,16 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>15.57</v>
+        <v>15.12</v>
       </c>
       <c r="C12" t="n">
-        <v>15.573</v>
+        <v>15.19</v>
       </c>
       <c r="D12" t="n">
         <v>0.624</v>
       </c>
       <c r="E12" t="n">
-        <v>0.20506</v>
+        <v>0.20508</v>
       </c>
     </row>
   </sheetData>
@@ -50730,25 +50730,25 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.001562</v>
+        <v>0.001559</v>
       </c>
       <c r="C9" t="n">
-        <v>4.15</v>
+        <v>3.97</v>
       </c>
       <c r="D9" t="n">
-        <v>99.25</v>
+        <v>98.76000000000001</v>
       </c>
       <c r="E9" t="n">
-        <v>37.87</v>
+        <v>37.19</v>
       </c>
       <c r="F9" t="n">
-        <v>42.97</v>
+        <v>42.26</v>
       </c>
       <c r="G9" t="n">
-        <v>1.18</v>
+        <v>0.74</v>
       </c>
       <c r="H9" t="n">
-        <v>5.7</v>
+        <v>5.92</v>
       </c>
     </row>
   </sheetData>
@@ -54302,10 +54302,10 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>15.57</v>
+        <v>15.12</v>
       </c>
       <c r="C12" t="n">
-        <v>20.202</v>
+        <v>20.2</v>
       </c>
       <c r="D12" t="n">
         <v>0.02404</v>
@@ -54314,7 +54314,7 @@
         <v>28.8</v>
       </c>
       <c r="F12" t="n">
-        <v>-4.632</v>
+        <v>-5.08</v>
       </c>
     </row>
   </sheetData>
@@ -54573,26 +54573,26 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>3.218</v>
+        <v>3.229</v>
       </c>
       <c r="D4" t="n">
-        <v>3.524</v>
+        <v>3.566</v>
       </c>
       <c r="E4" t="n">
-        <v>0.305</v>
+        <v>0.337</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.146</v>
+        <v>-0.104</v>
       </c>
       <c r="G4" t="n">
-        <v>0.732</v>
+        <v>0.754</v>
       </c>
       <c r="H4" t="n">
-        <v>0.586</v>
+        <v>0.65</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -54613,26 +54613,26 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>4.78</v>
+        <v>4.878</v>
       </c>
       <c r="D5" t="n">
-        <v>5.211</v>
+        <v>5.306</v>
       </c>
       <c r="E5" t="n">
-        <v>0.431</v>
+        <v>0.427</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.098</v>
+        <v>-0.089</v>
       </c>
       <c r="G5" t="n">
-        <v>0.499</v>
+        <v>0.651</v>
       </c>
       <c r="H5" t="n">
-        <v>0.402</v>
+        <v>0.5620000000000001</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -59350,10 +59350,10 @@
         <v>0.00882</v>
       </c>
       <c r="C12" t="n">
-        <v>0.0669</v>
+        <v>0.06707</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.03786</v>
+        <v>-0.03794</v>
       </c>
     </row>
   </sheetData>
@@ -69997,13 +69997,13 @@
         <v>89.40000000000001</v>
       </c>
       <c r="D3" t="n">
-        <v>4.02</v>
+        <v>4.06</v>
       </c>
       <c r="E3" t="n">
         <v>3.25</v>
       </c>
       <c r="F3" t="n">
-        <v>0.77</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="4">
@@ -70016,13 +70016,13 @@
         <v>12.9</v>
       </c>
       <c r="D4" t="n">
-        <v>5.21</v>
+        <v>5.31</v>
       </c>
       <c r="E4" t="n">
         <v>3.09</v>
       </c>
       <c r="F4" t="n">
-        <v>2.12</v>
+        <v>2.22</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-26T00:44Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-25 22:44 UTC</t>
+          <t>Genere le 2026-09-26 00:44 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-25 22:44 UTC</t>
+          <t>Rapport global — 2026-09-26 00:44 UTC</t>
         </is>
       </c>
     </row>
@@ -1009,7 +1009,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>**Rotation sectorielle** — classement momentum 3 mois (10 secteurs) : 1. Energie (XLE) : +15.23% | 2. Technologie (XLK) : +8.37% | 3. Sante (XLV) : +6.46% | 4. Finance (XLF) : +2.37% | 5. Consommation de base (XLP) : -3.13% _(observation : 2026-09-25)_</t>
+          <t>**Rotation sectorielle** — classement momentum 3 mois (10 secteurs) : 1. Energie (XLE) : +15.73% | 2. Sante (XLV) : +9.15% | 3. Technologie (XLK) : +5.49% | 4. Finance (XLF) : +2.02% | 5. Consommation de base (XLP) : -2.67% _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
@@ -1023,21 +1023,21 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>**Dispersion sectorielle** — 10 secteurs, rendement moyen 3m=-0.61%, dispersion (ecart-type)=8.31pt, etendue=29.71pt -- dispersion intermediaire _(observation : 2026-09-25)_</t>
+          <t>**Dispersion sectorielle** — 10 secteurs, rendement moyen 3m=-0.62%, dispersion (ecart-type)=8.40pt, etendue=29.89pt -- dispersion intermediaire _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>**Low volatility** — tercile bas-vol ['XLF', 'XLRE', 'XLU'] Sharpe=-0.566 vs tercile haut-vol ['XLY', 'XLE', 'XLK'] Sharpe=0.218 -- anomalie low-vol non confirmee sur cet echantillon (puissance statistique faible, n petit -- limite assumee) _(observation : 2026-09-25)_</t>
+          <t>**Low volatility** — tercile bas-vol ['XLF', 'XLRE', 'XLU'] Sharpe=-0.443 vs tercile haut-vol ['XLY', 'XLE', 'XLK'] Sharpe=0.258 -- anomalie low-vol non confirmee sur cet echantillon (puissance statistique faible, n petit -- limite assumee) _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>**Momentum cross sectional** — panier gagnant ['XLE', 'XLK', 'XLV'] (+10.02%) vs panier perdant ['XLI', 'XLRE', 'XLU'] (-9.52%) -- spread momentum=+19.54pt _(observation : 2026-09-25)_</t>
+          <t>**Momentum cross sectional** — panier gagnant ['XLE', 'XLV', 'XLK'] (+10.13%) vs panier perdant ['XLRE', 'XLI', 'XLU'] (-9.68%) -- spread momentum=+19.81pt _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>**Correlation facteurs** — correlation entre momentum 3m et beta-VIX, 10 secteurs : +0.062 (facteurs largement independants) _(observation : 2026-09-25)_</t>
+          <t>**Correlation facteurs** — correlation entre momentum 3m et beta-VIX, 10 secteurs : +0.174 (facteurs largement independants) _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
@@ -12755,7 +12755,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -15386,10 +15386,10 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>-2.6227</v>
+        <v>-2.6209</v>
       </c>
       <c r="D112" t="n">
-        <v>0.2286</v>
+        <v>0.2293</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -15409,10 +15409,10 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>-1.9044</v>
+        <v>-1.8796</v>
       </c>
       <c r="D113" t="n">
-        <v>0.5778</v>
+        <v>0.5903</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -15432,10 +15432,10 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>-2.0874</v>
+        <v>-2.1019</v>
       </c>
       <c r="D114" t="n">
-        <v>0.483</v>
+        <v>0.4754</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -15455,10 +15455,10 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>-2.3143</v>
+        <v>-2.3104</v>
       </c>
       <c r="D115" t="n">
-        <v>0.3664</v>
+        <v>0.3684</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -15478,10 +15478,10 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>-1.3337</v>
+        <v>-1.3042</v>
       </c>
       <c r="D116" t="n">
-        <v>0.8193</v>
+        <v>0.8285</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -15501,10 +15501,10 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>-0.0148</v>
+        <v>-0.0648</v>
       </c>
       <c r="D117" t="n">
-        <v>0.9856</v>
+        <v>0.9843</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -15524,10 +15524,10 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>-1.1895</v>
+        <v>-1.216</v>
       </c>
       <c r="D118" t="n">
-        <v>0.8606</v>
+        <v>0.8536</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -15547,10 +15547,10 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>-0.4625</v>
+        <v>-0.4936</v>
       </c>
       <c r="D119" t="n">
-        <v>0.9669</v>
+        <v>0.9648</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -15570,10 +15570,10 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>-2.1564</v>
+        <v>-2.1726</v>
       </c>
       <c r="D120" t="n">
-        <v>0.4469</v>
+        <v>0.4385</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -15593,10 +15593,10 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>-1.4682</v>
+        <v>-1.548</v>
       </c>
       <c r="D121" t="n">
-        <v>0.7732</v>
+        <v>0.7423</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -22383,7 +22383,7 @@
         <v>10</v>
       </c>
       <c r="C12" t="n">
-        <v>0.1431</v>
+        <v>0.1742</v>
       </c>
     </row>
     <row r="13">
@@ -42720,7 +42720,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D2" t="n">
         <v>91.5</v>
@@ -42749,7 +42749,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D3" t="n">
         <v>91.5</v>
@@ -42778,7 +42778,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D4" t="n">
         <v>91.5</v>
@@ -42807,7 +42807,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D5" t="n">
         <v>91.5</v>
@@ -42836,7 +42836,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D6" t="n">
         <v>91.5</v>
@@ -42865,7 +42865,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D7" t="n">
         <v>91.5</v>
@@ -42894,7 +42894,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D8" t="n">
         <v>91.5</v>
@@ -42923,7 +42923,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D9" t="n">
         <v>91.5</v>
@@ -42952,7 +42952,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D10" t="n">
         <v>91.5</v>
@@ -42981,7 +42981,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D11" t="n">
         <v>91.5</v>
@@ -43010,7 +43010,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D12" t="n">
         <v>91.5</v>
@@ -43039,7 +43039,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D13" t="n">
         <v>91.5</v>
@@ -43068,7 +43068,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D14" t="n">
         <v>91.5</v>
@@ -43097,7 +43097,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D15" t="n">
         <v>91.5</v>
@@ -43126,7 +43126,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D16" t="n">
         <v>92</v>
@@ -43155,7 +43155,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D17" t="n">
         <v>91.5</v>
@@ -43184,7 +43184,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D18" t="n">
         <v>91.5</v>
@@ -43213,7 +43213,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D19" t="n">
         <v>91.5</v>
@@ -43242,7 +43242,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D20" t="n">
         <v>91.5</v>
@@ -43271,7 +43271,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D21" t="n">
         <v>91.5</v>
@@ -43300,7 +43300,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D22" t="n">
         <v>91.5</v>
@@ -43329,7 +43329,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D23" t="n">
         <v>91.5</v>
@@ -43358,7 +43358,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D24" t="n">
         <v>91.5</v>
@@ -43387,7 +43387,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D25" t="n">
         <v>91</v>
@@ -43416,7 +43416,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D26" t="n">
         <v>31</v>
@@ -43445,7 +43445,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D27" t="n">
         <v>31</v>
@@ -43474,7 +43474,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D28" t="n">
         <v>31</v>
@@ -43503,7 +43503,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D29" t="n">
         <v>31</v>
@@ -43532,7 +43532,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D30" t="n">
         <v>31</v>
@@ -43561,7 +43561,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D31" t="n">
         <v>31</v>
@@ -43590,7 +43590,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D32" t="n">
         <v>31</v>
@@ -43619,7 +43619,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D33" t="n">
         <v>31</v>
@@ -43648,7 +43648,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D34" t="n">
         <v>31</v>
@@ -43677,7 +43677,7 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D35" t="n">
         <v>31</v>
@@ -43706,7 +43706,7 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D36" t="n">
         <v>31</v>
@@ -43735,7 +43735,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D37" t="n">
         <v>31</v>
@@ -43764,7 +43764,7 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D38" t="n">
         <v>31</v>
@@ -43793,7 +43793,7 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D39" t="n">
         <v>31</v>
@@ -43822,7 +43822,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D40" t="n">
         <v>31</v>
@@ -43851,7 +43851,7 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D41" t="n">
         <v>31</v>
@@ -43880,7 +43880,7 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D42" t="n">
         <v>31</v>
@@ -43909,7 +43909,7 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D43" t="n">
         <v>31</v>
@@ -43938,7 +43938,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D44" t="n">
         <v>31</v>
@@ -43967,7 +43967,7 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D45" t="n">
         <v>31</v>
@@ -43996,7 +43996,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D46" t="n">
         <v>31</v>
@@ -44025,7 +44025,7 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D47" t="n">
         <v>31</v>
@@ -44054,7 +44054,7 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D48" t="n">
         <v>31</v>
@@ -44083,7 +44083,7 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D49" t="n">
         <v>31</v>
@@ -44112,7 +44112,7 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D50" t="n">
         <v>31</v>
@@ -44141,7 +44141,7 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D51" t="n">
         <v>31</v>
@@ -44170,7 +44170,7 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D52" t="n">
         <v>31</v>
@@ -44199,7 +44199,7 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D53" t="n">
         <v>31</v>
@@ -44228,7 +44228,7 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D54" t="n">
         <v>31</v>
@@ -44257,7 +44257,7 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D55" t="n">
         <v>31</v>
@@ -44286,7 +44286,7 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D56" t="n">
         <v>31</v>
@@ -44315,7 +44315,7 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D57" t="n">
         <v>31</v>
@@ -44344,7 +44344,7 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D58" t="n">
         <v>31</v>
@@ -44373,7 +44373,7 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D59" t="n">
         <v>31</v>
@@ -44402,7 +44402,7 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D60" t="n">
         <v>31</v>
@@ -44431,7 +44431,7 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D61" t="n">
         <v>31</v>
@@ -44460,7 +44460,7 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D62" t="n">
         <v>31</v>
@@ -44489,7 +44489,7 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D63" t="n">
         <v>31</v>
@@ -44518,7 +44518,7 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D64" t="n">
         <v>31</v>
@@ -44547,7 +44547,7 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D65" t="n">
         <v>31</v>
@@ -44576,7 +44576,7 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D66" t="n">
         <v>31</v>
@@ -44605,7 +44605,7 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D67" t="n">
         <v>31</v>
@@ -44634,7 +44634,7 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D68" t="n">
         <v>31</v>
@@ -44663,7 +44663,7 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D69" t="n">
         <v>31</v>
@@ -44692,7 +44692,7 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D70" t="n">
         <v>31</v>
@@ -44721,7 +44721,7 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D71" t="n">
         <v>31</v>
@@ -44750,7 +44750,7 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D72" t="n">
         <v>31</v>
@@ -44779,7 +44779,7 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D73" t="n">
         <v>31</v>
@@ -44808,7 +44808,7 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D74" t="n">
         <v>31</v>
@@ -44837,7 +44837,7 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D75" t="n">
         <v>31</v>
@@ -44866,7 +44866,7 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D76" t="n">
         <v>31</v>
@@ -44895,7 +44895,7 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D77" t="n">
         <v>31</v>
@@ -44924,7 +44924,7 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D78" t="n">
         <v>31</v>
@@ -44953,7 +44953,7 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D79" t="n">
         <v>31</v>
@@ -44982,7 +44982,7 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D80" t="n">
         <v>31</v>
@@ -45011,7 +45011,7 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D81" t="n">
         <v>31</v>
@@ -45040,7 +45040,7 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D82" t="n">
         <v>31</v>
@@ -45069,7 +45069,7 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D83" t="n">
         <v>31</v>
@@ -45098,7 +45098,7 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D84" t="n">
         <v>31</v>
@@ -45127,7 +45127,7 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D85" t="n">
         <v>31</v>
@@ -45156,7 +45156,7 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D86" t="n">
         <v>31</v>
@@ -45185,7 +45185,7 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D87" t="n">
         <v>31</v>
@@ -45214,7 +45214,7 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D88" t="n">
         <v>31</v>
@@ -45243,7 +45243,7 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D89" t="n">
         <v>31</v>
@@ -45272,7 +45272,7 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D90" t="n">
         <v>31</v>
@@ -45301,7 +45301,7 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D91" t="n">
         <v>31</v>
@@ -45330,7 +45330,7 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D92" t="n">
         <v>31</v>
@@ -45359,7 +45359,7 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D93" t="n">
         <v>31</v>
@@ -45388,7 +45388,7 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D94" t="n">
         <v>31</v>
@@ -45417,7 +45417,7 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D95" t="n">
         <v>1</v>
@@ -45446,7 +45446,7 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D96" t="n">
         <v>1</v>
@@ -45475,7 +45475,7 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D97" t="n">
         <v>1</v>
@@ -45504,7 +45504,7 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D98" t="n">
         <v>1</v>
@@ -45533,7 +45533,7 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D99" t="n">
         <v>1</v>
@@ -45562,7 +45562,7 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D100" t="n">
         <v>31</v>
@@ -45591,7 +45591,7 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D101" t="n">
         <v>31</v>
@@ -45620,7 +45620,7 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D102" t="n">
         <v>7</v>
@@ -45649,7 +45649,7 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D103" t="n">
         <v>7</v>
@@ -45678,7 +45678,7 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D104" t="n">
         <v>1</v>
@@ -45707,7 +45707,7 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D105" t="n">
         <v>7</v>
@@ -45736,7 +45736,7 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D106" t="n">
         <v>1</v>
@@ -45765,7 +45765,7 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D107" t="n">
         <v>1</v>
@@ -45794,7 +45794,7 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D108" t="n">
         <v>7</v>
@@ -45823,7 +45823,7 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D109" t="n">
         <v>1</v>
@@ -45852,7 +45852,7 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D110" t="n">
         <v>1</v>
@@ -45881,7 +45881,7 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D111" t="n">
         <v>1</v>
@@ -45910,7 +45910,7 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D112" t="n">
         <v>1</v>
@@ -45939,7 +45939,7 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D113" t="n">
         <v>1</v>
@@ -45968,7 +45968,7 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D114" t="n">
         <v>1</v>
@@ -45997,7 +45997,7 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D115" t="n">
         <v>1</v>
@@ -46026,7 +46026,7 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D116" t="n">
         <v>1</v>
@@ -46055,7 +46055,7 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D117" t="n">
         <v>7</v>
@@ -46084,7 +46084,7 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D118" t="n">
         <v>7</v>
@@ -46113,7 +46113,7 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D119" t="n">
         <v>7</v>
@@ -46142,7 +46142,7 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D120" t="n">
         <v>7</v>
@@ -46171,7 +46171,7 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D121" t="n">
         <v>7</v>
@@ -46200,7 +46200,7 @@
         </is>
       </c>
       <c r="C122" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D122" t="n">
         <v>7</v>
@@ -46229,7 +46229,7 @@
         </is>
       </c>
       <c r="C123" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D123" t="n">
         <v>7</v>
@@ -46258,7 +46258,7 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D124" t="n">
         <v>7</v>
@@ -46287,7 +46287,7 @@
         </is>
       </c>
       <c r="C125" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D125" t="n">
         <v>7</v>
@@ -46316,7 +46316,7 @@
         </is>
       </c>
       <c r="C126" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D126" t="n">
         <v>7</v>
@@ -46345,7 +46345,7 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D127" t="n">
         <v>7</v>
@@ -46374,7 +46374,7 @@
         </is>
       </c>
       <c r="C128" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D128" t="n">
         <v>7</v>
@@ -46403,7 +46403,7 @@
         </is>
       </c>
       <c r="C129" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D129" t="n">
         <v>7</v>
@@ -46432,7 +46432,7 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D130" t="n">
         <v>7</v>
@@ -46461,7 +46461,7 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D131" t="n">
         <v>7</v>
@@ -46490,7 +46490,7 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D132" t="n">
         <v>7</v>
@@ -46519,7 +46519,7 @@
         </is>
       </c>
       <c r="C133" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D133" t="n">
         <v>7</v>
@@ -46548,7 +46548,7 @@
         </is>
       </c>
       <c r="C134" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D134" t="n">
         <v>7</v>
@@ -46577,7 +46577,7 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D135" t="n">
         <v>7</v>
@@ -46606,7 +46606,7 @@
         </is>
       </c>
       <c r="C136" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D136" t="n">
         <v>7</v>
@@ -46635,7 +46635,7 @@
         </is>
       </c>
       <c r="C137" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D137" t="n">
         <v>7</v>
@@ -46664,7 +46664,7 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D138" t="n">
         <v>7</v>
@@ -46693,7 +46693,7 @@
         </is>
       </c>
       <c r="C139" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D139" t="n">
         <v>7</v>
@@ -46722,7 +46722,7 @@
         </is>
       </c>
       <c r="C140" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D140" t="n">
         <v>7</v>
@@ -46751,7 +46751,7 @@
         </is>
       </c>
       <c r="C141" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D141" t="n">
         <v>7</v>
@@ -46780,7 +46780,7 @@
         </is>
       </c>
       <c r="C142" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D142" t="n">
         <v>7</v>
@@ -46809,7 +46809,7 @@
         </is>
       </c>
       <c r="C143" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D143" t="n">
         <v>7</v>
@@ -46838,7 +46838,7 @@
         </is>
       </c>
       <c r="C144" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D144" t="n">
         <v>7</v>
@@ -46867,7 +46867,7 @@
         </is>
       </c>
       <c r="C145" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D145" t="n">
         <v>7</v>
@@ -46896,7 +46896,7 @@
         </is>
       </c>
       <c r="C146" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D146" t="n">
         <v>7</v>
@@ -46925,7 +46925,7 @@
         </is>
       </c>
       <c r="C147" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D147" t="n">
         <v>7</v>
@@ -46954,7 +46954,7 @@
         </is>
       </c>
       <c r="C148" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D148" t="n">
         <v>7</v>
@@ -46983,7 +46983,7 @@
         </is>
       </c>
       <c r="C149" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D149" t="n">
         <v>7</v>
@@ -47012,7 +47012,7 @@
         </is>
       </c>
       <c r="C150" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D150" t="n">
         <v>7</v>
@@ -47041,7 +47041,7 @@
         </is>
       </c>
       <c r="C151" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D151" t="n">
         <v>7</v>
@@ -47070,7 +47070,7 @@
         </is>
       </c>
       <c r="C152" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D152" t="n">
         <v>7</v>
@@ -47099,7 +47099,7 @@
         </is>
       </c>
       <c r="C153" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D153" t="n">
         <v>7</v>
@@ -47128,7 +47128,7 @@
         </is>
       </c>
       <c r="C154" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D154" t="n">
         <v>7</v>
@@ -47157,7 +47157,7 @@
         </is>
       </c>
       <c r="C155" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D155" t="n">
         <v>7</v>
@@ -47186,7 +47186,7 @@
         </is>
       </c>
       <c r="C156" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D156" t="n">
         <v>7</v>
@@ -47215,7 +47215,7 @@
         </is>
       </c>
       <c r="C157" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D157" t="n">
         <v>7</v>
@@ -47244,7 +47244,7 @@
         </is>
       </c>
       <c r="C158" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D158" t="n">
         <v>7</v>
@@ -47273,7 +47273,7 @@
         </is>
       </c>
       <c r="C159" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D159" t="n">
         <v>7</v>
@@ -47302,7 +47302,7 @@
         </is>
       </c>
       <c r="C160" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D160" t="n">
         <v>7</v>
@@ -47331,7 +47331,7 @@
         </is>
       </c>
       <c r="C161" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D161" t="n">
         <v>7</v>
@@ -47360,7 +47360,7 @@
         </is>
       </c>
       <c r="C162" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D162" t="n">
         <v>7</v>
@@ -47389,7 +47389,7 @@
         </is>
       </c>
       <c r="C163" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D163" t="n">
         <v>7</v>
@@ -47418,7 +47418,7 @@
         </is>
       </c>
       <c r="C164" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D164" t="n">
         <v>7</v>
@@ -47447,7 +47447,7 @@
         </is>
       </c>
       <c r="C165" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D165" t="n">
         <v>7</v>
@@ -47476,7 +47476,7 @@
         </is>
       </c>
       <c r="C166" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D166" t="n">
         <v>7</v>
@@ -47505,7 +47505,7 @@
         </is>
       </c>
       <c r="C167" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D167" t="n">
         <v>7</v>
@@ -47534,7 +47534,7 @@
         </is>
       </c>
       <c r="C168" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D168" t="n">
         <v>7</v>
@@ -47563,7 +47563,7 @@
         </is>
       </c>
       <c r="C169" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D169" t="n">
         <v>7</v>
@@ -47592,7 +47592,7 @@
         </is>
       </c>
       <c r="C170" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D170" t="n">
         <v>7</v>
@@ -47621,7 +47621,7 @@
         </is>
       </c>
       <c r="C171" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D171" t="n">
         <v>7</v>
@@ -47650,7 +47650,7 @@
         </is>
       </c>
       <c r="C172" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D172" t="n">
         <v>7</v>
@@ -47679,7 +47679,7 @@
         </is>
       </c>
       <c r="C173" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D173" t="n">
         <v>7</v>
@@ -47708,7 +47708,7 @@
         </is>
       </c>
       <c r="C174" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D174" t="n">
         <v>7</v>
@@ -47737,7 +47737,7 @@
         </is>
       </c>
       <c r="C175" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D175" t="n">
         <v>1</v>
@@ -47766,7 +47766,7 @@
         </is>
       </c>
       <c r="C176" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D176" t="n">
         <v>7</v>
@@ -47795,7 +47795,7 @@
         </is>
       </c>
       <c r="C177" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D177" t="n">
         <v>7</v>
@@ -47824,7 +47824,7 @@
         </is>
       </c>
       <c r="C178" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D178" t="n">
         <v>7</v>
@@ -47853,7 +47853,7 @@
         </is>
       </c>
       <c r="C179" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D179" t="n">
         <v>7</v>
@@ -47882,7 +47882,7 @@
         </is>
       </c>
       <c r="C180" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D180" t="n">
         <v>7</v>
@@ -47911,7 +47911,7 @@
         </is>
       </c>
       <c r="C181" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D181" t="n">
         <v>7</v>
@@ -47940,7 +47940,7 @@
         </is>
       </c>
       <c r="C182" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D182" t="n">
         <v>7</v>
@@ -47969,7 +47969,7 @@
         </is>
       </c>
       <c r="C183" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D183" t="n">
         <v>7</v>
@@ -47998,7 +47998,7 @@
         </is>
       </c>
       <c r="C184" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D184" t="n">
         <v>1</v>
@@ -48027,7 +48027,7 @@
         </is>
       </c>
       <c r="C185" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D185" t="n">
         <v>1</v>
@@ -48056,7 +48056,7 @@
         </is>
       </c>
       <c r="C186" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D186" t="n">
         <v>1</v>
@@ -48085,7 +48085,7 @@
         </is>
       </c>
       <c r="C187" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D187" t="n">
         <v>1</v>
@@ -48114,7 +48114,7 @@
         </is>
       </c>
       <c r="C188" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D188" t="n">
         <v>1</v>
@@ -48143,7 +48143,7 @@
         </is>
       </c>
       <c r="C189" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D189" t="n">
         <v>1</v>
@@ -48172,7 +48172,7 @@
         </is>
       </c>
       <c r="C190" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D190" t="n">
         <v>1</v>
@@ -48201,7 +48201,7 @@
         </is>
       </c>
       <c r="C191" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D191" t="n">
         <v>1</v>
@@ -48230,7 +48230,7 @@
         </is>
       </c>
       <c r="C192" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D192" t="n">
         <v>1</v>
@@ -48259,7 +48259,7 @@
         </is>
       </c>
       <c r="C193" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D193" t="n">
         <v>1</v>
@@ -48288,7 +48288,7 @@
         </is>
       </c>
       <c r="C194" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D194" t="n">
         <v>1</v>
@@ -48317,7 +48317,7 @@
         </is>
       </c>
       <c r="C195" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D195" t="n">
         <v>1</v>
@@ -48346,7 +48346,7 @@
         </is>
       </c>
       <c r="C196" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D196" t="n">
         <v>1</v>
@@ -48375,7 +48375,7 @@
         </is>
       </c>
       <c r="C197" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D197" t="n">
         <v>1</v>
@@ -48404,7 +48404,7 @@
         </is>
       </c>
       <c r="C198" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D198" t="n">
         <v>1</v>
@@ -48433,7 +48433,7 @@
         </is>
       </c>
       <c r="C199" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D199" t="n">
         <v>1</v>
@@ -48462,7 +48462,7 @@
         </is>
       </c>
       <c r="C200" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D200" t="n">
         <v>1</v>
@@ -48491,7 +48491,7 @@
         </is>
       </c>
       <c r="C201" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D201" t="n">
         <v>1</v>
@@ -48520,7 +48520,7 @@
         </is>
       </c>
       <c r="C202" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D202" t="n">
         <v>1</v>
@@ -48549,7 +48549,7 @@
         </is>
       </c>
       <c r="C203" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D203" t="n">
         <v>1</v>
@@ -48578,7 +48578,7 @@
         </is>
       </c>
       <c r="C204" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D204" t="n">
         <v>1</v>
@@ -48607,7 +48607,7 @@
         </is>
       </c>
       <c r="C205" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D205" t="n">
         <v>1</v>
@@ -48636,7 +48636,7 @@
         </is>
       </c>
       <c r="C206" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D206" t="n">
         <v>1</v>
@@ -48665,7 +48665,7 @@
         </is>
       </c>
       <c r="C207" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D207" t="n">
         <v>1</v>
@@ -48694,7 +48694,7 @@
         </is>
       </c>
       <c r="C208" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D208" t="n">
         <v>1</v>
@@ -48723,7 +48723,7 @@
         </is>
       </c>
       <c r="C209" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D209" t="n">
         <v>1</v>
@@ -48752,7 +48752,7 @@
         </is>
       </c>
       <c r="C210" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D210" t="n">
         <v>1</v>
@@ -48781,7 +48781,7 @@
         </is>
       </c>
       <c r="C211" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D211" t="n">
         <v>7</v>
@@ -48810,7 +48810,7 @@
         </is>
       </c>
       <c r="C212" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D212" t="n">
         <v>1</v>
@@ -48839,7 +48839,7 @@
         </is>
       </c>
       <c r="C213" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D213" t="n">
         <v>1</v>
@@ -48859,7 +48859,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>marches/indices/HANGSENG.csv</t>
+          <t>marches/indices/FTSE100.csv</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -48868,7 +48868,7 @@
         </is>
       </c>
       <c r="C214" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D214" t="n">
         <v>1</v>
@@ -48877,7 +48877,7 @@
         <v>42</v>
       </c>
       <c r="F214" t="n">
-        <v>3689</v>
+        <v>3788</v>
       </c>
       <c r="G214" t="inlineStr">
         <is>
@@ -48888,7 +48888,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>marches/indices/NIKKEI225.csv</t>
+          <t>marches/indices/HANGSENG.csv</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -48897,7 +48897,7 @@
         </is>
       </c>
       <c r="C215" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D215" t="n">
         <v>1</v>
@@ -48906,7 +48906,7 @@
         <v>42</v>
       </c>
       <c r="F215" t="n">
-        <v>3667</v>
+        <v>3689</v>
       </c>
       <c r="G215" t="inlineStr">
         <is>
@@ -48917,7 +48917,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>souverains/CANADA_10A.csv</t>
+          <t>marches/indices/NIKKEI225.csv</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -48926,7 +48926,7 @@
         </is>
       </c>
       <c r="C216" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D216" t="n">
         <v>1</v>
@@ -48935,7 +48935,7 @@
         <v>42</v>
       </c>
       <c r="F216" t="n">
-        <v>6435</v>
+        <v>3667</v>
       </c>
       <c r="G216" t="inlineStr">
         <is>
@@ -48946,7 +48946,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>souverains/CANADA_2A.csv</t>
+          <t>souverains/CANADA_10A.csv</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -48955,7 +48955,7 @@
         </is>
       </c>
       <c r="C217" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D217" t="n">
         <v>1</v>
@@ -48964,7 +48964,7 @@
         <v>42</v>
       </c>
       <c r="F217" t="n">
-        <v>6434</v>
+        <v>6435</v>
       </c>
       <c r="G217" t="inlineStr">
         <is>
@@ -48975,7 +48975,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>souverains/CANADA_5A.csv</t>
+          <t>souverains/CANADA_2A.csv</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -48984,7 +48984,7 @@
         </is>
       </c>
       <c r="C218" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D218" t="n">
         <v>1</v>
@@ -49004,7 +49004,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>souverains/CANADA_LONG.csv</t>
+          <t>souverains/CANADA_5A.csv</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -49013,7 +49013,7 @@
         </is>
       </c>
       <c r="C219" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D219" t="n">
         <v>1</v>
@@ -49033,7 +49033,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_10A.csv</t>
+          <t>souverains/CANADA_LONG.csv</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -49042,7 +49042,7 @@
         </is>
       </c>
       <c r="C220" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D220" t="n">
         <v>1</v>
@@ -49051,7 +49051,7 @@
         <v>42</v>
       </c>
       <c r="F220" t="n">
-        <v>9201</v>
+        <v>6434</v>
       </c>
       <c r="G220" t="inlineStr">
         <is>
@@ -49062,7 +49062,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_2A.csv</t>
+          <t>souverains/SUEDE_10A.csv</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -49071,7 +49071,7 @@
         </is>
       </c>
       <c r="C221" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D221" t="n">
         <v>1</v>
@@ -49091,7 +49091,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_5A.csv</t>
+          <t>souverains/SUEDE_2A.csv</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -49100,7 +49100,7 @@
         </is>
       </c>
       <c r="C222" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D222" t="n">
         <v>1</v>
@@ -49109,7 +49109,7 @@
         <v>42</v>
       </c>
       <c r="F222" t="n">
-        <v>9203</v>
+        <v>9201</v>
       </c>
       <c r="G222" t="inlineStr">
         <is>
@@ -49120,7 +49120,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
+          <t>souverains/SUEDE_5A.csv</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -49129,7 +49129,7 @@
         </is>
       </c>
       <c r="C223" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D223" t="n">
         <v>1</v>
@@ -49138,7 +49138,7 @@
         <v>42</v>
       </c>
       <c r="F223" t="n">
-        <v>5638</v>
+        <v>9203</v>
       </c>
       <c r="G223" t="inlineStr">
         <is>
@@ -49149,7 +49149,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -49158,7 +49158,7 @@
         </is>
       </c>
       <c r="C224" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D224" t="n">
         <v>1</v>
@@ -49178,7 +49178,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
@@ -49187,7 +49187,7 @@
         </is>
       </c>
       <c r="C225" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D225" t="n">
         <v>1</v>
@@ -49207,7 +49207,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -49216,7 +49216,7 @@
         </is>
       </c>
       <c r="C226" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D226" t="n">
         <v>1</v>
@@ -49236,7 +49236,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -49245,7 +49245,7 @@
         </is>
       </c>
       <c r="C227" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D227" t="n">
         <v>1</v>
@@ -49265,7 +49265,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -49274,7 +49274,7 @@
         </is>
       </c>
       <c r="C228" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D228" t="n">
         <v>1</v>
@@ -49294,7 +49294,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -49303,7 +49303,7 @@
         </is>
       </c>
       <c r="C229" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D229" t="n">
         <v>1</v>
@@ -49323,7 +49323,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -49332,7 +49332,7 @@
         </is>
       </c>
       <c r="C230" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D230" t="n">
         <v>1</v>
@@ -49352,7 +49352,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -49361,7 +49361,7 @@
         </is>
       </c>
       <c r="C231" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D231" t="n">
         <v>1</v>
@@ -49381,7 +49381,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>tresor_us/dette_quotidienne.csv</t>
+          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -49390,7 +49390,7 @@
         </is>
       </c>
       <c r="C232" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D232" t="n">
         <v>1</v>
@@ -49399,7 +49399,7 @@
         <v>42</v>
       </c>
       <c r="F232" t="n">
-        <v>2000</v>
+        <v>5638</v>
       </c>
       <c r="G232" t="inlineStr">
         <is>
@@ -49410,7 +49410,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>tresor_us/solde_tresorerie.csv</t>
+          <t>tresor_us/dette_quotidienne.csv</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -49419,7 +49419,7 @@
         </is>
       </c>
       <c r="C233" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D233" t="n">
         <v>1</v>
@@ -49428,7 +49428,7 @@
         <v>42</v>
       </c>
       <c r="F233" t="n">
-        <v>500</v>
+        <v>2000</v>
       </c>
       <c r="G233" t="inlineStr">
         <is>
@@ -49439,16 +49439,16 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>fred/ECBDFR.csv</t>
+          <t>tresor_us/solde_tresorerie.csv</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C234" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D234" t="n">
         <v>1</v>
@@ -49457,7 +49457,7 @@
         <v>42</v>
       </c>
       <c r="F234" t="n">
-        <v>3000</v>
+        <v>500</v>
       </c>
       <c r="G234" t="inlineStr">
         <is>
@@ -49468,16 +49468,16 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>fred/RRPONTSYD.csv</t>
+          <t>yfinance/XLB.csv</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C235" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D235" t="n">
         <v>1</v>
@@ -49486,7 +49486,7 @@
         <v>42</v>
       </c>
       <c r="F235" t="n">
-        <v>3000</v>
+        <v>500</v>
       </c>
       <c r="G235" t="inlineStr">
         <is>
@@ -49497,16 +49497,16 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>fred/T10YIE.csv</t>
+          <t>yfinance/XLE.csv</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C236" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D236" t="n">
         <v>1</v>
@@ -49515,7 +49515,7 @@
         <v>42</v>
       </c>
       <c r="F236" t="n">
-        <v>3000</v>
+        <v>500</v>
       </c>
       <c r="G236" t="inlineStr">
         <is>
@@ -49526,16 +49526,16 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>marches/fx/AUDJPY.csv</t>
+          <t>yfinance/XLF.csv</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C237" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D237" t="n">
         <v>1</v>
@@ -49544,7 +49544,7 @@
         <v>42</v>
       </c>
       <c r="F237" t="n">
-        <v>3910</v>
+        <v>500</v>
       </c>
       <c r="G237" t="inlineStr">
         <is>
@@ -49555,16 +49555,16 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>marches/fx/AUDUSD.csv</t>
+          <t>yfinance/XLI.csv</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C238" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D238" t="n">
         <v>1</v>
@@ -49573,7 +49573,7 @@
         <v>42</v>
       </c>
       <c r="F238" t="n">
-        <v>3906</v>
+        <v>500</v>
       </c>
       <c r="G238" t="inlineStr">
         <is>
@@ -49584,16 +49584,16 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>marches/fx/DXY.csv</t>
+          <t>yfinance/XLK.csv</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C239" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D239" t="n">
         <v>1</v>
@@ -49602,7 +49602,7 @@
         <v>42</v>
       </c>
       <c r="F239" t="n">
-        <v>3773</v>
+        <v>500</v>
       </c>
       <c r="G239" t="inlineStr">
         <is>
@@ -49613,16 +49613,16 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>marches/fx/EURCHF.csv</t>
+          <t>yfinance/XLP.csv</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C240" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D240" t="n">
         <v>1</v>
@@ -49631,7 +49631,7 @@
         <v>42</v>
       </c>
       <c r="F240" t="n">
-        <v>3907</v>
+        <v>500</v>
       </c>
       <c r="G240" t="inlineStr">
         <is>
@@ -49642,16 +49642,16 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>marches/fx/EURGBP.csv</t>
+          <t>yfinance/XLRE.csv</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C241" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D241" t="n">
         <v>1</v>
@@ -49660,7 +49660,7 @@
         <v>42</v>
       </c>
       <c r="F241" t="n">
-        <v>3909</v>
+        <v>500</v>
       </c>
       <c r="G241" t="inlineStr">
         <is>
@@ -49671,16 +49671,16 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>marches/fx/EURJPY.csv</t>
+          <t>yfinance/XLU.csv</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C242" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D242" t="n">
         <v>1</v>
@@ -49689,7 +49689,7 @@
         <v>42</v>
       </c>
       <c r="F242" t="n">
-        <v>3909</v>
+        <v>500</v>
       </c>
       <c r="G242" t="inlineStr">
         <is>
@@ -49700,16 +49700,16 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>marches/fx/EURUSD.csv</t>
+          <t>yfinance/XLV.csv</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C243" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D243" t="n">
         <v>1</v>
@@ -49718,7 +49718,7 @@
         <v>42</v>
       </c>
       <c r="F243" t="n">
-        <v>3906</v>
+        <v>500</v>
       </c>
       <c r="G243" t="inlineStr">
         <is>
@@ -49729,16 +49729,16 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>marches/fx/GBPUSD.csv</t>
+          <t>yfinance/XLY.csv</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C244" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D244" t="n">
         <v>1</v>
@@ -49747,7 +49747,7 @@
         <v>42</v>
       </c>
       <c r="F244" t="n">
-        <v>3907</v>
+        <v>500</v>
       </c>
       <c r="G244" t="inlineStr">
         <is>
@@ -49758,7 +49758,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>marches/fx/NZDUSD.csv</t>
+          <t>fred/ECBDFR.csv</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -49767,7 +49767,7 @@
         </is>
       </c>
       <c r="C245" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D245" t="n">
         <v>1</v>
@@ -49776,7 +49776,7 @@
         <v>42</v>
       </c>
       <c r="F245" t="n">
-        <v>3907</v>
+        <v>3000</v>
       </c>
       <c r="G245" t="inlineStr">
         <is>
@@ -49787,7 +49787,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>marches/fx/USDCAD.csv</t>
+          <t>fred/RRPONTSYD.csv</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -49796,7 +49796,7 @@
         </is>
       </c>
       <c r="C246" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D246" t="n">
         <v>1</v>
@@ -49805,7 +49805,7 @@
         <v>42</v>
       </c>
       <c r="F246" t="n">
-        <v>3906</v>
+        <v>3000</v>
       </c>
       <c r="G246" t="inlineStr">
         <is>
@@ -49816,7 +49816,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>marches/fx/USDCHF.csv</t>
+          <t>fred/T10YIE.csv</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
@@ -49825,7 +49825,7 @@
         </is>
       </c>
       <c r="C247" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D247" t="n">
         <v>1</v>
@@ -49834,7 +49834,7 @@
         <v>42</v>
       </c>
       <c r="F247" t="n">
-        <v>3904</v>
+        <v>3000</v>
       </c>
       <c r="G247" t="inlineStr">
         <is>
@@ -49845,7 +49845,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>marches/fx/USDCNY.csv</t>
+          <t>marches/fx/AUDJPY.csv</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
@@ -49854,7 +49854,7 @@
         </is>
       </c>
       <c r="C248" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D248" t="n">
         <v>1</v>
@@ -49863,7 +49863,7 @@
         <v>42</v>
       </c>
       <c r="F248" t="n">
-        <v>3906</v>
+        <v>3910</v>
       </c>
       <c r="G248" t="inlineStr">
         <is>
@@ -49874,7 +49874,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>marches/fx/USDJPY.csv</t>
+          <t>marches/fx/AUDUSD.csv</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
@@ -49883,7 +49883,7 @@
         </is>
       </c>
       <c r="C249" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D249" t="n">
         <v>1</v>
@@ -49892,7 +49892,7 @@
         <v>42</v>
       </c>
       <c r="F249" t="n">
-        <v>3907</v>
+        <v>3906</v>
       </c>
       <c r="G249" t="inlineStr">
         <is>
@@ -49903,7 +49903,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>marches/fx/USDKRW.csv</t>
+          <t>marches/fx/DXY.csv</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
@@ -49912,7 +49912,7 @@
         </is>
       </c>
       <c r="C250" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D250" t="n">
         <v>1</v>
@@ -49921,7 +49921,7 @@
         <v>42</v>
       </c>
       <c r="F250" t="n">
-        <v>3906</v>
+        <v>3773</v>
       </c>
       <c r="G250" t="inlineStr">
         <is>
@@ -49932,7 +49932,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>marches/fx/USDNOK.csv</t>
+          <t>marches/fx/EURCHF.csv</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
@@ -49941,7 +49941,7 @@
         </is>
       </c>
       <c r="C251" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D251" t="n">
         <v>1</v>
@@ -49961,7 +49961,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>marches/fx/USDSEK.csv</t>
+          <t>marches/fx/EURGBP.csv</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -49970,7 +49970,7 @@
         </is>
       </c>
       <c r="C252" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D252" t="n">
         <v>1</v>
@@ -49979,7 +49979,7 @@
         <v>42</v>
       </c>
       <c r="F252" t="n">
-        <v>3907</v>
+        <v>3909</v>
       </c>
       <c r="G252" t="inlineStr">
         <is>
@@ -49990,7 +49990,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>marches/indices/FTSE100.csv</t>
+          <t>marches/fx/EURJPY.csv</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -49999,7 +49999,7 @@
         </is>
       </c>
       <c r="C253" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D253" t="n">
         <v>1</v>
@@ -50008,7 +50008,7 @@
         <v>42</v>
       </c>
       <c r="F253" t="n">
-        <v>3789</v>
+        <v>3909</v>
       </c>
       <c r="G253" t="inlineStr">
         <is>
@@ -50019,7 +50019,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>marches/matieres/BRENT.csv</t>
+          <t>marches/fx/EURUSD.csv</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
@@ -50028,7 +50028,7 @@
         </is>
       </c>
       <c r="C254" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D254" t="n">
         <v>1</v>
@@ -50037,7 +50037,7 @@
         <v>42</v>
       </c>
       <c r="F254" t="n">
-        <v>3751</v>
+        <v>3906</v>
       </c>
       <c r="G254" t="inlineStr">
         <is>
@@ -50048,7 +50048,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>marches/matieres/CUIVRE.csv</t>
+          <t>marches/fx/GBPUSD.csv</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
@@ -50057,7 +50057,7 @@
         </is>
       </c>
       <c r="C255" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D255" t="n">
         <v>1</v>
@@ -50066,7 +50066,7 @@
         <v>42</v>
       </c>
       <c r="F255" t="n">
-        <v>3772</v>
+        <v>3907</v>
       </c>
       <c r="G255" t="inlineStr">
         <is>
@@ -50077,7 +50077,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>marches/matieres/GAZ_HENRY_HUB.csv</t>
+          <t>marches/fx/NZDUSD.csv</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
@@ -50086,7 +50086,7 @@
         </is>
       </c>
       <c r="C256" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D256" t="n">
         <v>1</v>
@@ -50095,7 +50095,7 @@
         <v>42</v>
       </c>
       <c r="F256" t="n">
-        <v>3773</v>
+        <v>3907</v>
       </c>
       <c r="G256" t="inlineStr">
         <is>
@@ -50106,7 +50106,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>marches/matieres/OR.csv</t>
+          <t>marches/fx/USDCAD.csv</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
@@ -50115,7 +50115,7 @@
         </is>
       </c>
       <c r="C257" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D257" t="n">
         <v>1</v>
@@ -50124,7 +50124,7 @@
         <v>42</v>
       </c>
       <c r="F257" t="n">
-        <v>3772</v>
+        <v>3906</v>
       </c>
       <c r="G257" t="inlineStr">
         <is>
@@ -50135,7 +50135,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>marches/matieres/WTI.csv</t>
+          <t>marches/fx/USDCHF.csv</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
@@ -50144,7 +50144,7 @@
         </is>
       </c>
       <c r="C258" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D258" t="n">
         <v>1</v>
@@ -50153,7 +50153,7 @@
         <v>42</v>
       </c>
       <c r="F258" t="n">
-        <v>3772</v>
+        <v>3904</v>
       </c>
       <c r="G258" t="inlineStr">
         <is>
@@ -50164,7 +50164,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>marches/taux_futures/FED_FUNDS_FRONT.csv</t>
+          <t>marches/fx/USDCNY.csv</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
@@ -50173,7 +50173,7 @@
         </is>
       </c>
       <c r="C259" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D259" t="n">
         <v>1</v>
@@ -50182,7 +50182,7 @@
         <v>42</v>
       </c>
       <c r="F259" t="n">
-        <v>3773</v>
+        <v>3906</v>
       </c>
       <c r="G259" t="inlineStr">
         <is>
@@ -50193,7 +50193,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>marches/volatilite/GVZ.csv</t>
+          <t>marches/fx/USDJPY.csv</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
@@ -50202,7 +50202,7 @@
         </is>
       </c>
       <c r="C260" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D260" t="n">
         <v>1</v>
@@ -50211,7 +50211,7 @@
         <v>42</v>
       </c>
       <c r="F260" t="n">
-        <v>3772</v>
+        <v>3907</v>
       </c>
       <c r="G260" t="inlineStr">
         <is>
@@ -50222,7 +50222,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>marches/volatilite/MOVE.csv</t>
+          <t>marches/fx/USDKRW.csv</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
@@ -50231,7 +50231,7 @@
         </is>
       </c>
       <c r="C261" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D261" t="n">
         <v>1</v>
@@ -50240,7 +50240,7 @@
         <v>42</v>
       </c>
       <c r="F261" t="n">
-        <v>3691</v>
+        <v>3906</v>
       </c>
       <c r="G261" t="inlineStr">
         <is>
@@ -50251,7 +50251,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>marches/volatilite/OVX.csv</t>
+          <t>marches/fx/USDNOK.csv</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
@@ -50260,7 +50260,7 @@
         </is>
       </c>
       <c r="C262" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D262" t="n">
         <v>1</v>
@@ -50269,7 +50269,7 @@
         <v>42</v>
       </c>
       <c r="F262" t="n">
-        <v>3772</v>
+        <v>3907</v>
       </c>
       <c r="G262" t="inlineStr">
         <is>
@@ -50280,7 +50280,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>marches/volatilite/VVIX.csv</t>
+          <t>marches/fx/USDSEK.csv</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
@@ -50289,7 +50289,7 @@
         </is>
       </c>
       <c r="C263" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D263" t="n">
         <v>1</v>
@@ -50298,7 +50298,7 @@
         <v>42</v>
       </c>
       <c r="F263" t="n">
-        <v>3764</v>
+        <v>3907</v>
       </c>
       <c r="G263" t="inlineStr">
         <is>
@@ -50309,7 +50309,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>marches/volatilite/VXN.csv</t>
+          <t>marches/matieres/BRENT.csv</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
@@ -50318,7 +50318,7 @@
         </is>
       </c>
       <c r="C264" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D264" t="n">
         <v>1</v>
@@ -50327,7 +50327,7 @@
         <v>42</v>
       </c>
       <c r="F264" t="n">
-        <v>3772</v>
+        <v>3751</v>
       </c>
       <c r="G264" t="inlineStr">
         <is>
@@ -50338,7 +50338,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>yfinance/SP500.csv</t>
+          <t>marches/matieres/CUIVRE.csv</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
@@ -50347,7 +50347,7 @@
         </is>
       </c>
       <c r="C265" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D265" t="n">
         <v>1</v>
@@ -50356,7 +50356,7 @@
         <v>42</v>
       </c>
       <c r="F265" t="n">
-        <v>7547</v>
+        <v>3772</v>
       </c>
       <c r="G265" t="inlineStr">
         <is>
@@ -50367,7 +50367,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>yfinance/VIX.csv</t>
+          <t>marches/matieres/GAZ_HENRY_HUB.csv</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
@@ -50376,7 +50376,7 @@
         </is>
       </c>
       <c r="C266" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D266" t="n">
         <v>1</v>
@@ -50385,7 +50385,7 @@
         <v>42</v>
       </c>
       <c r="F266" t="n">
-        <v>7550</v>
+        <v>3773</v>
       </c>
       <c r="G266" t="inlineStr">
         <is>
@@ -50396,7 +50396,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>yfinance/XLB.csv</t>
+          <t>marches/matieres/OR.csv</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
@@ -50405,7 +50405,7 @@
         </is>
       </c>
       <c r="C267" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D267" t="n">
         <v>1</v>
@@ -50414,7 +50414,7 @@
         <v>42</v>
       </c>
       <c r="F267" t="n">
-        <v>501</v>
+        <v>3772</v>
       </c>
       <c r="G267" t="inlineStr">
         <is>
@@ -50425,7 +50425,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>yfinance/XLE.csv</t>
+          <t>marches/matieres/WTI.csv</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
@@ -50434,7 +50434,7 @@
         </is>
       </c>
       <c r="C268" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D268" t="n">
         <v>1</v>
@@ -50443,7 +50443,7 @@
         <v>42</v>
       </c>
       <c r="F268" t="n">
-        <v>501</v>
+        <v>3772</v>
       </c>
       <c r="G268" t="inlineStr">
         <is>
@@ -50454,7 +50454,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>yfinance/XLF.csv</t>
+          <t>marches/taux_futures/FED_FUNDS_FRONT.csv</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
@@ -50463,7 +50463,7 @@
         </is>
       </c>
       <c r="C269" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D269" t="n">
         <v>1</v>
@@ -50472,7 +50472,7 @@
         <v>42</v>
       </c>
       <c r="F269" t="n">
-        <v>501</v>
+        <v>3773</v>
       </c>
       <c r="G269" t="inlineStr">
         <is>
@@ -50483,7 +50483,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>yfinance/XLI.csv</t>
+          <t>marches/volatilite/GVZ.csv</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
@@ -50492,7 +50492,7 @@
         </is>
       </c>
       <c r="C270" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D270" t="n">
         <v>1</v>
@@ -50501,7 +50501,7 @@
         <v>42</v>
       </c>
       <c r="F270" t="n">
-        <v>501</v>
+        <v>3772</v>
       </c>
       <c r="G270" t="inlineStr">
         <is>
@@ -50512,7 +50512,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>yfinance/XLK.csv</t>
+          <t>marches/volatilite/MOVE.csv</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
@@ -50521,7 +50521,7 @@
         </is>
       </c>
       <c r="C271" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D271" t="n">
         <v>1</v>
@@ -50530,7 +50530,7 @@
         <v>42</v>
       </c>
       <c r="F271" t="n">
-        <v>501</v>
+        <v>3691</v>
       </c>
       <c r="G271" t="inlineStr">
         <is>
@@ -50541,7 +50541,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>yfinance/XLP.csv</t>
+          <t>marches/volatilite/OVX.csv</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
@@ -50550,7 +50550,7 @@
         </is>
       </c>
       <c r="C272" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D272" t="n">
         <v>1</v>
@@ -50559,7 +50559,7 @@
         <v>42</v>
       </c>
       <c r="F272" t="n">
-        <v>501</v>
+        <v>3772</v>
       </c>
       <c r="G272" t="inlineStr">
         <is>
@@ -50570,7 +50570,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>yfinance/XLRE.csv</t>
+          <t>marches/volatilite/VVIX.csv</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
@@ -50579,7 +50579,7 @@
         </is>
       </c>
       <c r="C273" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D273" t="n">
         <v>1</v>
@@ -50588,7 +50588,7 @@
         <v>42</v>
       </c>
       <c r="F273" t="n">
-        <v>501</v>
+        <v>3764</v>
       </c>
       <c r="G273" t="inlineStr">
         <is>
@@ -50599,7 +50599,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>yfinance/XLU.csv</t>
+          <t>marches/volatilite/VXN.csv</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
@@ -50608,7 +50608,7 @@
         </is>
       </c>
       <c r="C274" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D274" t="n">
         <v>1</v>
@@ -50617,7 +50617,7 @@
         <v>42</v>
       </c>
       <c r="F274" t="n">
-        <v>501</v>
+        <v>3772</v>
       </c>
       <c r="G274" t="inlineStr">
         <is>
@@ -50628,7 +50628,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>yfinance/XLV.csv</t>
+          <t>yfinance/SP500.csv</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
@@ -50637,7 +50637,7 @@
         </is>
       </c>
       <c r="C275" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D275" t="n">
         <v>1</v>
@@ -50646,7 +50646,7 @@
         <v>42</v>
       </c>
       <c r="F275" t="n">
-        <v>501</v>
+        <v>7547</v>
       </c>
       <c r="G275" t="inlineStr">
         <is>
@@ -50657,7 +50657,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>yfinance/XLY.csv</t>
+          <t>yfinance/VIX.csv</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
@@ -50666,7 +50666,7 @@
         </is>
       </c>
       <c r="C276" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D276" t="n">
         <v>1</v>
@@ -50675,7 +50675,7 @@
         <v>42</v>
       </c>
       <c r="F276" t="n">
-        <v>501</v>
+        <v>7550</v>
       </c>
       <c r="G276" t="inlineStr">
         <is>
@@ -50695,7 +50695,7 @@
         </is>
       </c>
       <c r="C277" t="n">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="D277" t="n">
         <v>2</v>
@@ -50724,7 +50724,7 @@
         </is>
       </c>
       <c r="C278" t="n">
-        <v>-438</v>
+        <v>-437</v>
       </c>
       <c r="D278" t="n">
         <v>42</v>
@@ -52198,17 +52198,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>10695.25</v>
+        <v>10680</v>
       </c>
       <c r="D5" t="n">
-        <v>1.78</v>
+        <v>1.43</v>
       </c>
       <c r="E5" t="n">
-        <v>16.08</v>
+        <v>15.45</v>
       </c>
     </row>
     <row r="6">
@@ -53963,7 +53963,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>-0.649</v>
+        <v>-0.443</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -53971,7 +53971,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0.123</v>
+        <v>0.258</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-26T05:35Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-26 00:44 UTC</t>
+          <t>Genere le 2026-09-26 05:35 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-26 00:44 UTC</t>
+          <t>Rapport global — 2026-09-26 05:35 UTC</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>**Matieres premieres macro** — ratio cuivre/or stable -- pas de signal net sur la croissance (+4.7% sur 3 mois). Brent 97.5$ (+35.4% sur 3 mois, +40.4% sur 12 mois), gaz +0.6% sur 3 mois, ecart Brent-WTI +5.0$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-25)_</t>
+          <t>**Matieres premieres macro** — ratio cuivre/or stable -- pas de signal net sur la croissance (+3.3% sur 3 mois). Brent 104.3$ (+44.9% sur 3 mois, +50.3% sur 12 mois), gaz -1.1% sur 3 mois, ecart Brent-WTI +11.9$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
@@ -960,7 +960,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>**Indices mondiaux** — 7 indices (devise locale) : Coree (KOSPI) +103.1% en tete sur 12 mois, Hong Kong (Hang Seng) -6.6% en queue -- ecart tres large entre blocs sur 12 mois (110pt) -- les cycles economiques ou les flux divergent nettement. ROTATION en cours : Coree (KOSPI) mene sur 12 mois mais Hong Kong (Hang Seng) a repris la tete sur 3 mois _(observation : 2026-09-25)_</t>
+          <t>**Indices mondiaux** — 7 indices (devise locale) : Coree (KOSPI) +103.1% en tete sur 12 mois, Hong Kong (Hang Seng) -7.5% en queue -- ecart tres large entre blocs sur 12 mois (111pt) -- les cycles economiques ou les flux divergent nettement. ROTATION en cours : Coree (KOSPI) mene sur 12 mois mais Hong Kong (Hang Seng) a repris la tete sur 3 mois _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
@@ -1009,7 +1009,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>**Rotation sectorielle** — classement momentum 3 mois (10 secteurs) : 1. Energie (XLE) : +15.73% | 2. Sante (XLV) : +9.15% | 3. Technologie (XLK) : +5.49% | 4. Finance (XLF) : +2.02% | 5. Consommation de base (XLP) : -2.67% _(observation : 2026-09-25)_</t>
+          <t>**Rotation sectorielle** — classement momentum 3 mois (10 secteurs) : 1. Energie (XLE) : +15.23% | 2. Technologie (XLK) : +8.37% | 3. Sante (XLV) : +6.46% | 4. Finance (XLF) : +2.37% | 5. Consommation de base (XLP) : -3.13% _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
@@ -1023,21 +1023,21 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>**Dispersion sectorielle** — 10 secteurs, rendement moyen 3m=-0.62%, dispersion (ecart-type)=8.40pt, etendue=29.89pt -- dispersion intermediaire _(observation : 2026-09-25)_</t>
+          <t>**Dispersion sectorielle** — 10 secteurs, rendement moyen 3m=-0.61%, dispersion (ecart-type)=8.31pt, etendue=29.71pt -- dispersion intermediaire _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>**Low volatility** — tercile bas-vol ['XLF', 'XLRE', 'XLU'] Sharpe=-0.443 vs tercile haut-vol ['XLY', 'XLE', 'XLK'] Sharpe=0.258 -- anomalie low-vol non confirmee sur cet echantillon (puissance statistique faible, n petit -- limite assumee) _(observation : 2026-09-25)_</t>
+          <t>**Low volatility** — tercile bas-vol ['XLF', 'XLRE', 'XLU'] Sharpe=-0.566 vs tercile haut-vol ['XLY', 'XLE', 'XLK'] Sharpe=0.218 -- anomalie low-vol non confirmee sur cet echantillon (puissance statistique faible, n petit -- limite assumee) _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>**Momentum cross sectional** — panier gagnant ['XLE', 'XLV', 'XLK'] (+10.13%) vs panier perdant ['XLRE', 'XLI', 'XLU'] (-9.68%) -- spread momentum=+19.81pt _(observation : 2026-09-25)_</t>
+          <t>**Momentum cross sectional** — panier gagnant ['XLE', 'XLK', 'XLV'] (+10.02%) vs panier perdant ['XLI', 'XLRE', 'XLU'] (-9.52%) -- spread momentum=+19.54pt _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>**Correlation facteurs** — correlation entre momentum 3m et beta-VIX, 10 secteurs : +0.174 (facteurs largement independants) _(observation : 2026-09-25)_</t>
+          <t>**Correlation facteurs** — correlation entre momentum 3m et beta-VIX, 10 secteurs : +0.062 (facteurs largement independants) _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
@@ -15386,10 +15386,10 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>-2.6209</v>
+        <v>-2.6227</v>
       </c>
       <c r="D112" t="n">
-        <v>0.2293</v>
+        <v>0.2286</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -15409,10 +15409,10 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>-1.8796</v>
+        <v>-1.9044</v>
       </c>
       <c r="D113" t="n">
-        <v>0.5903</v>
+        <v>0.5778</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -15432,10 +15432,10 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>-2.1019</v>
+        <v>-2.0874</v>
       </c>
       <c r="D114" t="n">
-        <v>0.4754</v>
+        <v>0.483</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -15455,10 +15455,10 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>-2.3104</v>
+        <v>-2.3143</v>
       </c>
       <c r="D115" t="n">
-        <v>0.3684</v>
+        <v>0.3664</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -15478,10 +15478,10 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>-1.3042</v>
+        <v>-1.3337</v>
       </c>
       <c r="D116" t="n">
-        <v>0.8285</v>
+        <v>0.8193</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -15501,10 +15501,10 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>-0.0648</v>
+        <v>-0.0148</v>
       </c>
       <c r="D117" t="n">
-        <v>0.9843</v>
+        <v>0.9856</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -15524,10 +15524,10 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>-1.216</v>
+        <v>-1.1895</v>
       </c>
       <c r="D118" t="n">
-        <v>0.8536</v>
+        <v>0.8606</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -15547,10 +15547,10 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>-0.4936</v>
+        <v>-0.4625</v>
       </c>
       <c r="D119" t="n">
-        <v>0.9648</v>
+        <v>0.9669</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -15570,10 +15570,10 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>-2.1726</v>
+        <v>-2.1564</v>
       </c>
       <c r="D120" t="n">
-        <v>0.4385</v>
+        <v>0.4469</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -15593,10 +15593,10 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>-1.548</v>
+        <v>-1.4682</v>
       </c>
       <c r="D121" t="n">
-        <v>0.7423</v>
+        <v>0.7732</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -48801,7 +48801,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>marches/indices/DAX.csv</t>
+          <t>souverains/CANADA_10A.csv</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -48819,7 +48819,7 @@
         <v>42</v>
       </c>
       <c r="F212" t="n">
-        <v>3802</v>
+        <v>6435</v>
       </c>
       <c r="G212" t="inlineStr">
         <is>
@@ -48830,7 +48830,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>marches/indices/EUROSTOXX50.csv</t>
+          <t>souverains/CANADA_2A.csv</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -48848,7 +48848,7 @@
         <v>42</v>
       </c>
       <c r="F213" t="n">
-        <v>3759</v>
+        <v>6434</v>
       </c>
       <c r="G213" t="inlineStr">
         <is>
@@ -48859,7 +48859,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>marches/indices/FTSE100.csv</t>
+          <t>souverains/CANADA_5A.csv</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -48877,7 +48877,7 @@
         <v>42</v>
       </c>
       <c r="F214" t="n">
-        <v>3788</v>
+        <v>6434</v>
       </c>
       <c r="G214" t="inlineStr">
         <is>
@@ -48888,7 +48888,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>marches/indices/HANGSENG.csv</t>
+          <t>souverains/CANADA_LONG.csv</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -48906,7 +48906,7 @@
         <v>42</v>
       </c>
       <c r="F215" t="n">
-        <v>3689</v>
+        <v>6434</v>
       </c>
       <c r="G215" t="inlineStr">
         <is>
@@ -48917,7 +48917,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>marches/indices/NIKKEI225.csv</t>
+          <t>souverains/SUEDE_10A.csv</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -48935,7 +48935,7 @@
         <v>42</v>
       </c>
       <c r="F216" t="n">
-        <v>3667</v>
+        <v>9201</v>
       </c>
       <c r="G216" t="inlineStr">
         <is>
@@ -48946,7 +48946,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>souverains/CANADA_10A.csv</t>
+          <t>souverains/SUEDE_2A.csv</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -48964,7 +48964,7 @@
         <v>42</v>
       </c>
       <c r="F217" t="n">
-        <v>6435</v>
+        <v>9201</v>
       </c>
       <c r="G217" t="inlineStr">
         <is>
@@ -48975,7 +48975,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>souverains/CANADA_2A.csv</t>
+          <t>souverains/SUEDE_5A.csv</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -48993,7 +48993,7 @@
         <v>42</v>
       </c>
       <c r="F218" t="n">
-        <v>6434</v>
+        <v>9203</v>
       </c>
       <c r="G218" t="inlineStr">
         <is>
@@ -49004,7 +49004,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>souverains/CANADA_5A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -49022,7 +49022,7 @@
         <v>42</v>
       </c>
       <c r="F219" t="n">
-        <v>6434</v>
+        <v>5638</v>
       </c>
       <c r="G219" t="inlineStr">
         <is>
@@ -49033,7 +49033,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>souverains/CANADA_LONG.csv</t>
+          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -49051,7 +49051,7 @@
         <v>42</v>
       </c>
       <c r="F220" t="n">
-        <v>6434</v>
+        <v>5638</v>
       </c>
       <c r="G220" t="inlineStr">
         <is>
@@ -49062,7 +49062,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_10A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -49080,7 +49080,7 @@
         <v>42</v>
       </c>
       <c r="F221" t="n">
-        <v>9201</v>
+        <v>5638</v>
       </c>
       <c r="G221" t="inlineStr">
         <is>
@@ -49091,7 +49091,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_2A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -49109,7 +49109,7 @@
         <v>42</v>
       </c>
       <c r="F222" t="n">
-        <v>9201</v>
+        <v>5638</v>
       </c>
       <c r="G222" t="inlineStr">
         <is>
@@ -49120,7 +49120,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_5A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -49138,7 +49138,7 @@
         <v>42</v>
       </c>
       <c r="F223" t="n">
-        <v>9203</v>
+        <v>5638</v>
       </c>
       <c r="G223" t="inlineStr">
         <is>
@@ -49149,7 +49149,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -49178,7 +49178,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
@@ -49207,7 +49207,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -49236,7 +49236,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
+          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -49265,7 +49265,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
+          <t>tresor_us/dette_quotidienne.csv</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -49283,7 +49283,7 @@
         <v>42</v>
       </c>
       <c r="F228" t="n">
-        <v>5638</v>
+        <v>2000</v>
       </c>
       <c r="G228" t="inlineStr">
         <is>
@@ -49294,7 +49294,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
+          <t>tresor_us/solde_tresorerie.csv</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -49312,7 +49312,7 @@
         <v>42</v>
       </c>
       <c r="F229" t="n">
-        <v>5638</v>
+        <v>500</v>
       </c>
       <c r="G229" t="inlineStr">
         <is>
@@ -49323,16 +49323,16 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
+          <t>fred/ECBDFR.csv</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C230" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D230" t="n">
         <v>1</v>
@@ -49341,7 +49341,7 @@
         <v>42</v>
       </c>
       <c r="F230" t="n">
-        <v>5638</v>
+        <v>3000</v>
       </c>
       <c r="G230" t="inlineStr">
         <is>
@@ -49352,16 +49352,16 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
+          <t>fred/RRPONTSYD.csv</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C231" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D231" t="n">
         <v>1</v>
@@ -49370,7 +49370,7 @@
         <v>42</v>
       </c>
       <c r="F231" t="n">
-        <v>5638</v>
+        <v>3000</v>
       </c>
       <c r="G231" t="inlineStr">
         <is>
@@ -49381,16 +49381,16 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
+          <t>fred/T10YIE.csv</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C232" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D232" t="n">
         <v>1</v>
@@ -49399,7 +49399,7 @@
         <v>42</v>
       </c>
       <c r="F232" t="n">
-        <v>5638</v>
+        <v>3000</v>
       </c>
       <c r="G232" t="inlineStr">
         <is>
@@ -49410,16 +49410,16 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>tresor_us/dette_quotidienne.csv</t>
+          <t>marches/fx/DXY.csv</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C233" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D233" t="n">
         <v>1</v>
@@ -49428,7 +49428,7 @@
         <v>42</v>
       </c>
       <c r="F233" t="n">
-        <v>2000</v>
+        <v>3773</v>
       </c>
       <c r="G233" t="inlineStr">
         <is>
@@ -49439,16 +49439,16 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>tresor_us/solde_tresorerie.csv</t>
+          <t>marches/fx/EURCHF.csv</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C234" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D234" t="n">
         <v>1</v>
@@ -49457,7 +49457,7 @@
         <v>42</v>
       </c>
       <c r="F234" t="n">
-        <v>500</v>
+        <v>3907</v>
       </c>
       <c r="G234" t="inlineStr">
         <is>
@@ -49468,16 +49468,16 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>yfinance/XLB.csv</t>
+          <t>marches/fx/EURGBP.csv</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C235" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D235" t="n">
         <v>1</v>
@@ -49486,7 +49486,7 @@
         <v>42</v>
       </c>
       <c r="F235" t="n">
-        <v>500</v>
+        <v>3909</v>
       </c>
       <c r="G235" t="inlineStr">
         <is>
@@ -49497,16 +49497,16 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>yfinance/XLE.csv</t>
+          <t>marches/fx/EURJPY.csv</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C236" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D236" t="n">
         <v>1</v>
@@ -49515,7 +49515,7 @@
         <v>42</v>
       </c>
       <c r="F236" t="n">
-        <v>500</v>
+        <v>3909</v>
       </c>
       <c r="G236" t="inlineStr">
         <is>
@@ -49526,16 +49526,16 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>yfinance/XLF.csv</t>
+          <t>marches/fx/EURUSD.csv</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C237" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D237" t="n">
         <v>1</v>
@@ -49544,7 +49544,7 @@
         <v>42</v>
       </c>
       <c r="F237" t="n">
-        <v>500</v>
+        <v>3906</v>
       </c>
       <c r="G237" t="inlineStr">
         <is>
@@ -49555,16 +49555,16 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>yfinance/XLI.csv</t>
+          <t>marches/fx/GBPUSD.csv</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C238" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D238" t="n">
         <v>1</v>
@@ -49573,7 +49573,7 @@
         <v>42</v>
       </c>
       <c r="F238" t="n">
-        <v>500</v>
+        <v>3907</v>
       </c>
       <c r="G238" t="inlineStr">
         <is>
@@ -49584,16 +49584,16 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>yfinance/XLK.csv</t>
+          <t>marches/fx/USDCHF.csv</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C239" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D239" t="n">
         <v>1</v>
@@ -49602,7 +49602,7 @@
         <v>42</v>
       </c>
       <c r="F239" t="n">
-        <v>500</v>
+        <v>3904</v>
       </c>
       <c r="G239" t="inlineStr">
         <is>
@@ -49613,16 +49613,16 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>yfinance/XLP.csv</t>
+          <t>marches/indices/DAX.csv</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C240" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D240" t="n">
         <v>1</v>
@@ -49631,7 +49631,7 @@
         <v>42</v>
       </c>
       <c r="F240" t="n">
-        <v>500</v>
+        <v>3803</v>
       </c>
       <c r="G240" t="inlineStr">
         <is>
@@ -49642,16 +49642,16 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>yfinance/XLRE.csv</t>
+          <t>marches/indices/EUROSTOXX50.csv</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C241" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D241" t="n">
         <v>1</v>
@@ -49660,7 +49660,7 @@
         <v>42</v>
       </c>
       <c r="F241" t="n">
-        <v>500</v>
+        <v>3760</v>
       </c>
       <c r="G241" t="inlineStr">
         <is>
@@ -49671,16 +49671,16 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>yfinance/XLU.csv</t>
+          <t>marches/indices/FTSE100.csv</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C242" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D242" t="n">
         <v>1</v>
@@ -49689,7 +49689,7 @@
         <v>42</v>
       </c>
       <c r="F242" t="n">
-        <v>500</v>
+        <v>3789</v>
       </c>
       <c r="G242" t="inlineStr">
         <is>
@@ -49700,16 +49700,16 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>yfinance/XLV.csv</t>
+          <t>marches/indices/HANGSENG.csv</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C243" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D243" t="n">
         <v>1</v>
@@ -49718,7 +49718,7 @@
         <v>42</v>
       </c>
       <c r="F243" t="n">
-        <v>500</v>
+        <v>3690</v>
       </c>
       <c r="G243" t="inlineStr">
         <is>
@@ -49729,16 +49729,16 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>yfinance/XLY.csv</t>
+          <t>marches/indices/NIKKEI225.csv</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C244" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D244" t="n">
         <v>1</v>
@@ -49747,7 +49747,7 @@
         <v>42</v>
       </c>
       <c r="F244" t="n">
-        <v>500</v>
+        <v>3668</v>
       </c>
       <c r="G244" t="inlineStr">
         <is>
@@ -49758,7 +49758,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>fred/ECBDFR.csv</t>
+          <t>marches/matieres/BRENT.csv</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -49776,7 +49776,7 @@
         <v>42</v>
       </c>
       <c r="F245" t="n">
-        <v>3000</v>
+        <v>3751</v>
       </c>
       <c r="G245" t="inlineStr">
         <is>
@@ -49787,7 +49787,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>fred/RRPONTSYD.csv</t>
+          <t>marches/matieres/CUIVRE.csv</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -49805,7 +49805,7 @@
         <v>42</v>
       </c>
       <c r="F246" t="n">
-        <v>3000</v>
+        <v>3772</v>
       </c>
       <c r="G246" t="inlineStr">
         <is>
@@ -49816,7 +49816,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>fred/T10YIE.csv</t>
+          <t>marches/matieres/GAZ_HENRY_HUB.csv</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
@@ -49834,7 +49834,7 @@
         <v>42</v>
       </c>
       <c r="F247" t="n">
-        <v>3000</v>
+        <v>3773</v>
       </c>
       <c r="G247" t="inlineStr">
         <is>
@@ -49845,7 +49845,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>marches/fx/AUDJPY.csv</t>
+          <t>marches/matieres/OR.csv</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
@@ -49863,7 +49863,7 @@
         <v>42</v>
       </c>
       <c r="F248" t="n">
-        <v>3910</v>
+        <v>3772</v>
       </c>
       <c r="G248" t="inlineStr">
         <is>
@@ -49874,7 +49874,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>marches/fx/AUDUSD.csv</t>
+          <t>marches/matieres/WTI.csv</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
@@ -49892,7 +49892,7 @@
         <v>42</v>
       </c>
       <c r="F249" t="n">
-        <v>3906</v>
+        <v>3772</v>
       </c>
       <c r="G249" t="inlineStr">
         <is>
@@ -49903,7 +49903,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>marches/fx/DXY.csv</t>
+          <t>marches/taux_futures/FED_FUNDS_FRONT.csv</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
@@ -49932,7 +49932,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>marches/fx/EURCHF.csv</t>
+          <t>marches/volatilite/GVZ.csv</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
@@ -49950,7 +49950,7 @@
         <v>42</v>
       </c>
       <c r="F251" t="n">
-        <v>3907</v>
+        <v>3772</v>
       </c>
       <c r="G251" t="inlineStr">
         <is>
@@ -49961,7 +49961,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>marches/fx/EURGBP.csv</t>
+          <t>marches/volatilite/MOVE.csv</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -49979,7 +49979,7 @@
         <v>42</v>
       </c>
       <c r="F252" t="n">
-        <v>3909</v>
+        <v>3691</v>
       </c>
       <c r="G252" t="inlineStr">
         <is>
@@ -49990,7 +49990,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>marches/fx/EURJPY.csv</t>
+          <t>marches/volatilite/OVX.csv</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -50008,7 +50008,7 @@
         <v>42</v>
       </c>
       <c r="F253" t="n">
-        <v>3909</v>
+        <v>3772</v>
       </c>
       <c r="G253" t="inlineStr">
         <is>
@@ -50019,7 +50019,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>marches/fx/EURUSD.csv</t>
+          <t>marches/volatilite/VVIX.csv</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
@@ -50037,7 +50037,7 @@
         <v>42</v>
       </c>
       <c r="F254" t="n">
-        <v>3906</v>
+        <v>3764</v>
       </c>
       <c r="G254" t="inlineStr">
         <is>
@@ -50048,7 +50048,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>marches/fx/GBPUSD.csv</t>
+          <t>marches/volatilite/VXN.csv</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
@@ -50066,7 +50066,7 @@
         <v>42</v>
       </c>
       <c r="F255" t="n">
-        <v>3907</v>
+        <v>3772</v>
       </c>
       <c r="G255" t="inlineStr">
         <is>
@@ -50077,7 +50077,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>marches/fx/NZDUSD.csv</t>
+          <t>yfinance/SP500.csv</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
@@ -50095,7 +50095,7 @@
         <v>42</v>
       </c>
       <c r="F256" t="n">
-        <v>3907</v>
+        <v>7547</v>
       </c>
       <c r="G256" t="inlineStr">
         <is>
@@ -50106,7 +50106,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>marches/fx/USDCAD.csv</t>
+          <t>yfinance/VIX.csv</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
@@ -50124,7 +50124,7 @@
         <v>42</v>
       </c>
       <c r="F257" t="n">
-        <v>3906</v>
+        <v>7550</v>
       </c>
       <c r="G257" t="inlineStr">
         <is>
@@ -50135,7 +50135,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>marches/fx/USDCHF.csv</t>
+          <t>yfinance/XLB.csv</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
@@ -50153,7 +50153,7 @@
         <v>42</v>
       </c>
       <c r="F258" t="n">
-        <v>3904</v>
+        <v>501</v>
       </c>
       <c r="G258" t="inlineStr">
         <is>
@@ -50164,7 +50164,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>marches/fx/USDCNY.csv</t>
+          <t>yfinance/XLE.csv</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
@@ -50182,7 +50182,7 @@
         <v>42</v>
       </c>
       <c r="F259" t="n">
-        <v>3906</v>
+        <v>501</v>
       </c>
       <c r="G259" t="inlineStr">
         <is>
@@ -50193,7 +50193,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>marches/fx/USDJPY.csv</t>
+          <t>yfinance/XLF.csv</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
@@ -50211,7 +50211,7 @@
         <v>42</v>
       </c>
       <c r="F260" t="n">
-        <v>3907</v>
+        <v>501</v>
       </c>
       <c r="G260" t="inlineStr">
         <is>
@@ -50222,7 +50222,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>marches/fx/USDKRW.csv</t>
+          <t>yfinance/XLI.csv</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
@@ -50240,7 +50240,7 @@
         <v>42</v>
       </c>
       <c r="F261" t="n">
-        <v>3906</v>
+        <v>501</v>
       </c>
       <c r="G261" t="inlineStr">
         <is>
@@ -50251,7 +50251,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>marches/fx/USDNOK.csv</t>
+          <t>yfinance/XLK.csv</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
@@ -50269,7 +50269,7 @@
         <v>42</v>
       </c>
       <c r="F262" t="n">
-        <v>3907</v>
+        <v>501</v>
       </c>
       <c r="G262" t="inlineStr">
         <is>
@@ -50280,7 +50280,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>marches/fx/USDSEK.csv</t>
+          <t>yfinance/XLP.csv</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
@@ -50298,7 +50298,7 @@
         <v>42</v>
       </c>
       <c r="F263" t="n">
-        <v>3907</v>
+        <v>501</v>
       </c>
       <c r="G263" t="inlineStr">
         <is>
@@ -50309,7 +50309,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>marches/matieres/BRENT.csv</t>
+          <t>yfinance/XLRE.csv</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
@@ -50327,7 +50327,7 @@
         <v>42</v>
       </c>
       <c r="F264" t="n">
-        <v>3751</v>
+        <v>501</v>
       </c>
       <c r="G264" t="inlineStr">
         <is>
@@ -50338,7 +50338,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>marches/matieres/CUIVRE.csv</t>
+          <t>yfinance/XLU.csv</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
@@ -50356,7 +50356,7 @@
         <v>42</v>
       </c>
       <c r="F265" t="n">
-        <v>3772</v>
+        <v>501</v>
       </c>
       <c r="G265" t="inlineStr">
         <is>
@@ -50367,7 +50367,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>marches/matieres/GAZ_HENRY_HUB.csv</t>
+          <t>yfinance/XLV.csv</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
@@ -50385,7 +50385,7 @@
         <v>42</v>
       </c>
       <c r="F266" t="n">
-        <v>3773</v>
+        <v>501</v>
       </c>
       <c r="G266" t="inlineStr">
         <is>
@@ -50396,7 +50396,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>marches/matieres/OR.csv</t>
+          <t>yfinance/XLY.csv</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
@@ -50414,7 +50414,7 @@
         <v>42</v>
       </c>
       <c r="F267" t="n">
-        <v>3772</v>
+        <v>501</v>
       </c>
       <c r="G267" t="inlineStr">
         <is>
@@ -50425,16 +50425,16 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>marches/matieres/WTI.csv</t>
+          <t>marches/fx/AUDJPY.csv</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="C268" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D268" t="n">
         <v>1</v>
@@ -50443,7 +50443,7 @@
         <v>42</v>
       </c>
       <c r="F268" t="n">
-        <v>3772</v>
+        <v>3910</v>
       </c>
       <c r="G268" t="inlineStr">
         <is>
@@ -50454,16 +50454,16 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>marches/taux_futures/FED_FUNDS_FRONT.csv</t>
+          <t>marches/fx/AUDUSD.csv</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="C269" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D269" t="n">
         <v>1</v>
@@ -50472,7 +50472,7 @@
         <v>42</v>
       </c>
       <c r="F269" t="n">
-        <v>3773</v>
+        <v>3906</v>
       </c>
       <c r="G269" t="inlineStr">
         <is>
@@ -50483,16 +50483,16 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>marches/volatilite/GVZ.csv</t>
+          <t>marches/fx/NZDUSD.csv</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="C270" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D270" t="n">
         <v>1</v>
@@ -50501,7 +50501,7 @@
         <v>42</v>
       </c>
       <c r="F270" t="n">
-        <v>3772</v>
+        <v>3907</v>
       </c>
       <c r="G270" t="inlineStr">
         <is>
@@ -50512,16 +50512,16 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>marches/volatilite/MOVE.csv</t>
+          <t>marches/fx/USDCAD.csv</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="C271" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D271" t="n">
         <v>1</v>
@@ -50530,7 +50530,7 @@
         <v>42</v>
       </c>
       <c r="F271" t="n">
-        <v>3691</v>
+        <v>3906</v>
       </c>
       <c r="G271" t="inlineStr">
         <is>
@@ -50541,16 +50541,16 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>marches/volatilite/OVX.csv</t>
+          <t>marches/fx/USDCNY.csv</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="C272" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D272" t="n">
         <v>1</v>
@@ -50559,7 +50559,7 @@
         <v>42</v>
       </c>
       <c r="F272" t="n">
-        <v>3772</v>
+        <v>3906</v>
       </c>
       <c r="G272" t="inlineStr">
         <is>
@@ -50570,16 +50570,16 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>marches/volatilite/VVIX.csv</t>
+          <t>marches/fx/USDJPY.csv</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="C273" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D273" t="n">
         <v>1</v>
@@ -50588,7 +50588,7 @@
         <v>42</v>
       </c>
       <c r="F273" t="n">
-        <v>3764</v>
+        <v>3907</v>
       </c>
       <c r="G273" t="inlineStr">
         <is>
@@ -50599,16 +50599,16 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>marches/volatilite/VXN.csv</t>
+          <t>marches/fx/USDKRW.csv</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="C274" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D274" t="n">
         <v>1</v>
@@ -50617,7 +50617,7 @@
         <v>42</v>
       </c>
       <c r="F274" t="n">
-        <v>3772</v>
+        <v>3906</v>
       </c>
       <c r="G274" t="inlineStr">
         <is>
@@ -50628,16 +50628,16 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>yfinance/SP500.csv</t>
+          <t>marches/fx/USDNOK.csv</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="C275" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D275" t="n">
         <v>1</v>
@@ -50646,7 +50646,7 @@
         <v>42</v>
       </c>
       <c r="F275" t="n">
-        <v>7547</v>
+        <v>3907</v>
       </c>
       <c r="G275" t="inlineStr">
         <is>
@@ -50657,16 +50657,16 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>yfinance/VIX.csv</t>
+          <t>marches/fx/USDSEK.csv</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="C276" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D276" t="n">
         <v>1</v>
@@ -50675,7 +50675,7 @@
         <v>42</v>
       </c>
       <c r="F276" t="n">
-        <v>7550</v>
+        <v>3907</v>
       </c>
       <c r="G276" t="inlineStr">
         <is>
@@ -52156,17 +52156,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>65513.99</v>
+        <v>66364.2</v>
       </c>
       <c r="D3" t="n">
-        <v>-9.470000000000001</v>
+        <v>-4.32</v>
       </c>
       <c r="E3" t="n">
-        <v>43.58</v>
+        <v>45.04</v>
       </c>
     </row>
     <row r="4">
@@ -52198,17 +52198,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>10680</v>
+        <v>10695.3</v>
       </c>
       <c r="D5" t="n">
-        <v>1.43</v>
+        <v>1.78</v>
       </c>
       <c r="E5" t="n">
-        <v>15.45</v>
+        <v>16.08</v>
       </c>
     </row>
     <row r="6">
@@ -52219,17 +52219,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>6272.5</v>
+        <v>6302.82</v>
       </c>
       <c r="D6" t="n">
-        <v>0.08</v>
+        <v>1.31</v>
       </c>
       <c r="E6" t="n">
-        <v>14.79</v>
+        <v>15.76</v>
       </c>
     </row>
     <row r="7">
@@ -52240,17 +52240,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>25266.53</v>
+        <v>25408.64</v>
       </c>
       <c r="D7" t="n">
-        <v>1.09</v>
+        <v>2.99</v>
       </c>
       <c r="E7" t="n">
-        <v>6.76</v>
+        <v>7.96</v>
       </c>
     </row>
     <row r="8">
@@ -52261,17 +52261,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>24761.13</v>
+        <v>24510.09</v>
       </c>
       <c r="D8" t="n">
-        <v>7.3</v>
+        <v>8.109999999999999</v>
       </c>
       <c r="E8" t="n">
-        <v>-6.63</v>
+        <v>-7.46</v>
       </c>
     </row>
   </sheetData>
@@ -54279,25 +54279,25 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.001569</v>
+        <v>0.001549</v>
       </c>
       <c r="C9" t="n">
-        <v>4.65</v>
+        <v>3.35</v>
       </c>
       <c r="D9" t="n">
-        <v>97.47</v>
+        <v>104.32</v>
       </c>
       <c r="E9" t="n">
-        <v>35.39</v>
+        <v>44.91</v>
       </c>
       <c r="F9" t="n">
-        <v>40.41</v>
+        <v>50.27</v>
       </c>
       <c r="G9" t="n">
-        <v>0.62</v>
+        <v>-1.08</v>
       </c>
       <c r="H9" t="n">
-        <v>5.03</v>
+        <v>11.91</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-26T10:09Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-26 05:35 UTC</t>
+          <t>Genere le 2026-09-26 10:09 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-26 05:35 UTC</t>
+          <t>Rapport global — 2026-09-26 10:09 UTC</t>
         </is>
       </c>
     </row>
@@ -876,7 +876,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>**Pentes courbes** — 7 courbes : pente de +0.30pt (Australie) a +1.20pt (Japon) -- aucune courbe inversee -- pas de signal recessif par la pente _(observation : 2026-09-24)_</t>
+          <t>**Pentes courbes** — 7 courbes : pente de +0.30pt (Australie) a +1.20pt (Japon) -- aucune courbe inversee -- pas de signal recessif par la pente _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
@@ -1240,7 +1240,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.3769116249569233 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.05237241130035915 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-25)_</t>
+          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.3769116249569233 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.052372411300360217 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
@@ -48917,7 +48917,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_10A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -48935,7 +48935,7 @@
         <v>42</v>
       </c>
       <c r="F216" t="n">
-        <v>9201</v>
+        <v>5638</v>
       </c>
       <c r="G216" t="inlineStr">
         <is>
@@ -48946,7 +48946,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_2A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -48964,7 +48964,7 @@
         <v>42</v>
       </c>
       <c r="F217" t="n">
-        <v>9201</v>
+        <v>5638</v>
       </c>
       <c r="G217" t="inlineStr">
         <is>
@@ -48975,7 +48975,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_5A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -48993,7 +48993,7 @@
         <v>42</v>
       </c>
       <c r="F218" t="n">
-        <v>9203</v>
+        <v>5638</v>
       </c>
       <c r="G218" t="inlineStr">
         <is>
@@ -49004,7 +49004,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -49033,7 +49033,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -49062,7 +49062,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -49091,7 +49091,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -49120,7 +49120,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -49149,7 +49149,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
+          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -49178,7 +49178,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
+          <t>tresor_us/dette_quotidienne.csv</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
@@ -49196,7 +49196,7 @@
         <v>42</v>
       </c>
       <c r="F225" t="n">
-        <v>5638</v>
+        <v>2000</v>
       </c>
       <c r="G225" t="inlineStr">
         <is>
@@ -49207,7 +49207,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
+          <t>tresor_us/solde_tresorerie.csv</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -49225,7 +49225,7 @@
         <v>42</v>
       </c>
       <c r="F226" t="n">
-        <v>5638</v>
+        <v>500</v>
       </c>
       <c r="G226" t="inlineStr">
         <is>
@@ -49236,16 +49236,16 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
+          <t>fred/ECBDFR.csv</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C227" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D227" t="n">
         <v>1</v>
@@ -49254,7 +49254,7 @@
         <v>42</v>
       </c>
       <c r="F227" t="n">
-        <v>5638</v>
+        <v>3000</v>
       </c>
       <c r="G227" t="inlineStr">
         <is>
@@ -49265,16 +49265,16 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>tresor_us/dette_quotidienne.csv</t>
+          <t>fred/RRPONTSYD.csv</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C228" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D228" t="n">
         <v>1</v>
@@ -49283,7 +49283,7 @@
         <v>42</v>
       </c>
       <c r="F228" t="n">
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="G228" t="inlineStr">
         <is>
@@ -49294,16 +49294,16 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>tresor_us/solde_tresorerie.csv</t>
+          <t>fred/T10YIE.csv</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C229" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D229" t="n">
         <v>1</v>
@@ -49312,7 +49312,7 @@
         <v>42</v>
       </c>
       <c r="F229" t="n">
-        <v>500</v>
+        <v>3000</v>
       </c>
       <c r="G229" t="inlineStr">
         <is>
@@ -49323,7 +49323,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>fred/ECBDFR.csv</t>
+          <t>marches/fx/DXY.csv</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -49341,7 +49341,7 @@
         <v>42</v>
       </c>
       <c r="F230" t="n">
-        <v>3000</v>
+        <v>3773</v>
       </c>
       <c r="G230" t="inlineStr">
         <is>
@@ -49352,7 +49352,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>fred/RRPONTSYD.csv</t>
+          <t>marches/fx/EURCHF.csv</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -49370,7 +49370,7 @@
         <v>42</v>
       </c>
       <c r="F231" t="n">
-        <v>3000</v>
+        <v>3907</v>
       </c>
       <c r="G231" t="inlineStr">
         <is>
@@ -49381,7 +49381,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>fred/T10YIE.csv</t>
+          <t>marches/fx/EURJPY.csv</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -49399,7 +49399,7 @@
         <v>42</v>
       </c>
       <c r="F232" t="n">
-        <v>3000</v>
+        <v>3909</v>
       </c>
       <c r="G232" t="inlineStr">
         <is>
@@ -49410,7 +49410,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>marches/fx/DXY.csv</t>
+          <t>marches/fx/USDCHF.csv</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -49428,7 +49428,7 @@
         <v>42</v>
       </c>
       <c r="F233" t="n">
-        <v>3773</v>
+        <v>3904</v>
       </c>
       <c r="G233" t="inlineStr">
         <is>
@@ -49439,7 +49439,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>marches/fx/EURCHF.csv</t>
+          <t>marches/indices/DAX.csv</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -49457,7 +49457,7 @@
         <v>42</v>
       </c>
       <c r="F234" t="n">
-        <v>3907</v>
+        <v>3803</v>
       </c>
       <c r="G234" t="inlineStr">
         <is>
@@ -49468,7 +49468,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>marches/fx/EURGBP.csv</t>
+          <t>marches/indices/EUROSTOXX50.csv</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -49486,7 +49486,7 @@
         <v>42</v>
       </c>
       <c r="F235" t="n">
-        <v>3909</v>
+        <v>3760</v>
       </c>
       <c r="G235" t="inlineStr">
         <is>
@@ -49497,7 +49497,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>marches/fx/EURJPY.csv</t>
+          <t>marches/indices/FTSE100.csv</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -49515,7 +49515,7 @@
         <v>42</v>
       </c>
       <c r="F236" t="n">
-        <v>3909</v>
+        <v>3789</v>
       </c>
       <c r="G236" t="inlineStr">
         <is>
@@ -49526,7 +49526,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>marches/fx/EURUSD.csv</t>
+          <t>marches/indices/HANGSENG.csv</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
@@ -49544,7 +49544,7 @@
         <v>42</v>
       </c>
       <c r="F237" t="n">
-        <v>3906</v>
+        <v>3690</v>
       </c>
       <c r="G237" t="inlineStr">
         <is>
@@ -49555,7 +49555,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>marches/fx/GBPUSD.csv</t>
+          <t>marches/indices/NIKKEI225.csv</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
@@ -49573,7 +49573,7 @@
         <v>42</v>
       </c>
       <c r="F238" t="n">
-        <v>3907</v>
+        <v>3668</v>
       </c>
       <c r="G238" t="inlineStr">
         <is>
@@ -49584,7 +49584,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>marches/fx/USDCHF.csv</t>
+          <t>marches/matieres/BRENT.csv</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
@@ -49602,7 +49602,7 @@
         <v>42</v>
       </c>
       <c r="F239" t="n">
-        <v>3904</v>
+        <v>3751</v>
       </c>
       <c r="G239" t="inlineStr">
         <is>
@@ -49613,7 +49613,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>marches/indices/DAX.csv</t>
+          <t>marches/matieres/CUIVRE.csv</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
@@ -49631,7 +49631,7 @@
         <v>42</v>
       </c>
       <c r="F240" t="n">
-        <v>3803</v>
+        <v>3772</v>
       </c>
       <c r="G240" t="inlineStr">
         <is>
@@ -49642,7 +49642,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>marches/indices/EUROSTOXX50.csv</t>
+          <t>marches/matieres/GAZ_HENRY_HUB.csv</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
@@ -49660,7 +49660,7 @@
         <v>42</v>
       </c>
       <c r="F241" t="n">
-        <v>3760</v>
+        <v>3773</v>
       </c>
       <c r="G241" t="inlineStr">
         <is>
@@ -49671,7 +49671,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>marches/indices/FTSE100.csv</t>
+          <t>marches/matieres/OR.csv</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
@@ -49689,7 +49689,7 @@
         <v>42</v>
       </c>
       <c r="F242" t="n">
-        <v>3789</v>
+        <v>3772</v>
       </c>
       <c r="G242" t="inlineStr">
         <is>
@@ -49700,7 +49700,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>marches/indices/HANGSENG.csv</t>
+          <t>marches/matieres/WTI.csv</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
@@ -49718,7 +49718,7 @@
         <v>42</v>
       </c>
       <c r="F243" t="n">
-        <v>3690</v>
+        <v>3772</v>
       </c>
       <c r="G243" t="inlineStr">
         <is>
@@ -49729,7 +49729,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>marches/indices/NIKKEI225.csv</t>
+          <t>marches/taux_futures/FED_FUNDS_FRONT.csv</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -49747,7 +49747,7 @@
         <v>42</v>
       </c>
       <c r="F244" t="n">
-        <v>3668</v>
+        <v>3773</v>
       </c>
       <c r="G244" t="inlineStr">
         <is>
@@ -49758,7 +49758,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>marches/matieres/BRENT.csv</t>
+          <t>marches/volatilite/GVZ.csv</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -49776,7 +49776,7 @@
         <v>42</v>
       </c>
       <c r="F245" t="n">
-        <v>3751</v>
+        <v>3772</v>
       </c>
       <c r="G245" t="inlineStr">
         <is>
@@ -49787,7 +49787,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>marches/matieres/CUIVRE.csv</t>
+          <t>marches/volatilite/MOVE.csv</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -49805,7 +49805,7 @@
         <v>42</v>
       </c>
       <c r="F246" t="n">
-        <v>3772</v>
+        <v>3691</v>
       </c>
       <c r="G246" t="inlineStr">
         <is>
@@ -49816,7 +49816,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>marches/matieres/GAZ_HENRY_HUB.csv</t>
+          <t>marches/volatilite/OVX.csv</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
@@ -49834,7 +49834,7 @@
         <v>42</v>
       </c>
       <c r="F247" t="n">
-        <v>3773</v>
+        <v>3772</v>
       </c>
       <c r="G247" t="inlineStr">
         <is>
@@ -49845,7 +49845,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>marches/matieres/OR.csv</t>
+          <t>marches/volatilite/VVIX.csv</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
@@ -49863,7 +49863,7 @@
         <v>42</v>
       </c>
       <c r="F248" t="n">
-        <v>3772</v>
+        <v>3764</v>
       </c>
       <c r="G248" t="inlineStr">
         <is>
@@ -49874,7 +49874,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>marches/matieres/WTI.csv</t>
+          <t>marches/volatilite/VXN.csv</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
@@ -49903,7 +49903,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>marches/taux_futures/FED_FUNDS_FRONT.csv</t>
+          <t>souverains/SUEDE_10A.csv</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
@@ -49921,7 +49921,7 @@
         <v>42</v>
       </c>
       <c r="F250" t="n">
-        <v>3773</v>
+        <v>9202</v>
       </c>
       <c r="G250" t="inlineStr">
         <is>
@@ -49932,7 +49932,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>marches/volatilite/GVZ.csv</t>
+          <t>souverains/SUEDE_2A.csv</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
@@ -49950,7 +49950,7 @@
         <v>42</v>
       </c>
       <c r="F251" t="n">
-        <v>3772</v>
+        <v>9202</v>
       </c>
       <c r="G251" t="inlineStr">
         <is>
@@ -49961,7 +49961,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>marches/volatilite/MOVE.csv</t>
+          <t>souverains/SUEDE_5A.csv</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -49979,7 +49979,7 @@
         <v>42</v>
       </c>
       <c r="F252" t="n">
-        <v>3691</v>
+        <v>9204</v>
       </c>
       <c r="G252" t="inlineStr">
         <is>
@@ -49990,7 +49990,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>marches/volatilite/OVX.csv</t>
+          <t>yfinance/SP500.csv</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -50008,7 +50008,7 @@
         <v>42</v>
       </c>
       <c r="F253" t="n">
-        <v>3772</v>
+        <v>7547</v>
       </c>
       <c r="G253" t="inlineStr">
         <is>
@@ -50019,7 +50019,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>marches/volatilite/VVIX.csv</t>
+          <t>yfinance/VIX.csv</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
@@ -50037,7 +50037,7 @@
         <v>42</v>
       </c>
       <c r="F254" t="n">
-        <v>3764</v>
+        <v>7550</v>
       </c>
       <c r="G254" t="inlineStr">
         <is>
@@ -50048,7 +50048,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>marches/volatilite/VXN.csv</t>
+          <t>yfinance/XLB.csv</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
@@ -50066,7 +50066,7 @@
         <v>42</v>
       </c>
       <c r="F255" t="n">
-        <v>3772</v>
+        <v>501</v>
       </c>
       <c r="G255" t="inlineStr">
         <is>
@@ -50077,7 +50077,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>yfinance/SP500.csv</t>
+          <t>yfinance/XLE.csv</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
@@ -50095,7 +50095,7 @@
         <v>42</v>
       </c>
       <c r="F256" t="n">
-        <v>7547</v>
+        <v>501</v>
       </c>
       <c r="G256" t="inlineStr">
         <is>
@@ -50106,7 +50106,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>yfinance/VIX.csv</t>
+          <t>yfinance/XLF.csv</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
@@ -50124,7 +50124,7 @@
         <v>42</v>
       </c>
       <c r="F257" t="n">
-        <v>7550</v>
+        <v>501</v>
       </c>
       <c r="G257" t="inlineStr">
         <is>
@@ -50135,7 +50135,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>yfinance/XLB.csv</t>
+          <t>yfinance/XLI.csv</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
@@ -50164,7 +50164,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>yfinance/XLE.csv</t>
+          <t>yfinance/XLK.csv</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
@@ -50193,7 +50193,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>yfinance/XLF.csv</t>
+          <t>yfinance/XLP.csv</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
@@ -50222,7 +50222,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>yfinance/XLI.csv</t>
+          <t>yfinance/XLRE.csv</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
@@ -50251,7 +50251,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>yfinance/XLK.csv</t>
+          <t>yfinance/XLU.csv</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
@@ -50280,7 +50280,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>yfinance/XLP.csv</t>
+          <t>yfinance/XLV.csv</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
@@ -50309,7 +50309,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>yfinance/XLRE.csv</t>
+          <t>yfinance/XLY.csv</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
@@ -50338,16 +50338,16 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>yfinance/XLU.csv</t>
+          <t>marches/fx/AUDJPY.csv</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="C265" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D265" t="n">
         <v>1</v>
@@ -50356,7 +50356,7 @@
         <v>42</v>
       </c>
       <c r="F265" t="n">
-        <v>501</v>
+        <v>3910</v>
       </c>
       <c r="G265" t="inlineStr">
         <is>
@@ -50367,16 +50367,16 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>yfinance/XLV.csv</t>
+          <t>marches/fx/AUDUSD.csv</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="C266" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D266" t="n">
         <v>1</v>
@@ -50385,7 +50385,7 @@
         <v>42</v>
       </c>
       <c r="F266" t="n">
-        <v>501</v>
+        <v>3906</v>
       </c>
       <c r="G266" t="inlineStr">
         <is>
@@ -50396,16 +50396,16 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>yfinance/XLY.csv</t>
+          <t>marches/fx/EURGBP.csv</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="C267" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D267" t="n">
         <v>1</v>
@@ -50414,7 +50414,7 @@
         <v>42</v>
       </c>
       <c r="F267" t="n">
-        <v>501</v>
+        <v>3909</v>
       </c>
       <c r="G267" t="inlineStr">
         <is>
@@ -50425,7 +50425,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>marches/fx/AUDJPY.csv</t>
+          <t>marches/fx/EURUSD.csv</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
@@ -50443,7 +50443,7 @@
         <v>42</v>
       </c>
       <c r="F268" t="n">
-        <v>3910</v>
+        <v>3906</v>
       </c>
       <c r="G268" t="inlineStr">
         <is>
@@ -50454,7 +50454,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>marches/fx/AUDUSD.csv</t>
+          <t>marches/fx/GBPUSD.csv</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
@@ -50472,7 +50472,7 @@
         <v>42</v>
       </c>
       <c r="F269" t="n">
-        <v>3906</v>
+        <v>3907</v>
       </c>
       <c r="G269" t="inlineStr">
         <is>
@@ -59011,26 +59011,26 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C6" t="n">
         <v>2.79</v>
       </c>
       <c r="D6" t="n">
-        <v>3.252</v>
+        <v>3.279</v>
       </c>
       <c r="E6" t="n">
-        <v>0.462</v>
+        <v>0.489</v>
       </c>
       <c r="F6" t="n">
-        <v>-0.074</v>
+        <v>-0.038</v>
       </c>
       <c r="G6" t="n">
-        <v>0.681</v>
+        <v>0.659</v>
       </c>
       <c r="H6" t="n">
-        <v>0.607</v>
+        <v>0.621</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-26T10:23Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-26 10:09 UTC</t>
+          <t>Genere le 2026-09-26 10:23 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-26 10:09 UTC</t>
+          <t>Rapport global — 2026-09-26 10:23 UTC</t>
         </is>
       </c>
     </row>
@@ -1240,7 +1240,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.3769116249569233 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.052372411300360217 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-25)_</t>
+          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.3769116249569233 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.05237241130035915 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-26T14:25Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-26 10:23 UTC</t>
+          <t>Genere le 2026-09-26 14:25 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-26 10:23 UTC</t>
+          <t>Rapport global — 2026-09-26 14:25 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-26T14:50Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-26 14:25 UTC</t>
+          <t>Genere le 2026-09-26 14:50 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-26 14:25 UTC</t>
+          <t>Rapport global — 2026-09-26 14:50 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-26T17:52Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-26 14:50 UTC</t>
+          <t>Genere le 2026-09-26 17:52 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-26 14:50 UTC</t>
+          <t>Rapport global — 2026-09-26 17:52 UTC</t>
         </is>
       </c>
     </row>
@@ -1240,7 +1240,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.3769116249569233 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.05237241130035915 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-25)_</t>
+          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.3769116249569233 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.052372411300360217 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-26T18:09Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-26 17:52 UTC</t>
+          <t>Genere le 2026-09-26 18:09 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-26 17:52 UTC</t>
+          <t>Rapport global — 2026-09-26 18:09 UTC</t>
         </is>
       </c>
     </row>
@@ -1240,7 +1240,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.3769116249569233 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.052372411300360217 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-25)_</t>
+          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.3769116249569233 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.05237241130035915 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-26T20:16Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-26 18:09 UTC</t>
+          <t>Genere le 2026-09-26 20:16 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-26 18:09 UTC</t>
+          <t>Rapport global — 2026-09-26 20:16 UTC</t>
         </is>
       </c>
     </row>
@@ -1240,7 +1240,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.3769116249569233 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.05237241130035915 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-25)_</t>
+          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.3769116249569233 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.052372411300360217 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-26T21:17Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-26 20:16 UTC</t>
+          <t>Genere le 2026-09-26 21:17 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-26 20:16 UTC</t>
+          <t>Rapport global — 2026-09-26 21:17 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-26T22:50Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-26 21:17 UTC</t>
+          <t>Genere le 2026-09-26 22:50 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-26 21:17 UTC</t>
+          <t>Rapport global — 2026-09-26 22:50 UTC</t>
         </is>
       </c>
     </row>
@@ -1240,7 +1240,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.3769116249569233 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.052372411300360217 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-25)_</t>
+          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.3769116249569233 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.05237241130035915 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-26T23:45Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-26 22:50 UTC</t>
+          <t>Genere le 2026-09-26 23:45 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-26 22:50 UTC</t>
+          <t>Rapport global — 2026-09-26 23:45 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-27T00:58Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-26 23:45 UTC</t>
+          <t>Genere le 2026-09-27 00:58 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-26 23:45 UTC</t>
+          <t>Rapport global — 2026-09-27 00:58 UTC</t>
         </is>
       </c>
     </row>
@@ -12755,7 +12755,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -42720,7 +42720,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D2" t="n">
         <v>91.5</v>
@@ -42749,7 +42749,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D3" t="n">
         <v>91.5</v>
@@ -42778,7 +42778,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D4" t="n">
         <v>91.5</v>
@@ -42807,7 +42807,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D5" t="n">
         <v>91.5</v>
@@ -42836,7 +42836,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D6" t="n">
         <v>91.5</v>
@@ -42865,7 +42865,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D7" t="n">
         <v>91.5</v>
@@ -42894,7 +42894,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D8" t="n">
         <v>91.5</v>
@@ -42923,7 +42923,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D9" t="n">
         <v>91.5</v>
@@ -42952,7 +42952,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D10" t="n">
         <v>91.5</v>
@@ -42981,7 +42981,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D11" t="n">
         <v>91.5</v>
@@ -43010,7 +43010,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D12" t="n">
         <v>91.5</v>
@@ -43039,7 +43039,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D13" t="n">
         <v>91.5</v>
@@ -43068,7 +43068,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D14" t="n">
         <v>91.5</v>
@@ -43097,7 +43097,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D15" t="n">
         <v>91.5</v>
@@ -43126,7 +43126,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D16" t="n">
         <v>92</v>
@@ -43155,7 +43155,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D17" t="n">
         <v>91.5</v>
@@ -43184,7 +43184,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D18" t="n">
         <v>91.5</v>
@@ -43213,7 +43213,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D19" t="n">
         <v>91.5</v>
@@ -43242,7 +43242,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D20" t="n">
         <v>91.5</v>
@@ -43271,7 +43271,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D21" t="n">
         <v>91.5</v>
@@ -43300,7 +43300,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D22" t="n">
         <v>91.5</v>
@@ -43329,7 +43329,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D23" t="n">
         <v>91.5</v>
@@ -43358,7 +43358,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D24" t="n">
         <v>91.5</v>
@@ -43387,7 +43387,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D25" t="n">
         <v>91</v>
@@ -43416,7 +43416,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D26" t="n">
         <v>31</v>
@@ -43445,7 +43445,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D27" t="n">
         <v>31</v>
@@ -43474,7 +43474,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D28" t="n">
         <v>31</v>
@@ -43503,7 +43503,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D29" t="n">
         <v>31</v>
@@ -43532,7 +43532,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D30" t="n">
         <v>31</v>
@@ -43561,7 +43561,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D31" t="n">
         <v>31</v>
@@ -43590,7 +43590,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D32" t="n">
         <v>31</v>
@@ -43619,7 +43619,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D33" t="n">
         <v>31</v>
@@ -43648,7 +43648,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D34" t="n">
         <v>31</v>
@@ -43677,7 +43677,7 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D35" t="n">
         <v>31</v>
@@ -43706,7 +43706,7 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D36" t="n">
         <v>31</v>
@@ -43735,7 +43735,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D37" t="n">
         <v>31</v>
@@ -43764,7 +43764,7 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D38" t="n">
         <v>31</v>
@@ -43793,7 +43793,7 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D39" t="n">
         <v>31</v>
@@ -43822,7 +43822,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D40" t="n">
         <v>31</v>
@@ -43851,7 +43851,7 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D41" t="n">
         <v>31</v>
@@ -43880,7 +43880,7 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D42" t="n">
         <v>31</v>
@@ -43909,7 +43909,7 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D43" t="n">
         <v>31</v>
@@ -43938,7 +43938,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D44" t="n">
         <v>31</v>
@@ -43967,7 +43967,7 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D45" t="n">
         <v>31</v>
@@ -43996,7 +43996,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D46" t="n">
         <v>31</v>
@@ -44025,7 +44025,7 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D47" t="n">
         <v>31</v>
@@ -44054,7 +44054,7 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D48" t="n">
         <v>31</v>
@@ -44083,7 +44083,7 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D49" t="n">
         <v>31</v>
@@ -44112,7 +44112,7 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D50" t="n">
         <v>31</v>
@@ -44141,7 +44141,7 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D51" t="n">
         <v>31</v>
@@ -44170,7 +44170,7 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D52" t="n">
         <v>31</v>
@@ -44199,7 +44199,7 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D53" t="n">
         <v>31</v>
@@ -44228,7 +44228,7 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D54" t="n">
         <v>31</v>
@@ -44257,7 +44257,7 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D55" t="n">
         <v>31</v>
@@ -44286,7 +44286,7 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D56" t="n">
         <v>31</v>
@@ -44315,7 +44315,7 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D57" t="n">
         <v>31</v>
@@ -44344,7 +44344,7 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D58" t="n">
         <v>31</v>
@@ -44373,7 +44373,7 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D59" t="n">
         <v>31</v>
@@ -44402,7 +44402,7 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D60" t="n">
         <v>31</v>
@@ -44431,7 +44431,7 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D61" t="n">
         <v>31</v>
@@ -44460,7 +44460,7 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D62" t="n">
         <v>31</v>
@@ -44489,7 +44489,7 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D63" t="n">
         <v>31</v>
@@ -44518,7 +44518,7 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D64" t="n">
         <v>31</v>
@@ -44547,7 +44547,7 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D65" t="n">
         <v>31</v>
@@ -44576,7 +44576,7 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D66" t="n">
         <v>31</v>
@@ -44605,7 +44605,7 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D67" t="n">
         <v>31</v>
@@ -44634,7 +44634,7 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D68" t="n">
         <v>31</v>
@@ -44663,7 +44663,7 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D69" t="n">
         <v>31</v>
@@ -44692,7 +44692,7 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D70" t="n">
         <v>31</v>
@@ -44721,7 +44721,7 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D71" t="n">
         <v>31</v>
@@ -44750,7 +44750,7 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D72" t="n">
         <v>31</v>
@@ -44779,7 +44779,7 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D73" t="n">
         <v>31</v>
@@ -44808,7 +44808,7 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D74" t="n">
         <v>31</v>
@@ -44837,7 +44837,7 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D75" t="n">
         <v>31</v>
@@ -44866,7 +44866,7 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D76" t="n">
         <v>31</v>
@@ -44895,7 +44895,7 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D77" t="n">
         <v>31</v>
@@ -44924,7 +44924,7 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D78" t="n">
         <v>31</v>
@@ -44953,7 +44953,7 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D79" t="n">
         <v>31</v>
@@ -44982,7 +44982,7 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D80" t="n">
         <v>31</v>
@@ -45011,7 +45011,7 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D81" t="n">
         <v>31</v>
@@ -45040,7 +45040,7 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D82" t="n">
         <v>31</v>
@@ -45069,7 +45069,7 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D83" t="n">
         <v>31</v>
@@ -45098,7 +45098,7 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D84" t="n">
         <v>31</v>
@@ -45127,7 +45127,7 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D85" t="n">
         <v>31</v>
@@ -45156,7 +45156,7 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D86" t="n">
         <v>31</v>
@@ -45185,7 +45185,7 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D87" t="n">
         <v>31</v>
@@ -45214,7 +45214,7 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D88" t="n">
         <v>31</v>
@@ -45243,7 +45243,7 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D89" t="n">
         <v>31</v>
@@ -45272,7 +45272,7 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D90" t="n">
         <v>31</v>
@@ -45301,7 +45301,7 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D91" t="n">
         <v>31</v>
@@ -45330,7 +45330,7 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D92" t="n">
         <v>31</v>
@@ -45359,7 +45359,7 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D93" t="n">
         <v>31</v>
@@ -45388,7 +45388,7 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D94" t="n">
         <v>31</v>
@@ -45417,7 +45417,7 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D95" t="n">
         <v>1</v>
@@ -45446,7 +45446,7 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D96" t="n">
         <v>1</v>
@@ -45475,7 +45475,7 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D97" t="n">
         <v>1</v>
@@ -45504,7 +45504,7 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D98" t="n">
         <v>1</v>
@@ -45533,7 +45533,7 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D99" t="n">
         <v>1</v>
@@ -45562,7 +45562,7 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D100" t="n">
         <v>31</v>
@@ -45591,7 +45591,7 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D101" t="n">
         <v>31</v>
@@ -45620,7 +45620,7 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D102" t="n">
         <v>7</v>
@@ -45649,7 +45649,7 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D103" t="n">
         <v>7</v>
@@ -45678,7 +45678,7 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D104" t="n">
         <v>1</v>
@@ -45707,7 +45707,7 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D105" t="n">
         <v>7</v>
@@ -45736,7 +45736,7 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D106" t="n">
         <v>1</v>
@@ -45765,7 +45765,7 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D107" t="n">
         <v>1</v>
@@ -45794,7 +45794,7 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D108" t="n">
         <v>7</v>
@@ -45823,7 +45823,7 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D109" t="n">
         <v>1</v>
@@ -45852,7 +45852,7 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D110" t="n">
         <v>1</v>
@@ -45881,7 +45881,7 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D111" t="n">
         <v>1</v>
@@ -45910,7 +45910,7 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D112" t="n">
         <v>1</v>
@@ -45939,7 +45939,7 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D113" t="n">
         <v>1</v>
@@ -45968,7 +45968,7 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D114" t="n">
         <v>1</v>
@@ -45997,7 +45997,7 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D115" t="n">
         <v>1</v>
@@ -46026,7 +46026,7 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D116" t="n">
         <v>1</v>
@@ -46055,7 +46055,7 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D117" t="n">
         <v>7</v>
@@ -46084,7 +46084,7 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D118" t="n">
         <v>7</v>
@@ -46113,7 +46113,7 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D119" t="n">
         <v>7</v>
@@ -46142,7 +46142,7 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D120" t="n">
         <v>7</v>
@@ -46171,7 +46171,7 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D121" t="n">
         <v>7</v>
@@ -46200,7 +46200,7 @@
         </is>
       </c>
       <c r="C122" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D122" t="n">
         <v>7</v>
@@ -46229,7 +46229,7 @@
         </is>
       </c>
       <c r="C123" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D123" t="n">
         <v>7</v>
@@ -46258,7 +46258,7 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D124" t="n">
         <v>7</v>
@@ -46287,7 +46287,7 @@
         </is>
       </c>
       <c r="C125" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D125" t="n">
         <v>7</v>
@@ -46316,7 +46316,7 @@
         </is>
       </c>
       <c r="C126" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D126" t="n">
         <v>7</v>
@@ -46345,7 +46345,7 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D127" t="n">
         <v>7</v>
@@ -46374,7 +46374,7 @@
         </is>
       </c>
       <c r="C128" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D128" t="n">
         <v>7</v>
@@ -46403,7 +46403,7 @@
         </is>
       </c>
       <c r="C129" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D129" t="n">
         <v>7</v>
@@ -46432,7 +46432,7 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D130" t="n">
         <v>7</v>
@@ -46461,7 +46461,7 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D131" t="n">
         <v>7</v>
@@ -46490,7 +46490,7 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D132" t="n">
         <v>7</v>
@@ -46519,7 +46519,7 @@
         </is>
       </c>
       <c r="C133" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D133" t="n">
         <v>7</v>
@@ -46548,7 +46548,7 @@
         </is>
       </c>
       <c r="C134" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D134" t="n">
         <v>7</v>
@@ -46577,7 +46577,7 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D135" t="n">
         <v>7</v>
@@ -46606,7 +46606,7 @@
         </is>
       </c>
       <c r="C136" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D136" t="n">
         <v>7</v>
@@ -46635,7 +46635,7 @@
         </is>
       </c>
       <c r="C137" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D137" t="n">
         <v>7</v>
@@ -46664,7 +46664,7 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D138" t="n">
         <v>7</v>
@@ -46693,7 +46693,7 @@
         </is>
       </c>
       <c r="C139" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D139" t="n">
         <v>7</v>
@@ -46722,7 +46722,7 @@
         </is>
       </c>
       <c r="C140" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D140" t="n">
         <v>7</v>
@@ -46751,7 +46751,7 @@
         </is>
       </c>
       <c r="C141" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D141" t="n">
         <v>7</v>
@@ -46780,7 +46780,7 @@
         </is>
       </c>
       <c r="C142" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D142" t="n">
         <v>7</v>
@@ -46809,7 +46809,7 @@
         </is>
       </c>
       <c r="C143" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D143" t="n">
         <v>7</v>
@@ -46838,7 +46838,7 @@
         </is>
       </c>
       <c r="C144" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D144" t="n">
         <v>7</v>
@@ -46867,7 +46867,7 @@
         </is>
       </c>
       <c r="C145" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D145" t="n">
         <v>7</v>
@@ -46896,7 +46896,7 @@
         </is>
       </c>
       <c r="C146" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D146" t="n">
         <v>7</v>
@@ -46925,7 +46925,7 @@
         </is>
       </c>
       <c r="C147" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D147" t="n">
         <v>7</v>
@@ -46954,7 +46954,7 @@
         </is>
       </c>
       <c r="C148" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D148" t="n">
         <v>7</v>
@@ -46983,7 +46983,7 @@
         </is>
       </c>
       <c r="C149" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D149" t="n">
         <v>7</v>
@@ -47012,7 +47012,7 @@
         </is>
       </c>
       <c r="C150" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D150" t="n">
         <v>7</v>
@@ -47041,7 +47041,7 @@
         </is>
       </c>
       <c r="C151" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D151" t="n">
         <v>7</v>
@@ -47070,7 +47070,7 @@
         </is>
       </c>
       <c r="C152" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D152" t="n">
         <v>7</v>
@@ -47099,7 +47099,7 @@
         </is>
       </c>
       <c r="C153" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D153" t="n">
         <v>7</v>
@@ -47128,7 +47128,7 @@
         </is>
       </c>
       <c r="C154" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D154" t="n">
         <v>7</v>
@@ -47157,7 +47157,7 @@
         </is>
       </c>
       <c r="C155" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D155" t="n">
         <v>7</v>
@@ -47186,7 +47186,7 @@
         </is>
       </c>
       <c r="C156" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D156" t="n">
         <v>7</v>
@@ -47215,7 +47215,7 @@
         </is>
       </c>
       <c r="C157" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D157" t="n">
         <v>7</v>
@@ -47244,7 +47244,7 @@
         </is>
       </c>
       <c r="C158" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D158" t="n">
         <v>7</v>
@@ -47273,7 +47273,7 @@
         </is>
       </c>
       <c r="C159" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D159" t="n">
         <v>7</v>
@@ -47302,7 +47302,7 @@
         </is>
       </c>
       <c r="C160" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D160" t="n">
         <v>7</v>
@@ -47331,7 +47331,7 @@
         </is>
       </c>
       <c r="C161" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D161" t="n">
         <v>7</v>
@@ -47360,7 +47360,7 @@
         </is>
       </c>
       <c r="C162" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D162" t="n">
         <v>7</v>
@@ -47389,7 +47389,7 @@
         </is>
       </c>
       <c r="C163" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D163" t="n">
         <v>7</v>
@@ -47418,7 +47418,7 @@
         </is>
       </c>
       <c r="C164" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D164" t="n">
         <v>7</v>
@@ -47447,7 +47447,7 @@
         </is>
       </c>
       <c r="C165" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D165" t="n">
         <v>7</v>
@@ -47476,7 +47476,7 @@
         </is>
       </c>
       <c r="C166" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D166" t="n">
         <v>7</v>
@@ -47505,7 +47505,7 @@
         </is>
       </c>
       <c r="C167" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D167" t="n">
         <v>7</v>
@@ -47534,7 +47534,7 @@
         </is>
       </c>
       <c r="C168" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D168" t="n">
         <v>7</v>
@@ -47563,7 +47563,7 @@
         </is>
       </c>
       <c r="C169" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D169" t="n">
         <v>7</v>
@@ -47592,7 +47592,7 @@
         </is>
       </c>
       <c r="C170" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D170" t="n">
         <v>7</v>
@@ -47621,7 +47621,7 @@
         </is>
       </c>
       <c r="C171" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D171" t="n">
         <v>7</v>
@@ -47650,7 +47650,7 @@
         </is>
       </c>
       <c r="C172" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D172" t="n">
         <v>7</v>
@@ -47679,7 +47679,7 @@
         </is>
       </c>
       <c r="C173" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D173" t="n">
         <v>7</v>
@@ -47708,7 +47708,7 @@
         </is>
       </c>
       <c r="C174" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D174" t="n">
         <v>7</v>
@@ -47737,7 +47737,7 @@
         </is>
       </c>
       <c r="C175" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D175" t="n">
         <v>1</v>
@@ -47766,7 +47766,7 @@
         </is>
       </c>
       <c r="C176" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D176" t="n">
         <v>7</v>
@@ -47795,7 +47795,7 @@
         </is>
       </c>
       <c r="C177" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D177" t="n">
         <v>7</v>
@@ -47824,7 +47824,7 @@
         </is>
       </c>
       <c r="C178" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D178" t="n">
         <v>7</v>
@@ -47853,7 +47853,7 @@
         </is>
       </c>
       <c r="C179" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D179" t="n">
         <v>7</v>
@@ -47882,7 +47882,7 @@
         </is>
       </c>
       <c r="C180" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D180" t="n">
         <v>7</v>
@@ -47911,7 +47911,7 @@
         </is>
       </c>
       <c r="C181" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D181" t="n">
         <v>7</v>
@@ -47940,7 +47940,7 @@
         </is>
       </c>
       <c r="C182" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D182" t="n">
         <v>7</v>
@@ -47969,7 +47969,7 @@
         </is>
       </c>
       <c r="C183" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D183" t="n">
         <v>7</v>
@@ -47998,7 +47998,7 @@
         </is>
       </c>
       <c r="C184" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D184" t="n">
         <v>1</v>
@@ -48027,7 +48027,7 @@
         </is>
       </c>
       <c r="C185" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D185" t="n">
         <v>1</v>
@@ -48056,7 +48056,7 @@
         </is>
       </c>
       <c r="C186" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D186" t="n">
         <v>1</v>
@@ -48085,7 +48085,7 @@
         </is>
       </c>
       <c r="C187" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D187" t="n">
         <v>1</v>
@@ -48114,7 +48114,7 @@
         </is>
       </c>
       <c r="C188" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D188" t="n">
         <v>1</v>
@@ -48143,7 +48143,7 @@
         </is>
       </c>
       <c r="C189" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D189" t="n">
         <v>1</v>
@@ -48172,7 +48172,7 @@
         </is>
       </c>
       <c r="C190" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D190" t="n">
         <v>1</v>
@@ -48201,7 +48201,7 @@
         </is>
       </c>
       <c r="C191" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D191" t="n">
         <v>1</v>
@@ -48230,7 +48230,7 @@
         </is>
       </c>
       <c r="C192" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D192" t="n">
         <v>1</v>
@@ -48259,7 +48259,7 @@
         </is>
       </c>
       <c r="C193" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D193" t="n">
         <v>1</v>
@@ -48288,7 +48288,7 @@
         </is>
       </c>
       <c r="C194" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D194" t="n">
         <v>1</v>
@@ -48317,7 +48317,7 @@
         </is>
       </c>
       <c r="C195" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D195" t="n">
         <v>1</v>
@@ -48346,7 +48346,7 @@
         </is>
       </c>
       <c r="C196" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D196" t="n">
         <v>1</v>
@@ -48375,7 +48375,7 @@
         </is>
       </c>
       <c r="C197" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D197" t="n">
         <v>1</v>
@@ -48404,7 +48404,7 @@
         </is>
       </c>
       <c r="C198" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D198" t="n">
         <v>1</v>
@@ -48433,7 +48433,7 @@
         </is>
       </c>
       <c r="C199" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D199" t="n">
         <v>1</v>
@@ -48462,7 +48462,7 @@
         </is>
       </c>
       <c r="C200" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D200" t="n">
         <v>1</v>
@@ -48491,7 +48491,7 @@
         </is>
       </c>
       <c r="C201" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D201" t="n">
         <v>1</v>
@@ -48520,7 +48520,7 @@
         </is>
       </c>
       <c r="C202" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D202" t="n">
         <v>1</v>
@@ -48549,7 +48549,7 @@
         </is>
       </c>
       <c r="C203" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D203" t="n">
         <v>1</v>
@@ -48578,7 +48578,7 @@
         </is>
       </c>
       <c r="C204" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D204" t="n">
         <v>1</v>
@@ -48607,7 +48607,7 @@
         </is>
       </c>
       <c r="C205" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D205" t="n">
         <v>1</v>
@@ -48636,7 +48636,7 @@
         </is>
       </c>
       <c r="C206" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D206" t="n">
         <v>1</v>
@@ -48665,7 +48665,7 @@
         </is>
       </c>
       <c r="C207" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D207" t="n">
         <v>1</v>
@@ -48694,7 +48694,7 @@
         </is>
       </c>
       <c r="C208" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D208" t="n">
         <v>1</v>
@@ -48723,7 +48723,7 @@
         </is>
       </c>
       <c r="C209" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D209" t="n">
         <v>1</v>
@@ -48752,7 +48752,7 @@
         </is>
       </c>
       <c r="C210" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D210" t="n">
         <v>1</v>
@@ -48781,7 +48781,7 @@
         </is>
       </c>
       <c r="C211" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D211" t="n">
         <v>7</v>
@@ -48810,7 +48810,7 @@
         </is>
       </c>
       <c r="C212" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D212" t="n">
         <v>1</v>
@@ -48839,7 +48839,7 @@
         </is>
       </c>
       <c r="C213" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D213" t="n">
         <v>1</v>
@@ -48868,7 +48868,7 @@
         </is>
       </c>
       <c r="C214" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D214" t="n">
         <v>1</v>
@@ -48897,7 +48897,7 @@
         </is>
       </c>
       <c r="C215" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D215" t="n">
         <v>1</v>
@@ -48926,7 +48926,7 @@
         </is>
       </c>
       <c r="C216" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D216" t="n">
         <v>1</v>
@@ -48955,7 +48955,7 @@
         </is>
       </c>
       <c r="C217" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D217" t="n">
         <v>1</v>
@@ -48984,7 +48984,7 @@
         </is>
       </c>
       <c r="C218" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D218" t="n">
         <v>1</v>
@@ -49013,7 +49013,7 @@
         </is>
       </c>
       <c r="C219" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D219" t="n">
         <v>1</v>
@@ -49042,7 +49042,7 @@
         </is>
       </c>
       <c r="C220" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D220" t="n">
         <v>1</v>
@@ -49071,7 +49071,7 @@
         </is>
       </c>
       <c r="C221" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D221" t="n">
         <v>1</v>
@@ -49100,7 +49100,7 @@
         </is>
       </c>
       <c r="C222" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D222" t="n">
         <v>1</v>
@@ -49129,7 +49129,7 @@
         </is>
       </c>
       <c r="C223" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D223" t="n">
         <v>1</v>
@@ -49158,7 +49158,7 @@
         </is>
       </c>
       <c r="C224" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D224" t="n">
         <v>1</v>
@@ -49187,7 +49187,7 @@
         </is>
       </c>
       <c r="C225" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D225" t="n">
         <v>1</v>
@@ -49216,7 +49216,7 @@
         </is>
       </c>
       <c r="C226" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D226" t="n">
         <v>1</v>
@@ -49245,7 +49245,7 @@
         </is>
       </c>
       <c r="C227" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D227" t="n">
         <v>1</v>
@@ -49274,7 +49274,7 @@
         </is>
       </c>
       <c r="C228" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D228" t="n">
         <v>1</v>
@@ -49303,7 +49303,7 @@
         </is>
       </c>
       <c r="C229" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D229" t="n">
         <v>1</v>
@@ -49332,7 +49332,7 @@
         </is>
       </c>
       <c r="C230" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D230" t="n">
         <v>1</v>
@@ -49361,7 +49361,7 @@
         </is>
       </c>
       <c r="C231" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D231" t="n">
         <v>1</v>
@@ -49390,7 +49390,7 @@
         </is>
       </c>
       <c r="C232" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D232" t="n">
         <v>1</v>
@@ -49419,7 +49419,7 @@
         </is>
       </c>
       <c r="C233" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D233" t="n">
         <v>1</v>
@@ -49448,7 +49448,7 @@
         </is>
       </c>
       <c r="C234" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D234" t="n">
         <v>1</v>
@@ -49477,7 +49477,7 @@
         </is>
       </c>
       <c r="C235" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D235" t="n">
         <v>1</v>
@@ -49506,7 +49506,7 @@
         </is>
       </c>
       <c r="C236" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D236" t="n">
         <v>1</v>
@@ -49535,7 +49535,7 @@
         </is>
       </c>
       <c r="C237" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D237" t="n">
         <v>1</v>
@@ -49564,7 +49564,7 @@
         </is>
       </c>
       <c r="C238" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D238" t="n">
         <v>1</v>
@@ -49593,7 +49593,7 @@
         </is>
       </c>
       <c r="C239" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D239" t="n">
         <v>1</v>
@@ -49622,7 +49622,7 @@
         </is>
       </c>
       <c r="C240" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D240" t="n">
         <v>1</v>
@@ -49651,7 +49651,7 @@
         </is>
       </c>
       <c r="C241" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D241" t="n">
         <v>1</v>
@@ -49680,7 +49680,7 @@
         </is>
       </c>
       <c r="C242" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D242" t="n">
         <v>1</v>
@@ -49709,7 +49709,7 @@
         </is>
       </c>
       <c r="C243" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D243" t="n">
         <v>1</v>
@@ -49738,7 +49738,7 @@
         </is>
       </c>
       <c r="C244" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D244" t="n">
         <v>1</v>
@@ -49767,7 +49767,7 @@
         </is>
       </c>
       <c r="C245" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D245" t="n">
         <v>1</v>
@@ -49796,7 +49796,7 @@
         </is>
       </c>
       <c r="C246" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D246" t="n">
         <v>1</v>
@@ -49825,7 +49825,7 @@
         </is>
       </c>
       <c r="C247" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D247" t="n">
         <v>1</v>
@@ -49854,7 +49854,7 @@
         </is>
       </c>
       <c r="C248" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D248" t="n">
         <v>1</v>
@@ -49883,7 +49883,7 @@
         </is>
       </c>
       <c r="C249" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D249" t="n">
         <v>1</v>
@@ -49912,7 +49912,7 @@
         </is>
       </c>
       <c r="C250" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D250" t="n">
         <v>1</v>
@@ -49941,7 +49941,7 @@
         </is>
       </c>
       <c r="C251" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D251" t="n">
         <v>1</v>
@@ -49970,7 +49970,7 @@
         </is>
       </c>
       <c r="C252" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D252" t="n">
         <v>1</v>
@@ -49999,7 +49999,7 @@
         </is>
       </c>
       <c r="C253" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D253" t="n">
         <v>1</v>
@@ -50028,7 +50028,7 @@
         </is>
       </c>
       <c r="C254" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D254" t="n">
         <v>1</v>
@@ -50057,7 +50057,7 @@
         </is>
       </c>
       <c r="C255" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D255" t="n">
         <v>1</v>
@@ -50086,7 +50086,7 @@
         </is>
       </c>
       <c r="C256" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D256" t="n">
         <v>1</v>
@@ -50115,7 +50115,7 @@
         </is>
       </c>
       <c r="C257" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D257" t="n">
         <v>1</v>
@@ -50144,7 +50144,7 @@
         </is>
       </c>
       <c r="C258" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D258" t="n">
         <v>1</v>
@@ -50173,7 +50173,7 @@
         </is>
       </c>
       <c r="C259" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D259" t="n">
         <v>1</v>
@@ -50202,7 +50202,7 @@
         </is>
       </c>
       <c r="C260" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D260" t="n">
         <v>1</v>
@@ -50231,7 +50231,7 @@
         </is>
       </c>
       <c r="C261" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D261" t="n">
         <v>1</v>
@@ -50260,7 +50260,7 @@
         </is>
       </c>
       <c r="C262" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D262" t="n">
         <v>1</v>
@@ -50289,7 +50289,7 @@
         </is>
       </c>
       <c r="C263" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D263" t="n">
         <v>1</v>
@@ -50318,7 +50318,7 @@
         </is>
       </c>
       <c r="C264" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D264" t="n">
         <v>1</v>
@@ -50347,7 +50347,7 @@
         </is>
       </c>
       <c r="C265" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D265" t="n">
         <v>1</v>
@@ -50376,7 +50376,7 @@
         </is>
       </c>
       <c r="C266" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D266" t="n">
         <v>1</v>
@@ -50405,7 +50405,7 @@
         </is>
       </c>
       <c r="C267" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D267" t="n">
         <v>1</v>
@@ -50434,7 +50434,7 @@
         </is>
       </c>
       <c r="C268" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D268" t="n">
         <v>1</v>
@@ -50454,7 +50454,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>marches/fx/GBPUSD.csv</t>
+          <t>marches/fx/NZDUSD.csv</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
@@ -50463,7 +50463,7 @@
         </is>
       </c>
       <c r="C269" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D269" t="n">
         <v>1</v>
@@ -50483,7 +50483,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>marches/fx/NZDUSD.csv</t>
+          <t>marches/fx/USDCAD.csv</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
@@ -50492,7 +50492,7 @@
         </is>
       </c>
       <c r="C270" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D270" t="n">
         <v>1</v>
@@ -50501,7 +50501,7 @@
         <v>42</v>
       </c>
       <c r="F270" t="n">
-        <v>3907</v>
+        <v>3906</v>
       </c>
       <c r="G270" t="inlineStr">
         <is>
@@ -50512,7 +50512,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>marches/fx/USDCAD.csv</t>
+          <t>marches/fx/USDCNY.csv</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
@@ -50521,7 +50521,7 @@
         </is>
       </c>
       <c r="C271" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D271" t="n">
         <v>1</v>
@@ -50541,7 +50541,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>marches/fx/USDCNY.csv</t>
+          <t>marches/fx/USDJPY.csv</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
@@ -50550,7 +50550,7 @@
         </is>
       </c>
       <c r="C272" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D272" t="n">
         <v>1</v>
@@ -50559,7 +50559,7 @@
         <v>42</v>
       </c>
       <c r="F272" t="n">
-        <v>3906</v>
+        <v>3907</v>
       </c>
       <c r="G272" t="inlineStr">
         <is>
@@ -50570,7 +50570,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>marches/fx/USDJPY.csv</t>
+          <t>marches/fx/USDKRW.csv</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
@@ -50579,7 +50579,7 @@
         </is>
       </c>
       <c r="C273" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D273" t="n">
         <v>1</v>
@@ -50588,7 +50588,7 @@
         <v>42</v>
       </c>
       <c r="F273" t="n">
-        <v>3907</v>
+        <v>3906</v>
       </c>
       <c r="G273" t="inlineStr">
         <is>
@@ -50599,7 +50599,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>marches/fx/USDKRW.csv</t>
+          <t>marches/fx/USDNOK.csv</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
@@ -50608,7 +50608,7 @@
         </is>
       </c>
       <c r="C274" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D274" t="n">
         <v>1</v>
@@ -50617,7 +50617,7 @@
         <v>42</v>
       </c>
       <c r="F274" t="n">
-        <v>3906</v>
+        <v>3907</v>
       </c>
       <c r="G274" t="inlineStr">
         <is>
@@ -50628,7 +50628,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>marches/fx/USDNOK.csv</t>
+          <t>marches/fx/USDSEK.csv</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
@@ -50637,7 +50637,7 @@
         </is>
       </c>
       <c r="C275" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D275" t="n">
         <v>1</v>
@@ -50657,12 +50657,12 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>marches/fx/USDSEK.csv</t>
+          <t>marches/fx/GBPUSD.csv</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="C276" t="n">
@@ -50695,7 +50695,7 @@
         </is>
       </c>
       <c r="C277" t="n">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="D277" t="n">
         <v>2</v>
@@ -50724,7 +50724,7 @@
         </is>
       </c>
       <c r="C278" t="n">
-        <v>-437</v>
+        <v>-436</v>
       </c>
       <c r="D278" t="n">
         <v>42</v>

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-27T01:56Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-27 00:58 UTC</t>
+          <t>Genere le 2026-09-27 01:56 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-27 00:58 UTC</t>
+          <t>Rapport global — 2026-09-27 01:56 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-27T05:58Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-27 01:56 UTC</t>
+          <t>Genere le 2026-09-27 05:58 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-27 01:56 UTC</t>
+          <t>Rapport global — 2026-09-27 05:58 UTC</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>**Matieres premieres macro** — ratio cuivre/or stable -- pas de signal net sur la croissance (+3.3% sur 3 mois). Brent 104.3$ (+44.9% sur 3 mois, +50.3% sur 12 mois), gaz -1.1% sur 3 mois, ecart Brent-WTI +11.9$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-25)_</t>
+          <t>**Matieres premieres macro** — ratio cuivre/or stable -- pas de signal net sur la croissance (+4.4% sur 3 mois). Brent 97.4$ (+35.4% sur 3 mois, +40.4% sur 12 mois), gaz -0.2% sur 3 mois, ecart Brent-WTI +5.0$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
@@ -1240,7 +1240,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.3769116249569233 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.05237241130035915 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-25)_</t>
+          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.3769116249569233 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.052372411300360217 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
@@ -49341,7 +49341,7 @@
         <v>42</v>
       </c>
       <c r="F230" t="n">
-        <v>3773</v>
+        <v>3772</v>
       </c>
       <c r="G230" t="inlineStr">
         <is>
@@ -49631,7 +49631,7 @@
         <v>42</v>
       </c>
       <c r="F240" t="n">
-        <v>3772</v>
+        <v>3771</v>
       </c>
       <c r="G240" t="inlineStr">
         <is>
@@ -49660,7 +49660,7 @@
         <v>42</v>
       </c>
       <c r="F241" t="n">
-        <v>3773</v>
+        <v>3772</v>
       </c>
       <c r="G241" t="inlineStr">
         <is>
@@ -49689,7 +49689,7 @@
         <v>42</v>
       </c>
       <c r="F242" t="n">
-        <v>3772</v>
+        <v>3771</v>
       </c>
       <c r="G242" t="inlineStr">
         <is>
@@ -49718,7 +49718,7 @@
         <v>42</v>
       </c>
       <c r="F243" t="n">
-        <v>3772</v>
+        <v>3771</v>
       </c>
       <c r="G243" t="inlineStr">
         <is>
@@ -49747,7 +49747,7 @@
         <v>42</v>
       </c>
       <c r="F244" t="n">
-        <v>3773</v>
+        <v>3772</v>
       </c>
       <c r="G244" t="inlineStr">
         <is>
@@ -50338,7 +50338,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>marches/fx/AUDJPY.csv</t>
+          <t>marches/fx/EURGBP.csv</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
@@ -50356,7 +50356,7 @@
         <v>42</v>
       </c>
       <c r="F265" t="n">
-        <v>3910</v>
+        <v>3909</v>
       </c>
       <c r="G265" t="inlineStr">
         <is>
@@ -50367,7 +50367,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>marches/fx/AUDUSD.csv</t>
+          <t>marches/fx/EURUSD.csv</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
@@ -50396,16 +50396,16 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>marches/fx/EURGBP.csv</t>
+          <t>marches/fx/AUDJPY.csv</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="C267" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D267" t="n">
         <v>1</v>
@@ -50414,7 +50414,7 @@
         <v>42</v>
       </c>
       <c r="F267" t="n">
-        <v>3909</v>
+        <v>3910</v>
       </c>
       <c r="G267" t="inlineStr">
         <is>
@@ -50425,16 +50425,16 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>marches/fx/EURUSD.csv</t>
+          <t>marches/fx/AUDUSD.csv</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="C268" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D268" t="n">
         <v>1</v>
@@ -50454,16 +50454,16 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>marches/fx/NZDUSD.csv</t>
+          <t>marches/fx/GBPUSD.csv</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="C269" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D269" t="n">
         <v>1</v>
@@ -50483,16 +50483,16 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>marches/fx/USDCAD.csv</t>
+          <t>marches/fx/NZDUSD.csv</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="C270" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D270" t="n">
         <v>1</v>
@@ -50501,7 +50501,7 @@
         <v>42</v>
       </c>
       <c r="F270" t="n">
-        <v>3906</v>
+        <v>3907</v>
       </c>
       <c r="G270" t="inlineStr">
         <is>
@@ -50512,16 +50512,16 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>marches/fx/USDCNY.csv</t>
+          <t>marches/fx/USDCAD.csv</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="C271" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D271" t="n">
         <v>1</v>
@@ -50541,16 +50541,16 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>marches/fx/USDJPY.csv</t>
+          <t>marches/fx/USDCNY.csv</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="C272" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D272" t="n">
         <v>1</v>
@@ -50559,7 +50559,7 @@
         <v>42</v>
       </c>
       <c r="F272" t="n">
-        <v>3907</v>
+        <v>3906</v>
       </c>
       <c r="G272" t="inlineStr">
         <is>
@@ -50570,16 +50570,16 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>marches/fx/USDKRW.csv</t>
+          <t>marches/fx/USDJPY.csv</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="C273" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D273" t="n">
         <v>1</v>
@@ -50588,7 +50588,7 @@
         <v>42</v>
       </c>
       <c r="F273" t="n">
-        <v>3906</v>
+        <v>3907</v>
       </c>
       <c r="G273" t="inlineStr">
         <is>
@@ -50599,16 +50599,16 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>marches/fx/USDNOK.csv</t>
+          <t>marches/fx/USDKRW.csv</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="C274" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D274" t="n">
         <v>1</v>
@@ -50617,7 +50617,7 @@
         <v>42</v>
       </c>
       <c r="F274" t="n">
-        <v>3907</v>
+        <v>3906</v>
       </c>
       <c r="G274" t="inlineStr">
         <is>
@@ -50628,16 +50628,16 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>marches/fx/USDSEK.csv</t>
+          <t>marches/fx/USDNOK.csv</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="C275" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D275" t="n">
         <v>1</v>
@@ -50657,7 +50657,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>marches/fx/GBPUSD.csv</t>
+          <t>marches/fx/USDSEK.csv</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
@@ -54279,25 +54279,25 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.001549</v>
+        <v>0.001566</v>
       </c>
       <c r="C9" t="n">
-        <v>3.35</v>
+        <v>4.43</v>
       </c>
       <c r="D9" t="n">
-        <v>104.32</v>
+        <v>97.44</v>
       </c>
       <c r="E9" t="n">
-        <v>44.91</v>
+        <v>35.35</v>
       </c>
       <c r="F9" t="n">
-        <v>50.27</v>
+        <v>40.36</v>
       </c>
       <c r="G9" t="n">
-        <v>-1.08</v>
+        <v>-0.19</v>
       </c>
       <c r="H9" t="n">
-        <v>11.91</v>
+        <v>5.03</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-27T08:19Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-27 05:58 UTC</t>
+          <t>Genere le 2026-09-27 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-27 05:58 UTC</t>
+          <t>Rapport global — 2026-09-27 08:19 UTC</t>
         </is>
       </c>
     </row>
@@ -1240,7 +1240,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.3769116249569233 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.052372411300360217 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-25)_</t>
+          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.3769116249569233 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.05237241130035915 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-27T10:55Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-27 08:19 UTC</t>
+          <t>Genere le 2026-09-27 10:55 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-27 08:19 UTC</t>
+          <t>Rapport global — 2026-09-27 10:55 UTC</t>
         </is>
       </c>
     </row>
@@ -1240,7 +1240,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.3769116249569233 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.05237241130035915 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-25)_</t>
+          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.3769116249569233 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.052372411300360217 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-27T14:08Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-27 10:55 UTC</t>
+          <t>Genere le 2026-09-27 14:08 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-27 10:55 UTC</t>
+          <t>Rapport global — 2026-09-27 14:08 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-27T15:26Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-27 14:08 UTC</t>
+          <t>Genere le 2026-09-27 15:26 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-27 14:08 UTC</t>
+          <t>Rapport global — 2026-09-27 15:26 UTC</t>
         </is>
       </c>
     </row>
@@ -1240,7 +1240,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.3769116249569233 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.052372411300360217 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-25)_</t>
+          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.3769116249569233 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.05237241130035915 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-27T18:33Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-27 15:26 UTC</t>
+          <t>Genere le 2026-09-27 18:33 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-27 15:26 UTC</t>
+          <t>Rapport global — 2026-09-27 18:33 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-27T21:44Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-27 18:33 UTC</t>
+          <t>Genere le 2026-09-27 21:44 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-27 18:33 UTC</t>
+          <t>Rapport global — 2026-09-27 21:44 UTC</t>
         </is>
       </c>
     </row>
@@ -49352,7 +49352,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>marches/fx/EURCHF.csv</t>
+          <t>marches/indices/DAX.csv</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -49370,7 +49370,7 @@
         <v>42</v>
       </c>
       <c r="F231" t="n">
-        <v>3907</v>
+        <v>3803</v>
       </c>
       <c r="G231" t="inlineStr">
         <is>
@@ -49381,7 +49381,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>marches/fx/EURJPY.csv</t>
+          <t>marches/indices/EUROSTOXX50.csv</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -49399,7 +49399,7 @@
         <v>42</v>
       </c>
       <c r="F232" t="n">
-        <v>3909</v>
+        <v>3760</v>
       </c>
       <c r="G232" t="inlineStr">
         <is>
@@ -49410,7 +49410,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>marches/fx/USDCHF.csv</t>
+          <t>marches/indices/FTSE100.csv</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -49428,7 +49428,7 @@
         <v>42</v>
       </c>
       <c r="F233" t="n">
-        <v>3904</v>
+        <v>3789</v>
       </c>
       <c r="G233" t="inlineStr">
         <is>
@@ -49439,7 +49439,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>marches/indices/DAX.csv</t>
+          <t>marches/indices/HANGSENG.csv</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -49457,7 +49457,7 @@
         <v>42</v>
       </c>
       <c r="F234" t="n">
-        <v>3803</v>
+        <v>3690</v>
       </c>
       <c r="G234" t="inlineStr">
         <is>
@@ -49468,7 +49468,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>marches/indices/EUROSTOXX50.csv</t>
+          <t>marches/indices/NIKKEI225.csv</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -49486,7 +49486,7 @@
         <v>42</v>
       </c>
       <c r="F235" t="n">
-        <v>3760</v>
+        <v>3668</v>
       </c>
       <c r="G235" t="inlineStr">
         <is>
@@ -49497,7 +49497,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>marches/indices/FTSE100.csv</t>
+          <t>marches/matieres/BRENT.csv</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -49515,7 +49515,7 @@
         <v>42</v>
       </c>
       <c r="F236" t="n">
-        <v>3789</v>
+        <v>3751</v>
       </c>
       <c r="G236" t="inlineStr">
         <is>
@@ -49526,7 +49526,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>marches/indices/HANGSENG.csv</t>
+          <t>marches/matieres/CUIVRE.csv</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
@@ -49544,7 +49544,7 @@
         <v>42</v>
       </c>
       <c r="F237" t="n">
-        <v>3690</v>
+        <v>3771</v>
       </c>
       <c r="G237" t="inlineStr">
         <is>
@@ -49555,7 +49555,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>marches/indices/NIKKEI225.csv</t>
+          <t>marches/matieres/GAZ_HENRY_HUB.csv</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
@@ -49573,7 +49573,7 @@
         <v>42</v>
       </c>
       <c r="F238" t="n">
-        <v>3668</v>
+        <v>3772</v>
       </c>
       <c r="G238" t="inlineStr">
         <is>
@@ -49584,7 +49584,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>marches/matieres/BRENT.csv</t>
+          <t>marches/matieres/OR.csv</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
@@ -49602,7 +49602,7 @@
         <v>42</v>
       </c>
       <c r="F239" t="n">
-        <v>3751</v>
+        <v>3771</v>
       </c>
       <c r="G239" t="inlineStr">
         <is>
@@ -49613,7 +49613,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>marches/matieres/CUIVRE.csv</t>
+          <t>marches/matieres/WTI.csv</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
@@ -49642,7 +49642,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>marches/matieres/GAZ_HENRY_HUB.csv</t>
+          <t>marches/taux_futures/FED_FUNDS_FRONT.csv</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
@@ -49671,7 +49671,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>marches/matieres/OR.csv</t>
+          <t>marches/volatilite/GVZ.csv</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
@@ -49689,7 +49689,7 @@
         <v>42</v>
       </c>
       <c r="F242" t="n">
-        <v>3771</v>
+        <v>3772</v>
       </c>
       <c r="G242" t="inlineStr">
         <is>
@@ -49700,7 +49700,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>marches/matieres/WTI.csv</t>
+          <t>marches/volatilite/MOVE.csv</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
@@ -49718,7 +49718,7 @@
         <v>42</v>
       </c>
       <c r="F243" t="n">
-        <v>3771</v>
+        <v>3691</v>
       </c>
       <c r="G243" t="inlineStr">
         <is>
@@ -49729,7 +49729,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>marches/taux_futures/FED_FUNDS_FRONT.csv</t>
+          <t>marches/volatilite/OVX.csv</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -49758,7 +49758,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>marches/volatilite/GVZ.csv</t>
+          <t>marches/volatilite/VVIX.csv</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -49776,7 +49776,7 @@
         <v>42</v>
       </c>
       <c r="F245" t="n">
-        <v>3772</v>
+        <v>3764</v>
       </c>
       <c r="G245" t="inlineStr">
         <is>
@@ -49787,7 +49787,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>marches/volatilite/MOVE.csv</t>
+          <t>marches/volatilite/VXN.csv</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -49805,7 +49805,7 @@
         <v>42</v>
       </c>
       <c r="F246" t="n">
-        <v>3691</v>
+        <v>3772</v>
       </c>
       <c r="G246" t="inlineStr">
         <is>
@@ -49816,7 +49816,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>marches/volatilite/OVX.csv</t>
+          <t>souverains/SUEDE_10A.csv</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
@@ -49834,7 +49834,7 @@
         <v>42</v>
       </c>
       <c r="F247" t="n">
-        <v>3772</v>
+        <v>9202</v>
       </c>
       <c r="G247" t="inlineStr">
         <is>
@@ -49845,7 +49845,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>marches/volatilite/VVIX.csv</t>
+          <t>souverains/SUEDE_2A.csv</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
@@ -49863,7 +49863,7 @@
         <v>42</v>
       </c>
       <c r="F248" t="n">
-        <v>3764</v>
+        <v>9202</v>
       </c>
       <c r="G248" t="inlineStr">
         <is>
@@ -49874,7 +49874,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>marches/volatilite/VXN.csv</t>
+          <t>souverains/SUEDE_5A.csv</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
@@ -49892,7 +49892,7 @@
         <v>42</v>
       </c>
       <c r="F249" t="n">
-        <v>3772</v>
+        <v>9204</v>
       </c>
       <c r="G249" t="inlineStr">
         <is>
@@ -49903,7 +49903,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_10A.csv</t>
+          <t>yfinance/SP500.csv</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
@@ -49921,7 +49921,7 @@
         <v>42</v>
       </c>
       <c r="F250" t="n">
-        <v>9202</v>
+        <v>7547</v>
       </c>
       <c r="G250" t="inlineStr">
         <is>
@@ -49932,7 +49932,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_2A.csv</t>
+          <t>yfinance/VIX.csv</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
@@ -49950,7 +49950,7 @@
         <v>42</v>
       </c>
       <c r="F251" t="n">
-        <v>9202</v>
+        <v>7550</v>
       </c>
       <c r="G251" t="inlineStr">
         <is>
@@ -49961,7 +49961,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_5A.csv</t>
+          <t>yfinance/XLB.csv</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -49979,7 +49979,7 @@
         <v>42</v>
       </c>
       <c r="F252" t="n">
-        <v>9204</v>
+        <v>501</v>
       </c>
       <c r="G252" t="inlineStr">
         <is>
@@ -49990,7 +49990,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>yfinance/SP500.csv</t>
+          <t>yfinance/XLE.csv</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -50008,7 +50008,7 @@
         <v>42</v>
       </c>
       <c r="F253" t="n">
-        <v>7547</v>
+        <v>501</v>
       </c>
       <c r="G253" t="inlineStr">
         <is>
@@ -50019,7 +50019,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>yfinance/VIX.csv</t>
+          <t>yfinance/XLF.csv</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
@@ -50037,7 +50037,7 @@
         <v>42</v>
       </c>
       <c r="F254" t="n">
-        <v>7550</v>
+        <v>501</v>
       </c>
       <c r="G254" t="inlineStr">
         <is>
@@ -50048,7 +50048,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>yfinance/XLB.csv</t>
+          <t>yfinance/XLI.csv</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
@@ -50077,7 +50077,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>yfinance/XLE.csv</t>
+          <t>yfinance/XLK.csv</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
@@ -50106,7 +50106,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>yfinance/XLF.csv</t>
+          <t>yfinance/XLP.csv</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
@@ -50135,7 +50135,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>yfinance/XLI.csv</t>
+          <t>yfinance/XLRE.csv</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
@@ -50164,7 +50164,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>yfinance/XLK.csv</t>
+          <t>yfinance/XLU.csv</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
@@ -50193,7 +50193,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>yfinance/XLP.csv</t>
+          <t>yfinance/XLV.csv</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
@@ -50222,7 +50222,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>yfinance/XLRE.csv</t>
+          <t>yfinance/XLY.csv</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
@@ -50251,16 +50251,16 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>yfinance/XLU.csv</t>
+          <t>marches/fx/AUDJPY.csv</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="C262" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D262" t="n">
         <v>1</v>
@@ -50269,7 +50269,7 @@
         <v>42</v>
       </c>
       <c r="F262" t="n">
-        <v>501</v>
+        <v>3910</v>
       </c>
       <c r="G262" t="inlineStr">
         <is>
@@ -50280,16 +50280,16 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>yfinance/XLV.csv</t>
+          <t>marches/fx/AUDUSD.csv</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="C263" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D263" t="n">
         <v>1</v>
@@ -50298,7 +50298,7 @@
         <v>42</v>
       </c>
       <c r="F263" t="n">
-        <v>501</v>
+        <v>3906</v>
       </c>
       <c r="G263" t="inlineStr">
         <is>
@@ -50309,16 +50309,16 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>yfinance/XLY.csv</t>
+          <t>marches/fx/EURCHF.csv</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="C264" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D264" t="n">
         <v>1</v>
@@ -50327,7 +50327,7 @@
         <v>42</v>
       </c>
       <c r="F264" t="n">
-        <v>501</v>
+        <v>3907</v>
       </c>
       <c r="G264" t="inlineStr">
         <is>
@@ -50343,11 +50343,11 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="C265" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D265" t="n">
         <v>1</v>
@@ -50367,16 +50367,16 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>marches/fx/EURUSD.csv</t>
+          <t>marches/fx/EURJPY.csv</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="C266" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D266" t="n">
         <v>1</v>
@@ -50385,7 +50385,7 @@
         <v>42</v>
       </c>
       <c r="F266" t="n">
-        <v>3906</v>
+        <v>3909</v>
       </c>
       <c r="G266" t="inlineStr">
         <is>
@@ -50396,7 +50396,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>marches/fx/AUDJPY.csv</t>
+          <t>marches/fx/EURUSD.csv</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
@@ -50414,7 +50414,7 @@
         <v>42</v>
       </c>
       <c r="F267" t="n">
-        <v>3910</v>
+        <v>3906</v>
       </c>
       <c r="G267" t="inlineStr">
         <is>
@@ -50425,7 +50425,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>marches/fx/AUDUSD.csv</t>
+          <t>marches/fx/GBPUSD.csv</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
@@ -50443,7 +50443,7 @@
         <v>42</v>
       </c>
       <c r="F268" t="n">
-        <v>3906</v>
+        <v>3907</v>
       </c>
       <c r="G268" t="inlineStr">
         <is>
@@ -50454,7 +50454,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>marches/fx/GBPUSD.csv</t>
+          <t>marches/fx/NZDUSD.csv</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
@@ -50483,7 +50483,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>marches/fx/NZDUSD.csv</t>
+          <t>marches/fx/USDCAD.csv</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
@@ -50501,7 +50501,7 @@
         <v>42</v>
       </c>
       <c r="F270" t="n">
-        <v>3907</v>
+        <v>3906</v>
       </c>
       <c r="G270" t="inlineStr">
         <is>
@@ -50512,7 +50512,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>marches/fx/USDCAD.csv</t>
+          <t>marches/fx/USDCHF.csv</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
@@ -50530,7 +50530,7 @@
         <v>42</v>
       </c>
       <c r="F271" t="n">
-        <v>3906</v>
+        <v>3904</v>
       </c>
       <c r="G271" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-28T00:09Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-27 21:44 UTC</t>
+          <t>Genere le 2026-09-28 00:09 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-27 21:44 UTC</t>
+          <t>Rapport global — 2026-09-28 00:09 UTC</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>**Matieres premieres macro** — ratio cuivre/or stable -- pas de signal net sur la croissance (+4.4% sur 3 mois). Brent 97.4$ (+35.4% sur 3 mois, +40.4% sur 12 mois), gaz -0.2% sur 3 mois, ecart Brent-WTI +5.0$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-25)_</t>
+          <t>**Matieres premieres macro** — ratio cuivre/or stable -- pas de signal net sur la croissance (+4.7% sur 3 mois). Brent 98.7$ (+37.0% sur 3 mois, +40.7% sur 12 mois), gaz -3.6% sur 3 mois, ecart Brent-WTI +5.2$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-27)_</t>
         </is>
       </c>
     </row>
@@ -12755,7 +12755,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -37294,10 +37294,10 @@
         <v>1.113</v>
       </c>
       <c r="D8" t="n">
-        <v>0.314</v>
+        <v>0.355</v>
       </c>
       <c r="E8" t="n">
-        <v>9.000000000000001e-05</v>
+        <v>1e-05</v>
       </c>
       <c r="F8" t="n">
         <v>150</v>
@@ -37323,10 +37323,10 @@
         <v>-1.549</v>
       </c>
       <c r="D9" t="n">
-        <v>0.343</v>
+        <v>0.355</v>
       </c>
       <c r="E9" t="n">
-        <v>1e-05</v>
+        <v>0</v>
       </c>
       <c r="F9" t="n">
         <v>158</v>
@@ -42720,7 +42720,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D2" t="n">
         <v>91.5</v>
@@ -42749,7 +42749,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D3" t="n">
         <v>91.5</v>
@@ -42778,7 +42778,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D4" t="n">
         <v>91.5</v>
@@ -42807,7 +42807,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D5" t="n">
         <v>91.5</v>
@@ -42836,7 +42836,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D6" t="n">
         <v>91.5</v>
@@ -42865,7 +42865,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D7" t="n">
         <v>91.5</v>
@@ -42894,7 +42894,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D8" t="n">
         <v>91.5</v>
@@ -42923,7 +42923,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D9" t="n">
         <v>91.5</v>
@@ -42952,7 +42952,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D10" t="n">
         <v>91.5</v>
@@ -42981,7 +42981,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D11" t="n">
         <v>91.5</v>
@@ -43010,7 +43010,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D12" t="n">
         <v>91.5</v>
@@ -43039,7 +43039,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D13" t="n">
         <v>91.5</v>
@@ -43068,7 +43068,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D14" t="n">
         <v>91.5</v>
@@ -43097,7 +43097,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D15" t="n">
         <v>91.5</v>
@@ -43126,7 +43126,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D16" t="n">
         <v>92</v>
@@ -43155,7 +43155,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D17" t="n">
         <v>91.5</v>
@@ -43184,7 +43184,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D18" t="n">
         <v>91.5</v>
@@ -43213,7 +43213,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D19" t="n">
         <v>91.5</v>
@@ -43242,7 +43242,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D20" t="n">
         <v>91.5</v>
@@ -43271,7 +43271,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D21" t="n">
         <v>91.5</v>
@@ -43300,7 +43300,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D22" t="n">
         <v>91.5</v>
@@ -43329,7 +43329,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D23" t="n">
         <v>91.5</v>
@@ -43358,7 +43358,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D24" t="n">
         <v>91.5</v>
@@ -43387,7 +43387,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D25" t="n">
         <v>91</v>
@@ -43416,7 +43416,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D26" t="n">
         <v>31</v>
@@ -43445,7 +43445,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D27" t="n">
         <v>31</v>
@@ -43474,7 +43474,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D28" t="n">
         <v>31</v>
@@ -43503,7 +43503,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D29" t="n">
         <v>31</v>
@@ -43532,7 +43532,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D30" t="n">
         <v>31</v>
@@ -43561,7 +43561,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D31" t="n">
         <v>31</v>
@@ -43590,7 +43590,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D32" t="n">
         <v>31</v>
@@ -43619,7 +43619,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D33" t="n">
         <v>31</v>
@@ -43648,7 +43648,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D34" t="n">
         <v>31</v>
@@ -43677,7 +43677,7 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D35" t="n">
         <v>31</v>
@@ -43706,7 +43706,7 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D36" t="n">
         <v>31</v>
@@ -43735,7 +43735,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D37" t="n">
         <v>31</v>
@@ -43764,7 +43764,7 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D38" t="n">
         <v>31</v>
@@ -43793,7 +43793,7 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D39" t="n">
         <v>31</v>
@@ -43822,7 +43822,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D40" t="n">
         <v>31</v>
@@ -43851,7 +43851,7 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D41" t="n">
         <v>31</v>
@@ -43880,7 +43880,7 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D42" t="n">
         <v>31</v>
@@ -43909,7 +43909,7 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D43" t="n">
         <v>31</v>
@@ -43938,7 +43938,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D44" t="n">
         <v>31</v>
@@ -43967,7 +43967,7 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D45" t="n">
         <v>31</v>
@@ -43996,7 +43996,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D46" t="n">
         <v>31</v>
@@ -44025,7 +44025,7 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D47" t="n">
         <v>31</v>
@@ -44054,7 +44054,7 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D48" t="n">
         <v>31</v>
@@ -44083,7 +44083,7 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D49" t="n">
         <v>31</v>
@@ -44112,7 +44112,7 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D50" t="n">
         <v>31</v>
@@ -44141,7 +44141,7 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D51" t="n">
         <v>31</v>
@@ -44170,7 +44170,7 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D52" t="n">
         <v>31</v>
@@ -44199,7 +44199,7 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D53" t="n">
         <v>31</v>
@@ -44228,7 +44228,7 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D54" t="n">
         <v>31</v>
@@ -44257,7 +44257,7 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D55" t="n">
         <v>31</v>
@@ -44286,7 +44286,7 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D56" t="n">
         <v>31</v>
@@ -44315,7 +44315,7 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D57" t="n">
         <v>31</v>
@@ -44344,7 +44344,7 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D58" t="n">
         <v>31</v>
@@ -44373,7 +44373,7 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D59" t="n">
         <v>31</v>
@@ -44402,7 +44402,7 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D60" t="n">
         <v>31</v>
@@ -44431,7 +44431,7 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D61" t="n">
         <v>31</v>
@@ -44460,7 +44460,7 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D62" t="n">
         <v>31</v>
@@ -44489,7 +44489,7 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D63" t="n">
         <v>31</v>
@@ -44518,7 +44518,7 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D64" t="n">
         <v>31</v>
@@ -44547,7 +44547,7 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D65" t="n">
         <v>31</v>
@@ -44576,7 +44576,7 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D66" t="n">
         <v>31</v>
@@ -44605,7 +44605,7 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D67" t="n">
         <v>31</v>
@@ -44634,7 +44634,7 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D68" t="n">
         <v>31</v>
@@ -44663,7 +44663,7 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D69" t="n">
         <v>31</v>
@@ -44692,7 +44692,7 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D70" t="n">
         <v>31</v>
@@ -44721,7 +44721,7 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D71" t="n">
         <v>31</v>
@@ -44750,7 +44750,7 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D72" t="n">
         <v>31</v>
@@ -44779,7 +44779,7 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D73" t="n">
         <v>31</v>
@@ -44808,7 +44808,7 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D74" t="n">
         <v>31</v>
@@ -44837,7 +44837,7 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D75" t="n">
         <v>31</v>
@@ -44866,7 +44866,7 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D76" t="n">
         <v>31</v>
@@ -44895,7 +44895,7 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D77" t="n">
         <v>31</v>
@@ -44924,7 +44924,7 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D78" t="n">
         <v>31</v>
@@ -44953,7 +44953,7 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D79" t="n">
         <v>31</v>
@@ -44982,7 +44982,7 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D80" t="n">
         <v>31</v>
@@ -45011,7 +45011,7 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D81" t="n">
         <v>31</v>
@@ -45040,7 +45040,7 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D82" t="n">
         <v>31</v>
@@ -45069,7 +45069,7 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D83" t="n">
         <v>31</v>
@@ -45098,7 +45098,7 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D84" t="n">
         <v>31</v>
@@ -45127,7 +45127,7 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D85" t="n">
         <v>31</v>
@@ -45156,7 +45156,7 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D86" t="n">
         <v>31</v>
@@ -45185,7 +45185,7 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D87" t="n">
         <v>31</v>
@@ -45214,7 +45214,7 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D88" t="n">
         <v>31</v>
@@ -45243,7 +45243,7 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D89" t="n">
         <v>31</v>
@@ -45272,7 +45272,7 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D90" t="n">
         <v>31</v>
@@ -45301,7 +45301,7 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D91" t="n">
         <v>31</v>
@@ -45330,7 +45330,7 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D92" t="n">
         <v>31</v>
@@ -45359,7 +45359,7 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D93" t="n">
         <v>31</v>
@@ -45388,7 +45388,7 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D94" t="n">
         <v>31</v>
@@ -45417,7 +45417,7 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D95" t="n">
         <v>1</v>
@@ -45446,7 +45446,7 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D96" t="n">
         <v>1</v>
@@ -45475,7 +45475,7 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D97" t="n">
         <v>1</v>
@@ -45504,7 +45504,7 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D98" t="n">
         <v>1</v>
@@ -45533,7 +45533,7 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D99" t="n">
         <v>1</v>
@@ -45562,7 +45562,7 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D100" t="n">
         <v>31</v>
@@ -45591,7 +45591,7 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D101" t="n">
         <v>31</v>
@@ -45620,7 +45620,7 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D102" t="n">
         <v>7</v>
@@ -45649,7 +45649,7 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D103" t="n">
         <v>7</v>
@@ -45678,7 +45678,7 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D104" t="n">
         <v>1</v>
@@ -45707,7 +45707,7 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D105" t="n">
         <v>7</v>
@@ -45736,7 +45736,7 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D106" t="n">
         <v>1</v>
@@ -45765,7 +45765,7 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D107" t="n">
         <v>1</v>
@@ -45794,7 +45794,7 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D108" t="n">
         <v>7</v>
@@ -45823,7 +45823,7 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D109" t="n">
         <v>1</v>
@@ -45852,7 +45852,7 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D110" t="n">
         <v>1</v>
@@ -45881,7 +45881,7 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D111" t="n">
         <v>1</v>
@@ -45910,7 +45910,7 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D112" t="n">
         <v>1</v>
@@ -45939,7 +45939,7 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D113" t="n">
         <v>1</v>
@@ -45968,7 +45968,7 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D114" t="n">
         <v>1</v>
@@ -45997,7 +45997,7 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D115" t="n">
         <v>1</v>
@@ -46026,7 +46026,7 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D116" t="n">
         <v>1</v>
@@ -46055,7 +46055,7 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D117" t="n">
         <v>7</v>
@@ -46084,7 +46084,7 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D118" t="n">
         <v>7</v>
@@ -46113,7 +46113,7 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D119" t="n">
         <v>7</v>
@@ -46142,7 +46142,7 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D120" t="n">
         <v>7</v>
@@ -46171,7 +46171,7 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D121" t="n">
         <v>7</v>
@@ -46200,7 +46200,7 @@
         </is>
       </c>
       <c r="C122" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D122" t="n">
         <v>7</v>
@@ -46229,7 +46229,7 @@
         </is>
       </c>
       <c r="C123" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D123" t="n">
         <v>7</v>
@@ -46258,7 +46258,7 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D124" t="n">
         <v>7</v>
@@ -46287,7 +46287,7 @@
         </is>
       </c>
       <c r="C125" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D125" t="n">
         <v>7</v>
@@ -46316,7 +46316,7 @@
         </is>
       </c>
       <c r="C126" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D126" t="n">
         <v>7</v>
@@ -46345,7 +46345,7 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D127" t="n">
         <v>7</v>
@@ -46374,7 +46374,7 @@
         </is>
       </c>
       <c r="C128" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D128" t="n">
         <v>7</v>
@@ -46403,7 +46403,7 @@
         </is>
       </c>
       <c r="C129" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D129" t="n">
         <v>7</v>
@@ -46432,7 +46432,7 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D130" t="n">
         <v>7</v>
@@ -46461,7 +46461,7 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D131" t="n">
         <v>7</v>
@@ -46490,7 +46490,7 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D132" t="n">
         <v>7</v>
@@ -46519,7 +46519,7 @@
         </is>
       </c>
       <c r="C133" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D133" t="n">
         <v>7</v>
@@ -46548,7 +46548,7 @@
         </is>
       </c>
       <c r="C134" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D134" t="n">
         <v>7</v>
@@ -46577,7 +46577,7 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D135" t="n">
         <v>7</v>
@@ -46606,7 +46606,7 @@
         </is>
       </c>
       <c r="C136" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D136" t="n">
         <v>7</v>
@@ -46635,7 +46635,7 @@
         </is>
       </c>
       <c r="C137" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D137" t="n">
         <v>7</v>
@@ -46664,7 +46664,7 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D138" t="n">
         <v>7</v>
@@ -46693,7 +46693,7 @@
         </is>
       </c>
       <c r="C139" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D139" t="n">
         <v>7</v>
@@ -46722,7 +46722,7 @@
         </is>
       </c>
       <c r="C140" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D140" t="n">
         <v>7</v>
@@ -46751,7 +46751,7 @@
         </is>
       </c>
       <c r="C141" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D141" t="n">
         <v>7</v>
@@ -46780,7 +46780,7 @@
         </is>
       </c>
       <c r="C142" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D142" t="n">
         <v>7</v>
@@ -46809,7 +46809,7 @@
         </is>
       </c>
       <c r="C143" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D143" t="n">
         <v>7</v>
@@ -46838,7 +46838,7 @@
         </is>
       </c>
       <c r="C144" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D144" t="n">
         <v>7</v>
@@ -46867,7 +46867,7 @@
         </is>
       </c>
       <c r="C145" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D145" t="n">
         <v>7</v>
@@ -46896,7 +46896,7 @@
         </is>
       </c>
       <c r="C146" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D146" t="n">
         <v>7</v>
@@ -46925,7 +46925,7 @@
         </is>
       </c>
       <c r="C147" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D147" t="n">
         <v>7</v>
@@ -46954,7 +46954,7 @@
         </is>
       </c>
       <c r="C148" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D148" t="n">
         <v>7</v>
@@ -46983,7 +46983,7 @@
         </is>
       </c>
       <c r="C149" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D149" t="n">
         <v>7</v>
@@ -47012,7 +47012,7 @@
         </is>
       </c>
       <c r="C150" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D150" t="n">
         <v>7</v>
@@ -47041,7 +47041,7 @@
         </is>
       </c>
       <c r="C151" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D151" t="n">
         <v>7</v>
@@ -47070,7 +47070,7 @@
         </is>
       </c>
       <c r="C152" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D152" t="n">
         <v>7</v>
@@ -47099,7 +47099,7 @@
         </is>
       </c>
       <c r="C153" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D153" t="n">
         <v>7</v>
@@ -47128,7 +47128,7 @@
         </is>
       </c>
       <c r="C154" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D154" t="n">
         <v>7</v>
@@ -47157,7 +47157,7 @@
         </is>
       </c>
       <c r="C155" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D155" t="n">
         <v>7</v>
@@ -47186,7 +47186,7 @@
         </is>
       </c>
       <c r="C156" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D156" t="n">
         <v>7</v>
@@ -47215,7 +47215,7 @@
         </is>
       </c>
       <c r="C157" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D157" t="n">
         <v>7</v>
@@ -47244,7 +47244,7 @@
         </is>
       </c>
       <c r="C158" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D158" t="n">
         <v>7</v>
@@ -47273,7 +47273,7 @@
         </is>
       </c>
       <c r="C159" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D159" t="n">
         <v>7</v>
@@ -47302,7 +47302,7 @@
         </is>
       </c>
       <c r="C160" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D160" t="n">
         <v>7</v>
@@ -47331,7 +47331,7 @@
         </is>
       </c>
       <c r="C161" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D161" t="n">
         <v>7</v>
@@ -47360,7 +47360,7 @@
         </is>
       </c>
       <c r="C162" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D162" t="n">
         <v>7</v>
@@ -47389,7 +47389,7 @@
         </is>
       </c>
       <c r="C163" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D163" t="n">
         <v>7</v>
@@ -47418,7 +47418,7 @@
         </is>
       </c>
       <c r="C164" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D164" t="n">
         <v>7</v>
@@ -47447,7 +47447,7 @@
         </is>
       </c>
       <c r="C165" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D165" t="n">
         <v>7</v>
@@ -47476,7 +47476,7 @@
         </is>
       </c>
       <c r="C166" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D166" t="n">
         <v>7</v>
@@ -47505,7 +47505,7 @@
         </is>
       </c>
       <c r="C167" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D167" t="n">
         <v>7</v>
@@ -47534,7 +47534,7 @@
         </is>
       </c>
       <c r="C168" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D168" t="n">
         <v>7</v>
@@ -47563,7 +47563,7 @@
         </is>
       </c>
       <c r="C169" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D169" t="n">
         <v>7</v>
@@ -47592,7 +47592,7 @@
         </is>
       </c>
       <c r="C170" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D170" t="n">
         <v>7</v>
@@ -47621,7 +47621,7 @@
         </is>
       </c>
       <c r="C171" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D171" t="n">
         <v>7</v>
@@ -47650,7 +47650,7 @@
         </is>
       </c>
       <c r="C172" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D172" t="n">
         <v>7</v>
@@ -47679,7 +47679,7 @@
         </is>
       </c>
       <c r="C173" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D173" t="n">
         <v>7</v>
@@ -47708,7 +47708,7 @@
         </is>
       </c>
       <c r="C174" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D174" t="n">
         <v>7</v>
@@ -47737,7 +47737,7 @@
         </is>
       </c>
       <c r="C175" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D175" t="n">
         <v>1</v>
@@ -47766,7 +47766,7 @@
         </is>
       </c>
       <c r="C176" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D176" t="n">
         <v>7</v>
@@ -47795,7 +47795,7 @@
         </is>
       </c>
       <c r="C177" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D177" t="n">
         <v>7</v>
@@ -47824,7 +47824,7 @@
         </is>
       </c>
       <c r="C178" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D178" t="n">
         <v>7</v>
@@ -47853,7 +47853,7 @@
         </is>
       </c>
       <c r="C179" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D179" t="n">
         <v>7</v>
@@ -47882,7 +47882,7 @@
         </is>
       </c>
       <c r="C180" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D180" t="n">
         <v>7</v>
@@ -47911,7 +47911,7 @@
         </is>
       </c>
       <c r="C181" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D181" t="n">
         <v>7</v>
@@ -47940,7 +47940,7 @@
         </is>
       </c>
       <c r="C182" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D182" t="n">
         <v>7</v>
@@ -47969,7 +47969,7 @@
         </is>
       </c>
       <c r="C183" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D183" t="n">
         <v>7</v>
@@ -47998,7 +47998,7 @@
         </is>
       </c>
       <c r="C184" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D184" t="n">
         <v>1</v>
@@ -48007,7 +48007,7 @@
         <v>42</v>
       </c>
       <c r="F184" t="n">
-        <v>3683</v>
+        <v>3680</v>
       </c>
       <c r="G184" t="inlineStr">
         <is>
@@ -48027,7 +48027,7 @@
         </is>
       </c>
       <c r="C185" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D185" t="n">
         <v>1</v>
@@ -48056,7 +48056,7 @@
         </is>
       </c>
       <c r="C186" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D186" t="n">
         <v>1</v>
@@ -48085,7 +48085,7 @@
         </is>
       </c>
       <c r="C187" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D187" t="n">
         <v>1</v>
@@ -48114,7 +48114,7 @@
         </is>
       </c>
       <c r="C188" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D188" t="n">
         <v>1</v>
@@ -48143,7 +48143,7 @@
         </is>
       </c>
       <c r="C189" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D189" t="n">
         <v>1</v>
@@ -48172,7 +48172,7 @@
         </is>
       </c>
       <c r="C190" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D190" t="n">
         <v>1</v>
@@ -48201,7 +48201,7 @@
         </is>
       </c>
       <c r="C191" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D191" t="n">
         <v>1</v>
@@ -48230,7 +48230,7 @@
         </is>
       </c>
       <c r="C192" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D192" t="n">
         <v>1</v>
@@ -48259,7 +48259,7 @@
         </is>
       </c>
       <c r="C193" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D193" t="n">
         <v>1</v>
@@ -48288,7 +48288,7 @@
         </is>
       </c>
       <c r="C194" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D194" t="n">
         <v>1</v>
@@ -48317,7 +48317,7 @@
         </is>
       </c>
       <c r="C195" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D195" t="n">
         <v>1</v>
@@ -48346,7 +48346,7 @@
         </is>
       </c>
       <c r="C196" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D196" t="n">
         <v>1</v>
@@ -48375,7 +48375,7 @@
         </is>
       </c>
       <c r="C197" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D197" t="n">
         <v>1</v>
@@ -48404,7 +48404,7 @@
         </is>
       </c>
       <c r="C198" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D198" t="n">
         <v>1</v>
@@ -48433,7 +48433,7 @@
         </is>
       </c>
       <c r="C199" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D199" t="n">
         <v>1</v>
@@ -48462,7 +48462,7 @@
         </is>
       </c>
       <c r="C200" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D200" t="n">
         <v>1</v>
@@ -48491,7 +48491,7 @@
         </is>
       </c>
       <c r="C201" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D201" t="n">
         <v>1</v>
@@ -48520,7 +48520,7 @@
         </is>
       </c>
       <c r="C202" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D202" t="n">
         <v>1</v>
@@ -48549,7 +48549,7 @@
         </is>
       </c>
       <c r="C203" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D203" t="n">
         <v>1</v>
@@ -48578,7 +48578,7 @@
         </is>
       </c>
       <c r="C204" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D204" t="n">
         <v>1</v>
@@ -48607,7 +48607,7 @@
         </is>
       </c>
       <c r="C205" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D205" t="n">
         <v>1</v>
@@ -48636,7 +48636,7 @@
         </is>
       </c>
       <c r="C206" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D206" t="n">
         <v>1</v>
@@ -48665,7 +48665,7 @@
         </is>
       </c>
       <c r="C207" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D207" t="n">
         <v>1</v>
@@ -48694,7 +48694,7 @@
         </is>
       </c>
       <c r="C208" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D208" t="n">
         <v>1</v>
@@ -48723,7 +48723,7 @@
         </is>
       </c>
       <c r="C209" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D209" t="n">
         <v>1</v>
@@ -48752,7 +48752,7 @@
         </is>
       </c>
       <c r="C210" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D210" t="n">
         <v>1</v>
@@ -48781,7 +48781,7 @@
         </is>
       </c>
       <c r="C211" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D211" t="n">
         <v>7</v>
@@ -48810,7 +48810,7 @@
         </is>
       </c>
       <c r="C212" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D212" t="n">
         <v>1</v>
@@ -48839,7 +48839,7 @@
         </is>
       </c>
       <c r="C213" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D213" t="n">
         <v>1</v>
@@ -48868,7 +48868,7 @@
         </is>
       </c>
       <c r="C214" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D214" t="n">
         <v>1</v>
@@ -48897,7 +48897,7 @@
         </is>
       </c>
       <c r="C215" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D215" t="n">
         <v>1</v>
@@ -48926,7 +48926,7 @@
         </is>
       </c>
       <c r="C216" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D216" t="n">
         <v>1</v>
@@ -48955,7 +48955,7 @@
         </is>
       </c>
       <c r="C217" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D217" t="n">
         <v>1</v>
@@ -48984,7 +48984,7 @@
         </is>
       </c>
       <c r="C218" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D218" t="n">
         <v>1</v>
@@ -49013,7 +49013,7 @@
         </is>
       </c>
       <c r="C219" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D219" t="n">
         <v>1</v>
@@ -49042,7 +49042,7 @@
         </is>
       </c>
       <c r="C220" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D220" t="n">
         <v>1</v>
@@ -49071,7 +49071,7 @@
         </is>
       </c>
       <c r="C221" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D221" t="n">
         <v>1</v>
@@ -49100,7 +49100,7 @@
         </is>
       </c>
       <c r="C222" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D222" t="n">
         <v>1</v>
@@ -49129,7 +49129,7 @@
         </is>
       </c>
       <c r="C223" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D223" t="n">
         <v>1</v>
@@ -49158,7 +49158,7 @@
         </is>
       </c>
       <c r="C224" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D224" t="n">
         <v>1</v>
@@ -49187,7 +49187,7 @@
         </is>
       </c>
       <c r="C225" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D225" t="n">
         <v>1</v>
@@ -49216,7 +49216,7 @@
         </is>
       </c>
       <c r="C226" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D226" t="n">
         <v>1</v>
@@ -49245,7 +49245,7 @@
         </is>
       </c>
       <c r="C227" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D227" t="n">
         <v>1</v>
@@ -49274,7 +49274,7 @@
         </is>
       </c>
       <c r="C228" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D228" t="n">
         <v>1</v>
@@ -49303,7 +49303,7 @@
         </is>
       </c>
       <c r="C229" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D229" t="n">
         <v>1</v>
@@ -49332,7 +49332,7 @@
         </is>
       </c>
       <c r="C230" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D230" t="n">
         <v>1</v>
@@ -49361,7 +49361,7 @@
         </is>
       </c>
       <c r="C231" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D231" t="n">
         <v>1</v>
@@ -49390,7 +49390,7 @@
         </is>
       </c>
       <c r="C232" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D232" t="n">
         <v>1</v>
@@ -49419,7 +49419,7 @@
         </is>
       </c>
       <c r="C233" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D233" t="n">
         <v>1</v>
@@ -49448,7 +49448,7 @@
         </is>
       </c>
       <c r="C234" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D234" t="n">
         <v>1</v>
@@ -49477,7 +49477,7 @@
         </is>
       </c>
       <c r="C235" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D235" t="n">
         <v>1</v>
@@ -49486,7 +49486,7 @@
         <v>42</v>
       </c>
       <c r="F235" t="n">
-        <v>3668</v>
+        <v>3666</v>
       </c>
       <c r="G235" t="inlineStr">
         <is>
@@ -49497,7 +49497,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>marches/matieres/BRENT.csv</t>
+          <t>marches/volatilite/GVZ.csv</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -49506,7 +49506,7 @@
         </is>
       </c>
       <c r="C236" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D236" t="n">
         <v>1</v>
@@ -49515,7 +49515,7 @@
         <v>42</v>
       </c>
       <c r="F236" t="n">
-        <v>3751</v>
+        <v>3772</v>
       </c>
       <c r="G236" t="inlineStr">
         <is>
@@ -49526,7 +49526,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>marches/matieres/CUIVRE.csv</t>
+          <t>marches/volatilite/MOVE.csv</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
@@ -49535,7 +49535,7 @@
         </is>
       </c>
       <c r="C237" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D237" t="n">
         <v>1</v>
@@ -49544,7 +49544,7 @@
         <v>42</v>
       </c>
       <c r="F237" t="n">
-        <v>3771</v>
+        <v>3691</v>
       </c>
       <c r="G237" t="inlineStr">
         <is>
@@ -49555,7 +49555,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>marches/matieres/GAZ_HENRY_HUB.csv</t>
+          <t>marches/volatilite/OVX.csv</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
@@ -49564,7 +49564,7 @@
         </is>
       </c>
       <c r="C238" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D238" t="n">
         <v>1</v>
@@ -49584,7 +49584,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>marches/matieres/OR.csv</t>
+          <t>marches/volatilite/VVIX.csv</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
@@ -49593,7 +49593,7 @@
         </is>
       </c>
       <c r="C239" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D239" t="n">
         <v>1</v>
@@ -49602,7 +49602,7 @@
         <v>42</v>
       </c>
       <c r="F239" t="n">
-        <v>3771</v>
+        <v>3764</v>
       </c>
       <c r="G239" t="inlineStr">
         <is>
@@ -49613,7 +49613,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>marches/matieres/WTI.csv</t>
+          <t>marches/volatilite/VXN.csv</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
@@ -49622,7 +49622,7 @@
         </is>
       </c>
       <c r="C240" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D240" t="n">
         <v>1</v>
@@ -49631,7 +49631,7 @@
         <v>42</v>
       </c>
       <c r="F240" t="n">
-        <v>3771</v>
+        <v>3772</v>
       </c>
       <c r="G240" t="inlineStr">
         <is>
@@ -49642,7 +49642,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>marches/taux_futures/FED_FUNDS_FRONT.csv</t>
+          <t>souverains/SUEDE_10A.csv</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
@@ -49651,7 +49651,7 @@
         </is>
       </c>
       <c r="C241" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D241" t="n">
         <v>1</v>
@@ -49660,7 +49660,7 @@
         <v>42</v>
       </c>
       <c r="F241" t="n">
-        <v>3772</v>
+        <v>9202</v>
       </c>
       <c r="G241" t="inlineStr">
         <is>
@@ -49671,7 +49671,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>marches/volatilite/GVZ.csv</t>
+          <t>souverains/SUEDE_2A.csv</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
@@ -49680,7 +49680,7 @@
         </is>
       </c>
       <c r="C242" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D242" t="n">
         <v>1</v>
@@ -49689,7 +49689,7 @@
         <v>42</v>
       </c>
       <c r="F242" t="n">
-        <v>3772</v>
+        <v>9202</v>
       </c>
       <c r="G242" t="inlineStr">
         <is>
@@ -49700,7 +49700,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>marches/volatilite/MOVE.csv</t>
+          <t>souverains/SUEDE_5A.csv</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
@@ -49709,7 +49709,7 @@
         </is>
       </c>
       <c r="C243" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D243" t="n">
         <v>1</v>
@@ -49718,7 +49718,7 @@
         <v>42</v>
       </c>
       <c r="F243" t="n">
-        <v>3691</v>
+        <v>9204</v>
       </c>
       <c r="G243" t="inlineStr">
         <is>
@@ -49729,7 +49729,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>marches/volatilite/OVX.csv</t>
+          <t>yfinance/SP500.csv</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -49738,7 +49738,7 @@
         </is>
       </c>
       <c r="C244" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D244" t="n">
         <v>1</v>
@@ -49747,7 +49747,7 @@
         <v>42</v>
       </c>
       <c r="F244" t="n">
-        <v>3772</v>
+        <v>7547</v>
       </c>
       <c r="G244" t="inlineStr">
         <is>
@@ -49758,7 +49758,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>marches/volatilite/VVIX.csv</t>
+          <t>yfinance/VIX.csv</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -49767,7 +49767,7 @@
         </is>
       </c>
       <c r="C245" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D245" t="n">
         <v>1</v>
@@ -49776,7 +49776,7 @@
         <v>42</v>
       </c>
       <c r="F245" t="n">
-        <v>3764</v>
+        <v>7550</v>
       </c>
       <c r="G245" t="inlineStr">
         <is>
@@ -49787,7 +49787,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>marches/volatilite/VXN.csv</t>
+          <t>yfinance/XLB.csv</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -49796,7 +49796,7 @@
         </is>
       </c>
       <c r="C246" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D246" t="n">
         <v>1</v>
@@ -49805,7 +49805,7 @@
         <v>42</v>
       </c>
       <c r="F246" t="n">
-        <v>3772</v>
+        <v>501</v>
       </c>
       <c r="G246" t="inlineStr">
         <is>
@@ -49816,7 +49816,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_10A.csv</t>
+          <t>yfinance/XLE.csv</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
@@ -49825,7 +49825,7 @@
         </is>
       </c>
       <c r="C247" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D247" t="n">
         <v>1</v>
@@ -49834,7 +49834,7 @@
         <v>42</v>
       </c>
       <c r="F247" t="n">
-        <v>9202</v>
+        <v>501</v>
       </c>
       <c r="G247" t="inlineStr">
         <is>
@@ -49845,7 +49845,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_2A.csv</t>
+          <t>yfinance/XLF.csv</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
@@ -49854,7 +49854,7 @@
         </is>
       </c>
       <c r="C248" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D248" t="n">
         <v>1</v>
@@ -49863,7 +49863,7 @@
         <v>42</v>
       </c>
       <c r="F248" t="n">
-        <v>9202</v>
+        <v>501</v>
       </c>
       <c r="G248" t="inlineStr">
         <is>
@@ -49874,7 +49874,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_5A.csv</t>
+          <t>yfinance/XLI.csv</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
@@ -49883,7 +49883,7 @@
         </is>
       </c>
       <c r="C249" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D249" t="n">
         <v>1</v>
@@ -49892,7 +49892,7 @@
         <v>42</v>
       </c>
       <c r="F249" t="n">
-        <v>9204</v>
+        <v>501</v>
       </c>
       <c r="G249" t="inlineStr">
         <is>
@@ -49903,7 +49903,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>yfinance/SP500.csv</t>
+          <t>yfinance/XLK.csv</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
@@ -49912,7 +49912,7 @@
         </is>
       </c>
       <c r="C250" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D250" t="n">
         <v>1</v>
@@ -49921,7 +49921,7 @@
         <v>42</v>
       </c>
       <c r="F250" t="n">
-        <v>7547</v>
+        <v>501</v>
       </c>
       <c r="G250" t="inlineStr">
         <is>
@@ -49932,7 +49932,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>yfinance/VIX.csv</t>
+          <t>yfinance/XLP.csv</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
@@ -49941,7 +49941,7 @@
         </is>
       </c>
       <c r="C251" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D251" t="n">
         <v>1</v>
@@ -49950,7 +49950,7 @@
         <v>42</v>
       </c>
       <c r="F251" t="n">
-        <v>7550</v>
+        <v>501</v>
       </c>
       <c r="G251" t="inlineStr">
         <is>
@@ -49961,7 +49961,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>yfinance/XLB.csv</t>
+          <t>yfinance/XLRE.csv</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -49970,7 +49970,7 @@
         </is>
       </c>
       <c r="C252" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D252" t="n">
         <v>1</v>
@@ -49990,7 +49990,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>yfinance/XLE.csv</t>
+          <t>yfinance/XLU.csv</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -49999,7 +49999,7 @@
         </is>
       </c>
       <c r="C253" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D253" t="n">
         <v>1</v>
@@ -50019,7 +50019,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>yfinance/XLF.csv</t>
+          <t>yfinance/XLV.csv</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
@@ -50028,7 +50028,7 @@
         </is>
       </c>
       <c r="C254" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D254" t="n">
         <v>1</v>
@@ -50048,7 +50048,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>yfinance/XLI.csv</t>
+          <t>yfinance/XLY.csv</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
@@ -50057,7 +50057,7 @@
         </is>
       </c>
       <c r="C255" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D255" t="n">
         <v>1</v>
@@ -50077,16 +50077,16 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>yfinance/XLK.csv</t>
+          <t>marches/fx/AUDUSD.csv</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="C256" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D256" t="n">
         <v>1</v>
@@ -50095,7 +50095,7 @@
         <v>42</v>
       </c>
       <c r="F256" t="n">
-        <v>501</v>
+        <v>3904</v>
       </c>
       <c r="G256" t="inlineStr">
         <is>
@@ -50106,16 +50106,16 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>yfinance/XLP.csv</t>
+          <t>marches/fx/EURUSD.csv</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="C257" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D257" t="n">
         <v>1</v>
@@ -50124,7 +50124,7 @@
         <v>42</v>
       </c>
       <c r="F257" t="n">
-        <v>501</v>
+        <v>3904</v>
       </c>
       <c r="G257" t="inlineStr">
         <is>
@@ -50135,16 +50135,16 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>yfinance/XLRE.csv</t>
+          <t>marches/fx/GBPUSD.csv</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="C258" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D258" t="n">
         <v>1</v>
@@ -50153,7 +50153,7 @@
         <v>42</v>
       </c>
       <c r="F258" t="n">
-        <v>501</v>
+        <v>3905</v>
       </c>
       <c r="G258" t="inlineStr">
         <is>
@@ -50164,16 +50164,16 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>yfinance/XLU.csv</t>
+          <t>marches/fx/NZDUSD.csv</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="C259" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D259" t="n">
         <v>1</v>
@@ -50182,7 +50182,7 @@
         <v>42</v>
       </c>
       <c r="F259" t="n">
-        <v>501</v>
+        <v>3905</v>
       </c>
       <c r="G259" t="inlineStr">
         <is>
@@ -50193,16 +50193,16 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>yfinance/XLV.csv</t>
+          <t>marches/fx/USDCNY.csv</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="C260" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D260" t="n">
         <v>1</v>
@@ -50211,7 +50211,7 @@
         <v>42</v>
       </c>
       <c r="F260" t="n">
-        <v>501</v>
+        <v>3904</v>
       </c>
       <c r="G260" t="inlineStr">
         <is>
@@ -50222,16 +50222,16 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>yfinance/XLY.csv</t>
+          <t>marches/matieres/BRENT.csv</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-27</t>
         </is>
       </c>
       <c r="C261" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D261" t="n">
         <v>1</v>
@@ -50240,7 +50240,7 @@
         <v>42</v>
       </c>
       <c r="F261" t="n">
-        <v>501</v>
+        <v>3752</v>
       </c>
       <c r="G261" t="inlineStr">
         <is>
@@ -50251,7 +50251,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>marches/fx/AUDJPY.csv</t>
+          <t>marches/matieres/CUIVRE.csv</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
@@ -50260,7 +50260,7 @@
         </is>
       </c>
       <c r="C262" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D262" t="n">
         <v>1</v>
@@ -50269,7 +50269,7 @@
         <v>42</v>
       </c>
       <c r="F262" t="n">
-        <v>3910</v>
+        <v>3772</v>
       </c>
       <c r="G262" t="inlineStr">
         <is>
@@ -50280,7 +50280,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>marches/fx/AUDUSD.csv</t>
+          <t>marches/matieres/GAZ_HENRY_HUB.csv</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
@@ -50289,7 +50289,7 @@
         </is>
       </c>
       <c r="C263" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D263" t="n">
         <v>1</v>
@@ -50298,7 +50298,7 @@
         <v>42</v>
       </c>
       <c r="F263" t="n">
-        <v>3906</v>
+        <v>3773</v>
       </c>
       <c r="G263" t="inlineStr">
         <is>
@@ -50309,7 +50309,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>marches/fx/EURCHF.csv</t>
+          <t>marches/matieres/OR.csv</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
@@ -50318,7 +50318,7 @@
         </is>
       </c>
       <c r="C264" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D264" t="n">
         <v>1</v>
@@ -50327,7 +50327,7 @@
         <v>42</v>
       </c>
       <c r="F264" t="n">
-        <v>3907</v>
+        <v>3772</v>
       </c>
       <c r="G264" t="inlineStr">
         <is>
@@ -50338,7 +50338,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>marches/fx/EURGBP.csv</t>
+          <t>marches/matieres/WTI.csv</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
@@ -50347,7 +50347,7 @@
         </is>
       </c>
       <c r="C265" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D265" t="n">
         <v>1</v>
@@ -50356,7 +50356,7 @@
         <v>42</v>
       </c>
       <c r="F265" t="n">
-        <v>3909</v>
+        <v>3772</v>
       </c>
       <c r="G265" t="inlineStr">
         <is>
@@ -50367,7 +50367,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>marches/fx/EURJPY.csv</t>
+          <t>marches/taux_futures/FED_FUNDS_FRONT.csv</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
@@ -50376,7 +50376,7 @@
         </is>
       </c>
       <c r="C266" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D266" t="n">
         <v>1</v>
@@ -50385,7 +50385,7 @@
         <v>42</v>
       </c>
       <c r="F266" t="n">
-        <v>3909</v>
+        <v>3773</v>
       </c>
       <c r="G266" t="inlineStr">
         <is>
@@ -50396,12 +50396,12 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>marches/fx/EURUSD.csv</t>
+          <t>marches/fx/AUDJPY.csv</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -50414,7 +50414,7 @@
         <v>42</v>
       </c>
       <c r="F267" t="n">
-        <v>3906</v>
+        <v>3908</v>
       </c>
       <c r="G267" t="inlineStr">
         <is>
@@ -50425,12 +50425,12 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>marches/fx/GBPUSD.csv</t>
+          <t>marches/fx/EURCHF.csv</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -50443,7 +50443,7 @@
         <v>42</v>
       </c>
       <c r="F268" t="n">
-        <v>3907</v>
+        <v>3905</v>
       </c>
       <c r="G268" t="inlineStr">
         <is>
@@ -50454,12 +50454,12 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>marches/fx/NZDUSD.csv</t>
+          <t>marches/fx/EURGBP.csv</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -50483,12 +50483,12 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>marches/fx/USDCAD.csv</t>
+          <t>marches/fx/EURJPY.csv</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -50501,7 +50501,7 @@
         <v>42</v>
       </c>
       <c r="F270" t="n">
-        <v>3906</v>
+        <v>3907</v>
       </c>
       <c r="G270" t="inlineStr">
         <is>
@@ -50512,12 +50512,12 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>marches/fx/USDCHF.csv</t>
+          <t>marches/fx/USDCAD.csv</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C271" t="n">
@@ -50541,12 +50541,12 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>marches/fx/USDCNY.csv</t>
+          <t>marches/fx/USDCHF.csv</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C272" t="n">
@@ -50559,7 +50559,7 @@
         <v>42</v>
       </c>
       <c r="F272" t="n">
-        <v>3906</v>
+        <v>3902</v>
       </c>
       <c r="G272" t="inlineStr">
         <is>
@@ -50575,7 +50575,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -50588,7 +50588,7 @@
         <v>42</v>
       </c>
       <c r="F273" t="n">
-        <v>3907</v>
+        <v>3905</v>
       </c>
       <c r="G273" t="inlineStr">
         <is>
@@ -50604,7 +50604,7 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C274" t="n">
@@ -50617,7 +50617,7 @@
         <v>42</v>
       </c>
       <c r="F274" t="n">
-        <v>3906</v>
+        <v>3904</v>
       </c>
       <c r="G274" t="inlineStr">
         <is>
@@ -50633,7 +50633,7 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -50646,7 +50646,7 @@
         <v>42</v>
       </c>
       <c r="F275" t="n">
-        <v>3907</v>
+        <v>3905</v>
       </c>
       <c r="G275" t="inlineStr">
         <is>
@@ -50662,7 +50662,7 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C276" t="n">
@@ -50675,7 +50675,7 @@
         <v>42</v>
       </c>
       <c r="F276" t="n">
-        <v>3907</v>
+        <v>3905</v>
       </c>
       <c r="G276" t="inlineStr">
         <is>
@@ -50695,7 +50695,7 @@
         </is>
       </c>
       <c r="C277" t="n">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="D277" t="n">
         <v>2</v>
@@ -50724,7 +50724,7 @@
         </is>
       </c>
       <c r="C278" t="n">
-        <v>-436</v>
+        <v>-435</v>
       </c>
       <c r="D278" t="n">
         <v>42</v>
@@ -54021,7 +54021,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -54298,6 +54298,34 @@
       </c>
       <c r="H9" t="n">
         <v>5.03</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0.001569</v>
+      </c>
+      <c r="C10" t="n">
+        <v>4.67</v>
+      </c>
+      <c r="D10" t="n">
+        <v>98.66</v>
+      </c>
+      <c r="E10" t="n">
+        <v>37.05</v>
+      </c>
+      <c r="F10" t="n">
+        <v>40.68</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-3.56</v>
+      </c>
+      <c r="H10" t="n">
+        <v>5.23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-28T05:20Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-28 00:09 UTC</t>
+          <t>Genere le 2026-09-28 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-28 00:09 UTC</t>
+          <t>Rapport global — 2026-09-28 05:20 UTC</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>**Matieres premieres macro** — ratio cuivre/or stable -- pas de signal net sur la croissance (+4.7% sur 3 mois). Brent 98.7$ (+37.0% sur 3 mois, +40.7% sur 12 mois), gaz -3.6% sur 3 mois, ecart Brent-WTI +5.2$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-27)_</t>
+          <t>**Matieres premieres macro** — ratio cuivre/or stable -- pas de signal net sur la croissance (+4.6% sur 3 mois). Brent 99.2$ (+35.6% sur 3 mois, +41.4% sur 12 mois), gaz -2.0% sur 3 mois, ecart Brent-WTI +5.1$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -960,7 +960,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>**Indices mondiaux** — 7 indices (devise locale) : Coree (KOSPI) +103.1% en tete sur 12 mois, Hong Kong (Hang Seng) -7.5% en queue -- ecart tres large entre blocs sur 12 mois (111pt) -- les cycles economiques ou les flux divergent nettement. ROTATION en cours : Coree (KOSPI) mene sur 12 mois mais Hong Kong (Hang Seng) a repris la tete sur 3 mois _(observation : 2026-09-25)_</t>
+          <t>**Indices mondiaux** — 7 indices (devise locale) : Coree (KOSPI) +104.5% en tete sur 12 mois, Hong Kong (Hang Seng) -5.6% en queue -- ecart tres large entre blocs sur 12 mois (110pt) -- les cycles economiques ou les flux divergent nettement. ROTATION en cours : Coree (KOSPI) mene sur 12 mois mais Hong Kong (Hang Seng) a repris la tete sur 3 mois _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1240,7 +1240,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.3769116249569233 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.05237241130035915 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-25)_</t>
+          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.3769116249569233 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.052372411300360217 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
@@ -47989,7 +47989,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>marches/indices/KOSPI.csv</t>
+          <t>souverains/AUSTRALIE_10A.csv</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -48007,7 +48007,7 @@
         <v>42</v>
       </c>
       <c r="F184" t="n">
-        <v>3680</v>
+        <v>3361</v>
       </c>
       <c r="G184" t="inlineStr">
         <is>
@@ -48018,7 +48018,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>souverains/AUSTRALIE_10A.csv</t>
+          <t>souverains/AUSTRALIE_2A.csv</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -48036,7 +48036,7 @@
         <v>42</v>
       </c>
       <c r="F185" t="n">
-        <v>3361</v>
+        <v>3283</v>
       </c>
       <c r="G185" t="inlineStr">
         <is>
@@ -48047,7 +48047,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>souverains/AUSTRALIE_2A.csv</t>
+          <t>souverains/AUSTRALIE_5A.csv</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -48076,7 +48076,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>souverains/AUSTRALIE_5A.csv</t>
+          <t>souverains/UK_10A.csv</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -48094,7 +48094,7 @@
         <v>42</v>
       </c>
       <c r="F187" t="n">
-        <v>3283</v>
+        <v>9282</v>
       </c>
       <c r="G187" t="inlineStr">
         <is>
@@ -48105,7 +48105,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>souverains/UK_10A.csv</t>
+          <t>souverains/UK_20A.csv</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -48123,7 +48123,7 @@
         <v>42</v>
       </c>
       <c r="F188" t="n">
-        <v>9282</v>
+        <v>6753</v>
       </c>
       <c r="G188" t="inlineStr">
         <is>
@@ -48134,7 +48134,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>souverains/UK_20A.csv</t>
+          <t>souverains/UK_5A.csv</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -48152,7 +48152,7 @@
         <v>42</v>
       </c>
       <c r="F189" t="n">
-        <v>6753</v>
+        <v>8290</v>
       </c>
       <c r="G189" t="inlineStr">
         <is>
@@ -48163,16 +48163,16 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>souverains/UK_5A.csv</t>
+          <t>fred/BAMLC0A0CM.csv</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C190" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D190" t="n">
         <v>1</v>
@@ -48181,7 +48181,7 @@
         <v>42</v>
       </c>
       <c r="F190" t="n">
-        <v>8290</v>
+        <v>795</v>
       </c>
       <c r="G190" t="inlineStr">
         <is>
@@ -48192,7 +48192,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>fred/BAMLC0A0CM.csv</t>
+          <t>fred/BAMLC0A0CMEY.csv</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -48221,7 +48221,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>fred/BAMLC0A0CMEY.csv</t>
+          <t>fred/BAMLEMCBPIOAS.csv</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -48250,7 +48250,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>fred/BAMLEMCBPIOAS.csv</t>
+          <t>fred/BAMLEMFSFCRPIOAS.csv</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -48279,7 +48279,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>fred/BAMLEMFSFCRPIOAS.csv</t>
+          <t>fred/BAMLEMHBHYCRPIOAS.csv</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -48308,7 +48308,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>fred/BAMLEMHBHYCRPIOAS.csv</t>
+          <t>fred/BAMLEMPBPUBSICRPIOAS.csv</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -48337,7 +48337,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>fred/BAMLEMPBPUBSICRPIOAS.csv</t>
+          <t>fred/BAMLH0A0HYM2.csv</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -48366,7 +48366,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>fred/BAMLH0A0HYM2.csv</t>
+          <t>fred/BAMLHE00EHYIEY.csv</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -48395,7 +48395,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>fred/BAMLHE00EHYIEY.csv</t>
+          <t>fred/BAMLHE00EHYIOAS.csv</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -48424,7 +48424,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>fred/BAMLHE00EHYIOAS.csv</t>
+          <t>fred/DFF.csv</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -48442,7 +48442,7 @@
         <v>42</v>
       </c>
       <c r="F199" t="n">
-        <v>795</v>
+        <v>3000</v>
       </c>
       <c r="G199" t="inlineStr">
         <is>
@@ -48453,7 +48453,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>fred/DFF.csv</t>
+          <t>fred/DFII10.csv</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -48482,7 +48482,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>fred/DFII10.csv</t>
+          <t>fred/DFII5.csv</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -48511,7 +48511,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>fred/DFII5.csv</t>
+          <t>fred/DGS1.csv</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -48540,7 +48540,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>fred/DGS1.csv</t>
+          <t>fred/DGS10.csv</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -48569,7 +48569,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>fred/DGS10.csv</t>
+          <t>fred/DGS1MO.csv</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
@@ -48598,7 +48598,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>fred/DGS1MO.csv</t>
+          <t>fred/DGS2.csv</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -48627,7 +48627,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>fred/DGS2.csv</t>
+          <t>fred/DGS30.csv</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -48656,7 +48656,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>fred/DGS30.csv</t>
+          <t>fred/DGS3MO.csv</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -48685,7 +48685,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>fred/DGS3MO.csv</t>
+          <t>fred/DGS5.csv</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -48714,7 +48714,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>fred/DGS5.csv</t>
+          <t>fred/DGS6MO.csv</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -48743,7 +48743,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>fred/DGS6MO.csv</t>
+          <t>fred/MORTGAGE30US.csv</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -48755,13 +48755,13 @@
         <v>4</v>
       </c>
       <c r="D210" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E210" t="n">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="F210" t="n">
-        <v>3000</v>
+        <v>2896</v>
       </c>
       <c r="G210" t="inlineStr">
         <is>
@@ -48772,7 +48772,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>fred/MORTGAGE30US.csv</t>
+          <t>souverains/CANADA_10A.csv</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
@@ -48784,13 +48784,13 @@
         <v>4</v>
       </c>
       <c r="D211" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E211" t="n">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="F211" t="n">
-        <v>2896</v>
+        <v>6435</v>
       </c>
       <c r="G211" t="inlineStr">
         <is>
@@ -48801,7 +48801,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>souverains/CANADA_10A.csv</t>
+          <t>souverains/CANADA_2A.csv</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -48819,7 +48819,7 @@
         <v>42</v>
       </c>
       <c r="F212" t="n">
-        <v>6435</v>
+        <v>6434</v>
       </c>
       <c r="G212" t="inlineStr">
         <is>
@@ -48830,7 +48830,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>souverains/CANADA_2A.csv</t>
+          <t>souverains/CANADA_5A.csv</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -48859,7 +48859,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>souverains/CANADA_5A.csv</t>
+          <t>souverains/CANADA_LONG.csv</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -48888,7 +48888,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>souverains/CANADA_LONG.csv</t>
+          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -48906,7 +48906,7 @@
         <v>42</v>
       </c>
       <c r="F215" t="n">
-        <v>6434</v>
+        <v>5638</v>
       </c>
       <c r="G215" t="inlineStr">
         <is>
@@ -48917,7 +48917,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -48946,7 +48946,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -48975,7 +48975,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -49004,7 +49004,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -49033,7 +49033,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -49062,7 +49062,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -49091,7 +49091,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -49120,7 +49120,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
+          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -49149,7 +49149,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
+          <t>tresor_us/dette_quotidienne.csv</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -49167,7 +49167,7 @@
         <v>42</v>
       </c>
       <c r="F224" t="n">
-        <v>5638</v>
+        <v>2000</v>
       </c>
       <c r="G224" t="inlineStr">
         <is>
@@ -49178,7 +49178,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>tresor_us/dette_quotidienne.csv</t>
+          <t>tresor_us/solde_tresorerie.csv</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
@@ -49196,7 +49196,7 @@
         <v>42</v>
       </c>
       <c r="F225" t="n">
-        <v>2000</v>
+        <v>500</v>
       </c>
       <c r="G225" t="inlineStr">
         <is>
@@ -49207,16 +49207,16 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>tresor_us/solde_tresorerie.csv</t>
+          <t>fred/ECBDFR.csv</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C226" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D226" t="n">
         <v>1</v>
@@ -49225,7 +49225,7 @@
         <v>42</v>
       </c>
       <c r="F226" t="n">
-        <v>500</v>
+        <v>3000</v>
       </c>
       <c r="G226" t="inlineStr">
         <is>
@@ -49236,7 +49236,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>fred/ECBDFR.csv</t>
+          <t>fred/RRPONTSYD.csv</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -49265,7 +49265,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>fred/RRPONTSYD.csv</t>
+          <t>fred/T10YIE.csv</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -49294,7 +49294,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>fred/T10YIE.csv</t>
+          <t>marches/indices/DAX.csv</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -49312,7 +49312,7 @@
         <v>42</v>
       </c>
       <c r="F229" t="n">
-        <v>3000</v>
+        <v>3803</v>
       </c>
       <c r="G229" t="inlineStr">
         <is>
@@ -49323,7 +49323,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>marches/fx/DXY.csv</t>
+          <t>marches/indices/EUROSTOXX50.csv</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -49341,7 +49341,7 @@
         <v>42</v>
       </c>
       <c r="F230" t="n">
-        <v>3772</v>
+        <v>3760</v>
       </c>
       <c r="G230" t="inlineStr">
         <is>
@@ -49352,7 +49352,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>marches/indices/DAX.csv</t>
+          <t>marches/indices/FTSE100.csv</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -49370,7 +49370,7 @@
         <v>42</v>
       </c>
       <c r="F231" t="n">
-        <v>3803</v>
+        <v>3789</v>
       </c>
       <c r="G231" t="inlineStr">
         <is>
@@ -49381,7 +49381,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>marches/indices/EUROSTOXX50.csv</t>
+          <t>marches/volatilite/GVZ.csv</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -49399,7 +49399,7 @@
         <v>42</v>
       </c>
       <c r="F232" t="n">
-        <v>3760</v>
+        <v>3772</v>
       </c>
       <c r="G232" t="inlineStr">
         <is>
@@ -49410,7 +49410,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>marches/indices/FTSE100.csv</t>
+          <t>marches/volatilite/MOVE.csv</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -49428,7 +49428,7 @@
         <v>42</v>
       </c>
       <c r="F233" t="n">
-        <v>3789</v>
+        <v>3691</v>
       </c>
       <c r="G233" t="inlineStr">
         <is>
@@ -49439,7 +49439,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>marches/indices/HANGSENG.csv</t>
+          <t>marches/volatilite/OVX.csv</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -49457,7 +49457,7 @@
         <v>42</v>
       </c>
       <c r="F234" t="n">
-        <v>3690</v>
+        <v>3772</v>
       </c>
       <c r="G234" t="inlineStr">
         <is>
@@ -49468,7 +49468,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>marches/indices/NIKKEI225.csv</t>
+          <t>marches/volatilite/VVIX.csv</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -49486,7 +49486,7 @@
         <v>42</v>
       </c>
       <c r="F235" t="n">
-        <v>3666</v>
+        <v>3764</v>
       </c>
       <c r="G235" t="inlineStr">
         <is>
@@ -49497,7 +49497,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>marches/volatilite/GVZ.csv</t>
+          <t>marches/volatilite/VXN.csv</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -49526,7 +49526,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>marches/volatilite/MOVE.csv</t>
+          <t>souverains/SUEDE_10A.csv</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
@@ -49544,7 +49544,7 @@
         <v>42</v>
       </c>
       <c r="F237" t="n">
-        <v>3691</v>
+        <v>9202</v>
       </c>
       <c r="G237" t="inlineStr">
         <is>
@@ -49555,7 +49555,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>marches/volatilite/OVX.csv</t>
+          <t>souverains/SUEDE_2A.csv</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
@@ -49573,7 +49573,7 @@
         <v>42</v>
       </c>
       <c r="F238" t="n">
-        <v>3772</v>
+        <v>9202</v>
       </c>
       <c r="G238" t="inlineStr">
         <is>
@@ -49584,7 +49584,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>marches/volatilite/VVIX.csv</t>
+          <t>souverains/SUEDE_5A.csv</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
@@ -49602,7 +49602,7 @@
         <v>42</v>
       </c>
       <c r="F239" t="n">
-        <v>3764</v>
+        <v>9204</v>
       </c>
       <c r="G239" t="inlineStr">
         <is>
@@ -49613,7 +49613,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>marches/volatilite/VXN.csv</t>
+          <t>yfinance/SP500.csv</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
@@ -49631,7 +49631,7 @@
         <v>42</v>
       </c>
       <c r="F240" t="n">
-        <v>3772</v>
+        <v>7547</v>
       </c>
       <c r="G240" t="inlineStr">
         <is>
@@ -49642,7 +49642,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_10A.csv</t>
+          <t>yfinance/VIX.csv</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
@@ -49660,7 +49660,7 @@
         <v>42</v>
       </c>
       <c r="F241" t="n">
-        <v>9202</v>
+        <v>7550</v>
       </c>
       <c r="G241" t="inlineStr">
         <is>
@@ -49671,7 +49671,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_2A.csv</t>
+          <t>yfinance/XLB.csv</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
@@ -49689,7 +49689,7 @@
         <v>42</v>
       </c>
       <c r="F242" t="n">
-        <v>9202</v>
+        <v>501</v>
       </c>
       <c r="G242" t="inlineStr">
         <is>
@@ -49700,7 +49700,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_5A.csv</t>
+          <t>yfinance/XLE.csv</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
@@ -49718,7 +49718,7 @@
         <v>42</v>
       </c>
       <c r="F243" t="n">
-        <v>9204</v>
+        <v>501</v>
       </c>
       <c r="G243" t="inlineStr">
         <is>
@@ -49729,7 +49729,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>yfinance/SP500.csv</t>
+          <t>yfinance/XLF.csv</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -49747,7 +49747,7 @@
         <v>42</v>
       </c>
       <c r="F244" t="n">
-        <v>7547</v>
+        <v>501</v>
       </c>
       <c r="G244" t="inlineStr">
         <is>
@@ -49758,7 +49758,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>yfinance/VIX.csv</t>
+          <t>yfinance/XLI.csv</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -49776,7 +49776,7 @@
         <v>42</v>
       </c>
       <c r="F245" t="n">
-        <v>7550</v>
+        <v>501</v>
       </c>
       <c r="G245" t="inlineStr">
         <is>
@@ -49787,7 +49787,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>yfinance/XLB.csv</t>
+          <t>yfinance/XLK.csv</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -49816,7 +49816,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>yfinance/XLE.csv</t>
+          <t>yfinance/XLP.csv</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
@@ -49845,7 +49845,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>yfinance/XLF.csv</t>
+          <t>yfinance/XLRE.csv</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
@@ -49874,7 +49874,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>yfinance/XLI.csv</t>
+          <t>yfinance/XLU.csv</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
@@ -49903,7 +49903,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>yfinance/XLK.csv</t>
+          <t>yfinance/XLV.csv</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
@@ -49932,7 +49932,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>yfinance/XLP.csv</t>
+          <t>yfinance/XLY.csv</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
@@ -49961,16 +49961,16 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>yfinance/XLRE.csv</t>
+          <t>marches/fx/AUDJPY.csv</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C252" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D252" t="n">
         <v>1</v>
@@ -49979,7 +49979,7 @@
         <v>42</v>
       </c>
       <c r="F252" t="n">
-        <v>501</v>
+        <v>3908</v>
       </c>
       <c r="G252" t="inlineStr">
         <is>
@@ -49990,16 +49990,16 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>yfinance/XLU.csv</t>
+          <t>marches/fx/AUDUSD.csv</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C253" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D253" t="n">
         <v>1</v>
@@ -50008,7 +50008,7 @@
         <v>42</v>
       </c>
       <c r="F253" t="n">
-        <v>501</v>
+        <v>3904</v>
       </c>
       <c r="G253" t="inlineStr">
         <is>
@@ -50019,16 +50019,16 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>yfinance/XLV.csv</t>
+          <t>marches/fx/DXY.csv</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C254" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D254" t="n">
         <v>1</v>
@@ -50037,7 +50037,7 @@
         <v>42</v>
       </c>
       <c r="F254" t="n">
-        <v>501</v>
+        <v>3772</v>
       </c>
       <c r="G254" t="inlineStr">
         <is>
@@ -50048,16 +50048,16 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>yfinance/XLY.csv</t>
+          <t>marches/fx/EURCHF.csv</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C255" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D255" t="n">
         <v>1</v>
@@ -50066,7 +50066,7 @@
         <v>42</v>
       </c>
       <c r="F255" t="n">
-        <v>501</v>
+        <v>3905</v>
       </c>
       <c r="G255" t="inlineStr">
         <is>
@@ -50077,16 +50077,16 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>marches/fx/AUDUSD.csv</t>
+          <t>marches/fx/EURGBP.csv</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C256" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D256" t="n">
         <v>1</v>
@@ -50095,7 +50095,7 @@
         <v>42</v>
       </c>
       <c r="F256" t="n">
-        <v>3904</v>
+        <v>3907</v>
       </c>
       <c r="G256" t="inlineStr">
         <is>
@@ -50106,16 +50106,16 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>marches/fx/EURUSD.csv</t>
+          <t>marches/fx/EURJPY.csv</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C257" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D257" t="n">
         <v>1</v>
@@ -50124,7 +50124,7 @@
         <v>42</v>
       </c>
       <c r="F257" t="n">
-        <v>3904</v>
+        <v>3907</v>
       </c>
       <c r="G257" t="inlineStr">
         <is>
@@ -50135,16 +50135,16 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>marches/fx/GBPUSD.csv</t>
+          <t>marches/fx/EURUSD.csv</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C258" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D258" t="n">
         <v>1</v>
@@ -50153,7 +50153,7 @@
         <v>42</v>
       </c>
       <c r="F258" t="n">
-        <v>3905</v>
+        <v>3904</v>
       </c>
       <c r="G258" t="inlineStr">
         <is>
@@ -50164,16 +50164,16 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>marches/fx/NZDUSD.csv</t>
+          <t>marches/fx/GBPUSD.csv</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C259" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D259" t="n">
         <v>1</v>
@@ -50193,16 +50193,16 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>marches/fx/USDCNY.csv</t>
+          <t>marches/fx/NZDUSD.csv</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C260" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D260" t="n">
         <v>1</v>
@@ -50211,7 +50211,7 @@
         <v>42</v>
       </c>
       <c r="F260" t="n">
-        <v>3904</v>
+        <v>3905</v>
       </c>
       <c r="G260" t="inlineStr">
         <is>
@@ -50222,16 +50222,16 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>marches/matieres/BRENT.csv</t>
+          <t>marches/fx/USDCAD.csv</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C261" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D261" t="n">
         <v>1</v>
@@ -50240,7 +50240,7 @@
         <v>42</v>
       </c>
       <c r="F261" t="n">
-        <v>3752</v>
+        <v>3904</v>
       </c>
       <c r="G261" t="inlineStr">
         <is>
@@ -50251,16 +50251,16 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>marches/matieres/CUIVRE.csv</t>
+          <t>marches/fx/USDCHF.csv</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C262" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D262" t="n">
         <v>1</v>
@@ -50269,7 +50269,7 @@
         <v>42</v>
       </c>
       <c r="F262" t="n">
-        <v>3772</v>
+        <v>3902</v>
       </c>
       <c r="G262" t="inlineStr">
         <is>
@@ -50280,16 +50280,16 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>marches/matieres/GAZ_HENRY_HUB.csv</t>
+          <t>marches/fx/USDCNY.csv</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C263" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D263" t="n">
         <v>1</v>
@@ -50298,7 +50298,7 @@
         <v>42</v>
       </c>
       <c r="F263" t="n">
-        <v>3773</v>
+        <v>3904</v>
       </c>
       <c r="G263" t="inlineStr">
         <is>
@@ -50309,16 +50309,16 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>marches/matieres/OR.csv</t>
+          <t>marches/fx/USDJPY.csv</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C264" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D264" t="n">
         <v>1</v>
@@ -50327,7 +50327,7 @@
         <v>42</v>
       </c>
       <c r="F264" t="n">
-        <v>3772</v>
+        <v>3905</v>
       </c>
       <c r="G264" t="inlineStr">
         <is>
@@ -50338,16 +50338,16 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>marches/matieres/WTI.csv</t>
+          <t>marches/fx/USDKRW.csv</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C265" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D265" t="n">
         <v>1</v>
@@ -50356,7 +50356,7 @@
         <v>42</v>
       </c>
       <c r="F265" t="n">
-        <v>3772</v>
+        <v>3904</v>
       </c>
       <c r="G265" t="inlineStr">
         <is>
@@ -50367,16 +50367,16 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>marches/taux_futures/FED_FUNDS_FRONT.csv</t>
+          <t>marches/fx/USDNOK.csv</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-09-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C266" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D266" t="n">
         <v>1</v>
@@ -50385,7 +50385,7 @@
         <v>42</v>
       </c>
       <c r="F266" t="n">
-        <v>3773</v>
+        <v>3905</v>
       </c>
       <c r="G266" t="inlineStr">
         <is>
@@ -50396,7 +50396,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>marches/fx/AUDJPY.csv</t>
+          <t>marches/fx/USDSEK.csv</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
@@ -50414,7 +50414,7 @@
         <v>42</v>
       </c>
       <c r="F267" t="n">
-        <v>3908</v>
+        <v>3905</v>
       </c>
       <c r="G267" t="inlineStr">
         <is>
@@ -50425,7 +50425,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>marches/fx/EURCHF.csv</t>
+          <t>marches/indices/HANGSENG.csv</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
@@ -50443,7 +50443,7 @@
         <v>42</v>
       </c>
       <c r="F268" t="n">
-        <v>3905</v>
+        <v>3689</v>
       </c>
       <c r="G268" t="inlineStr">
         <is>
@@ -50454,7 +50454,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>marches/fx/EURGBP.csv</t>
+          <t>marches/indices/KOSPI.csv</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
@@ -50472,7 +50472,7 @@
         <v>42</v>
       </c>
       <c r="F269" t="n">
-        <v>3907</v>
+        <v>3681</v>
       </c>
       <c r="G269" t="inlineStr">
         <is>
@@ -50483,7 +50483,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>marches/fx/EURJPY.csv</t>
+          <t>marches/indices/NIKKEI225.csv</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
@@ -50501,7 +50501,7 @@
         <v>42</v>
       </c>
       <c r="F270" t="n">
-        <v>3907</v>
+        <v>3667</v>
       </c>
       <c r="G270" t="inlineStr">
         <is>
@@ -50512,7 +50512,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>marches/fx/USDCAD.csv</t>
+          <t>marches/matieres/BRENT.csv</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
@@ -50530,7 +50530,7 @@
         <v>42</v>
       </c>
       <c r="F271" t="n">
-        <v>3904</v>
+        <v>3751</v>
       </c>
       <c r="G271" t="inlineStr">
         <is>
@@ -50541,7 +50541,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>marches/fx/USDCHF.csv</t>
+          <t>marches/matieres/CUIVRE.csv</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
@@ -50559,7 +50559,7 @@
         <v>42</v>
       </c>
       <c r="F272" t="n">
-        <v>3902</v>
+        <v>3771</v>
       </c>
       <c r="G272" t="inlineStr">
         <is>
@@ -50570,7 +50570,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>marches/fx/USDJPY.csv</t>
+          <t>marches/matieres/GAZ_HENRY_HUB.csv</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
@@ -50588,7 +50588,7 @@
         <v>42</v>
       </c>
       <c r="F273" t="n">
-        <v>3905</v>
+        <v>3772</v>
       </c>
       <c r="G273" t="inlineStr">
         <is>
@@ -50599,7 +50599,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>marches/fx/USDKRW.csv</t>
+          <t>marches/matieres/OR.csv</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
@@ -50617,7 +50617,7 @@
         <v>42</v>
       </c>
       <c r="F274" t="n">
-        <v>3904</v>
+        <v>3771</v>
       </c>
       <c r="G274" t="inlineStr">
         <is>
@@ -50628,7 +50628,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>marches/fx/USDNOK.csv</t>
+          <t>marches/matieres/WTI.csv</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
@@ -50646,7 +50646,7 @@
         <v>42</v>
       </c>
       <c r="F275" t="n">
-        <v>3905</v>
+        <v>3771</v>
       </c>
       <c r="G275" t="inlineStr">
         <is>
@@ -50657,7 +50657,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>marches/fx/USDSEK.csv</t>
+          <t>marches/taux_futures/FED_FUNDS_FRONT.csv</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
@@ -50675,7 +50675,7 @@
         <v>42</v>
       </c>
       <c r="F276" t="n">
-        <v>3905</v>
+        <v>3772</v>
       </c>
       <c r="G276" t="inlineStr">
         <is>
@@ -52135,17 +52135,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7080.92</v>
+        <v>6924.2</v>
       </c>
       <c r="D2" t="n">
-        <v>-16.41</v>
+        <v>-17.52</v>
       </c>
       <c r="E2" t="n">
-        <v>103.11</v>
+        <v>104.49</v>
       </c>
     </row>
     <row r="3">
@@ -52156,17 +52156,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>66364.2</v>
+        <v>66346.41</v>
       </c>
       <c r="D3" t="n">
-        <v>-4.32</v>
+        <v>-4.49</v>
       </c>
       <c r="E3" t="n">
-        <v>45.04</v>
+        <v>46.28</v>
       </c>
     </row>
     <row r="4">
@@ -52261,17 +52261,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>24510.09</v>
+        <v>24668.25</v>
       </c>
       <c r="D8" t="n">
-        <v>8.109999999999999</v>
+        <v>7.13</v>
       </c>
       <c r="E8" t="n">
-        <v>-7.46</v>
+        <v>-5.59</v>
       </c>
     </row>
   </sheetData>
@@ -54021,7 +54021,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -54326,6 +54326,34 @@
       </c>
       <c r="H10" t="n">
         <v>5.23</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.00158</v>
+      </c>
+      <c r="C11" t="n">
+        <v>4.62</v>
+      </c>
+      <c r="D11" t="n">
+        <v>99.17</v>
+      </c>
+      <c r="E11" t="n">
+        <v>35.57</v>
+      </c>
+      <c r="F11" t="n">
+        <v>41.41</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-1.98</v>
+      </c>
+      <c r="H11" t="n">
+        <v>5.06</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-28T05:32Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-28 05:20 UTC</t>
+          <t>Genere le 2026-09-28 05:32 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-28 05:20 UTC</t>
+          <t>Rapport global — 2026-09-28 05:32 UTC</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>**Matieres premieres macro** — ratio cuivre/or stable -- pas de signal net sur la croissance (+4.6% sur 3 mois). Brent 99.2$ (+35.6% sur 3 mois, +41.4% sur 12 mois), gaz -2.0% sur 3 mois, ecart Brent-WTI +5.1$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-28)_</t>
+          <t>**Matieres premieres macro** — ratio cuivre/or stable -- pas de signal net sur la croissance (+4.6% sur 3 mois). Brent 99.2$ (+35.7% sur 3 mois, +41.5% sur 12 mois), gaz -1.9% sur 3 mois, ecart Brent-WTI +5.1$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -960,7 +960,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>**Indices mondiaux** — 7 indices (devise locale) : Coree (KOSPI) +104.5% en tete sur 12 mois, Hong Kong (Hang Seng) -5.6% en queue -- ecart tres large entre blocs sur 12 mois (110pt) -- les cycles economiques ou les flux divergent nettement. ROTATION en cours : Coree (KOSPI) mene sur 12 mois mais Hong Kong (Hang Seng) a repris la tete sur 3 mois _(observation : 2026-09-28)_</t>
+          <t>**Indices mondiaux** — 7 indices (devise locale) : Coree (KOSPI) +105.0% en tete sur 12 mois, Hong Kong (Hang Seng) -5.5% en queue -- ecart tres large entre blocs sur 12 mois (110pt) -- les cycles economiques ou les flux divergent nettement. ROTATION en cours : Coree (KOSPI) mene sur 12 mois mais Hong Kong (Hang Seng) a repris la tete sur 3 mois _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -52139,13 +52139,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>6924.2</v>
+        <v>6942.46</v>
       </c>
       <c r="D2" t="n">
-        <v>-17.52</v>
+        <v>-17.3</v>
       </c>
       <c r="E2" t="n">
-        <v>104.49</v>
+        <v>105.03</v>
       </c>
     </row>
     <row r="3">
@@ -52160,13 +52160,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>66346.41</v>
+        <v>66308.45</v>
       </c>
       <c r="D3" t="n">
-        <v>-4.49</v>
+        <v>-4.55</v>
       </c>
       <c r="E3" t="n">
-        <v>46.28</v>
+        <v>46.2</v>
       </c>
     </row>
     <row r="4">
@@ -52265,13 +52265,13 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>24668.25</v>
+        <v>24700.5</v>
       </c>
       <c r="D8" t="n">
-        <v>7.13</v>
+        <v>7.27</v>
       </c>
       <c r="E8" t="n">
-        <v>-5.59</v>
+        <v>-5.46</v>
       </c>
     </row>
   </sheetData>
@@ -54338,19 +54338,19 @@
         <v>0.00158</v>
       </c>
       <c r="C11" t="n">
-        <v>4.62</v>
+        <v>4.63</v>
       </c>
       <c r="D11" t="n">
-        <v>99.17</v>
+        <v>99.23999999999999</v>
       </c>
       <c r="E11" t="n">
-        <v>35.57</v>
+        <v>35.67</v>
       </c>
       <c r="F11" t="n">
-        <v>41.41</v>
+        <v>41.51</v>
       </c>
       <c r="G11" t="n">
-        <v>-1.98</v>
+        <v>-1.92</v>
       </c>
       <c r="H11" t="n">
         <v>5.06</v>

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-28T11:47Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-28 05:32 UTC</t>
+          <t>Genere le 2026-09-28 11:47 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-28 05:32 UTC</t>
+          <t>Rapport global — 2026-09-28 11:47 UTC</t>
         </is>
       </c>
     </row>
@@ -792,14 +792,14 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>**Soutenabilite dette** — 8 pays. charge la plus lourde : Canada a 25.5% du revenu. taux 10 ans AU-DESSUS de l'inflation dans 5 pays -- Royaume-Uni (+2.2pt), Etats-Unis (+1.8pt), Japon (+1.0pt), Canada (+0.9pt), Zone euro (+0.8pt). Configuration ou le ratio d'endettement monte meme a budget primaire equilibre (approximation : croissance nominale reduite a l'inflation) _(observation : date non exposee)_</t>
+          <t>**Soutenabilite dette** — 8 pays. charge la plus lourde : Canada a 25.5% du revenu. taux 10 ans AU-DESSUS de l'inflation dans 5 pays -- Royaume-Uni (+2.3pt), Etats-Unis (+1.8pt), Japon (+1.0pt), Canada (+0.9pt), Zone euro (+0.9pt). Configuration ou le ratio d'endettement monte meme a budget primaire equilibre (approximation : croissance nominale reduite a l'inflation) _(observation : date non exposee)_</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>**Matieres premieres macro** — ratio cuivre/or stable -- pas de signal net sur la croissance (+4.6% sur 3 mois). Brent 99.2$ (+35.7% sur 3 mois, +41.5% sur 12 mois), gaz -1.9% sur 3 mois, ecart Brent-WTI +5.1$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-28)_</t>
+          <t>**Matieres premieres macro** — le ratio cuivre/or monte -- la croissance domine la peur (+5.0% sur 3 mois). Brent 100.4$ (+37.3% sur 3 mois, +43.2% sur 12 mois), gaz -1.9% sur 3 mois, ecart Brent-WTI +4.7$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -862,7 +862,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>**Conditions financieres** — indice conditions financieres=+0.064 (3 composantes: {'taux_directeur': 0.5985724560125544, 'courbe_inversee': 0.2531563730537784, 'vix': -0.6597998970697634}) -- conditions proches de la normale _(observation : 2026-09-24)_</t>
+          <t>**Conditions financieres** — indice conditions financieres=+0.121 (3 composantes: {'taux_directeur': 0.5985724560125544, 'courbe_inversee': 0.2531563730537784, 'vix': -0.48919720777532755}) -- conditions proches de la normale _(observation : 2026-09-24)_</t>
         </is>
       </c>
     </row>
@@ -960,7 +960,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>**Indices mondiaux** — 7 indices (devise locale) : Coree (KOSPI) +105.0% en tete sur 12 mois, Hong Kong (Hang Seng) -5.5% en queue -- ecart tres large entre blocs sur 12 mois (110pt) -- les cycles economiques ou les flux divergent nettement. ROTATION en cours : Coree (KOSPI) mene sur 12 mois mais Hong Kong (Hang Seng) a repris la tete sur 3 mois _(observation : 2026-09-28)_</t>
+          <t>**Indices mondiaux** — 7 indices (devise locale) : Coree (KOSPI) +103.5% en tete sur 12 mois, Hong Kong (Hang Seng) -5.7% en queue -- ecart tres large entre blocs sur 12 mois (109pt) -- les cycles economiques ou les flux divergent nettement. ROTATION en cours : Coree (KOSPI) mene sur 12 mois mais Hong Kong (Hang Seng) a repris la tete sur 3 mois _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1191,7 +1191,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>**Vol cross asset** — 6 mesures de volatilite : Petrole (OVX) 88e pct, Or (GVZ) 80e pct, Taux US (MOVE) 43e pct, Nasdaq (VXN) 38e pct, Vol de la vol (VVIX) 27e pct, Actions US (VIX) 21e pct -- stress LOCALISE sur Petrole (OVX), Or (GVZ) pendant que le reste ne l'est pas -- episode propre a cette classe d'actifs, pas une aversion au risque d'ensemble _(observation : 2026-09-25)_</t>
+          <t>**Vol cross asset** — 6 mesures de volatilite : Petrole (OVX) 88e pct, Or (GVZ) 80e pct, Taux US (MOVE) 43e pct, Nasdaq (VXN) 38e pct, Actions US (VIX) 34e pct, Vol de la vol (VVIX) 27e pct -- stress LOCALISE sur Petrole (OVX), Or (GVZ) pendant que le reste ne l'est pas -- episode propre a cette classe d'actifs, pas une aversion au risque d'ensemble _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1219,7 +1219,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>**Ornstein uhlenbeck vix** — VIX actuel=14.87, niveau moyen estime (mu)=20.20, demi-vie=28.8j, ecart actuel=-5.33 -- VIX actuel en-dessous de son niveau moyen de long terme _(observation : 2026-09-25)_</t>
+          <t>**Ornstein uhlenbeck vix** — VIX actuel=16.25, niveau moyen estime (mu)=20.20, demi-vie=28.8j, ecart actuel=-3.95 -- VIX actuel en-dessous de son niveau moyen de long terme _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1233,21 +1233,21 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>**Kalman niveau local** — VIX observe=14.87, filtre Kalman=14.98 (ecart-type=0.62), ratio signal/bruit=0.2051 -- le filtre lisse fortement le bruit, reagit lentement (ecart obs.-filtre=-0.11) _(observation : 2026-09-25)_</t>
+          <t>**Kalman niveau local** — VIX observe=16.25, filtre Kalman=16.06 (ecart-type=0.62), ratio signal/bruit=0.2052 -- le filtre lisse fortement le bruit, reagit lentement (ecart obs.-filtre=+0.19) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.3769116249569233 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.052372411300360217 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-25)_</t>
+          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.37012183452205605 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.05233908530492189 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>**Analyse spectrale** — 3 periodes dominantes (jours de bourse) : [2.2, 4.0, 5.3] -- cycle(s) connu(s) qui ressortent : 4.0j~hebdomadaire, 5.3j~hebdomadaire _(observation : 2026-09-25)_</t>
+          <t>**Analyse spectrale** — 3 periodes dominantes (jours de bourse) : [2.2, 3.0, 2.4] -- aucune des 3 periodes dominantes ne correspond a un cycle connu (hebdo/mensuel/trimestriel) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1317,7 +1317,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>**Qualite regime macro** — instabilite taux=0.0088, instabilite VIX=0.0679 -- score qualite du regime=-0.0383 (plus haut = regime plus stable/previsible) _(observation : 2026-09-24)_</t>
+          <t>**Qualite regime macro** — instabilite taux=0.0088, instabilite VIX=0.0686 -- score qualite du regime=-0.0387 (plus haut = regime plus stable/previsible) _(observation : 2026-09-24)_</t>
         </is>
       </c>
     </row>
@@ -1331,14 +1331,14 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>**Decomposition stl** — VIX : tendance=15.52, composante saisonniere (periode 5j)=-0.665, residu=+0.016 -- la saisonnalite explique 0.71% de la variance totale (negligeable) _(observation : 2026-09-25)_</t>
+          <t>**Decomposition stl** — VIX : tendance=15.59, composante saisonniere (periode 5j)=+0.177, residu=+0.480 -- la saisonnalite explique 0.72% de la variance totale (negligeable) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>**Ratios conditionnels regime** — Sharpe regime haut-vol=-1.107, bas-vol=2.406, global=0.423 -- meilleur en regime calme, comme attendu _(observation : 2026-09-25)_</t>
+          <t>**Ratios conditionnels regime** — Sharpe regime haut-vol=-1.107, bas-vol=2.406, global=0.422 -- meilleur en regime calme, comme attendu _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
@@ -1373,7 +1373,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>**Dependance queue** — 518/7546 jours conjointement extremes (SP500 pire 10% ET VIX pire 10%), P observee=0.0686 vs P sous independance=0.0100 -- coefficient de dependance de queue=6.86 (dependance reelle) _(observation : 2026-09-25)_</t>
+          <t>**Dependance queue** — 518/7544 jours conjointement extremes (SP500 pire 10% ET VIX pire 10%), P observee=0.0687 vs P sous independance=0.0100 -- coefficient de dependance de queue=6.87 (dependance reelle) _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
@@ -1415,7 +1415,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>**Ensemble signaux** — 7516 predictions -- momentum=0.4960, vix=0.4988, ensemble=0.4988, baseline=0.5375 -- ensemble NE BAT PAS la baseline _(observation : 2026-09-25)_</t>
+          <t>**Ensemble signaux** — 7514 predictions -- momentum=0.4959, vix=0.4988, ensemble=0.4988, baseline=0.5374 -- ensemble NE BAT PAS la baseline _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1436,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>**Regression multifeatures** — coefs (intercept=0.00029, momentum5j=-0.0325, var_vix=0.00027) -- R2 out-of-sample=0.0103 (modele bat la moyenne) _(observation : 2026-09-25)_</t>
+          <t>**Regression multifeatures** — coefs (intercept=0.00029, momentum5j=-0.0326, var_vix=0.00027) -- R2 out-of-sample=0.0102 (modele bat la moyenne) _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
@@ -1457,7 +1457,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>**Arima** — ARIMA(1,1,1) sur 100 previsions 1-jour test : RMSE=2.325 vs baseline naive MSE=5.474 -- ARIMA bat la persistance simple _(observation : 2026-09-25)_</t>
+          <t>**Arima** — ARIMA(1,1,1) sur 100 previsions 1-jour test : RMSE=2.327 vs baseline naive MSE=5.430 -- ARIMA bat la persistance simple _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1471,14 +1471,14 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>**Decision stump** — seuil appris=-1.530 (sens=False) -- accuracy stump=0.5459 vs baseline=0.5477 sur 2264 points test -- stump NE BAT PAS la baseline _(observation : 2026-09-25)_</t>
+          <t>**Decision stump** — seuil appris=-1.530 (sens=False) -- accuracy stump=0.5457 vs baseline=0.5475 sur 2263 points test -- stump NE BAT PAS la baseline _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>**Importance permutation** — R2 base=0.0103 -- importance momentum5j=0.00424, importance variation_vix=0.01648 -- VIX plus important _(observation : 2026-09-25)_</t>
+          <t>**Importance permutation** — R2 base=0.0102 -- importance momentum5j=-0.00094, importance variation_vix=0.01231 -- VIX plus important _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
@@ -4607,10 +4607,10 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>-0.159</v>
+        <v>-0.1568</v>
       </c>
       <c r="E59" t="n">
-        <v>0.9432</v>
+        <v>0.9435</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
@@ -6884,10 +6884,10 @@
         <v>5</v>
       </c>
       <c r="C13" t="n">
-        <v>0.07804</v>
+        <v>0.07636999999999999</v>
       </c>
       <c r="D13" t="n">
-        <v>0.00439</v>
+        <v>0.00433</v>
       </c>
     </row>
   </sheetData>
@@ -8063,10 +8063,10 @@
         <v>10</v>
       </c>
       <c r="C13" t="n">
-        <v>0.37691</v>
+        <v>0.37012</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.052372</v>
+        <v>-0.052339</v>
       </c>
     </row>
   </sheetData>
@@ -8230,19 +8230,19 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Vol de la vol (VVIX)</t>
+          <t>Actions US (VIX)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>87.84</v>
+        <v>16.25</v>
       </c>
       <c r="D6" t="n">
-        <v>27.3</v>
+        <v>34</v>
       </c>
       <c r="E6" t="n">
         <v>1260</v>
@@ -8256,7 +8256,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Actions US (VIX)</t>
+          <t>Vol de la vol (VVIX)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -8265,10 +8265,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>14.87</v>
+        <v>87.84</v>
       </c>
       <c r="D7" t="n">
-        <v>20.6</v>
+        <v>27.3</v>
       </c>
       <c r="E7" t="n">
         <v>1260</v>
@@ -18951,10 +18951,10 @@
         </is>
       </c>
       <c r="D119" t="n">
-        <v>-1.9682</v>
+        <v>-1.9783</v>
       </c>
       <c r="E119" t="n">
-        <v>0.545</v>
+        <v>0.5399</v>
       </c>
       <c r="F119" t="inlineStr">
         <is>
@@ -18979,10 +18979,10 @@
         </is>
       </c>
       <c r="D120" t="n">
-        <v>-2.2144</v>
+        <v>-2.213</v>
       </c>
       <c r="E120" t="n">
-        <v>0.4169</v>
+        <v>0.4177</v>
       </c>
       <c r="F120" t="inlineStr">
         <is>
@@ -22122,7 +22122,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.064</v>
+        <v>0.1208</v>
       </c>
       <c r="C13" t="n">
         <v>3</v>
@@ -22134,7 +22134,7 @@
         <v>0.2532</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.6598000000000001</v>
+        <v>-0.4892</v>
       </c>
     </row>
   </sheetData>
@@ -34634,7 +34634,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -34956,6 +34956,31 @@
       </c>
       <c r="G12" t="n">
         <v>320.82</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="C13" t="n">
+        <v>468.17</v>
+      </c>
+      <c r="D13" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" t="n">
+        <v>416.86</v>
+      </c>
+      <c r="F13" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="G13" t="n">
+        <v>372.23</v>
       </c>
     </row>
   </sheetData>
@@ -36011,13 +36036,13 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>2264</v>
+        <v>2263</v>
       </c>
       <c r="E13" t="n">
-        <v>0.5459000000000001</v>
+        <v>0.5457</v>
       </c>
       <c r="F13" t="n">
-        <v>0.5477</v>
+        <v>0.5475</v>
       </c>
     </row>
   </sheetData>
@@ -36031,7 +36056,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -36275,6 +36300,25 @@
       </c>
       <c r="E12" t="n">
         <v>0.71</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>15.593</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.177</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.72</v>
       </c>
     </row>
   </sheetData>
@@ -36772,19 +36816,19 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>7546</v>
+        <v>7544</v>
       </c>
       <c r="C13" t="n">
         <v>518</v>
       </c>
       <c r="D13" t="n">
-        <v>0.06865</v>
+        <v>0.06866</v>
       </c>
       <c r="E13" t="n">
         <v>0.01</v>
       </c>
       <c r="F13" t="n">
-        <v>6.86</v>
+        <v>6.87</v>
       </c>
     </row>
   </sheetData>
@@ -37171,11 +37215,11 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>-0.112</v>
+        <v>-0.106</v>
       </c>
       <c r="D4" t="n">
         <v>0.067</v>
@@ -37316,11 +37360,11 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>-1.549</v>
+        <v>-1.581</v>
       </c>
       <c r="D9" t="n">
         <v>0.355</v>
@@ -39241,10 +39285,10 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>7516</v>
+        <v>7514</v>
       </c>
       <c r="C13" t="n">
-        <v>0.496</v>
+        <v>0.4959</v>
       </c>
       <c r="D13" t="n">
         <v>0.4988</v>
@@ -39253,7 +39297,7 @@
         <v>0.4988</v>
       </c>
       <c r="F13" t="n">
-        <v>0.5375</v>
+        <v>0.5374</v>
       </c>
     </row>
   </sheetData>
@@ -42380,7 +42424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -42643,6 +42687,27 @@
         <v>5.4737</v>
       </c>
       <c r="E12" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>100</v>
+      </c>
+      <c r="C13" t="n">
+        <v>2.3274</v>
+      </c>
+      <c r="D13" t="n">
+        <v>5.4303</v>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>True</t>
         </is>
@@ -45640,7 +45705,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>bilans/BOE_BILAN_TOTAL.csv</t>
+          <t>bis/taux_directeurs/NO.csv</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -45652,13 +45717,13 @@
         <v>12</v>
       </c>
       <c r="D103" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E103" t="n">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="F103" t="n">
-        <v>1609</v>
+        <v>14772</v>
       </c>
       <c r="G103" t="inlineStr">
         <is>
@@ -45669,7 +45734,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>bis/taux_directeurs/NO.csv</t>
+          <t>fred/TOTBKCR.csv</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -45681,13 +45746,13 @@
         <v>12</v>
       </c>
       <c r="D104" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E104" t="n">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="F104" t="n">
-        <v>14772</v>
+        <v>2803</v>
       </c>
       <c r="G104" t="inlineStr">
         <is>
@@ -45698,25 +45763,25 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>fred/TOTBKCR.csv</t>
+          <t>bis/taux_directeurs/AU.csv</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D105" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E105" t="n">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="F105" t="n">
-        <v>2803</v>
+        <v>12882</v>
       </c>
       <c r="G105" t="inlineStr">
         <is>
@@ -45727,16 +45792,16 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>bis/taux_directeurs/AU.csv</t>
+          <t>bis/taux_directeurs/NZ.csv</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D106" t="n">
         <v>1</v>
@@ -45745,7 +45810,7 @@
         <v>42</v>
       </c>
       <c r="F106" t="n">
-        <v>12882</v>
+        <v>15211</v>
       </c>
       <c r="G106" t="inlineStr">
         <is>
@@ -45756,7 +45821,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>bis/taux_directeurs/NZ.csv</t>
+          <t>fred/ECBASSETSW.csv</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -45768,13 +45833,13 @@
         <v>10</v>
       </c>
       <c r="D107" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E107" t="n">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="F107" t="n">
-        <v>15211</v>
+        <v>1447</v>
       </c>
       <c r="G107" t="inlineStr">
         <is>
@@ -45785,25 +45850,25 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>fred/ECBASSETSW.csv</t>
+          <t>bis/taux_directeurs/CN.csv</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D108" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E108" t="n">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="F108" t="n">
-        <v>1447</v>
+        <v>10949</v>
       </c>
       <c r="G108" t="inlineStr">
         <is>
@@ -45814,16 +45879,16 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>bis/taux_directeurs/CN.csv</t>
+          <t>bis/taux_directeurs/CA.csv</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D109" t="n">
         <v>1</v>
@@ -45832,7 +45897,7 @@
         <v>42</v>
       </c>
       <c r="F109" t="n">
-        <v>10949</v>
+        <v>23147</v>
       </c>
       <c r="G109" t="inlineStr">
         <is>
@@ -45843,7 +45908,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>bis/taux_directeurs/CA.csv</t>
+          <t>bis/taux_directeurs/GB.csv</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -45861,7 +45926,7 @@
         <v>42</v>
       </c>
       <c r="F110" t="n">
-        <v>23147</v>
+        <v>23865</v>
       </c>
       <c r="G110" t="inlineStr">
         <is>
@@ -45872,16 +45937,16 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>bis/taux_directeurs/GB.csv</t>
+          <t>bis/taux_directeurs/CH.csv</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D111" t="n">
         <v>1</v>
@@ -45890,7 +45955,7 @@
         <v>42</v>
       </c>
       <c r="F111" t="n">
-        <v>23865</v>
+        <v>21061</v>
       </c>
       <c r="G111" t="inlineStr">
         <is>
@@ -45901,7 +45966,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>bis/taux_directeurs/CH.csv</t>
+          <t>bis/taux_directeurs/JP.csv</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -45919,7 +45984,7 @@
         <v>42</v>
       </c>
       <c r="F112" t="n">
-        <v>21061</v>
+        <v>24889</v>
       </c>
       <c r="G112" t="inlineStr">
         <is>
@@ -45930,7 +45995,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>bis/taux_directeurs/JP.csv</t>
+          <t>bis/taux_directeurs/SE.csv</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -45948,7 +46013,7 @@
         <v>42</v>
       </c>
       <c r="F113" t="n">
-        <v>24889</v>
+        <v>22804</v>
       </c>
       <c r="G113" t="inlineStr">
         <is>
@@ -45959,7 +46024,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>bis/taux_directeurs/SE.csv</t>
+          <t>bis/taux_directeurs/US.csv</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -45977,7 +46042,7 @@
         <v>42</v>
       </c>
       <c r="F114" t="n">
-        <v>22804</v>
+        <v>26381</v>
       </c>
       <c r="G114" t="inlineStr">
         <is>
@@ -45988,7 +46053,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>bis/taux_directeurs/US.csv</t>
+          <t>bis/taux_directeurs/XM.csv</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -46006,7 +46071,7 @@
         <v>42</v>
       </c>
       <c r="F115" t="n">
-        <v>26381</v>
+        <v>10127</v>
       </c>
       <c r="G115" t="inlineStr">
         <is>
@@ -46017,7 +46082,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>bis/taux_directeurs/XM.csv</t>
+          <t>cftc/AUD_FX.csv</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -46029,13 +46094,13 @@
         <v>6</v>
       </c>
       <c r="D116" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E116" t="n">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="F116" t="n">
-        <v>10127</v>
+        <v>1000</v>
       </c>
       <c r="G116" t="inlineStr">
         <is>
@@ -46046,7 +46111,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>cftc/AUD_FX.csv</t>
+          <t>cftc/BRENT_CRUDE.csv</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -46064,7 +46129,7 @@
         <v>63</v>
       </c>
       <c r="F117" t="n">
-        <v>1000</v>
+        <v>242</v>
       </c>
       <c r="G117" t="inlineStr">
         <is>
@@ -46075,7 +46140,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>cftc/BRENT_CRUDE.csv</t>
+          <t>cftc/CAD_FX.csv</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -46093,7 +46158,7 @@
         <v>63</v>
       </c>
       <c r="F118" t="n">
-        <v>242</v>
+        <v>1000</v>
       </c>
       <c r="G118" t="inlineStr">
         <is>
@@ -46104,7 +46169,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>cftc/CAD_FX.csv</t>
+          <t>cftc/CHF_FX.csv</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -46133,7 +46198,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>cftc/CHF_FX.csv</t>
+          <t>cftc/COPPER.csv</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -46151,7 +46216,7 @@
         <v>63</v>
       </c>
       <c r="F120" t="n">
-        <v>1000</v>
+        <v>242</v>
       </c>
       <c r="G120" t="inlineStr">
         <is>
@@ -46162,7 +46227,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>cftc/COPPER.csv</t>
+          <t>cftc/CORN.csv</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -46180,7 +46245,7 @@
         <v>63</v>
       </c>
       <c r="F121" t="n">
-        <v>242</v>
+        <v>1000</v>
       </c>
       <c r="G121" t="inlineStr">
         <is>
@@ -46191,7 +46256,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>cftc/CORN.csv</t>
+          <t>cftc/EUR_FX.csv</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -46220,7 +46285,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>cftc/EUR_FX.csv</t>
+          <t>cftc/FED_FUNDS.csv</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -46238,7 +46303,7 @@
         <v>63</v>
       </c>
       <c r="F123" t="n">
-        <v>1000</v>
+        <v>242</v>
       </c>
       <c r="G123" t="inlineStr">
         <is>
@@ -46249,7 +46314,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>cftc/FED_FUNDS.csv</t>
+          <t>cftc/GBP_FX.csv</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -46278,7 +46343,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>cftc/GBP_FX.csv</t>
+          <t>cftc/GOLD.csv</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -46296,7 +46361,7 @@
         <v>63</v>
       </c>
       <c r="F125" t="n">
-        <v>242</v>
+        <v>1000</v>
       </c>
       <c r="G125" t="inlineStr">
         <is>
@@ -46307,7 +46372,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>cftc/GOLD.csv</t>
+          <t>cftc/JPY_FX.csv</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -46336,7 +46401,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>cftc/JPY_FX.csv</t>
+          <t>cftc/MXN_FX.csv</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -46365,7 +46430,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>cftc/MXN_FX.csv</t>
+          <t>cftc/NASDAQ_MINI.csv</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -46383,7 +46448,7 @@
         <v>63</v>
       </c>
       <c r="F128" t="n">
-        <v>1000</v>
+        <v>242</v>
       </c>
       <c r="G128" t="inlineStr">
         <is>
@@ -46394,7 +46459,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>cftc/NASDAQ_MINI.csv</t>
+          <t>cftc/NAT_GAS.csv</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -46423,7 +46488,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>cftc/NAT_GAS.csv</t>
+          <t>cftc/NZD_FX.csv</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -46452,7 +46517,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>cftc/NZD_FX.csv</t>
+          <t>cftc/PALLADIUM.csv</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -46470,7 +46535,7 @@
         <v>63</v>
       </c>
       <c r="F131" t="n">
-        <v>242</v>
+        <v>1000</v>
       </c>
       <c r="G131" t="inlineStr">
         <is>
@@ -46481,7 +46546,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>cftc/PALLADIUM.csv</t>
+          <t>cftc/PLATINUM.csv</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -46510,7 +46575,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>cftc/PLATINUM.csv</t>
+          <t>cftc/RUSSELL_MINI.csv</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -46528,7 +46593,7 @@
         <v>63</v>
       </c>
       <c r="F133" t="n">
-        <v>1000</v>
+        <v>242</v>
       </c>
       <c r="G133" t="inlineStr">
         <is>
@@ -46539,7 +46604,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>cftc/RUSSELL_MINI.csv</t>
+          <t>cftc/SILVER.csv</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -46557,7 +46622,7 @@
         <v>63</v>
       </c>
       <c r="F134" t="n">
-        <v>242</v>
+        <v>1000</v>
       </c>
       <c r="G134" t="inlineStr">
         <is>
@@ -46568,7 +46633,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>cftc/SILVER.csv</t>
+          <t>cftc/SOFR_3M.csv</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -46586,7 +46651,7 @@
         <v>63</v>
       </c>
       <c r="F135" t="n">
-        <v>1000</v>
+        <v>242</v>
       </c>
       <c r="G135" t="inlineStr">
         <is>
@@ -46597,7 +46662,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>cftc/SOFR_3M.csv</t>
+          <t>cftc/SOYBEANS.csv</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -46615,7 +46680,7 @@
         <v>63</v>
       </c>
       <c r="F136" t="n">
-        <v>242</v>
+        <v>1000</v>
       </c>
       <c r="G136" t="inlineStr">
         <is>
@@ -46626,7 +46691,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>cftc/SOYBEANS.csv</t>
+          <t>cftc/SP500_EMINI.csv</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -46644,7 +46709,7 @@
         <v>63</v>
       </c>
       <c r="F137" t="n">
-        <v>1000</v>
+        <v>242</v>
       </c>
       <c r="G137" t="inlineStr">
         <is>
@@ -46655,7 +46720,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>cftc/SP500_EMINI.csv</t>
+          <t>cftc/USD_INDEX.csv</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -46684,7 +46749,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>cftc/USD_INDEX.csv</t>
+          <t>cftc/UST_10Y.csv</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -46713,7 +46778,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>cftc/UST_10Y.csv</t>
+          <t>cftc/UST_2Y.csv</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -46742,7 +46807,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>cftc/UST_2Y.csv</t>
+          <t>cftc/UST_5Y.csv</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -46771,7 +46836,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>cftc/UST_5Y.csv</t>
+          <t>cftc/UST_BOND.csv</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -46800,7 +46865,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>cftc/UST_BOND.csv</t>
+          <t>cftc/UST_ULTRA_10Y.csv</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -46829,7 +46894,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>cftc/UST_ULTRA_10Y.csv</t>
+          <t>cftc/UST_ULTRA_BOND.csv</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -46847,7 +46912,7 @@
         <v>63</v>
       </c>
       <c r="F144" t="n">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="G144" t="inlineStr">
         <is>
@@ -46858,7 +46923,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>cftc/UST_ULTRA_BOND.csv</t>
+          <t>cftc/VIX_FUT.csv</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -46876,7 +46941,7 @@
         <v>63</v>
       </c>
       <c r="F145" t="n">
-        <v>240</v>
+        <v>1000</v>
       </c>
       <c r="G145" t="inlineStr">
         <is>
@@ -46887,7 +46952,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>cftc/VIX_FUT.csv</t>
+          <t>cftc/WHEAT.csv</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -46905,7 +46970,7 @@
         <v>63</v>
       </c>
       <c r="F146" t="n">
-        <v>1000</v>
+        <v>667</v>
       </c>
       <c r="G146" t="inlineStr">
         <is>
@@ -46916,7 +46981,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>cftc/WHEAT.csv</t>
+          <t>cftc/WTI_CRUDE.csv</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -46934,7 +46999,7 @@
         <v>63</v>
       </c>
       <c r="F147" t="n">
-        <v>667</v>
+        <v>242</v>
       </c>
       <c r="G147" t="inlineStr">
         <is>
@@ -46945,16 +47010,16 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>cftc/WTI_CRUDE.csv</t>
+          <t>bilans/BOC_V1038114416.csv</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D148" t="n">
         <v>7</v>
@@ -46963,7 +47028,7 @@
         <v>63</v>
       </c>
       <c r="F148" t="n">
-        <v>242</v>
+        <v>405</v>
       </c>
       <c r="G148" t="inlineStr">
         <is>
@@ -46974,7 +47039,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>bilans/BOC_V1038114416.csv</t>
+          <t>bilans/BOC_V1146067261.csv</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -46992,7 +47057,7 @@
         <v>63</v>
       </c>
       <c r="F149" t="n">
-        <v>405</v>
+        <v>340</v>
       </c>
       <c r="G149" t="inlineStr">
         <is>
@@ -47003,7 +47068,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>bilans/BOC_V1146067261.csv</t>
+          <t>bilans/BOC_V1146067262.csv</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -47032,7 +47097,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>bilans/BOC_V1146067262.csv</t>
+          <t>bilans/BOC_V1146067263.csv</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -47050,7 +47115,7 @@
         <v>63</v>
       </c>
       <c r="F151" t="n">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="G151" t="inlineStr">
         <is>
@@ -47061,7 +47126,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>bilans/BOC_V1146067263.csv</t>
+          <t>bilans/BOC_V1146067264.csv</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -47079,7 +47144,7 @@
         <v>63</v>
       </c>
       <c r="F152" t="n">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="G152" t="inlineStr">
         <is>
@@ -47090,7 +47155,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>bilans/BOC_V1146067264.csv</t>
+          <t>bilans/BOC_V1154426989.csv</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -47108,7 +47173,7 @@
         <v>63</v>
       </c>
       <c r="F153" t="n">
-        <v>340</v>
+        <v>333</v>
       </c>
       <c r="G153" t="inlineStr">
         <is>
@@ -47119,7 +47184,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>bilans/BOC_V1154426989.csv</t>
+          <t>bilans/BOC_V1154426990.csv</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -47137,7 +47202,7 @@
         <v>63</v>
       </c>
       <c r="F154" t="n">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="G154" t="inlineStr">
         <is>
@@ -47148,7 +47213,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>bilans/BOC_V1154426990.csv</t>
+          <t>bilans/BOC_V1154426991.csv</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -47166,7 +47231,7 @@
         <v>63</v>
       </c>
       <c r="F155" t="n">
-        <v>330</v>
+        <v>308</v>
       </c>
       <c r="G155" t="inlineStr">
         <is>
@@ -47177,7 +47242,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>bilans/BOC_V1154426991.csv</t>
+          <t>bilans/BOC_V1160788296.csv</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -47195,7 +47260,7 @@
         <v>63</v>
       </c>
       <c r="F156" t="n">
-        <v>308</v>
+        <v>330</v>
       </c>
       <c r="G156" t="inlineStr">
         <is>
@@ -47206,7 +47271,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>bilans/BOC_V1160788296.csv</t>
+          <t>bilans/BOC_V1203435186.csv</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -47224,7 +47289,7 @@
         <v>63</v>
       </c>
       <c r="F157" t="n">
-        <v>330</v>
+        <v>322</v>
       </c>
       <c r="G157" t="inlineStr">
         <is>
@@ -47235,7 +47300,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>bilans/BOC_V1203435186.csv</t>
+          <t>bilans/BOC_V1210798115.csv</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -47253,7 +47318,7 @@
         <v>63</v>
       </c>
       <c r="F158" t="n">
-        <v>322</v>
+        <v>326</v>
       </c>
       <c r="G158" t="inlineStr">
         <is>
@@ -47264,7 +47329,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>bilans/BOC_V1210798115.csv</t>
+          <t>bilans/BOC_V1490410223.csv</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -47282,7 +47347,7 @@
         <v>63</v>
       </c>
       <c r="F159" t="n">
-        <v>326</v>
+        <v>195</v>
       </c>
       <c r="G159" t="inlineStr">
         <is>
@@ -47293,7 +47358,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>bilans/BOC_V1490410223.csv</t>
+          <t>bilans/BOC_V1490410224.csv</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -47322,7 +47387,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>bilans/BOC_V1490410224.csv</t>
+          <t>bilans/BOC_V36610.csv</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -47340,7 +47405,7 @@
         <v>63</v>
       </c>
       <c r="F161" t="n">
-        <v>195</v>
+        <v>1917</v>
       </c>
       <c r="G161" t="inlineStr">
         <is>
@@ -47351,7 +47416,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>bilans/BOC_V36610.csv</t>
+          <t>bilans/BOC_V36612.csv</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -47380,7 +47445,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>bilans/BOC_V36612.csv</t>
+          <t>bilans/BOC_V36613.csv</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -47409,7 +47474,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>bilans/BOC_V36613.csv</t>
+          <t>bilans/BOC_V36624.csv</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -47438,7 +47503,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>bilans/BOC_V36624.csv</t>
+          <t>bilans/BOC_V36625.csv</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
@@ -47467,7 +47532,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>bilans/BOC_V36625.csv</t>
+          <t>bilans/BOC_V36628.csv</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -47496,7 +47561,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>bilans/BOC_V36628.csv</t>
+          <t>bilans/BOC_V36634.csv</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -47525,7 +47590,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>bilans/BOC_V36634.csv</t>
+          <t>bilans/BOC_V36635.csv</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -47554,7 +47619,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>bilans/BOC_V36635.csv</t>
+          <t>bilans/BOC_V36636.csv</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
@@ -47583,7 +47648,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>bilans/BOC_V36636.csv</t>
+          <t>bilans/BOC_V44201362.csv</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -47601,7 +47666,7 @@
         <v>63</v>
       </c>
       <c r="F170" t="n">
-        <v>1917</v>
+        <v>991</v>
       </c>
       <c r="G170" t="inlineStr">
         <is>
@@ -47612,7 +47677,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>bilans/BOC_V44201362.csv</t>
+          <t>bilans/BOE_BILAN_TOTAL.csv</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -47630,7 +47695,7 @@
         <v>63</v>
       </c>
       <c r="F171" t="n">
-        <v>991</v>
+        <v>1610</v>
       </c>
       <c r="G171" t="inlineStr">
         <is>
@@ -47728,7 +47793,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>fred/IUDSOIA.csv</t>
+          <t>fred/RESPPLLOPNWW.csv</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -47740,13 +47805,13 @@
         <v>5</v>
       </c>
       <c r="D175" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E175" t="n">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="F175" t="n">
-        <v>3000</v>
+        <v>1241</v>
       </c>
       <c r="G175" t="inlineStr">
         <is>
@@ -47757,7 +47822,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>fred/RESPPLLOPNWW.csv</t>
+          <t>fred/TREAST.csv</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -47786,7 +47851,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>fred/TREAST.csv</t>
+          <t>fred/WALCL.csv</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
@@ -47815,7 +47880,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>fred/WALCL.csv</t>
+          <t>fred/WLRRAL.csv</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -47844,7 +47909,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>fred/WLRRAL.csv</t>
+          <t>fred/WRESBAL.csv</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -47862,7 +47927,7 @@
         <v>63</v>
       </c>
       <c r="F179" t="n">
-        <v>1241</v>
+        <v>2230</v>
       </c>
       <c r="G179" t="inlineStr">
         <is>
@@ -47873,7 +47938,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>fred/WRESBAL.csv</t>
+          <t>fred/WSHOMCB.csv</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -47891,7 +47956,7 @@
         <v>63</v>
       </c>
       <c r="F180" t="n">
-        <v>2230</v>
+        <v>1241</v>
       </c>
       <c r="G180" t="inlineStr">
         <is>
@@ -47902,7 +47967,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>fred/WSHOMCB.csv</t>
+          <t>fred/WSHOSHO.csv</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -47931,7 +47996,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>fred/WSHOSHO.csv</t>
+          <t>fred/WTREGEN.csv</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
@@ -47949,7 +48014,7 @@
         <v>63</v>
       </c>
       <c r="F182" t="n">
-        <v>1241</v>
+        <v>2125</v>
       </c>
       <c r="G182" t="inlineStr">
         <is>
@@ -47960,7 +48025,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>fred/WTREGEN.csv</t>
+          <t>souverains/AUSTRALIE_10A.csv</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -47972,13 +48037,13 @@
         <v>5</v>
       </c>
       <c r="D183" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E183" t="n">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="F183" t="n">
-        <v>2125</v>
+        <v>3361</v>
       </c>
       <c r="G183" t="inlineStr">
         <is>
@@ -47989,7 +48054,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>souverains/AUSTRALIE_10A.csv</t>
+          <t>souverains/AUSTRALIE_2A.csv</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -48007,7 +48072,7 @@
         <v>42</v>
       </c>
       <c r="F184" t="n">
-        <v>3361</v>
+        <v>3283</v>
       </c>
       <c r="G184" t="inlineStr">
         <is>
@@ -48018,7 +48083,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>souverains/AUSTRALIE_2A.csv</t>
+          <t>souverains/AUSTRALIE_5A.csv</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -48047,16 +48112,16 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>souverains/AUSTRALIE_5A.csv</t>
+          <t>fred/BAMLC0A0CM.csv</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C186" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D186" t="n">
         <v>1</v>
@@ -48065,7 +48130,7 @@
         <v>42</v>
       </c>
       <c r="F186" t="n">
-        <v>3283</v>
+        <v>795</v>
       </c>
       <c r="G186" t="inlineStr">
         <is>
@@ -48076,16 +48141,16 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>souverains/UK_10A.csv</t>
+          <t>fred/BAMLC0A0CMEY.csv</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C187" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D187" t="n">
         <v>1</v>
@@ -48094,7 +48159,7 @@
         <v>42</v>
       </c>
       <c r="F187" t="n">
-        <v>9282</v>
+        <v>795</v>
       </c>
       <c r="G187" t="inlineStr">
         <is>
@@ -48105,16 +48170,16 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>souverains/UK_20A.csv</t>
+          <t>fred/BAMLEMCBPIOAS.csv</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C188" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D188" t="n">
         <v>1</v>
@@ -48123,7 +48188,7 @@
         <v>42</v>
       </c>
       <c r="F188" t="n">
-        <v>6753</v>
+        <v>795</v>
       </c>
       <c r="G188" t="inlineStr">
         <is>
@@ -48134,16 +48199,16 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>souverains/UK_5A.csv</t>
+          <t>fred/BAMLEMFSFCRPIOAS.csv</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C189" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D189" t="n">
         <v>1</v>
@@ -48152,7 +48217,7 @@
         <v>42</v>
       </c>
       <c r="F189" t="n">
-        <v>8290</v>
+        <v>795</v>
       </c>
       <c r="G189" t="inlineStr">
         <is>
@@ -48163,7 +48228,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>fred/BAMLC0A0CM.csv</t>
+          <t>fred/BAMLEMHBHYCRPIOAS.csv</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -48192,7 +48257,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>fred/BAMLC0A0CMEY.csv</t>
+          <t>fred/BAMLEMPBPUBSICRPIOAS.csv</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -48221,7 +48286,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>fred/BAMLEMCBPIOAS.csv</t>
+          <t>fred/BAMLH0A0HYM2.csv</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -48250,7 +48315,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>fred/BAMLEMFSFCRPIOAS.csv</t>
+          <t>fred/BAMLHE00EHYIEY.csv</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -48279,7 +48344,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>fred/BAMLEMHBHYCRPIOAS.csv</t>
+          <t>fred/BAMLHE00EHYIOAS.csv</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -48308,7 +48373,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>fred/BAMLEMPBPUBSICRPIOAS.csv</t>
+          <t>fred/DFF.csv</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -48326,7 +48391,7 @@
         <v>42</v>
       </c>
       <c r="F195" t="n">
-        <v>795</v>
+        <v>3000</v>
       </c>
       <c r="G195" t="inlineStr">
         <is>
@@ -48337,7 +48402,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>fred/BAMLH0A0HYM2.csv</t>
+          <t>fred/DFII10.csv</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -48355,7 +48420,7 @@
         <v>42</v>
       </c>
       <c r="F196" t="n">
-        <v>795</v>
+        <v>3000</v>
       </c>
       <c r="G196" t="inlineStr">
         <is>
@@ -48366,7 +48431,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>fred/BAMLHE00EHYIEY.csv</t>
+          <t>fred/DFII5.csv</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -48384,7 +48449,7 @@
         <v>42</v>
       </c>
       <c r="F197" t="n">
-        <v>795</v>
+        <v>3000</v>
       </c>
       <c r="G197" t="inlineStr">
         <is>
@@ -48395,7 +48460,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>fred/BAMLHE00EHYIOAS.csv</t>
+          <t>fred/DGS1.csv</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -48413,7 +48478,7 @@
         <v>42</v>
       </c>
       <c r="F198" t="n">
-        <v>795</v>
+        <v>3000</v>
       </c>
       <c r="G198" t="inlineStr">
         <is>
@@ -48424,7 +48489,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>fred/DFF.csv</t>
+          <t>fred/DGS10.csv</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -48453,7 +48518,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>fred/DFII10.csv</t>
+          <t>fred/DGS1MO.csv</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -48482,7 +48547,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>fred/DFII5.csv</t>
+          <t>fred/DGS2.csv</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -48511,7 +48576,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>fred/DGS1.csv</t>
+          <t>fred/DGS30.csv</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -48540,7 +48605,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>fred/DGS10.csv</t>
+          <t>fred/DGS3MO.csv</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -48569,7 +48634,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>fred/DGS1MO.csv</t>
+          <t>fred/DGS5.csv</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
@@ -48598,7 +48663,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>fred/DGS2.csv</t>
+          <t>fred/DGS6MO.csv</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -48627,7 +48692,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>fred/DGS30.csv</t>
+          <t>fred/IUDSOIA.csv</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -48656,7 +48721,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>fred/DGS3MO.csv</t>
+          <t>fred/MORTGAGE30US.csv</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -48668,13 +48733,13 @@
         <v>4</v>
       </c>
       <c r="D207" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E207" t="n">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="F207" t="n">
-        <v>3000</v>
+        <v>2896</v>
       </c>
       <c r="G207" t="inlineStr">
         <is>
@@ -48685,7 +48750,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>fred/DGS5.csv</t>
+          <t>souverains/CANADA_10A.csv</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -48703,7 +48768,7 @@
         <v>42</v>
       </c>
       <c r="F208" t="n">
-        <v>3000</v>
+        <v>6435</v>
       </c>
       <c r="G208" t="inlineStr">
         <is>
@@ -48714,7 +48779,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>fred/DGS6MO.csv</t>
+          <t>souverains/CANADA_2A.csv</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -48732,7 +48797,7 @@
         <v>42</v>
       </c>
       <c r="F209" t="n">
-        <v>3000</v>
+        <v>6434</v>
       </c>
       <c r="G209" t="inlineStr">
         <is>
@@ -48743,7 +48808,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>fred/MORTGAGE30US.csv</t>
+          <t>souverains/CANADA_5A.csv</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -48755,13 +48820,13 @@
         <v>4</v>
       </c>
       <c r="D210" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E210" t="n">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="F210" t="n">
-        <v>2896</v>
+        <v>6434</v>
       </c>
       <c r="G210" t="inlineStr">
         <is>
@@ -48772,7 +48837,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>souverains/CANADA_10A.csv</t>
+          <t>souverains/CANADA_LONG.csv</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
@@ -48790,7 +48855,7 @@
         <v>42</v>
       </c>
       <c r="F211" t="n">
-        <v>6435</v>
+        <v>6434</v>
       </c>
       <c r="G211" t="inlineStr">
         <is>
@@ -48801,7 +48866,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>souverains/CANADA_2A.csv</t>
+          <t>souverains/UK_10A.csv</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -48819,7 +48884,7 @@
         <v>42</v>
       </c>
       <c r="F212" t="n">
-        <v>6434</v>
+        <v>9283</v>
       </c>
       <c r="G212" t="inlineStr">
         <is>
@@ -48830,7 +48895,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>souverains/CANADA_5A.csv</t>
+          <t>souverains/UK_20A.csv</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -48848,7 +48913,7 @@
         <v>42</v>
       </c>
       <c r="F213" t="n">
-        <v>6434</v>
+        <v>6754</v>
       </c>
       <c r="G213" t="inlineStr">
         <is>
@@ -48859,7 +48924,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>souverains/CANADA_LONG.csv</t>
+          <t>souverains/UK_5A.csv</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -48877,7 +48942,7 @@
         <v>42</v>
       </c>
       <c r="F214" t="n">
-        <v>6434</v>
+        <v>8291</v>
       </c>
       <c r="G214" t="inlineStr">
         <is>
@@ -48888,7 +48953,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
+          <t>tresor_us/dette_quotidienne.csv</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -48906,7 +48971,7 @@
         <v>42</v>
       </c>
       <c r="F215" t="n">
-        <v>5638</v>
+        <v>2000</v>
       </c>
       <c r="G215" t="inlineStr">
         <is>
@@ -48917,7 +48982,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
+          <t>tresor_us/solde_tresorerie.csv</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -48935,7 +49000,7 @@
         <v>42</v>
       </c>
       <c r="F216" t="n">
-        <v>5638</v>
+        <v>500</v>
       </c>
       <c r="G216" t="inlineStr">
         <is>
@@ -48946,16 +49011,16 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
+          <t>fred/ECBDFR.csv</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C217" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D217" t="n">
         <v>1</v>
@@ -48964,7 +49029,7 @@
         <v>42</v>
       </c>
       <c r="F217" t="n">
-        <v>5638</v>
+        <v>3000</v>
       </c>
       <c r="G217" t="inlineStr">
         <is>
@@ -48975,16 +49040,16 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
+          <t>fred/RRPONTSYD.csv</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C218" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D218" t="n">
         <v>1</v>
@@ -48993,7 +49058,7 @@
         <v>42</v>
       </c>
       <c r="F218" t="n">
-        <v>5638</v>
+        <v>3000</v>
       </c>
       <c r="G218" t="inlineStr">
         <is>
@@ -49004,16 +49069,16 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
+          <t>fred/T10YIE.csv</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C219" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D219" t="n">
         <v>1</v>
@@ -49022,7 +49087,7 @@
         <v>42</v>
       </c>
       <c r="F219" t="n">
-        <v>5638</v>
+        <v>3000</v>
       </c>
       <c r="G219" t="inlineStr">
         <is>
@@ -49033,16 +49098,16 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
+          <t>marches/volatilite/GVZ.csv</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C220" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D220" t="n">
         <v>1</v>
@@ -49051,7 +49116,7 @@
         <v>42</v>
       </c>
       <c r="F220" t="n">
-        <v>5638</v>
+        <v>3772</v>
       </c>
       <c r="G220" t="inlineStr">
         <is>
@@ -49062,16 +49127,16 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
+          <t>marches/volatilite/MOVE.csv</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C221" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D221" t="n">
         <v>1</v>
@@ -49080,7 +49145,7 @@
         <v>42</v>
       </c>
       <c r="F221" t="n">
-        <v>5638</v>
+        <v>3691</v>
       </c>
       <c r="G221" t="inlineStr">
         <is>
@@ -49091,16 +49156,16 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
+          <t>marches/volatilite/OVX.csv</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C222" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D222" t="n">
         <v>1</v>
@@ -49109,7 +49174,7 @@
         <v>42</v>
       </c>
       <c r="F222" t="n">
-        <v>5638</v>
+        <v>3772</v>
       </c>
       <c r="G222" t="inlineStr">
         <is>
@@ -49120,16 +49185,16 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
+          <t>marches/volatilite/VVIX.csv</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C223" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D223" t="n">
         <v>1</v>
@@ -49138,7 +49203,7 @@
         <v>42</v>
       </c>
       <c r="F223" t="n">
-        <v>5638</v>
+        <v>3764</v>
       </c>
       <c r="G223" t="inlineStr">
         <is>
@@ -49149,16 +49214,16 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>tresor_us/dette_quotidienne.csv</t>
+          <t>marches/volatilite/VXN.csv</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C224" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D224" t="n">
         <v>1</v>
@@ -49167,7 +49232,7 @@
         <v>42</v>
       </c>
       <c r="F224" t="n">
-        <v>2000</v>
+        <v>3772</v>
       </c>
       <c r="G224" t="inlineStr">
         <is>
@@ -49178,16 +49243,16 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>tresor_us/solde_tresorerie.csv</t>
+          <t>souverains/SUEDE_10A.csv</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C225" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D225" t="n">
         <v>1</v>
@@ -49196,7 +49261,7 @@
         <v>42</v>
       </c>
       <c r="F225" t="n">
-        <v>500</v>
+        <v>9202</v>
       </c>
       <c r="G225" t="inlineStr">
         <is>
@@ -49207,7 +49272,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>fred/ECBDFR.csv</t>
+          <t>souverains/SUEDE_2A.csv</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -49225,7 +49290,7 @@
         <v>42</v>
       </c>
       <c r="F226" t="n">
-        <v>3000</v>
+        <v>9202</v>
       </c>
       <c r="G226" t="inlineStr">
         <is>
@@ -49236,7 +49301,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>fred/RRPONTSYD.csv</t>
+          <t>souverains/SUEDE_5A.csv</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -49254,7 +49319,7 @@
         <v>42</v>
       </c>
       <c r="F227" t="n">
-        <v>3000</v>
+        <v>9204</v>
       </c>
       <c r="G227" t="inlineStr">
         <is>
@@ -49265,7 +49330,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>fred/T10YIE.csv</t>
+          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -49283,7 +49348,7 @@
         <v>42</v>
       </c>
       <c r="F228" t="n">
-        <v>3000</v>
+        <v>5639</v>
       </c>
       <c r="G228" t="inlineStr">
         <is>
@@ -49294,7 +49359,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>marches/indices/DAX.csv</t>
+          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -49312,7 +49377,7 @@
         <v>42</v>
       </c>
       <c r="F229" t="n">
-        <v>3803</v>
+        <v>5639</v>
       </c>
       <c r="G229" t="inlineStr">
         <is>
@@ -49323,7 +49388,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>marches/indices/EUROSTOXX50.csv</t>
+          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -49341,7 +49406,7 @@
         <v>42</v>
       </c>
       <c r="F230" t="n">
-        <v>3760</v>
+        <v>5639</v>
       </c>
       <c r="G230" t="inlineStr">
         <is>
@@ -49352,7 +49417,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>marches/indices/FTSE100.csv</t>
+          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -49370,7 +49435,7 @@
         <v>42</v>
       </c>
       <c r="F231" t="n">
-        <v>3789</v>
+        <v>5639</v>
       </c>
       <c r="G231" t="inlineStr">
         <is>
@@ -49381,7 +49446,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>marches/volatilite/GVZ.csv</t>
+          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -49399,7 +49464,7 @@
         <v>42</v>
       </c>
       <c r="F232" t="n">
-        <v>3772</v>
+        <v>5639</v>
       </c>
       <c r="G232" t="inlineStr">
         <is>
@@ -49410,7 +49475,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>marches/volatilite/MOVE.csv</t>
+          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -49428,7 +49493,7 @@
         <v>42</v>
       </c>
       <c r="F233" t="n">
-        <v>3691</v>
+        <v>5639</v>
       </c>
       <c r="G233" t="inlineStr">
         <is>
@@ -49439,7 +49504,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>marches/volatilite/OVX.csv</t>
+          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -49457,7 +49522,7 @@
         <v>42</v>
       </c>
       <c r="F234" t="n">
-        <v>3772</v>
+        <v>5639</v>
       </c>
       <c r="G234" t="inlineStr">
         <is>
@@ -49468,7 +49533,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>marches/volatilite/VVIX.csv</t>
+          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -49486,7 +49551,7 @@
         <v>42</v>
       </c>
       <c r="F235" t="n">
-        <v>3764</v>
+        <v>5639</v>
       </c>
       <c r="G235" t="inlineStr">
         <is>
@@ -49497,7 +49562,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>marches/volatilite/VXN.csv</t>
+          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -49515,7 +49580,7 @@
         <v>42</v>
       </c>
       <c r="F236" t="n">
-        <v>3772</v>
+        <v>5639</v>
       </c>
       <c r="G236" t="inlineStr">
         <is>
@@ -49526,7 +49591,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_10A.csv</t>
+          <t>yfinance/SP500.csv</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
@@ -49544,7 +49609,7 @@
         <v>42</v>
       </c>
       <c r="F237" t="n">
-        <v>9202</v>
+        <v>7547</v>
       </c>
       <c r="G237" t="inlineStr">
         <is>
@@ -49555,7 +49620,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_2A.csv</t>
+          <t>yfinance/XLB.csv</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
@@ -49573,7 +49638,7 @@
         <v>42</v>
       </c>
       <c r="F238" t="n">
-        <v>9202</v>
+        <v>501</v>
       </c>
       <c r="G238" t="inlineStr">
         <is>
@@ -49584,7 +49649,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_5A.csv</t>
+          <t>yfinance/XLE.csv</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
@@ -49602,7 +49667,7 @@
         <v>42</v>
       </c>
       <c r="F239" t="n">
-        <v>9204</v>
+        <v>501</v>
       </c>
       <c r="G239" t="inlineStr">
         <is>
@@ -49613,7 +49678,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>yfinance/SP500.csv</t>
+          <t>yfinance/XLF.csv</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
@@ -49631,7 +49696,7 @@
         <v>42</v>
       </c>
       <c r="F240" t="n">
-        <v>7547</v>
+        <v>501</v>
       </c>
       <c r="G240" t="inlineStr">
         <is>
@@ -49642,7 +49707,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>yfinance/VIX.csv</t>
+          <t>yfinance/XLI.csv</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
@@ -49660,7 +49725,7 @@
         <v>42</v>
       </c>
       <c r="F241" t="n">
-        <v>7550</v>
+        <v>501</v>
       </c>
       <c r="G241" t="inlineStr">
         <is>
@@ -49671,7 +49736,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>yfinance/XLB.csv</t>
+          <t>yfinance/XLK.csv</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
@@ -49700,7 +49765,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>yfinance/XLE.csv</t>
+          <t>yfinance/XLP.csv</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
@@ -49729,7 +49794,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>yfinance/XLF.csv</t>
+          <t>yfinance/XLRE.csv</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -49758,7 +49823,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>yfinance/XLI.csv</t>
+          <t>yfinance/XLU.csv</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -49787,7 +49852,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>yfinance/XLK.csv</t>
+          <t>yfinance/XLV.csv</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -49816,7 +49881,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>yfinance/XLP.csv</t>
+          <t>yfinance/XLY.csv</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
@@ -49845,16 +49910,16 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>yfinance/XLRE.csv</t>
+          <t>marches/fx/AUDJPY.csv</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C248" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D248" t="n">
         <v>1</v>
@@ -49863,7 +49928,7 @@
         <v>42</v>
       </c>
       <c r="F248" t="n">
-        <v>501</v>
+        <v>3908</v>
       </c>
       <c r="G248" t="inlineStr">
         <is>
@@ -49874,16 +49939,16 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>yfinance/XLU.csv</t>
+          <t>marches/fx/AUDUSD.csv</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C249" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D249" t="n">
         <v>1</v>
@@ -49892,7 +49957,7 @@
         <v>42</v>
       </c>
       <c r="F249" t="n">
-        <v>501</v>
+        <v>3904</v>
       </c>
       <c r="G249" t="inlineStr">
         <is>
@@ -49903,16 +49968,16 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>yfinance/XLV.csv</t>
+          <t>marches/fx/DXY.csv</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C250" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D250" t="n">
         <v>1</v>
@@ -49921,7 +49986,7 @@
         <v>42</v>
       </c>
       <c r="F250" t="n">
-        <v>501</v>
+        <v>3772</v>
       </c>
       <c r="G250" t="inlineStr">
         <is>
@@ -49932,16 +49997,16 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>yfinance/XLY.csv</t>
+          <t>marches/fx/EURCHF.csv</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C251" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D251" t="n">
         <v>1</v>
@@ -49950,7 +50015,7 @@
         <v>42</v>
       </c>
       <c r="F251" t="n">
-        <v>501</v>
+        <v>3905</v>
       </c>
       <c r="G251" t="inlineStr">
         <is>
@@ -49961,7 +50026,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>marches/fx/AUDJPY.csv</t>
+          <t>marches/fx/EURGBP.csv</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -49979,7 +50044,7 @@
         <v>42</v>
       </c>
       <c r="F252" t="n">
-        <v>3908</v>
+        <v>3907</v>
       </c>
       <c r="G252" t="inlineStr">
         <is>
@@ -49990,7 +50055,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>marches/fx/AUDUSD.csv</t>
+          <t>marches/fx/EURJPY.csv</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -50008,7 +50073,7 @@
         <v>42</v>
       </c>
       <c r="F253" t="n">
-        <v>3904</v>
+        <v>3907</v>
       </c>
       <c r="G253" t="inlineStr">
         <is>
@@ -50019,7 +50084,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>marches/fx/DXY.csv</t>
+          <t>marches/fx/EURUSD.csv</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
@@ -50037,7 +50102,7 @@
         <v>42</v>
       </c>
       <c r="F254" t="n">
-        <v>3772</v>
+        <v>3904</v>
       </c>
       <c r="G254" t="inlineStr">
         <is>
@@ -50048,7 +50113,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>marches/fx/EURCHF.csv</t>
+          <t>marches/fx/GBPUSD.csv</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
@@ -50077,7 +50142,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>marches/fx/EURGBP.csv</t>
+          <t>marches/fx/NZDUSD.csv</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
@@ -50095,7 +50160,7 @@
         <v>42</v>
       </c>
       <c r="F256" t="n">
-        <v>3907</v>
+        <v>3905</v>
       </c>
       <c r="G256" t="inlineStr">
         <is>
@@ -50106,7 +50171,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>marches/fx/EURJPY.csv</t>
+          <t>marches/fx/USDCAD.csv</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
@@ -50124,7 +50189,7 @@
         <v>42</v>
       </c>
       <c r="F257" t="n">
-        <v>3907</v>
+        <v>3904</v>
       </c>
       <c r="G257" t="inlineStr">
         <is>
@@ -50135,7 +50200,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>marches/fx/EURUSD.csv</t>
+          <t>marches/fx/USDCHF.csv</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
@@ -50153,7 +50218,7 @@
         <v>42</v>
       </c>
       <c r="F258" t="n">
-        <v>3904</v>
+        <v>3902</v>
       </c>
       <c r="G258" t="inlineStr">
         <is>
@@ -50164,7 +50229,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>marches/fx/GBPUSD.csv</t>
+          <t>marches/fx/USDCNY.csv</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
@@ -50182,7 +50247,7 @@
         <v>42</v>
       </c>
       <c r="F259" t="n">
-        <v>3905</v>
+        <v>3904</v>
       </c>
       <c r="G259" t="inlineStr">
         <is>
@@ -50193,7 +50258,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>marches/fx/NZDUSD.csv</t>
+          <t>marches/fx/USDJPY.csv</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
@@ -50222,7 +50287,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>marches/fx/USDCAD.csv</t>
+          <t>marches/fx/USDKRW.csv</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
@@ -50251,7 +50316,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>marches/fx/USDCHF.csv</t>
+          <t>marches/fx/USDNOK.csv</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
@@ -50269,7 +50334,7 @@
         <v>42</v>
       </c>
       <c r="F262" t="n">
-        <v>3902</v>
+        <v>3905</v>
       </c>
       <c r="G262" t="inlineStr">
         <is>
@@ -50280,7 +50345,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>marches/fx/USDCNY.csv</t>
+          <t>marches/fx/USDSEK.csv</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
@@ -50298,7 +50363,7 @@
         <v>42</v>
       </c>
       <c r="F263" t="n">
-        <v>3904</v>
+        <v>3905</v>
       </c>
       <c r="G263" t="inlineStr">
         <is>
@@ -50309,7 +50374,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>marches/fx/USDJPY.csv</t>
+          <t>marches/indices/DAX.csv</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
@@ -50327,7 +50392,7 @@
         <v>42</v>
       </c>
       <c r="F264" t="n">
-        <v>3905</v>
+        <v>3802</v>
       </c>
       <c r="G264" t="inlineStr">
         <is>
@@ -50338,7 +50403,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>marches/fx/USDKRW.csv</t>
+          <t>marches/indices/EUROSTOXX50.csv</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
@@ -50356,7 +50421,7 @@
         <v>42</v>
       </c>
       <c r="F265" t="n">
-        <v>3904</v>
+        <v>3759</v>
       </c>
       <c r="G265" t="inlineStr">
         <is>
@@ -50367,7 +50432,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>marches/fx/USDNOK.csv</t>
+          <t>marches/indices/FTSE100.csv</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
@@ -50385,7 +50450,7 @@
         <v>42</v>
       </c>
       <c r="F266" t="n">
-        <v>3905</v>
+        <v>3788</v>
       </c>
       <c r="G266" t="inlineStr">
         <is>
@@ -50396,7 +50461,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>marches/fx/USDSEK.csv</t>
+          <t>marches/indices/HANGSENG.csv</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
@@ -50414,7 +50479,7 @@
         <v>42</v>
       </c>
       <c r="F267" t="n">
-        <v>3905</v>
+        <v>3689</v>
       </c>
       <c r="G267" t="inlineStr">
         <is>
@@ -50425,7 +50490,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>marches/indices/HANGSENG.csv</t>
+          <t>marches/indices/KOSPI.csv</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
@@ -50443,7 +50508,7 @@
         <v>42</v>
       </c>
       <c r="F268" t="n">
-        <v>3689</v>
+        <v>3681</v>
       </c>
       <c r="G268" t="inlineStr">
         <is>
@@ -50454,7 +50519,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>marches/indices/KOSPI.csv</t>
+          <t>marches/indices/NIKKEI225.csv</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
@@ -50472,7 +50537,7 @@
         <v>42</v>
       </c>
       <c r="F269" t="n">
-        <v>3681</v>
+        <v>3667</v>
       </c>
       <c r="G269" t="inlineStr">
         <is>
@@ -50483,7 +50548,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>marches/indices/NIKKEI225.csv</t>
+          <t>marches/matieres/BRENT.csv</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
@@ -50501,7 +50566,7 @@
         <v>42</v>
       </c>
       <c r="F270" t="n">
-        <v>3667</v>
+        <v>3751</v>
       </c>
       <c r="G270" t="inlineStr">
         <is>
@@ -50512,7 +50577,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>marches/matieres/BRENT.csv</t>
+          <t>marches/matieres/CUIVRE.csv</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
@@ -50530,7 +50595,7 @@
         <v>42</v>
       </c>
       <c r="F271" t="n">
-        <v>3751</v>
+        <v>3771</v>
       </c>
       <c r="G271" t="inlineStr">
         <is>
@@ -50541,7 +50606,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>marches/matieres/CUIVRE.csv</t>
+          <t>marches/matieres/GAZ_HENRY_HUB.csv</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
@@ -50559,7 +50624,7 @@
         <v>42</v>
       </c>
       <c r="F272" t="n">
-        <v>3771</v>
+        <v>3772</v>
       </c>
       <c r="G272" t="inlineStr">
         <is>
@@ -50570,7 +50635,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>marches/matieres/GAZ_HENRY_HUB.csv</t>
+          <t>marches/matieres/OR.csv</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
@@ -50588,7 +50653,7 @@
         <v>42</v>
       </c>
       <c r="F273" t="n">
-        <v>3772</v>
+        <v>3771</v>
       </c>
       <c r="G273" t="inlineStr">
         <is>
@@ -50599,7 +50664,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>marches/matieres/OR.csv</t>
+          <t>marches/matieres/WTI.csv</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
@@ -50628,7 +50693,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>marches/matieres/WTI.csv</t>
+          <t>marches/taux_futures/FED_FUNDS_FRONT.csv</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
@@ -50646,7 +50711,7 @@
         <v>42</v>
       </c>
       <c r="F275" t="n">
-        <v>3771</v>
+        <v>3772</v>
       </c>
       <c r="G275" t="inlineStr">
         <is>
@@ -50657,7 +50722,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>marches/taux_futures/FED_FUNDS_FRONT.csv</t>
+          <t>yfinance/VIX.csv</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
@@ -50675,7 +50740,7 @@
         <v>42</v>
       </c>
       <c r="F276" t="n">
-        <v>3772</v>
+        <v>7548</v>
       </c>
       <c r="G276" t="inlineStr">
         <is>
@@ -52070,13 +52135,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.01025</v>
+        <v>0.01024</v>
       </c>
       <c r="C13" t="n">
-        <v>0.00424</v>
+        <v>-0.00094</v>
       </c>
       <c r="D13" t="n">
-        <v>0.01648</v>
+        <v>0.01231</v>
       </c>
     </row>
   </sheetData>
@@ -52139,13 +52204,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>6942.46</v>
+        <v>6889.74</v>
       </c>
       <c r="D2" t="n">
-        <v>-17.3</v>
+        <v>-17.93</v>
       </c>
       <c r="E2" t="n">
-        <v>105.03</v>
+        <v>103.47</v>
       </c>
     </row>
     <row r="3">
@@ -52160,13 +52225,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>66308.45</v>
+        <v>65877.62</v>
       </c>
       <c r="D3" t="n">
-        <v>-4.55</v>
+        <v>-5.17</v>
       </c>
       <c r="E3" t="n">
-        <v>46.2</v>
+        <v>45.25</v>
       </c>
     </row>
     <row r="4">
@@ -52198,17 +52263,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>10695.3</v>
+        <v>10724.08</v>
       </c>
       <c r="D5" t="n">
-        <v>1.78</v>
+        <v>2.29</v>
       </c>
       <c r="E5" t="n">
-        <v>16.08</v>
+        <v>15.5</v>
       </c>
     </row>
     <row r="6">
@@ -52219,17 +52284,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>6302.82</v>
+        <v>6307.73</v>
       </c>
       <c r="D6" t="n">
-        <v>1.31</v>
+        <v>1.22</v>
       </c>
       <c r="E6" t="n">
-        <v>15.76</v>
+        <v>14.69</v>
       </c>
     </row>
     <row r="7">
@@ -52240,17 +52305,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>25408.64</v>
+        <v>25420.36</v>
       </c>
       <c r="D7" t="n">
-        <v>2.99</v>
+        <v>3.22</v>
       </c>
       <c r="E7" t="n">
-        <v>7.96</v>
+        <v>7.08</v>
       </c>
     </row>
     <row r="8">
@@ -52265,13 +52330,13 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>24700.5</v>
+        <v>24642.51</v>
       </c>
       <c r="D8" t="n">
-        <v>7.27</v>
+        <v>7.02</v>
       </c>
       <c r="E8" t="n">
-        <v>-5.46</v>
+        <v>-5.69</v>
       </c>
     </row>
   </sheetData>
@@ -52694,7 +52759,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -52938,6 +53003,25 @@
       </c>
       <c r="E12" t="n">
         <v>0.2051</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>16.25</v>
+      </c>
+      <c r="C13" t="n">
+        <v>16.06</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.20517</v>
       </c>
     </row>
   </sheetData>
@@ -54335,25 +54419,25 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.00158</v>
+        <v>0.001586</v>
       </c>
       <c r="C11" t="n">
-        <v>4.63</v>
+        <v>5.03</v>
       </c>
       <c r="D11" t="n">
-        <v>99.23999999999999</v>
+        <v>100.43</v>
       </c>
       <c r="E11" t="n">
-        <v>35.67</v>
+        <v>37.29</v>
       </c>
       <c r="F11" t="n">
-        <v>41.51</v>
+        <v>43.21</v>
       </c>
       <c r="G11" t="n">
-        <v>-1.92</v>
+        <v>-1.89</v>
       </c>
       <c r="H11" t="n">
-        <v>5.06</v>
+        <v>4.71</v>
       </c>
     </row>
   </sheetData>
@@ -58446,7 +58530,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -58729,6 +58813,28 @@
       </c>
       <c r="F12" t="n">
         <v>-5.328</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>16.25</v>
+      </c>
+      <c r="C13" t="n">
+        <v>20.202</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.02405</v>
+      </c>
+      <c r="E13" t="n">
+        <v>28.8</v>
+      </c>
+      <c r="F13" t="n">
+        <v>-3.952</v>
       </c>
     </row>
   </sheetData>
@@ -58987,26 +59093,26 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>3.229</v>
+        <v>3.251</v>
       </c>
       <c r="D4" t="n">
-        <v>3.566</v>
+        <v>3.615</v>
       </c>
       <c r="E4" t="n">
-        <v>0.337</v>
+        <v>0.364</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.104</v>
+        <v>-0.106</v>
       </c>
       <c r="G4" t="n">
-        <v>0.754</v>
+        <v>0.798</v>
       </c>
       <c r="H4" t="n">
-        <v>0.65</v>
+        <v>0.6919999999999999</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -59027,26 +59133,26 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>4.878</v>
+        <v>4.924</v>
       </c>
       <c r="D5" t="n">
-        <v>5.306</v>
+        <v>5.361</v>
       </c>
       <c r="E5" t="n">
-        <v>0.427</v>
+        <v>0.437</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.089</v>
+        <v>-0.098</v>
       </c>
       <c r="G5" t="n">
-        <v>0.651</v>
+        <v>0.697</v>
       </c>
       <c r="H5" t="n">
-        <v>0.5620000000000001</v>
+        <v>0.599</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -65036,10 +65142,10 @@
         <v>0.00881</v>
       </c>
       <c r="C13" t="n">
-        <v>0.06784999999999999</v>
+        <v>0.06857000000000001</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.03833</v>
+        <v>-0.03869</v>
       </c>
     </row>
   </sheetData>
@@ -68213,7 +68319,7 @@
         <v>2.406</v>
       </c>
       <c r="D13" t="n">
-        <v>0.423</v>
+        <v>0.422</v>
       </c>
     </row>
   </sheetData>
@@ -71340,22 +71446,22 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.000294</v>
+        <v>0.00029</v>
       </c>
       <c r="C13" t="n">
-        <v>-0.032546</v>
+        <v>-0.032596</v>
       </c>
       <c r="D13" t="n">
         <v>0.000269</v>
       </c>
       <c r="E13" t="n">
-        <v>5278</v>
+        <v>5277</v>
       </c>
       <c r="F13" t="n">
-        <v>2263</v>
+        <v>2262</v>
       </c>
       <c r="G13" t="n">
-        <v>0.01025</v>
+        <v>0.01024</v>
       </c>
     </row>
   </sheetData>
@@ -71552,14 +71658,14 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.84</v>
+        <v>0.74</v>
       </c>
       <c r="D8" t="n">
-        <v>5.2</v>
+        <v>5.13</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -76443,10 +76549,10 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>-0.0293</v>
+        <v>-0.0294</v>
       </c>
       <c r="D46" t="n">
-        <v>0.011</v>
+        <v>0.0106</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -76466,10 +76572,10 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>-0.0114</v>
+        <v>-0.0113</v>
       </c>
       <c r="D47" t="n">
-        <v>0.3246</v>
+        <v>0.3286</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -76489,10 +76595,10 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>-0.0039</v>
+        <v>-0.0037</v>
       </c>
       <c r="D48" t="n">
-        <v>0.7371</v>
+        <v>0.7453</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -76515,7 +76621,7 @@
         <v>0.0305</v>
       </c>
       <c r="D49" t="n">
-        <v>0.008</v>
+        <v>0.0081</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -77160,13 +77266,13 @@
         <v>89.40000000000001</v>
       </c>
       <c r="D3" t="n">
-        <v>4.06</v>
+        <v>4.11</v>
       </c>
       <c r="E3" t="n">
         <v>3.25</v>
       </c>
       <c r="F3" t="n">
-        <v>0.82</v>
+        <v>0.86</v>
       </c>
     </row>
     <row r="4">
@@ -77179,13 +77285,13 @@
         <v>12.9</v>
       </c>
       <c r="D4" t="n">
-        <v>5.31</v>
+        <v>5.36</v>
       </c>
       <c r="E4" t="n">
         <v>3.09</v>
       </c>
       <c r="F4" t="n">
-        <v>2.22</v>
+        <v>2.27</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-28T12:10Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-28 11:47 UTC</t>
+          <t>Genere le 2026-09-28 12:10 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-28 11:47 UTC</t>
+          <t>Rapport global — 2026-09-28 12:10 UTC</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>**Matieres premieres macro** — le ratio cuivre/or monte -- la croissance domine la peur (+5.0% sur 3 mois). Brent 100.4$ (+37.3% sur 3 mois, +43.2% sur 12 mois), gaz -1.9% sur 3 mois, ecart Brent-WTI +4.7$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-28)_</t>
+          <t>**Matieres premieres macro** — le ratio cuivre/or monte -- la croissance domine la peur (+5.0% sur 3 mois). Brent 100.5$ (+37.4% sur 3 mois, +43.3% sur 12 mois), gaz -1.0% sur 3 mois, ecart Brent-WTI +4.8$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -862,7 +862,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>**Conditions financieres** — indice conditions financieres=+0.121 (3 composantes: {'taux_directeur': 0.5985724560125544, 'courbe_inversee': 0.2531563730537784, 'vix': -0.48919720777532755}) -- conditions proches de la normale _(observation : 2026-09-24)_</t>
+          <t>**Conditions financieres** — indice conditions financieres=+0.122 (3 composantes: {'taux_directeur': 0.5985724560125544, 'courbe_inversee': 0.2531563730537784, 'vix': -0.4867240951306789}) -- conditions proches de la normale _(observation : 2026-09-24)_</t>
         </is>
       </c>
     </row>
@@ -1219,7 +1219,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>**Ornstein uhlenbeck vix** — VIX actuel=16.25, niveau moyen estime (mu)=20.20, demi-vie=28.8j, ecart actuel=-3.95 -- VIX actuel en-dessous de son niveau moyen de long terme _(observation : 2026-09-28)_</t>
+          <t>**Ornstein uhlenbeck vix** — VIX actuel=16.27, niveau moyen estime (mu)=20.20, demi-vie=28.8j, ecart actuel=-3.93 -- VIX actuel en-dessous de son niveau moyen de long terme _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1233,14 +1233,14 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>**Kalman niveau local** — VIX observe=16.25, filtre Kalman=16.06 (ecart-type=0.62), ratio signal/bruit=0.2052 -- le filtre lisse fortement le bruit, reagit lentement (ecart obs.-filtre=+0.19) _(observation : 2026-09-28)_</t>
+          <t>**Kalman niveau local** — VIX observe=16.27, filtre Kalman=16.08 (ecart-type=0.62), ratio signal/bruit=0.2052 -- le filtre lisse fortement le bruit, reagit lentement (ecart obs.-filtre=+0.19) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.37012183452205605 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.05233908530492189 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-25)_</t>
+          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.37012183452189085 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.05233908530492146 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1331,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>**Decomposition stl** — VIX : tendance=15.59, composante saisonniere (periode 5j)=+0.177, residu=+0.480 -- la saisonnalite explique 0.72% de la variance totale (negligeable) _(observation : 2026-09-28)_</t>
+          <t>**Decomposition stl** — VIX : tendance=15.60, composante saisonniere (periode 5j)=+0.181, residu=+0.493 -- la saisonnalite explique 0.72% de la variance totale (negligeable) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -4579,10 +4579,10 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>-0.5789</v>
+        <v>-0.5818</v>
       </c>
       <c r="E58" t="n">
-        <v>0.8757</v>
+        <v>0.875</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
@@ -8239,10 +8239,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>16.25</v>
+        <v>16.27</v>
       </c>
       <c r="D6" t="n">
-        <v>34</v>
+        <v>34.3</v>
       </c>
       <c r="E6" t="n">
         <v>1260</v>
@@ -18979,10 +18979,10 @@
         </is>
       </c>
       <c r="D120" t="n">
-        <v>-2.213</v>
+        <v>-2.2116</v>
       </c>
       <c r="E120" t="n">
-        <v>0.4177</v>
+        <v>0.4184</v>
       </c>
       <c r="F120" t="inlineStr">
         <is>
@@ -19007,10 +19007,10 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>-1.6022</v>
+        <v>-1.6032</v>
       </c>
       <c r="E121" t="n">
-        <v>0.72</v>
+        <v>0.7195</v>
       </c>
       <c r="F121" t="inlineStr">
         <is>
@@ -22122,7 +22122,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1208</v>
+        <v>0.1217</v>
       </c>
       <c r="C13" t="n">
         <v>3</v>
@@ -22134,7 +22134,7 @@
         <v>0.2532</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.4892</v>
+        <v>-0.4867</v>
       </c>
     </row>
   </sheetData>
@@ -34968,19 +34968,19 @@
         <v>2.2</v>
       </c>
       <c r="C13" t="n">
-        <v>468.17</v>
+        <v>468.21</v>
       </c>
       <c r="D13" t="n">
         <v>3</v>
       </c>
       <c r="E13" t="n">
-        <v>416.86</v>
+        <v>416.81</v>
       </c>
       <c r="F13" t="n">
         <v>2.4</v>
       </c>
       <c r="G13" t="n">
-        <v>372.23</v>
+        <v>372.25</v>
       </c>
     </row>
   </sheetData>
@@ -36309,13 +36309,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>15.593</v>
+        <v>15.596</v>
       </c>
       <c r="C13" t="n">
-        <v>0.177</v>
+        <v>0.181</v>
       </c>
       <c r="D13" t="n">
-        <v>0.48</v>
+        <v>0.493</v>
       </c>
       <c r="E13" t="n">
         <v>0.72</v>
@@ -49011,7 +49011,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>fred/ECBDFR.csv</t>
+          <t>fred/RRPONTSYD.csv</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -49040,7 +49040,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>fred/RRPONTSYD.csv</t>
+          <t>fred/T10YIE.csv</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -49069,7 +49069,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>fred/T10YIE.csv</t>
+          <t>marches/volatilite/GVZ.csv</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -49087,7 +49087,7 @@
         <v>42</v>
       </c>
       <c r="F219" t="n">
-        <v>3000</v>
+        <v>3772</v>
       </c>
       <c r="G219" t="inlineStr">
         <is>
@@ -49098,7 +49098,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>marches/volatilite/GVZ.csv</t>
+          <t>marches/volatilite/MOVE.csv</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -49116,7 +49116,7 @@
         <v>42</v>
       </c>
       <c r="F220" t="n">
-        <v>3772</v>
+        <v>3691</v>
       </c>
       <c r="G220" t="inlineStr">
         <is>
@@ -49127,7 +49127,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>marches/volatilite/MOVE.csv</t>
+          <t>marches/volatilite/OVX.csv</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -49145,7 +49145,7 @@
         <v>42</v>
       </c>
       <c r="F221" t="n">
-        <v>3691</v>
+        <v>3772</v>
       </c>
       <c r="G221" t="inlineStr">
         <is>
@@ -49156,7 +49156,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>marches/volatilite/OVX.csv</t>
+          <t>marches/volatilite/VVIX.csv</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -49174,7 +49174,7 @@
         <v>42</v>
       </c>
       <c r="F222" t="n">
-        <v>3772</v>
+        <v>3764</v>
       </c>
       <c r="G222" t="inlineStr">
         <is>
@@ -49185,7 +49185,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>marches/volatilite/VVIX.csv</t>
+          <t>marches/volatilite/VXN.csv</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -49203,7 +49203,7 @@
         <v>42</v>
       </c>
       <c r="F223" t="n">
-        <v>3764</v>
+        <v>3772</v>
       </c>
       <c r="G223" t="inlineStr">
         <is>
@@ -49214,7 +49214,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>marches/volatilite/VXN.csv</t>
+          <t>souverains/SUEDE_10A.csv</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -49232,7 +49232,7 @@
         <v>42</v>
       </c>
       <c r="F224" t="n">
-        <v>3772</v>
+        <v>9202</v>
       </c>
       <c r="G224" t="inlineStr">
         <is>
@@ -49243,7 +49243,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_10A.csv</t>
+          <t>souverains/SUEDE_2A.csv</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
@@ -49272,7 +49272,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_2A.csv</t>
+          <t>souverains/SUEDE_5A.csv</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -49290,7 +49290,7 @@
         <v>42</v>
       </c>
       <c r="F226" t="n">
-        <v>9202</v>
+        <v>9204</v>
       </c>
       <c r="G226" t="inlineStr">
         <is>
@@ -49301,7 +49301,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_5A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -49319,7 +49319,7 @@
         <v>42</v>
       </c>
       <c r="F227" t="n">
-        <v>9204</v>
+        <v>5639</v>
       </c>
       <c r="G227" t="inlineStr">
         <is>
@@ -49330,7 +49330,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -49359,7 +49359,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -49388,7 +49388,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -49417,7 +49417,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -49446,7 +49446,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -49475,7 +49475,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -49504,7 +49504,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -49533,7 +49533,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
+          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -49562,7 +49562,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
+          <t>yfinance/SP500.csv</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -49580,7 +49580,7 @@
         <v>42</v>
       </c>
       <c r="F236" t="n">
-        <v>5639</v>
+        <v>7547</v>
       </c>
       <c r="G236" t="inlineStr">
         <is>
@@ -49591,7 +49591,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>yfinance/SP500.csv</t>
+          <t>yfinance/XLB.csv</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
@@ -49609,7 +49609,7 @@
         <v>42</v>
       </c>
       <c r="F237" t="n">
-        <v>7547</v>
+        <v>501</v>
       </c>
       <c r="G237" t="inlineStr">
         <is>
@@ -49620,7 +49620,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>yfinance/XLB.csv</t>
+          <t>yfinance/XLE.csv</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
@@ -49649,7 +49649,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>yfinance/XLE.csv</t>
+          <t>yfinance/XLF.csv</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
@@ -49678,7 +49678,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>yfinance/XLF.csv</t>
+          <t>yfinance/XLI.csv</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
@@ -49707,7 +49707,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>yfinance/XLI.csv</t>
+          <t>yfinance/XLK.csv</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
@@ -49736,7 +49736,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>yfinance/XLK.csv</t>
+          <t>yfinance/XLP.csv</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
@@ -49765,7 +49765,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>yfinance/XLP.csv</t>
+          <t>yfinance/XLRE.csv</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
@@ -49794,7 +49794,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>yfinance/XLRE.csv</t>
+          <t>yfinance/XLU.csv</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -49823,7 +49823,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>yfinance/XLU.csv</t>
+          <t>yfinance/XLV.csv</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -49852,7 +49852,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>yfinance/XLV.csv</t>
+          <t>yfinance/XLY.csv</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -49881,16 +49881,16 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>yfinance/XLY.csv</t>
+          <t>fred/ECBDFR.csv</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C247" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D247" t="n">
         <v>1</v>
@@ -49899,7 +49899,7 @@
         <v>42</v>
       </c>
       <c r="F247" t="n">
-        <v>501</v>
+        <v>3000</v>
       </c>
       <c r="G247" t="inlineStr">
         <is>
@@ -52267,13 +52267,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>10724.08</v>
+        <v>10730.11</v>
       </c>
       <c r="D5" t="n">
-        <v>2.29</v>
+        <v>2.35</v>
       </c>
       <c r="E5" t="n">
-        <v>15.5</v>
+        <v>15.57</v>
       </c>
     </row>
     <row r="6">
@@ -52288,13 +52288,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>6307.73</v>
+        <v>6310.18</v>
       </c>
       <c r="D6" t="n">
-        <v>1.22</v>
+        <v>1.26</v>
       </c>
       <c r="E6" t="n">
-        <v>14.69</v>
+        <v>14.74</v>
       </c>
     </row>
     <row r="7">
@@ -52309,13 +52309,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>25420.36</v>
+        <v>25417.97</v>
       </c>
       <c r="D7" t="n">
-        <v>3.22</v>
+        <v>3.21</v>
       </c>
       <c r="E7" t="n">
-        <v>7.08</v>
+        <v>7.07</v>
       </c>
     </row>
     <row r="8">
@@ -53012,16 +53012,16 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>16.25</v>
+        <v>16.27</v>
       </c>
       <c r="C13" t="n">
-        <v>16.06</v>
+        <v>16.077</v>
       </c>
       <c r="D13" t="n">
         <v>0.625</v>
       </c>
       <c r="E13" t="n">
-        <v>0.20517</v>
+        <v>0.20518</v>
       </c>
     </row>
   </sheetData>
@@ -54419,25 +54419,25 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.001586</v>
+        <v>0.001585</v>
       </c>
       <c r="C11" t="n">
-        <v>5.03</v>
+        <v>5.02</v>
       </c>
       <c r="D11" t="n">
-        <v>100.43</v>
+        <v>100.53</v>
       </c>
       <c r="E11" t="n">
-        <v>37.29</v>
+        <v>37.43</v>
       </c>
       <c r="F11" t="n">
-        <v>43.21</v>
+        <v>43.35</v>
       </c>
       <c r="G11" t="n">
-        <v>-1.89</v>
+        <v>-1.04</v>
       </c>
       <c r="H11" t="n">
-        <v>4.71</v>
+        <v>4.81</v>
       </c>
     </row>
   </sheetData>
@@ -58822,7 +58822,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>16.25</v>
+        <v>16.27</v>
       </c>
       <c r="C13" t="n">
         <v>20.202</v>
@@ -58834,7 +58834,7 @@
         <v>28.8</v>
       </c>
       <c r="F13" t="n">
-        <v>-3.952</v>
+        <v>-3.932</v>
       </c>
     </row>
   </sheetData>
@@ -65142,10 +65142,10 @@
         <v>0.00881</v>
       </c>
       <c r="C13" t="n">
-        <v>0.06857000000000001</v>
+        <v>0.06859999999999999</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.03869</v>
+        <v>-0.0387</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-28T18:49Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-28 12:10 UTC</t>
+          <t>Genere le 2026-09-28 18:49 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-28 12:10 UTC</t>
+          <t>Rapport global — 2026-09-28 18:49 UTC</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>**Matieres premieres macro** — le ratio cuivre/or monte -- la croissance domine la peur (+5.0% sur 3 mois). Brent 100.5$ (+37.4% sur 3 mois, +43.3% sur 12 mois), gaz -1.0% sur 3 mois, ecart Brent-WTI +4.8$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-28)_</t>
+          <t>**Matieres premieres macro** — le ratio cuivre/or monte -- la croissance domine la peur (+5.4% sur 3 mois). Brent 97.8$ (+33.7% sur 3 mois, +39.4% sur 12 mois), gaz -2.4% sur 3 mois, ecart Brent-WTI +5.2$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -862,7 +862,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>**Conditions financieres** — indice conditions financieres=+0.122 (3 composantes: {'taux_directeur': 0.5985724560125544, 'courbe_inversee': 0.2531563730537784, 'vix': -0.4867240951306789}) -- conditions proches de la normale _(observation : 2026-09-24)_</t>
+          <t>**Conditions financieres** — indice conditions financieres=+0.106 (3 composantes: {'taux_directeur': 0.5985724560125544, 'courbe_inversee': 0.2531563730537784, 'vix': -0.5337130261637928}) -- conditions proches de la normale _(observation : 2026-09-24)_</t>
         </is>
       </c>
     </row>
@@ -911,21 +911,21 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>**Facteur qualite credit** — spread HY=2.80, IG=0.79, ecart=2.01pt (niveau contenu), variation 6m=-13.7% -- se resserre (risque credit percu en baisse) _(observation : 2026-09-24)_</t>
+          <t>**Facteur qualite credit** — spread HY=2.93, IG=0.81, ecart=2.12pt (niveau contenu), variation 6m=-15.5% -- se resserre (risque credit percu en baisse) _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>**Ornstein uhlenbeck credit** — spread HY actuel=2.80, niveau moyen estime=3.02, demi-vie=41.9j, ecart actuel=-0.22 -- spread HY actuel en-dessous de son niveau moyen de long terme _(observation : 2026-09-24)_</t>
+          <t>**Ornstein uhlenbeck credit** — spread HY actuel=2.93, niveau moyen estime=3.02, demi-vie=40.5j, ecart actuel=-0.09 -- spread HY actuel en-dessous de son niveau moyen de long terme _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>**Momentum credit** — momentum credit 12-1 mois=+0.00pt -- stable _(observation : 2026-09-24)_</t>
+          <t>**Momentum credit** — momentum credit 12-1 mois=-0.09pt -- stable _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
@@ -960,14 +960,14 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>**Indices mondiaux** — 7 indices (devise locale) : Coree (KOSPI) +103.5% en tete sur 12 mois, Hong Kong (Hang Seng) -5.7% en queue -- ecart tres large entre blocs sur 12 mois (109pt) -- les cycles economiques ou les flux divergent nettement. ROTATION en cours : Coree (KOSPI) mene sur 12 mois mais Hong Kong (Hang Seng) a repris la tete sur 3 mois _(observation : 2026-09-28)_</t>
+          <t>**Indices mondiaux** — 7 indices (devise locale) : Coree (KOSPI) +103.1% en tete sur 12 mois, Hong Kong (Hang Seng) -7.5% en queue -- ecart tres large entre blocs sur 12 mois (111pt) -- les cycles economiques ou les flux divergent nettement. ROTATION en cours : Coree (KOSPI) mene sur 12 mois mais Hong Kong (Hang Seng) a repris la tete sur 3 mois _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>**Correlation glissante** — correlation glissante 60j SP500/VIX = -0.750 (min=-0.955, max=-0.429 sur la fenetre d'historique disponible) -- dans la zone intermediaire de sa fourchette historique _(observation : 2026-09-25)_</t>
+          <t>**Correlation glissante** — correlation glissante 60j SP500/VIX = -0.752 (min=-0.955, max=-0.429 sur la fenetre d'historique disponible) -- dans la zone intermediaire de sa fourchette historique _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -988,7 +988,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>**Momentum prix** — SP500 momentum 12-1 mois = 16.22% -- haussier (momentum positif), detail 1/3/6/12m = [0.88, 5.29, 21.58, 17.24] _(observation : 2026-09-25)_</t>
+          <t>**Momentum prix** — SP500 momentum 12-1 mois = 16.08% -- haussier (momentum positif), detail 1/3/6/12m = [-0.17, 3.47, 21.35, 15.87] _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1002,56 +1002,56 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>**Beta vol** — beta SP500/VIX (60j) = -0.00484 (rendement SP500 pour +1pt VIX) -- sensibilite normale, relation inverse attendue (normale) _(observation : 2026-09-25)_</t>
+          <t>**Beta vol** — beta SP500/VIX (60j) = -0.00488 (rendement SP500 pour +1pt VIX) -- sensibilite normale, relation inverse attendue (normale) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>**Rotation sectorielle** — classement momentum 3 mois (10 secteurs) : 1. Energie (XLE) : +15.23% | 2. Technologie (XLK) : +8.37% | 3. Sante (XLV) : +6.46% | 4. Finance (XLF) : +2.37% | 5. Consommation de base (XLP) : -3.13% _(observation : 2026-09-25)_</t>
+          <t>**Rotation sectorielle** — classement momentum 3 mois (10 secteurs) : 1. Energie (XLE) : +15.97% | 2. Sante (XLV) : +6.53% | 3. Technologie (XLK) : +5.06% | 4. Finance (XLF) : +1.09% | 5. Materiaux (XLB) : -2.06% _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>**Saisonnalite** — rendement journalier moyen ete=+0.0182%, hiver=+0.0465% (t=-1.02, p=0.3081) -- non significatif (attendu vu la faible puissance sur seulement ~2 ans) _(observation : 2026-09-25)_</t>
+          <t>**Saisonnalite** — rendement journalier moyen ete=+0.0180%, hiver=+0.0465% (t=-1.03, p=0.3047) -- non significatif (attendu vu la faible puissance sur seulement ~2 ans) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>**Dispersion sectorielle** — 10 secteurs, rendement moyen 3m=-0.61%, dispersion (ecart-type)=8.31pt, etendue=29.71pt -- dispersion intermediaire _(observation : 2026-09-25)_</t>
+          <t>**Dispersion sectorielle** — 10 secteurs, rendement moyen 3m=-1.24%, dispersion (ecart-type)=8.31pt, etendue=30.42pt -- dispersion intermediaire _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>**Low volatility** — tercile bas-vol ['XLF', 'XLRE', 'XLU'] Sharpe=-0.566 vs tercile haut-vol ['XLY', 'XLE', 'XLK'] Sharpe=0.218 -- anomalie low-vol non confirmee sur cet echantillon (puissance statistique faible, n petit -- limite assumee) _(observation : 2026-09-25)_</t>
+          <t>**Low volatility** — tercile bas-vol ['XLF', 'XLRE', 'XLU'] Sharpe=-0.682 vs tercile haut-vol ['XLY', 'XLE', 'XLK'] Sharpe=0.175 -- anomalie low-vol non confirmee sur cet echantillon (puissance statistique faible, n petit -- limite assumee) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>**Momentum cross sectional** — panier gagnant ['XLE', 'XLK', 'XLV'] (+10.02%) vs panier perdant ['XLI', 'XLRE', 'XLU'] (-9.52%) -- spread momentum=+19.54pt _(observation : 2026-09-25)_</t>
+          <t>**Momentum cross sectional** — panier gagnant ['XLE', 'XLV', 'XLK'] (+9.18%) vs panier perdant ['XLI', 'XLRE', 'XLU'] (-9.95%) -- spread momentum=+19.13pt _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>**Cointegration secteurs** — 0/10 secteurs cointegres avec SP500 -- decouples : ['XLK', 'XLF', 'XLE', 'XLV', 'XLI', 'XLY', 'XLP', 'XLU', 'XLB', 'XLRE']  _(sans synthese)_ _(observation : 2026-09-25)_</t>
+          <t>**Cointegration secteurs** — 0/10 secteurs cointegres avec SP500 -- decouples : ['XLK', 'XLF', 'XLE', 'XLV', 'XLI', 'XLY', 'XLP', 'XLU', 'XLB', 'XLRE']  _(sans synthese)_ _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>**Correlation facteurs** — correlation entre momentum 3m et beta-VIX, 10 secteurs : +0.062 (facteurs largement independants) _(observation : 2026-09-25)_</t>
+          <t>**Correlation facteurs** — correlation entre momentum 3m et beta-VIX, 10 secteurs : +0.206 (facteurs largement independants) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1107,7 +1107,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>**Divergence cot prix** — SP500 +0.88% sur 30j, COT net -10560 -&gt; -133228 -- DIVERGENCE (prix monte, positionnement recule) _(observation : 2026-09-25)_</t>
+          <t>**Divergence cot prix** — SP500 -0.17% sur 30j, COT net -10560 -&gt; -133228 -- pas de divergence _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1191,56 +1191,56 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>**Vol cross asset** — 6 mesures de volatilite : Petrole (OVX) 88e pct, Or (GVZ) 80e pct, Taux US (MOVE) 43e pct, Nasdaq (VXN) 38e pct, Actions US (VIX) 34e pct, Vol de la vol (VVIX) 27e pct -- stress LOCALISE sur Petrole (OVX), Or (GVZ) pendant que le reste ne l'est pas -- episode propre a cette classe d'actifs, pas une aversion au risque d'ensemble _(observation : 2026-09-28)_</t>
+          <t>**Vol cross asset** — 6 mesures de volatilite : Petrole (OVX) 88e pct, Or (GVZ) 86e pct, Nasdaq (VXN) 48e pct, Taux US (MOVE) 43e pct, Vol de la vol (VVIX) 35e pct, Actions US (VIX) 31e pct -- stress LOCALISE sur Petrole (OVX), Or (GVZ) pendant que le reste ne l'est pas -- episode propre a cette classe d'actifs, pas une aversion au risque d'ensemble _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>**Volatilite ewma** — vol realisee 60j=0.11153026065780319, EWMA=0.1081 (tendance 10 runs: stable) _(observation : 2026-09-25)_</t>
+          <t>**Volatilite ewma** — vol realisee 60j=0.11229567008242833, EWMA=0.1072 (tendance 10 runs: stable) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>**Garch** — vol GARCH(1,1) annualisee=0.1233 (alpha=0.114, beta=0.868, persistance=0.983 -- tres proche de 1 -- chocs de volatilite tres durables) _(observation : 2026-09-25)_</t>
+          <t>**Garch** — vol GARCH(1,1) annualisee=0.1207 (alpha=0.114, beta=0.868, persistance=0.983 -- tres proche de 1 -- chocs de volatilite tres durables) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>**Hurst** — Hurst=0.5535 (R2 regression=1.000) -- persistant (tendanciel) _(observation : 2026-09-25)_</t>
+          <t>**Hurst** — Hurst=0.5507 (R2 regression=1.000) -- persistant (tendanciel) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>**Ornstein uhlenbeck vix** — VIX actuel=16.27, niveau moyen estime (mu)=20.20, demi-vie=28.8j, ecart actuel=-3.93 -- VIX actuel en-dessous de son niveau moyen de long terme _(observation : 2026-09-28)_</t>
+          <t>**Ornstein uhlenbeck vix** — VIX actuel=15.89, niveau moyen estime (mu)=20.20, demi-vie=28.8j, ecart actuel=-4.31 -- VIX actuel en-dessous de son niveau moyen de long terme _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>**Changepoint volatilite** — rupture detectee le 2011-12-21 -- vol avant=0.2129, vol apres=0.1666 (reduction SSE=0.5%) -- baisse de la vol au point de rupture (-21.7%) _(observation : 2026-09-25)_</t>
+          <t>**Changepoint volatilite** — rupture detectee le 2011-12-21 -- vol avant=0.2130, vol apres=0.1666 (reduction SSE=0.5%) -- baisse de la vol au point de rupture (-21.8%) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>**Kalman niveau local** — VIX observe=16.27, filtre Kalman=16.08 (ecart-type=0.62), ratio signal/bruit=0.2052 -- le filtre lisse fortement le bruit, reagit lentement (ecart obs.-filtre=+0.19) _(observation : 2026-09-28)_</t>
+          <t>**Kalman niveau local** — VIX observe=15.89, filtre Kalman=15.75 (ecart-type=0.62), ratio signal/bruit=0.2052 -- le filtre lisse fortement le bruit, reagit lentement (ecart obs.-filtre=+0.14) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.37012183452189085 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.05233908530492146 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-25)_</t>
+          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.37239521716456103 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.05235750065322864 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1254,42 +1254,42 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>**Var drawdown** — VaR95=-1.45% CVaR95=-1.80% VaR99=-2.08% CVaR99=-2.50% drawdown_max_252j=-9.10% -- soit l'equivalent de ~6 jours de VaR95 d'affilee _(observation : 2026-09-25)_</t>
+          <t>**Var drawdown** — VaR95=-1.45% CVaR95=-1.80% VaR99=-2.08% CVaR99=-2.50% drawdown_max_252j=-9.10% -- soit l'equivalent de ~6 jours de VaR95 d'affilee _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>**Skew kurtosis** — skewness=-0.201 (asymetrie negative (pertes extremes &gt; gains extremes)), kurtosis exces=+1.031 (queues epaisses (risque extreme sous-estime par une hypothese normale)) _(observation : 2026-09-25)_</t>
+          <t>**Skew kurtosis** — skewness=-0.201 (asymetrie negative (pertes extremes &gt; gains extremes)), kurtosis exces=+1.026 (queues epaisses (risque extreme sous-estime par une hypothese normale)) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>**Ratios performance** — Sharpe=1.230 (bon), Sortino=1.207 (bon), Calmar=1.755 (bon) -- lecture sur fenetre 252j (~1 an, echantillon limite), seuils academiques standards, taux sans risque suppose nul _(observation : 2026-09-25)_</t>
+          <t>**Ratios performance** — Sharpe=1.139 (bon), Sortino=1.120 (bon), Calmar=1.626 (bon) -- lecture sur fenetre 252j (~1 an, echantillon limite), seuils academiques standards, taux sans risque suppose nul _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>**Covar** — VaR95 inconditionnelle=-1.84%, VaR95|VIX detresse(&gt;=29.5)=-4.37%, VaR95|VIX normal=-1.52% -- DeltaCoVaR=-2.86pt (755 jours de detresse dans l'echantillon) -- contagion notable -- VaR 2.9x plus severe en detresse _(observation : 2026-09-25)_</t>
+          <t>**Covar** — VaR95 inconditionnelle=-1.84%, VaR95|VIX detresse(&gt;=29.5)=-4.37%, VaR95|VIX normal=-1.52% -- DeltaCoVaR=-2.86pt (755 jours de detresse dans l'echantillon) -- contagion notable -- VaR 2.9x plus severe en detresse _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>**Stress test historique** — COVID_2020 (2020-02-19 -&gt; 2020-03-23) : chute historique=-33.9% -- rejouee sur le niveau actuel (7743) -&gt; 5116  _(sans synthese)_ _(observation : 2026-09-25)_</t>
+          <t>**Stress test historique** — COVID_2020 (2020-02-19 -&gt; 2020-03-23) : chute historique=-33.9% -- rejouee sur le niveau actuel (7698) -&gt; 5087  _(sans synthese)_ _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>**Sizing robuste** — vol point estimate=0.1297, IC90%=[0.1184, 0.1411] (1000 tirages bootstrap) -- intervalle etroit (17% du point estimate) -- estimation relativement fiable _(observation : 2026-09-25)_</t>
+          <t>**Sizing robuste** — vol point estimate=0.1298, IC90%=[0.1171, 0.1412] (1000 tirages bootstrap) -- intervalle etroit (19% du point estimate) -- estimation relativement fiable _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1303,7 +1303,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>**Detection saut** — Z-stat BNS (fenetre 22j)=1.336 (seuil ±1.96) -- pas de saut isole detecte _(observation : 2026-09-25)_</t>
+          <t>**Detection saut** — Z-stat BNS (fenetre 22j)=1.206 (seuil ±1.96) -- pas de saut isole detecte _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1317,35 +1317,35 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>**Qualite regime macro** — instabilite taux=0.0088, instabilite VIX=0.0686 -- score qualite du regime=-0.0387 (plus haut = regime plus stable/previsible) _(observation : 2026-09-24)_</t>
+          <t>**Qualite regime macro** — instabilite taux=0.0088, instabilite VIX=0.0682 -- score qualite du regime=-0.0385 (plus haut = regime plus stable/previsible) _(observation : 2026-09-24)_</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>**Var conditionnelle regime** — regime VIX actuel=bas (rang percentile=32) -- VaR95 applicable maintenant=-1.14% (vs VaR95 globale non-conditionnelle=-1.84%) _(observation : 2026-09-25)_</t>
+          <t>**Var conditionnelle regime** — regime VIX actuel=bas (rang percentile=32) -- VaR95 applicable maintenant=-1.14% (vs VaR95 globale non-conditionnelle=-1.84%) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>**Decomposition stl** — VIX : tendance=15.60, composante saisonniere (periode 5j)=+0.181, residu=+0.493 -- la saisonnalite explique 0.72% de la variance totale (negligeable) _(observation : 2026-09-28)_</t>
+          <t>**Decomposition stl** — VIX : tendance=15.52, composante saisonniere (periode 5j)=+0.101, residu=+0.266 -- la saisonnalite explique 0.72% de la variance totale (negligeable) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>**Ratios conditionnels regime** — Sharpe regime haut-vol=-1.107, bas-vol=2.406, global=0.422 -- meilleur en regime calme, comme attendu _(observation : 2026-09-25)_</t>
+          <t>**Ratios conditionnels regime** — Sharpe regime haut-vol=-1.107, bas-vol=2.403, global=0.421 -- meilleur en regime calme, comme attendu _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>**Choc vol parametrique** — vol actuelle=12.97%, scenarios x1/x2/x3 calcules -- pire scenario (x3) = -3.97%/jour, soit 3.1x le scenario de base _(observation : 2026-09-25)_</t>
+          <t>**Choc vol parametrique** — vol actuelle=12.98%, scenarios x1/x2/x3 calcules -- pire scenario (x3) = -3.97%/jour, soit 3.1x le scenario de base _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1366,42 +1366,42 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>**Causalite granger** — causalite Granger detectee : SP500_cause_VIX (lag=5) _(observation : 2026-09-25)_</t>
+          <t>**Causalite granger** — causalite Granger detectee : SP500_cause_VIX (lag=5) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>**Dependance queue** — 518/7544 jours conjointement extremes (SP500 pire 10% ET VIX pire 10%), P observee=0.0687 vs P sous independance=0.0100 -- coefficient de dependance de queue=6.87 (dependance reelle) _(observation : 2026-09-25)_</t>
+          <t>**Dependance queue** — 518/7545 jours conjointement extremes (SP500 pire 10% ET VIX pire 10%), P observee=0.0687 vs P sous independance=0.0100 -- coefficient de dependance de queue=6.87 (dependance reelle) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>**Walkforward direction** — 7516 predictions walk-forward -- momentum 5j=0.4960 vs baseline majoritaire=0.5375 -- NE BAT PAS la baseline (resultat honnete, pas ajuste pour paraitre mieux) _(observation : 2026-09-25)_</t>
+          <t>**Walkforward direction** — 7515 predictions walk-forward -- momentum 5j=0.4958 vs baseline majoritaire=0.5373 -- NE BAT PAS la baseline (resultat honnete, pas ajuste pour paraitre mieux) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>**Anomalie multivariee** — distance de Mahalanobis=0.557 (seuil 3.0) -- jour ordinaire _(observation : 2026-09-25)_</t>
+          <t>**Anomalie multivariee** — distance de Mahalanobis=0.788 (seuil 3.0) -- jour ordinaire _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>**Test overfitting** — meilleure fenetre in-sample=23j (accuracy=0.5164) vs meme fenetre en walk-forward=0.5162 -- ecart=+0.0002 (ecart faible) _(observation : 2026-09-25)_</t>
+          <t>**Test overfitting** — meilleure fenetre in-sample=23j (accuracy=0.5164) vs meme fenetre en walk-forward=0.5160 -- ecart=+0.0003 (ecart faible) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>**Prevision vol regression** — regression AR(1) (a=0.000116, b=0.2096) MSE=2.9848e-07 vs baseline persistance MSE=3.8343e-07 -- BAT la baseline (resultat honnete, pas ajuste) _(observation : 2026-09-25)_</t>
+          <t>**Prevision vol regression** — regression AR(1) (a=0.000116, b=0.2096) MSE=2.9848e-07 vs baseline persistance MSE=3.8343e-07 -- BAT la baseline (resultat honnete, pas ajuste) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1415,28 +1415,28 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>**Ensemble signaux** — 7514 predictions -- momentum=0.4959, vix=0.4988, ensemble=0.4988, baseline=0.5374 -- ensemble NE BAT PAS la baseline _(observation : 2026-09-25)_</t>
+          <t>**Ensemble signaux** — 7515 predictions -- momentum=0.4958, vix=0.4987, ensemble=0.4987, baseline=0.5373 -- ensemble NE BAT PAS la baseline _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>**Screening features** — 2/4 features avec un lien univarie significatif (p&lt;0.05, sans correction multiple-testing ici -- seulement 4 tests)  _(sans synthese)_ _(observation : 2026-09-25)_</t>
+          <t>**Screening features** — 2/4 features avec un lien univarie significatif (p&lt;0.05, sans correction multiple-testing ici -- seulement 4 tests)  _(sans synthese)_ _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>**Couts transaction** — 7516 predictions, 1512 changements de position (5pb/changement) -- rendement cumule brut=-93.11%, cout total=53.05%, net=-96.76% -- les frais mangent une part importante du rendement (&gt;50% du brut) _(observation : 2026-09-25)_</t>
+          <t>**Couts transaction** — 7515 predictions, 1512 changements de position (5pb/changement) -- rendement cumule brut=-93.19%, cout total=53.05%, net=-96.80% -- les frais mangent une part importante du rendement (&gt;50% du brut) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>**Regression multifeatures** — coefs (intercept=0.00029, momentum5j=-0.0326, var_vix=0.00027) -- R2 out-of-sample=0.0102 (modele bat la moyenne) _(observation : 2026-09-25)_</t>
+          <t>**Regression multifeatures** — coefs (intercept=0.00029, momentum5j=-0.0326, var_vix=0.00027) -- R2 out-of-sample=0.0103 (modele bat la moyenne) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1464,21 +1464,21 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>**Stacking** — poids appris (momentum=-0.080, baseline=0.090, biais=0.090) -- accuracy stacking=0.5463 vs momentum seul=0.5024, baseline seule=0.5463 sur 2255 points test -- stacking NE BAT PAS la baseline, meilleur=stacking / baseline (ex-aequo) _(observation : 2026-09-25)_</t>
+          <t>**Stacking** — poids appris (momentum=-0.081, baseline=0.090, biais=0.090) -- accuracy stacking=0.5459 vs momentum seul=0.5020, baseline seule=0.5459 sur 2255 points test -- stacking NE BAT PAS la baseline, meilleur=stacking / baseline (ex-aequo) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>**Decision stump** — seuil appris=-1.530 (sens=False) -- accuracy stump=0.5457 vs baseline=0.5475 sur 2263 points test -- stump NE BAT PAS la baseline _(observation : 2026-09-25)_</t>
+          <t>**Decision stump** — seuil appris=-1.530 (sens=False) -- accuracy stump=0.5455 vs baseline=0.5473 sur 2264 points test -- stump NE BAT PAS la baseline _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>**Importance permutation** — R2 base=0.0102 -- importance momentum5j=-0.00094, importance variation_vix=0.01231 -- VIX plus important _(observation : 2026-09-25)_</t>
+          <t>**Importance permutation** — R2 base=0.0103 -- importance momentum5j=0.00041, importance variation_vix=0.01282 -- VIX plus important _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -2549,7 +2549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2938,6 +2938,34 @@
       </c>
       <c r="H13" t="n">
         <v>0.5463</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>-0.0809</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.08989999999999999</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.08989999999999999</v>
+      </c>
+      <c r="E14" t="n">
+        <v>2255</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.5459000000000001</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.502</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.5459000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -4685,7 +4713,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5398,6 +5426,62 @@
       </c>
       <c r="F25" t="n">
         <v>5116.46</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>GFC_2008</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>2007-10-09</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>2009-03-09</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>-56.78</v>
+      </c>
+      <c r="F26" t="n">
+        <v>3327.59</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>COVID_2020</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>2020-02-19</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>2020-03-23</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>-33.92</v>
+      </c>
+      <c r="F27" t="n">
+        <v>5086.7</v>
       </c>
     </row>
   </sheetData>
@@ -6053,7 +6137,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6316,6 +6400,25 @@
       </c>
       <c r="E13" t="n">
         <v>0.0002</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>23</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.5164</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.516</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.0003</v>
       </c>
     </row>
   </sheetData>
@@ -6667,7 +6770,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6888,6 +6991,22 @@
       </c>
       <c r="D13" t="n">
         <v>0.00433</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>5</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.07575999999999999</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.00419</v>
       </c>
     </row>
   </sheetData>
@@ -7144,7 +7263,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7517,6 +7636,33 @@
         <v>-1.141</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>bas</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="D14" t="n">
+        <v>-2.847</v>
+      </c>
+      <c r="E14" t="n">
+        <v>-1.141</v>
+      </c>
+      <c r="F14" t="n">
+        <v>-1.845</v>
+      </c>
+      <c r="G14" t="n">
+        <v>-1.141</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7528,7 +7674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7835,6 +7981,28 @@
         <v>-9.098000000000001</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>-1.447</v>
+      </c>
+      <c r="C14" t="n">
+        <v>-1.803</v>
+      </c>
+      <c r="D14" t="n">
+        <v>-2.084</v>
+      </c>
+      <c r="E14" t="n">
+        <v>-2.504</v>
+      </c>
+      <c r="F14" t="n">
+        <v>-9.098000000000001</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7846,7 +8014,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8067,6 +8235,22 @@
       </c>
       <c r="D13" t="n">
         <v>-0.052339</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>10</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.3724</v>
+      </c>
+      <c r="D14" t="n">
+        <v>-0.052358</v>
       </c>
     </row>
   </sheetData>
@@ -8131,14 +8315,14 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>55.09</v>
+        <v>55.65</v>
       </c>
       <c r="D2" t="n">
-        <v>87.90000000000001</v>
+        <v>88.3</v>
       </c>
       <c r="E2" t="n">
         <v>1260</v>
@@ -8157,14 +8341,14 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>22.44</v>
+        <v>24.65</v>
       </c>
       <c r="D3" t="n">
-        <v>80.2</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="E3" t="n">
         <v>1260</v>
@@ -8178,19 +8362,19 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Taux US (MOVE)</t>
+          <t>Nasdaq (VXN)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>96</v>
+        <v>22.17</v>
       </c>
       <c r="D4" t="n">
-        <v>43.3</v>
+        <v>48</v>
       </c>
       <c r="E4" t="n">
         <v>1260</v>
@@ -8204,7 +8388,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Nasdaq (VXN)</t>
+          <t>Taux US (MOVE)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -8213,10 +8397,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>20.87</v>
+        <v>96</v>
       </c>
       <c r="D5" t="n">
-        <v>37.5</v>
+        <v>43.3</v>
       </c>
       <c r="E5" t="n">
         <v>1260</v>
@@ -8230,7 +8414,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Actions US (VIX)</t>
+          <t>Vol de la vol (VVIX)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -8239,10 +8423,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>16.27</v>
+        <v>90.47</v>
       </c>
       <c r="D6" t="n">
-        <v>34.3</v>
+        <v>35.2</v>
       </c>
       <c r="E6" t="n">
         <v>1260</v>
@@ -8256,19 +8440,19 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Vol de la vol (VVIX)</t>
+          <t>Actions US (VIX)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>87.84</v>
+        <v>15.89</v>
       </c>
       <c r="D7" t="n">
-        <v>27.3</v>
+        <v>30.9</v>
       </c>
       <c r="E7" t="n">
         <v>1260</v>
@@ -8290,7 +8474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8555,6 +8739,25 @@
         <v>0.1115</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.1072</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.0804</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.1096</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.1123</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8566,7 +8769,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8855,6 +9058,27 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>7515</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.4958</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.5373</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8866,7 +9090,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9152,6 +9376,27 @@
         <v>0.1666</v>
       </c>
       <c r="E13" t="n">
+        <v>0.0048</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2011-12-21</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>0.213</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.1666</v>
+      </c>
+      <c r="E14" t="n">
         <v>0.0048</v>
       </c>
     </row>
@@ -10708,7 +10953,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10971,6 +11216,25 @@
       </c>
       <c r="E13" t="n">
         <v>-3.972</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>12.976</v>
+      </c>
+      <c r="C14" t="n">
+        <v>-1.284</v>
+      </c>
+      <c r="D14" t="n">
+        <v>-2.629</v>
+      </c>
+      <c r="E14" t="n">
+        <v>-3.973</v>
       </c>
     </row>
   </sheetData>
@@ -12807,7 +13071,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E121"/>
+  <dimension ref="A1:E131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -15599,6 +15863,236 @@
         <v>0.7732</v>
       </c>
       <c r="E121" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>XLK</t>
+        </is>
+      </c>
+      <c r="C122" t="n">
+        <v>-2.5552</v>
+      </c>
+      <c r="D122" t="n">
+        <v>0.2553</v>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>XLF</t>
+        </is>
+      </c>
+      <c r="C123" t="n">
+        <v>-1.8586</v>
+      </c>
+      <c r="D123" t="n">
+        <v>0.6008</v>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>XLE</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>-2.142</v>
+      </c>
+      <c r="D124" t="n">
+        <v>0.4545</v>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>XLV</t>
+        </is>
+      </c>
+      <c r="C125" t="n">
+        <v>-2.3931</v>
+      </c>
+      <c r="D125" t="n">
+        <v>0.3281</v>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>XLI</t>
+        </is>
+      </c>
+      <c r="C126" t="n">
+        <v>-1.3476</v>
+      </c>
+      <c r="D126" t="n">
+        <v>0.8149</v>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>XLY</t>
+        </is>
+      </c>
+      <c r="C127" t="n">
+        <v>0.06279999999999999</v>
+      </c>
+      <c r="D127" t="n">
+        <v>0.9873</v>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>XLP</t>
+        </is>
+      </c>
+      <c r="C128" t="n">
+        <v>-1.204</v>
+      </c>
+      <c r="D128" t="n">
+        <v>0.8568</v>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>XLU</t>
+        </is>
+      </c>
+      <c r="C129" t="n">
+        <v>-0.5289</v>
+      </c>
+      <c r="D129" t="n">
+        <v>0.9622000000000001</v>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>XLB</t>
+        </is>
+      </c>
+      <c r="C130" t="n">
+        <v>-2.1897</v>
+      </c>
+      <c r="D130" t="n">
+        <v>0.4297</v>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>XLRE</t>
+        </is>
+      </c>
+      <c r="C131" t="n">
+        <v>-1.6061</v>
+      </c>
+      <c r="D131" t="n">
+        <v>0.7183</v>
+      </c>
+      <c r="E131" t="inlineStr">
         <is>
           <t>False</t>
         </is>
@@ -22122,7 +22616,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1217</v>
+        <v>0.106</v>
       </c>
       <c r="C13" t="n">
         <v>3</v>
@@ -22134,7 +22628,7 @@
         <v>0.2532</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.4867</v>
+        <v>-0.5337</v>
       </c>
     </row>
   </sheetData>
@@ -22218,7 +22712,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -22397,6 +22891,19 @@
       </c>
       <c r="C13" t="n">
         <v>0.0619</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>10</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.2065</v>
       </c>
     </row>
   </sheetData>
@@ -22410,7 +22917,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -22547,6 +23054,16 @@
       </c>
       <c r="B13" t="n">
         <v>-0.7498</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>-0.7519</v>
       </c>
     </row>
   </sheetData>
@@ -34316,7 +34833,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -34621,6 +35138,28 @@
       </c>
       <c r="F13" t="n">
         <v>-96.76000000000001</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>7515</v>
+      </c>
+      <c r="C14" t="n">
+        <v>1512</v>
+      </c>
+      <c r="D14" t="n">
+        <v>53.05</v>
+      </c>
+      <c r="E14" t="n">
+        <v>-93.19</v>
+      </c>
+      <c r="F14" t="n">
+        <v>-96.8</v>
       </c>
     </row>
   </sheetData>
@@ -34968,19 +35507,19 @@
         <v>2.2</v>
       </c>
       <c r="C13" t="n">
-        <v>468.21</v>
+        <v>467.44</v>
       </c>
       <c r="D13" t="n">
         <v>3</v>
       </c>
       <c r="E13" t="n">
-        <v>416.81</v>
+        <v>417.73</v>
       </c>
       <c r="F13" t="n">
         <v>2.4</v>
       </c>
       <c r="G13" t="n">
-        <v>372.25</v>
+        <v>371.99</v>
       </c>
     </row>
   </sheetData>
@@ -34994,7 +35533,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -35340,6 +35879,31 @@
         <v>-2.858</v>
       </c>
       <c r="G13" t="n">
+        <v>755</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>29.55</v>
+      </c>
+      <c r="C14" t="n">
+        <v>-1.845</v>
+      </c>
+      <c r="D14" t="n">
+        <v>-4.373</v>
+      </c>
+      <c r="E14" t="n">
+        <v>-1.515</v>
+      </c>
+      <c r="F14" t="n">
+        <v>-2.858</v>
+      </c>
+      <c r="G14" t="n">
         <v>755</v>
       </c>
     </row>
@@ -35714,7 +36278,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -36043,6 +36607,30 @@
       </c>
       <c r="F13" t="n">
         <v>0.5475</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>-1.53</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>2264</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.5455</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.5473</v>
       </c>
     </row>
   </sheetData>
@@ -36309,13 +36897,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>15.596</v>
+        <v>15.523</v>
       </c>
       <c r="C13" t="n">
-        <v>0.181</v>
+        <v>0.101</v>
       </c>
       <c r="D13" t="n">
-        <v>0.493</v>
+        <v>0.266</v>
       </c>
       <c r="E13" t="n">
         <v>0.72</v>
@@ -36524,7 +37112,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -36831,6 +37419,28 @@
         <v>6.87</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>7545</v>
+      </c>
+      <c r="C14" t="n">
+        <v>518</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.06865</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F14" t="n">
+        <v>6.87</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -36842,7 +37452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -37086,6 +37696,24 @@
         </is>
       </c>
       <c r="D13" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1.206</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
         <v>22</v>
       </c>
     </row>
@@ -37392,7 +38020,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -37681,6 +38309,27 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>-0.00583</v>
+      </c>
+      <c r="C14" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.788</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -37692,7 +38341,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -37957,6 +38606,25 @@
         <v>29.711</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>10</v>
+      </c>
+      <c r="C14" t="n">
+        <v>-1.238</v>
+      </c>
+      <c r="D14" t="n">
+        <v>8.31</v>
+      </c>
+      <c r="E14" t="n">
+        <v>30.417</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -37968,7 +38636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -38254,6 +38922,27 @@
       <c r="E13" t="inlineStr">
         <is>
           <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>-0.174</v>
+      </c>
+      <c r="C14" t="n">
+        <v>-133228</v>
+      </c>
+      <c r="D14" t="n">
+        <v>-10560</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -38993,7 +39682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -39298,6 +39987,28 @@
       </c>
       <c r="F13" t="n">
         <v>0.5374</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>7515</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.4958</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.4987</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.4987</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.5373</v>
       </c>
     </row>
   </sheetData>
@@ -42148,7 +42859,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -42411,6 +43122,25 @@
       </c>
       <c r="E13" t="n">
         <v>-13.7</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="D14" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="E14" t="n">
+        <v>-15.5</v>
       </c>
     </row>
   </sheetData>
@@ -48025,7 +48755,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>souverains/AUSTRALIE_10A.csv</t>
+          <t>marches/indices/KOSPI.csv</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -48043,7 +48773,7 @@
         <v>42</v>
       </c>
       <c r="F183" t="n">
-        <v>3361</v>
+        <v>3680</v>
       </c>
       <c r="G183" t="inlineStr">
         <is>
@@ -48054,7 +48784,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>souverains/AUSTRALIE_2A.csv</t>
+          <t>souverains/AUSTRALIE_10A.csv</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -48072,7 +48802,7 @@
         <v>42</v>
       </c>
       <c r="F184" t="n">
-        <v>3283</v>
+        <v>3361</v>
       </c>
       <c r="G184" t="inlineStr">
         <is>
@@ -48083,7 +48813,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>souverains/AUSTRALIE_5A.csv</t>
+          <t>souverains/AUSTRALIE_2A.csv</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -48112,16 +48842,16 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>fred/BAMLC0A0CM.csv</t>
+          <t>souverains/AUSTRALIE_5A.csv</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="C186" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D186" t="n">
         <v>1</v>
@@ -48130,7 +48860,7 @@
         <v>42</v>
       </c>
       <c r="F186" t="n">
-        <v>795</v>
+        <v>3283</v>
       </c>
       <c r="G186" t="inlineStr">
         <is>
@@ -48141,7 +48871,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>fred/BAMLC0A0CMEY.csv</t>
+          <t>fred/DFF.csv</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -48159,7 +48889,7 @@
         <v>42</v>
       </c>
       <c r="F187" t="n">
-        <v>795</v>
+        <v>3000</v>
       </c>
       <c r="G187" t="inlineStr">
         <is>
@@ -48170,7 +48900,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>fred/BAMLEMCBPIOAS.csv</t>
+          <t>fred/DFII10.csv</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -48188,7 +48918,7 @@
         <v>42</v>
       </c>
       <c r="F188" t="n">
-        <v>795</v>
+        <v>3000</v>
       </c>
       <c r="G188" t="inlineStr">
         <is>
@@ -48199,7 +48929,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>fred/BAMLEMFSFCRPIOAS.csv</t>
+          <t>fred/DFII5.csv</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -48217,7 +48947,7 @@
         <v>42</v>
       </c>
       <c r="F189" t="n">
-        <v>795</v>
+        <v>3000</v>
       </c>
       <c r="G189" t="inlineStr">
         <is>
@@ -48228,7 +48958,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>fred/BAMLEMHBHYCRPIOAS.csv</t>
+          <t>fred/DGS1.csv</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -48246,7 +48976,7 @@
         <v>42</v>
       </c>
       <c r="F190" t="n">
-        <v>795</v>
+        <v>3000</v>
       </c>
       <c r="G190" t="inlineStr">
         <is>
@@ -48257,7 +48987,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>fred/BAMLEMPBPUBSICRPIOAS.csv</t>
+          <t>fred/DGS10.csv</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -48275,7 +49005,7 @@
         <v>42</v>
       </c>
       <c r="F191" t="n">
-        <v>795</v>
+        <v>3000</v>
       </c>
       <c r="G191" t="inlineStr">
         <is>
@@ -48286,7 +49016,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>fred/BAMLH0A0HYM2.csv</t>
+          <t>fred/DGS1MO.csv</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -48304,7 +49034,7 @@
         <v>42</v>
       </c>
       <c r="F192" t="n">
-        <v>795</v>
+        <v>3000</v>
       </c>
       <c r="G192" t="inlineStr">
         <is>
@@ -48315,7 +49045,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>fred/BAMLHE00EHYIEY.csv</t>
+          <t>fred/DGS2.csv</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -48333,7 +49063,7 @@
         <v>42</v>
       </c>
       <c r="F193" t="n">
-        <v>795</v>
+        <v>3000</v>
       </c>
       <c r="G193" t="inlineStr">
         <is>
@@ -48344,7 +49074,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>fred/BAMLHE00EHYIOAS.csv</t>
+          <t>fred/DGS30.csv</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -48362,7 +49092,7 @@
         <v>42</v>
       </c>
       <c r="F194" t="n">
-        <v>795</v>
+        <v>3000</v>
       </c>
       <c r="G194" t="inlineStr">
         <is>
@@ -48373,7 +49103,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>fred/DFF.csv</t>
+          <t>fred/DGS3MO.csv</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -48402,7 +49132,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>fred/DFII10.csv</t>
+          <t>fred/DGS5.csv</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -48431,7 +49161,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>fred/DFII5.csv</t>
+          <t>fred/DGS6MO.csv</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -48460,7 +49190,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>fred/DGS1.csv</t>
+          <t>fred/IUDSOIA.csv</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -48489,7 +49219,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>fred/DGS10.csv</t>
+          <t>fred/MORTGAGE30US.csv</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -48501,13 +49231,13 @@
         <v>4</v>
       </c>
       <c r="D199" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E199" t="n">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="F199" t="n">
-        <v>3000</v>
+        <v>2896</v>
       </c>
       <c r="G199" t="inlineStr">
         <is>
@@ -48518,7 +49248,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>fred/DGS1MO.csv</t>
+          <t>souverains/UK_10A.csv</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -48536,7 +49266,7 @@
         <v>42</v>
       </c>
       <c r="F200" t="n">
-        <v>3000</v>
+        <v>9283</v>
       </c>
       <c r="G200" t="inlineStr">
         <is>
@@ -48547,7 +49277,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>fred/DGS2.csv</t>
+          <t>souverains/UK_20A.csv</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -48565,7 +49295,7 @@
         <v>42</v>
       </c>
       <c r="F201" t="n">
-        <v>3000</v>
+        <v>6754</v>
       </c>
       <c r="G201" t="inlineStr">
         <is>
@@ -48576,7 +49306,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>fred/DGS30.csv</t>
+          <t>souverains/UK_5A.csv</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -48594,7 +49324,7 @@
         <v>42</v>
       </c>
       <c r="F202" t="n">
-        <v>3000</v>
+        <v>8291</v>
       </c>
       <c r="G202" t="inlineStr">
         <is>
@@ -48605,7 +49335,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>fred/DGS3MO.csv</t>
+          <t>tresor_us/dette_quotidienne.csv</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -48623,7 +49353,7 @@
         <v>42</v>
       </c>
       <c r="F203" t="n">
-        <v>3000</v>
+        <v>2000</v>
       </c>
       <c r="G203" t="inlineStr">
         <is>
@@ -48634,7 +49364,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>fred/DGS5.csv</t>
+          <t>tresor_us/solde_tresorerie.csv</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
@@ -48652,7 +49382,7 @@
         <v>42</v>
       </c>
       <c r="F204" t="n">
-        <v>3000</v>
+        <v>500</v>
       </c>
       <c r="G204" t="inlineStr">
         <is>
@@ -48663,16 +49393,16 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>fred/DGS6MO.csv</t>
+          <t>fred/BAMLC0A0CM.csv</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C205" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D205" t="n">
         <v>1</v>
@@ -48681,7 +49411,7 @@
         <v>42</v>
       </c>
       <c r="F205" t="n">
-        <v>3000</v>
+        <v>793</v>
       </c>
       <c r="G205" t="inlineStr">
         <is>
@@ -48692,16 +49422,16 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>fred/IUDSOIA.csv</t>
+          <t>fred/BAMLC0A0CMEY.csv</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C206" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D206" t="n">
         <v>1</v>
@@ -48710,7 +49440,7 @@
         <v>42</v>
       </c>
       <c r="F206" t="n">
-        <v>3000</v>
+        <v>793</v>
       </c>
       <c r="G206" t="inlineStr">
         <is>
@@ -48721,25 +49451,25 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>fred/MORTGAGE30US.csv</t>
+          <t>fred/BAMLEMCBPIOAS.csv</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C207" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D207" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E207" t="n">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="F207" t="n">
-        <v>2896</v>
+        <v>793</v>
       </c>
       <c r="G207" t="inlineStr">
         <is>
@@ -48750,16 +49480,16 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>souverains/CANADA_10A.csv</t>
+          <t>fred/BAMLEMFSFCRPIOAS.csv</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C208" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D208" t="n">
         <v>1</v>
@@ -48768,7 +49498,7 @@
         <v>42</v>
       </c>
       <c r="F208" t="n">
-        <v>6435</v>
+        <v>793</v>
       </c>
       <c r="G208" t="inlineStr">
         <is>
@@ -48779,16 +49509,16 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>souverains/CANADA_2A.csv</t>
+          <t>fred/BAMLEMHBHYCRPIOAS.csv</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C209" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D209" t="n">
         <v>1</v>
@@ -48797,7 +49527,7 @@
         <v>42</v>
       </c>
       <c r="F209" t="n">
-        <v>6434</v>
+        <v>793</v>
       </c>
       <c r="G209" t="inlineStr">
         <is>
@@ -48808,16 +49538,16 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>souverains/CANADA_5A.csv</t>
+          <t>fred/BAMLEMPBPUBSICRPIOAS.csv</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C210" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D210" t="n">
         <v>1</v>
@@ -48826,7 +49556,7 @@
         <v>42</v>
       </c>
       <c r="F210" t="n">
-        <v>6434</v>
+        <v>793</v>
       </c>
       <c r="G210" t="inlineStr">
         <is>
@@ -48837,16 +49567,16 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>souverains/CANADA_LONG.csv</t>
+          <t>fred/BAMLH0A0HYM2.csv</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C211" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D211" t="n">
         <v>1</v>
@@ -48855,7 +49585,7 @@
         <v>42</v>
       </c>
       <c r="F211" t="n">
-        <v>6434</v>
+        <v>793</v>
       </c>
       <c r="G211" t="inlineStr">
         <is>
@@ -48866,16 +49596,16 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>souverains/UK_10A.csv</t>
+          <t>fred/BAMLHE00EHYIEY.csv</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C212" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D212" t="n">
         <v>1</v>
@@ -48884,7 +49614,7 @@
         <v>42</v>
       </c>
       <c r="F212" t="n">
-        <v>9283</v>
+        <v>793</v>
       </c>
       <c r="G212" t="inlineStr">
         <is>
@@ -48895,16 +49625,16 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>souverains/UK_20A.csv</t>
+          <t>fred/BAMLHE00EHYIOAS.csv</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C213" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D213" t="n">
         <v>1</v>
@@ -48913,7 +49643,7 @@
         <v>42</v>
       </c>
       <c r="F213" t="n">
-        <v>6754</v>
+        <v>793</v>
       </c>
       <c r="G213" t="inlineStr">
         <is>
@@ -48924,16 +49654,16 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>souverains/UK_5A.csv</t>
+          <t>fred/T10YIE.csv</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C214" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D214" t="n">
         <v>1</v>
@@ -48942,7 +49672,7 @@
         <v>42</v>
       </c>
       <c r="F214" t="n">
-        <v>8291</v>
+        <v>3000</v>
       </c>
       <c r="G214" t="inlineStr">
         <is>
@@ -48953,16 +49683,16 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>tresor_us/dette_quotidienne.csv</t>
+          <t>marches/indices/HANGSENG.csv</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C215" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D215" t="n">
         <v>1</v>
@@ -48971,7 +49701,7 @@
         <v>42</v>
       </c>
       <c r="F215" t="n">
-        <v>2000</v>
+        <v>3688</v>
       </c>
       <c r="G215" t="inlineStr">
         <is>
@@ -48982,16 +49712,16 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>tresor_us/solde_tresorerie.csv</t>
+          <t>marches/indices/NIKKEI225.csv</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C216" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D216" t="n">
         <v>1</v>
@@ -49000,7 +49730,7 @@
         <v>42</v>
       </c>
       <c r="F216" t="n">
-        <v>500</v>
+        <v>3666</v>
       </c>
       <c r="G216" t="inlineStr">
         <is>
@@ -49011,7 +49741,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>fred/RRPONTSYD.csv</t>
+          <t>marches/volatilite/MOVE.csv</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -49029,7 +49759,7 @@
         <v>42</v>
       </c>
       <c r="F217" t="n">
-        <v>3000</v>
+        <v>3689</v>
       </c>
       <c r="G217" t="inlineStr">
         <is>
@@ -49040,7 +49770,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>fred/T10YIE.csv</t>
+          <t>souverains/CANADA_10A.csv</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -49058,7 +49788,7 @@
         <v>42</v>
       </c>
       <c r="F218" t="n">
-        <v>3000</v>
+        <v>6436</v>
       </c>
       <c r="G218" t="inlineStr">
         <is>
@@ -49069,7 +49799,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>marches/volatilite/GVZ.csv</t>
+          <t>souverains/CANADA_2A.csv</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -49087,7 +49817,7 @@
         <v>42</v>
       </c>
       <c r="F219" t="n">
-        <v>3772</v>
+        <v>6435</v>
       </c>
       <c r="G219" t="inlineStr">
         <is>
@@ -49098,7 +49828,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>marches/volatilite/MOVE.csv</t>
+          <t>souverains/CANADA_5A.csv</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -49116,7 +49846,7 @@
         <v>42</v>
       </c>
       <c r="F220" t="n">
-        <v>3691</v>
+        <v>6435</v>
       </c>
       <c r="G220" t="inlineStr">
         <is>
@@ -49127,7 +49857,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>marches/volatilite/OVX.csv</t>
+          <t>souverains/CANADA_LONG.csv</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -49145,7 +49875,7 @@
         <v>42</v>
       </c>
       <c r="F221" t="n">
-        <v>3772</v>
+        <v>6435</v>
       </c>
       <c r="G221" t="inlineStr">
         <is>
@@ -49156,7 +49886,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>marches/volatilite/VVIX.csv</t>
+          <t>souverains/SUEDE_10A.csv</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -49174,7 +49904,7 @@
         <v>42</v>
       </c>
       <c r="F222" t="n">
-        <v>3764</v>
+        <v>9202</v>
       </c>
       <c r="G222" t="inlineStr">
         <is>
@@ -49185,7 +49915,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>marches/volatilite/VXN.csv</t>
+          <t>souverains/SUEDE_2A.csv</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -49203,7 +49933,7 @@
         <v>42</v>
       </c>
       <c r="F223" t="n">
-        <v>3772</v>
+        <v>9202</v>
       </c>
       <c r="G223" t="inlineStr">
         <is>
@@ -49214,7 +49944,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_10A.csv</t>
+          <t>souverains/SUEDE_5A.csv</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -49232,7 +49962,7 @@
         <v>42</v>
       </c>
       <c r="F224" t="n">
-        <v>9202</v>
+        <v>9204</v>
       </c>
       <c r="G224" t="inlineStr">
         <is>
@@ -49243,7 +49973,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_2A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
@@ -49261,7 +49991,7 @@
         <v>42</v>
       </c>
       <c r="F225" t="n">
-        <v>9202</v>
+        <v>5639</v>
       </c>
       <c r="G225" t="inlineStr">
         <is>
@@ -49272,7 +50002,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_5A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -49290,7 +50020,7 @@
         <v>42</v>
       </c>
       <c r="F226" t="n">
-        <v>9204</v>
+        <v>5639</v>
       </c>
       <c r="G226" t="inlineStr">
         <is>
@@ -49301,7 +50031,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -49330,7 +50060,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -49359,7 +50089,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -49388,7 +50118,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -49417,7 +50147,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -49446,7 +50176,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -49475,7 +50205,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
+          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -49504,16 +50234,16 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
+          <t>fred/ECBDFR.csv</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C234" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D234" t="n">
         <v>1</v>
@@ -49522,7 +50252,7 @@
         <v>42</v>
       </c>
       <c r="F234" t="n">
-        <v>5639</v>
+        <v>3000</v>
       </c>
       <c r="G234" t="inlineStr">
         <is>
@@ -49533,16 +50263,16 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
+          <t>fred/RRPONTSYD.csv</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C235" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D235" t="n">
         <v>1</v>
@@ -49551,7 +50281,7 @@
         <v>42</v>
       </c>
       <c r="F235" t="n">
-        <v>5639</v>
+        <v>3000</v>
       </c>
       <c r="G235" t="inlineStr">
         <is>
@@ -49562,16 +50292,16 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>yfinance/SP500.csv</t>
+          <t>marches/fx/AUDJPY.csv</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C236" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D236" t="n">
         <v>1</v>
@@ -49580,7 +50310,7 @@
         <v>42</v>
       </c>
       <c r="F236" t="n">
-        <v>7547</v>
+        <v>3908</v>
       </c>
       <c r="G236" t="inlineStr">
         <is>
@@ -49591,16 +50321,16 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>yfinance/XLB.csv</t>
+          <t>marches/fx/AUDUSD.csv</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C237" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D237" t="n">
         <v>1</v>
@@ -49609,7 +50339,7 @@
         <v>42</v>
       </c>
       <c r="F237" t="n">
-        <v>501</v>
+        <v>3904</v>
       </c>
       <c r="G237" t="inlineStr">
         <is>
@@ -49620,16 +50350,16 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>yfinance/XLE.csv</t>
+          <t>marches/fx/DXY.csv</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C238" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D238" t="n">
         <v>1</v>
@@ -49638,7 +50368,7 @@
         <v>42</v>
       </c>
       <c r="F238" t="n">
-        <v>501</v>
+        <v>3772</v>
       </c>
       <c r="G238" t="inlineStr">
         <is>
@@ -49649,16 +50379,16 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>yfinance/XLF.csv</t>
+          <t>marches/fx/EURCHF.csv</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C239" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D239" t="n">
         <v>1</v>
@@ -49667,7 +50397,7 @@
         <v>42</v>
       </c>
       <c r="F239" t="n">
-        <v>501</v>
+        <v>3905</v>
       </c>
       <c r="G239" t="inlineStr">
         <is>
@@ -49678,16 +50408,16 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>yfinance/XLI.csv</t>
+          <t>marches/fx/EURGBP.csv</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C240" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D240" t="n">
         <v>1</v>
@@ -49696,7 +50426,7 @@
         <v>42</v>
       </c>
       <c r="F240" t="n">
-        <v>501</v>
+        <v>3907</v>
       </c>
       <c r="G240" t="inlineStr">
         <is>
@@ -49707,16 +50437,16 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>yfinance/XLK.csv</t>
+          <t>marches/fx/EURJPY.csv</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C241" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D241" t="n">
         <v>1</v>
@@ -49725,7 +50455,7 @@
         <v>42</v>
       </c>
       <c r="F241" t="n">
-        <v>501</v>
+        <v>3907</v>
       </c>
       <c r="G241" t="inlineStr">
         <is>
@@ -49736,16 +50466,16 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>yfinance/XLP.csv</t>
+          <t>marches/fx/EURUSD.csv</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C242" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D242" t="n">
         <v>1</v>
@@ -49754,7 +50484,7 @@
         <v>42</v>
       </c>
       <c r="F242" t="n">
-        <v>501</v>
+        <v>3904</v>
       </c>
       <c r="G242" t="inlineStr">
         <is>
@@ -49765,16 +50495,16 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>yfinance/XLRE.csv</t>
+          <t>marches/fx/GBPUSD.csv</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C243" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D243" t="n">
         <v>1</v>
@@ -49783,7 +50513,7 @@
         <v>42</v>
       </c>
       <c r="F243" t="n">
-        <v>501</v>
+        <v>3905</v>
       </c>
       <c r="G243" t="inlineStr">
         <is>
@@ -49794,16 +50524,16 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>yfinance/XLU.csv</t>
+          <t>marches/fx/NZDUSD.csv</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C244" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D244" t="n">
         <v>1</v>
@@ -49812,7 +50542,7 @@
         <v>42</v>
       </c>
       <c r="F244" t="n">
-        <v>501</v>
+        <v>3905</v>
       </c>
       <c r="G244" t="inlineStr">
         <is>
@@ -49823,16 +50553,16 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>yfinance/XLV.csv</t>
+          <t>marches/fx/USDCAD.csv</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C245" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D245" t="n">
         <v>1</v>
@@ -49841,7 +50571,7 @@
         <v>42</v>
       </c>
       <c r="F245" t="n">
-        <v>501</v>
+        <v>3904</v>
       </c>
       <c r="G245" t="inlineStr">
         <is>
@@ -49852,16 +50582,16 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>yfinance/XLY.csv</t>
+          <t>marches/fx/USDCHF.csv</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C246" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D246" t="n">
         <v>1</v>
@@ -49870,7 +50600,7 @@
         <v>42</v>
       </c>
       <c r="F246" t="n">
-        <v>501</v>
+        <v>3902</v>
       </c>
       <c r="G246" t="inlineStr">
         <is>
@@ -49881,7 +50611,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>fred/ECBDFR.csv</t>
+          <t>marches/fx/USDCNY.csv</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
@@ -49899,7 +50629,7 @@
         <v>42</v>
       </c>
       <c r="F247" t="n">
-        <v>3000</v>
+        <v>3904</v>
       </c>
       <c r="G247" t="inlineStr">
         <is>
@@ -49910,7 +50640,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>marches/fx/AUDJPY.csv</t>
+          <t>marches/fx/USDJPY.csv</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
@@ -49928,7 +50658,7 @@
         <v>42</v>
       </c>
       <c r="F248" t="n">
-        <v>3908</v>
+        <v>3905</v>
       </c>
       <c r="G248" t="inlineStr">
         <is>
@@ -49939,7 +50669,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>marches/fx/AUDUSD.csv</t>
+          <t>marches/fx/USDKRW.csv</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
@@ -49968,7 +50698,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>marches/fx/DXY.csv</t>
+          <t>marches/fx/USDNOK.csv</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
@@ -49986,7 +50716,7 @@
         <v>42</v>
       </c>
       <c r="F250" t="n">
-        <v>3772</v>
+        <v>3905</v>
       </c>
       <c r="G250" t="inlineStr">
         <is>
@@ -49997,7 +50727,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>marches/fx/EURCHF.csv</t>
+          <t>marches/fx/USDSEK.csv</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
@@ -50026,7 +50756,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>marches/fx/EURGBP.csv</t>
+          <t>marches/indices/DAX.csv</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -50044,7 +50774,7 @@
         <v>42</v>
       </c>
       <c r="F252" t="n">
-        <v>3907</v>
+        <v>3802</v>
       </c>
       <c r="G252" t="inlineStr">
         <is>
@@ -50055,7 +50785,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>marches/fx/EURJPY.csv</t>
+          <t>marches/indices/EUROSTOXX50.csv</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -50073,7 +50803,7 @@
         <v>42</v>
       </c>
       <c r="F253" t="n">
-        <v>3907</v>
+        <v>3759</v>
       </c>
       <c r="G253" t="inlineStr">
         <is>
@@ -50084,7 +50814,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>marches/fx/EURUSD.csv</t>
+          <t>marches/indices/FTSE100.csv</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
@@ -50102,7 +50832,7 @@
         <v>42</v>
       </c>
       <c r="F254" t="n">
-        <v>3904</v>
+        <v>3788</v>
       </c>
       <c r="G254" t="inlineStr">
         <is>
@@ -50113,7 +50843,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>marches/fx/GBPUSD.csv</t>
+          <t>marches/matieres/BRENT.csv</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
@@ -50131,7 +50861,7 @@
         <v>42</v>
       </c>
       <c r="F255" t="n">
-        <v>3905</v>
+        <v>3751</v>
       </c>
       <c r="G255" t="inlineStr">
         <is>
@@ -50142,7 +50872,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>marches/fx/NZDUSD.csv</t>
+          <t>marches/matieres/CUIVRE.csv</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
@@ -50160,7 +50890,7 @@
         <v>42</v>
       </c>
       <c r="F256" t="n">
-        <v>3905</v>
+        <v>3771</v>
       </c>
       <c r="G256" t="inlineStr">
         <is>
@@ -50171,7 +50901,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>marches/fx/USDCAD.csv</t>
+          <t>marches/matieres/GAZ_HENRY_HUB.csv</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
@@ -50189,7 +50919,7 @@
         <v>42</v>
       </c>
       <c r="F257" t="n">
-        <v>3904</v>
+        <v>3772</v>
       </c>
       <c r="G257" t="inlineStr">
         <is>
@@ -50200,7 +50930,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>marches/fx/USDCHF.csv</t>
+          <t>marches/matieres/OR.csv</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
@@ -50218,7 +50948,7 @@
         <v>42</v>
       </c>
       <c r="F258" t="n">
-        <v>3902</v>
+        <v>3771</v>
       </c>
       <c r="G258" t="inlineStr">
         <is>
@@ -50229,7 +50959,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>marches/fx/USDCNY.csv</t>
+          <t>marches/matieres/WTI.csv</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
@@ -50247,7 +50977,7 @@
         <v>42</v>
       </c>
       <c r="F259" t="n">
-        <v>3904</v>
+        <v>3771</v>
       </c>
       <c r="G259" t="inlineStr">
         <is>
@@ -50258,7 +50988,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>marches/fx/USDJPY.csv</t>
+          <t>marches/taux_futures/FED_FUNDS_FRONT.csv</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
@@ -50276,7 +51006,7 @@
         <v>42</v>
       </c>
       <c r="F260" t="n">
-        <v>3905</v>
+        <v>3772</v>
       </c>
       <c r="G260" t="inlineStr">
         <is>
@@ -50287,7 +51017,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>marches/fx/USDKRW.csv</t>
+          <t>marches/volatilite/GVZ.csv</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
@@ -50305,7 +51035,7 @@
         <v>42</v>
       </c>
       <c r="F261" t="n">
-        <v>3904</v>
+        <v>3771</v>
       </c>
       <c r="G261" t="inlineStr">
         <is>
@@ -50316,7 +51046,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>marches/fx/USDNOK.csv</t>
+          <t>marches/volatilite/OVX.csv</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
@@ -50334,7 +51064,7 @@
         <v>42</v>
       </c>
       <c r="F262" t="n">
-        <v>3905</v>
+        <v>3771</v>
       </c>
       <c r="G262" t="inlineStr">
         <is>
@@ -50345,7 +51075,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>marches/fx/USDSEK.csv</t>
+          <t>marches/volatilite/VVIX.csv</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
@@ -50363,7 +51093,7 @@
         <v>42</v>
       </c>
       <c r="F263" t="n">
-        <v>3905</v>
+        <v>3763</v>
       </c>
       <c r="G263" t="inlineStr">
         <is>
@@ -50374,7 +51104,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>marches/indices/DAX.csv</t>
+          <t>marches/volatilite/VXN.csv</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
@@ -50392,7 +51122,7 @@
         <v>42</v>
       </c>
       <c r="F264" t="n">
-        <v>3802</v>
+        <v>3771</v>
       </c>
       <c r="G264" t="inlineStr">
         <is>
@@ -50403,7 +51133,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>marches/indices/EUROSTOXX50.csv</t>
+          <t>yfinance/SP500.csv</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
@@ -50421,7 +51151,7 @@
         <v>42</v>
       </c>
       <c r="F265" t="n">
-        <v>3759</v>
+        <v>7546</v>
       </c>
       <c r="G265" t="inlineStr">
         <is>
@@ -50432,7 +51162,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>marches/indices/FTSE100.csv</t>
+          <t>yfinance/VIX.csv</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
@@ -50450,7 +51180,7 @@
         <v>42</v>
       </c>
       <c r="F266" t="n">
-        <v>3788</v>
+        <v>7548</v>
       </c>
       <c r="G266" t="inlineStr">
         <is>
@@ -50461,7 +51191,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>marches/indices/HANGSENG.csv</t>
+          <t>yfinance/XLB.csv</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
@@ -50479,7 +51209,7 @@
         <v>42</v>
       </c>
       <c r="F267" t="n">
-        <v>3689</v>
+        <v>500</v>
       </c>
       <c r="G267" t="inlineStr">
         <is>
@@ -50490,7 +51220,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>marches/indices/KOSPI.csv</t>
+          <t>yfinance/XLE.csv</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
@@ -50508,7 +51238,7 @@
         <v>42</v>
       </c>
       <c r="F268" t="n">
-        <v>3681</v>
+        <v>500</v>
       </c>
       <c r="G268" t="inlineStr">
         <is>
@@ -50519,7 +51249,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>marches/indices/NIKKEI225.csv</t>
+          <t>yfinance/XLF.csv</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
@@ -50537,7 +51267,7 @@
         <v>42</v>
       </c>
       <c r="F269" t="n">
-        <v>3667</v>
+        <v>500</v>
       </c>
       <c r="G269" t="inlineStr">
         <is>
@@ -50548,7 +51278,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>marches/matieres/BRENT.csv</t>
+          <t>yfinance/XLI.csv</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
@@ -50566,7 +51296,7 @@
         <v>42</v>
       </c>
       <c r="F270" t="n">
-        <v>3751</v>
+        <v>500</v>
       </c>
       <c r="G270" t="inlineStr">
         <is>
@@ -50577,7 +51307,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>marches/matieres/CUIVRE.csv</t>
+          <t>yfinance/XLK.csv</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
@@ -50595,7 +51325,7 @@
         <v>42</v>
       </c>
       <c r="F271" t="n">
-        <v>3771</v>
+        <v>500</v>
       </c>
       <c r="G271" t="inlineStr">
         <is>
@@ -50606,7 +51336,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>marches/matieres/GAZ_HENRY_HUB.csv</t>
+          <t>yfinance/XLP.csv</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
@@ -50624,7 +51354,7 @@
         <v>42</v>
       </c>
       <c r="F272" t="n">
-        <v>3772</v>
+        <v>500</v>
       </c>
       <c r="G272" t="inlineStr">
         <is>
@@ -50635,7 +51365,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>marches/matieres/OR.csv</t>
+          <t>yfinance/XLRE.csv</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
@@ -50653,7 +51383,7 @@
         <v>42</v>
       </c>
       <c r="F273" t="n">
-        <v>3771</v>
+        <v>500</v>
       </c>
       <c r="G273" t="inlineStr">
         <is>
@@ -50664,7 +51394,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>marches/matieres/WTI.csv</t>
+          <t>yfinance/XLU.csv</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
@@ -50682,7 +51412,7 @@
         <v>42</v>
       </c>
       <c r="F274" t="n">
-        <v>3771</v>
+        <v>500</v>
       </c>
       <c r="G274" t="inlineStr">
         <is>
@@ -50693,7 +51423,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>marches/taux_futures/FED_FUNDS_FRONT.csv</t>
+          <t>yfinance/XLV.csv</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
@@ -50711,7 +51441,7 @@
         <v>42</v>
       </c>
       <c r="F275" t="n">
-        <v>3772</v>
+        <v>500</v>
       </c>
       <c r="G275" t="inlineStr">
         <is>
@@ -50722,7 +51452,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>yfinance/VIX.csv</t>
+          <t>yfinance/XLY.csv</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
@@ -50740,7 +51470,7 @@
         <v>42</v>
       </c>
       <c r="F276" t="n">
-        <v>7548</v>
+        <v>500</v>
       </c>
       <c r="G276" t="inlineStr">
         <is>
@@ -51153,7 +51883,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -51415,6 +52145,25 @@
         <v>0.8685</v>
       </c>
       <c r="E13" t="n">
+        <v>0.9826</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.1207</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.1141</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.8683999999999999</v>
+      </c>
+      <c r="E14" t="n">
         <v>0.9826</v>
       </c>
     </row>
@@ -51663,7 +52412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -51905,6 +52654,24 @@
         <v>0.9997</v>
       </c>
       <c r="D13" t="inlineStr">
+        <is>
+          <t>persistant (tendanciel)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.5507</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.9996</v>
+      </c>
+      <c r="D14" t="inlineStr">
         <is>
           <t>persistant (tendanciel)</t>
         </is>
@@ -51921,7 +52688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -52142,6 +52909,22 @@
       </c>
       <c r="D13" t="n">
         <v>0.01231</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.01026</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.00041</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.01282</v>
       </c>
     </row>
   </sheetData>
@@ -52200,17 +52983,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>6889.74</v>
+        <v>7080.92</v>
       </c>
       <c r="D2" t="n">
-        <v>-17.93</v>
+        <v>-16.41</v>
       </c>
       <c r="E2" t="n">
-        <v>103.47</v>
+        <v>103.11</v>
       </c>
     </row>
     <row r="3">
@@ -52221,17 +53004,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>65877.62</v>
+        <v>66364.2</v>
       </c>
       <c r="D3" t="n">
-        <v>-5.17</v>
+        <v>-4.32</v>
       </c>
       <c r="E3" t="n">
-        <v>45.25</v>
+        <v>45.04</v>
       </c>
     </row>
     <row r="4">
@@ -52242,17 +53025,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>7743.41</v>
+        <v>7698.37</v>
       </c>
       <c r="D4" t="n">
-        <v>5.29</v>
+        <v>3.47</v>
       </c>
       <c r="E4" t="n">
-        <v>17.24</v>
+        <v>15.87</v>
       </c>
     </row>
     <row r="5">
@@ -52267,13 +53050,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>10730.11</v>
+        <v>10684.88</v>
       </c>
       <c r="D5" t="n">
-        <v>2.35</v>
+        <v>1.91</v>
       </c>
       <c r="E5" t="n">
-        <v>15.57</v>
+        <v>15.08</v>
       </c>
     </row>
     <row r="6">
@@ -52288,13 +53071,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>6310.18</v>
+        <v>6301.28</v>
       </c>
       <c r="D6" t="n">
-        <v>1.26</v>
+        <v>1.12</v>
       </c>
       <c r="E6" t="n">
-        <v>14.74</v>
+        <v>14.57</v>
       </c>
     </row>
     <row r="7">
@@ -52309,13 +53092,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>25417.97</v>
+        <v>25374.42</v>
       </c>
       <c r="D7" t="n">
-        <v>3.21</v>
+        <v>3.04</v>
       </c>
       <c r="E7" t="n">
-        <v>7.07</v>
+        <v>6.89</v>
       </c>
     </row>
     <row r="8">
@@ -52326,17 +53109,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>24642.51</v>
+        <v>24510.09</v>
       </c>
       <c r="D8" t="n">
-        <v>7.02</v>
+        <v>8.109999999999999</v>
       </c>
       <c r="E8" t="n">
-        <v>-5.69</v>
+        <v>-7.46</v>
       </c>
     </row>
   </sheetData>
@@ -53012,16 +53795,16 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>16.27</v>
+        <v>15.89</v>
       </c>
       <c r="C13" t="n">
-        <v>16.077</v>
+        <v>15.754</v>
       </c>
       <c r="D13" t="n">
         <v>0.625</v>
       </c>
       <c r="E13" t="n">
-        <v>0.20518</v>
+        <v>0.20516</v>
       </c>
     </row>
   </sheetData>
@@ -53673,7 +54456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -54089,6 +54872,37 @@
         <v>0.218</v>
       </c>
       <c r="G13" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>10</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>XLF;XLRE;XLU</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>-0.6820000000000001</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>XLY;XLE;XLK</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>0.175</v>
+      </c>
+      <c r="G14" t="inlineStr">
         <is>
           <t>False</t>
         </is>
@@ -54419,25 +55233,25 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.001585</v>
+        <v>0.001592</v>
       </c>
       <c r="C11" t="n">
-        <v>5.02</v>
+        <v>5.44</v>
       </c>
       <c r="D11" t="n">
-        <v>100.53</v>
+        <v>97.78</v>
       </c>
       <c r="E11" t="n">
-        <v>37.43</v>
+        <v>33.67</v>
       </c>
       <c r="F11" t="n">
-        <v>43.35</v>
+        <v>39.43</v>
       </c>
       <c r="G11" t="n">
-        <v>-1.04</v>
+        <v>-2.42</v>
       </c>
       <c r="H11" t="n">
-        <v>4.81</v>
+        <v>5.24</v>
       </c>
     </row>
   </sheetData>
@@ -54575,7 +55389,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -54840,6 +55654,25 @@
         <v>0.1</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="C14" t="n">
+        <v>2.76</v>
+      </c>
+      <c r="D14" t="n">
+        <v>-0.09</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.17</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -54851,7 +55684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -55204,6 +56037,32 @@
       </c>
       <c r="F13" t="n">
         <v>19.54</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>XLE;XLV;XLK</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>9.183999999999999</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>XLI;XLRE;XLU</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>-9.948</v>
+      </c>
+      <c r="F14" t="n">
+        <v>19.132</v>
       </c>
     </row>
   </sheetData>
@@ -57788,7 +58647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -58093,6 +58952,28 @@
       </c>
       <c r="F13" t="n">
         <v>16.215</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>-0.174</v>
+      </c>
+      <c r="C14" t="n">
+        <v>3.467</v>
+      </c>
+      <c r="D14" t="n">
+        <v>21.354</v>
+      </c>
+      <c r="E14" t="n">
+        <v>15.875</v>
+      </c>
+      <c r="F14" t="n">
+        <v>16.076</v>
       </c>
     </row>
   </sheetData>
@@ -58212,7 +59093,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -58517,6 +59398,28 @@
       </c>
       <c r="F13" t="n">
         <v>-0.216</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="C14" t="n">
+        <v>3.025</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.017113</v>
+      </c>
+      <c r="E14" t="n">
+        <v>40.5</v>
+      </c>
+      <c r="F14" t="n">
+        <v>-0.095</v>
       </c>
     </row>
   </sheetData>
@@ -58822,19 +59725,19 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>16.27</v>
+        <v>15.89</v>
       </c>
       <c r="C13" t="n">
-        <v>20.202</v>
+        <v>20.2</v>
       </c>
       <c r="D13" t="n">
-        <v>0.02405</v>
+        <v>0.02404</v>
       </c>
       <c r="E13" t="n">
         <v>28.8</v>
       </c>
       <c r="F13" t="n">
-        <v>-3.932</v>
+        <v>-4.31</v>
       </c>
     </row>
   </sheetData>
@@ -59213,26 +60116,26 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>3.39</v>
+        <v>3.35</v>
       </c>
       <c r="D7" t="n">
-        <v>3.97</v>
+        <v>3.94</v>
       </c>
       <c r="E7" t="n">
-        <v>0.58</v>
+        <v>0.59</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.06</v>
+        <v>-0.05</v>
       </c>
       <c r="G7" t="n">
-        <v>0.64</v>
+        <v>0.6</v>
       </c>
       <c r="H7" t="n">
-        <v>0.58</v>
+        <v>0.55</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -63952,7 +64855,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -64089,6 +64992,16 @@
       </c>
       <c r="B13" t="n">
         <v>-0.004842</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>-0.004876</v>
       </c>
     </row>
   </sheetData>
@@ -64499,7 +65412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -64909,6 +65822,36 @@
         <v>3.834e-07</v>
       </c>
       <c r="H13" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>5281</v>
+      </c>
+      <c r="C14" t="n">
+        <v>2264</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.00011628</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.20963</v>
+      </c>
+      <c r="F14" t="n">
+        <v>2.985e-07</v>
+      </c>
+      <c r="G14" t="n">
+        <v>3.834e-07</v>
+      </c>
+      <c r="H14" t="inlineStr">
         <is>
           <t>True</t>
         </is>
@@ -65142,10 +66085,10 @@
         <v>0.00881</v>
       </c>
       <c r="C13" t="n">
-        <v>0.06859999999999999</v>
+        <v>0.06818</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.0387</v>
+        <v>-0.0385</v>
       </c>
     </row>
   </sheetData>
@@ -68099,7 +69042,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -68320,6 +69263,22 @@
       </c>
       <c r="D13" t="n">
         <v>0.422</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>-1.107</v>
+      </c>
+      <c r="C14" t="n">
+        <v>2.403</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.421</v>
       </c>
     </row>
   </sheetData>
@@ -68333,7 +69292,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -68554,6 +69513,22 @@
       </c>
       <c r="D13" t="n">
         <v>1.7553</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1.1387</v>
+      </c>
+      <c r="C14" t="n">
+        <v>1.1201</v>
+      </c>
+      <c r="D14" t="n">
+        <v>1.626</v>
       </c>
     </row>
   </sheetData>
@@ -71115,7 +72090,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -71462,6 +72437,31 @@
       </c>
       <c r="G13" t="n">
         <v>0.01024</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.00029</v>
+      </c>
+      <c r="C14" t="n">
+        <v>-0.032596</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.000269</v>
+      </c>
+      <c r="E14" t="n">
+        <v>5278</v>
+      </c>
+      <c r="F14" t="n">
+        <v>2262</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.01026</v>
       </c>
     </row>
   </sheetData>
@@ -71862,7 +72862,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E121"/>
+  <dimension ref="A1:E131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -74657,6 +75657,236 @@
       </c>
       <c r="E121" t="n">
         <v>-14.481</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B122" t="n">
+        <v>1</v>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>XLE</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Energie</t>
+        </is>
+      </c>
+      <c r="E122" t="n">
+        <v>15.967</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B123" t="n">
+        <v>2</v>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>XLV</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Sante</t>
+        </is>
+      </c>
+      <c r="E123" t="n">
+        <v>6.526</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B124" t="n">
+        <v>3</v>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>XLK</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Technologie</t>
+        </is>
+      </c>
+      <c r="E124" t="n">
+        <v>5.059</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B125" t="n">
+        <v>4</v>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>XLF</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="E125" t="n">
+        <v>1.089</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B126" t="n">
+        <v>5</v>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>XLB</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Materiaux</t>
+        </is>
+      </c>
+      <c r="E126" t="n">
+        <v>-2.063</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B127" t="n">
+        <v>6</v>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>XLP</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Consommation de base</t>
+        </is>
+      </c>
+      <c r="E127" t="n">
+        <v>-2.495</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B128" t="n">
+        <v>7</v>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>XLY</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Consommation discretionnaire</t>
+        </is>
+      </c>
+      <c r="E128" t="n">
+        <v>-6.617</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B129" t="n">
+        <v>8</v>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>XLI</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Industrie</t>
+        </is>
+      </c>
+      <c r="E129" t="n">
+        <v>-7.514</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B130" t="n">
+        <v>9</v>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>XLRE</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Immobilier</t>
+        </is>
+      </c>
+      <c r="E130" t="n">
+        <v>-7.881</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B131" t="n">
+        <v>10</v>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>XLU</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Services collectifs</t>
+        </is>
+      </c>
+      <c r="E131" t="n">
+        <v>-14.45</v>
       </c>
     </row>
   </sheetData>
@@ -75062,7 +76292,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -75477,6 +76707,36 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>3840</v>
+      </c>
+      <c r="C14" t="n">
+        <v>3705</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.04655</v>
+      </c>
+      <c r="F14" t="n">
+        <v>-1.026</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.3047</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -75488,7 +76748,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -76624,6 +77884,98 @@
         <v>0.0081</v>
       </c>
       <c r="E49" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>momentum_5j</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>-0.0295</v>
+      </c>
+      <c r="D50" t="n">
+        <v>0.0104</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>momentum_20j</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>-0.0112</v>
+      </c>
+      <c r="D51" t="n">
+        <v>0.3294</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>niveau_vix</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>-0.0036</v>
+      </c>
+      <c r="D52" t="n">
+        <v>0.7514999999999999</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>variation_vix</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>0.0306</v>
+      </c>
+      <c r="D53" t="n">
+        <v>0.008</v>
+      </c>
+      <c r="E53" t="inlineStr">
         <is>
           <t>True</t>
         </is>
@@ -76723,7 +78075,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -76988,6 +78340,25 @@
         <v>1000</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.1298</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.1171</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.1412</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1000</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -76999,7 +78370,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -77178,6 +78549,19 @@
       </c>
       <c r="C13" t="n">
         <v>1.0307</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>-0.2008</v>
+      </c>
+      <c r="C14" t="n">
+        <v>1.0264</v>
       </c>
     </row>
   </sheetData>
@@ -77362,13 +78746,13 @@
         <v>25.5</v>
       </c>
       <c r="D9" t="n">
-        <v>3.97</v>
+        <v>3.94</v>
       </c>
       <c r="E9" t="n">
         <v>3.03</v>
       </c>
       <c r="F9" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.91</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-28T19:47Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-28 18:49 UTC</t>
+          <t>Genere le 2026-09-28 19:47 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-28 18:49 UTC</t>
+          <t>Rapport global — 2026-09-28 19:47 UTC</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>**Matieres premieres macro** — le ratio cuivre/or monte -- la croissance domine la peur (+5.4% sur 3 mois). Brent 97.8$ (+33.7% sur 3 mois, +39.4% sur 12 mois), gaz -2.4% sur 3 mois, ecart Brent-WTI +5.2$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-28)_</t>
+          <t>**Matieres premieres macro** — le ratio cuivre/or monte -- la croissance domine la peur (+5.3% sur 3 mois). Brent 98.0$ (+34.0% sur 3 mois, +39.8% sur 12 mois), gaz -1.0% sur 3 mois, ecart Brent-WTI +5.2$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -862,7 +862,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>**Conditions financieres** — indice conditions financieres=+0.106 (3 composantes: {'taux_directeur': 0.5985724560125544, 'courbe_inversee': 0.2531563730537784, 'vix': -0.5337130261637928}) -- conditions proches de la normale _(observation : 2026-09-24)_</t>
+          <t>**Conditions financieres** — indice conditions financieres=+0.111 (3 composantes: {'taux_directeur': 0.5985724560125544, 'courbe_inversee': 0.2531563730537784, 'vix': -0.5188744650175076}) -- conditions proches de la normale _(observation : 2026-09-24)_</t>
         </is>
       </c>
     </row>
@@ -988,7 +988,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>**Momentum prix** — SP500 momentum 12-1 mois = 16.08% -- haussier (momentum positif), detail 1/3/6/12m = [-0.17, 3.47, 21.35, 15.87] _(observation : 2026-09-28)_</t>
+          <t>**Momentum prix** — SP500 momentum 12-1 mois = 16.08% -- haussier (momentum positif), detail 1/3/6/12m = [-0.38, 3.25, 21.1, 15.63] _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1002,42 +1002,42 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>**Beta vol** — beta SP500/VIX (60j) = -0.00488 (rendement SP500 pour +1pt VIX) -- sensibilite normale, relation inverse attendue (normale) _(observation : 2026-09-28)_</t>
+          <t>**Beta vol** — beta SP500/VIX (60j) = -0.00490 (rendement SP500 pour +1pt VIX) -- sensibilite normale, relation inverse attendue (normale) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>**Rotation sectorielle** — classement momentum 3 mois (10 secteurs) : 1. Energie (XLE) : +15.97% | 2. Sante (XLV) : +6.53% | 3. Technologie (XLK) : +5.06% | 4. Finance (XLF) : +1.09% | 5. Materiaux (XLB) : -2.06% _(observation : 2026-09-28)_</t>
+          <t>**Rotation sectorielle** — classement momentum 3 mois (10 secteurs) : 1. Energie (XLE) : +16.10% | 2. Sante (XLV) : +6.54% | 3. Technologie (XLK) : +4.82% | 4. Finance (XLF) : +0.92% | 5. Materiaux (XLB) : -2.20% _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>**Saisonnalite** — rendement journalier moyen ete=+0.0180%, hiver=+0.0465% (t=-1.03, p=0.3047) -- non significatif (attendu vu la faible puissance sur seulement ~2 ans) _(observation : 2026-09-28)_</t>
+          <t>**Saisonnalite** — rendement journalier moyen ete=+0.0179%, hiver=+0.0465% (t=-1.03, p=0.3038) -- non significatif (attendu vu la faible puissance sur seulement ~2 ans) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>**Dispersion sectorielle** — 10 secteurs, rendement moyen 3m=-1.24%, dispersion (ecart-type)=8.31pt, etendue=30.42pt -- dispersion intermediaire _(observation : 2026-09-28)_</t>
+          <t>**Dispersion sectorielle** — 10 secteurs, rendement moyen 3m=-1.33%, dispersion (ecart-type)=8.38pt, etendue=30.71pt -- dispersion intermediaire _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>**Low volatility** — tercile bas-vol ['XLF', 'XLRE', 'XLU'] Sharpe=-0.682 vs tercile haut-vol ['XLY', 'XLE', 'XLK'] Sharpe=0.175 -- anomalie low-vol non confirmee sur cet echantillon (puissance statistique faible, n petit -- limite assumee) _(observation : 2026-09-28)_</t>
+          <t>**Low volatility** — tercile bas-vol ['XLF', 'XLRE', 'XLU'] Sharpe=-0.712 vs tercile haut-vol ['XLY', 'XLE', 'XLK'] Sharpe=0.164 -- anomalie low-vol non confirmee sur cet echantillon (puissance statistique faible, n petit -- limite assumee) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>**Momentum cross sectional** — panier gagnant ['XLE', 'XLV', 'XLK'] (+9.18%) vs panier perdant ['XLI', 'XLRE', 'XLU'] (-9.95%) -- spread momentum=+19.13pt _(observation : 2026-09-28)_</t>
+          <t>**Momentum cross sectional** — panier gagnant ['XLE', 'XLV', 'XLK'] (+9.15%) vs panier perdant ['XLI', 'XLRE', 'XLU'] (-10.09%) -- spread momentum=+19.25pt _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>**Correlation facteurs** — correlation entre momentum 3m et beta-VIX, 10 secteurs : +0.206 (facteurs largement independants) _(observation : 2026-09-28)_</t>
+          <t>**Correlation facteurs** — correlation entre momentum 3m et beta-VIX, 10 secteurs : +0.219 (facteurs largement independants) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1107,7 +1107,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>**Divergence cot prix** — SP500 -0.17% sur 30j, COT net -10560 -&gt; -133228 -- pas de divergence _(observation : 2026-09-28)_</t>
+          <t>**Divergence cot prix** — SP500 -0.38% sur 30j, COT net -10560 -&gt; -133228 -- pas de divergence _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1191,14 +1191,14 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>**Vol cross asset** — 6 mesures de volatilite : Petrole (OVX) 88e pct, Or (GVZ) 86e pct, Nasdaq (VXN) 48e pct, Taux US (MOVE) 43e pct, Vol de la vol (VVIX) 35e pct, Actions US (VIX) 31e pct -- stress LOCALISE sur Petrole (OVX), Or (GVZ) pendant que le reste ne l'est pas -- episode propre a cette classe d'actifs, pas une aversion au risque d'ensemble _(observation : 2026-09-28)_</t>
+          <t>**Vol cross asset** — 6 mesures de volatilite : Petrole (OVX) 88e pct, Or (GVZ) 86e pct, Nasdaq (VXN) 48e pct, Taux US (MOVE) 43e pct, Vol de la vol (VVIX) 37e pct, Actions US (VIX) 32e pct -- stress LOCALISE sur Petrole (OVX), Or (GVZ) pendant que le reste ne l'est pas -- episode propre a cette classe d'actifs, pas une aversion au risque d'ensemble _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>**Volatilite ewma** — vol realisee 60j=0.11229567008242833, EWMA=0.1072 (tendance 10 runs: stable) _(observation : 2026-09-28)_</t>
+          <t>**Volatilite ewma** — vol realisee 60j=0.11287248847520996, EWMA=0.1092 (tendance 10 runs: stable) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1219,7 +1219,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>**Ornstein uhlenbeck vix** — VIX actuel=15.89, niveau moyen estime (mu)=20.20, demi-vie=28.8j, ecart actuel=-4.31 -- VIX actuel en-dessous de son niveau moyen de long terme _(observation : 2026-09-28)_</t>
+          <t>**Ornstein uhlenbeck vix** — VIX actuel=16.01, niveau moyen estime (mu)=20.20, demi-vie=28.8j, ecart actuel=-4.19 -- VIX actuel en-dessous de son niveau moyen de long terme _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1233,14 +1233,14 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>**Kalman niveau local** — VIX observe=15.89, filtre Kalman=15.75 (ecart-type=0.62), ratio signal/bruit=0.2052 -- le filtre lisse fortement le bruit, reagit lentement (ecart obs.-filtre=+0.14) _(observation : 2026-09-28)_</t>
+          <t>**Kalman niveau local** — VIX observe=16.01, filtre Kalman=15.86 (ecart-type=0.62), ratio signal/bruit=0.2052 -- le filtre lisse fortement le bruit, reagit lentement (ecart obs.-filtre=+0.15) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.37239521716456103 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.05235750065322864 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-28)_</t>
+          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.37280971577723143 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.05236466910626937 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1261,14 +1261,14 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>**Skew kurtosis** — skewness=-0.201 (asymetrie negative (pertes extremes &gt; gains extremes)), kurtosis exces=+1.026 (queues epaisses (risque extreme sous-estime par une hypothese normale)) _(observation : 2026-09-28)_</t>
+          <t>**Skew kurtosis** — skewness=-0.200 (asymetrie negative (pertes extremes &gt; gains extremes)), kurtosis exces=+1.014 (queues epaisses (risque extreme sous-estime par une hypothese normale)) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>**Ratios performance** — Sharpe=1.139 (bon), Sortino=1.120 (bon), Calmar=1.626 (bon) -- lecture sur fenetre 252j (~1 an, echantillon limite), seuils academiques standards, taux sans risque suppose nul _(observation : 2026-09-28)_</t>
+          <t>**Ratios performance** — Sharpe=1.122 (bon), Sortino=1.102 (bon), Calmar=1.603 (bon) -- lecture sur fenetre 252j (~1 an, echantillon limite), seuils academiques standards, taux sans risque suppose nul _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1282,14 +1282,14 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>**Stress test historique** — COVID_2020 (2020-02-19 -&gt; 2020-03-23) : chute historique=-33.9% -- rejouee sur le niveau actuel (7698) -&gt; 5087  _(sans synthese)_ _(observation : 2026-09-28)_</t>
+          <t>**Stress test historique** — COVID_2020 (2020-02-19 -&gt; 2020-03-23) : chute historique=-33.9% -- rejouee sur le niveau actuel (7682) -&gt; 5076  _(sans synthese)_ _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>**Sizing robuste** — vol point estimate=0.1298, IC90%=[0.1171, 0.1412] (1000 tirages bootstrap) -- intervalle etroit (19% du point estimate) -- estimation relativement fiable _(observation : 2026-09-28)_</t>
+          <t>**Sizing robuste** — vol point estimate=0.1299, IC90%=[0.1173, 0.1413] (1000 tirages bootstrap) -- intervalle etroit (18% du point estimate) -- estimation relativement fiable _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1303,7 +1303,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>**Detection saut** — Z-stat BNS (fenetre 22j)=1.206 (seuil ±1.96) -- pas de saut isole detecte _(observation : 2026-09-28)_</t>
+          <t>**Detection saut** — Z-stat BNS (fenetre 22j)=1.270 (seuil ±1.96) -- pas de saut isole detecte _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1317,7 +1317,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>**Qualite regime macro** — instabilite taux=0.0088, instabilite VIX=0.0682 -- score qualite du regime=-0.0385 (plus haut = regime plus stable/previsible) _(observation : 2026-09-24)_</t>
+          <t>**Qualite regime macro** — instabilite taux=0.0088, instabilite VIX=0.0683 -- score qualite du regime=-0.0386 (plus haut = regime plus stable/previsible) _(observation : 2026-09-24)_</t>
         </is>
       </c>
     </row>
@@ -1331,21 +1331,21 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>**Decomposition stl** — VIX : tendance=15.52, composante saisonniere (periode 5j)=+0.101, residu=+0.266 -- la saisonnalite explique 0.72% de la variance totale (negligeable) _(observation : 2026-09-28)_</t>
+          <t>**Decomposition stl** — VIX : tendance=15.55, composante saisonniere (periode 5j)=+0.128, residu=+0.335 -- la saisonnalite explique 0.72% de la variance totale (negligeable) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>**Ratios conditionnels regime** — Sharpe regime haut-vol=-1.107, bas-vol=2.403, global=0.421 -- meilleur en regime calme, comme attendu _(observation : 2026-09-28)_</t>
+          <t>**Ratios conditionnels regime** — Sharpe regime haut-vol=-1.107, bas-vol=2.402, global=0.421 -- meilleur en regime calme, comme attendu _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>**Choc vol parametrique** — vol actuelle=12.98%, scenarios x1/x2/x3 calcules -- pire scenario (x3) = -3.97%/jour, soit 3.1x le scenario de base _(observation : 2026-09-28)_</t>
+          <t>**Choc vol parametrique** — vol actuelle=12.99%, scenarios x1/x2/x3 calcules -- pire scenario (x3) = -3.98%/jour, soit 3.1x le scenario de base _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1387,7 +1387,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>**Anomalie multivariee** — distance de Mahalanobis=0.788 (seuil 3.0) -- jour ordinaire _(observation : 2026-09-28)_</t>
+          <t>**Anomalie multivariee** — distance de Mahalanobis=1.062 (seuil 3.0) -- jour ordinaire _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>**Couts transaction** — 7515 predictions, 1512 changements de position (5pb/changement) -- rendement cumule brut=-93.19%, cout total=53.05%, net=-96.80% -- les frais mangent une part importante du rendement (&gt;50% du brut) _(observation : 2026-09-28)_</t>
+          <t>**Couts transaction** — 7515 predictions, 1512 changements de position (5pb/changement) -- rendement cumule brut=-93.20%, cout total=53.05%, net=-96.81% -- les frais mangent une part importante du rendement (&gt;50% du brut) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>**Importance permutation** — R2 base=0.0103 -- importance momentum5j=0.00041, importance variation_vix=0.01282 -- VIX plus important _(observation : 2026-09-28)_</t>
+          <t>**Importance permutation** — R2 base=0.0103 -- importance momentum5j=0.00042, importance variation_vix=0.01282 -- VIX plus important _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -5453,7 +5453,7 @@
         <v>-56.78</v>
       </c>
       <c r="F26" t="n">
-        <v>3327.59</v>
+        <v>3320.69</v>
       </c>
     </row>
     <row r="27">
@@ -5481,7 +5481,7 @@
         <v>-33.92</v>
       </c>
       <c r="F27" t="n">
-        <v>5086.7</v>
+        <v>5076.16</v>
       </c>
     </row>
   </sheetData>
@@ -7003,10 +7003,10 @@
         <v>5</v>
       </c>
       <c r="C14" t="n">
-        <v>0.07575999999999999</v>
+        <v>0.07554</v>
       </c>
       <c r="D14" t="n">
-        <v>0.00419</v>
+        <v>0.00417</v>
       </c>
     </row>
   </sheetData>
@@ -8247,10 +8247,10 @@
         <v>10</v>
       </c>
       <c r="C14" t="n">
-        <v>0.3724</v>
+        <v>0.37281</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.052358</v>
+        <v>-0.052365</v>
       </c>
     </row>
   </sheetData>
@@ -8319,7 +8319,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>55.65</v>
+        <v>55.7</v>
       </c>
       <c r="D2" t="n">
         <v>88.3</v>
@@ -8345,10 +8345,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>24.65</v>
+        <v>24.78</v>
       </c>
       <c r="D3" t="n">
-        <v>85.90000000000001</v>
+        <v>86.3</v>
       </c>
       <c r="E3" t="n">
         <v>1260</v>
@@ -8371,10 +8371,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>22.17</v>
+        <v>22.18</v>
       </c>
       <c r="D4" t="n">
-        <v>48</v>
+        <v>48.1</v>
       </c>
       <c r="E4" t="n">
         <v>1260</v>
@@ -8423,10 +8423,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>90.47</v>
+        <v>90.83</v>
       </c>
       <c r="D6" t="n">
-        <v>35.2</v>
+        <v>36.9</v>
       </c>
       <c r="E6" t="n">
         <v>1260</v>
@@ -8449,10 +8449,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>15.89</v>
+        <v>16.01</v>
       </c>
       <c r="D7" t="n">
-        <v>30.9</v>
+        <v>32</v>
       </c>
       <c r="E7" t="n">
         <v>1260</v>
@@ -8746,16 +8746,16 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.1072</v>
+        <v>0.1092</v>
       </c>
       <c r="C14" t="n">
-        <v>0.0804</v>
+        <v>0.0881</v>
       </c>
       <c r="D14" t="n">
-        <v>0.1096</v>
+        <v>0.1112</v>
       </c>
       <c r="E14" t="n">
-        <v>0.1123</v>
+        <v>0.1129</v>
       </c>
     </row>
   </sheetData>
@@ -11225,16 +11225,16 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>12.976</v>
+        <v>12.988</v>
       </c>
       <c r="C14" t="n">
-        <v>-1.284</v>
+        <v>-1.286</v>
       </c>
       <c r="D14" t="n">
-        <v>-2.629</v>
+        <v>-2.632</v>
       </c>
       <c r="E14" t="n">
-        <v>-3.973</v>
+        <v>-3.978</v>
       </c>
     </row>
   </sheetData>
@@ -15880,10 +15880,10 @@
         </is>
       </c>
       <c r="C122" t="n">
-        <v>-2.5552</v>
+        <v>-2.544</v>
       </c>
       <c r="D122" t="n">
-        <v>0.2553</v>
+        <v>0.26</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -15903,10 +15903,10 @@
         </is>
       </c>
       <c r="C123" t="n">
-        <v>-1.8586</v>
+        <v>-1.8576</v>
       </c>
       <c r="D123" t="n">
-        <v>0.6008</v>
+        <v>0.6014</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -15926,10 +15926,10 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>-2.142</v>
+        <v>-2.1473</v>
       </c>
       <c r="D124" t="n">
-        <v>0.4545</v>
+        <v>0.4517</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -15949,10 +15949,10 @@
         </is>
       </c>
       <c r="C125" t="n">
-        <v>-2.3931</v>
+        <v>-2.3953</v>
       </c>
       <c r="D125" t="n">
-        <v>0.3281</v>
+        <v>0.3271</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -15972,10 +15972,10 @@
         </is>
       </c>
       <c r="C126" t="n">
-        <v>-1.3476</v>
+        <v>-1.3606</v>
       </c>
       <c r="D126" t="n">
-        <v>0.8149</v>
+        <v>0.8107</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -15995,10 +15995,10 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>0.06279999999999999</v>
+        <v>0.0595</v>
       </c>
       <c r="D127" t="n">
-        <v>0.9873</v>
+        <v>0.9872</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -16018,10 +16018,10 @@
         </is>
       </c>
       <c r="C128" t="n">
-        <v>-1.204</v>
+        <v>-1.2254</v>
       </c>
       <c r="D128" t="n">
-        <v>0.8568</v>
+        <v>0.8511</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -16041,10 +16041,10 @@
         </is>
       </c>
       <c r="C129" t="n">
-        <v>-0.5289</v>
+        <v>-0.5329</v>
       </c>
       <c r="D129" t="n">
-        <v>0.9622000000000001</v>
+        <v>0.9619</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -16064,10 +16064,10 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>-2.1897</v>
+        <v>-2.1975</v>
       </c>
       <c r="D130" t="n">
-        <v>0.4297</v>
+        <v>0.4257</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -16087,10 +16087,10 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>-1.6061</v>
+        <v>-1.6132</v>
       </c>
       <c r="D131" t="n">
-        <v>0.7183</v>
+        <v>0.7153</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -22616,7 +22616,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.106</v>
+        <v>0.111</v>
       </c>
       <c r="C13" t="n">
         <v>3</v>
@@ -22628,7 +22628,7 @@
         <v>0.2532</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.5337</v>
+        <v>-0.5189</v>
       </c>
     </row>
   </sheetData>
@@ -22903,7 +22903,7 @@
         <v>10</v>
       </c>
       <c r="C14" t="n">
-        <v>0.2065</v>
+        <v>0.2189</v>
       </c>
     </row>
   </sheetData>
@@ -35156,10 +35156,10 @@
         <v>53.05</v>
       </c>
       <c r="E14" t="n">
-        <v>-93.19</v>
+        <v>-93.2</v>
       </c>
       <c r="F14" t="n">
-        <v>-96.8</v>
+        <v>-96.81</v>
       </c>
     </row>
   </sheetData>
@@ -35507,19 +35507,19 @@
         <v>2.2</v>
       </c>
       <c r="C13" t="n">
-        <v>467.44</v>
+        <v>467.68</v>
       </c>
       <c r="D13" t="n">
         <v>3</v>
       </c>
       <c r="E13" t="n">
-        <v>417.73</v>
+        <v>417.44</v>
       </c>
       <c r="F13" t="n">
         <v>2.4</v>
       </c>
       <c r="G13" t="n">
-        <v>371.99</v>
+        <v>372.07</v>
       </c>
     </row>
   </sheetData>
@@ -36897,13 +36897,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>15.523</v>
+        <v>15.547</v>
       </c>
       <c r="C13" t="n">
-        <v>0.101</v>
+        <v>0.128</v>
       </c>
       <c r="D13" t="n">
-        <v>0.266</v>
+        <v>0.335</v>
       </c>
       <c r="E13" t="n">
         <v>0.72</v>
@@ -37706,7 +37706,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1.206</v>
+        <v>1.27</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -38316,13 +38316,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>-0.00583</v>
+        <v>-0.00791</v>
       </c>
       <c r="C14" t="n">
-        <v>1.02</v>
+        <v>1.14</v>
       </c>
       <c r="D14" t="n">
-        <v>0.788</v>
+        <v>1.062</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -38616,13 +38616,13 @@
         <v>10</v>
       </c>
       <c r="C14" t="n">
-        <v>-1.238</v>
+        <v>-1.332</v>
       </c>
       <c r="D14" t="n">
-        <v>8.31</v>
+        <v>8.375999999999999</v>
       </c>
       <c r="E14" t="n">
-        <v>30.417</v>
+        <v>30.711</v>
       </c>
     </row>
   </sheetData>
@@ -38932,7 +38932,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>-0.174</v>
+        <v>-0.381</v>
       </c>
       <c r="C14" t="n">
         <v>-133228</v>
@@ -52918,10 +52918,10 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.01026</v>
+        <v>0.01027</v>
       </c>
       <c r="C14" t="n">
-        <v>0.00041</v>
+        <v>0.00042</v>
       </c>
       <c r="D14" t="n">
         <v>0.01282</v>
@@ -53029,13 +53029,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>7698.37</v>
+        <v>7682.41</v>
       </c>
       <c r="D4" t="n">
-        <v>3.47</v>
+        <v>3.25</v>
       </c>
       <c r="E4" t="n">
-        <v>15.87</v>
+        <v>15.63</v>
       </c>
     </row>
     <row r="5">
@@ -53795,10 +53795,10 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>15.89</v>
+        <v>16.01</v>
       </c>
       <c r="C13" t="n">
-        <v>15.754</v>
+        <v>15.856</v>
       </c>
       <c r="D13" t="n">
         <v>0.625</v>
@@ -54892,7 +54892,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>-0.6820000000000001</v>
+        <v>-0.712</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -54900,7 +54900,7 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0.175</v>
+        <v>0.164</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -55233,25 +55233,25 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.001592</v>
+        <v>0.00159</v>
       </c>
       <c r="C11" t="n">
-        <v>5.44</v>
+        <v>5.33</v>
       </c>
       <c r="D11" t="n">
-        <v>97.78</v>
+        <v>98.01000000000001</v>
       </c>
       <c r="E11" t="n">
-        <v>33.67</v>
+        <v>33.98</v>
       </c>
       <c r="F11" t="n">
-        <v>39.43</v>
+        <v>39.75</v>
       </c>
       <c r="G11" t="n">
-        <v>-2.42</v>
+        <v>-0.97</v>
       </c>
       <c r="H11" t="n">
-        <v>5.24</v>
+        <v>5.21</v>
       </c>
     </row>
   </sheetData>
@@ -56051,7 +56051,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>9.183999999999999</v>
+        <v>9.154</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -56059,10 +56059,10 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>-9.948</v>
+        <v>-10.092</v>
       </c>
       <c r="F14" t="n">
-        <v>19.132</v>
+        <v>19.247</v>
       </c>
     </row>
   </sheetData>
@@ -58961,16 +58961,16 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>-0.174</v>
+        <v>-0.381</v>
       </c>
       <c r="C14" t="n">
-        <v>3.467</v>
+        <v>3.252</v>
       </c>
       <c r="D14" t="n">
-        <v>21.354</v>
+        <v>21.103</v>
       </c>
       <c r="E14" t="n">
-        <v>15.875</v>
+        <v>15.635</v>
       </c>
       <c r="F14" t="n">
         <v>16.076</v>
@@ -59725,10 +59725,10 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>15.89</v>
+        <v>16.01</v>
       </c>
       <c r="C13" t="n">
-        <v>20.2</v>
+        <v>20.201</v>
       </c>
       <c r="D13" t="n">
         <v>0.02404</v>
@@ -59737,7 +59737,7 @@
         <v>28.8</v>
       </c>
       <c r="F13" t="n">
-        <v>-4.31</v>
+        <v>-4.191</v>
       </c>
     </row>
   </sheetData>
@@ -65001,7 +65001,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>-0.004876</v>
+        <v>-0.004902</v>
       </c>
     </row>
   </sheetData>
@@ -66085,10 +66085,10 @@
         <v>0.00881</v>
       </c>
       <c r="C13" t="n">
-        <v>0.06818</v>
+        <v>0.0683</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.0385</v>
+        <v>-0.03855</v>
       </c>
     </row>
   </sheetData>
@@ -69275,7 +69275,7 @@
         <v>-1.107</v>
       </c>
       <c r="C14" t="n">
-        <v>2.403</v>
+        <v>2.402</v>
       </c>
       <c r="D14" t="n">
         <v>0.421</v>
@@ -69522,13 +69522,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1.1387</v>
+        <v>1.1216</v>
       </c>
       <c r="C14" t="n">
-        <v>1.1201</v>
+        <v>1.1024</v>
       </c>
       <c r="D14" t="n">
-        <v>1.626</v>
+        <v>1.6031</v>
       </c>
     </row>
   </sheetData>
@@ -72461,7 +72461,7 @@
         <v>2262</v>
       </c>
       <c r="G14" t="n">
-        <v>0.01026</v>
+        <v>0.01027</v>
       </c>
     </row>
   </sheetData>
@@ -75679,7 +75679,7 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>15.967</v>
+        <v>16.097</v>
       </c>
     </row>
     <row r="123">
@@ -75702,7 +75702,7 @@
         </is>
       </c>
       <c r="E123" t="n">
-        <v>6.526</v>
+        <v>6.542</v>
       </c>
     </row>
     <row r="124">
@@ -75725,7 +75725,7 @@
         </is>
       </c>
       <c r="E124" t="n">
-        <v>5.059</v>
+        <v>4.824</v>
       </c>
     </row>
     <row r="125">
@@ -75748,7 +75748,7 @@
         </is>
       </c>
       <c r="E125" t="n">
-        <v>1.089</v>
+        <v>0.921</v>
       </c>
     </row>
     <row r="126">
@@ -75771,7 +75771,7 @@
         </is>
       </c>
       <c r="E126" t="n">
-        <v>-2.063</v>
+        <v>-2.201</v>
       </c>
     </row>
     <row r="127">
@@ -75794,7 +75794,7 @@
         </is>
       </c>
       <c r="E127" t="n">
-        <v>-2.495</v>
+        <v>-2.424</v>
       </c>
     </row>
     <row r="128">
@@ -75817,7 +75817,7 @@
         </is>
       </c>
       <c r="E128" t="n">
-        <v>-6.617</v>
+        <v>-6.801</v>
       </c>
     </row>
     <row r="129">
@@ -75840,7 +75840,7 @@
         </is>
       </c>
       <c r="E129" t="n">
-        <v>-7.514</v>
+        <v>-7.682</v>
       </c>
     </row>
     <row r="130">
@@ -75863,7 +75863,7 @@
         </is>
       </c>
       <c r="E130" t="n">
-        <v>-7.881</v>
+        <v>-7.981</v>
       </c>
     </row>
     <row r="131">
@@ -75886,7 +75886,7 @@
         </is>
       </c>
       <c r="E131" t="n">
-        <v>-14.45</v>
+        <v>-14.613</v>
       </c>
     </row>
   </sheetData>
@@ -76720,16 +76720,16 @@
         <v>3705</v>
       </c>
       <c r="D14" t="n">
-        <v>0.018</v>
+        <v>0.01795</v>
       </c>
       <c r="E14" t="n">
         <v>0.04655</v>
       </c>
       <c r="F14" t="n">
-        <v>-1.026</v>
+        <v>-1.028</v>
       </c>
       <c r="G14" t="n">
-        <v>0.3047</v>
+        <v>0.3038</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -78347,13 +78347,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.1298</v>
+        <v>0.1299</v>
       </c>
       <c r="C14" t="n">
-        <v>0.1171</v>
+        <v>0.1173</v>
       </c>
       <c r="D14" t="n">
-        <v>0.1412</v>
+        <v>0.1413</v>
       </c>
       <c r="E14" t="n">
         <v>1000</v>
@@ -78558,10 +78558,10 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>-0.2008</v>
+        <v>-0.1997</v>
       </c>
       <c r="C14" t="n">
-        <v>1.0264</v>
+        <v>1.0139</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-28T23:35Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-28 19:47 UTC</t>
+          <t>Genere le 2026-09-28 23:35 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-28 19:47 UTC</t>
+          <t>Rapport global — 2026-09-28 23:35 UTC</t>
         </is>
       </c>
     </row>
@@ -617,21 +617,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>**Regime monetaire emploi** — Chine : taux 1.54% (stable, niveau bas) -- chomage non_couvert  _(sans synthese)_ _(observation : 2026-09-24)_</t>
+          <t>**Regime monetaire emploi** — Chine : taux 1.54% (stable, niveau bas) -- chomage non_couvert  _(sans synthese)_ _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>**Regle taylor** — Taylor (2 termes, sans output gap)=6.03%, Fed reel=3.88%, ecart=-2.15pt -- accommodant (Fed en-dessous de la regle) _(observation : 2026-09-24)_</t>
+          <t>**Regle taylor** — Taylor (2 termes, sans output gap)=6.03%, Fed reel=3.88%, ecart=-2.15pt -- accommodant (Fed en-dessous de la regle) _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>**Chemin taux fed** — chemin de taux (pas des probabilites) : DFF=3.88%, prochaine reunion 2026-10-27 (11 a venir dans le calendrier) -- 0-1 mois: +13pb (hausse, confiance faible) | 1-3 mois: +48pb (hausse, confiance faible) | 3-6 mois: +56pb (hausse, confiance faible) | 6-12 mois: +80pb (hausse, confiance faible) _(observation : 2026-09-24)_</t>
+          <t>**Chemin taux fed** — chemin de taux (pas des probabilites) : DFF=3.88%, prochaine reunion 2026-10-27 (11 a venir dans le calendrier) -- 0-1 mois: +16pb (hausse, confiance faible) | 1-3 mois: +46pb (hausse, confiance faible) | 3-6 mois: +54pb (hausse, confiance faible) | 6-12 mois: +79pb (hausse, confiance faible) _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>**Matieres premieres macro** — le ratio cuivre/or monte -- la croissance domine la peur (+5.3% sur 3 mois). Brent 98.0$ (+34.0% sur 3 mois, +39.8% sur 12 mois), gaz -1.0% sur 3 mois, ecart Brent-WTI +5.2$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-28)_</t>
+          <t>**Matieres premieres macro** — le ratio cuivre/or monte -- la croissance domine la peur (+5.5% sur 3 mois). Brent 98.5$ (+34.7% sur 3 mois, +40.5% sur 12 mois), gaz -1.2% sur 3 mois, ecart Brent-WTI +5.4$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -841,14 +841,14 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>**Taux reel us** — nominal=3.88%, inflation YoY=3.35%, reel=0.53% -- restrictif (taux reel positif et eleve) _(observation : 2026-09-24)_</t>
+          <t>**Taux reel us** — nominal=3.88%, inflation YoY=3.35%, reel=0.53% -- restrictif (taux reel positif et eleve) _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>**Courbe taux us** — 10 ans=5.18%, 2 ans=4.87%, spread=+0.31pt -- normale (0 run(s) consecutif(s) dans l'historique accumule) _(observation : 2026-09-24)_</t>
+          <t>**Courbe taux us** — 10 ans=5.17%, 2 ans=4.81%, spread=+0.36pt -- normale (0 run(s) consecutif(s) dans l'historique accumule) _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
@@ -862,7 +862,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>**Conditions financieres** — indice conditions financieres=+0.111 (3 composantes: {'taux_directeur': 0.5985724560125544, 'courbe_inversee': 0.2531563730537784, 'vix': -0.5188744650175076}) -- conditions proches de la normale _(observation : 2026-09-24)_</t>
+          <t>**Conditions financieres** — indice conditions financieres=+0.086 (3 composantes: {'taux_directeur': 0.5982151864455719, 'courbe_inversee': 0.17031877422284264, 'vix': -0.5114551673321737}) -- conditions proches de la normale _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
@@ -883,14 +883,14 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>**Stationnarite taux** — 1/5 series stationnaires (niveau, pas en difference) -- a garder en tete avant toute correlation/regression sur ces series telles quelles  _(sans synthese)_ _(observation : 2026-09-24)_</t>
+          <t>**Stationnarite taux** — 1/5 series stationnaires (niveau, pas en difference) -- a garder en tete avant toute correlation/regression sur ces series telles quelles  _(sans synthese)_ _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>**Cointegration taux** — 1/10 paires cointegrees  _(sans synthese)_ _(observation : 2026-09-24)_</t>
+          <t>**Cointegration taux** — 1/10 paires cointegrees  _(sans synthese)_ _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
@@ -904,7 +904,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>**Hp filter taux** — taux 10 ans observe=5.180%, tendance HP=4.960%, ecart cyclique=+0.220pt -- au-dessus de sa tendance locale _(observation : 2026-09-24)_</t>
+          <t>**Hp filter taux** — taux 10 ans observe=5.170%, tendance HP=4.983%, ecart cyclique=+0.187pt -- au-dessus de sa tendance locale _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
@@ -953,7 +953,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>**Differentiel taux change** — 8 paires testees sur variations a 21 jours -- le lien taux/change tient sur 7 paire(s) apres correction pour tests multiples : EURUSD, USDJPY, USDCAD, AUDUSD, USDSEK, EURJPY, EURGBP _(observation : 2026-09-24)_</t>
+          <t>**Differentiel taux change** — 8 paires testees sur variations a 21 jours -- le lien taux/change tient sur 6 paire(s) apres correction pour tests multiples : EURUSD, USDJPY, USDCAD, AUDUSD, USDSEK, EURJPY _(observation : 2026-09-24)_</t>
         </is>
       </c>
     </row>
@@ -981,21 +981,21 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>**Beta facteur macro** — beta SP500/DGS10 (60j) = -0.0790 (rendement SP500 pour +1pt de taux 10 ans, 57/60 jours avec variation reelle) -- sensibilite elevee au facteur macro (choc de +100pb extrapole = -7.6%) _(observation : 2026-09-24)_</t>
+          <t>**Beta facteur macro** — beta SP500/DGS10 (60j) = -0.0794 (rendement SP500 pour +1pt de taux 10 ans, 57/60 jours avec variation reelle) -- sensibilite elevee au facteur macro (choc de +100pb extrapole = -7.6%) _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>**Momentum prix** — SP500 momentum 12-1 mois = 16.08% -- haussier (momentum positif), detail 1/3/6/12m = [-0.38, 3.25, 21.1, 15.63] _(observation : 2026-09-28)_</t>
+          <t>**Momentum prix** — SP500 momentum 12-1 mois = 16.08% -- haussier (momentum positif), detail 1/3/6/12m = [-0.36, 3.27, 21.12, 15.65] _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>**Carry proxy** — Chine : 1.54% vs US 3.88% -- diff=-2.34pt (carry negatif (taux &lt; US))  _(sans synthese)_ _(observation : 2026-09-24)_</t>
+          <t>**Carry proxy** — Chine : 1.54% vs US 3.88% -- diff=-2.34pt (carry negatif (taux &lt; US))  _(sans synthese)_ _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
@@ -1009,35 +1009,35 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>**Rotation sectorielle** — classement momentum 3 mois (10 secteurs) : 1. Energie (XLE) : +16.10% | 2. Sante (XLV) : +6.54% | 3. Technologie (XLK) : +4.82% | 4. Finance (XLF) : +0.92% | 5. Materiaux (XLB) : -2.20% _(observation : 2026-09-28)_</t>
+          <t>**Rotation sectorielle** — classement momentum 3 mois (10 secteurs) : 1. Energie (XLE) : +15.90% | 2. Sante (XLV) : +6.54% | 3. Technologie (XLK) : +4.92% | 4. Finance (XLF) : +0.88% | 5. Materiaux (XLB) : -2.35% _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>**Saisonnalite** — rendement journalier moyen ete=+0.0179%, hiver=+0.0465% (t=-1.03, p=0.3038) -- non significatif (attendu vu la faible puissance sur seulement ~2 ans) _(observation : 2026-09-28)_</t>
+          <t>**Saisonnalite** — rendement journalier moyen ete=+0.0180%, hiver=+0.0465% (t=-1.03, p=0.3039) -- non significatif (attendu vu la faible puissance sur seulement ~2 ans) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>**Dispersion sectorielle** — 10 secteurs, rendement moyen 3m=-1.33%, dispersion (ecart-type)=8.38pt, etendue=30.71pt -- dispersion intermediaire _(observation : 2026-09-28)_</t>
+          <t>**Dispersion sectorielle** — 10 secteurs, rendement moyen 3m=-1.38%, dispersion (ecart-type)=8.36pt, etendue=30.61pt -- dispersion intermediaire _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>**Low volatility** — tercile bas-vol ['XLF', 'XLRE', 'XLU'] Sharpe=-0.712 vs tercile haut-vol ['XLY', 'XLE', 'XLK'] Sharpe=0.164 -- anomalie low-vol non confirmee sur cet echantillon (puissance statistique faible, n petit -- limite assumee) _(observation : 2026-09-28)_</t>
+          <t>**Low volatility** — tercile bas-vol ['XLF', 'XLRE', 'XLU'] Sharpe=-0.720 vs tercile haut-vol ['XLY', 'XLE', 'XLK'] Sharpe=0.153 -- anomalie low-vol non confirmee sur cet echantillon (puissance statistique faible, n petit -- limite assumee) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>**Momentum cross sectional** — panier gagnant ['XLE', 'XLV', 'XLK'] (+9.15%) vs panier perdant ['XLI', 'XLRE', 'XLU'] (-10.09%) -- spread momentum=+19.25pt _(observation : 2026-09-28)_</t>
+          <t>**Momentum cross sectional** — panier gagnant ['XLE', 'XLV', 'XLK'] (+9.12%) vs panier perdant ['XLI', 'XLRE', 'XLU'] (-10.10%) -- spread momentum=+19.22pt _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>**Correlation facteurs** — correlation entre momentum 3m et beta-VIX, 10 secteurs : +0.219 (facteurs largement independants) _(observation : 2026-09-28)_</t>
+          <t>**Correlation facteurs** — correlation entre momentum 3m et beta-VIX, 10 secteurs : +0.215 (facteurs largement independants) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1107,7 +1107,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>**Divergence cot prix** — SP500 -0.38% sur 30j, COT net -10560 -&gt; -133228 -- pas de divergence _(observation : 2026-09-28)_</t>
+          <t>**Divergence cot prix** — SP500 -0.36% sur 30j, COT net -10560 -&gt; -133228 -- pas de divergence _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1191,14 +1191,14 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>**Vol cross asset** — 6 mesures de volatilite : Petrole (OVX) 88e pct, Or (GVZ) 86e pct, Nasdaq (VXN) 48e pct, Taux US (MOVE) 43e pct, Vol de la vol (VVIX) 37e pct, Actions US (VIX) 32e pct -- stress LOCALISE sur Petrole (OVX), Or (GVZ) pendant que le reste ne l'est pas -- episode propre a cette classe d'actifs, pas une aversion au risque d'ensemble _(observation : 2026-09-28)_</t>
+          <t>**Vol cross asset** — 6 mesures de volatilite : Petrole (OVX) 89e pct, Or (GVZ) 87e pct, Taux US (MOVE) 51e pct, Nasdaq (VXN) 48e pct, Vol de la vol (VVIX) 37e pct, Actions US (VIX) 32e pct -- stress LOCALISE sur Petrole (OVX), Or (GVZ) pendant que le reste ne l'est pas -- episode propre a cette classe d'actifs, pas une aversion au risque d'ensemble _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>**Volatilite ewma** — vol realisee 60j=0.11287248847520996, EWMA=0.1092 (tendance 10 runs: stable) _(observation : 2026-09-28)_</t>
+          <t>**Volatilite ewma** — vol realisee 60j=0.1128203817439559, EWMA=0.1090 (tendance 10 runs: stable) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1219,7 +1219,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>**Ornstein uhlenbeck vix** — VIX actuel=16.01, niveau moyen estime (mu)=20.20, demi-vie=28.8j, ecart actuel=-4.19 -- VIX actuel en-dessous de son niveau moyen de long terme _(observation : 2026-09-28)_</t>
+          <t>**Ornstein uhlenbeck vix** — VIX actuel=16.07, niveau moyen estime (mu)=20.20, demi-vie=28.8j, ecart actuel=-4.13 -- VIX actuel en-dessous de son niveau moyen de long terme _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1233,14 +1233,14 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>**Kalman niveau local** — VIX observe=16.01, filtre Kalman=15.86 (ecart-type=0.62), ratio signal/bruit=0.2052 -- le filtre lisse fortement le bruit, reagit lentement (ecart obs.-filtre=+0.15) _(observation : 2026-09-28)_</t>
+          <t>**Kalman niveau local** — VIX observe=16.07, filtre Kalman=15.91 (ecart-type=0.62), ratio signal/bruit=0.2052 -- le filtre lisse fortement le bruit, reagit lentement (ecart obs.-filtre=+0.16) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.37280971577723143 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.05236466910626937 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-28)_</t>
+          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.3730169650835773 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.052364093738951525 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1261,14 +1261,14 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>**Skew kurtosis** — skewness=-0.200 (asymetrie negative (pertes extremes &gt; gains extremes)), kurtosis exces=+1.014 (queues epaisses (risque extreme sous-estime par une hypothese normale)) _(observation : 2026-09-28)_</t>
+          <t>**Skew kurtosis** — skewness=-0.200 (asymetrie negative (pertes extremes &gt; gains extremes)), kurtosis exces=+1.015 (queues epaisses (risque extreme sous-estime par une hypothese normale)) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>**Ratios performance** — Sharpe=1.122 (bon), Sortino=1.102 (bon), Calmar=1.603 (bon) -- lecture sur fenetre 252j (~1 an, echantillon limite), seuils academiques standards, taux sans risque suppose nul _(observation : 2026-09-28)_</t>
+          <t>**Ratios performance** — Sharpe=1.123 (bon), Sortino=1.104 (bon), Calmar=1.605 (bon) -- lecture sur fenetre 252j (~1 an, echantillon limite), seuils academiques standards, taux sans risque suppose nul _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1282,14 +1282,14 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>**Stress test historique** — COVID_2020 (2020-02-19 -&gt; 2020-03-23) : chute historique=-33.9% -- rejouee sur le niveau actuel (7682) -&gt; 5076  _(sans synthese)_ _(observation : 2026-09-28)_</t>
+          <t>**Stress test historique** — COVID_2020 (2020-02-19 -&gt; 2020-03-23) : chute historique=-33.9% -- rejouee sur le niveau actuel (7684) -&gt; 5077  _(sans synthese)_ _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>**Sizing robuste** — vol point estimate=0.1299, IC90%=[0.1173, 0.1413] (1000 tirages bootstrap) -- intervalle etroit (18% du point estimate) -- estimation relativement fiable _(observation : 2026-09-28)_</t>
+          <t>**Sizing robuste** — vol point estimate=0.1299, IC90%=[0.1173, 0.1413] (1000 tirages bootstrap) -- intervalle etroit (19% du point estimate) -- estimation relativement fiable _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1303,21 +1303,21 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>**Detection saut** — Z-stat BNS (fenetre 22j)=1.270 (seuil ±1.96) -- pas de saut isole detecte _(observation : 2026-09-28)_</t>
+          <t>**Detection saut** — Z-stat BNS (fenetre 22j)=1.262 (seuil ±1.96) -- pas de saut isole detecte _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>**Choc taux** — beta SP500/DGS10=-0.0790 -- choc +100pb : -7.90% (SP500 7704 -&gt; 7096) ; choc -100pb : +7.90% (-&gt; 8313) _(observation : 2026-09-24)_</t>
+          <t>**Choc taux** — beta SP500/DGS10=-0.0794 -- choc +100pb : -7.94% (SP500 7743 -&gt; 7129) ; choc -100pb : +7.94% (-&gt; 8358) _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>**Qualite regime macro** — instabilite taux=0.0088, instabilite VIX=0.0683 -- score qualite du regime=-0.0386 (plus haut = regime plus stable/previsible) _(observation : 2026-09-24)_</t>
+          <t>**Qualite regime macro** — instabilite taux=0.0088, instabilite VIX=0.0684 -- score qualite du regime=-0.0386 (plus haut = regime plus stable/previsible) _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1331,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>**Decomposition stl** — VIX : tendance=15.55, composante saisonniere (periode 5j)=+0.128, residu=+0.335 -- la saisonnalite explique 0.72% de la variance totale (negligeable) _(observation : 2026-09-28)_</t>
+          <t>**Decomposition stl** — VIX : tendance=15.56, composante saisonniere (periode 5j)=+0.141, residu=+0.371 -- la saisonnalite explique 0.72% de la variance totale (negligeable) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1387,7 +1387,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>**Anomalie multivariee** — distance de Mahalanobis=1.062 (seuil 3.0) -- jour ordinaire _(observation : 2026-09-28)_</t>
+          <t>**Anomalie multivariee** — distance de Mahalanobis=1.027 (seuil 3.0) -- jour ordinaire _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1408,7 +1408,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>**Kmeans regimes** — 2050 points, k=3 -- point actuel (VIX=15.7, spread=+0.31, taux=3.88%) -&gt; cluster 1 (tailles : {0: 357, 1: 1369, 2: 324}) -- regime calme (VIX du cluster en-dessous de la moyenne historique) _(observation : 2026-09-24)_</t>
+          <t>**Kmeans regimes** — 2050 points, k=3 -- point actuel (VIX=14.9, spread=+0.36, taux=3.88%) -&gt; cluster 1 (tailles : {0: 357, 1: 1369, 2: 324}) -- regime calme (VIX du cluster en-dessous de la moyenne historique) _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
@@ -1443,14 +1443,14 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>**Decomposition variance** — R² SP500~DGS10 (60j) = 0.2696 -- 27.0% de la variance des rendements SP500 expliquee par les variations du taux 10 ans (le reste = idiosyncratique/autres facteurs) _(observation : 2026-09-24)_</t>
+          <t>**Decomposition variance** — R² SP500~DGS10 (60j) = 0.2703 -- 27.0% de la variance des rendements SP500 expliquee par les variations du taux 10 ans (le reste = idiosyncratique/autres facteurs) _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>**Test chow** — test de Chow (taux 10 ans, 1ere vs 2eme moitie des 12 derniers mois) : F=567.167, p=0.0000 -- RUPTURE structurelle significative _(observation : 2026-09-24)_</t>
+          <t>**Test chow** — test de Chow (taux 10 ans, 1ere vs 2eme moitie des 12 derniers mois) : F=560.405, p=0.0000 -- RUPTURE structurelle significative _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
@@ -1493,7 +1493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2535,6 +2535,90 @@
         <v>3.88</v>
       </c>
       <c r="E49" t="n">
+        <v>-2.34</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Zone_euro</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D50" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="E50" t="n">
+        <v>-1.38</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Royaume-Uni</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>3.7305</v>
+      </c>
+      <c r="D51" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="E51" t="n">
+        <v>-0.149</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Japon</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>0.977</v>
+      </c>
+      <c r="D52" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="E52" t="n">
+        <v>-2.903</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Chine</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="D53" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="E53" t="n">
         <v>-2.34</v>
       </c>
     </row>
@@ -2979,7 +3063,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F61"/>
+  <dimension ref="A1:F66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4697,6 +4781,146 @@
         <v>0.0002</v>
       </c>
       <c r="F61" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>DFF</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>-0.5032</v>
+      </c>
+      <c r="E62" t="n">
+        <v>0.8914</v>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Zone_euro</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>ECBDFR</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>-0.5818</v>
+      </c>
+      <c r="E63" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Royaume-Uni</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>IUDSOIA</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>-0.1568</v>
+      </c>
+      <c r="E64" t="n">
+        <v>0.9435</v>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Japon</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>IRSTCI01JPM156N</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>-1.9195</v>
+      </c>
+      <c r="E65" t="n">
+        <v>0.3229</v>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Chine</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>IR3TIB01CNM156N</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>-4.4511</v>
+      </c>
+      <c r="E66" t="n">
+        <v>0.0002</v>
+      </c>
+      <c r="F66" t="inlineStr">
         <is>
           <t>True</t>
         </is>
@@ -5453,7 +5677,7 @@
         <v>-56.78</v>
       </c>
       <c r="F26" t="n">
-        <v>3320.69</v>
+        <v>3321.25</v>
       </c>
     </row>
     <row r="27">
@@ -5481,7 +5705,7 @@
         <v>-33.92</v>
       </c>
       <c r="F27" t="n">
-        <v>5076.16</v>
+        <v>5077</v>
       </c>
     </row>
   </sheetData>
@@ -5645,7 +5869,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5865,6 +6089,22 @@
         <v>3.353</v>
       </c>
       <c r="D13" t="n">
+        <v>0.527</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="C14" t="n">
+        <v>3.353</v>
+      </c>
+      <c r="D14" t="n">
         <v>0.527</v>
       </c>
     </row>
@@ -5879,7 +6119,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6121,6 +6361,24 @@
         <v>0</v>
       </c>
       <c r="D13" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>560.405</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" t="inlineStr">
         <is>
           <t>True</t>
         </is>
@@ -7003,10 +7261,10 @@
         <v>5</v>
       </c>
       <c r="C14" t="n">
-        <v>0.07554</v>
+        <v>0.07556</v>
       </c>
       <c r="D14" t="n">
-        <v>0.00417</v>
+        <v>0.00416</v>
       </c>
     </row>
   </sheetData>
@@ -8247,10 +8505,10 @@
         <v>10</v>
       </c>
       <c r="C14" t="n">
-        <v>0.37281</v>
+        <v>0.37302</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.052365</v>
+        <v>-0.052364</v>
       </c>
     </row>
   </sheetData>
@@ -8319,10 +8577,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>55.7</v>
+        <v>56.11</v>
       </c>
       <c r="D2" t="n">
-        <v>88.3</v>
+        <v>88.8</v>
       </c>
       <c r="E2" t="n">
         <v>1260</v>
@@ -8345,10 +8603,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>24.78</v>
+        <v>24.83</v>
       </c>
       <c r="D3" t="n">
-        <v>86.3</v>
+        <v>86.7</v>
       </c>
       <c r="E3" t="n">
         <v>1260</v>
@@ -8362,7 +8620,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Nasdaq (VXN)</t>
+          <t>Taux US (MOVE)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -8371,10 +8629,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>22.18</v>
+        <v>101.82</v>
       </c>
       <c r="D4" t="n">
-        <v>48.1</v>
+        <v>51.3</v>
       </c>
       <c r="E4" t="n">
         <v>1260</v>
@@ -8388,19 +8646,19 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Taux US (MOVE)</t>
+          <t>Nasdaq (VXN)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>96</v>
+        <v>22.13</v>
       </c>
       <c r="D5" t="n">
-        <v>43.3</v>
+        <v>47.8</v>
       </c>
       <c r="E5" t="n">
         <v>1260</v>
@@ -8423,10 +8681,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>90.83</v>
+        <v>91.02</v>
       </c>
       <c r="D6" t="n">
-        <v>36.9</v>
+        <v>37.4</v>
       </c>
       <c r="E6" t="n">
         <v>1260</v>
@@ -8449,10 +8707,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>16.01</v>
+        <v>16.07</v>
       </c>
       <c r="D7" t="n">
-        <v>32</v>
+        <v>32.5</v>
       </c>
       <c r="E7" t="n">
         <v>1260</v>
@@ -8746,16 +9004,16 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.1092</v>
+        <v>0.109</v>
       </c>
       <c r="C14" t="n">
-        <v>0.0881</v>
+        <v>0.08740000000000001</v>
       </c>
       <c r="D14" t="n">
-        <v>0.1112</v>
+        <v>0.1111</v>
       </c>
       <c r="E14" t="n">
-        <v>0.1129</v>
+        <v>0.1128</v>
       </c>
     </row>
   </sheetData>
@@ -9411,7 +9669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:J29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10582,6 +10840,190 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>0-1 mois</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" t="n">
+        <v>4.04</v>
+      </c>
+      <c r="F26" t="n">
+        <v>16</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>hausse</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>forward_treasury_proxy</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>mouvement net de fenetre; aucune probabilite isolee par reunion</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>1-3 mois</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>2026-12-25</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>2</v>
+      </c>
+      <c r="E27" t="n">
+        <v>4.34</v>
+      </c>
+      <c r="F27" t="n">
+        <v>46</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>hausse</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>forward_treasury_proxy</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>mouvement net de fenetre; aucune probabilite isolee par reunion</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>3-6 mois</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>2027-03-26</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>5</v>
+      </c>
+      <c r="E28" t="n">
+        <v>4.42</v>
+      </c>
+      <c r="F28" t="n">
+        <v>54</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>hausse</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>forward_treasury_proxy</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>mouvement net de fenetre; aucune probabilite isolee par reunion</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>6-12 mois</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>2027-09-25</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>9</v>
+      </c>
+      <c r="E29" t="n">
+        <v>4.67</v>
+      </c>
+      <c r="F29" t="n">
+        <v>79</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>hausse</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>forward_treasury_proxy</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>mouvement net de fenetre; aucune probabilite isolee par reunion</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10593,7 +11035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10940,6 +11382,31 @@
       </c>
       <c r="G13" t="n">
         <v>8312.6</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>-0.07937</v>
+      </c>
+      <c r="C14" t="n">
+        <v>7743.41</v>
+      </c>
+      <c r="D14" t="n">
+        <v>-7.94</v>
+      </c>
+      <c r="E14" t="n">
+        <v>7128.8</v>
+      </c>
+      <c r="F14" t="n">
+        <v>7.94</v>
+      </c>
+      <c r="G14" t="n">
+        <v>8358</v>
       </c>
     </row>
   </sheetData>
@@ -11225,7 +11692,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>12.988</v>
+        <v>12.987</v>
       </c>
       <c r="C14" t="n">
         <v>-1.286</v>
@@ -11234,7 +11701,7 @@
         <v>-2.632</v>
       </c>
       <c r="E14" t="n">
-        <v>-3.978</v>
+        <v>-3.977</v>
       </c>
     </row>
   </sheetData>
@@ -15880,10 +16347,10 @@
         </is>
       </c>
       <c r="C122" t="n">
-        <v>-2.544</v>
+        <v>-2.5374</v>
       </c>
       <c r="D122" t="n">
-        <v>0.26</v>
+        <v>0.2628</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -15903,10 +16370,10 @@
         </is>
       </c>
       <c r="C123" t="n">
-        <v>-1.8576</v>
+        <v>-1.8514</v>
       </c>
       <c r="D123" t="n">
-        <v>0.6014</v>
+        <v>0.6044</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -15926,10 +16393,10 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>-2.1473</v>
+        <v>-2.1451</v>
       </c>
       <c r="D124" t="n">
-        <v>0.4517</v>
+        <v>0.4528</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -15949,7 +16416,7 @@
         </is>
       </c>
       <c r="C125" t="n">
-        <v>-2.3953</v>
+        <v>-2.3952</v>
       </c>
       <c r="D125" t="n">
         <v>0.3271</v>
@@ -15972,10 +16439,10 @@
         </is>
       </c>
       <c r="C126" t="n">
-        <v>-1.3606</v>
+        <v>-1.3635</v>
       </c>
       <c r="D126" t="n">
-        <v>0.8107</v>
+        <v>0.8097</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -15995,10 +16462,10 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>0.0595</v>
+        <v>0.0851</v>
       </c>
       <c r="D127" t="n">
-        <v>0.9872</v>
+        <v>0.9877</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -16018,10 +16485,10 @@
         </is>
       </c>
       <c r="C128" t="n">
-        <v>-1.2254</v>
+        <v>-1.2195</v>
       </c>
       <c r="D128" t="n">
-        <v>0.8511</v>
+        <v>0.8527</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -16041,10 +16508,10 @@
         </is>
       </c>
       <c r="C129" t="n">
-        <v>-0.5329</v>
+        <v>-0.5135999999999999</v>
       </c>
       <c r="D129" t="n">
-        <v>0.9619</v>
+        <v>0.9634</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -16064,10 +16531,10 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>-2.1975</v>
+        <v>-2.1811</v>
       </c>
       <c r="D130" t="n">
-        <v>0.4257</v>
+        <v>0.4341</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -16087,10 +16554,10 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>-1.6132</v>
+        <v>-1.6158</v>
       </c>
       <c r="D131" t="n">
-        <v>0.7153</v>
+        <v>0.7141999999999999</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -16109,7 +16576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F121"/>
+  <dimension ref="A1:F131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19507,6 +19974,286 @@
         <v>0.7195</v>
       </c>
       <c r="F121" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Chine</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Japon</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>-3.6969</v>
+      </c>
+      <c r="E122" t="n">
+        <v>0.0185</v>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Chine</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Royaume-Uni</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>-2.417</v>
+      </c>
+      <c r="E123" t="n">
+        <v>0.3168</v>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Chine</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>-2.0335</v>
+      </c>
+      <c r="E124" t="n">
+        <v>0.5111</v>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Chine</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Zone_euro</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>-2.1259</v>
+      </c>
+      <c r="E125" t="n">
+        <v>0.4628</v>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Japon</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Royaume-Uni</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>-1.975</v>
+      </c>
+      <c r="E126" t="n">
+        <v>0.5415</v>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Japon</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>-0.3664</v>
+      </c>
+      <c r="E127" t="n">
+        <v>0.9726</v>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Japon</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Zone_euro</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>-0.7129</v>
+      </c>
+      <c r="E128" t="n">
+        <v>0.9452</v>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Royaume-Uni</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>-1.9784</v>
+      </c>
+      <c r="E129" t="n">
+        <v>0.5397999999999999</v>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Royaume-Uni</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Zone_euro</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>-2.2116</v>
+      </c>
+      <c r="E130" t="n">
+        <v>0.4184</v>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Zone_euro</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>-1.6051</v>
+      </c>
+      <c r="E131" t="n">
+        <v>0.7187</v>
+      </c>
+      <c r="F131" t="inlineStr">
         <is>
           <t>False</t>
         </is>
@@ -22324,7 +23071,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -22629,6 +23376,28 @@
       </c>
       <c r="F13" t="n">
         <v>-0.5189</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.0857</v>
+      </c>
+      <c r="C14" t="n">
+        <v>3</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.5982</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.1703</v>
+      </c>
+      <c r="F14" t="n">
+        <v>-0.5115</v>
       </c>
     </row>
   </sheetData>
@@ -22903,7 +23672,7 @@
         <v>10</v>
       </c>
       <c r="C14" t="n">
-        <v>0.2189</v>
+        <v>0.2152</v>
       </c>
     </row>
   </sheetData>
@@ -34533,7 +35302,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -34817,6 +35586,27 @@
         <v>0.31</v>
       </c>
       <c r="E13" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>5.17</v>
+      </c>
+      <c r="C14" t="n">
+        <v>4.81</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="E14" t="inlineStr">
         <is>
           <t>False</t>
         </is>
@@ -35507,19 +36297,19 @@
         <v>2.2</v>
       </c>
       <c r="C13" t="n">
-        <v>467.68</v>
+        <v>467.8</v>
       </c>
       <c r="D13" t="n">
         <v>3</v>
       </c>
       <c r="E13" t="n">
-        <v>417.44</v>
+        <v>417.29</v>
       </c>
       <c r="F13" t="n">
         <v>2.4</v>
       </c>
       <c r="G13" t="n">
-        <v>372.07</v>
+        <v>372.11</v>
       </c>
     </row>
   </sheetData>
@@ -36897,13 +37687,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>15.547</v>
+        <v>15.559</v>
       </c>
       <c r="C13" t="n">
-        <v>0.128</v>
+        <v>0.141</v>
       </c>
       <c r="D13" t="n">
-        <v>0.335</v>
+        <v>0.371</v>
       </c>
       <c r="E13" t="n">
         <v>0.72</v>
@@ -36920,7 +37710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -37099,6 +37889,19 @@
       </c>
       <c r="C13" t="n">
         <v>26.96</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.27034</v>
+      </c>
+      <c r="C14" t="n">
+        <v>27.03</v>
       </c>
     </row>
   </sheetData>
@@ -37706,7 +38509,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1.27</v>
+        <v>1.262</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -37792,10 +38595,10 @@
         <v>-1.641</v>
       </c>
       <c r="D2" t="n">
-        <v>0.305</v>
+        <v>0.314</v>
       </c>
       <c r="E2" t="n">
-        <v>0.00078</v>
+        <v>0.00054</v>
       </c>
       <c r="F2" t="n">
         <v>118</v>
@@ -37821,7 +38624,7 @@
         <v>2.597</v>
       </c>
       <c r="D3" t="n">
-        <v>0.555</v>
+        <v>0.513</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
@@ -37850,10 +38653,10 @@
         <v>-0.106</v>
       </c>
       <c r="D4" t="n">
-        <v>0.067</v>
+        <v>0.134</v>
       </c>
       <c r="E4" t="n">
-        <v>0.475</v>
+        <v>0.14953</v>
       </c>
       <c r="F4" t="n">
         <v>117</v>
@@ -37879,7 +38682,7 @@
         <v>1.48</v>
       </c>
       <c r="D5" t="n">
-        <v>0.536</v>
+        <v>0.505</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
@@ -37908,10 +38711,10 @@
         <v>0.097</v>
       </c>
       <c r="D6" t="n">
-        <v>0.338</v>
+        <v>0.342</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0002</v>
+        <v>0.00017</v>
       </c>
       <c r="F6" t="n">
         <v>116</v>
@@ -37937,13 +38740,13 @@
         <v>2.08</v>
       </c>
       <c r="D7" t="n">
-        <v>0.281</v>
+        <v>0.307</v>
       </c>
       <c r="E7" t="n">
-        <v>0.00213</v>
+        <v>0.0008</v>
       </c>
       <c r="F7" t="n">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -37966,10 +38769,10 @@
         <v>1.113</v>
       </c>
       <c r="D8" t="n">
-        <v>0.355</v>
+        <v>0.337</v>
       </c>
       <c r="E8" t="n">
-        <v>1e-05</v>
+        <v>2e-05</v>
       </c>
       <c r="F8" t="n">
         <v>150</v>
@@ -37995,17 +38798,17 @@
         <v>-1.581</v>
       </c>
       <c r="D9" t="n">
-        <v>0.355</v>
+        <v>0.09</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>0.26214</v>
       </c>
       <c r="F9" t="n">
         <v>158</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>oui</t>
+          <t>non</t>
         </is>
       </c>
     </row>
@@ -38316,13 +39119,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>-0.00791</v>
+        <v>-0.00774</v>
       </c>
       <c r="C14" t="n">
-        <v>1.14</v>
+        <v>1.2</v>
       </c>
       <c r="D14" t="n">
-        <v>1.062</v>
+        <v>1.027</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -38616,13 +39419,13 @@
         <v>10</v>
       </c>
       <c r="C14" t="n">
-        <v>-1.332</v>
+        <v>-1.383</v>
       </c>
       <c r="D14" t="n">
-        <v>8.375999999999999</v>
+        <v>8.363</v>
       </c>
       <c r="E14" t="n">
-        <v>30.711</v>
+        <v>30.612</v>
       </c>
     </row>
   </sheetData>
@@ -38932,7 +39735,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>-0.381</v>
+        <v>-0.364</v>
       </c>
       <c r="C14" t="n">
         <v>-133228</v>
@@ -48871,7 +49674,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>fred/DFF.csv</t>
+          <t>fred/IUDSOIA.csv</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -48900,7 +49703,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>fred/DFII10.csv</t>
+          <t>fred/MORTGAGE30US.csv</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -48912,13 +49715,13 @@
         <v>4</v>
       </c>
       <c r="D188" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E188" t="n">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="F188" t="n">
-        <v>3000</v>
+        <v>2896</v>
       </c>
       <c r="G188" t="inlineStr">
         <is>
@@ -48929,7 +49732,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>fred/DFII5.csv</t>
+          <t>souverains/UK_10A.csv</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -48947,7 +49750,7 @@
         <v>42</v>
       </c>
       <c r="F189" t="n">
-        <v>3000</v>
+        <v>9283</v>
       </c>
       <c r="G189" t="inlineStr">
         <is>
@@ -48958,7 +49761,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>fred/DGS1.csv</t>
+          <t>souverains/UK_20A.csv</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -48976,7 +49779,7 @@
         <v>42</v>
       </c>
       <c r="F190" t="n">
-        <v>3000</v>
+        <v>6754</v>
       </c>
       <c r="G190" t="inlineStr">
         <is>
@@ -48987,7 +49790,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>fred/DGS10.csv</t>
+          <t>souverains/UK_5A.csv</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -49005,7 +49808,7 @@
         <v>42</v>
       </c>
       <c r="F191" t="n">
-        <v>3000</v>
+        <v>8291</v>
       </c>
       <c r="G191" t="inlineStr">
         <is>
@@ -49016,16 +49819,16 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>fred/DGS1MO.csv</t>
+          <t>fred/BAMLC0A0CM.csv</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C192" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D192" t="n">
         <v>1</v>
@@ -49034,7 +49837,7 @@
         <v>42</v>
       </c>
       <c r="F192" t="n">
-        <v>3000</v>
+        <v>793</v>
       </c>
       <c r="G192" t="inlineStr">
         <is>
@@ -49045,16 +49848,16 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>fred/DGS2.csv</t>
+          <t>fred/BAMLC0A0CMEY.csv</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C193" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D193" t="n">
         <v>1</v>
@@ -49063,7 +49866,7 @@
         <v>42</v>
       </c>
       <c r="F193" t="n">
-        <v>3000</v>
+        <v>793</v>
       </c>
       <c r="G193" t="inlineStr">
         <is>
@@ -49074,16 +49877,16 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>fred/DGS30.csv</t>
+          <t>fred/BAMLEMCBPIOAS.csv</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C194" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D194" t="n">
         <v>1</v>
@@ -49092,7 +49895,7 @@
         <v>42</v>
       </c>
       <c r="F194" t="n">
-        <v>3000</v>
+        <v>793</v>
       </c>
       <c r="G194" t="inlineStr">
         <is>
@@ -49103,16 +49906,16 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>fred/DGS3MO.csv</t>
+          <t>fred/BAMLEMFSFCRPIOAS.csv</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C195" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D195" t="n">
         <v>1</v>
@@ -49121,7 +49924,7 @@
         <v>42</v>
       </c>
       <c r="F195" t="n">
-        <v>3000</v>
+        <v>793</v>
       </c>
       <c r="G195" t="inlineStr">
         <is>
@@ -49132,16 +49935,16 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>fred/DGS5.csv</t>
+          <t>fred/BAMLEMHBHYCRPIOAS.csv</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C196" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D196" t="n">
         <v>1</v>
@@ -49150,7 +49953,7 @@
         <v>42</v>
       </c>
       <c r="F196" t="n">
-        <v>3000</v>
+        <v>793</v>
       </c>
       <c r="G196" t="inlineStr">
         <is>
@@ -49161,16 +49964,16 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>fred/DGS6MO.csv</t>
+          <t>fred/BAMLEMPBPUBSICRPIOAS.csv</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C197" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D197" t="n">
         <v>1</v>
@@ -49179,7 +49982,7 @@
         <v>42</v>
       </c>
       <c r="F197" t="n">
-        <v>3000</v>
+        <v>793</v>
       </c>
       <c r="G197" t="inlineStr">
         <is>
@@ -49190,16 +49993,16 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>fred/IUDSOIA.csv</t>
+          <t>fred/BAMLH0A0HYM2.csv</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C198" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D198" t="n">
         <v>1</v>
@@ -49208,7 +50011,7 @@
         <v>42</v>
       </c>
       <c r="F198" t="n">
-        <v>3000</v>
+        <v>793</v>
       </c>
       <c r="G198" t="inlineStr">
         <is>
@@ -49219,25 +50022,25 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>fred/MORTGAGE30US.csv</t>
+          <t>fred/BAMLHE00EHYIEY.csv</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C199" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D199" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E199" t="n">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="F199" t="n">
-        <v>2896</v>
+        <v>793</v>
       </c>
       <c r="G199" t="inlineStr">
         <is>
@@ -49248,16 +50051,16 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>souverains/UK_10A.csv</t>
+          <t>fred/BAMLHE00EHYIOAS.csv</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C200" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D200" t="n">
         <v>1</v>
@@ -49266,7 +50069,7 @@
         <v>42</v>
       </c>
       <c r="F200" t="n">
-        <v>9283</v>
+        <v>793</v>
       </c>
       <c r="G200" t="inlineStr">
         <is>
@@ -49277,16 +50080,16 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>souverains/UK_20A.csv</t>
+          <t>fred/DFF.csv</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C201" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D201" t="n">
         <v>1</v>
@@ -49295,7 +50098,7 @@
         <v>42</v>
       </c>
       <c r="F201" t="n">
-        <v>6754</v>
+        <v>3000</v>
       </c>
       <c r="G201" t="inlineStr">
         <is>
@@ -49306,16 +50109,16 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>souverains/UK_5A.csv</t>
+          <t>fred/DFII10.csv</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C202" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D202" t="n">
         <v>1</v>
@@ -49324,7 +50127,7 @@
         <v>42</v>
       </c>
       <c r="F202" t="n">
-        <v>8291</v>
+        <v>3000</v>
       </c>
       <c r="G202" t="inlineStr">
         <is>
@@ -49335,16 +50138,16 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>tresor_us/dette_quotidienne.csv</t>
+          <t>fred/DFII5.csv</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C203" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D203" t="n">
         <v>1</v>
@@ -49353,7 +50156,7 @@
         <v>42</v>
       </c>
       <c r="F203" t="n">
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="G203" t="inlineStr">
         <is>
@@ -49364,16 +50167,16 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>tresor_us/solde_tresorerie.csv</t>
+          <t>fred/DGS1.csv</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C204" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D204" t="n">
         <v>1</v>
@@ -49382,7 +50185,7 @@
         <v>42</v>
       </c>
       <c r="F204" t="n">
-        <v>500</v>
+        <v>3000</v>
       </c>
       <c r="G204" t="inlineStr">
         <is>
@@ -49393,7 +50196,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>fred/BAMLC0A0CM.csv</t>
+          <t>fred/DGS10.csv</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -49411,7 +50214,7 @@
         <v>42</v>
       </c>
       <c r="F205" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G205" t="inlineStr">
         <is>
@@ -49422,7 +50225,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>fred/BAMLC0A0CMEY.csv</t>
+          <t>fred/DGS1MO.csv</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -49440,7 +50243,7 @@
         <v>42</v>
       </c>
       <c r="F206" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G206" t="inlineStr">
         <is>
@@ -49451,7 +50254,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>fred/BAMLEMCBPIOAS.csv</t>
+          <t>fred/DGS2.csv</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -49469,7 +50272,7 @@
         <v>42</v>
       </c>
       <c r="F207" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G207" t="inlineStr">
         <is>
@@ -49480,7 +50283,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>fred/BAMLEMFSFCRPIOAS.csv</t>
+          <t>fred/DGS30.csv</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -49498,7 +50301,7 @@
         <v>42</v>
       </c>
       <c r="F208" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G208" t="inlineStr">
         <is>
@@ -49509,7 +50312,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>fred/BAMLEMHBHYCRPIOAS.csv</t>
+          <t>fred/DGS3MO.csv</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -49527,7 +50330,7 @@
         <v>42</v>
       </c>
       <c r="F209" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G209" t="inlineStr">
         <is>
@@ -49538,7 +50341,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>fred/BAMLEMPBPUBSICRPIOAS.csv</t>
+          <t>fred/DGS5.csv</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -49556,7 +50359,7 @@
         <v>42</v>
       </c>
       <c r="F210" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G210" t="inlineStr">
         <is>
@@ -49567,7 +50370,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>fred/BAMLH0A0HYM2.csv</t>
+          <t>fred/DGS6MO.csv</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
@@ -49585,7 +50388,7 @@
         <v>42</v>
       </c>
       <c r="F211" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G211" t="inlineStr">
         <is>
@@ -49596,7 +50399,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>fred/BAMLHE00EHYIEY.csv</t>
+          <t>marches/indices/DAX.csv</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -49614,7 +50417,7 @@
         <v>42</v>
       </c>
       <c r="F212" t="n">
-        <v>793</v>
+        <v>3801</v>
       </c>
       <c r="G212" t="inlineStr">
         <is>
@@ -49625,7 +50428,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>fred/BAMLHE00EHYIOAS.csv</t>
+          <t>marches/indices/EUROSTOXX50.csv</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -49643,7 +50446,7 @@
         <v>42</v>
       </c>
       <c r="F213" t="n">
-        <v>793</v>
+        <v>3758</v>
       </c>
       <c r="G213" t="inlineStr">
         <is>
@@ -49654,7 +50457,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>fred/T10YIE.csv</t>
+          <t>marches/indices/FTSE100.csv</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -49672,7 +50475,7 @@
         <v>42</v>
       </c>
       <c r="F214" t="n">
-        <v>3000</v>
+        <v>3787</v>
       </c>
       <c r="G214" t="inlineStr">
         <is>
@@ -49741,7 +50544,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>marches/volatilite/MOVE.csv</t>
+          <t>souverains/CANADA_10A.csv</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -49759,7 +50562,7 @@
         <v>42</v>
       </c>
       <c r="F217" t="n">
-        <v>3689</v>
+        <v>6436</v>
       </c>
       <c r="G217" t="inlineStr">
         <is>
@@ -49770,7 +50573,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>souverains/CANADA_10A.csv</t>
+          <t>souverains/CANADA_2A.csv</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -49788,7 +50591,7 @@
         <v>42</v>
       </c>
       <c r="F218" t="n">
-        <v>6436</v>
+        <v>6435</v>
       </c>
       <c r="G218" t="inlineStr">
         <is>
@@ -49799,7 +50602,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>souverains/CANADA_2A.csv</t>
+          <t>souverains/CANADA_5A.csv</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -49828,7 +50631,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>souverains/CANADA_5A.csv</t>
+          <t>souverains/CANADA_LONG.csv</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -49857,7 +50660,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>souverains/CANADA_LONG.csv</t>
+          <t>souverains/SUEDE_10A.csv</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -49875,7 +50678,7 @@
         <v>42</v>
       </c>
       <c r="F221" t="n">
-        <v>6435</v>
+        <v>9202</v>
       </c>
       <c r="G221" t="inlineStr">
         <is>
@@ -49886,7 +50689,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_10A.csv</t>
+          <t>souverains/SUEDE_2A.csv</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -49915,7 +50718,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_2A.csv</t>
+          <t>souverains/SUEDE_5A.csv</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -49933,7 +50736,7 @@
         <v>42</v>
       </c>
       <c r="F223" t="n">
-        <v>9202</v>
+        <v>9204</v>
       </c>
       <c r="G223" t="inlineStr">
         <is>
@@ -49944,7 +50747,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_5A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -49962,7 +50765,7 @@
         <v>42</v>
       </c>
       <c r="F224" t="n">
-        <v>9204</v>
+        <v>5639</v>
       </c>
       <c r="G224" t="inlineStr">
         <is>
@@ -49973,7 +50776,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
@@ -50002,7 +50805,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -50031,7 +50834,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -50060,7 +50863,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -50089,7 +50892,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -50118,7 +50921,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -50147,7 +50950,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -50176,7 +50979,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
+          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -50205,7 +51008,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
+          <t>tresor_us/dette_quotidienne.csv</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -50223,7 +51026,7 @@
         <v>42</v>
       </c>
       <c r="F233" t="n">
-        <v>5639</v>
+        <v>2000</v>
       </c>
       <c r="G233" t="inlineStr">
         <is>
@@ -50234,16 +51037,16 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>fred/ECBDFR.csv</t>
+          <t>tresor_us/solde_tresorerie.csv</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C234" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D234" t="n">
         <v>1</v>
@@ -50252,7 +51055,7 @@
         <v>42</v>
       </c>
       <c r="F234" t="n">
-        <v>3000</v>
+        <v>500</v>
       </c>
       <c r="G234" t="inlineStr">
         <is>
@@ -50263,7 +51066,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>fred/RRPONTSYD.csv</t>
+          <t>fred/ECBDFR.csv</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -50292,7 +51095,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>marches/fx/AUDJPY.csv</t>
+          <t>fred/RRPONTSYD.csv</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -50310,7 +51113,7 @@
         <v>42</v>
       </c>
       <c r="F236" t="n">
-        <v>3908</v>
+        <v>3000</v>
       </c>
       <c r="G236" t="inlineStr">
         <is>
@@ -50321,7 +51124,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>marches/fx/AUDUSD.csv</t>
+          <t>fred/T10YIE.csv</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
@@ -50339,7 +51142,7 @@
         <v>42</v>
       </c>
       <c r="F237" t="n">
-        <v>3904</v>
+        <v>3000</v>
       </c>
       <c r="G237" t="inlineStr">
         <is>
@@ -50350,7 +51153,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>marches/fx/DXY.csv</t>
+          <t>marches/fx/AUDJPY.csv</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
@@ -50368,7 +51171,7 @@
         <v>42</v>
       </c>
       <c r="F238" t="n">
-        <v>3772</v>
+        <v>3908</v>
       </c>
       <c r="G238" t="inlineStr">
         <is>
@@ -50379,7 +51182,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>marches/fx/EURCHF.csv</t>
+          <t>marches/fx/AUDUSD.csv</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
@@ -50397,7 +51200,7 @@
         <v>42</v>
       </c>
       <c r="F239" t="n">
-        <v>3905</v>
+        <v>3904</v>
       </c>
       <c r="G239" t="inlineStr">
         <is>
@@ -50408,7 +51211,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>marches/fx/EURGBP.csv</t>
+          <t>marches/fx/DXY.csv</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
@@ -50426,7 +51229,7 @@
         <v>42</v>
       </c>
       <c r="F240" t="n">
-        <v>3907</v>
+        <v>3772</v>
       </c>
       <c r="G240" t="inlineStr">
         <is>
@@ -50437,7 +51240,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>marches/fx/EURJPY.csv</t>
+          <t>marches/fx/EURCHF.csv</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
@@ -50455,7 +51258,7 @@
         <v>42</v>
       </c>
       <c r="F241" t="n">
-        <v>3907</v>
+        <v>3905</v>
       </c>
       <c r="G241" t="inlineStr">
         <is>
@@ -50466,7 +51269,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>marches/fx/EURUSD.csv</t>
+          <t>marches/fx/EURGBP.csv</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
@@ -50484,7 +51287,7 @@
         <v>42</v>
       </c>
       <c r="F242" t="n">
-        <v>3904</v>
+        <v>3907</v>
       </c>
       <c r="G242" t="inlineStr">
         <is>
@@ -50495,7 +51298,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>marches/fx/GBPUSD.csv</t>
+          <t>marches/fx/EURJPY.csv</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
@@ -50513,7 +51316,7 @@
         <v>42</v>
       </c>
       <c r="F243" t="n">
-        <v>3905</v>
+        <v>3907</v>
       </c>
       <c r="G243" t="inlineStr">
         <is>
@@ -50524,7 +51327,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>marches/fx/NZDUSD.csv</t>
+          <t>marches/fx/EURUSD.csv</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -50542,7 +51345,7 @@
         <v>42</v>
       </c>
       <c r="F244" t="n">
-        <v>3905</v>
+        <v>3904</v>
       </c>
       <c r="G244" t="inlineStr">
         <is>
@@ -50553,7 +51356,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>marches/fx/USDCAD.csv</t>
+          <t>marches/fx/GBPUSD.csv</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -50571,7 +51374,7 @@
         <v>42</v>
       </c>
       <c r="F245" t="n">
-        <v>3904</v>
+        <v>3905</v>
       </c>
       <c r="G245" t="inlineStr">
         <is>
@@ -50582,7 +51385,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>marches/fx/USDCHF.csv</t>
+          <t>marches/fx/NZDUSD.csv</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -50600,7 +51403,7 @@
         <v>42</v>
       </c>
       <c r="F246" t="n">
-        <v>3902</v>
+        <v>3905</v>
       </c>
       <c r="G246" t="inlineStr">
         <is>
@@ -50611,7 +51414,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>marches/fx/USDCNY.csv</t>
+          <t>marches/fx/USDCAD.csv</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
@@ -50640,7 +51443,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>marches/fx/USDJPY.csv</t>
+          <t>marches/fx/USDCHF.csv</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
@@ -50658,7 +51461,7 @@
         <v>42</v>
       </c>
       <c r="F248" t="n">
-        <v>3905</v>
+        <v>3902</v>
       </c>
       <c r="G248" t="inlineStr">
         <is>
@@ -50669,7 +51472,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>marches/fx/USDKRW.csv</t>
+          <t>marches/fx/USDCNY.csv</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
@@ -50698,7 +51501,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>marches/fx/USDNOK.csv</t>
+          <t>marches/fx/USDJPY.csv</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
@@ -50727,7 +51530,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>marches/fx/USDSEK.csv</t>
+          <t>marches/fx/USDKRW.csv</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
@@ -50745,7 +51548,7 @@
         <v>42</v>
       </c>
       <c r="F251" t="n">
-        <v>3905</v>
+        <v>3904</v>
       </c>
       <c r="G251" t="inlineStr">
         <is>
@@ -50756,7 +51559,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>marches/indices/DAX.csv</t>
+          <t>marches/fx/USDNOK.csv</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -50774,7 +51577,7 @@
         <v>42</v>
       </c>
       <c r="F252" t="n">
-        <v>3802</v>
+        <v>3905</v>
       </c>
       <c r="G252" t="inlineStr">
         <is>
@@ -50785,7 +51588,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>marches/indices/EUROSTOXX50.csv</t>
+          <t>marches/fx/USDSEK.csv</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -50803,7 +51606,7 @@
         <v>42</v>
       </c>
       <c r="F253" t="n">
-        <v>3759</v>
+        <v>3905</v>
       </c>
       <c r="G253" t="inlineStr">
         <is>
@@ -50814,7 +51617,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>marches/indices/FTSE100.csv</t>
+          <t>marches/matieres/BRENT.csv</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
@@ -50832,7 +51635,7 @@
         <v>42</v>
       </c>
       <c r="F254" t="n">
-        <v>3788</v>
+        <v>3751</v>
       </c>
       <c r="G254" t="inlineStr">
         <is>
@@ -50843,7 +51646,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>marches/matieres/BRENT.csv</t>
+          <t>marches/matieres/CUIVRE.csv</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
@@ -50861,7 +51664,7 @@
         <v>42</v>
       </c>
       <c r="F255" t="n">
-        <v>3751</v>
+        <v>3771</v>
       </c>
       <c r="G255" t="inlineStr">
         <is>
@@ -50872,7 +51675,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>marches/matieres/CUIVRE.csv</t>
+          <t>marches/matieres/GAZ_HENRY_HUB.csv</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
@@ -50890,7 +51693,7 @@
         <v>42</v>
       </c>
       <c r="F256" t="n">
-        <v>3771</v>
+        <v>3772</v>
       </c>
       <c r="G256" t="inlineStr">
         <is>
@@ -50901,7 +51704,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>marches/matieres/GAZ_HENRY_HUB.csv</t>
+          <t>marches/matieres/OR.csv</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
@@ -50919,7 +51722,7 @@
         <v>42</v>
       </c>
       <c r="F257" t="n">
-        <v>3772</v>
+        <v>3771</v>
       </c>
       <c r="G257" t="inlineStr">
         <is>
@@ -50930,7 +51733,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>marches/matieres/OR.csv</t>
+          <t>marches/matieres/WTI.csv</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
@@ -50959,7 +51762,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>marches/matieres/WTI.csv</t>
+          <t>marches/taux_futures/FED_FUNDS_FRONT.csv</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
@@ -50977,7 +51780,7 @@
         <v>42</v>
       </c>
       <c r="F259" t="n">
-        <v>3771</v>
+        <v>3772</v>
       </c>
       <c r="G259" t="inlineStr">
         <is>
@@ -50988,7 +51791,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>marches/taux_futures/FED_FUNDS_FRONT.csv</t>
+          <t>marches/volatilite/GVZ.csv</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
@@ -51006,7 +51809,7 @@
         <v>42</v>
       </c>
       <c r="F260" t="n">
-        <v>3772</v>
+        <v>3770</v>
       </c>
       <c r="G260" t="inlineStr">
         <is>
@@ -51017,7 +51820,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>marches/volatilite/GVZ.csv</t>
+          <t>marches/volatilite/MOVE.csv</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
@@ -51035,7 +51838,7 @@
         <v>42</v>
       </c>
       <c r="F261" t="n">
-        <v>3771</v>
+        <v>3689</v>
       </c>
       <c r="G261" t="inlineStr">
         <is>
@@ -51064,7 +51867,7 @@
         <v>42</v>
       </c>
       <c r="F262" t="n">
-        <v>3771</v>
+        <v>3770</v>
       </c>
       <c r="G262" t="inlineStr">
         <is>
@@ -51093,7 +51896,7 @@
         <v>42</v>
       </c>
       <c r="F263" t="n">
-        <v>3763</v>
+        <v>3762</v>
       </c>
       <c r="G263" t="inlineStr">
         <is>
@@ -51122,7 +51925,7 @@
         <v>42</v>
       </c>
       <c r="F264" t="n">
-        <v>3771</v>
+        <v>3770</v>
       </c>
       <c r="G264" t="inlineStr">
         <is>
@@ -52178,7 +52981,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -52399,6 +53202,22 @@
       </c>
       <c r="D13" t="n">
         <v>0.2202</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>5.17</v>
+      </c>
+      <c r="C14" t="n">
+        <v>4.9834</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.1866</v>
       </c>
     </row>
   </sheetData>
@@ -53020,49 +53839,49 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Etats-Unis (S&amp;P 500)</t>
+          <t>Royaume-Uni (FTSE 100)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>7682.41</v>
+        <v>10695.3</v>
       </c>
       <c r="D4" t="n">
-        <v>3.25</v>
+        <v>1.78</v>
       </c>
       <c r="E4" t="n">
-        <v>15.63</v>
+        <v>16.08</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Royaume-Uni (FTSE 100)</t>
+          <t>Zone euro (Euro Stoxx 50)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>10684.88</v>
+        <v>6302.82</v>
       </c>
       <c r="D5" t="n">
-        <v>1.91</v>
+        <v>1.31</v>
       </c>
       <c r="E5" t="n">
-        <v>15.08</v>
+        <v>15.76</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Zone euro (Euro Stoxx 50)</t>
+          <t>Etats-Unis (S&amp;P 500)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -53071,13 +53890,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>6301.28</v>
+        <v>7683.69</v>
       </c>
       <c r="D6" t="n">
-        <v>1.12</v>
+        <v>3.27</v>
       </c>
       <c r="E6" t="n">
-        <v>14.57</v>
+        <v>15.65</v>
       </c>
     </row>
     <row r="7">
@@ -53088,17 +53907,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>25374.42</v>
+        <v>25408.64</v>
       </c>
       <c r="D7" t="n">
-        <v>3.04</v>
+        <v>2.99</v>
       </c>
       <c r="E7" t="n">
-        <v>6.89</v>
+        <v>7.96</v>
       </c>
     </row>
     <row r="8">
@@ -53795,16 +54614,16 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>16.01</v>
+        <v>16.07</v>
       </c>
       <c r="C13" t="n">
-        <v>15.856</v>
+        <v>15.907</v>
       </c>
       <c r="D13" t="n">
         <v>0.625</v>
       </c>
       <c r="E13" t="n">
-        <v>0.20516</v>
+        <v>0.20517</v>
       </c>
     </row>
   </sheetData>
@@ -53818,7 +54637,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -54144,6 +54963,30 @@
         <v>1</v>
       </c>
       <c r="F13" t="inlineStr">
+        <is>
+          <t>{0: 357, 1: 1369, 2: 324}</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>14.87</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="D14" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" t="inlineStr">
         <is>
           <t>{0: 357, 1: 1369, 2: 324}</t>
         </is>
@@ -54892,7 +55735,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>-0.712</v>
+        <v>-0.72</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -54900,7 +55743,7 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0.164</v>
+        <v>0.153</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -55233,25 +56076,25 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.00159</v>
+        <v>0.001592</v>
       </c>
       <c r="C11" t="n">
-        <v>5.33</v>
+        <v>5.45</v>
       </c>
       <c r="D11" t="n">
-        <v>98.01000000000001</v>
+        <v>98.54000000000001</v>
       </c>
       <c r="E11" t="n">
-        <v>33.98</v>
+        <v>34.71</v>
       </c>
       <c r="F11" t="n">
-        <v>39.75</v>
+        <v>40.51</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.97</v>
+        <v>-1.23</v>
       </c>
       <c r="H11" t="n">
-        <v>5.21</v>
+        <v>5.42</v>
       </c>
     </row>
   </sheetData>
@@ -56051,7 +56894,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>9.154</v>
+        <v>9.122</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -56059,10 +56902,10 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>-10.092</v>
+        <v>-10.103</v>
       </c>
       <c r="F14" t="n">
-        <v>19.247</v>
+        <v>19.224</v>
       </c>
     </row>
   </sheetData>
@@ -56076,7 +56919,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -56254,6 +57097,19 @@
         <v>-0.07897999999999999</v>
       </c>
       <c r="C13" t="n">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>-0.07937</v>
+      </c>
+      <c r="C14" t="n">
         <v>57</v>
       </c>
     </row>
@@ -58961,16 +59817,16 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>-0.381</v>
+        <v>-0.364</v>
       </c>
       <c r="C14" t="n">
-        <v>3.252</v>
+        <v>3.269</v>
       </c>
       <c r="D14" t="n">
-        <v>21.103</v>
+        <v>21.123</v>
       </c>
       <c r="E14" t="n">
-        <v>15.635</v>
+        <v>15.654</v>
       </c>
       <c r="F14" t="n">
         <v>16.076</v>
@@ -59725,7 +60581,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>16.01</v>
+        <v>16.07</v>
       </c>
       <c r="C13" t="n">
         <v>20.201</v>
@@ -59737,7 +60593,7 @@
         <v>28.8</v>
       </c>
       <c r="F13" t="n">
-        <v>-4.191</v>
+        <v>-4.131</v>
       </c>
     </row>
   </sheetData>
@@ -59956,26 +60812,26 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>4.87</v>
+        <v>4.81</v>
       </c>
       <c r="D3" t="n">
-        <v>5.18</v>
+        <v>5.17</v>
       </c>
       <c r="E3" t="n">
-        <v>0.31</v>
+        <v>0.36</v>
       </c>
       <c r="F3" t="n">
-        <v>-0</v>
+        <v>0.05</v>
       </c>
       <c r="G3" t="n">
-        <v>0.78</v>
+        <v>0.74</v>
       </c>
       <c r="H3" t="n">
-        <v>0.78</v>
+        <v>0.79</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -65001,7 +65857,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>-0.004902</v>
+        <v>-0.004897</v>
       </c>
     </row>
   </sheetData>
@@ -65868,7 +66724,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -66089,6 +66945,22 @@
       </c>
       <c r="D13" t="n">
         <v>-0.03855</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.008800000000000001</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.06836</v>
+      </c>
+      <c r="D14" t="n">
+        <v>-0.03858</v>
       </c>
     </row>
   </sheetData>
@@ -69522,13 +70394,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1.1216</v>
+        <v>1.123</v>
       </c>
       <c r="C14" t="n">
-        <v>1.1024</v>
+        <v>1.1038</v>
       </c>
       <c r="D14" t="n">
-        <v>1.6031</v>
+        <v>1.6049</v>
       </c>
     </row>
   </sheetData>
@@ -69600,7 +70472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G66"/>
+  <dimension ref="A1:G71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -71737,6 +72609,165 @@
         </is>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>stable</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>moyen</t>
+        </is>
+      </c>
+      <c r="F67" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>stable</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Zone euro</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>hausse</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>haut</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>non_couvert</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Royaume-Uni</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>3.7305</v>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>stable</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>haut</t>
+        </is>
+      </c>
+      <c r="F69" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>stable</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Japon</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>0.977</v>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>stable</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>haut</t>
+        </is>
+      </c>
+      <c r="F70" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>stable</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Chine</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>stable</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>bas</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>non_couvert</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -71748,7 +72779,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -72074,6 +73105,30 @@
         <v>-2.15</v>
       </c>
       <c r="F13" t="inlineStr">
+        <is>
+          <t>2_termes_sans_output_gap</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>3.353</v>
+      </c>
+      <c r="C14" t="n">
+        <v>6.03</v>
+      </c>
+      <c r="D14" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="E14" t="n">
+        <v>-2.15</v>
+      </c>
+      <c r="F14" t="inlineStr">
         <is>
           <t>2_termes_sans_output_gap</t>
         </is>
@@ -75679,7 +76734,7 @@
         </is>
       </c>
       <c r="E122" t="n">
-        <v>16.097</v>
+        <v>15.901</v>
       </c>
     </row>
     <row r="123">
@@ -75702,7 +76757,7 @@
         </is>
       </c>
       <c r="E123" t="n">
-        <v>6.542</v>
+        <v>6.545</v>
       </c>
     </row>
     <row r="124">
@@ -75725,7 +76780,7 @@
         </is>
       </c>
       <c r="E124" t="n">
-        <v>4.824</v>
+        <v>4.919</v>
       </c>
     </row>
     <row r="125">
@@ -75748,7 +76803,7 @@
         </is>
       </c>
       <c r="E125" t="n">
-        <v>0.921</v>
+        <v>0.875</v>
       </c>
     </row>
     <row r="126">
@@ -75771,7 +76826,7 @@
         </is>
       </c>
       <c r="E126" t="n">
-        <v>-2.201</v>
+        <v>-2.349</v>
       </c>
     </row>
     <row r="127">
@@ -75794,7 +76849,7 @@
         </is>
       </c>
       <c r="E127" t="n">
-        <v>-2.424</v>
+        <v>-2.477</v>
       </c>
     </row>
     <row r="128">
@@ -75817,7 +76872,7 @@
         </is>
       </c>
       <c r="E128" t="n">
-        <v>-6.801</v>
+        <v>-6.933</v>
       </c>
     </row>
     <row r="129">
@@ -75840,7 +76895,7 @@
         </is>
       </c>
       <c r="E129" t="n">
-        <v>-7.682</v>
+        <v>-7.649</v>
       </c>
     </row>
     <row r="130">
@@ -75863,7 +76918,7 @@
         </is>
       </c>
       <c r="E130" t="n">
-        <v>-7.981</v>
+        <v>-7.947</v>
       </c>
     </row>
     <row r="131">
@@ -75886,7 +76941,7 @@
         </is>
       </c>
       <c r="E131" t="n">
-        <v>-14.613</v>
+        <v>-14.711</v>
       </c>
     </row>
   </sheetData>
@@ -76729,7 +77784,7 @@
         <v>-1.028</v>
       </c>
       <c r="G14" t="n">
-        <v>0.3038</v>
+        <v>0.3039</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -78558,10 +79613,10 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>-0.1997</v>
+        <v>-0.1998</v>
       </c>
       <c r="C14" t="n">
-        <v>1.0139</v>
+        <v>1.0149</v>
       </c>
     </row>
   </sheetData>
@@ -78631,13 +79686,13 @@
         <v>13.8</v>
       </c>
       <c r="D2" t="n">
-        <v>5.18</v>
+        <v>5.17</v>
       </c>
       <c r="E2" t="n">
         <v>3.4</v>
       </c>
       <c r="F2" t="n">
-        <v>1.78</v>
+        <v>1.77</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-29T00:04Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-28 23:35 UTC</t>
+          <t>Genere le 2026-09-29 00:04 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-28 23:35 UTC</t>
+          <t>Rapport global — 2026-09-29 00:04 UTC</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>**Matieres premieres macro** — le ratio cuivre/or monte -- la croissance domine la peur (+5.5% sur 3 mois). Brent 98.5$ (+34.7% sur 3 mois, +40.5% sur 12 mois), gaz -1.2% sur 3 mois, ecart Brent-WTI +5.4$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-28)_</t>
+          <t>**Matieres premieres macro** — le ratio cuivre/or monte -- la croissance domine la peur (+5.5% sur 3 mois). Brent 98.6$ (+34.8% sur 3 mois, +40.6% sur 12 mois), gaz -1.3% sur 3 mois, ecart Brent-WTI +5.4$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -869,7 +869,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>**Emission tresor us** — 84 derniers jours, 7886 Mds$ offerts : court (moins d'un an) 6798 Mds$ (86%), intermediaire (2 a 10 ans) 969 Mds$ (12%), long (20 a 30 ans) 119 Mds$ (2%) -- financement concentre sur le court et l'intermediaire, part longue a 2% -- peu de pression par la duration _(observation : date non exposee)_</t>
+          <t>**Emission tresor us** — 84 derniers jours, 7715 Mds$ offerts : court (moins d'un an) 6627 Mds$ (86%), intermediaire (2 a 10 ans) 969 Mds$ (13%), long (20 a 30 ans) 119 Mds$ (2%) -- financement concentre sur le court et l'intermediaire, part longue a 2% -- peu de pression par la duration _(observation : date non exposee)_</t>
         </is>
       </c>
     </row>
@@ -1240,7 +1240,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.3730169650835773 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.052364093738951525 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-28)_</t>
+          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.37301696508358795 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.05236409373895107 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -13486,7 +13486,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -40424,13 +40424,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C2" t="n">
-        <v>6798</v>
+        <v>6627</v>
       </c>
       <c r="D2" t="n">
-        <v>86.2</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="E2" t="n">
         <v>2.85</v>
@@ -40449,7 +40449,7 @@
         <v>969</v>
       </c>
       <c r="D3" t="n">
-        <v>12.3</v>
+        <v>12.6</v>
       </c>
       <c r="E3" t="n">
         <v>2.59</v>
@@ -44318,7 +44318,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D2" t="n">
         <v>91.5</v>
@@ -44347,7 +44347,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D3" t="n">
         <v>91.5</v>
@@ -44376,7 +44376,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D4" t="n">
         <v>91.5</v>
@@ -44405,7 +44405,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D5" t="n">
         <v>91.5</v>
@@ -44434,7 +44434,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D6" t="n">
         <v>91.5</v>
@@ -44463,7 +44463,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D7" t="n">
         <v>91.5</v>
@@ -44492,7 +44492,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D8" t="n">
         <v>91.5</v>
@@ -44521,7 +44521,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D9" t="n">
         <v>91.5</v>
@@ -44550,7 +44550,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D10" t="n">
         <v>91.5</v>
@@ -44579,7 +44579,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D11" t="n">
         <v>91.5</v>
@@ -44608,7 +44608,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D12" t="n">
         <v>91.5</v>
@@ -44637,7 +44637,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D13" t="n">
         <v>91.5</v>
@@ -44666,7 +44666,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D14" t="n">
         <v>91.5</v>
@@ -44695,7 +44695,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D15" t="n">
         <v>91.5</v>
@@ -44724,7 +44724,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D16" t="n">
         <v>92</v>
@@ -44753,7 +44753,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D17" t="n">
         <v>91.5</v>
@@ -44782,7 +44782,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D18" t="n">
         <v>91.5</v>
@@ -44811,7 +44811,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D19" t="n">
         <v>91.5</v>
@@ -44840,7 +44840,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D20" t="n">
         <v>91.5</v>
@@ -44869,7 +44869,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D21" t="n">
         <v>91.5</v>
@@ -44898,7 +44898,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D22" t="n">
         <v>91.5</v>
@@ -44927,7 +44927,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D23" t="n">
         <v>91.5</v>
@@ -44956,7 +44956,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D24" t="n">
         <v>91.5</v>
@@ -44985,7 +44985,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D25" t="n">
         <v>91</v>
@@ -45014,7 +45014,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D26" t="n">
         <v>31</v>
@@ -45043,7 +45043,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D27" t="n">
         <v>31</v>
@@ -45072,7 +45072,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D28" t="n">
         <v>31</v>
@@ -45101,7 +45101,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D29" t="n">
         <v>31</v>
@@ -45130,7 +45130,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D30" t="n">
         <v>31</v>
@@ -45159,7 +45159,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D31" t="n">
         <v>31</v>
@@ -45188,7 +45188,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D32" t="n">
         <v>31</v>
@@ -45217,7 +45217,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D33" t="n">
         <v>31</v>
@@ -45246,7 +45246,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D34" t="n">
         <v>31</v>
@@ -45275,7 +45275,7 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D35" t="n">
         <v>31</v>
@@ -45304,7 +45304,7 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D36" t="n">
         <v>31</v>
@@ -45333,7 +45333,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D37" t="n">
         <v>31</v>
@@ -45362,7 +45362,7 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D38" t="n">
         <v>31</v>
@@ -45391,7 +45391,7 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D39" t="n">
         <v>31</v>
@@ -45420,7 +45420,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D40" t="n">
         <v>31</v>
@@ -45449,7 +45449,7 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D41" t="n">
         <v>31</v>
@@ -45478,7 +45478,7 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D42" t="n">
         <v>31</v>
@@ -45507,7 +45507,7 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D43" t="n">
         <v>31</v>
@@ -45536,7 +45536,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D44" t="n">
         <v>31</v>
@@ -45565,7 +45565,7 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D45" t="n">
         <v>31</v>
@@ -45594,7 +45594,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D46" t="n">
         <v>31</v>
@@ -45623,7 +45623,7 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D47" t="n">
         <v>31</v>
@@ -45652,7 +45652,7 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D48" t="n">
         <v>31</v>
@@ -45681,7 +45681,7 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D49" t="n">
         <v>31</v>
@@ -45710,7 +45710,7 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D50" t="n">
         <v>31</v>
@@ -45739,7 +45739,7 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D51" t="n">
         <v>31</v>
@@ -45768,7 +45768,7 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D52" t="n">
         <v>31</v>
@@ -45797,7 +45797,7 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D53" t="n">
         <v>31</v>
@@ -45826,7 +45826,7 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D54" t="n">
         <v>31</v>
@@ -45855,7 +45855,7 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D55" t="n">
         <v>31</v>
@@ -45884,7 +45884,7 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D56" t="n">
         <v>31</v>
@@ -45913,7 +45913,7 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D57" t="n">
         <v>31</v>
@@ -45942,7 +45942,7 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D58" t="n">
         <v>31</v>
@@ -45971,7 +45971,7 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D59" t="n">
         <v>31</v>
@@ -46000,7 +46000,7 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D60" t="n">
         <v>31</v>
@@ -46029,7 +46029,7 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D61" t="n">
         <v>31</v>
@@ -46058,7 +46058,7 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D62" t="n">
         <v>31</v>
@@ -46087,7 +46087,7 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D63" t="n">
         <v>31</v>
@@ -46116,7 +46116,7 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D64" t="n">
         <v>31</v>
@@ -46145,7 +46145,7 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D65" t="n">
         <v>31</v>
@@ -46174,7 +46174,7 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D66" t="n">
         <v>31</v>
@@ -46203,7 +46203,7 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D67" t="n">
         <v>31</v>
@@ -46232,7 +46232,7 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D68" t="n">
         <v>31</v>
@@ -46261,7 +46261,7 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D69" t="n">
         <v>31</v>
@@ -46290,7 +46290,7 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D70" t="n">
         <v>31</v>
@@ -46319,7 +46319,7 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D71" t="n">
         <v>31</v>
@@ -46348,7 +46348,7 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D72" t="n">
         <v>31</v>
@@ -46377,7 +46377,7 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D73" t="n">
         <v>31</v>
@@ -46406,7 +46406,7 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D74" t="n">
         <v>31</v>
@@ -46435,7 +46435,7 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D75" t="n">
         <v>31</v>
@@ -46464,7 +46464,7 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D76" t="n">
         <v>31</v>
@@ -46493,7 +46493,7 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D77" t="n">
         <v>31</v>
@@ -46522,7 +46522,7 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D78" t="n">
         <v>31</v>
@@ -46551,7 +46551,7 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D79" t="n">
         <v>31</v>
@@ -46580,7 +46580,7 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D80" t="n">
         <v>31</v>
@@ -46609,7 +46609,7 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D81" t="n">
         <v>31</v>
@@ -46638,7 +46638,7 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D82" t="n">
         <v>31</v>
@@ -46667,7 +46667,7 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D83" t="n">
         <v>31</v>
@@ -46696,7 +46696,7 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D84" t="n">
         <v>31</v>
@@ -46725,7 +46725,7 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D85" t="n">
         <v>31</v>
@@ -46754,7 +46754,7 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D86" t="n">
         <v>31</v>
@@ -46783,7 +46783,7 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D87" t="n">
         <v>31</v>
@@ -46812,7 +46812,7 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D88" t="n">
         <v>31</v>
@@ -46841,7 +46841,7 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D89" t="n">
         <v>31</v>
@@ -46870,7 +46870,7 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D90" t="n">
         <v>31</v>
@@ -46899,7 +46899,7 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D91" t="n">
         <v>31</v>
@@ -46928,7 +46928,7 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D92" t="n">
         <v>31</v>
@@ -46957,7 +46957,7 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D93" t="n">
         <v>31</v>
@@ -46986,7 +46986,7 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D94" t="n">
         <v>31</v>
@@ -47015,7 +47015,7 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D95" t="n">
         <v>1</v>
@@ -47044,7 +47044,7 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D96" t="n">
         <v>1</v>
@@ -47073,7 +47073,7 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D97" t="n">
         <v>1</v>
@@ -47102,7 +47102,7 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D98" t="n">
         <v>1</v>
@@ -47131,7 +47131,7 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D99" t="n">
         <v>1</v>
@@ -47160,7 +47160,7 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D100" t="n">
         <v>31</v>
@@ -47189,7 +47189,7 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D101" t="n">
         <v>31</v>
@@ -47218,7 +47218,7 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D102" t="n">
         <v>7</v>
@@ -47247,7 +47247,7 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D103" t="n">
         <v>1</v>
@@ -47276,7 +47276,7 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D104" t="n">
         <v>7</v>
@@ -47305,7 +47305,7 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D105" t="n">
         <v>1</v>
@@ -47334,7 +47334,7 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D106" t="n">
         <v>1</v>
@@ -47363,7 +47363,7 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D107" t="n">
         <v>7</v>
@@ -47392,7 +47392,7 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D108" t="n">
         <v>1</v>
@@ -47421,7 +47421,7 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D109" t="n">
         <v>1</v>
@@ -47450,7 +47450,7 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D110" t="n">
         <v>1</v>
@@ -47479,7 +47479,7 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D111" t="n">
         <v>1</v>
@@ -47508,7 +47508,7 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D112" t="n">
         <v>1</v>
@@ -47537,7 +47537,7 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D113" t="n">
         <v>1</v>
@@ -47566,7 +47566,7 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D114" t="n">
         <v>1</v>
@@ -47595,7 +47595,7 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D115" t="n">
         <v>1</v>
@@ -47624,7 +47624,7 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D116" t="n">
         <v>7</v>
@@ -47653,7 +47653,7 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D117" t="n">
         <v>7</v>
@@ -47682,7 +47682,7 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D118" t="n">
         <v>7</v>
@@ -47711,7 +47711,7 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D119" t="n">
         <v>7</v>
@@ -47740,7 +47740,7 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D120" t="n">
         <v>7</v>
@@ -47769,7 +47769,7 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D121" t="n">
         <v>7</v>
@@ -47798,7 +47798,7 @@
         </is>
       </c>
       <c r="C122" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D122" t="n">
         <v>7</v>
@@ -47827,7 +47827,7 @@
         </is>
       </c>
       <c r="C123" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D123" t="n">
         <v>7</v>
@@ -47856,7 +47856,7 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D124" t="n">
         <v>7</v>
@@ -47885,7 +47885,7 @@
         </is>
       </c>
       <c r="C125" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D125" t="n">
         <v>7</v>
@@ -47914,7 +47914,7 @@
         </is>
       </c>
       <c r="C126" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D126" t="n">
         <v>7</v>
@@ -47943,7 +47943,7 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D127" t="n">
         <v>7</v>
@@ -47972,7 +47972,7 @@
         </is>
       </c>
       <c r="C128" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D128" t="n">
         <v>7</v>
@@ -48001,7 +48001,7 @@
         </is>
       </c>
       <c r="C129" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D129" t="n">
         <v>7</v>
@@ -48030,7 +48030,7 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D130" t="n">
         <v>7</v>
@@ -48059,7 +48059,7 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D131" t="n">
         <v>7</v>
@@ -48088,7 +48088,7 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D132" t="n">
         <v>7</v>
@@ -48117,7 +48117,7 @@
         </is>
       </c>
       <c r="C133" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D133" t="n">
         <v>7</v>
@@ -48146,7 +48146,7 @@
         </is>
       </c>
       <c r="C134" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D134" t="n">
         <v>7</v>
@@ -48175,7 +48175,7 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D135" t="n">
         <v>7</v>
@@ -48204,7 +48204,7 @@
         </is>
       </c>
       <c r="C136" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D136" t="n">
         <v>7</v>
@@ -48233,7 +48233,7 @@
         </is>
       </c>
       <c r="C137" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D137" t="n">
         <v>7</v>
@@ -48262,7 +48262,7 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D138" t="n">
         <v>7</v>
@@ -48291,7 +48291,7 @@
         </is>
       </c>
       <c r="C139" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D139" t="n">
         <v>7</v>
@@ -48320,7 +48320,7 @@
         </is>
       </c>
       <c r="C140" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D140" t="n">
         <v>7</v>
@@ -48349,7 +48349,7 @@
         </is>
       </c>
       <c r="C141" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D141" t="n">
         <v>7</v>
@@ -48378,7 +48378,7 @@
         </is>
       </c>
       <c r="C142" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D142" t="n">
         <v>7</v>
@@ -48407,7 +48407,7 @@
         </is>
       </c>
       <c r="C143" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D143" t="n">
         <v>7</v>
@@ -48436,7 +48436,7 @@
         </is>
       </c>
       <c r="C144" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D144" t="n">
         <v>7</v>
@@ -48465,7 +48465,7 @@
         </is>
       </c>
       <c r="C145" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D145" t="n">
         <v>7</v>
@@ -48494,7 +48494,7 @@
         </is>
       </c>
       <c r="C146" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D146" t="n">
         <v>7</v>
@@ -48523,7 +48523,7 @@
         </is>
       </c>
       <c r="C147" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D147" t="n">
         <v>7</v>
@@ -48552,7 +48552,7 @@
         </is>
       </c>
       <c r="C148" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D148" t="n">
         <v>7</v>
@@ -48581,7 +48581,7 @@
         </is>
       </c>
       <c r="C149" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D149" t="n">
         <v>7</v>
@@ -48610,7 +48610,7 @@
         </is>
       </c>
       <c r="C150" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D150" t="n">
         <v>7</v>
@@ -48639,7 +48639,7 @@
         </is>
       </c>
       <c r="C151" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D151" t="n">
         <v>7</v>
@@ -48668,7 +48668,7 @@
         </is>
       </c>
       <c r="C152" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D152" t="n">
         <v>7</v>
@@ -48697,7 +48697,7 @@
         </is>
       </c>
       <c r="C153" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D153" t="n">
         <v>7</v>
@@ -48726,7 +48726,7 @@
         </is>
       </c>
       <c r="C154" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D154" t="n">
         <v>7</v>
@@ -48755,7 +48755,7 @@
         </is>
       </c>
       <c r="C155" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D155" t="n">
         <v>7</v>
@@ -48784,7 +48784,7 @@
         </is>
       </c>
       <c r="C156" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D156" t="n">
         <v>7</v>
@@ -48813,7 +48813,7 @@
         </is>
       </c>
       <c r="C157" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D157" t="n">
         <v>7</v>
@@ -48842,7 +48842,7 @@
         </is>
       </c>
       <c r="C158" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D158" t="n">
         <v>7</v>
@@ -48871,7 +48871,7 @@
         </is>
       </c>
       <c r="C159" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D159" t="n">
         <v>7</v>
@@ -48900,7 +48900,7 @@
         </is>
       </c>
       <c r="C160" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D160" t="n">
         <v>7</v>
@@ -48929,7 +48929,7 @@
         </is>
       </c>
       <c r="C161" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D161" t="n">
         <v>7</v>
@@ -48958,7 +48958,7 @@
         </is>
       </c>
       <c r="C162" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D162" t="n">
         <v>7</v>
@@ -48987,7 +48987,7 @@
         </is>
       </c>
       <c r="C163" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D163" t="n">
         <v>7</v>
@@ -49016,7 +49016,7 @@
         </is>
       </c>
       <c r="C164" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D164" t="n">
         <v>7</v>
@@ -49045,7 +49045,7 @@
         </is>
       </c>
       <c r="C165" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D165" t="n">
         <v>7</v>
@@ -49074,7 +49074,7 @@
         </is>
       </c>
       <c r="C166" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D166" t="n">
         <v>7</v>
@@ -49103,7 +49103,7 @@
         </is>
       </c>
       <c r="C167" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D167" t="n">
         <v>7</v>
@@ -49132,7 +49132,7 @@
         </is>
       </c>
       <c r="C168" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D168" t="n">
         <v>7</v>
@@ -49161,7 +49161,7 @@
         </is>
       </c>
       <c r="C169" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D169" t="n">
         <v>7</v>
@@ -49190,7 +49190,7 @@
         </is>
       </c>
       <c r="C170" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D170" t="n">
         <v>7</v>
@@ -49219,7 +49219,7 @@
         </is>
       </c>
       <c r="C171" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D171" t="n">
         <v>7</v>
@@ -49248,7 +49248,7 @@
         </is>
       </c>
       <c r="C172" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D172" t="n">
         <v>7</v>
@@ -49277,7 +49277,7 @@
         </is>
       </c>
       <c r="C173" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D173" t="n">
         <v>7</v>
@@ -49306,7 +49306,7 @@
         </is>
       </c>
       <c r="C174" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D174" t="n">
         <v>7</v>
@@ -49335,7 +49335,7 @@
         </is>
       </c>
       <c r="C175" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D175" t="n">
         <v>7</v>
@@ -49364,7 +49364,7 @@
         </is>
       </c>
       <c r="C176" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D176" t="n">
         <v>7</v>
@@ -49393,7 +49393,7 @@
         </is>
       </c>
       <c r="C177" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D177" t="n">
         <v>7</v>
@@ -49422,7 +49422,7 @@
         </is>
       </c>
       <c r="C178" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D178" t="n">
         <v>7</v>
@@ -49451,7 +49451,7 @@
         </is>
       </c>
       <c r="C179" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D179" t="n">
         <v>7</v>
@@ -49480,7 +49480,7 @@
         </is>
       </c>
       <c r="C180" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D180" t="n">
         <v>7</v>
@@ -49509,7 +49509,7 @@
         </is>
       </c>
       <c r="C181" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D181" t="n">
         <v>7</v>
@@ -49538,7 +49538,7 @@
         </is>
       </c>
       <c r="C182" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D182" t="n">
         <v>7</v>
@@ -49567,7 +49567,7 @@
         </is>
       </c>
       <c r="C183" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D183" t="n">
         <v>1</v>
@@ -49596,7 +49596,7 @@
         </is>
       </c>
       <c r="C184" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D184" t="n">
         <v>1</v>
@@ -49625,7 +49625,7 @@
         </is>
       </c>
       <c r="C185" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D185" t="n">
         <v>1</v>
@@ -49654,7 +49654,7 @@
         </is>
       </c>
       <c r="C186" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D186" t="n">
         <v>1</v>
@@ -49683,7 +49683,7 @@
         </is>
       </c>
       <c r="C187" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D187" t="n">
         <v>1</v>
@@ -49712,7 +49712,7 @@
         </is>
       </c>
       <c r="C188" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D188" t="n">
         <v>7</v>
@@ -49741,7 +49741,7 @@
         </is>
       </c>
       <c r="C189" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D189" t="n">
         <v>1</v>
@@ -49770,7 +49770,7 @@
         </is>
       </c>
       <c r="C190" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D190" t="n">
         <v>1</v>
@@ -49799,7 +49799,7 @@
         </is>
       </c>
       <c r="C191" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D191" t="n">
         <v>1</v>
@@ -49828,7 +49828,7 @@
         </is>
       </c>
       <c r="C192" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D192" t="n">
         <v>1</v>
@@ -49857,7 +49857,7 @@
         </is>
       </c>
       <c r="C193" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D193" t="n">
         <v>1</v>
@@ -49886,7 +49886,7 @@
         </is>
       </c>
       <c r="C194" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D194" t="n">
         <v>1</v>
@@ -49915,7 +49915,7 @@
         </is>
       </c>
       <c r="C195" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D195" t="n">
         <v>1</v>
@@ -49944,7 +49944,7 @@
         </is>
       </c>
       <c r="C196" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D196" t="n">
         <v>1</v>
@@ -49973,7 +49973,7 @@
         </is>
       </c>
       <c r="C197" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D197" t="n">
         <v>1</v>
@@ -50002,7 +50002,7 @@
         </is>
       </c>
       <c r="C198" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D198" t="n">
         <v>1</v>
@@ -50031,7 +50031,7 @@
         </is>
       </c>
       <c r="C199" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D199" t="n">
         <v>1</v>
@@ -50060,7 +50060,7 @@
         </is>
       </c>
       <c r="C200" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D200" t="n">
         <v>1</v>
@@ -50089,7 +50089,7 @@
         </is>
       </c>
       <c r="C201" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D201" t="n">
         <v>1</v>
@@ -50118,7 +50118,7 @@
         </is>
       </c>
       <c r="C202" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D202" t="n">
         <v>1</v>
@@ -50147,7 +50147,7 @@
         </is>
       </c>
       <c r="C203" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D203" t="n">
         <v>1</v>
@@ -50176,7 +50176,7 @@
         </is>
       </c>
       <c r="C204" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D204" t="n">
         <v>1</v>
@@ -50205,7 +50205,7 @@
         </is>
       </c>
       <c r="C205" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D205" t="n">
         <v>1</v>
@@ -50234,7 +50234,7 @@
         </is>
       </c>
       <c r="C206" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D206" t="n">
         <v>1</v>
@@ -50263,7 +50263,7 @@
         </is>
       </c>
       <c r="C207" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D207" t="n">
         <v>1</v>
@@ -50292,7 +50292,7 @@
         </is>
       </c>
       <c r="C208" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D208" t="n">
         <v>1</v>
@@ -50321,7 +50321,7 @@
         </is>
       </c>
       <c r="C209" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D209" t="n">
         <v>1</v>
@@ -50350,7 +50350,7 @@
         </is>
       </c>
       <c r="C210" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D210" t="n">
         <v>1</v>
@@ -50379,7 +50379,7 @@
         </is>
       </c>
       <c r="C211" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D211" t="n">
         <v>1</v>
@@ -50408,7 +50408,7 @@
         </is>
       </c>
       <c r="C212" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D212" t="n">
         <v>1</v>
@@ -50437,7 +50437,7 @@
         </is>
       </c>
       <c r="C213" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D213" t="n">
         <v>1</v>
@@ -50466,7 +50466,7 @@
         </is>
       </c>
       <c r="C214" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D214" t="n">
         <v>1</v>
@@ -50495,7 +50495,7 @@
         </is>
       </c>
       <c r="C215" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D215" t="n">
         <v>1</v>
@@ -50524,7 +50524,7 @@
         </is>
       </c>
       <c r="C216" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D216" t="n">
         <v>1</v>
@@ -50553,7 +50553,7 @@
         </is>
       </c>
       <c r="C217" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D217" t="n">
         <v>1</v>
@@ -50582,7 +50582,7 @@
         </is>
       </c>
       <c r="C218" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D218" t="n">
         <v>1</v>
@@ -50611,7 +50611,7 @@
         </is>
       </c>
       <c r="C219" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D219" t="n">
         <v>1</v>
@@ -50640,7 +50640,7 @@
         </is>
       </c>
       <c r="C220" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D220" t="n">
         <v>1</v>
@@ -50669,7 +50669,7 @@
         </is>
       </c>
       <c r="C221" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D221" t="n">
         <v>1</v>
@@ -50698,7 +50698,7 @@
         </is>
       </c>
       <c r="C222" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D222" t="n">
         <v>1</v>
@@ -50727,7 +50727,7 @@
         </is>
       </c>
       <c r="C223" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D223" t="n">
         <v>1</v>
@@ -50756,7 +50756,7 @@
         </is>
       </c>
       <c r="C224" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D224" t="n">
         <v>1</v>
@@ -50785,7 +50785,7 @@
         </is>
       </c>
       <c r="C225" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D225" t="n">
         <v>1</v>
@@ -50814,7 +50814,7 @@
         </is>
       </c>
       <c r="C226" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D226" t="n">
         <v>1</v>
@@ -50843,7 +50843,7 @@
         </is>
       </c>
       <c r="C227" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D227" t="n">
         <v>1</v>
@@ -50872,7 +50872,7 @@
         </is>
       </c>
       <c r="C228" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D228" t="n">
         <v>1</v>
@@ -50901,7 +50901,7 @@
         </is>
       </c>
       <c r="C229" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D229" t="n">
         <v>1</v>
@@ -50930,7 +50930,7 @@
         </is>
       </c>
       <c r="C230" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D230" t="n">
         <v>1</v>
@@ -50959,7 +50959,7 @@
         </is>
       </c>
       <c r="C231" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D231" t="n">
         <v>1</v>
@@ -50988,7 +50988,7 @@
         </is>
       </c>
       <c r="C232" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D232" t="n">
         <v>1</v>
@@ -51017,7 +51017,7 @@
         </is>
       </c>
       <c r="C233" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D233" t="n">
         <v>1</v>
@@ -51046,7 +51046,7 @@
         </is>
       </c>
       <c r="C234" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D234" t="n">
         <v>1</v>
@@ -51075,7 +51075,7 @@
         </is>
       </c>
       <c r="C235" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D235" t="n">
         <v>1</v>
@@ -51104,7 +51104,7 @@
         </is>
       </c>
       <c r="C236" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D236" t="n">
         <v>1</v>
@@ -51133,7 +51133,7 @@
         </is>
       </c>
       <c r="C237" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D237" t="n">
         <v>1</v>
@@ -51162,7 +51162,7 @@
         </is>
       </c>
       <c r="C238" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D238" t="n">
         <v>1</v>
@@ -51191,7 +51191,7 @@
         </is>
       </c>
       <c r="C239" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D239" t="n">
         <v>1</v>
@@ -51220,7 +51220,7 @@
         </is>
       </c>
       <c r="C240" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D240" t="n">
         <v>1</v>
@@ -51249,7 +51249,7 @@
         </is>
       </c>
       <c r="C241" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D241" t="n">
         <v>1</v>
@@ -51278,7 +51278,7 @@
         </is>
       </c>
       <c r="C242" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D242" t="n">
         <v>1</v>
@@ -51307,7 +51307,7 @@
         </is>
       </c>
       <c r="C243" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D243" t="n">
         <v>1</v>
@@ -51336,7 +51336,7 @@
         </is>
       </c>
       <c r="C244" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D244" t="n">
         <v>1</v>
@@ -51365,7 +51365,7 @@
         </is>
       </c>
       <c r="C245" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D245" t="n">
         <v>1</v>
@@ -51394,7 +51394,7 @@
         </is>
       </c>
       <c r="C246" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D246" t="n">
         <v>1</v>
@@ -51423,7 +51423,7 @@
         </is>
       </c>
       <c r="C247" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D247" t="n">
         <v>1</v>
@@ -51452,7 +51452,7 @@
         </is>
       </c>
       <c r="C248" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D248" t="n">
         <v>1</v>
@@ -51481,7 +51481,7 @@
         </is>
       </c>
       <c r="C249" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D249" t="n">
         <v>1</v>
@@ -51510,7 +51510,7 @@
         </is>
       </c>
       <c r="C250" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D250" t="n">
         <v>1</v>
@@ -51539,7 +51539,7 @@
         </is>
       </c>
       <c r="C251" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D251" t="n">
         <v>1</v>
@@ -51568,7 +51568,7 @@
         </is>
       </c>
       <c r="C252" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D252" t="n">
         <v>1</v>
@@ -51597,7 +51597,7 @@
         </is>
       </c>
       <c r="C253" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D253" t="n">
         <v>1</v>
@@ -51626,7 +51626,7 @@
         </is>
       </c>
       <c r="C254" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D254" t="n">
         <v>1</v>
@@ -51655,7 +51655,7 @@
         </is>
       </c>
       <c r="C255" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D255" t="n">
         <v>1</v>
@@ -51684,7 +51684,7 @@
         </is>
       </c>
       <c r="C256" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D256" t="n">
         <v>1</v>
@@ -51713,7 +51713,7 @@
         </is>
       </c>
       <c r="C257" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D257" t="n">
         <v>1</v>
@@ -51742,7 +51742,7 @@
         </is>
       </c>
       <c r="C258" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D258" t="n">
         <v>1</v>
@@ -51771,7 +51771,7 @@
         </is>
       </c>
       <c r="C259" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D259" t="n">
         <v>1</v>
@@ -51800,7 +51800,7 @@
         </is>
       </c>
       <c r="C260" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D260" t="n">
         <v>1</v>
@@ -51829,7 +51829,7 @@
         </is>
       </c>
       <c r="C261" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D261" t="n">
         <v>1</v>
@@ -51858,7 +51858,7 @@
         </is>
       </c>
       <c r="C262" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D262" t="n">
         <v>1</v>
@@ -51887,7 +51887,7 @@
         </is>
       </c>
       <c r="C263" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D263" t="n">
         <v>1</v>
@@ -51916,7 +51916,7 @@
         </is>
       </c>
       <c r="C264" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D264" t="n">
         <v>1</v>
@@ -51945,7 +51945,7 @@
         </is>
       </c>
       <c r="C265" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D265" t="n">
         <v>1</v>
@@ -51974,7 +51974,7 @@
         </is>
       </c>
       <c r="C266" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D266" t="n">
         <v>1</v>
@@ -52003,7 +52003,7 @@
         </is>
       </c>
       <c r="C267" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D267" t="n">
         <v>1</v>
@@ -52032,7 +52032,7 @@
         </is>
       </c>
       <c r="C268" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D268" t="n">
         <v>1</v>
@@ -52061,7 +52061,7 @@
         </is>
       </c>
       <c r="C269" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D269" t="n">
         <v>1</v>
@@ -52090,7 +52090,7 @@
         </is>
       </c>
       <c r="C270" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D270" t="n">
         <v>1</v>
@@ -52119,7 +52119,7 @@
         </is>
       </c>
       <c r="C271" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D271" t="n">
         <v>1</v>
@@ -52148,7 +52148,7 @@
         </is>
       </c>
       <c r="C272" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D272" t="n">
         <v>1</v>
@@ -52177,7 +52177,7 @@
         </is>
       </c>
       <c r="C273" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D273" t="n">
         <v>1</v>
@@ -52206,7 +52206,7 @@
         </is>
       </c>
       <c r="C274" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D274" t="n">
         <v>1</v>
@@ -52235,7 +52235,7 @@
         </is>
       </c>
       <c r="C275" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D275" t="n">
         <v>1</v>
@@ -52264,7 +52264,7 @@
         </is>
       </c>
       <c r="C276" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D276" t="n">
         <v>1</v>
@@ -52293,7 +52293,7 @@
         </is>
       </c>
       <c r="C277" t="n">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="D277" t="n">
         <v>2</v>
@@ -52322,7 +52322,7 @@
         </is>
       </c>
       <c r="C278" t="n">
-        <v>-435</v>
+        <v>-434</v>
       </c>
       <c r="D278" t="n">
         <v>42</v>
@@ -56076,25 +56076,25 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.001592</v>
+        <v>0.001593</v>
       </c>
       <c r="C11" t="n">
-        <v>5.45</v>
+        <v>5.53</v>
       </c>
       <c r="D11" t="n">
-        <v>98.54000000000001</v>
+        <v>98.61</v>
       </c>
       <c r="E11" t="n">
-        <v>34.71</v>
+        <v>34.81</v>
       </c>
       <c r="F11" t="n">
-        <v>40.51</v>
+        <v>40.61</v>
       </c>
       <c r="G11" t="n">
-        <v>-1.23</v>
+        <v>-1.29</v>
       </c>
       <c r="H11" t="n">
-        <v>5.42</v>
+        <v>5.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-29T02:45Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-29 00:04 UTC</t>
+          <t>Genere le 2026-09-29 02:45 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-29 00:04 UTC</t>
+          <t>Rapport global — 2026-09-29 02:45 UTC</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>**Matieres premieres macro** — le ratio cuivre/or monte -- la croissance domine la peur (+5.5% sur 3 mois). Brent 98.6$ (+34.8% sur 3 mois, +40.6% sur 12 mois), gaz -1.3% sur 3 mois, ecart Brent-WTI +5.4$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-28)_</t>
+          <t>**Matieres premieres macro** — ratio cuivre/or stable -- pas de signal net sur la croissance (+3.7% sur 3 mois). Brent 99.1$ (+35.9% sur 3 mois, +45.8% sur 12 mois), gaz -4.2% sur 3 mois, ecart Brent-WTI +5.6$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -960,7 +960,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>**Indices mondiaux** — 7 indices (devise locale) : Coree (KOSPI) +103.1% en tete sur 12 mois, Hong Kong (Hang Seng) -7.5% en queue -- ecart tres large entre blocs sur 12 mois (111pt) -- les cycles economiques ou les flux divergent nettement. ROTATION en cours : Coree (KOSPI) mene sur 12 mois mais Hong Kong (Hang Seng) a repris la tete sur 3 mois _(observation : 2026-09-28)_</t>
+          <t>**Indices mondiaux** — 7 indices (devise locale) : Coree (KOSPI) +100.4% en tete sur 12 mois, Hong Kong (Hang Seng) -8.0% en queue -- ecart tres large entre blocs sur 12 mois (108pt) -- les cycles economiques ou les flux divergent nettement. ROTATION en cours : Coree (KOSPI) mene sur 12 mois mais Hong Kong (Hang Seng) a repris la tete sur 3 mois _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -49558,7 +49558,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>marches/indices/KOSPI.csv</t>
+          <t>souverains/AUSTRALIE_10A.csv</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -49576,7 +49576,7 @@
         <v>42</v>
       </c>
       <c r="F183" t="n">
-        <v>3680</v>
+        <v>3361</v>
       </c>
       <c r="G183" t="inlineStr">
         <is>
@@ -49587,7 +49587,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>souverains/AUSTRALIE_10A.csv</t>
+          <t>souverains/AUSTRALIE_2A.csv</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -49605,7 +49605,7 @@
         <v>42</v>
       </c>
       <c r="F184" t="n">
-        <v>3361</v>
+        <v>3283</v>
       </c>
       <c r="G184" t="inlineStr">
         <is>
@@ -49616,7 +49616,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>souverains/AUSTRALIE_2A.csv</t>
+          <t>souverains/AUSTRALIE_5A.csv</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -49645,16 +49645,16 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>souverains/AUSTRALIE_5A.csv</t>
+          <t>fred/IUDSOIA.csv</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C186" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D186" t="n">
         <v>1</v>
@@ -49663,7 +49663,7 @@
         <v>42</v>
       </c>
       <c r="F186" t="n">
-        <v>3283</v>
+        <v>3000</v>
       </c>
       <c r="G186" t="inlineStr">
         <is>
@@ -49674,7 +49674,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>fred/IUDSOIA.csv</t>
+          <t>fred/MORTGAGE30US.csv</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -49686,13 +49686,13 @@
         <v>5</v>
       </c>
       <c r="D187" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E187" t="n">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="F187" t="n">
-        <v>3000</v>
+        <v>2896</v>
       </c>
       <c r="G187" t="inlineStr">
         <is>
@@ -49703,7 +49703,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>fred/MORTGAGE30US.csv</t>
+          <t>souverains/UK_10A.csv</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -49715,13 +49715,13 @@
         <v>5</v>
       </c>
       <c r="D188" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E188" t="n">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="F188" t="n">
-        <v>2896</v>
+        <v>9283</v>
       </c>
       <c r="G188" t="inlineStr">
         <is>
@@ -49732,7 +49732,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>souverains/UK_10A.csv</t>
+          <t>souverains/UK_20A.csv</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -49750,7 +49750,7 @@
         <v>42</v>
       </c>
       <c r="F189" t="n">
-        <v>9283</v>
+        <v>6754</v>
       </c>
       <c r="G189" t="inlineStr">
         <is>
@@ -49761,7 +49761,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>souverains/UK_20A.csv</t>
+          <t>souverains/UK_5A.csv</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -49779,7 +49779,7 @@
         <v>42</v>
       </c>
       <c r="F190" t="n">
-        <v>6754</v>
+        <v>8291</v>
       </c>
       <c r="G190" t="inlineStr">
         <is>
@@ -49790,16 +49790,16 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>souverains/UK_5A.csv</t>
+          <t>fred/BAMLC0A0CM.csv</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C191" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D191" t="n">
         <v>1</v>
@@ -49808,7 +49808,7 @@
         <v>42</v>
       </c>
       <c r="F191" t="n">
-        <v>8291</v>
+        <v>793</v>
       </c>
       <c r="G191" t="inlineStr">
         <is>
@@ -49819,7 +49819,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>fred/BAMLC0A0CM.csv</t>
+          <t>fred/BAMLC0A0CMEY.csv</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -49848,7 +49848,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>fred/BAMLC0A0CMEY.csv</t>
+          <t>fred/BAMLEMCBPIOAS.csv</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -49877,7 +49877,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>fred/BAMLEMCBPIOAS.csv</t>
+          <t>fred/BAMLEMFSFCRPIOAS.csv</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -49906,7 +49906,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>fred/BAMLEMFSFCRPIOAS.csv</t>
+          <t>fred/BAMLEMHBHYCRPIOAS.csv</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -49935,7 +49935,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>fred/BAMLEMHBHYCRPIOAS.csv</t>
+          <t>fred/BAMLEMPBPUBSICRPIOAS.csv</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -49964,7 +49964,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>fred/BAMLEMPBPUBSICRPIOAS.csv</t>
+          <t>fred/BAMLH0A0HYM2.csv</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -49993,7 +49993,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>fred/BAMLH0A0HYM2.csv</t>
+          <t>fred/BAMLHE00EHYIEY.csv</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -50022,7 +50022,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>fred/BAMLHE00EHYIEY.csv</t>
+          <t>fred/BAMLHE00EHYIOAS.csv</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -50051,7 +50051,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>fred/BAMLHE00EHYIOAS.csv</t>
+          <t>fred/DFF.csv</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -50069,7 +50069,7 @@
         <v>42</v>
       </c>
       <c r="F200" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G200" t="inlineStr">
         <is>
@@ -50080,7 +50080,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>fred/DFF.csv</t>
+          <t>fred/DFII10.csv</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -50109,7 +50109,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>fred/DFII10.csv</t>
+          <t>fred/DFII5.csv</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -50138,7 +50138,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>fred/DFII5.csv</t>
+          <t>fred/DGS1.csv</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -50167,7 +50167,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>fred/DGS1.csv</t>
+          <t>fred/DGS10.csv</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
@@ -50196,7 +50196,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>fred/DGS10.csv</t>
+          <t>fred/DGS1MO.csv</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -50225,7 +50225,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>fred/DGS1MO.csv</t>
+          <t>fred/DGS2.csv</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -50254,7 +50254,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>fred/DGS2.csv</t>
+          <t>fred/DGS30.csv</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -50283,7 +50283,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>fred/DGS30.csv</t>
+          <t>fred/DGS3MO.csv</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -50312,7 +50312,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>fred/DGS3MO.csv</t>
+          <t>fred/DGS5.csv</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -50341,7 +50341,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>fred/DGS5.csv</t>
+          <t>fred/DGS6MO.csv</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -50370,7 +50370,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>fred/DGS6MO.csv</t>
+          <t>souverains/CANADA_10A.csv</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
@@ -50388,7 +50388,7 @@
         <v>42</v>
       </c>
       <c r="F211" t="n">
-        <v>3000</v>
+        <v>6436</v>
       </c>
       <c r="G211" t="inlineStr">
         <is>
@@ -50399,7 +50399,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>marches/indices/DAX.csv</t>
+          <t>souverains/CANADA_2A.csv</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -50417,7 +50417,7 @@
         <v>42</v>
       </c>
       <c r="F212" t="n">
-        <v>3801</v>
+        <v>6435</v>
       </c>
       <c r="G212" t="inlineStr">
         <is>
@@ -50428,7 +50428,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>marches/indices/EUROSTOXX50.csv</t>
+          <t>souverains/CANADA_5A.csv</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -50446,7 +50446,7 @@
         <v>42</v>
       </c>
       <c r="F213" t="n">
-        <v>3758</v>
+        <v>6435</v>
       </c>
       <c r="G213" t="inlineStr">
         <is>
@@ -50457,7 +50457,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>marches/indices/FTSE100.csv</t>
+          <t>souverains/CANADA_LONG.csv</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -50475,7 +50475,7 @@
         <v>42</v>
       </c>
       <c r="F214" t="n">
-        <v>3787</v>
+        <v>6435</v>
       </c>
       <c r="G214" t="inlineStr">
         <is>
@@ -50486,7 +50486,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>marches/indices/HANGSENG.csv</t>
+          <t>souverains/SUEDE_10A.csv</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -50504,7 +50504,7 @@
         <v>42</v>
       </c>
       <c r="F215" t="n">
-        <v>3688</v>
+        <v>9202</v>
       </c>
       <c r="G215" t="inlineStr">
         <is>
@@ -50515,7 +50515,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>marches/indices/NIKKEI225.csv</t>
+          <t>souverains/SUEDE_2A.csv</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -50533,7 +50533,7 @@
         <v>42</v>
       </c>
       <c r="F216" t="n">
-        <v>3666</v>
+        <v>9202</v>
       </c>
       <c r="G216" t="inlineStr">
         <is>
@@ -50544,7 +50544,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>souverains/CANADA_10A.csv</t>
+          <t>souverains/SUEDE_5A.csv</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -50562,7 +50562,7 @@
         <v>42</v>
       </c>
       <c r="F217" t="n">
-        <v>6436</v>
+        <v>9204</v>
       </c>
       <c r="G217" t="inlineStr">
         <is>
@@ -50573,7 +50573,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>souverains/CANADA_2A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -50591,7 +50591,7 @@
         <v>42</v>
       </c>
       <c r="F218" t="n">
-        <v>6435</v>
+        <v>5639</v>
       </c>
       <c r="G218" t="inlineStr">
         <is>
@@ -50602,7 +50602,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>souverains/CANADA_5A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -50620,7 +50620,7 @@
         <v>42</v>
       </c>
       <c r="F219" t="n">
-        <v>6435</v>
+        <v>5639</v>
       </c>
       <c r="G219" t="inlineStr">
         <is>
@@ -50631,7 +50631,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>souverains/CANADA_LONG.csv</t>
+          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -50649,7 +50649,7 @@
         <v>42</v>
       </c>
       <c r="F220" t="n">
-        <v>6435</v>
+        <v>5639</v>
       </c>
       <c r="G220" t="inlineStr">
         <is>
@@ -50660,7 +50660,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_10A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -50678,7 +50678,7 @@
         <v>42</v>
       </c>
       <c r="F221" t="n">
-        <v>9202</v>
+        <v>5639</v>
       </c>
       <c r="G221" t="inlineStr">
         <is>
@@ -50689,7 +50689,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_2A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -50707,7 +50707,7 @@
         <v>42</v>
       </c>
       <c r="F222" t="n">
-        <v>9202</v>
+        <v>5639</v>
       </c>
       <c r="G222" t="inlineStr">
         <is>
@@ -50718,7 +50718,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_5A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -50736,7 +50736,7 @@
         <v>42</v>
       </c>
       <c r="F223" t="n">
-        <v>9204</v>
+        <v>5639</v>
       </c>
       <c r="G223" t="inlineStr">
         <is>
@@ -50747,7 +50747,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -50776,7 +50776,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
@@ -50805,7 +50805,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
+          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -50834,7 +50834,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
+          <t>tresor_us/dette_quotidienne.csv</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -50852,7 +50852,7 @@
         <v>42</v>
       </c>
       <c r="F227" t="n">
-        <v>5639</v>
+        <v>2000</v>
       </c>
       <c r="G227" t="inlineStr">
         <is>
@@ -50863,7 +50863,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
+          <t>tresor_us/solde_tresorerie.csv</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -50881,7 +50881,7 @@
         <v>42</v>
       </c>
       <c r="F228" t="n">
-        <v>5639</v>
+        <v>500</v>
       </c>
       <c r="G228" t="inlineStr">
         <is>
@@ -50892,16 +50892,16 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
+          <t>fred/ECBDFR.csv</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C229" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D229" t="n">
         <v>1</v>
@@ -50910,7 +50910,7 @@
         <v>42</v>
       </c>
       <c r="F229" t="n">
-        <v>5639</v>
+        <v>3000</v>
       </c>
       <c r="G229" t="inlineStr">
         <is>
@@ -50921,16 +50921,16 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
+          <t>fred/RRPONTSYD.csv</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C230" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D230" t="n">
         <v>1</v>
@@ -50939,7 +50939,7 @@
         <v>42</v>
       </c>
       <c r="F230" t="n">
-        <v>5639</v>
+        <v>3000</v>
       </c>
       <c r="G230" t="inlineStr">
         <is>
@@ -50950,16 +50950,16 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
+          <t>fred/T10YIE.csv</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C231" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D231" t="n">
         <v>1</v>
@@ -50968,7 +50968,7 @@
         <v>42</v>
       </c>
       <c r="F231" t="n">
-        <v>5639</v>
+        <v>3000</v>
       </c>
       <c r="G231" t="inlineStr">
         <is>
@@ -50979,16 +50979,16 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
+          <t>marches/indices/DAX.csv</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C232" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D232" t="n">
         <v>1</v>
@@ -50997,7 +50997,7 @@
         <v>42</v>
       </c>
       <c r="F232" t="n">
-        <v>5639</v>
+        <v>3802</v>
       </c>
       <c r="G232" t="inlineStr">
         <is>
@@ -51008,16 +51008,16 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>tresor_us/dette_quotidienne.csv</t>
+          <t>marches/indices/EUROSTOXX50.csv</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C233" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D233" t="n">
         <v>1</v>
@@ -51026,7 +51026,7 @@
         <v>42</v>
       </c>
       <c r="F233" t="n">
-        <v>2000</v>
+        <v>3759</v>
       </c>
       <c r="G233" t="inlineStr">
         <is>
@@ -51037,16 +51037,16 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>tresor_us/solde_tresorerie.csv</t>
+          <t>marches/indices/FTSE100.csv</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C234" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D234" t="n">
         <v>1</v>
@@ -51055,7 +51055,7 @@
         <v>42</v>
       </c>
       <c r="F234" t="n">
-        <v>500</v>
+        <v>3788</v>
       </c>
       <c r="G234" t="inlineStr">
         <is>
@@ -51066,7 +51066,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>fred/ECBDFR.csv</t>
+          <t>marches/volatilite/GVZ.csv</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -51084,7 +51084,7 @@
         <v>42</v>
       </c>
       <c r="F235" t="n">
-        <v>3000</v>
+        <v>3770</v>
       </c>
       <c r="G235" t="inlineStr">
         <is>
@@ -51095,7 +51095,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>fred/RRPONTSYD.csv</t>
+          <t>marches/volatilite/MOVE.csv</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -51113,7 +51113,7 @@
         <v>42</v>
       </c>
       <c r="F236" t="n">
-        <v>3000</v>
+        <v>3689</v>
       </c>
       <c r="G236" t="inlineStr">
         <is>
@@ -51124,7 +51124,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>fred/T10YIE.csv</t>
+          <t>marches/volatilite/OVX.csv</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
@@ -51142,7 +51142,7 @@
         <v>42</v>
       </c>
       <c r="F237" t="n">
-        <v>3000</v>
+        <v>3770</v>
       </c>
       <c r="G237" t="inlineStr">
         <is>
@@ -51153,7 +51153,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>marches/fx/AUDJPY.csv</t>
+          <t>marches/volatilite/VVIX.csv</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
@@ -51171,7 +51171,7 @@
         <v>42</v>
       </c>
       <c r="F238" t="n">
-        <v>3908</v>
+        <v>3762</v>
       </c>
       <c r="G238" t="inlineStr">
         <is>
@@ -51182,7 +51182,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>marches/fx/AUDUSD.csv</t>
+          <t>marches/volatilite/VXN.csv</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
@@ -51200,7 +51200,7 @@
         <v>42</v>
       </c>
       <c r="F239" t="n">
-        <v>3904</v>
+        <v>3770</v>
       </c>
       <c r="G239" t="inlineStr">
         <is>
@@ -51211,7 +51211,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>marches/fx/DXY.csv</t>
+          <t>yfinance/SP500.csv</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
@@ -51229,7 +51229,7 @@
         <v>42</v>
       </c>
       <c r="F240" t="n">
-        <v>3772</v>
+        <v>7546</v>
       </c>
       <c r="G240" t="inlineStr">
         <is>
@@ -51240,7 +51240,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>marches/fx/EURCHF.csv</t>
+          <t>yfinance/VIX.csv</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
@@ -51258,7 +51258,7 @@
         <v>42</v>
       </c>
       <c r="F241" t="n">
-        <v>3905</v>
+        <v>7548</v>
       </c>
       <c r="G241" t="inlineStr">
         <is>
@@ -51269,7 +51269,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>marches/fx/EURGBP.csv</t>
+          <t>yfinance/XLB.csv</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
@@ -51287,7 +51287,7 @@
         <v>42</v>
       </c>
       <c r="F242" t="n">
-        <v>3907</v>
+        <v>500</v>
       </c>
       <c r="G242" t="inlineStr">
         <is>
@@ -51298,7 +51298,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>marches/fx/EURJPY.csv</t>
+          <t>yfinance/XLE.csv</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
@@ -51316,7 +51316,7 @@
         <v>42</v>
       </c>
       <c r="F243" t="n">
-        <v>3907</v>
+        <v>500</v>
       </c>
       <c r="G243" t="inlineStr">
         <is>
@@ -51327,7 +51327,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>marches/fx/EURUSD.csv</t>
+          <t>yfinance/XLF.csv</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -51345,7 +51345,7 @@
         <v>42</v>
       </c>
       <c r="F244" t="n">
-        <v>3904</v>
+        <v>500</v>
       </c>
       <c r="G244" t="inlineStr">
         <is>
@@ -51356,7 +51356,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>marches/fx/GBPUSD.csv</t>
+          <t>yfinance/XLI.csv</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -51374,7 +51374,7 @@
         <v>42</v>
       </c>
       <c r="F245" t="n">
-        <v>3905</v>
+        <v>500</v>
       </c>
       <c r="G245" t="inlineStr">
         <is>
@@ -51385,7 +51385,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>marches/fx/NZDUSD.csv</t>
+          <t>yfinance/XLK.csv</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -51403,7 +51403,7 @@
         <v>42</v>
       </c>
       <c r="F246" t="n">
-        <v>3905</v>
+        <v>500</v>
       </c>
       <c r="G246" t="inlineStr">
         <is>
@@ -51414,7 +51414,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>marches/fx/USDCAD.csv</t>
+          <t>yfinance/XLP.csv</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
@@ -51432,7 +51432,7 @@
         <v>42</v>
       </c>
       <c r="F247" t="n">
-        <v>3904</v>
+        <v>500</v>
       </c>
       <c r="G247" t="inlineStr">
         <is>
@@ -51443,7 +51443,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>marches/fx/USDCHF.csv</t>
+          <t>yfinance/XLRE.csv</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
@@ -51461,7 +51461,7 @@
         <v>42</v>
       </c>
       <c r="F248" t="n">
-        <v>3902</v>
+        <v>500</v>
       </c>
       <c r="G248" t="inlineStr">
         <is>
@@ -51472,7 +51472,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>marches/fx/USDCNY.csv</t>
+          <t>yfinance/XLU.csv</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
@@ -51490,7 +51490,7 @@
         <v>42</v>
       </c>
       <c r="F249" t="n">
-        <v>3904</v>
+        <v>500</v>
       </c>
       <c r="G249" t="inlineStr">
         <is>
@@ -51501,7 +51501,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>marches/fx/USDJPY.csv</t>
+          <t>yfinance/XLV.csv</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
@@ -51519,7 +51519,7 @@
         <v>42</v>
       </c>
       <c r="F250" t="n">
-        <v>3905</v>
+        <v>500</v>
       </c>
       <c r="G250" t="inlineStr">
         <is>
@@ -51530,7 +51530,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>marches/fx/USDKRW.csv</t>
+          <t>yfinance/XLY.csv</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
@@ -51548,7 +51548,7 @@
         <v>42</v>
       </c>
       <c r="F251" t="n">
-        <v>3904</v>
+        <v>500</v>
       </c>
       <c r="G251" t="inlineStr">
         <is>
@@ -51559,16 +51559,16 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>marches/fx/USDNOK.csv</t>
+          <t>marches/fx/AUDJPY.csv</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C252" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D252" t="n">
         <v>1</v>
@@ -51577,7 +51577,7 @@
         <v>42</v>
       </c>
       <c r="F252" t="n">
-        <v>3905</v>
+        <v>3908</v>
       </c>
       <c r="G252" t="inlineStr">
         <is>
@@ -51588,16 +51588,16 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>marches/fx/USDSEK.csv</t>
+          <t>marches/fx/AUDUSD.csv</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C253" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D253" t="n">
         <v>1</v>
@@ -51606,7 +51606,7 @@
         <v>42</v>
       </c>
       <c r="F253" t="n">
-        <v>3905</v>
+        <v>3904</v>
       </c>
       <c r="G253" t="inlineStr">
         <is>
@@ -51617,16 +51617,16 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>marches/matieres/BRENT.csv</t>
+          <t>marches/fx/DXY.csv</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C254" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D254" t="n">
         <v>1</v>
@@ -51635,7 +51635,7 @@
         <v>42</v>
       </c>
       <c r="F254" t="n">
-        <v>3751</v>
+        <v>3773</v>
       </c>
       <c r="G254" t="inlineStr">
         <is>
@@ -51646,16 +51646,16 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>marches/matieres/CUIVRE.csv</t>
+          <t>marches/fx/EURCHF.csv</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C255" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D255" t="n">
         <v>1</v>
@@ -51664,7 +51664,7 @@
         <v>42</v>
       </c>
       <c r="F255" t="n">
-        <v>3771</v>
+        <v>3905</v>
       </c>
       <c r="G255" t="inlineStr">
         <is>
@@ -51675,16 +51675,16 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>marches/matieres/GAZ_HENRY_HUB.csv</t>
+          <t>marches/fx/EURGBP.csv</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C256" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D256" t="n">
         <v>1</v>
@@ -51693,7 +51693,7 @@
         <v>42</v>
       </c>
       <c r="F256" t="n">
-        <v>3772</v>
+        <v>3907</v>
       </c>
       <c r="G256" t="inlineStr">
         <is>
@@ -51704,16 +51704,16 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>marches/matieres/OR.csv</t>
+          <t>marches/fx/EURJPY.csv</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C257" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D257" t="n">
         <v>1</v>
@@ -51722,7 +51722,7 @@
         <v>42</v>
       </c>
       <c r="F257" t="n">
-        <v>3771</v>
+        <v>3907</v>
       </c>
       <c r="G257" t="inlineStr">
         <is>
@@ -51733,16 +51733,16 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>marches/matieres/WTI.csv</t>
+          <t>marches/fx/EURUSD.csv</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C258" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D258" t="n">
         <v>1</v>
@@ -51751,7 +51751,7 @@
         <v>42</v>
       </c>
       <c r="F258" t="n">
-        <v>3771</v>
+        <v>3904</v>
       </c>
       <c r="G258" t="inlineStr">
         <is>
@@ -51762,16 +51762,16 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>marches/taux_futures/FED_FUNDS_FRONT.csv</t>
+          <t>marches/fx/GBPUSD.csv</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C259" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D259" t="n">
         <v>1</v>
@@ -51780,7 +51780,7 @@
         <v>42</v>
       </c>
       <c r="F259" t="n">
-        <v>3772</v>
+        <v>3905</v>
       </c>
       <c r="G259" t="inlineStr">
         <is>
@@ -51791,16 +51791,16 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>marches/volatilite/GVZ.csv</t>
+          <t>marches/fx/NZDUSD.csv</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C260" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D260" t="n">
         <v>1</v>
@@ -51809,7 +51809,7 @@
         <v>42</v>
       </c>
       <c r="F260" t="n">
-        <v>3770</v>
+        <v>3905</v>
       </c>
       <c r="G260" t="inlineStr">
         <is>
@@ -51820,16 +51820,16 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>marches/volatilite/MOVE.csv</t>
+          <t>marches/fx/USDCAD.csv</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C261" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D261" t="n">
         <v>1</v>
@@ -51838,7 +51838,7 @@
         <v>42</v>
       </c>
       <c r="F261" t="n">
-        <v>3689</v>
+        <v>3904</v>
       </c>
       <c r="G261" t="inlineStr">
         <is>
@@ -51849,16 +51849,16 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>marches/volatilite/OVX.csv</t>
+          <t>marches/fx/USDCHF.csv</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C262" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D262" t="n">
         <v>1</v>
@@ -51867,7 +51867,7 @@
         <v>42</v>
       </c>
       <c r="F262" t="n">
-        <v>3770</v>
+        <v>3902</v>
       </c>
       <c r="G262" t="inlineStr">
         <is>
@@ -51878,16 +51878,16 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>marches/volatilite/VVIX.csv</t>
+          <t>marches/fx/USDCNY.csv</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C263" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D263" t="n">
         <v>1</v>
@@ -51896,7 +51896,7 @@
         <v>42</v>
       </c>
       <c r="F263" t="n">
-        <v>3762</v>
+        <v>3904</v>
       </c>
       <c r="G263" t="inlineStr">
         <is>
@@ -51907,16 +51907,16 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>marches/volatilite/VXN.csv</t>
+          <t>marches/fx/USDJPY.csv</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C264" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D264" t="n">
         <v>1</v>
@@ -51925,7 +51925,7 @@
         <v>42</v>
       </c>
       <c r="F264" t="n">
-        <v>3770</v>
+        <v>3905</v>
       </c>
       <c r="G264" t="inlineStr">
         <is>
@@ -51936,16 +51936,16 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>yfinance/SP500.csv</t>
+          <t>marches/fx/USDKRW.csv</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C265" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D265" t="n">
         <v>1</v>
@@ -51954,7 +51954,7 @@
         <v>42</v>
       </c>
       <c r="F265" t="n">
-        <v>7546</v>
+        <v>3904</v>
       </c>
       <c r="G265" t="inlineStr">
         <is>
@@ -51965,16 +51965,16 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>yfinance/VIX.csv</t>
+          <t>marches/fx/USDNOK.csv</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C266" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D266" t="n">
         <v>1</v>
@@ -51983,7 +51983,7 @@
         <v>42</v>
       </c>
       <c r="F266" t="n">
-        <v>7548</v>
+        <v>3905</v>
       </c>
       <c r="G266" t="inlineStr">
         <is>
@@ -51994,16 +51994,16 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>yfinance/XLB.csv</t>
+          <t>marches/fx/USDSEK.csv</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C267" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D267" t="n">
         <v>1</v>
@@ -52012,7 +52012,7 @@
         <v>42</v>
       </c>
       <c r="F267" t="n">
-        <v>500</v>
+        <v>3905</v>
       </c>
       <c r="G267" t="inlineStr">
         <is>
@@ -52023,16 +52023,16 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>yfinance/XLE.csv</t>
+          <t>marches/indices/HANGSENG.csv</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C268" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D268" t="n">
         <v>1</v>
@@ -52041,7 +52041,7 @@
         <v>42</v>
       </c>
       <c r="F268" t="n">
-        <v>500</v>
+        <v>3689</v>
       </c>
       <c r="G268" t="inlineStr">
         <is>
@@ -52052,16 +52052,16 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>yfinance/XLF.csv</t>
+          <t>marches/indices/KOSPI.csv</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C269" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D269" t="n">
         <v>1</v>
@@ -52070,7 +52070,7 @@
         <v>42</v>
       </c>
       <c r="F269" t="n">
-        <v>500</v>
+        <v>3681</v>
       </c>
       <c r="G269" t="inlineStr">
         <is>
@@ -52081,16 +52081,16 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>yfinance/XLI.csv</t>
+          <t>marches/indices/NIKKEI225.csv</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C270" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D270" t="n">
         <v>1</v>
@@ -52099,7 +52099,7 @@
         <v>42</v>
       </c>
       <c r="F270" t="n">
-        <v>500</v>
+        <v>3667</v>
       </c>
       <c r="G270" t="inlineStr">
         <is>
@@ -52110,16 +52110,16 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>yfinance/XLK.csv</t>
+          <t>marches/matieres/BRENT.csv</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C271" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D271" t="n">
         <v>1</v>
@@ -52128,7 +52128,7 @@
         <v>42</v>
       </c>
       <c r="F271" t="n">
-        <v>500</v>
+        <v>3751</v>
       </c>
       <c r="G271" t="inlineStr">
         <is>
@@ -52139,16 +52139,16 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>yfinance/XLP.csv</t>
+          <t>marches/matieres/CUIVRE.csv</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C272" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D272" t="n">
         <v>1</v>
@@ -52157,7 +52157,7 @@
         <v>42</v>
       </c>
       <c r="F272" t="n">
-        <v>500</v>
+        <v>3772</v>
       </c>
       <c r="G272" t="inlineStr">
         <is>
@@ -52168,16 +52168,16 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>yfinance/XLRE.csv</t>
+          <t>marches/matieres/GAZ_HENRY_HUB.csv</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C273" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D273" t="n">
         <v>1</v>
@@ -52186,7 +52186,7 @@
         <v>42</v>
       </c>
       <c r="F273" t="n">
-        <v>500</v>
+        <v>3773</v>
       </c>
       <c r="G273" t="inlineStr">
         <is>
@@ -52197,16 +52197,16 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>yfinance/XLU.csv</t>
+          <t>marches/matieres/OR.csv</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C274" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D274" t="n">
         <v>1</v>
@@ -52215,7 +52215,7 @@
         <v>42</v>
       </c>
       <c r="F274" t="n">
-        <v>500</v>
+        <v>3772</v>
       </c>
       <c r="G274" t="inlineStr">
         <is>
@@ -52226,16 +52226,16 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>yfinance/XLV.csv</t>
+          <t>marches/matieres/WTI.csv</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C275" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D275" t="n">
         <v>1</v>
@@ -52244,7 +52244,7 @@
         <v>42</v>
       </c>
       <c r="F275" t="n">
-        <v>500</v>
+        <v>3772</v>
       </c>
       <c r="G275" t="inlineStr">
         <is>
@@ -52255,16 +52255,16 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>yfinance/XLY.csv</t>
+          <t>marches/taux_futures/FED_FUNDS_FRONT.csv</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C276" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D276" t="n">
         <v>1</v>
@@ -52273,7 +52273,7 @@
         <v>42</v>
       </c>
       <c r="F276" t="n">
-        <v>500</v>
+        <v>3772</v>
       </c>
       <c r="G276" t="inlineStr">
         <is>
@@ -53802,17 +53802,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7080.92</v>
+        <v>6876.98</v>
       </c>
       <c r="D2" t="n">
-        <v>-16.41</v>
+        <v>-18.87</v>
       </c>
       <c r="E2" t="n">
-        <v>103.11</v>
+        <v>100.42</v>
       </c>
     </row>
     <row r="3">
@@ -53823,65 +53823,65 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>66364.2</v>
+        <v>65281.24</v>
       </c>
       <c r="D3" t="n">
-        <v>-4.32</v>
+        <v>-6.82</v>
       </c>
       <c r="E3" t="n">
-        <v>45.04</v>
+        <v>44.93</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Royaume-Uni (FTSE 100)</t>
+          <t>Etats-Unis (S&amp;P 500)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>10695.3</v>
+        <v>7683.69</v>
       </c>
       <c r="D4" t="n">
-        <v>1.78</v>
+        <v>3.27</v>
       </c>
       <c r="E4" t="n">
-        <v>16.08</v>
+        <v>15.65</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Zone euro (Euro Stoxx 50)</t>
+          <t>Royaume-Uni (FTSE 100)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>6302.82</v>
+        <v>10684.9</v>
       </c>
       <c r="D5" t="n">
-        <v>1.31</v>
+        <v>1.91</v>
       </c>
       <c r="E5" t="n">
-        <v>15.76</v>
+        <v>15.08</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Etats-Unis (S&amp;P 500)</t>
+          <t>Zone euro (Euro Stoxx 50)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -53890,13 +53890,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>7683.69</v>
+        <v>6301.28</v>
       </c>
       <c r="D6" t="n">
-        <v>3.27</v>
+        <v>1.12</v>
       </c>
       <c r="E6" t="n">
-        <v>15.65</v>
+        <v>14.57</v>
       </c>
     </row>
     <row r="7">
@@ -53907,17 +53907,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>25408.64</v>
+        <v>25374.42</v>
       </c>
       <c r="D7" t="n">
-        <v>2.99</v>
+        <v>3.04</v>
       </c>
       <c r="E7" t="n">
-        <v>7.96</v>
+        <v>6.89</v>
       </c>
     </row>
     <row r="8">
@@ -53928,17 +53928,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>24510.09</v>
+        <v>24507.08</v>
       </c>
       <c r="D8" t="n">
-        <v>8.109999999999999</v>
+        <v>7.11</v>
       </c>
       <c r="E8" t="n">
-        <v>-7.46</v>
+        <v>-7.95</v>
       </c>
     </row>
   </sheetData>
@@ -55762,7 +55762,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -56095,6 +56095,34 @@
       </c>
       <c r="H11" t="n">
         <v>5.4</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.00159</v>
+      </c>
+      <c r="C12" t="n">
+        <v>3.68</v>
+      </c>
+      <c r="D12" t="n">
+        <v>99.09</v>
+      </c>
+      <c r="E12" t="n">
+        <v>35.89</v>
+      </c>
+      <c r="F12" t="n">
+        <v>45.78</v>
+      </c>
+      <c r="G12" t="n">
+        <v>-4.24</v>
+      </c>
+      <c r="H12" t="n">
+        <v>5.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-29T05:52Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-29 02:45 UTC</t>
+          <t>Genere le 2026-09-29 05:52 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-29 02:45 UTC</t>
+          <t>Rapport global — 2026-09-29 05:52 UTC</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>**Matieres premieres macro** — ratio cuivre/or stable -- pas de signal net sur la croissance (+3.7% sur 3 mois). Brent 99.1$ (+35.9% sur 3 mois, +45.8% sur 12 mois), gaz -4.2% sur 3 mois, ecart Brent-WTI +5.6$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-29)_</t>
+          <t>**Matieres premieres macro** — ratio cuivre/or stable -- pas de signal net sur la croissance (+3.8% sur 3 mois). Brent 100.1$ (+37.3% sur 3 mois, +47.3% sur 12 mois), gaz -4.6% sur 3 mois, ecart Brent-WTI +5.5$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -876,7 +876,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>**Pentes courbes** — 7 courbes : pente de +0.30pt (Australie) a +1.20pt (Japon) -- aucune courbe inversee -- pas de signal recessif par la pente _(observation : 2026-09-25)_</t>
+          <t>**Pentes courbes** — 7 courbes : pente de +0.30pt (Australie) a +1.20pt (Japon) -- aucune courbe inversee -- pas de signal recessif par la pente _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -960,7 +960,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>**Indices mondiaux** — 7 indices (devise locale) : Coree (KOSPI) +100.4% en tete sur 12 mois, Hong Kong (Hang Seng) -8.0% en queue -- ecart tres large entre blocs sur 12 mois (108pt) -- les cycles economiques ou les flux divergent nettement. ROTATION en cours : Coree (KOSPI) mene sur 12 mois mais Hong Kong (Hang Seng) a repris la tete sur 3 mois _(observation : 2026-09-29)_</t>
+          <t>**Indices mondiaux** — 7 indices (devise locale) : Coree (KOSPI) +98.3% en tete sur 12 mois, Hong Kong (Hang Seng) -8.0% en queue -- ecart tres large entre blocs sur 12 mois (106pt) -- les cycles economiques ou les flux divergent nettement. ROTATION en cours : Coree (KOSPI) mene sur 12 mois mais Hong Kong (Hang Seng) a repris la tete sur 3 mois _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1240,7 +1240,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.37301696508358795 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.05236409373895107 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-28)_</t>
+          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.3730169650835773 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.052364093738951525 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -50486,7 +50486,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_10A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -50504,7 +50504,7 @@
         <v>42</v>
       </c>
       <c r="F215" t="n">
-        <v>9202</v>
+        <v>5639</v>
       </c>
       <c r="G215" t="inlineStr">
         <is>
@@ -50515,7 +50515,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_2A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -50533,7 +50533,7 @@
         <v>42</v>
       </c>
       <c r="F216" t="n">
-        <v>9202</v>
+        <v>5639</v>
       </c>
       <c r="G216" t="inlineStr">
         <is>
@@ -50544,7 +50544,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_5A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -50562,7 +50562,7 @@
         <v>42</v>
       </c>
       <c r="F217" t="n">
-        <v>9204</v>
+        <v>5639</v>
       </c>
       <c r="G217" t="inlineStr">
         <is>
@@ -50573,7 +50573,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -50602,7 +50602,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -50631,7 +50631,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -50660,7 +50660,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -50689,7 +50689,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -50718,7 +50718,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
+          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -50747,7 +50747,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
+          <t>tresor_us/dette_quotidienne.csv</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -50765,7 +50765,7 @@
         <v>42</v>
       </c>
       <c r="F224" t="n">
-        <v>5639</v>
+        <v>2000</v>
       </c>
       <c r="G224" t="inlineStr">
         <is>
@@ -50776,7 +50776,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
+          <t>tresor_us/solde_tresorerie.csv</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
@@ -50794,7 +50794,7 @@
         <v>42</v>
       </c>
       <c r="F225" t="n">
-        <v>5639</v>
+        <v>500</v>
       </c>
       <c r="G225" t="inlineStr">
         <is>
@@ -50805,16 +50805,16 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
+          <t>fred/ECBDFR.csv</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C226" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D226" t="n">
         <v>1</v>
@@ -50823,7 +50823,7 @@
         <v>42</v>
       </c>
       <c r="F226" t="n">
-        <v>5639</v>
+        <v>3000</v>
       </c>
       <c r="G226" t="inlineStr">
         <is>
@@ -50834,16 +50834,16 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>tresor_us/dette_quotidienne.csv</t>
+          <t>fred/RRPONTSYD.csv</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C227" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D227" t="n">
         <v>1</v>
@@ -50852,7 +50852,7 @@
         <v>42</v>
       </c>
       <c r="F227" t="n">
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="G227" t="inlineStr">
         <is>
@@ -50863,16 +50863,16 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>tresor_us/solde_tresorerie.csv</t>
+          <t>fred/T10YIE.csv</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C228" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D228" t="n">
         <v>1</v>
@@ -50881,7 +50881,7 @@
         <v>42</v>
       </c>
       <c r="F228" t="n">
-        <v>500</v>
+        <v>3000</v>
       </c>
       <c r="G228" t="inlineStr">
         <is>
@@ -50892,7 +50892,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>fred/ECBDFR.csv</t>
+          <t>marches/indices/DAX.csv</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -50910,7 +50910,7 @@
         <v>42</v>
       </c>
       <c r="F229" t="n">
-        <v>3000</v>
+        <v>3802</v>
       </c>
       <c r="G229" t="inlineStr">
         <is>
@@ -50921,7 +50921,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>fred/RRPONTSYD.csv</t>
+          <t>marches/indices/EUROSTOXX50.csv</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -50939,7 +50939,7 @@
         <v>42</v>
       </c>
       <c r="F230" t="n">
-        <v>3000</v>
+        <v>3759</v>
       </c>
       <c r="G230" t="inlineStr">
         <is>
@@ -50950,7 +50950,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>fred/T10YIE.csv</t>
+          <t>marches/indices/FTSE100.csv</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -50968,7 +50968,7 @@
         <v>42</v>
       </c>
       <c r="F231" t="n">
-        <v>3000</v>
+        <v>3788</v>
       </c>
       <c r="G231" t="inlineStr">
         <is>
@@ -50979,7 +50979,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>marches/indices/DAX.csv</t>
+          <t>marches/volatilite/GVZ.csv</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -50997,7 +50997,7 @@
         <v>42</v>
       </c>
       <c r="F232" t="n">
-        <v>3802</v>
+        <v>3770</v>
       </c>
       <c r="G232" t="inlineStr">
         <is>
@@ -51008,7 +51008,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>marches/indices/EUROSTOXX50.csv</t>
+          <t>marches/volatilite/MOVE.csv</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -51026,7 +51026,7 @@
         <v>42</v>
       </c>
       <c r="F233" t="n">
-        <v>3759</v>
+        <v>3689</v>
       </c>
       <c r="G233" t="inlineStr">
         <is>
@@ -51037,7 +51037,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>marches/indices/FTSE100.csv</t>
+          <t>marches/volatilite/OVX.csv</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -51055,7 +51055,7 @@
         <v>42</v>
       </c>
       <c r="F234" t="n">
-        <v>3788</v>
+        <v>3770</v>
       </c>
       <c r="G234" t="inlineStr">
         <is>
@@ -51066,7 +51066,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>marches/volatilite/GVZ.csv</t>
+          <t>marches/volatilite/VVIX.csv</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -51084,7 +51084,7 @@
         <v>42</v>
       </c>
       <c r="F235" t="n">
-        <v>3770</v>
+        <v>3762</v>
       </c>
       <c r="G235" t="inlineStr">
         <is>
@@ -51095,7 +51095,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>marches/volatilite/MOVE.csv</t>
+          <t>marches/volatilite/VXN.csv</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -51113,7 +51113,7 @@
         <v>42</v>
       </c>
       <c r="F236" t="n">
-        <v>3689</v>
+        <v>3770</v>
       </c>
       <c r="G236" t="inlineStr">
         <is>
@@ -51124,7 +51124,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>marches/volatilite/OVX.csv</t>
+          <t>souverains/SUEDE_10A.csv</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
@@ -51142,7 +51142,7 @@
         <v>42</v>
       </c>
       <c r="F237" t="n">
-        <v>3770</v>
+        <v>9203</v>
       </c>
       <c r="G237" t="inlineStr">
         <is>
@@ -51153,7 +51153,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>marches/volatilite/VVIX.csv</t>
+          <t>souverains/SUEDE_2A.csv</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
@@ -51171,7 +51171,7 @@
         <v>42</v>
       </c>
       <c r="F238" t="n">
-        <v>3762</v>
+        <v>9203</v>
       </c>
       <c r="G238" t="inlineStr">
         <is>
@@ -51182,7 +51182,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>marches/volatilite/VXN.csv</t>
+          <t>souverains/SUEDE_5A.csv</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
@@ -51200,7 +51200,7 @@
         <v>42</v>
       </c>
       <c r="F239" t="n">
-        <v>3770</v>
+        <v>9205</v>
       </c>
       <c r="G239" t="inlineStr">
         <is>
@@ -51635,7 +51635,7 @@
         <v>42</v>
       </c>
       <c r="F254" t="n">
-        <v>3773</v>
+        <v>3772</v>
       </c>
       <c r="G254" t="inlineStr">
         <is>
@@ -52157,7 +52157,7 @@
         <v>42</v>
       </c>
       <c r="F272" t="n">
-        <v>3772</v>
+        <v>3771</v>
       </c>
       <c r="G272" t="inlineStr">
         <is>
@@ -52186,7 +52186,7 @@
         <v>42</v>
       </c>
       <c r="F273" t="n">
-        <v>3773</v>
+        <v>3772</v>
       </c>
       <c r="G273" t="inlineStr">
         <is>
@@ -52215,7 +52215,7 @@
         <v>42</v>
       </c>
       <c r="F274" t="n">
-        <v>3772</v>
+        <v>3771</v>
       </c>
       <c r="G274" t="inlineStr">
         <is>
@@ -52244,7 +52244,7 @@
         <v>42</v>
       </c>
       <c r="F275" t="n">
-        <v>3772</v>
+        <v>3771</v>
       </c>
       <c r="G275" t="inlineStr">
         <is>
@@ -53806,13 +53806,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>6876.98</v>
+        <v>6804.68</v>
       </c>
       <c r="D2" t="n">
-        <v>-18.87</v>
+        <v>-19.72</v>
       </c>
       <c r="E2" t="n">
-        <v>100.42</v>
+        <v>98.31999999999999</v>
       </c>
     </row>
     <row r="3">
@@ -53827,13 +53827,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>65281.24</v>
+        <v>64842.17</v>
       </c>
       <c r="D3" t="n">
-        <v>-6.82</v>
+        <v>-7.45</v>
       </c>
       <c r="E3" t="n">
-        <v>44.93</v>
+        <v>43.95</v>
       </c>
     </row>
     <row r="4">
@@ -53932,13 +53932,13 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>24507.08</v>
+        <v>24504.65</v>
       </c>
       <c r="D8" t="n">
-        <v>7.11</v>
+        <v>7.1</v>
       </c>
       <c r="E8" t="n">
-        <v>-7.95</v>
+        <v>-7.96</v>
       </c>
     </row>
   </sheetData>
@@ -56104,25 +56104,25 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.00159</v>
+        <v>0.001591</v>
       </c>
       <c r="C12" t="n">
-        <v>3.68</v>
+        <v>3.77</v>
       </c>
       <c r="D12" t="n">
-        <v>99.09</v>
+        <v>100.11</v>
       </c>
       <c r="E12" t="n">
-        <v>35.89</v>
+        <v>37.29</v>
       </c>
       <c r="F12" t="n">
-        <v>45.78</v>
+        <v>47.29</v>
       </c>
       <c r="G12" t="n">
-        <v>-4.24</v>
+        <v>-4.64</v>
       </c>
       <c r="H12" t="n">
-        <v>5.6</v>
+        <v>5.52</v>
       </c>
     </row>
   </sheetData>
@@ -60960,26 +60960,26 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>2.79</v>
+        <v>2.793</v>
       </c>
       <c r="D6" t="n">
-        <v>3.279</v>
+        <v>3.285</v>
       </c>
       <c r="E6" t="n">
-        <v>0.489</v>
+        <v>0.492</v>
       </c>
       <c r="F6" t="n">
-        <v>-0.038</v>
+        <v>-0.028</v>
       </c>
       <c r="G6" t="n">
-        <v>0.659</v>
+        <v>0.657</v>
       </c>
       <c r="H6" t="n">
-        <v>0.621</v>
+        <v>0.629</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-29T09:09Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-29 05:52 UTC</t>
+          <t>Genere le 2026-09-29 09:09 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-29 05:52 UTC</t>
+          <t>Rapport global — 2026-09-29 09:09 UTC</t>
         </is>
       </c>
     </row>
@@ -785,7 +785,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>**Activite zone euro** — zone euro : Production industrielle -0.2 % sur 12 mois, Ventes de detail +0.8 % sur 12 mois, Taux de chomage +0.1 pt sur 12 mois, Confiance industrielle +1.2 pt vs moyenne longue -- production industrielle DIVERGENTE entre grands pays -- en hausse : Espagne ; en baisse : Allemagne, France, Italie _(observation : date non exposee)_</t>
+          <t>**Activite zone euro** — zone euro : Production industrielle -0.2 % sur 12 mois, Ventes de detail +0.8 % sur 12 mois, Taux de chomage +0.1 pt sur 12 mois, Confiance industrielle +2.7 pt vs moyenne longue -- production industrielle DIVERGENTE entre grands pays -- en hausse : Espagne ; en baisse : Allemagne, France, Italie _(observation : date non exposee)_</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>**Matieres premieres macro** — ratio cuivre/or stable -- pas de signal net sur la croissance (+3.8% sur 3 mois). Brent 100.1$ (+37.3% sur 3 mois, +47.3% sur 12 mois), gaz -4.6% sur 3 mois, ecart Brent-WTI +5.5$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-29)_</t>
+          <t>**Matieres premieres macro** — ratio cuivre/or stable -- pas de signal net sur la croissance (+3.1% sur 3 mois). Brent 97.9$ (+34.2% sur 3 mois, +44.0% sur 12 mois), gaz -5.2% sur 3 mois, ecart Brent-WTI +5.1$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -862,7 +862,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>**Conditions financieres** — indice conditions financieres=+0.086 (3 composantes: {'taux_directeur': 0.5982151864455719, 'courbe_inversee': 0.17031877422284264, 'vix': -0.5114551673321737}) -- conditions proches de la normale _(observation : 2026-09-25)_</t>
+          <t>**Conditions financieres** — indice conditions financieres=+0.083 (3 composantes: {'taux_directeur': 0.5982151864455719, 'courbe_inversee': 0.17031877422284264, 'vix': -0.5188320907186125}) -- conditions proches de la normale _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
@@ -960,7 +960,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>**Indices mondiaux** — 7 indices (devise locale) : Coree (KOSPI) +98.3% en tete sur 12 mois, Hong Kong (Hang Seng) -8.0% en queue -- ecart tres large entre blocs sur 12 mois (106pt) -- les cycles economiques ou les flux divergent nettement. ROTATION en cours : Coree (KOSPI) mene sur 12 mois mais Hong Kong (Hang Seng) a repris la tete sur 3 mois _(observation : 2026-09-29)_</t>
+          <t>**Indices mondiaux** — 7 indices (devise locale) : Coree (KOSPI) +100.2% en tete sur 12 mois, Hong Kong (Hang Seng) -7.9% en queue -- ecart tres large entre blocs sur 12 mois (108pt) -- les cycles economiques ou les flux divergent nettement. ROTATION en cours : Coree (KOSPI) mene sur 12 mois mais Hong Kong (Hang Seng) a repris la tete sur 3 mois _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1191,7 +1191,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>**Vol cross asset** — 6 mesures de volatilite : Petrole (OVX) 89e pct, Or (GVZ) 87e pct, Taux US (MOVE) 51e pct, Nasdaq (VXN) 48e pct, Vol de la vol (VVIX) 37e pct, Actions US (VIX) 32e pct -- stress LOCALISE sur Petrole (OVX), Or (GVZ) pendant que le reste ne l'est pas -- episode propre a cette classe d'actifs, pas une aversion au risque d'ensemble _(observation : 2026-09-28)_</t>
+          <t>**Vol cross asset** — 6 mesures de volatilite : Petrole (OVX) 89e pct, Or (GVZ) 87e pct, Taux US (MOVE) 51e pct, Nasdaq (VXN) 48e pct, Vol de la vol (VVIX) 37e pct, Actions US (VIX) 32e pct -- stress LOCALISE sur Petrole (OVX), Or (GVZ) pendant que le reste ne l'est pas -- episode propre a cette classe d'actifs, pas une aversion au risque d'ensemble _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1219,7 +1219,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>**Ornstein uhlenbeck vix** — VIX actuel=16.07, niveau moyen estime (mu)=20.20, demi-vie=28.8j, ecart actuel=-4.13 -- VIX actuel en-dessous de son niveau moyen de long terme _(observation : 2026-09-28)_</t>
+          <t>**Ornstein uhlenbeck vix** — VIX actuel=16.01, niveau moyen estime (mu)=20.20, demi-vie=28.8j, ecart actuel=-4.19 -- VIX actuel en-dessous de son niveau moyen de long terme _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1233,7 +1233,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>**Kalman niveau local** — VIX observe=16.07, filtre Kalman=15.91 (ecart-type=0.62), ratio signal/bruit=0.2052 -- le filtre lisse fortement le bruit, reagit lentement (ecart obs.-filtre=+0.16) _(observation : 2026-09-28)_</t>
+          <t>**Kalman niveau local** — VIX observe=16.01, filtre Kalman=15.99 (ecart-type=0.62), ratio signal/bruit=0.2052 -- le filtre lisse fortement le bruit, reagit lentement (ecart obs.-filtre=+0.02) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1247,7 +1247,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>**Analyse spectrale** — 3 periodes dominantes (jours de bourse) : [2.2, 3.0, 2.4] -- aucune des 3 periodes dominantes ne correspond a un cycle connu (hebdo/mensuel/trimestriel) _(observation : 2026-09-28)_</t>
+          <t>**Analyse spectrale** — 3 periodes dominantes (jours de bourse) : [2.2, 4.0, 5.4] -- cycle(s) connu(s) qui ressortent : 4.0j~hebdomadaire, 5.4j~hebdomadaire _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1317,7 +1317,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>**Qualite regime macro** — instabilite taux=0.0088, instabilite VIX=0.0684 -- score qualite du regime=-0.0386 (plus haut = regime plus stable/previsible) _(observation : 2026-09-25)_</t>
+          <t>**Qualite regime macro** — instabilite taux=0.0088, instabilite VIX=0.0681 -- score qualite du regime=-0.0384 (plus haut = regime plus stable/previsible) _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1331,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>**Decomposition stl** — VIX : tendance=15.56, composante saisonniere (periode 5j)=+0.141, residu=+0.371 -- la saisonnalite explique 0.72% de la variance totale (negligeable) _(observation : 2026-09-28)_</t>
+          <t>**Decomposition stl** — VIX : tendance=15.51, composante saisonniere (periode 5j)=+0.574, residu=-0.075 -- la saisonnalite explique 0.72% de la variance totale (negligeable) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1457,7 +1457,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>**Arima** — ARIMA(1,1,1) sur 100 previsions 1-jour test : RMSE=2.327 vs baseline naive MSE=5.430 -- ARIMA bat la persistance simple _(observation : 2026-09-28)_</t>
+          <t>**Arima** — ARIMA(1,1,1) sur 100 previsions 1-jour test : RMSE=2.319 vs baseline naive MSE=5.450 -- ARIMA bat la persistance simple _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -8703,14 +8703,14 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>16.07</v>
+        <v>16.01</v>
       </c>
       <c r="D7" t="n">
-        <v>32.5</v>
+        <v>32</v>
       </c>
       <c r="E7" t="n">
         <v>1260</v>
@@ -20746,14 +20746,14 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-09</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>-5.3</v>
+        <v>-3.8</v>
       </c>
       <c r="E17" t="n">
-        <v>1.17</v>
+        <v>2.66</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -20774,14 +20774,14 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-09</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>-11</v>
+        <v>-8.199999999999999</v>
       </c>
       <c r="E18" t="n">
-        <v>-3.47</v>
+        <v>-0.67</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -20802,14 +20802,14 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-09</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>-3.6</v>
+        <v>-5.2</v>
       </c>
       <c r="E19" t="n">
-        <v>3.32</v>
+        <v>1.71</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -20830,14 +20830,14 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-09</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>-4.8</v>
+        <v>-3.2</v>
       </c>
       <c r="E20" t="n">
-        <v>1.09</v>
+        <v>2.68</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -20858,14 +20858,14 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-09</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>-3.7</v>
+        <v>-1</v>
       </c>
       <c r="E21" t="n">
-        <v>3.92</v>
+        <v>6.6</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -23385,7 +23385,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.0857</v>
+        <v>0.0832</v>
       </c>
       <c r="C14" t="n">
         <v>3</v>
@@ -23397,7 +23397,7 @@
         <v>0.1703</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.5115</v>
+        <v>-0.5188</v>
       </c>
     </row>
   </sheetData>
@@ -35963,7 +35963,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -36310,6 +36310,31 @@
       </c>
       <c r="G13" t="n">
         <v>372.11</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="C14" t="n">
+        <v>428.38</v>
+      </c>
+      <c r="D14" t="n">
+        <v>4</v>
+      </c>
+      <c r="E14" t="n">
+        <v>354.78</v>
+      </c>
+      <c r="F14" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="G14" t="n">
+        <v>351.64</v>
       </c>
     </row>
   </sheetData>
@@ -37434,7 +37459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -37696,6 +37721,25 @@
         <v>0.371</v>
       </c>
       <c r="E13" t="n">
+        <v>0.72</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>15.511</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.574</v>
+      </c>
+      <c r="D14" t="n">
+        <v>-0.075</v>
+      </c>
+      <c r="E14" t="n">
         <v>0.72</v>
       </c>
     </row>
@@ -43957,7 +44001,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -44241,6 +44285,27 @@
         <v>5.4303</v>
       </c>
       <c r="E13" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>100</v>
+      </c>
+      <c r="C14" t="n">
+        <v>2.3191</v>
+      </c>
+      <c r="D14" t="n">
+        <v>5.4495</v>
+      </c>
+      <c r="E14" t="inlineStr">
         <is>
           <t>True</t>
         </is>
@@ -46078,7 +46143,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>eurostat/confiance_industrielle/DE.csv</t>
+          <t>fred/BOGMBASE.csv</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -46096,7 +46161,7 @@
         <v>279</v>
       </c>
       <c r="F63" t="n">
-        <v>560</v>
+        <v>812</v>
       </c>
       <c r="G63" t="inlineStr">
         <is>
@@ -46107,7 +46172,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>eurostat/confiance_industrielle/EA21.csv</t>
+          <t>fred/CFNAI.csv</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -46125,7 +46190,7 @@
         <v>279</v>
       </c>
       <c r="F64" t="n">
-        <v>560</v>
+        <v>714</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
@@ -46136,7 +46201,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>eurostat/confiance_industrielle/ES.csv</t>
+          <t>fred/CPIAUCSL.csv</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -46154,7 +46219,7 @@
         <v>279</v>
       </c>
       <c r="F65" t="n">
-        <v>473</v>
+        <v>956</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
@@ -46165,7 +46230,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>eurostat/confiance_industrielle/FR.csv</t>
+          <t>fred/HOUST.csv</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -46183,7 +46248,7 @@
         <v>279</v>
       </c>
       <c r="F66" t="n">
-        <v>499</v>
+        <v>812</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
@@ -46194,7 +46259,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>eurostat/confiance_industrielle/IT.csv</t>
+          <t>fred/INDPRO.csv</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -46212,7 +46277,7 @@
         <v>279</v>
       </c>
       <c r="F67" t="n">
-        <v>559</v>
+        <v>1292</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
@@ -46223,7 +46288,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>fred/BOGMBASE.csv</t>
+          <t>fred/IR3TIB01CHM156N.csv</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -46241,7 +46306,7 @@
         <v>279</v>
       </c>
       <c r="F68" t="n">
-        <v>812</v>
+        <v>632</v>
       </c>
       <c r="G68" t="inlineStr">
         <is>
@@ -46252,7 +46317,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>fred/CFNAI.csv</t>
+          <t>fred/IR3TIB01NZM156N.csv</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -46270,7 +46335,7 @@
         <v>279</v>
       </c>
       <c r="F69" t="n">
-        <v>714</v>
+        <v>633</v>
       </c>
       <c r="G69" t="inlineStr">
         <is>
@@ -46281,7 +46346,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>fred/CPIAUCSL.csv</t>
+          <t>fred/IR3TIB01SEM156N.csv</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -46299,7 +46364,7 @@
         <v>279</v>
       </c>
       <c r="F70" t="n">
-        <v>956</v>
+        <v>536</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
@@ -46310,7 +46375,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>fred/HOUST.csv</t>
+          <t>fred/IRLTLT01CAM156N.csv</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -46328,7 +46393,7 @@
         <v>279</v>
       </c>
       <c r="F71" t="n">
-        <v>812</v>
+        <v>860</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
@@ -46339,7 +46404,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>fred/INDPRO.csv</t>
+          <t>fred/IRLTLT01DEM156N.csv</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -46357,7 +46422,7 @@
         <v>279</v>
       </c>
       <c r="F72" t="n">
-        <v>1292</v>
+        <v>844</v>
       </c>
       <c r="G72" t="inlineStr">
         <is>
@@ -46368,7 +46433,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>fred/IR3TIB01CHM156N.csv</t>
+          <t>fred/IRLTLT01GBM156N.csv</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -46386,7 +46451,7 @@
         <v>279</v>
       </c>
       <c r="F73" t="n">
-        <v>632</v>
+        <v>800</v>
       </c>
       <c r="G73" t="inlineStr">
         <is>
@@ -46397,7 +46462,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>fred/IR3TIB01NZM156N.csv</t>
+          <t>fred/IRLTLT01JPM156N.csv</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -46415,7 +46480,7 @@
         <v>279</v>
       </c>
       <c r="F74" t="n">
-        <v>633</v>
+        <v>452</v>
       </c>
       <c r="G74" t="inlineStr">
         <is>
@@ -46426,7 +46491,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>fred/IR3TIB01SEM156N.csv</t>
+          <t>fred/IRLTLT01KRM156N.csv</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -46444,7 +46509,7 @@
         <v>279</v>
       </c>
       <c r="F75" t="n">
-        <v>536</v>
+        <v>311</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
@@ -46455,7 +46520,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>fred/IRLTLT01CAM156N.csv</t>
+          <t>fred/IRSTCI01AUM156N.csv</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -46473,7 +46538,7 @@
         <v>279</v>
       </c>
       <c r="F76" t="n">
-        <v>860</v>
+        <v>433</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
@@ -46484,7 +46549,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>fred/IRLTLT01DEM156N.csv</t>
+          <t>fred/IRSTCI01CAM156N.csv</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -46502,7 +46567,7 @@
         <v>279</v>
       </c>
       <c r="F77" t="n">
-        <v>844</v>
+        <v>620</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -46513,7 +46578,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>fred/IRLTLT01GBM156N.csv</t>
+          <t>fred/IRSTCI01JPM156N.csv</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -46531,7 +46596,7 @@
         <v>279</v>
       </c>
       <c r="F78" t="n">
-        <v>800</v>
+        <v>494</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -46542,7 +46607,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>fred/IRLTLT01JPM156N.csv</t>
+          <t>fred/IRSTCI01KRM156N.csv</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -46560,7 +46625,7 @@
         <v>279</v>
       </c>
       <c r="F79" t="n">
-        <v>452</v>
+        <v>428</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -46571,7 +46636,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>fred/IRLTLT01KRM156N.csv</t>
+          <t>fred/IRSTCI01NOM156N.csv</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -46589,7 +46654,7 @@
         <v>279</v>
       </c>
       <c r="F80" t="n">
-        <v>311</v>
+        <v>536</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -46600,7 +46665,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>fred/IRSTCI01AUM156N.csv</t>
+          <t>fred/JPNASSETS.csv</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -46618,7 +46683,7 @@
         <v>279</v>
       </c>
       <c r="F81" t="n">
-        <v>433</v>
+        <v>341</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
@@ -46629,7 +46694,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>fred/IRSTCI01CAM156N.csv</t>
+          <t>fred/LRHUTTTTCAM156S.csv</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -46647,7 +46712,7 @@
         <v>279</v>
       </c>
       <c r="F82" t="n">
-        <v>620</v>
+        <v>860</v>
       </c>
       <c r="G82" t="inlineStr">
         <is>
@@ -46658,7 +46723,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>fred/IRSTCI01JPM156N.csv</t>
+          <t>fred/MTSDS133FMS.csv</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -46676,7 +46741,7 @@
         <v>279</v>
       </c>
       <c r="F83" t="n">
-        <v>494</v>
+        <v>551</v>
       </c>
       <c r="G83" t="inlineStr">
         <is>
@@ -46687,7 +46752,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>fred/IRSTCI01KRM156N.csv</t>
+          <t>fred/PERMIT.csv</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -46705,7 +46770,7 @@
         <v>279</v>
       </c>
       <c r="F84" t="n">
-        <v>428</v>
+        <v>800</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
@@ -46716,7 +46781,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>fred/IRSTCI01NOM156N.csv</t>
+          <t>fred/RSAFS.csv</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -46734,7 +46799,7 @@
         <v>279</v>
       </c>
       <c r="F85" t="n">
-        <v>536</v>
+        <v>416</v>
       </c>
       <c r="G85" t="inlineStr">
         <is>
@@ -46745,7 +46810,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>fred/JPNASSETS.csv</t>
+          <t>fred/TOTRESNS.csv</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -46763,7 +46828,7 @@
         <v>279</v>
       </c>
       <c r="F86" t="n">
-        <v>341</v>
+        <v>812</v>
       </c>
       <c r="G86" t="inlineStr">
         <is>
@@ -46774,7 +46839,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>fred/LRHUTTTTCAM156S.csv</t>
+          <t>fred/TRESEGUSM052N.csv</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -46792,7 +46857,7 @@
         <v>279</v>
       </c>
       <c r="F87" t="n">
-        <v>860</v>
+        <v>909</v>
       </c>
       <c r="G87" t="inlineStr">
         <is>
@@ -46803,7 +46868,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>fred/MTSDS133FMS.csv</t>
+          <t>fred/UMCSENT.csv</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -46821,7 +46886,7 @@
         <v>279</v>
       </c>
       <c r="F88" t="n">
-        <v>551</v>
+        <v>886</v>
       </c>
       <c r="G88" t="inlineStr">
         <is>
@@ -46832,7 +46897,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>fred/PERMIT.csv</t>
+          <t>fred/UNRATE.csv</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -46850,7 +46915,7 @@
         <v>279</v>
       </c>
       <c r="F89" t="n">
-        <v>800</v>
+        <v>944</v>
       </c>
       <c r="G89" t="inlineStr">
         <is>
@@ -46861,25 +46926,25 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>fred/RSAFS.csv</t>
+          <t>bis/taux_directeurs/KR.csv</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>59</v>
+        <v>32</v>
       </c>
       <c r="D90" t="n">
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="E90" t="n">
-        <v>279</v>
+        <v>70</v>
       </c>
       <c r="F90" t="n">
-        <v>416</v>
+        <v>6815</v>
       </c>
       <c r="G90" t="inlineStr">
         <is>
@@ -46890,25 +46955,25 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>fred/TOTRESNS.csv</t>
+          <t>souverains/JAPON_10A.csv</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>59</v>
+        <v>29</v>
       </c>
       <c r="D91" t="n">
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="E91" t="n">
-        <v>279</v>
+        <v>90</v>
       </c>
       <c r="F91" t="n">
-        <v>812</v>
+        <v>9929</v>
       </c>
       <c r="G91" t="inlineStr">
         <is>
@@ -46919,25 +46984,25 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>fred/TRESEGUSM052N.csv</t>
+          <t>souverains/JAPON_2A.csv</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>59</v>
+        <v>29</v>
       </c>
       <c r="D92" t="n">
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="E92" t="n">
-        <v>279</v>
+        <v>90</v>
       </c>
       <c r="F92" t="n">
-        <v>909</v>
+        <v>12929</v>
       </c>
       <c r="G92" t="inlineStr">
         <is>
@@ -46948,25 +47013,25 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>fred/UMCSENT.csv</t>
+          <t>souverains/JAPON_30A.csv</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>59</v>
+        <v>29</v>
       </c>
       <c r="D93" t="n">
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="E93" t="n">
-        <v>279</v>
+        <v>90</v>
       </c>
       <c r="F93" t="n">
-        <v>886</v>
+        <v>6613</v>
       </c>
       <c r="G93" t="inlineStr">
         <is>
@@ -46977,25 +47042,25 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>fred/UNRATE.csv</t>
+          <t>souverains/JAPON_5A.csv</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>59</v>
+        <v>29</v>
       </c>
       <c r="D94" t="n">
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="E94" t="n">
-        <v>279</v>
+        <v>90</v>
       </c>
       <c r="F94" t="n">
-        <v>944</v>
+        <v>13290</v>
       </c>
       <c r="G94" t="inlineStr">
         <is>
@@ -47006,25 +47071,25 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>bis/taux_directeurs/KR.csv</t>
+          <t>eurostat/confiance_industrielle/DE.csv</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="D95" t="n">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="E95" t="n">
-        <v>70</v>
+        <v>279</v>
       </c>
       <c r="F95" t="n">
-        <v>6815</v>
+        <v>561</v>
       </c>
       <c r="G95" t="inlineStr">
         <is>
@@ -47035,25 +47100,25 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>souverains/JAPON_10A.csv</t>
+          <t>eurostat/confiance_industrielle/EA21.csv</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D96" t="n">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="E96" t="n">
-        <v>90</v>
+        <v>279</v>
       </c>
       <c r="F96" t="n">
-        <v>9929</v>
+        <v>561</v>
       </c>
       <c r="G96" t="inlineStr">
         <is>
@@ -47064,25 +47129,25 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>souverains/JAPON_2A.csv</t>
+          <t>eurostat/confiance_industrielle/ES.csv</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D97" t="n">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="E97" t="n">
-        <v>90</v>
+        <v>279</v>
       </c>
       <c r="F97" t="n">
-        <v>12929</v>
+        <v>474</v>
       </c>
       <c r="G97" t="inlineStr">
         <is>
@@ -47093,25 +47158,25 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>souverains/JAPON_30A.csv</t>
+          <t>eurostat/confiance_industrielle/FR.csv</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D98" t="n">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="E98" t="n">
-        <v>90</v>
+        <v>279</v>
       </c>
       <c r="F98" t="n">
-        <v>6613</v>
+        <v>500</v>
       </c>
       <c r="G98" t="inlineStr">
         <is>
@@ -47122,25 +47187,25 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>souverains/JAPON_5A.csv</t>
+          <t>eurostat/confiance_industrielle/IT.csv</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D99" t="n">
-        <v>1</v>
+        <v>31</v>
       </c>
       <c r="E99" t="n">
-        <v>90</v>
+        <v>279</v>
       </c>
       <c r="F99" t="n">
-        <v>13290</v>
+        <v>560</v>
       </c>
       <c r="G99" t="inlineStr">
         <is>
@@ -49703,16 +49768,16 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>souverains/UK_10A.csv</t>
+          <t>fred/BAMLC0A0CM.csv</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C188" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D188" t="n">
         <v>1</v>
@@ -49721,7 +49786,7 @@
         <v>42</v>
       </c>
       <c r="F188" t="n">
-        <v>9283</v>
+        <v>793</v>
       </c>
       <c r="G188" t="inlineStr">
         <is>
@@ -49732,16 +49797,16 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>souverains/UK_20A.csv</t>
+          <t>fred/BAMLC0A0CMEY.csv</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C189" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D189" t="n">
         <v>1</v>
@@ -49750,7 +49815,7 @@
         <v>42</v>
       </c>
       <c r="F189" t="n">
-        <v>6754</v>
+        <v>793</v>
       </c>
       <c r="G189" t="inlineStr">
         <is>
@@ -49761,16 +49826,16 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>souverains/UK_5A.csv</t>
+          <t>fred/BAMLEMCBPIOAS.csv</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C190" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D190" t="n">
         <v>1</v>
@@ -49779,7 +49844,7 @@
         <v>42</v>
       </c>
       <c r="F190" t="n">
-        <v>8291</v>
+        <v>793</v>
       </c>
       <c r="G190" t="inlineStr">
         <is>
@@ -49790,7 +49855,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>fred/BAMLC0A0CM.csv</t>
+          <t>fred/BAMLEMFSFCRPIOAS.csv</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -49819,7 +49884,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>fred/BAMLC0A0CMEY.csv</t>
+          <t>fred/BAMLEMHBHYCRPIOAS.csv</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -49848,7 +49913,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>fred/BAMLEMCBPIOAS.csv</t>
+          <t>fred/BAMLEMPBPUBSICRPIOAS.csv</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -49877,7 +49942,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>fred/BAMLEMFSFCRPIOAS.csv</t>
+          <t>fred/BAMLH0A0HYM2.csv</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -49906,7 +49971,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>fred/BAMLEMHBHYCRPIOAS.csv</t>
+          <t>fred/BAMLHE00EHYIEY.csv</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -49935,7 +50000,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>fred/BAMLEMPBPUBSICRPIOAS.csv</t>
+          <t>fred/BAMLHE00EHYIOAS.csv</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -49964,7 +50029,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>fred/BAMLH0A0HYM2.csv</t>
+          <t>fred/DFF.csv</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -49982,7 +50047,7 @@
         <v>42</v>
       </c>
       <c r="F197" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G197" t="inlineStr">
         <is>
@@ -49993,7 +50058,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>fred/BAMLHE00EHYIEY.csv</t>
+          <t>fred/DFII10.csv</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -50011,7 +50076,7 @@
         <v>42</v>
       </c>
       <c r="F198" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G198" t="inlineStr">
         <is>
@@ -50022,7 +50087,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>fred/BAMLHE00EHYIOAS.csv</t>
+          <t>fred/DFII5.csv</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -50040,7 +50105,7 @@
         <v>42</v>
       </c>
       <c r="F199" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G199" t="inlineStr">
         <is>
@@ -50051,7 +50116,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>fred/DFF.csv</t>
+          <t>fred/DGS1.csv</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -50080,7 +50145,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>fred/DFII10.csv</t>
+          <t>fred/DGS10.csv</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -50109,7 +50174,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>fred/DFII5.csv</t>
+          <t>fred/DGS1MO.csv</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -50138,7 +50203,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>fred/DGS1.csv</t>
+          <t>fred/DGS2.csv</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -50167,7 +50232,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>fred/DGS10.csv</t>
+          <t>fred/DGS30.csv</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
@@ -50196,7 +50261,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>fred/DGS1MO.csv</t>
+          <t>fred/DGS3MO.csv</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -50225,7 +50290,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>fred/DGS2.csv</t>
+          <t>fred/DGS5.csv</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -50254,7 +50319,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>fred/DGS30.csv</t>
+          <t>fred/DGS6MO.csv</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -50283,7 +50348,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>fred/DGS3MO.csv</t>
+          <t>souverains/CANADA_10A.csv</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -50301,7 +50366,7 @@
         <v>42</v>
       </c>
       <c r="F208" t="n">
-        <v>3000</v>
+        <v>6436</v>
       </c>
       <c r="G208" t="inlineStr">
         <is>
@@ -50312,7 +50377,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>fred/DGS5.csv</t>
+          <t>souverains/CANADA_2A.csv</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -50330,7 +50395,7 @@
         <v>42</v>
       </c>
       <c r="F209" t="n">
-        <v>3000</v>
+        <v>6435</v>
       </c>
       <c r="G209" t="inlineStr">
         <is>
@@ -50341,7 +50406,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>fred/DGS6MO.csv</t>
+          <t>souverains/CANADA_5A.csv</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -50359,7 +50424,7 @@
         <v>42</v>
       </c>
       <c r="F210" t="n">
-        <v>3000</v>
+        <v>6435</v>
       </c>
       <c r="G210" t="inlineStr">
         <is>
@@ -50370,7 +50435,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>souverains/CANADA_10A.csv</t>
+          <t>souverains/CANADA_LONG.csv</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
@@ -50388,7 +50453,7 @@
         <v>42</v>
       </c>
       <c r="F211" t="n">
-        <v>6436</v>
+        <v>6435</v>
       </c>
       <c r="G211" t="inlineStr">
         <is>
@@ -50399,7 +50464,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>souverains/CANADA_2A.csv</t>
+          <t>souverains/UK_10A.csv</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -50417,7 +50482,7 @@
         <v>42</v>
       </c>
       <c r="F212" t="n">
-        <v>6435</v>
+        <v>9284</v>
       </c>
       <c r="G212" t="inlineStr">
         <is>
@@ -50428,7 +50493,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>souverains/CANADA_5A.csv</t>
+          <t>souverains/UK_20A.csv</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -50446,7 +50511,7 @@
         <v>42</v>
       </c>
       <c r="F213" t="n">
-        <v>6435</v>
+        <v>6755</v>
       </c>
       <c r="G213" t="inlineStr">
         <is>
@@ -50457,7 +50522,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>souverains/CANADA_LONG.csv</t>
+          <t>souverains/UK_5A.csv</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -50475,7 +50540,7 @@
         <v>42</v>
       </c>
       <c r="F214" t="n">
-        <v>6435</v>
+        <v>8292</v>
       </c>
       <c r="G214" t="inlineStr">
         <is>
@@ -50892,7 +50957,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>marches/indices/DAX.csv</t>
+          <t>marches/volatilite/GVZ.csv</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -50910,7 +50975,7 @@
         <v>42</v>
       </c>
       <c r="F229" t="n">
-        <v>3802</v>
+        <v>3770</v>
       </c>
       <c r="G229" t="inlineStr">
         <is>
@@ -50921,7 +50986,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>marches/indices/EUROSTOXX50.csv</t>
+          <t>marches/volatilite/MOVE.csv</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -50939,7 +51004,7 @@
         <v>42</v>
       </c>
       <c r="F230" t="n">
-        <v>3759</v>
+        <v>3689</v>
       </c>
       <c r="G230" t="inlineStr">
         <is>
@@ -50950,7 +51015,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>marches/indices/FTSE100.csv</t>
+          <t>marches/volatilite/OVX.csv</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -50968,7 +51033,7 @@
         <v>42</v>
       </c>
       <c r="F231" t="n">
-        <v>3788</v>
+        <v>3770</v>
       </c>
       <c r="G231" t="inlineStr">
         <is>
@@ -50979,7 +51044,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>marches/volatilite/GVZ.csv</t>
+          <t>marches/volatilite/VVIX.csv</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -50997,7 +51062,7 @@
         <v>42</v>
       </c>
       <c r="F232" t="n">
-        <v>3770</v>
+        <v>3762</v>
       </c>
       <c r="G232" t="inlineStr">
         <is>
@@ -51008,7 +51073,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>marches/volatilite/MOVE.csv</t>
+          <t>marches/volatilite/VXN.csv</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -51026,7 +51091,7 @@
         <v>42</v>
       </c>
       <c r="F233" t="n">
-        <v>3689</v>
+        <v>3770</v>
       </c>
       <c r="G233" t="inlineStr">
         <is>
@@ -51037,7 +51102,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>marches/volatilite/OVX.csv</t>
+          <t>souverains/SUEDE_10A.csv</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -51055,7 +51120,7 @@
         <v>42</v>
       </c>
       <c r="F234" t="n">
-        <v>3770</v>
+        <v>9203</v>
       </c>
       <c r="G234" t="inlineStr">
         <is>
@@ -51066,7 +51131,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>marches/volatilite/VVIX.csv</t>
+          <t>souverains/SUEDE_2A.csv</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -51084,7 +51149,7 @@
         <v>42</v>
       </c>
       <c r="F235" t="n">
-        <v>3762</v>
+        <v>9203</v>
       </c>
       <c r="G235" t="inlineStr">
         <is>
@@ -51095,7 +51160,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>marches/volatilite/VXN.csv</t>
+          <t>souverains/SUEDE_5A.csv</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -51113,7 +51178,7 @@
         <v>42</v>
       </c>
       <c r="F236" t="n">
-        <v>3770</v>
+        <v>9205</v>
       </c>
       <c r="G236" t="inlineStr">
         <is>
@@ -51124,7 +51189,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_10A.csv</t>
+          <t>yfinance/SP500.csv</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
@@ -51142,7 +51207,7 @@
         <v>42</v>
       </c>
       <c r="F237" t="n">
-        <v>9203</v>
+        <v>7546</v>
       </c>
       <c r="G237" t="inlineStr">
         <is>
@@ -51153,7 +51218,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_2A.csv</t>
+          <t>yfinance/XLB.csv</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
@@ -51171,7 +51236,7 @@
         <v>42</v>
       </c>
       <c r="F238" t="n">
-        <v>9203</v>
+        <v>500</v>
       </c>
       <c r="G238" t="inlineStr">
         <is>
@@ -51182,7 +51247,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_5A.csv</t>
+          <t>yfinance/XLE.csv</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
@@ -51200,7 +51265,7 @@
         <v>42</v>
       </c>
       <c r="F239" t="n">
-        <v>9205</v>
+        <v>500</v>
       </c>
       <c r="G239" t="inlineStr">
         <is>
@@ -51211,7 +51276,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>yfinance/SP500.csv</t>
+          <t>yfinance/XLF.csv</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
@@ -51229,7 +51294,7 @@
         <v>42</v>
       </c>
       <c r="F240" t="n">
-        <v>7546</v>
+        <v>500</v>
       </c>
       <c r="G240" t="inlineStr">
         <is>
@@ -51240,7 +51305,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>yfinance/VIX.csv</t>
+          <t>yfinance/XLI.csv</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
@@ -51258,7 +51323,7 @@
         <v>42</v>
       </c>
       <c r="F241" t="n">
-        <v>7548</v>
+        <v>500</v>
       </c>
       <c r="G241" t="inlineStr">
         <is>
@@ -51269,7 +51334,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>yfinance/XLB.csv</t>
+          <t>yfinance/XLK.csv</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
@@ -51298,7 +51363,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>yfinance/XLE.csv</t>
+          <t>yfinance/XLP.csv</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
@@ -51327,7 +51392,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>yfinance/XLF.csv</t>
+          <t>yfinance/XLRE.csv</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -51356,7 +51421,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>yfinance/XLI.csv</t>
+          <t>yfinance/XLU.csv</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -51385,7 +51450,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>yfinance/XLK.csv</t>
+          <t>yfinance/XLV.csv</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -51414,7 +51479,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>yfinance/XLP.csv</t>
+          <t>yfinance/XLY.csv</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
@@ -51443,16 +51508,16 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>yfinance/XLRE.csv</t>
+          <t>marches/fx/AUDJPY.csv</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C248" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D248" t="n">
         <v>1</v>
@@ -51461,7 +51526,7 @@
         <v>42</v>
       </c>
       <c r="F248" t="n">
-        <v>500</v>
+        <v>3908</v>
       </c>
       <c r="G248" t="inlineStr">
         <is>
@@ -51472,16 +51537,16 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>yfinance/XLU.csv</t>
+          <t>marches/fx/AUDUSD.csv</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C249" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D249" t="n">
         <v>1</v>
@@ -51490,7 +51555,7 @@
         <v>42</v>
       </c>
       <c r="F249" t="n">
-        <v>500</v>
+        <v>3904</v>
       </c>
       <c r="G249" t="inlineStr">
         <is>
@@ -51501,16 +51566,16 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>yfinance/XLV.csv</t>
+          <t>marches/fx/DXY.csv</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C250" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D250" t="n">
         <v>1</v>
@@ -51519,7 +51584,7 @@
         <v>42</v>
       </c>
       <c r="F250" t="n">
-        <v>500</v>
+        <v>3772</v>
       </c>
       <c r="G250" t="inlineStr">
         <is>
@@ -51530,16 +51595,16 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>yfinance/XLY.csv</t>
+          <t>marches/fx/EURCHF.csv</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C251" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D251" t="n">
         <v>1</v>
@@ -51548,7 +51613,7 @@
         <v>42</v>
       </c>
       <c r="F251" t="n">
-        <v>500</v>
+        <v>3905</v>
       </c>
       <c r="G251" t="inlineStr">
         <is>
@@ -51559,7 +51624,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>marches/fx/AUDJPY.csv</t>
+          <t>marches/fx/EURGBP.csv</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -51577,7 +51642,7 @@
         <v>42</v>
       </c>
       <c r="F252" t="n">
-        <v>3908</v>
+        <v>3907</v>
       </c>
       <c r="G252" t="inlineStr">
         <is>
@@ -51588,7 +51653,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>marches/fx/AUDUSD.csv</t>
+          <t>marches/fx/EURJPY.csv</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -51606,7 +51671,7 @@
         <v>42</v>
       </c>
       <c r="F253" t="n">
-        <v>3904</v>
+        <v>3907</v>
       </c>
       <c r="G253" t="inlineStr">
         <is>
@@ -51617,7 +51682,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>marches/fx/DXY.csv</t>
+          <t>marches/fx/EURUSD.csv</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
@@ -51635,7 +51700,7 @@
         <v>42</v>
       </c>
       <c r="F254" t="n">
-        <v>3772</v>
+        <v>3904</v>
       </c>
       <c r="G254" t="inlineStr">
         <is>
@@ -51646,7 +51711,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>marches/fx/EURCHF.csv</t>
+          <t>marches/fx/GBPUSD.csv</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
@@ -51675,7 +51740,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>marches/fx/EURGBP.csv</t>
+          <t>marches/fx/NZDUSD.csv</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
@@ -51693,7 +51758,7 @@
         <v>42</v>
       </c>
       <c r="F256" t="n">
-        <v>3907</v>
+        <v>3905</v>
       </c>
       <c r="G256" t="inlineStr">
         <is>
@@ -51704,7 +51769,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>marches/fx/EURJPY.csv</t>
+          <t>marches/fx/USDCAD.csv</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
@@ -51722,7 +51787,7 @@
         <v>42</v>
       </c>
       <c r="F257" t="n">
-        <v>3907</v>
+        <v>3904</v>
       </c>
       <c r="G257" t="inlineStr">
         <is>
@@ -51733,7 +51798,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>marches/fx/EURUSD.csv</t>
+          <t>marches/fx/USDCHF.csv</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
@@ -51751,7 +51816,7 @@
         <v>42</v>
       </c>
       <c r="F258" t="n">
-        <v>3904</v>
+        <v>3902</v>
       </c>
       <c r="G258" t="inlineStr">
         <is>
@@ -51762,7 +51827,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>marches/fx/GBPUSD.csv</t>
+          <t>marches/fx/USDCNY.csv</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
@@ -51780,7 +51845,7 @@
         <v>42</v>
       </c>
       <c r="F259" t="n">
-        <v>3905</v>
+        <v>3904</v>
       </c>
       <c r="G259" t="inlineStr">
         <is>
@@ -51791,7 +51856,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>marches/fx/NZDUSD.csv</t>
+          <t>marches/fx/USDJPY.csv</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
@@ -51820,7 +51885,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>marches/fx/USDCAD.csv</t>
+          <t>marches/fx/USDKRW.csv</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
@@ -51849,7 +51914,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>marches/fx/USDCHF.csv</t>
+          <t>marches/fx/USDNOK.csv</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
@@ -51867,7 +51932,7 @@
         <v>42</v>
       </c>
       <c r="F262" t="n">
-        <v>3902</v>
+        <v>3905</v>
       </c>
       <c r="G262" t="inlineStr">
         <is>
@@ -51878,7 +51943,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>marches/fx/USDCNY.csv</t>
+          <t>marches/fx/USDSEK.csv</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
@@ -51896,7 +51961,7 @@
         <v>42</v>
       </c>
       <c r="F263" t="n">
-        <v>3904</v>
+        <v>3905</v>
       </c>
       <c r="G263" t="inlineStr">
         <is>
@@ -51907,7 +51972,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>marches/fx/USDJPY.csv</t>
+          <t>marches/indices/DAX.csv</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
@@ -51925,7 +51990,7 @@
         <v>42</v>
       </c>
       <c r="F264" t="n">
-        <v>3905</v>
+        <v>3802</v>
       </c>
       <c r="G264" t="inlineStr">
         <is>
@@ -51936,7 +52001,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>marches/fx/USDKRW.csv</t>
+          <t>marches/indices/EUROSTOXX50.csv</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
@@ -51954,7 +52019,7 @@
         <v>42</v>
       </c>
       <c r="F265" t="n">
-        <v>3904</v>
+        <v>3759</v>
       </c>
       <c r="G265" t="inlineStr">
         <is>
@@ -51965,7 +52030,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>marches/fx/USDNOK.csv</t>
+          <t>marches/indices/FTSE100.csv</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
@@ -51983,7 +52048,7 @@
         <v>42</v>
       </c>
       <c r="F266" t="n">
-        <v>3905</v>
+        <v>3788</v>
       </c>
       <c r="G266" t="inlineStr">
         <is>
@@ -51994,7 +52059,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>marches/fx/USDSEK.csv</t>
+          <t>marches/indices/HANGSENG.csv</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
@@ -52012,7 +52077,7 @@
         <v>42</v>
       </c>
       <c r="F267" t="n">
-        <v>3905</v>
+        <v>3689</v>
       </c>
       <c r="G267" t="inlineStr">
         <is>
@@ -52023,7 +52088,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>marches/indices/HANGSENG.csv</t>
+          <t>marches/indices/KOSPI.csv</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
@@ -52041,7 +52106,7 @@
         <v>42</v>
       </c>
       <c r="F268" t="n">
-        <v>3689</v>
+        <v>3681</v>
       </c>
       <c r="G268" t="inlineStr">
         <is>
@@ -52052,7 +52117,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>marches/indices/KOSPI.csv</t>
+          <t>marches/indices/NIKKEI225.csv</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
@@ -52070,7 +52135,7 @@
         <v>42</v>
       </c>
       <c r="F269" t="n">
-        <v>3681</v>
+        <v>3667</v>
       </c>
       <c r="G269" t="inlineStr">
         <is>
@@ -52081,7 +52146,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>marches/indices/NIKKEI225.csv</t>
+          <t>marches/matieres/BRENT.csv</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
@@ -52099,7 +52164,7 @@
         <v>42</v>
       </c>
       <c r="F270" t="n">
-        <v>3667</v>
+        <v>3751</v>
       </c>
       <c r="G270" t="inlineStr">
         <is>
@@ -52110,7 +52175,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>marches/matieres/BRENT.csv</t>
+          <t>marches/matieres/CUIVRE.csv</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
@@ -52128,7 +52193,7 @@
         <v>42</v>
       </c>
       <c r="F271" t="n">
-        <v>3751</v>
+        <v>3771</v>
       </c>
       <c r="G271" t="inlineStr">
         <is>
@@ -52139,7 +52204,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>marches/matieres/CUIVRE.csv</t>
+          <t>marches/matieres/GAZ_HENRY_HUB.csv</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
@@ -52157,7 +52222,7 @@
         <v>42</v>
       </c>
       <c r="F272" t="n">
-        <v>3771</v>
+        <v>3772</v>
       </c>
       <c r="G272" t="inlineStr">
         <is>
@@ -52168,7 +52233,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>marches/matieres/GAZ_HENRY_HUB.csv</t>
+          <t>marches/matieres/OR.csv</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
@@ -52186,7 +52251,7 @@
         <v>42</v>
       </c>
       <c r="F273" t="n">
-        <v>3772</v>
+        <v>3770</v>
       </c>
       <c r="G273" t="inlineStr">
         <is>
@@ -52197,7 +52262,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>marches/matieres/OR.csv</t>
+          <t>marches/matieres/WTI.csv</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
@@ -52226,7 +52291,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>marches/matieres/WTI.csv</t>
+          <t>marches/taux_futures/FED_FUNDS_FRONT.csv</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
@@ -52244,7 +52309,7 @@
         <v>42</v>
       </c>
       <c r="F275" t="n">
-        <v>3771</v>
+        <v>3772</v>
       </c>
       <c r="G275" t="inlineStr">
         <is>
@@ -52255,7 +52320,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>marches/taux_futures/FED_FUNDS_FRONT.csv</t>
+          <t>yfinance/VIX.csv</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
@@ -52273,7 +52338,7 @@
         <v>42</v>
       </c>
       <c r="F276" t="n">
-        <v>3772</v>
+        <v>7549</v>
       </c>
       <c r="G276" t="inlineStr">
         <is>
@@ -53806,13 +53871,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>6804.68</v>
+        <v>6870.81</v>
       </c>
       <c r="D2" t="n">
-        <v>-19.72</v>
+        <v>-18.94</v>
       </c>
       <c r="E2" t="n">
-        <v>98.31999999999999</v>
+        <v>100.24</v>
       </c>
     </row>
     <row r="3">
@@ -53827,13 +53892,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>64842.17</v>
+        <v>65481.27</v>
       </c>
       <c r="D3" t="n">
-        <v>-7.45</v>
+        <v>-6.54</v>
       </c>
       <c r="E3" t="n">
-        <v>43.95</v>
+        <v>45.37</v>
       </c>
     </row>
     <row r="4">
@@ -53865,17 +53930,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>10684.9</v>
+        <v>10713.6</v>
       </c>
       <c r="D5" t="n">
-        <v>1.91</v>
+        <v>2.06</v>
       </c>
       <c r="E5" t="n">
-        <v>15.08</v>
+        <v>15.2</v>
       </c>
     </row>
     <row r="6">
@@ -53886,17 +53951,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>6301.28</v>
+        <v>6342.69</v>
       </c>
       <c r="D6" t="n">
-        <v>1.12</v>
+        <v>0.23</v>
       </c>
       <c r="E6" t="n">
-        <v>14.57</v>
+        <v>15.18</v>
       </c>
     </row>
     <row r="7">
@@ -53907,17 +53972,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>25374.42</v>
+        <v>25450.15</v>
       </c>
       <c r="D7" t="n">
-        <v>3.04</v>
+        <v>1.82</v>
       </c>
       <c r="E7" t="n">
-        <v>6.89</v>
+        <v>7.18</v>
       </c>
     </row>
     <row r="8">
@@ -53932,13 +53997,13 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>24504.65</v>
+        <v>24523.57</v>
       </c>
       <c r="D8" t="n">
-        <v>7.1</v>
+        <v>7.18</v>
       </c>
       <c r="E8" t="n">
-        <v>-7.96</v>
+        <v>-7.89</v>
       </c>
     </row>
   </sheetData>
@@ -54361,7 +54426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -54624,6 +54689,25 @@
       </c>
       <c r="E13" t="n">
         <v>0.20517</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>16.01</v>
+      </c>
+      <c r="C14" t="n">
+        <v>15.995</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.625</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.20516</v>
       </c>
     </row>
   </sheetData>
@@ -56104,25 +56188,25 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.001591</v>
+        <v>0.001581</v>
       </c>
       <c r="C12" t="n">
-        <v>3.77</v>
+        <v>3.13</v>
       </c>
       <c r="D12" t="n">
-        <v>100.11</v>
+        <v>97.87</v>
       </c>
       <c r="E12" t="n">
-        <v>37.29</v>
+        <v>34.22</v>
       </c>
       <c r="F12" t="n">
-        <v>47.29</v>
+        <v>43.99</v>
       </c>
       <c r="G12" t="n">
-        <v>-4.64</v>
+        <v>-5.22</v>
       </c>
       <c r="H12" t="n">
-        <v>5.52</v>
+        <v>5.11</v>
       </c>
     </row>
   </sheetData>
@@ -60317,7 +60401,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -60622,6 +60706,28 @@
       </c>
       <c r="F13" t="n">
         <v>-4.131</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>16.01</v>
+      </c>
+      <c r="C14" t="n">
+        <v>20.2</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.02404</v>
+      </c>
+      <c r="E14" t="n">
+        <v>28.8</v>
+      </c>
+      <c r="F14" t="n">
+        <v>-4.19</v>
       </c>
     </row>
   </sheetData>
@@ -60920,26 +61026,26 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>4.924</v>
+        <v>4.916</v>
       </c>
       <c r="D5" t="n">
-        <v>5.361</v>
+        <v>5.384</v>
       </c>
       <c r="E5" t="n">
-        <v>0.437</v>
+        <v>0.468</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.098</v>
+        <v>-0.079</v>
       </c>
       <c r="G5" t="n">
-        <v>0.697</v>
+        <v>0.668</v>
       </c>
       <c r="H5" t="n">
-        <v>0.599</v>
+        <v>0.589</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -66985,10 +67091,10 @@
         <v>0.008800000000000001</v>
       </c>
       <c r="C14" t="n">
-        <v>0.06836</v>
+        <v>0.06808</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.03858</v>
+        <v>-0.03844</v>
       </c>
     </row>
   </sheetData>
@@ -79752,13 +79858,13 @@
         <v>12.9</v>
       </c>
       <c r="D4" t="n">
-        <v>5.36</v>
+        <v>5.38</v>
       </c>
       <c r="E4" t="n">
         <v>3.09</v>
       </c>
       <c r="F4" t="n">
-        <v>2.27</v>
+        <v>2.3</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-29T11:41Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-29 09:09 UTC</t>
+          <t>Genere le 2026-09-29 11:41 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-29 09:09 UTC</t>
+          <t>Rapport global — 2026-09-29 11:41 UTC</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>**Matieres premieres macro** — ratio cuivre/or stable -- pas de signal net sur la croissance (+3.1% sur 3 mois). Brent 97.9$ (+34.2% sur 3 mois, +44.0% sur 12 mois), gaz -5.2% sur 3 mois, ecart Brent-WTI +5.1$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-29)_</t>
+          <t>**Matieres premieres macro** — ratio cuivre/or stable -- pas de signal net sur la croissance (+3.1% sur 3 mois). Brent 96.9$ (+32.9% sur 3 mois, +42.5% sur 12 mois), gaz -5.5% sur 3 mois, ecart Brent-WTI +5.2$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -862,7 +862,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>**Conditions financieres** — indice conditions financieres=+0.083 (3 composantes: {'taux_directeur': 0.5982151864455719, 'courbe_inversee': 0.17031877422284264, 'vix': -0.5188320907186125}) -- conditions proches de la normale _(observation : 2026-09-25)_</t>
+          <t>**Conditions financieres** — indice conditions financieres=+0.077 (3 composantes: {'taux_directeur': 0.5982151864455719, 'courbe_inversee': 0.17031877422284264, 'vix': -0.5373811926967677}) -- conditions proches de la normale _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
@@ -1191,7 +1191,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>**Vol cross asset** — 6 mesures de volatilite : Petrole (OVX) 89e pct, Or (GVZ) 87e pct, Taux US (MOVE) 51e pct, Nasdaq (VXN) 48e pct, Vol de la vol (VVIX) 37e pct, Actions US (VIX) 32e pct -- stress LOCALISE sur Petrole (OVX), Or (GVZ) pendant que le reste ne l'est pas -- episode propre a cette classe d'actifs, pas une aversion au risque d'ensemble _(observation : 2026-09-29)_</t>
+          <t>**Vol cross asset** — 6 mesures de volatilite : Petrole (OVX) 89e pct, Or (GVZ) 87e pct, Taux US (MOVE) 51e pct, Nasdaq (VXN) 48e pct, Vol de la vol (VVIX) 37e pct, Actions US (VIX) 31e pct -- stress LOCALISE sur Petrole (OVX), Or (GVZ) pendant que le reste ne l'est pas -- episode propre a cette classe d'actifs, pas une aversion au risque d'ensemble _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1219,7 +1219,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>**Ornstein uhlenbeck vix** — VIX actuel=16.01, niveau moyen estime (mu)=20.20, demi-vie=28.8j, ecart actuel=-4.19 -- VIX actuel en-dessous de son niveau moyen de long terme _(observation : 2026-09-29)_</t>
+          <t>**Ornstein uhlenbeck vix** — VIX actuel=15.86, niveau moyen estime (mu)=20.20, demi-vie=28.8j, ecart actuel=-4.34 -- VIX actuel en-dessous de son niveau moyen de long terme _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1233,14 +1233,14 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>**Kalman niveau local** — VIX observe=16.01, filtre Kalman=15.99 (ecart-type=0.62), ratio signal/bruit=0.2052 -- le filtre lisse fortement le bruit, reagit lentement (ecart obs.-filtre=+0.02) _(observation : 2026-09-29)_</t>
+          <t>**Kalman niveau local** — VIX observe=15.86, filtre Kalman=15.87 (ecart-type=0.62), ratio signal/bruit=0.2052 -- le filtre lisse fortement le bruit, reagit lentement (ecart obs.-filtre=-0.01) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.3730169650835773 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.052364093738951525 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-28)_</t>
+          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.37301696508358795 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.05236409373895107 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1317,7 +1317,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>**Qualite regime macro** — instabilite taux=0.0088, instabilite VIX=0.0681 -- score qualite du regime=-0.0384 (plus haut = regime plus stable/previsible) _(observation : 2026-09-25)_</t>
+          <t>**Qualite regime macro** — instabilite taux=0.0088, instabilite VIX=0.0681 -- score qualite du regime=-0.0385 (plus haut = regime plus stable/previsible) _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1331,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>**Decomposition stl** — VIX : tendance=15.51, composante saisonniere (periode 5j)=+0.574, residu=-0.075 -- la saisonnalite explique 0.72% de la variance totale (negligeable) _(observation : 2026-09-29)_</t>
+          <t>**Decomposition stl** — VIX : tendance=15.47, composante saisonniere (periode 5j)=+0.516, residu=-0.124 -- la saisonnalite explique 0.72% de la variance totale (negligeable) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -2571,13 +2571,13 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>3.7305</v>
+        <v>3.73</v>
       </c>
       <c r="D51" t="n">
         <v>3.88</v>
       </c>
       <c r="E51" t="n">
-        <v>-0.149</v>
+        <v>-0.15</v>
       </c>
     </row>
     <row r="52">
@@ -4859,10 +4859,10 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>-0.1568</v>
+        <v>-0.159</v>
       </c>
       <c r="E64" t="n">
-        <v>0.9435</v>
+        <v>0.9432</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
@@ -8707,10 +8707,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>16.01</v>
+        <v>15.86</v>
       </c>
       <c r="D7" t="n">
-        <v>32</v>
+        <v>30.6</v>
       </c>
       <c r="E7" t="n">
         <v>1260</v>
@@ -20192,10 +20192,10 @@
         </is>
       </c>
       <c r="D129" t="n">
-        <v>-1.9784</v>
+        <v>-1.9798</v>
       </c>
       <c r="E129" t="n">
-        <v>0.5397999999999999</v>
+        <v>0.5391</v>
       </c>
       <c r="F129" t="inlineStr">
         <is>
@@ -20220,10 +20220,10 @@
         </is>
       </c>
       <c r="D130" t="n">
-        <v>-2.2116</v>
+        <v>-2.2119</v>
       </c>
       <c r="E130" t="n">
-        <v>0.4184</v>
+        <v>0.4182</v>
       </c>
       <c r="F130" t="inlineStr">
         <is>
@@ -23385,7 +23385,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.0832</v>
+        <v>0.0771</v>
       </c>
       <c r="C14" t="n">
         <v>3</v>
@@ -23397,7 +23397,7 @@
         <v>0.1703</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.5188</v>
+        <v>-0.5374</v>
       </c>
     </row>
   </sheetData>
@@ -36322,19 +36322,19 @@
         <v>2.2</v>
       </c>
       <c r="C14" t="n">
-        <v>428.38</v>
+        <v>428.16</v>
       </c>
       <c r="D14" t="n">
         <v>4</v>
       </c>
       <c r="E14" t="n">
-        <v>354.78</v>
+        <v>354.75</v>
       </c>
       <c r="F14" t="n">
         <v>5.4</v>
       </c>
       <c r="G14" t="n">
-        <v>351.64</v>
+        <v>351.49</v>
       </c>
     </row>
   </sheetData>
@@ -37731,13 +37731,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>15.511</v>
+        <v>15.469</v>
       </c>
       <c r="C14" t="n">
-        <v>0.574</v>
+        <v>0.516</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.075</v>
+        <v>-0.124</v>
       </c>
       <c r="E14" t="n">
         <v>0.72</v>
@@ -49710,7 +49710,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>fred/IUDSOIA.csv</t>
+          <t>fred/MORTGAGE30US.csv</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -49722,13 +49722,13 @@
         <v>5</v>
       </c>
       <c r="D186" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E186" t="n">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="F186" t="n">
-        <v>3000</v>
+        <v>2896</v>
       </c>
       <c r="G186" t="inlineStr">
         <is>
@@ -49739,25 +49739,25 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>fred/MORTGAGE30US.csv</t>
+          <t>fred/BAMLC0A0CM.csv</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C187" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D187" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E187" t="n">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="F187" t="n">
-        <v>2896</v>
+        <v>793</v>
       </c>
       <c r="G187" t="inlineStr">
         <is>
@@ -49768,7 +49768,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>fred/BAMLC0A0CM.csv</t>
+          <t>fred/BAMLC0A0CMEY.csv</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -49797,7 +49797,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>fred/BAMLC0A0CMEY.csv</t>
+          <t>fred/BAMLEMCBPIOAS.csv</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -49826,7 +49826,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>fred/BAMLEMCBPIOAS.csv</t>
+          <t>fred/BAMLEMFSFCRPIOAS.csv</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -49855,7 +49855,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>fred/BAMLEMFSFCRPIOAS.csv</t>
+          <t>fred/BAMLEMHBHYCRPIOAS.csv</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -49884,7 +49884,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>fred/BAMLEMHBHYCRPIOAS.csv</t>
+          <t>fred/BAMLEMPBPUBSICRPIOAS.csv</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -49913,7 +49913,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>fred/BAMLEMPBPUBSICRPIOAS.csv</t>
+          <t>fred/BAMLH0A0HYM2.csv</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -49942,7 +49942,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>fred/BAMLH0A0HYM2.csv</t>
+          <t>fred/BAMLHE00EHYIEY.csv</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -49971,7 +49971,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>fred/BAMLHE00EHYIEY.csv</t>
+          <t>fred/BAMLHE00EHYIOAS.csv</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -50000,7 +50000,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>fred/BAMLHE00EHYIOAS.csv</t>
+          <t>fred/DFF.csv</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -50018,7 +50018,7 @@
         <v>42</v>
       </c>
       <c r="F196" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G196" t="inlineStr">
         <is>
@@ -50029,7 +50029,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>fred/DFF.csv</t>
+          <t>fred/DFII10.csv</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -50058,7 +50058,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>fred/DFII10.csv</t>
+          <t>fred/DFII5.csv</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -50087,7 +50087,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>fred/DFII5.csv</t>
+          <t>fred/DGS1.csv</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -50116,7 +50116,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>fred/DGS1.csv</t>
+          <t>fred/DGS10.csv</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -50145,7 +50145,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>fred/DGS10.csv</t>
+          <t>fred/DGS1MO.csv</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -50174,7 +50174,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>fred/DGS1MO.csv</t>
+          <t>fred/DGS2.csv</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -50203,7 +50203,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>fred/DGS2.csv</t>
+          <t>fred/DGS30.csv</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -50232,7 +50232,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>fred/DGS30.csv</t>
+          <t>fred/DGS3MO.csv</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
@@ -50261,7 +50261,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>fred/DGS3MO.csv</t>
+          <t>fred/DGS5.csv</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -50290,7 +50290,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>fred/DGS5.csv</t>
+          <t>fred/DGS6MO.csv</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -50319,7 +50319,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>fred/DGS6MO.csv</t>
+          <t>fred/IUDSOIA.csv</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -50551,7 +50551,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
+          <t>tresor_us/dette_quotidienne.csv</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -50569,7 +50569,7 @@
         <v>42</v>
       </c>
       <c r="F215" t="n">
-        <v>5639</v>
+        <v>2000</v>
       </c>
       <c r="G215" t="inlineStr">
         <is>
@@ -50580,7 +50580,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
+          <t>tresor_us/solde_tresorerie.csv</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -50598,7 +50598,7 @@
         <v>42</v>
       </c>
       <c r="F216" t="n">
-        <v>5639</v>
+        <v>500</v>
       </c>
       <c r="G216" t="inlineStr">
         <is>
@@ -50609,16 +50609,16 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
+          <t>fred/ECBDFR.csv</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C217" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D217" t="n">
         <v>1</v>
@@ -50627,7 +50627,7 @@
         <v>42</v>
       </c>
       <c r="F217" t="n">
-        <v>5639</v>
+        <v>3000</v>
       </c>
       <c r="G217" t="inlineStr">
         <is>
@@ -50638,16 +50638,16 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
+          <t>fred/RRPONTSYD.csv</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C218" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D218" t="n">
         <v>1</v>
@@ -50656,7 +50656,7 @@
         <v>42</v>
       </c>
       <c r="F218" t="n">
-        <v>5639</v>
+        <v>3000</v>
       </c>
       <c r="G218" t="inlineStr">
         <is>
@@ -50667,16 +50667,16 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
+          <t>fred/T10YIE.csv</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C219" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D219" t="n">
         <v>1</v>
@@ -50685,7 +50685,7 @@
         <v>42</v>
       </c>
       <c r="F219" t="n">
-        <v>5639</v>
+        <v>3000</v>
       </c>
       <c r="G219" t="inlineStr">
         <is>
@@ -50696,16 +50696,16 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
+          <t>marches/volatilite/GVZ.csv</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C220" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D220" t="n">
         <v>1</v>
@@ -50714,7 +50714,7 @@
         <v>42</v>
       </c>
       <c r="F220" t="n">
-        <v>5639</v>
+        <v>3770</v>
       </c>
       <c r="G220" t="inlineStr">
         <is>
@@ -50725,16 +50725,16 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
+          <t>marches/volatilite/MOVE.csv</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C221" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D221" t="n">
         <v>1</v>
@@ -50743,7 +50743,7 @@
         <v>42</v>
       </c>
       <c r="F221" t="n">
-        <v>5639</v>
+        <v>3689</v>
       </c>
       <c r="G221" t="inlineStr">
         <is>
@@ -50754,16 +50754,16 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
+          <t>marches/volatilite/OVX.csv</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C222" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D222" t="n">
         <v>1</v>
@@ -50772,7 +50772,7 @@
         <v>42</v>
       </c>
       <c r="F222" t="n">
-        <v>5639</v>
+        <v>3770</v>
       </c>
       <c r="G222" t="inlineStr">
         <is>
@@ -50783,16 +50783,16 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
+          <t>marches/volatilite/VVIX.csv</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C223" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D223" t="n">
         <v>1</v>
@@ -50801,7 +50801,7 @@
         <v>42</v>
       </c>
       <c r="F223" t="n">
-        <v>5639</v>
+        <v>3762</v>
       </c>
       <c r="G223" t="inlineStr">
         <is>
@@ -50812,16 +50812,16 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>tresor_us/dette_quotidienne.csv</t>
+          <t>marches/volatilite/VXN.csv</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C224" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D224" t="n">
         <v>1</v>
@@ -50830,7 +50830,7 @@
         <v>42</v>
       </c>
       <c r="F224" t="n">
-        <v>2000</v>
+        <v>3770</v>
       </c>
       <c r="G224" t="inlineStr">
         <is>
@@ -50841,16 +50841,16 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>tresor_us/solde_tresorerie.csv</t>
+          <t>souverains/SUEDE_10A.csv</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C225" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D225" t="n">
         <v>1</v>
@@ -50859,7 +50859,7 @@
         <v>42</v>
       </c>
       <c r="F225" t="n">
-        <v>500</v>
+        <v>9203</v>
       </c>
       <c r="G225" t="inlineStr">
         <is>
@@ -50870,7 +50870,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>fred/ECBDFR.csv</t>
+          <t>souverains/SUEDE_2A.csv</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -50888,7 +50888,7 @@
         <v>42</v>
       </c>
       <c r="F226" t="n">
-        <v>3000</v>
+        <v>9203</v>
       </c>
       <c r="G226" t="inlineStr">
         <is>
@@ -50899,7 +50899,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>fred/RRPONTSYD.csv</t>
+          <t>souverains/SUEDE_5A.csv</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -50917,7 +50917,7 @@
         <v>42</v>
       </c>
       <c r="F227" t="n">
-        <v>3000</v>
+        <v>9205</v>
       </c>
       <c r="G227" t="inlineStr">
         <is>
@@ -50928,7 +50928,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>fred/T10YIE.csv</t>
+          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -50946,7 +50946,7 @@
         <v>42</v>
       </c>
       <c r="F228" t="n">
-        <v>3000</v>
+        <v>5640</v>
       </c>
       <c r="G228" t="inlineStr">
         <is>
@@ -50957,7 +50957,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>marches/volatilite/GVZ.csv</t>
+          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -50975,7 +50975,7 @@
         <v>42</v>
       </c>
       <c r="F229" t="n">
-        <v>3770</v>
+        <v>5640</v>
       </c>
       <c r="G229" t="inlineStr">
         <is>
@@ -50986,7 +50986,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>marches/volatilite/MOVE.csv</t>
+          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -51004,7 +51004,7 @@
         <v>42</v>
       </c>
       <c r="F230" t="n">
-        <v>3689</v>
+        <v>5640</v>
       </c>
       <c r="G230" t="inlineStr">
         <is>
@@ -51015,7 +51015,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>marches/volatilite/OVX.csv</t>
+          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -51033,7 +51033,7 @@
         <v>42</v>
       </c>
       <c r="F231" t="n">
-        <v>3770</v>
+        <v>5640</v>
       </c>
       <c r="G231" t="inlineStr">
         <is>
@@ -51044,7 +51044,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>marches/volatilite/VVIX.csv</t>
+          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -51062,7 +51062,7 @@
         <v>42</v>
       </c>
       <c r="F232" t="n">
-        <v>3762</v>
+        <v>5640</v>
       </c>
       <c r="G232" t="inlineStr">
         <is>
@@ -51073,7 +51073,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>marches/volatilite/VXN.csv</t>
+          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -51091,7 +51091,7 @@
         <v>42</v>
       </c>
       <c r="F233" t="n">
-        <v>3770</v>
+        <v>5640</v>
       </c>
       <c r="G233" t="inlineStr">
         <is>
@@ -51102,7 +51102,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_10A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -51120,7 +51120,7 @@
         <v>42</v>
       </c>
       <c r="F234" t="n">
-        <v>9203</v>
+        <v>5640</v>
       </c>
       <c r="G234" t="inlineStr">
         <is>
@@ -51131,7 +51131,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_2A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -51149,7 +51149,7 @@
         <v>42</v>
       </c>
       <c r="F235" t="n">
-        <v>9203</v>
+        <v>5640</v>
       </c>
       <c r="G235" t="inlineStr">
         <is>
@@ -51160,7 +51160,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_5A.csv</t>
+          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -51178,7 +51178,7 @@
         <v>42</v>
       </c>
       <c r="F236" t="n">
-        <v>9205</v>
+        <v>5640</v>
       </c>
       <c r="G236" t="inlineStr">
         <is>
@@ -52251,7 +52251,7 @@
         <v>42</v>
       </c>
       <c r="F273" t="n">
-        <v>3770</v>
+        <v>3771</v>
       </c>
       <c r="G273" t="inlineStr">
         <is>
@@ -53925,7 +53925,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Royaume-Uni (FTSE 100)</t>
+          <t>Zone euro (Euro Stoxx 50)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -53934,19 +53934,19 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>10713.6</v>
+        <v>6357.46</v>
       </c>
       <c r="D5" t="n">
-        <v>2.06</v>
+        <v>0.46</v>
       </c>
       <c r="E5" t="n">
-        <v>15.2</v>
+        <v>15.45</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Zone euro (Euro Stoxx 50)</t>
+          <t>Royaume-Uni (FTSE 100)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -53955,13 +53955,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>6342.69</v>
+        <v>10724.63</v>
       </c>
       <c r="D6" t="n">
-        <v>0.23</v>
+        <v>2.17</v>
       </c>
       <c r="E6" t="n">
-        <v>15.18</v>
+        <v>15.32</v>
       </c>
     </row>
     <row r="7">
@@ -53976,13 +53976,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>25450.15</v>
+        <v>25549.71</v>
       </c>
       <c r="D7" t="n">
-        <v>1.82</v>
+        <v>2.22</v>
       </c>
       <c r="E7" t="n">
-        <v>7.18</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="8">
@@ -54698,16 +54698,16 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>16.01</v>
+        <v>15.86</v>
       </c>
       <c r="C14" t="n">
-        <v>15.995</v>
+        <v>15.867</v>
       </c>
       <c r="D14" t="n">
         <v>0.625</v>
       </c>
       <c r="E14" t="n">
-        <v>0.20516</v>
+        <v>0.20517</v>
       </c>
     </row>
   </sheetData>
@@ -56194,19 +56194,19 @@
         <v>3.13</v>
       </c>
       <c r="D12" t="n">
-        <v>97.87</v>
+        <v>96.89</v>
       </c>
       <c r="E12" t="n">
-        <v>34.22</v>
+        <v>32.87</v>
       </c>
       <c r="F12" t="n">
-        <v>43.99</v>
+        <v>42.55</v>
       </c>
       <c r="G12" t="n">
-        <v>-5.22</v>
+        <v>-5.5</v>
       </c>
       <c r="H12" t="n">
-        <v>5.11</v>
+        <v>5.19</v>
       </c>
     </row>
   </sheetData>
@@ -60715,10 +60715,10 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>16.01</v>
+        <v>15.86</v>
       </c>
       <c r="C14" t="n">
-        <v>20.2</v>
+        <v>20.199</v>
       </c>
       <c r="D14" t="n">
         <v>0.02404</v>
@@ -60727,7 +60727,7 @@
         <v>28.8</v>
       </c>
       <c r="F14" t="n">
-        <v>-4.19</v>
+        <v>-4.339</v>
       </c>
     </row>
   </sheetData>
@@ -60842,7 +60842,7 @@
     <col width="23" customWidth="1" min="6" max="6"/>
     <col width="30" customWidth="1" min="7" max="7"/>
     <col width="30" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -60986,30 +60986,30 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>3.251</v>
+        <v>3.233</v>
       </c>
       <c r="D4" t="n">
-        <v>3.615</v>
+        <v>3.631</v>
       </c>
       <c r="E4" t="n">
-        <v>0.364</v>
+        <v>0.398</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.106</v>
+        <v>-0.048</v>
       </c>
       <c r="G4" t="n">
-        <v>0.798</v>
+        <v>0.756</v>
       </c>
       <c r="H4" t="n">
-        <v>0.6919999999999999</v>
+        <v>0.708</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>aplatissement</t>
+          <t>stable</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -67091,10 +67091,10 @@
         <v>0.008800000000000001</v>
       </c>
       <c r="C14" t="n">
-        <v>0.06808</v>
+        <v>0.06811</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.03844</v>
+        <v>-0.03845</v>
       </c>
     </row>
   </sheetData>
@@ -72818,7 +72818,7 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>3.7305</v>
+        <v>3.73</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
@@ -79839,13 +79839,13 @@
         <v>89.40000000000001</v>
       </c>
       <c r="D3" t="n">
-        <v>4.11</v>
+        <v>4.13</v>
       </c>
       <c r="E3" t="n">
         <v>3.25</v>
       </c>
       <c r="F3" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-29T17:08Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-29 15:30 UTC</t>
+          <t>Genere le 2026-09-29 17:08 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-29 15:30 UTC</t>
+          <t>Rapport global — 2026-09-29 17:08 UTC</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>**Matieres premieres macro** — ratio cuivre/or stable -- pas de signal net sur la croissance (+3.0% sur 3 mois). Brent 97.1$ (+33.1% sur 3 mois, +42.8% sur 12 mois), gaz -7.5% sur 3 mois, ecart Brent-WTI +5.5$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-29)_</t>
+          <t>**Matieres premieres macro** — ratio cuivre/or stable -- pas de signal net sur la croissance (+3.1% sur 3 mois). Brent 96.7$ (+32.7% sur 3 mois, +42.3% sur 12 mois), gaz -7.4% sur 3 mois, ecart Brent-WTI +6.4$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -862,7 +862,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>**Conditions financieres** — indice conditions financieres=+0.085 (3 composantes: {'taux_directeur': 0.5982151864455719, 'courbe_inversee': 0.17031877422284264, 'vix': -0.5126491644940797}) -- conditions proches de la normale _(observation : 2026-09-25)_</t>
+          <t>**Conditions financieres** — indice conditions financieres=+0.096 (3 composantes: {'taux_directeur': 0.5982151864455719, 'courbe_inversee': 0.17031877422284264, 'vix': -0.48049705797506703}) -- conditions proches de la normale _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
@@ -960,7 +960,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>**Indices mondiaux** — 7 indices (devise locale) : Coree (KOSPI) +103.5% en tete sur 12 mois, Hong Kong (Hang Seng) -7.9% en queue -- ecart tres large entre blocs sur 12 mois (111pt) -- les cycles economiques ou les flux divergent nettement. ROTATION en cours : Coree (KOSPI) mene sur 12 mois mais Hong Kong (Hang Seng) a repris la tete sur 3 mois _(observation : 2026-09-29)_</t>
+          <t>**Indices mondiaux** — 7 indices (devise locale) : Coree (KOSPI) +103.5% en tete sur 12 mois, Hong Kong (Hang Seng) -5.7% en queue -- ecart tres large entre blocs sur 12 mois (109pt) -- les cycles economiques ou les flux divergent nettement. ROTATION en cours : Coree (KOSPI) mene sur 12 mois mais Hong Kong (Hang Seng) a repris la tete sur 3 mois _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -988,7 +988,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>**Momentum prix** — SP500 momentum 12-1 mois = 15.77% -- haussier (momentum positif), detail 1/3/6/12m = [-0.7, 2.11, 17.3, 14.96] _(observation : 2026-09-29)_</t>
+          <t>**Momentum prix** — SP500 momentum 12-1 mois = 15.77% -- haussier (momentum positif), detail 1/3/6/12m = [-0.73, 2.08, 17.27, 14.93] _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1002,42 +1002,42 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>**Beta vol** — beta SP500/VIX (60j) = -0.00486 (rendement SP500 pour +1pt VIX) -- sensibilite normale, relation inverse attendue (normale) _(observation : 2026-09-29)_</t>
+          <t>**Beta vol** — beta SP500/VIX (60j) = -0.00487 (rendement SP500 pour +1pt VIX) -- sensibilite normale, relation inverse attendue (normale) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>**Rotation sectorielle** — classement momentum 3 mois (10 secteurs) : 1. Energie (XLE) : +15.95% | 2. Sante (XLV) : +6.67% | 3. Technologie (XLK) : +2.22% | 4. Finance (XLF) : +0.44% | 5. Consommation de base (XLP) : -2.02% _(observation : 2026-09-29)_</t>
+          <t>**Rotation sectorielle** — classement momentum 3 mois (10 secteurs) : 1. Energie (XLE) : +16.16% | 2. Sante (XLV) : +6.93% | 3. Technologie (XLK) : +1.96% | 4. Finance (XLF) : +0.48% | 5. Consommation de base (XLP) : -1.89% _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>**Saisonnalite** — rendement journalier moyen ete=+0.0179%, hiver=+0.0465% (t=-1.03, p=0.3023) -- non significatif (attendu vu la faible puissance sur seulement ~2 ans) _(observation : 2026-09-29)_</t>
+          <t>**Saisonnalite** — rendement journalier moyen ete=+0.0179%, hiver=+0.0465% (t=-1.03, p=0.3022) -- non significatif (attendu vu la faible puissance sur seulement ~2 ans) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>**Dispersion sectorielle** — 10 secteurs, rendement moyen 3m=-1.63%, dispersion (ecart-type)=8.03pt, etendue=29.17pt -- dispersion intermediaire _(observation : 2026-09-29)_</t>
+          <t>**Dispersion sectorielle** — 10 secteurs, rendement moyen 3m=-1.57%, dispersion (ecart-type)=8.06pt, etendue=29.13pt -- dispersion intermediaire _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>**Low volatility** — tercile bas-vol ['XLF', 'XLRE', 'XLU'] Sharpe=-0.943 vs tercile haut-vol ['XLY', 'XLE', 'XLK'] Sharpe=0.030 -- anomalie low-vol non confirmee sur cet echantillon (puissance statistique faible, n petit -- limite assumee) _(observation : 2026-09-29)_</t>
+          <t>**Low volatility** — tercile bas-vol ['XLF', 'XLRE', 'XLU'] Sharpe=-0.932 vs tercile haut-vol ['XLY', 'XLE', 'XLK'] Sharpe=0.031 -- anomalie low-vol non confirmee sur cet echantillon (puissance statistique faible, n petit -- limite assumee) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>**Momentum cross sectional** — panier gagnant ['XLE', 'XLV', 'XLK'] (+8.28%) vs panier perdant ['XLY', 'XLI', 'XLU'] (-9.85%) -- spread momentum=+18.13pt _(observation : 2026-09-29)_</t>
+          <t>**Momentum cross sectional** — panier gagnant ['XLE', 'XLV', 'XLK'] (+8.35%) vs panier perdant ['XLY', 'XLI', 'XLU'] (-9.73%) -- spread momentum=+18.08pt _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>**Correlation facteurs** — correlation entre momentum 3m et beta-VIX, 10 secteurs : +0.341 (facteurs largement independants) _(observation : 2026-09-29)_</t>
+          <t>**Correlation facteurs** — correlation entre momentum 3m et beta-VIX, 10 secteurs : +0.350 (facteurs largement independants) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1107,7 +1107,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>**Divergence cot prix** — SP500 -0.70% sur 30j, COT net -10560 -&gt; -133228 -- pas de divergence _(observation : 2026-09-29)_</t>
+          <t>**Divergence cot prix** — SP500 -0.73% sur 30j, COT net -10560 -&gt; -133228 -- pas de divergence _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1191,14 +1191,14 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>**Vol cross asset** — 6 mesures de volatilite : Petrole (OVX) 88e pct, Or (GVZ) 84e pct, Taux US (MOVE) 54e pct, Nasdaq (VXN) 46e pct, Vol de la vol (VVIX) 35e pct, Actions US (VIX) 32e pct -- stress LOCALISE sur Petrole (OVX), Or (GVZ) pendant que le reste ne l'est pas -- episode propre a cette classe d'actifs, pas une aversion au risque d'ensemble _(observation : 2026-09-29)_</t>
+          <t>**Vol cross asset** — 6 mesures de volatilite : Petrole (OVX) 88e pct, Or (GVZ) 85e pct, Taux US (MOVE) 58e pct, Nasdaq (VXN) 52e pct, Vol de la vol (VVIX) 39e pct, Actions US (VIX) 35e pct -- stress LOCALISE sur Petrole (OVX), Or (GVZ) pendant que le reste ne l'est pas -- episode propre a cette classe d'actifs, pas une aversion au risque d'ensemble _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>**Volatilite ewma** — vol realisee 60j=0.11218875196487915, EWMA=0.1065 (tendance 10 runs: stable) _(observation : 2026-09-29)_</t>
+          <t>**Volatilite ewma** — vol realisee 60j=0.11222961500219901, EWMA=0.1067 (tendance 10 runs: stable) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1219,7 +1219,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>**Ornstein uhlenbeck vix** — VIX actuel=16.06, niveau moyen estime (mu)=20.20, demi-vie=28.8j, ecart actuel=-4.14 -- VIX actuel en-dessous de son niveau moyen de long terme _(observation : 2026-09-29)_</t>
+          <t>**Ornstein uhlenbeck vix** — VIX actuel=16.32, niveau moyen estime (mu)=20.20, demi-vie=28.8j, ecart actuel=-3.88 -- VIX actuel en-dessous de son niveau moyen de long terme _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1233,14 +1233,14 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>**Kalman niveau local** — VIX observe=16.06, filtre Kalman=16.04 (ecart-type=0.62), ratio signal/bruit=0.2052 -- le filtre lisse fortement le bruit, reagit lentement (ecart obs.-filtre=+0.02) _(observation : 2026-09-29)_</t>
+          <t>**Kalman niveau local** — VIX observe=16.32, filtre Kalman=16.26 (ecart-type=0.62), ratio signal/bruit=0.2051 -- le filtre lisse fortement le bruit, reagit lentement (ecart obs.-filtre=+0.06) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.3725135374594988 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.05233957080408232 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-29)_</t>
+          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.37076270871109074 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.05233765339827812 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1261,14 +1261,14 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>**Skew kurtosis** — skewness=-0.188 (asymetrie negative (pertes extremes &gt; gains extremes)), kurtosis exces=+1.017 (queues epaisses (risque extreme sous-estime par une hypothese normale)) _(observation : 2026-09-29)_</t>
+          <t>**Skew kurtosis** — skewness=-0.188 (asymetrie negative (pertes extremes &gt; gains extremes)), kurtosis exces=+1.016 (queues epaisses (risque extreme sous-estime par une hypothese normale)) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>**Ratios performance** — Sharpe=1.076 (bon), Sortino=1.062 (bon), Calmar=1.539 (bon) -- lecture sur fenetre 252j (~1 an, echantillon limite), seuils academiques standards, taux sans risque suppose nul _(observation : 2026-09-29)_</t>
+          <t>**Ratios performance** — Sharpe=1.074 (bon), Sortino=1.060 (bon), Calmar=1.536 (bon) -- lecture sur fenetre 252j (~1 an, echantillon limite), seuils academiques standards, taux sans risque suppose nul _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1282,7 +1282,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>**Stress test historique** — COVID_2020 (2020-02-19 -&gt; 2020-03-23) : chute historique=-33.9% -- rejouee sur le niveau actuel (7658) -&gt; 5060  _(sans synthese)_ _(observation : 2026-09-29)_</t>
+          <t>**Stress test historique** — COVID_2020 (2020-02-19 -&gt; 2020-03-23) : chute historique=-33.9% -- rejouee sur le niveau actuel (7656) -&gt; 5059  _(sans synthese)_ _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1303,7 +1303,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>**Detection saut** — Z-stat BNS (fenetre 22j)=0.859 (seuil ±1.96) -- pas de saut isole detecte _(observation : 2026-09-29)_</t>
+          <t>**Detection saut** — Z-stat BNS (fenetre 22j)=0.845 (seuil ±1.96) -- pas de saut isole detecte _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1331,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>**Decomposition stl** — VIX : tendance=15.52, composante saisonniere (periode 5j)=+0.593, residu=-0.056 -- la saisonnalite explique 0.72% de la variance totale (negligeable) _(observation : 2026-09-29)_</t>
+          <t>**Decomposition stl** — VIX : tendance=15.58, composante saisonniere (periode 5j)=+0.674, residu=+0.061 -- la saisonnalite explique 0.72% de la variance totale (negligeable) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1387,7 +1387,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>**Anomalie multivariee** — distance de Mahalanobis=0.853 (seuil 3.0) -- jour ordinaire _(observation : 2026-09-29)_</t>
+          <t>**Anomalie multivariee** — distance de Mahalanobis=0.694 (seuil 3.0) -- jour ordinaire _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>**Importance permutation** — R2 base=0.0103 -- importance momentum5j=0.00088, importance variation_vix=0.01377 -- VIX plus important _(observation : 2026-09-29)_</t>
+          <t>**Importance permutation** — R2 base=0.0103 -- importance momentum5j=0.00088, importance variation_vix=0.01376 -- VIX plus important _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -5761,7 +5761,7 @@
         <v>-56.78</v>
       </c>
       <c r="F28" t="n">
-        <v>3310.08</v>
+        <v>3309.14</v>
       </c>
     </row>
     <row r="29">
@@ -5789,7 +5789,7 @@
         <v>-33.92</v>
       </c>
       <c r="F29" t="n">
-        <v>5059.94</v>
+        <v>5058.5</v>
       </c>
     </row>
   </sheetData>
@@ -7383,7 +7383,7 @@
         <v>0.07562000000000001</v>
       </c>
       <c r="D15" t="n">
-        <v>0.00416</v>
+        <v>0.00417</v>
       </c>
     </row>
   </sheetData>
@@ -8052,7 +8052,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>32.8</v>
+        <v>32.9</v>
       </c>
       <c r="D15" t="n">
         <v>-2.847</v>
@@ -8689,10 +8689,10 @@
         <v>10</v>
       </c>
       <c r="C15" t="n">
-        <v>0.37251</v>
+        <v>0.37076</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.05234</v>
+        <v>-0.052338</v>
       </c>
     </row>
   </sheetData>
@@ -8761,10 +8761,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>55.55</v>
+        <v>55.04</v>
       </c>
       <c r="D2" t="n">
-        <v>88.2</v>
+        <v>87.7</v>
       </c>
       <c r="E2" t="n">
         <v>1260</v>
@@ -8787,10 +8787,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>24.04</v>
+        <v>24.36</v>
       </c>
       <c r="D3" t="n">
-        <v>84</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="E3" t="n">
         <v>1260</v>
@@ -8813,10 +8813,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>104.06</v>
+        <v>106.81</v>
       </c>
       <c r="D4" t="n">
-        <v>53.6</v>
+        <v>58.2</v>
       </c>
       <c r="E4" t="n">
         <v>1260</v>
@@ -8839,10 +8839,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>21.91</v>
+        <v>22.74</v>
       </c>
       <c r="D5" t="n">
-        <v>45.9</v>
+        <v>52.2</v>
       </c>
       <c r="E5" t="n">
         <v>1260</v>
@@ -8865,10 +8865,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>90.16</v>
+        <v>91.34</v>
       </c>
       <c r="D6" t="n">
-        <v>34.8</v>
+        <v>38.7</v>
       </c>
       <c r="E6" t="n">
         <v>1260</v>
@@ -8891,10 +8891,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>16.06</v>
+        <v>16.32</v>
       </c>
       <c r="D7" t="n">
-        <v>32.5</v>
+        <v>35</v>
       </c>
       <c r="E7" t="n">
         <v>1260</v>
@@ -9207,13 +9207,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.1065</v>
+        <v>0.1067</v>
       </c>
       <c r="C15" t="n">
-        <v>0.0856</v>
+        <v>0.0857</v>
       </c>
       <c r="D15" t="n">
-        <v>0.1111</v>
+        <v>0.1112</v>
       </c>
       <c r="E15" t="n">
         <v>0.1122</v>
@@ -11956,13 +11956,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>12.982</v>
+        <v>12.983</v>
       </c>
       <c r="C15" t="n">
         <v>-1.289</v>
       </c>
       <c r="D15" t="n">
-        <v>-2.634</v>
+        <v>-2.635</v>
       </c>
       <c r="E15" t="n">
         <v>-3.98</v>
@@ -16841,10 +16841,10 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>-2.4654</v>
+        <v>-2.4889</v>
       </c>
       <c r="D132" t="n">
-        <v>0.2945</v>
+        <v>0.284</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -16864,10 +16864,10 @@
         </is>
       </c>
       <c r="C133" t="n">
-        <v>-1.8132</v>
+        <v>-1.8208</v>
       </c>
       <c r="D133" t="n">
-        <v>0.6233</v>
+        <v>0.6196</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -16887,10 +16887,10 @@
         </is>
       </c>
       <c r="C134" t="n">
-        <v>-2.1452</v>
+        <v>-2.1474</v>
       </c>
       <c r="D134" t="n">
-        <v>0.4528</v>
+        <v>0.4516</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -16910,10 +16910,10 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>-2.3905</v>
+        <v>-2.3936</v>
       </c>
       <c r="D135" t="n">
-        <v>0.3294</v>
+        <v>0.3279</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -16933,10 +16933,10 @@
         </is>
       </c>
       <c r="C136" t="n">
-        <v>-1.4035</v>
+        <v>-1.4247</v>
       </c>
       <c r="D136" t="n">
-        <v>0.7963</v>
+        <v>0.7889</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -16956,10 +16956,10 @@
         </is>
       </c>
       <c r="C137" t="n">
-        <v>0.0658</v>
+        <v>0.0564</v>
       </c>
       <c r="D137" t="n">
-        <v>0.9873</v>
+        <v>0.9871</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -16979,10 +16979,10 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>-1.1624</v>
+        <v>-1.1751</v>
       </c>
       <c r="D138" t="n">
-        <v>0.8675</v>
+        <v>0.8643</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -17002,10 +17002,10 @@
         </is>
       </c>
       <c r="C139" t="n">
-        <v>-0.5915</v>
+        <v>-0.6355</v>
       </c>
       <c r="D139" t="n">
-        <v>0.9571</v>
+        <v>0.9532</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -17025,10 +17025,10 @@
         </is>
       </c>
       <c r="C140" t="n">
-        <v>-2.1199</v>
+        <v>-2.1189</v>
       </c>
       <c r="D140" t="n">
-        <v>0.466</v>
+        <v>0.4665</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -17048,10 +17048,10 @@
         </is>
       </c>
       <c r="C141" t="n">
-        <v>-1.6036</v>
+        <v>-1.5882</v>
       </c>
       <c r="D141" t="n">
-        <v>0.7194</v>
+        <v>0.7259</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -23879,7 +23879,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.0853</v>
+        <v>0.096</v>
       </c>
       <c r="C14" t="n">
         <v>3</v>
@@ -23891,7 +23891,7 @@
         <v>0.1703</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.5125999999999999</v>
+        <v>-0.4805</v>
       </c>
     </row>
   </sheetData>
@@ -24179,7 +24179,7 @@
         <v>10</v>
       </c>
       <c r="C15" t="n">
-        <v>0.3414</v>
+        <v>0.3504</v>
       </c>
     </row>
   </sheetData>
@@ -36861,19 +36861,19 @@
         <v>2.2</v>
       </c>
       <c r="C14" t="n">
-        <v>428.46</v>
+        <v>428.85</v>
       </c>
       <c r="D14" t="n">
         <v>4</v>
       </c>
       <c r="E14" t="n">
-        <v>354.79</v>
+        <v>354.84</v>
       </c>
       <c r="F14" t="n">
         <v>5.4</v>
       </c>
       <c r="G14" t="n">
-        <v>351.69</v>
+        <v>351.96</v>
       </c>
     </row>
   </sheetData>
@@ -38319,13 +38319,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>15.524</v>
+        <v>15.585</v>
       </c>
       <c r="C14" t="n">
-        <v>0.593</v>
+        <v>0.674</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.056</v>
+        <v>0.061</v>
       </c>
       <c r="E14" t="n">
         <v>0.72</v>
@@ -39181,7 +39181,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.859</v>
+        <v>0.845</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -39812,13 +39812,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>-0.00337</v>
+        <v>-0.00365</v>
       </c>
       <c r="C15" t="n">
-        <v>-0.01</v>
+        <v>0.25</v>
       </c>
       <c r="D15" t="n">
-        <v>0.853</v>
+        <v>0.694</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -40131,13 +40131,13 @@
         <v>10</v>
       </c>
       <c r="C15" t="n">
-        <v>-1.628</v>
+        <v>-1.574</v>
       </c>
       <c r="D15" t="n">
-        <v>8.029</v>
+        <v>8.058</v>
       </c>
       <c r="E15" t="n">
-        <v>29.17</v>
+        <v>29.135</v>
       </c>
     </row>
   </sheetData>
@@ -40468,7 +40468,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>-0.699</v>
+        <v>-0.727</v>
       </c>
       <c r="C15" t="n">
         <v>-133228</v>
@@ -51281,7 +51281,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>marches/indices/KOSPI.csv</t>
+          <t>marches/indices/HANGSENG.csv</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -51299,7 +51299,7 @@
         <v>42</v>
       </c>
       <c r="F215" t="n">
-        <v>3680</v>
+        <v>3688</v>
       </c>
       <c r="G215" t="inlineStr">
         <is>
@@ -51310,7 +51310,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>marches/indices/NIKKEI225.csv</t>
+          <t>marches/indices/KOSPI.csv</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -51328,7 +51328,7 @@
         <v>42</v>
       </c>
       <c r="F216" t="n">
-        <v>3666</v>
+        <v>3680</v>
       </c>
       <c r="G216" t="inlineStr">
         <is>
@@ -51339,7 +51339,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>souverains/CANADA_10A.csv</t>
+          <t>marches/indices/NIKKEI225.csv</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -51357,7 +51357,7 @@
         <v>42</v>
       </c>
       <c r="F217" t="n">
-        <v>6437</v>
+        <v>3666</v>
       </c>
       <c r="G217" t="inlineStr">
         <is>
@@ -51368,7 +51368,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>souverains/CANADA_2A.csv</t>
+          <t>souverains/CANADA_10A.csv</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -51386,7 +51386,7 @@
         <v>42</v>
       </c>
       <c r="F218" t="n">
-        <v>6436</v>
+        <v>6437</v>
       </c>
       <c r="G218" t="inlineStr">
         <is>
@@ -51397,7 +51397,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>souverains/CANADA_5A.csv</t>
+          <t>souverains/CANADA_2A.csv</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -51426,7 +51426,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>souverains/CANADA_LONG.csv</t>
+          <t>souverains/CANADA_5A.csv</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -51455,7 +51455,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_10A.csv</t>
+          <t>souverains/CANADA_LONG.csv</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -51473,7 +51473,7 @@
         <v>42</v>
       </c>
       <c r="F221" t="n">
-        <v>9203</v>
+        <v>6436</v>
       </c>
       <c r="G221" t="inlineStr">
         <is>
@@ -51484,7 +51484,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_2A.csv</t>
+          <t>souverains/SUEDE_10A.csv</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -51513,7 +51513,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_5A.csv</t>
+          <t>souverains/SUEDE_2A.csv</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -51531,7 +51531,7 @@
         <v>42</v>
       </c>
       <c r="F223" t="n">
-        <v>9205</v>
+        <v>9203</v>
       </c>
       <c r="G223" t="inlineStr">
         <is>
@@ -51542,7 +51542,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
+          <t>souverains/SUEDE_5A.csv</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -51560,7 +51560,7 @@
         <v>42</v>
       </c>
       <c r="F224" t="n">
-        <v>5640</v>
+        <v>9205</v>
       </c>
       <c r="G224" t="inlineStr">
         <is>
@@ -51571,7 +51571,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
@@ -51600,7 +51600,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -51629,7 +51629,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -51658,7 +51658,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -51687,7 +51687,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -51716,7 +51716,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -51745,7 +51745,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -51774,7 +51774,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -51803,16 +51803,16 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>fred/ECBDFR.csv</t>
+          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C233" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D233" t="n">
         <v>1</v>
@@ -51821,7 +51821,7 @@
         <v>42</v>
       </c>
       <c r="F233" t="n">
-        <v>3000</v>
+        <v>5640</v>
       </c>
       <c r="G233" t="inlineStr">
         <is>
@@ -51832,7 +51832,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>marches/fx/AUDJPY.csv</t>
+          <t>fred/ECBDFR.csv</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -51850,7 +51850,7 @@
         <v>42</v>
       </c>
       <c r="F234" t="n">
-        <v>3908</v>
+        <v>3000</v>
       </c>
       <c r="G234" t="inlineStr">
         <is>
@@ -51861,7 +51861,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>marches/fx/AUDUSD.csv</t>
+          <t>marches/fx/AUDJPY.csv</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -51879,7 +51879,7 @@
         <v>42</v>
       </c>
       <c r="F235" t="n">
-        <v>3904</v>
+        <v>3908</v>
       </c>
       <c r="G235" t="inlineStr">
         <is>
@@ -51890,7 +51890,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>marches/fx/DXY.csv</t>
+          <t>marches/fx/AUDUSD.csv</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -51908,7 +51908,7 @@
         <v>42</v>
       </c>
       <c r="F236" t="n">
-        <v>3772</v>
+        <v>3904</v>
       </c>
       <c r="G236" t="inlineStr">
         <is>
@@ -51919,7 +51919,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>marches/fx/EURCHF.csv</t>
+          <t>marches/fx/DXY.csv</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
@@ -51937,7 +51937,7 @@
         <v>42</v>
       </c>
       <c r="F237" t="n">
-        <v>3905</v>
+        <v>3772</v>
       </c>
       <c r="G237" t="inlineStr">
         <is>
@@ -51948,7 +51948,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>marches/fx/EURGBP.csv</t>
+          <t>marches/fx/EURCHF.csv</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
@@ -51966,7 +51966,7 @@
         <v>42</v>
       </c>
       <c r="F238" t="n">
-        <v>3907</v>
+        <v>3905</v>
       </c>
       <c r="G238" t="inlineStr">
         <is>
@@ -51977,7 +51977,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>marches/fx/EURJPY.csv</t>
+          <t>marches/fx/EURGBP.csv</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
@@ -52006,7 +52006,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>marches/fx/EURUSD.csv</t>
+          <t>marches/fx/EURJPY.csv</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
@@ -52024,7 +52024,7 @@
         <v>42</v>
       </c>
       <c r="F240" t="n">
-        <v>3904</v>
+        <v>3907</v>
       </c>
       <c r="G240" t="inlineStr">
         <is>
@@ -52035,7 +52035,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>marches/fx/GBPUSD.csv</t>
+          <t>marches/fx/EURUSD.csv</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
@@ -52053,7 +52053,7 @@
         <v>42</v>
       </c>
       <c r="F241" t="n">
-        <v>3905</v>
+        <v>3904</v>
       </c>
       <c r="G241" t="inlineStr">
         <is>
@@ -52064,7 +52064,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>marches/fx/NZDUSD.csv</t>
+          <t>marches/fx/GBPUSD.csv</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
@@ -52093,7 +52093,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>marches/fx/USDCAD.csv</t>
+          <t>marches/fx/NZDUSD.csv</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
@@ -52111,7 +52111,7 @@
         <v>42</v>
       </c>
       <c r="F243" t="n">
-        <v>3904</v>
+        <v>3905</v>
       </c>
       <c r="G243" t="inlineStr">
         <is>
@@ -52122,7 +52122,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>marches/fx/USDCHF.csv</t>
+          <t>marches/fx/USDCAD.csv</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -52140,7 +52140,7 @@
         <v>42</v>
       </c>
       <c r="F244" t="n">
-        <v>3902</v>
+        <v>3904</v>
       </c>
       <c r="G244" t="inlineStr">
         <is>
@@ -52151,7 +52151,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>marches/fx/USDCNY.csv</t>
+          <t>marches/fx/USDCHF.csv</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -52169,7 +52169,7 @@
         <v>42</v>
       </c>
       <c r="F245" t="n">
-        <v>3904</v>
+        <v>3902</v>
       </c>
       <c r="G245" t="inlineStr">
         <is>
@@ -52180,7 +52180,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>marches/fx/USDJPY.csv</t>
+          <t>marches/fx/USDCNY.csv</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -52198,7 +52198,7 @@
         <v>42</v>
       </c>
       <c r="F246" t="n">
-        <v>3905</v>
+        <v>3904</v>
       </c>
       <c r="G246" t="inlineStr">
         <is>
@@ -52209,7 +52209,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>marches/fx/USDKRW.csv</t>
+          <t>marches/fx/USDJPY.csv</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
@@ -52227,7 +52227,7 @@
         <v>42</v>
       </c>
       <c r="F247" t="n">
-        <v>3904</v>
+        <v>3905</v>
       </c>
       <c r="G247" t="inlineStr">
         <is>
@@ -52238,7 +52238,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>marches/fx/USDNOK.csv</t>
+          <t>marches/fx/USDKRW.csv</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
@@ -52256,7 +52256,7 @@
         <v>42</v>
       </c>
       <c r="F248" t="n">
-        <v>3905</v>
+        <v>3904</v>
       </c>
       <c r="G248" t="inlineStr">
         <is>
@@ -52267,7 +52267,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>marches/fx/USDSEK.csv</t>
+          <t>marches/fx/USDNOK.csv</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
@@ -52296,7 +52296,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>marches/indices/DAX.csv</t>
+          <t>marches/fx/USDSEK.csv</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
@@ -52314,7 +52314,7 @@
         <v>42</v>
       </c>
       <c r="F250" t="n">
-        <v>3802</v>
+        <v>3905</v>
       </c>
       <c r="G250" t="inlineStr">
         <is>
@@ -52325,7 +52325,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>marches/indices/EUROSTOXX50.csv</t>
+          <t>marches/indices/DAX.csv</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
@@ -52343,7 +52343,7 @@
         <v>42</v>
       </c>
       <c r="F251" t="n">
-        <v>3759</v>
+        <v>3802</v>
       </c>
       <c r="G251" t="inlineStr">
         <is>
@@ -52354,7 +52354,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>marches/indices/FTSE100.csv</t>
+          <t>marches/indices/EUROSTOXX50.csv</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -52372,7 +52372,7 @@
         <v>42</v>
       </c>
       <c r="F252" t="n">
-        <v>3788</v>
+        <v>3759</v>
       </c>
       <c r="G252" t="inlineStr">
         <is>
@@ -52383,7 +52383,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>marches/indices/HANGSENG.csv</t>
+          <t>marches/indices/FTSE100.csv</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -52401,7 +52401,7 @@
         <v>42</v>
       </c>
       <c r="F253" t="n">
-        <v>3689</v>
+        <v>3788</v>
       </c>
       <c r="G253" t="inlineStr">
         <is>
@@ -52517,7 +52517,7 @@
         <v>42</v>
       </c>
       <c r="F257" t="n">
-        <v>3771</v>
+        <v>3770</v>
       </c>
       <c r="G257" t="inlineStr">
         <is>
@@ -54591,7 +54591,7 @@
         <v>0.00088</v>
       </c>
       <c r="D15" t="n">
-        <v>0.01377</v>
+        <v>0.01376</v>
       </c>
     </row>
   </sheetData>
@@ -54696,13 +54696,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>7657.87</v>
+        <v>7655.69</v>
       </c>
       <c r="D4" t="n">
-        <v>2.11</v>
+        <v>2.08</v>
       </c>
       <c r="E4" t="n">
-        <v>14.96</v>
+        <v>14.93</v>
       </c>
     </row>
     <row r="5">
@@ -54717,13 +54717,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>6329.09</v>
+        <v>6320.26</v>
       </c>
       <c r="D5" t="n">
-        <v>0.02</v>
+        <v>-0.12</v>
       </c>
       <c r="E5" t="n">
-        <v>14.93</v>
+        <v>14.77</v>
       </c>
     </row>
     <row r="6">
@@ -54738,13 +54738,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>10647.23</v>
+        <v>10636.71</v>
       </c>
       <c r="D6" t="n">
-        <v>1.43</v>
+        <v>1.33</v>
       </c>
       <c r="E6" t="n">
-        <v>14.49</v>
+        <v>14.38</v>
       </c>
     </row>
     <row r="7">
@@ -54759,13 +54759,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>25421.12</v>
+        <v>25399.21</v>
       </c>
       <c r="D7" t="n">
-        <v>1.7</v>
+        <v>1.61</v>
       </c>
       <c r="E7" t="n">
-        <v>7.06</v>
+        <v>6.97</v>
       </c>
     </row>
     <row r="8">
@@ -54776,17 +54776,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>24523.57</v>
+        <v>24642.51</v>
       </c>
       <c r="D8" t="n">
-        <v>7.18</v>
+        <v>7.02</v>
       </c>
       <c r="E8" t="n">
-        <v>-7.89</v>
+        <v>-5.69</v>
       </c>
     </row>
   </sheetData>
@@ -55481,16 +55481,16 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>16.059999</v>
+        <v>16.32</v>
       </c>
       <c r="C14" t="n">
-        <v>16.037</v>
+        <v>16.259</v>
       </c>
       <c r="D14" t="n">
         <v>0.625</v>
       </c>
       <c r="E14" t="n">
-        <v>0.20515</v>
+        <v>0.20513</v>
       </c>
     </row>
   </sheetData>
@@ -56633,7 +56633,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>-0.9429999999999999</v>
+        <v>-0.9320000000000001</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -56641,7 +56641,7 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0.03</v>
+        <v>0.031</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -57002,25 +57002,25 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.00158</v>
+        <v>0.001581</v>
       </c>
       <c r="C12" t="n">
-        <v>3.04</v>
+        <v>3.09</v>
       </c>
       <c r="D12" t="n">
-        <v>97.06</v>
+        <v>96.73999999999999</v>
       </c>
       <c r="E12" t="n">
-        <v>33.1</v>
+        <v>32.67</v>
       </c>
       <c r="F12" t="n">
-        <v>42.8</v>
+        <v>42.33</v>
       </c>
       <c r="G12" t="n">
-        <v>-7.45</v>
+        <v>-7.36</v>
       </c>
       <c r="H12" t="n">
-        <v>5.53</v>
+        <v>6.38</v>
       </c>
     </row>
   </sheetData>
@@ -57865,7 +57865,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>8.279</v>
+        <v>8.35</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -57873,10 +57873,10 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>-9.847</v>
+        <v>-9.733000000000001</v>
       </c>
       <c r="F15" t="n">
-        <v>18.126</v>
+        <v>18.084</v>
       </c>
     </row>
   </sheetData>
@@ -60810,16 +60810,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>-0.699</v>
+        <v>-0.727</v>
       </c>
       <c r="C15" t="n">
-        <v>2.114</v>
+        <v>2.085</v>
       </c>
       <c r="D15" t="n">
-        <v>17.299</v>
+        <v>17.265</v>
       </c>
       <c r="E15" t="n">
-        <v>14.962</v>
+        <v>14.929</v>
       </c>
       <c r="F15" t="n">
         <v>15.771</v>
@@ -61618,19 +61618,19 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>16.059999</v>
+        <v>16.32</v>
       </c>
       <c r="C14" t="n">
-        <v>20.201</v>
+        <v>20.202</v>
       </c>
       <c r="D14" t="n">
-        <v>0.02404</v>
+        <v>0.02405</v>
       </c>
       <c r="E14" t="n">
         <v>28.8</v>
       </c>
       <c r="F14" t="n">
-        <v>-4.141</v>
+        <v>-3.882</v>
       </c>
     </row>
   </sheetData>
@@ -66904,7 +66904,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>-0.004863</v>
+        <v>-0.004874</v>
       </c>
     </row>
   </sheetData>
@@ -68034,10 +68034,10 @@
         <v>0.008800000000000001</v>
       </c>
       <c r="C14" t="n">
-        <v>0.06808</v>
+        <v>0.06809</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.03844</v>
+        <v>-0.03845</v>
       </c>
     </row>
   </sheetData>
@@ -71503,13 +71503,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1.0763</v>
+        <v>1.074</v>
       </c>
       <c r="C15" t="n">
-        <v>1.0621</v>
+        <v>1.0598</v>
       </c>
       <c r="D15" t="n">
-        <v>1.5388</v>
+        <v>1.5356</v>
       </c>
     </row>
   </sheetData>
@@ -78098,7 +78098,7 @@
         </is>
       </c>
       <c r="E132" t="n">
-        <v>15.948</v>
+        <v>16.155</v>
       </c>
     </row>
     <row r="133">
@@ -78121,7 +78121,7 @@
         </is>
       </c>
       <c r="E133" t="n">
-        <v>6.665</v>
+        <v>6.933</v>
       </c>
     </row>
     <row r="134">
@@ -78144,7 +78144,7 @@
         </is>
       </c>
       <c r="E134" t="n">
-        <v>2.223</v>
+        <v>1.963</v>
       </c>
     </row>
     <row r="135">
@@ -78167,7 +78167,7 @@
         </is>
       </c>
       <c r="E135" t="n">
-        <v>0.438</v>
+        <v>0.485</v>
       </c>
     </row>
     <row r="136">
@@ -78190,7 +78190,7 @@
         </is>
       </c>
       <c r="E136" t="n">
-        <v>-2.016</v>
+        <v>-1.89</v>
       </c>
     </row>
     <row r="137">
@@ -78213,7 +78213,7 @@
         </is>
       </c>
       <c r="E137" t="n">
-        <v>-3.64</v>
+        <v>-3.679</v>
       </c>
     </row>
     <row r="138">
@@ -78236,7 +78236,7 @@
         </is>
       </c>
       <c r="E138" t="n">
-        <v>-6.359</v>
+        <v>-6.507</v>
       </c>
     </row>
     <row r="139">
@@ -78259,7 +78259,7 @@
         </is>
       </c>
       <c r="E139" t="n">
-        <v>-7.265</v>
+        <v>-7.239</v>
       </c>
     </row>
     <row r="140">
@@ -78282,7 +78282,7 @@
         </is>
       </c>
       <c r="E140" t="n">
-        <v>-9.054</v>
+        <v>-8.981</v>
       </c>
     </row>
     <row r="141">
@@ -78305,7 +78305,7 @@
         </is>
       </c>
       <c r="E141" t="n">
-        <v>-13.222</v>
+        <v>-12.98</v>
       </c>
     </row>
   </sheetData>
@@ -79169,7 +79169,7 @@
         <v>3705</v>
       </c>
       <c r="D15" t="n">
-        <v>0.01786</v>
+        <v>0.01785</v>
       </c>
       <c r="E15" t="n">
         <v>0.04655</v>
@@ -79178,7 +79178,7 @@
         <v>-1.032</v>
       </c>
       <c r="G15" t="n">
-        <v>0.3023</v>
+        <v>0.3022</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -81131,10 +81131,10 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>-0.188</v>
+        <v>-0.1877</v>
       </c>
       <c r="C15" t="n">
-        <v>1.0169</v>
+        <v>1.0158</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-29T20:09Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-29 17:08 UTC</t>
+          <t>Genere le 2026-09-29 20:09 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-29 17:08 UTC</t>
+          <t>Rapport global — 2026-09-29 20:09 UTC</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>**Matieres premieres macro** — ratio cuivre/or stable -- pas de signal net sur la croissance (+3.1% sur 3 mois). Brent 96.7$ (+32.7% sur 3 mois, +42.3% sur 12 mois), gaz -7.4% sur 3 mois, ecart Brent-WTI +6.4$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-29)_</t>
+          <t>**Matieres premieres macro** — ratio cuivre/or stable -- pas de signal net sur la croissance (+3.1% sur 3 mois). Brent 95.9$ (+31.5% sur 3 mois, +41.1% sur 12 mois), gaz -8.0% sur 3 mois, ecart Brent-WTI +6.7$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -862,7 +862,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>**Conditions financieres** — indice conditions financieres=+0.096 (3 composantes: {'taux_directeur': 0.5982151864455719, 'courbe_inversee': 0.17031877422284264, 'vix': -0.48049705797506703}) -- conditions proches de la normale _(observation : 2026-09-25)_</t>
+          <t>**Conditions financieres** — indice conditions financieres=+0.088 (3 composantes: {'taux_directeur': 0.5982151864455719, 'courbe_inversee': 0.17031877422284264, 'vix': -0.5039928815884913}) -- conditions proches de la normale _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
@@ -988,7 +988,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>**Momentum prix** — SP500 momentum 12-1 mois = 15.77% -- haussier (momentum positif), detail 1/3/6/12m = [-0.73, 2.08, 17.27, 14.93] _(observation : 2026-09-29)_</t>
+          <t>**Momentum prix** — SP500 momentum 12-1 mois = 15.77% -- haussier (momentum positif), detail 1/3/6/12m = [-0.53, 2.29, 17.5, 15.16] _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1009,35 +1009,35 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>**Rotation sectorielle** — classement momentum 3 mois (10 secteurs) : 1. Energie (XLE) : +16.16% | 2. Sante (XLV) : +6.93% | 3. Technologie (XLK) : +1.96% | 4. Finance (XLF) : +0.48% | 5. Consommation de base (XLP) : -1.89% _(observation : 2026-09-29)_</t>
+          <t>**Rotation sectorielle** — classement momentum 3 mois (10 secteurs) : 1. Energie (XLE) : +15.89% | 2. Sante (XLV) : +7.61% | 3. Technologie (XLK) : +2.08% | 4. Finance (XLF) : +0.75% | 5. Consommation de base (XLP) : -1.48% _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>**Saisonnalite** — rendement journalier moyen ete=+0.0179%, hiver=+0.0465% (t=-1.03, p=0.3022) -- non significatif (attendu vu la faible puissance sur seulement ~2 ans) _(observation : 2026-09-29)_</t>
+          <t>**Saisonnalite** — rendement journalier moyen ete=+0.0179%, hiver=+0.0465% (t=-1.03, p=0.3030) -- non significatif (attendu vu la faible puissance sur seulement ~2 ans) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>**Dispersion sectorielle** — 10 secteurs, rendement moyen 3m=-1.57%, dispersion (ecart-type)=8.06pt, etendue=29.13pt -- dispersion intermediaire _(observation : 2026-09-29)_</t>
+          <t>**Dispersion sectorielle** — 10 secteurs, rendement moyen 3m=-1.27%, dispersion (ecart-type)=7.92pt, etendue=28.29pt -- dispersion intermediaire _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>**Low volatility** — tercile bas-vol ['XLF', 'XLRE', 'XLU'] Sharpe=-0.932 vs tercile haut-vol ['XLY', 'XLE', 'XLK'] Sharpe=0.031 -- anomalie low-vol non confirmee sur cet echantillon (puissance statistique faible, n petit -- limite assumee) _(observation : 2026-09-29)_</t>
+          <t>**Low volatility** — tercile bas-vol ['XLF', 'XLRE', 'XLU'] Sharpe=-0.838 vs tercile haut-vol ['XLY', 'XLE', 'XLK'] Sharpe=0.040 -- anomalie low-vol non confirmee sur cet echantillon (puissance statistique faible, n petit -- limite assumee) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>**Momentum cross sectional** — panier gagnant ['XLE', 'XLV', 'XLK'] (+8.35%) vs panier perdant ['XLY', 'XLI', 'XLU'] (-9.73%) -- spread momentum=+18.08pt _(observation : 2026-09-29)_</t>
+          <t>**Momentum cross sectional** — panier gagnant ['XLE', 'XLV', 'XLK'] (+8.53%) vs panier perdant ['XLY', 'XLI', 'XLU'] (-9.34%) -- spread momentum=+17.87pt _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>**Correlation facteurs** — correlation entre momentum 3m et beta-VIX, 10 secteurs : +0.350 (facteurs largement independants) _(observation : 2026-09-29)_</t>
+          <t>**Correlation facteurs** — correlation entre momentum 3m et beta-VIX, 10 secteurs : +0.360 (facteurs largement independants) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1107,7 +1107,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>**Divergence cot prix** — SP500 -0.73% sur 30j, COT net -10560 -&gt; -133228 -- pas de divergence _(observation : 2026-09-29)_</t>
+          <t>**Divergence cot prix** — SP500 -0.53% sur 30j, COT net -10560 -&gt; -133228 -- pas de divergence _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1191,14 +1191,14 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>**Vol cross asset** — 6 mesures de volatilite : Petrole (OVX) 88e pct, Or (GVZ) 85e pct, Taux US (MOVE) 58e pct, Nasdaq (VXN) 52e pct, Vol de la vol (VVIX) 39e pct, Actions US (VIX) 35e pct -- stress LOCALISE sur Petrole (OVX), Or (GVZ) pendant que le reste ne l'est pas -- episode propre a cette classe d'actifs, pas une aversion au risque d'ensemble _(observation : 2026-09-29)_</t>
+          <t>**Vol cross asset** — 6 mesures de volatilite : Petrole (OVX) 86e pct, Or (GVZ) 85e pct, Taux US (MOVE) 58e pct, Nasdaq (VXN) 49e pct, Vol de la vol (VVIX) 34e pct, Actions US (VIX) 33e pct -- stress LOCALISE sur Petrole (OVX), Or (GVZ) pendant que le reste ne l'est pas -- episode propre a cette classe d'actifs, pas une aversion au risque d'ensemble _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>**Volatilite ewma** — vol realisee 60j=0.11222961500219901, EWMA=0.1067 (tendance 10 runs: stable) _(observation : 2026-09-29)_</t>
+          <t>**Volatilite ewma** — vol realisee 60j=0.11200610147428887, EWMA=0.1059 (tendance 10 runs: stable) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1219,7 +1219,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>**Ornstein uhlenbeck vix** — VIX actuel=16.32, niveau moyen estime (mu)=20.20, demi-vie=28.8j, ecart actuel=-3.88 -- VIX actuel en-dessous de son niveau moyen de long terme _(observation : 2026-09-29)_</t>
+          <t>**Ornstein uhlenbeck vix** — VIX actuel=16.13, niveau moyen estime (mu)=20.20, demi-vie=28.8j, ecart actuel=-4.07 -- VIX actuel en-dessous de son niveau moyen de long terme _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1233,14 +1233,14 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>**Kalman niveau local** — VIX observe=16.32, filtre Kalman=16.26 (ecart-type=0.62), ratio signal/bruit=0.2051 -- le filtre lisse fortement le bruit, reagit lentement (ecart obs.-filtre=+0.06) _(observation : 2026-09-29)_</t>
+          <t>**Kalman niveau local** — VIX observe=16.13, filtre Kalman=16.10 (ecart-type=0.62), ratio signal/bruit=0.2051 -- le filtre lisse fortement le bruit, reagit lentement (ecart obs.-filtre=+0.03) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.37076270871109074 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.05233765339827812 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-29)_</t>
+          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.37204216230183995 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.052351167944674745 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1261,14 +1261,14 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>**Skew kurtosis** — skewness=-0.188 (asymetrie negative (pertes extremes &gt; gains extremes)), kurtosis exces=+1.016 (queues epaisses (risque extreme sous-estime par une hypothese normale)) _(observation : 2026-09-29)_</t>
+          <t>**Skew kurtosis** — skewness=-0.190 (asymetrie negative (pertes extremes &gt; gains extremes)), kurtosis exces=+1.022 (queues epaisses (risque extreme sous-estime par une hypothese normale)) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>**Ratios performance** — Sharpe=1.074 (bon), Sortino=1.060 (bon), Calmar=1.536 (bon) -- lecture sur fenetre 252j (~1 an, echantillon limite), seuils academiques standards, taux sans risque suppose nul _(observation : 2026-09-29)_</t>
+          <t>**Ratios performance** — Sharpe=1.090 (bon), Sortino=1.076 (bon), Calmar=1.558 (bon) -- lecture sur fenetre 252j (~1 an, echantillon limite), seuils academiques standards, taux sans risque suppose nul _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1282,7 +1282,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>**Stress test historique** — COVID_2020 (2020-02-19 -&gt; 2020-03-23) : chute historique=-33.9% -- rejouee sur le niveau actuel (7656) -&gt; 5059  _(sans synthese)_ _(observation : 2026-09-29)_</t>
+          <t>**Stress test historique** — COVID_2020 (2020-02-19 -&gt; 2020-03-23) : chute historique=-33.9% -- rejouee sur le niveau actuel (7671) -&gt; 5069  _(sans synthese)_ _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1303,7 +1303,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>**Detection saut** — Z-stat BNS (fenetre 22j)=0.845 (seuil ±1.96) -- pas de saut isole detecte _(observation : 2026-09-29)_</t>
+          <t>**Detection saut** — Z-stat BNS (fenetre 22j)=0.973 (seuil ±1.96) -- pas de saut isole detecte _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1331,14 +1331,14 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>**Decomposition stl** — VIX : tendance=15.58, composante saisonniere (periode 5j)=+0.674, residu=+0.061 -- la saisonnalite explique 0.72% de la variance totale (negligeable) _(observation : 2026-09-29)_</t>
+          <t>**Decomposition stl** — VIX : tendance=15.54, composante saisonniere (periode 5j)=+0.616, residu=-0.027 -- la saisonnalite explique 0.72% de la variance totale (negligeable) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>**Ratios conditionnels regime** — Sharpe regime haut-vol=-1.107, bas-vol=2.400, global=0.420 -- meilleur en regime calme, comme attendu _(observation : 2026-09-29)_</t>
+          <t>**Ratios conditionnels regime** — Sharpe regime haut-vol=-1.107, bas-vol=2.401, global=0.421 -- meilleur en regime calme, comme attendu _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1387,7 +1387,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>**Anomalie multivariee** — distance de Mahalanobis=0.694 (seuil 3.0) -- jour ordinaire _(observation : 2026-09-29)_</t>
+          <t>**Anomalie multivariee** — distance de Mahalanobis=0.424 (seuil 3.0) -- jour ordinaire _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>**Couts transaction** — 7516 predictions, 1513 changements de position (5pb/changement) -- rendement cumule brut=-93.18%, cout total=53.08%, net=-96.80% -- les frais mangent une part importante du rendement (&gt;50% du brut) _(observation : 2026-09-29)_</t>
+          <t>**Couts transaction** — 7516 predictions, 1513 changements de position (5pb/changement) -- rendement cumule brut=-93.19%, cout total=53.08%, net=-96.80% -- les frais mangent une part importante du rendement (&gt;50% du brut) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>**Importance permutation** — R2 base=0.0103 -- importance momentum5j=0.00088, importance variation_vix=0.01376 -- VIX plus important _(observation : 2026-09-29)_</t>
+          <t>**Importance permutation** — R2 base=0.0103 -- importance momentum5j=0.00088, importance variation_vix=0.01377 -- VIX plus important _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -5761,7 +5761,7 @@
         <v>-56.78</v>
       </c>
       <c r="F28" t="n">
-        <v>3309.14</v>
+        <v>3315.79</v>
       </c>
     </row>
     <row r="29">
@@ -5789,7 +5789,7 @@
         <v>-33.92</v>
       </c>
       <c r="F29" t="n">
-        <v>5058.5</v>
+        <v>5068.66</v>
       </c>
     </row>
   </sheetData>
@@ -7380,10 +7380,10 @@
         <v>5</v>
       </c>
       <c r="C15" t="n">
-        <v>0.07562000000000001</v>
+        <v>0.07557999999999999</v>
       </c>
       <c r="D15" t="n">
-        <v>0.00417</v>
+        <v>0.00416</v>
       </c>
     </row>
   </sheetData>
@@ -8052,7 +8052,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>32.9</v>
+        <v>32.8</v>
       </c>
       <c r="D15" t="n">
         <v>-2.847</v>
@@ -8689,10 +8689,10 @@
         <v>10</v>
       </c>
       <c r="C15" t="n">
-        <v>0.37076</v>
+        <v>0.37204</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.052338</v>
+        <v>-0.052351</v>
       </c>
     </row>
   </sheetData>
@@ -8761,10 +8761,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>55.04</v>
+        <v>53.65</v>
       </c>
       <c r="D2" t="n">
-        <v>87.7</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="E2" t="n">
         <v>1260</v>
@@ -8787,10 +8787,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>24.36</v>
+        <v>24.27</v>
       </c>
       <c r="D3" t="n">
-        <v>84.90000000000001</v>
+        <v>84.8</v>
       </c>
       <c r="E3" t="n">
         <v>1260</v>
@@ -8813,10 +8813,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>106.81</v>
+        <v>106.6</v>
       </c>
       <c r="D4" t="n">
-        <v>58.2</v>
+        <v>57.7</v>
       </c>
       <c r="E4" t="n">
         <v>1260</v>
@@ -8839,10 +8839,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>22.74</v>
+        <v>22.34</v>
       </c>
       <c r="D5" t="n">
-        <v>52.2</v>
+        <v>49.4</v>
       </c>
       <c r="E5" t="n">
         <v>1260</v>
@@ -8865,10 +8865,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>91.34</v>
+        <v>90.08</v>
       </c>
       <c r="D6" t="n">
-        <v>38.7</v>
+        <v>34.5</v>
       </c>
       <c r="E6" t="n">
         <v>1260</v>
@@ -8891,10 +8891,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>16.32</v>
+        <v>16.13</v>
       </c>
       <c r="D7" t="n">
-        <v>35</v>
+        <v>33.4</v>
       </c>
       <c r="E7" t="n">
         <v>1260</v>
@@ -9207,16 +9207,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.1067</v>
+        <v>0.1059</v>
       </c>
       <c r="C15" t="n">
         <v>0.0857</v>
       </c>
       <c r="D15" t="n">
-        <v>0.1112</v>
+        <v>0.1106</v>
       </c>
       <c r="E15" t="n">
-        <v>0.1122</v>
+        <v>0.112</v>
       </c>
     </row>
   </sheetData>
@@ -11956,16 +11956,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>12.983</v>
+        <v>12.978</v>
       </c>
       <c r="C15" t="n">
-        <v>-1.289</v>
+        <v>-1.288</v>
       </c>
       <c r="D15" t="n">
-        <v>-2.635</v>
+        <v>-2.633</v>
       </c>
       <c r="E15" t="n">
-        <v>-3.98</v>
+        <v>-3.978</v>
       </c>
     </row>
   </sheetData>
@@ -16841,10 +16841,10 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>-2.4889</v>
+        <v>-2.5118</v>
       </c>
       <c r="D132" t="n">
-        <v>0.284</v>
+        <v>0.2739</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -16864,10 +16864,10 @@
         </is>
       </c>
       <c r="C133" t="n">
-        <v>-1.8208</v>
+        <v>-1.8329</v>
       </c>
       <c r="D133" t="n">
-        <v>0.6196</v>
+        <v>0.6136</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -16887,10 +16887,10 @@
         </is>
       </c>
       <c r="C134" t="n">
-        <v>-2.1474</v>
+        <v>-2.1418</v>
       </c>
       <c r="D134" t="n">
-        <v>0.4516</v>
+        <v>0.4546</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -16910,10 +16910,10 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>-2.3936</v>
+        <v>-2.3975</v>
       </c>
       <c r="D135" t="n">
-        <v>0.3279</v>
+        <v>0.326</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -16933,10 +16933,10 @@
         </is>
       </c>
       <c r="C136" t="n">
-        <v>-1.4247</v>
+        <v>-1.4407</v>
       </c>
       <c r="D136" t="n">
-        <v>0.7889</v>
+        <v>0.7832</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -16956,10 +16956,10 @@
         </is>
       </c>
       <c r="C137" t="n">
-        <v>0.0564</v>
+        <v>0.0391</v>
       </c>
       <c r="D137" t="n">
-        <v>0.9871</v>
+        <v>0.9868</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -16979,10 +16979,10 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>-1.1751</v>
+        <v>-1.196</v>
       </c>
       <c r="D138" t="n">
-        <v>0.8643</v>
+        <v>0.8589</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -17002,10 +17002,10 @@
         </is>
       </c>
       <c r="C139" t="n">
-        <v>-0.6355</v>
+        <v>-0.7012</v>
       </c>
       <c r="D139" t="n">
-        <v>0.9532</v>
+        <v>0.9465</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -17025,10 +17025,10 @@
         </is>
       </c>
       <c r="C140" t="n">
-        <v>-2.1189</v>
+        <v>-2.1228</v>
       </c>
       <c r="D140" t="n">
-        <v>0.4665</v>
+        <v>0.4644</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -17048,10 +17048,10 @@
         </is>
       </c>
       <c r="C141" t="n">
-        <v>-1.5882</v>
+        <v>-1.6207</v>
       </c>
       <c r="D141" t="n">
-        <v>0.7259</v>
+        <v>0.7121</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -23879,7 +23879,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.096</v>
+        <v>0.0882</v>
       </c>
       <c r="C14" t="n">
         <v>3</v>
@@ -23891,7 +23891,7 @@
         <v>0.1703</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.4805</v>
+        <v>-0.504</v>
       </c>
     </row>
   </sheetData>
@@ -24179,7 +24179,7 @@
         <v>10</v>
       </c>
       <c r="C15" t="n">
-        <v>0.3504</v>
+        <v>0.36</v>
       </c>
     </row>
   </sheetData>
@@ -36485,7 +36485,7 @@
         <v>53.08</v>
       </c>
       <c r="E15" t="n">
-        <v>-93.18000000000001</v>
+        <v>-93.19</v>
       </c>
       <c r="F15" t="n">
         <v>-96.8</v>
@@ -36861,19 +36861,19 @@
         <v>2.2</v>
       </c>
       <c r="C14" t="n">
-        <v>428.85</v>
+        <v>428.56</v>
       </c>
       <c r="D14" t="n">
         <v>4</v>
       </c>
       <c r="E14" t="n">
-        <v>354.84</v>
+        <v>354.8</v>
       </c>
       <c r="F14" t="n">
         <v>5.4</v>
       </c>
       <c r="G14" t="n">
-        <v>351.96</v>
+        <v>351.77</v>
       </c>
     </row>
   </sheetData>
@@ -38319,13 +38319,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>15.585</v>
+        <v>15.541</v>
       </c>
       <c r="C14" t="n">
-        <v>0.674</v>
+        <v>0.616</v>
       </c>
       <c r="D14" t="n">
-        <v>0.061</v>
+        <v>-0.027</v>
       </c>
       <c r="E14" t="n">
         <v>0.72</v>
@@ -39181,7 +39181,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.845</v>
+        <v>0.973</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -39812,13 +39812,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>-0.00365</v>
+        <v>-0.00164</v>
       </c>
       <c r="C15" t="n">
-        <v>0.25</v>
+        <v>0.06</v>
       </c>
       <c r="D15" t="n">
-        <v>0.694</v>
+        <v>0.424</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -40131,13 +40131,13 @@
         <v>10</v>
       </c>
       <c r="C15" t="n">
-        <v>-1.574</v>
+        <v>-1.269</v>
       </c>
       <c r="D15" t="n">
-        <v>8.058</v>
+        <v>7.921</v>
       </c>
       <c r="E15" t="n">
-        <v>29.135</v>
+        <v>28.287</v>
       </c>
     </row>
   </sheetData>
@@ -40468,7 +40468,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>-0.727</v>
+        <v>-0.528</v>
       </c>
       <c r="C15" t="n">
         <v>-133228</v>
@@ -50933,16 +50933,16 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>tresor_us/solde_tresorerie.csv</t>
+          <t>fred/BAMLC0A0CM.csv</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C203" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D203" t="n">
         <v>1</v>
@@ -50951,7 +50951,7 @@
         <v>42</v>
       </c>
       <c r="F203" t="n">
-        <v>500</v>
+        <v>793</v>
       </c>
       <c r="G203" t="inlineStr">
         <is>
@@ -50962,7 +50962,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>fred/BAMLC0A0CM.csv</t>
+          <t>fred/BAMLC0A0CMEY.csv</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
@@ -50991,7 +50991,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>fred/BAMLC0A0CMEY.csv</t>
+          <t>fred/BAMLEMCBPIOAS.csv</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -51020,7 +51020,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>fred/BAMLEMCBPIOAS.csv</t>
+          <t>fred/BAMLEMFSFCRPIOAS.csv</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -51049,7 +51049,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>fred/BAMLEMFSFCRPIOAS.csv</t>
+          <t>fred/BAMLEMHBHYCRPIOAS.csv</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -51078,7 +51078,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>fred/BAMLEMHBHYCRPIOAS.csv</t>
+          <t>fred/BAMLEMPBPUBSICRPIOAS.csv</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -51107,7 +51107,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>fred/BAMLEMPBPUBSICRPIOAS.csv</t>
+          <t>fred/BAMLH0A0HYM2.csv</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -51136,7 +51136,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>fred/BAMLH0A0HYM2.csv</t>
+          <t>fred/BAMLHE00EHYIEY.csv</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -51165,7 +51165,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>fred/BAMLHE00EHYIEY.csv</t>
+          <t>fred/BAMLHE00EHYIOAS.csv</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
@@ -51194,7 +51194,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>fred/BAMLHE00EHYIOAS.csv</t>
+          <t>fred/T10YIE.csv</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -51212,7 +51212,7 @@
         <v>42</v>
       </c>
       <c r="F212" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G212" t="inlineStr">
         <is>
@@ -51223,7 +51223,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>fred/RRPONTSYD.csv</t>
+          <t>marches/indices/HANGSENG.csv</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -51241,7 +51241,7 @@
         <v>42</v>
       </c>
       <c r="F213" t="n">
-        <v>3000</v>
+        <v>3688</v>
       </c>
       <c r="G213" t="inlineStr">
         <is>
@@ -51252,7 +51252,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>fred/T10YIE.csv</t>
+          <t>marches/indices/KOSPI.csv</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -51270,7 +51270,7 @@
         <v>42</v>
       </c>
       <c r="F214" t="n">
-        <v>3000</v>
+        <v>3680</v>
       </c>
       <c r="G214" t="inlineStr">
         <is>
@@ -51281,7 +51281,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>marches/indices/HANGSENG.csv</t>
+          <t>marches/indices/NIKKEI225.csv</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -51299,7 +51299,7 @@
         <v>42</v>
       </c>
       <c r="F215" t="n">
-        <v>3688</v>
+        <v>3666</v>
       </c>
       <c r="G215" t="inlineStr">
         <is>
@@ -51310,7 +51310,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>marches/indices/KOSPI.csv</t>
+          <t>souverains/CANADA_10A.csv</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -51328,7 +51328,7 @@
         <v>42</v>
       </c>
       <c r="F216" t="n">
-        <v>3680</v>
+        <v>6437</v>
       </c>
       <c r="G216" t="inlineStr">
         <is>
@@ -51339,7 +51339,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>marches/indices/NIKKEI225.csv</t>
+          <t>souverains/CANADA_2A.csv</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -51357,7 +51357,7 @@
         <v>42</v>
       </c>
       <c r="F217" t="n">
-        <v>3666</v>
+        <v>6436</v>
       </c>
       <c r="G217" t="inlineStr">
         <is>
@@ -51368,7 +51368,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>souverains/CANADA_10A.csv</t>
+          <t>souverains/CANADA_5A.csv</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -51386,7 +51386,7 @@
         <v>42</v>
       </c>
       <c r="F218" t="n">
-        <v>6437</v>
+        <v>6436</v>
       </c>
       <c r="G218" t="inlineStr">
         <is>
@@ -51397,7 +51397,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>souverains/CANADA_2A.csv</t>
+          <t>souverains/CANADA_LONG.csv</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -51426,7 +51426,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>souverains/CANADA_5A.csv</t>
+          <t>souverains/SUEDE_10A.csv</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -51444,7 +51444,7 @@
         <v>42</v>
       </c>
       <c r="F220" t="n">
-        <v>6436</v>
+        <v>9203</v>
       </c>
       <c r="G220" t="inlineStr">
         <is>
@@ -51455,7 +51455,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>souverains/CANADA_LONG.csv</t>
+          <t>souverains/SUEDE_2A.csv</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -51473,7 +51473,7 @@
         <v>42</v>
       </c>
       <c r="F221" t="n">
-        <v>6436</v>
+        <v>9203</v>
       </c>
       <c r="G221" t="inlineStr">
         <is>
@@ -51484,7 +51484,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_10A.csv</t>
+          <t>souverains/SUEDE_5A.csv</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -51502,7 +51502,7 @@
         <v>42</v>
       </c>
       <c r="F222" t="n">
-        <v>9203</v>
+        <v>9205</v>
       </c>
       <c r="G222" t="inlineStr">
         <is>
@@ -51513,7 +51513,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_2A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -51531,7 +51531,7 @@
         <v>42</v>
       </c>
       <c r="F223" t="n">
-        <v>9203</v>
+        <v>5640</v>
       </c>
       <c r="G223" t="inlineStr">
         <is>
@@ -51542,7 +51542,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_5A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -51560,7 +51560,7 @@
         <v>42</v>
       </c>
       <c r="F224" t="n">
-        <v>9205</v>
+        <v>5640</v>
       </c>
       <c r="G224" t="inlineStr">
         <is>
@@ -51571,7 +51571,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
@@ -51600,7 +51600,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -51629,7 +51629,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -51658,7 +51658,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -51687,7 +51687,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -51716,7 +51716,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -51745,7 +51745,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
+          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -51774,7 +51774,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
+          <t>tresor_us/solde_tresorerie.csv</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -51792,7 +51792,7 @@
         <v>42</v>
       </c>
       <c r="F232" t="n">
-        <v>5640</v>
+        <v>500</v>
       </c>
       <c r="G232" t="inlineStr">
         <is>
@@ -51803,16 +51803,16 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
+          <t>fred/ECBDFR.csv</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C233" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D233" t="n">
         <v>1</v>
@@ -51821,7 +51821,7 @@
         <v>42</v>
       </c>
       <c r="F233" t="n">
-        <v>5640</v>
+        <v>3000</v>
       </c>
       <c r="G233" t="inlineStr">
         <is>
@@ -51832,7 +51832,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>fred/ECBDFR.csv</t>
+          <t>fred/RRPONTSYD.csv</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -51879,7 +51879,7 @@
         <v>42</v>
       </c>
       <c r="F235" t="n">
-        <v>3908</v>
+        <v>3909</v>
       </c>
       <c r="G235" t="inlineStr">
         <is>
@@ -51908,7 +51908,7 @@
         <v>42</v>
       </c>
       <c r="F236" t="n">
-        <v>3904</v>
+        <v>3905</v>
       </c>
       <c r="G236" t="inlineStr">
         <is>
@@ -51966,7 +51966,7 @@
         <v>42</v>
       </c>
       <c r="F238" t="n">
-        <v>3905</v>
+        <v>3906</v>
       </c>
       <c r="G238" t="inlineStr">
         <is>
@@ -51995,7 +51995,7 @@
         <v>42</v>
       </c>
       <c r="F239" t="n">
-        <v>3907</v>
+        <v>3908</v>
       </c>
       <c r="G239" t="inlineStr">
         <is>
@@ -52024,7 +52024,7 @@
         <v>42</v>
       </c>
       <c r="F240" t="n">
-        <v>3907</v>
+        <v>3908</v>
       </c>
       <c r="G240" t="inlineStr">
         <is>
@@ -52053,7 +52053,7 @@
         <v>42</v>
       </c>
       <c r="F241" t="n">
-        <v>3904</v>
+        <v>3905</v>
       </c>
       <c r="G241" t="inlineStr">
         <is>
@@ -52082,7 +52082,7 @@
         <v>42</v>
       </c>
       <c r="F242" t="n">
-        <v>3905</v>
+        <v>3906</v>
       </c>
       <c r="G242" t="inlineStr">
         <is>
@@ -52111,7 +52111,7 @@
         <v>42</v>
       </c>
       <c r="F243" t="n">
-        <v>3905</v>
+        <v>3906</v>
       </c>
       <c r="G243" t="inlineStr">
         <is>
@@ -52140,7 +52140,7 @@
         <v>42</v>
       </c>
       <c r="F244" t="n">
-        <v>3904</v>
+        <v>3905</v>
       </c>
       <c r="G244" t="inlineStr">
         <is>
@@ -52169,7 +52169,7 @@
         <v>42</v>
       </c>
       <c r="F245" t="n">
-        <v>3902</v>
+        <v>3903</v>
       </c>
       <c r="G245" t="inlineStr">
         <is>
@@ -52198,7 +52198,7 @@
         <v>42</v>
       </c>
       <c r="F246" t="n">
-        <v>3904</v>
+        <v>3905</v>
       </c>
       <c r="G246" t="inlineStr">
         <is>
@@ -52227,7 +52227,7 @@
         <v>42</v>
       </c>
       <c r="F247" t="n">
-        <v>3905</v>
+        <v>3906</v>
       </c>
       <c r="G247" t="inlineStr">
         <is>
@@ -52256,7 +52256,7 @@
         <v>42</v>
       </c>
       <c r="F248" t="n">
-        <v>3904</v>
+        <v>3905</v>
       </c>
       <c r="G248" t="inlineStr">
         <is>
@@ -52285,7 +52285,7 @@
         <v>42</v>
       </c>
       <c r="F249" t="n">
-        <v>3905</v>
+        <v>3906</v>
       </c>
       <c r="G249" t="inlineStr">
         <is>
@@ -52314,7 +52314,7 @@
         <v>42</v>
       </c>
       <c r="F250" t="n">
-        <v>3905</v>
+        <v>3906</v>
       </c>
       <c r="G250" t="inlineStr">
         <is>
@@ -52604,7 +52604,7 @@
         <v>42</v>
       </c>
       <c r="F260" t="n">
-        <v>3771</v>
+        <v>3770</v>
       </c>
       <c r="G260" t="inlineStr">
         <is>
@@ -52633,7 +52633,7 @@
         <v>42</v>
       </c>
       <c r="F261" t="n">
-        <v>3690</v>
+        <v>3689</v>
       </c>
       <c r="G261" t="inlineStr">
         <is>
@@ -52662,7 +52662,7 @@
         <v>42</v>
       </c>
       <c r="F262" t="n">
-        <v>3771</v>
+        <v>3770</v>
       </c>
       <c r="G262" t="inlineStr">
         <is>
@@ -52691,7 +52691,7 @@
         <v>42</v>
       </c>
       <c r="F263" t="n">
-        <v>3763</v>
+        <v>3762</v>
       </c>
       <c r="G263" t="inlineStr">
         <is>
@@ -52720,7 +52720,7 @@
         <v>42</v>
       </c>
       <c r="F264" t="n">
-        <v>3771</v>
+        <v>3770</v>
       </c>
       <c r="G264" t="inlineStr">
         <is>
@@ -54585,13 +54585,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.01026</v>
+        <v>0.01027</v>
       </c>
       <c r="C15" t="n">
         <v>0.00088</v>
       </c>
       <c r="D15" t="n">
-        <v>0.01376</v>
+        <v>0.01377</v>
       </c>
     </row>
   </sheetData>
@@ -54696,13 +54696,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>7655.69</v>
+        <v>7671.07</v>
       </c>
       <c r="D4" t="n">
-        <v>2.08</v>
+        <v>2.29</v>
       </c>
       <c r="E4" t="n">
-        <v>14.93</v>
+        <v>15.16</v>
       </c>
     </row>
     <row r="5">
@@ -55481,16 +55481,16 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>16.32</v>
+        <v>16.129999</v>
       </c>
       <c r="C14" t="n">
-        <v>16.259</v>
+        <v>16.097</v>
       </c>
       <c r="D14" t="n">
         <v>0.625</v>
       </c>
       <c r="E14" t="n">
-        <v>0.20513</v>
+        <v>0.20515</v>
       </c>
     </row>
   </sheetData>
@@ -56633,7 +56633,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>-0.9320000000000001</v>
+        <v>-0.838</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -56641,7 +56641,7 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0.031</v>
+        <v>0.04</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -57008,19 +57008,19 @@
         <v>3.09</v>
       </c>
       <c r="D12" t="n">
-        <v>96.73999999999999</v>
+        <v>95.90000000000001</v>
       </c>
       <c r="E12" t="n">
-        <v>32.67</v>
+        <v>31.51</v>
       </c>
       <c r="F12" t="n">
-        <v>42.33</v>
+        <v>41.09</v>
       </c>
       <c r="G12" t="n">
-        <v>-7.36</v>
+        <v>-8.029999999999999</v>
       </c>
       <c r="H12" t="n">
-        <v>6.38</v>
+        <v>6.7</v>
       </c>
     </row>
   </sheetData>
@@ -57865,7 +57865,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>8.35</v>
+        <v>8.526</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -57873,10 +57873,10 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>-9.733000000000001</v>
+        <v>-9.34</v>
       </c>
       <c r="F15" t="n">
-        <v>18.084</v>
+        <v>17.866</v>
       </c>
     </row>
   </sheetData>
@@ -60810,16 +60810,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>-0.727</v>
+        <v>-0.528</v>
       </c>
       <c r="C15" t="n">
-        <v>2.085</v>
+        <v>2.29</v>
       </c>
       <c r="D15" t="n">
-        <v>17.265</v>
+        <v>17.501</v>
       </c>
       <c r="E15" t="n">
-        <v>14.929</v>
+        <v>15.16</v>
       </c>
       <c r="F15" t="n">
         <v>15.771</v>
@@ -61618,19 +61618,19 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>16.32</v>
+        <v>16.129999</v>
       </c>
       <c r="C14" t="n">
-        <v>20.202</v>
+        <v>20.201</v>
       </c>
       <c r="D14" t="n">
-        <v>0.02405</v>
+        <v>0.02404</v>
       </c>
       <c r="E14" t="n">
         <v>28.8</v>
       </c>
       <c r="F14" t="n">
-        <v>-3.882</v>
+        <v>-4.071</v>
       </c>
     </row>
   </sheetData>
@@ -66904,7 +66904,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>-0.004874</v>
+        <v>-0.004866</v>
       </c>
     </row>
   </sheetData>
@@ -68034,10 +68034,10 @@
         <v>0.008800000000000001</v>
       </c>
       <c r="C14" t="n">
-        <v>0.06809</v>
+        <v>0.06807000000000001</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.03845</v>
+        <v>-0.03844</v>
       </c>
     </row>
   </sheetData>
@@ -71240,10 +71240,10 @@
         <v>-1.107</v>
       </c>
       <c r="C15" t="n">
-        <v>2.4</v>
+        <v>2.401</v>
       </c>
       <c r="D15" t="n">
-        <v>0.42</v>
+        <v>0.421</v>
       </c>
     </row>
   </sheetData>
@@ -71503,13 +71503,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1.074</v>
+        <v>1.0899</v>
       </c>
       <c r="C15" t="n">
-        <v>1.0598</v>
+        <v>1.0758</v>
       </c>
       <c r="D15" t="n">
-        <v>1.5356</v>
+        <v>1.5578</v>
       </c>
     </row>
   </sheetData>
@@ -74650,7 +74650,7 @@
         <v>2263</v>
       </c>
       <c r="G15" t="n">
-        <v>0.01026</v>
+        <v>0.01027</v>
       </c>
     </row>
   </sheetData>
@@ -78098,7 +78098,7 @@
         </is>
       </c>
       <c r="E132" t="n">
-        <v>16.155</v>
+        <v>15.892</v>
       </c>
     </row>
     <row r="133">
@@ -78121,7 +78121,7 @@
         </is>
       </c>
       <c r="E133" t="n">
-        <v>6.933</v>
+        <v>7.607</v>
       </c>
     </row>
     <row r="134">
@@ -78144,7 +78144,7 @@
         </is>
       </c>
       <c r="E134" t="n">
-        <v>1.963</v>
+        <v>2.079</v>
       </c>
     </row>
     <row r="135">
@@ -78167,7 +78167,7 @@
         </is>
       </c>
       <c r="E135" t="n">
-        <v>0.485</v>
+        <v>0.746</v>
       </c>
     </row>
     <row r="136">
@@ -78190,7 +78190,7 @@
         </is>
       </c>
       <c r="E136" t="n">
-        <v>-1.89</v>
+        <v>-1.475</v>
       </c>
     </row>
     <row r="137">
@@ -78213,7 +78213,7 @@
         </is>
       </c>
       <c r="E137" t="n">
-        <v>-3.679</v>
+        <v>-3.433</v>
       </c>
     </row>
     <row r="138">
@@ -78236,7 +78236,7 @@
         </is>
       </c>
       <c r="E138" t="n">
-        <v>-6.507</v>
+        <v>-6.087</v>
       </c>
     </row>
     <row r="139">
@@ -78259,7 +78259,7 @@
         </is>
       </c>
       <c r="E139" t="n">
-        <v>-7.239</v>
+        <v>-6.945</v>
       </c>
     </row>
     <row r="140">
@@ -78282,7 +78282,7 @@
         </is>
       </c>
       <c r="E140" t="n">
-        <v>-8.981</v>
+        <v>-8.680999999999999</v>
       </c>
     </row>
     <row r="141">
@@ -78305,7 +78305,7 @@
         </is>
       </c>
       <c r="E141" t="n">
-        <v>-12.98</v>
+        <v>-12.395</v>
       </c>
     </row>
   </sheetData>
@@ -79169,16 +79169,16 @@
         <v>3705</v>
       </c>
       <c r="D15" t="n">
-        <v>0.01785</v>
+        <v>0.01791</v>
       </c>
       <c r="E15" t="n">
         <v>0.04655</v>
       </c>
       <c r="F15" t="n">
-        <v>-1.032</v>
+        <v>-1.03</v>
       </c>
       <c r="G15" t="n">
-        <v>0.3022</v>
+        <v>0.303</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -81131,10 +81131,10 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>-0.1877</v>
+        <v>-0.1904</v>
       </c>
       <c r="C15" t="n">
-        <v>1.0158</v>
+        <v>1.0224</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-29T21:30Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-29 20:09 UTC</t>
+          <t>Genere le 2026-09-29 21:30 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-29 20:09 UTC</t>
+          <t>Rapport global — 2026-09-29 21:30 UTC</t>
         </is>
       </c>
     </row>
@@ -617,21 +617,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>**Regime monetaire emploi** — Chine : taux 1.54% (stable, niveau bas) -- chomage non_couvert  _(sans synthese)_ _(observation : 2026-09-25)_</t>
+          <t>**Regime monetaire emploi** — Chine : taux 1.54% (stable, niveau bas) -- chomage non_couvert  _(sans synthese)_ _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>**Regle taylor** — Taylor (2 termes, sans output gap)=6.03%, Fed reel=3.88%, ecart=-2.15pt -- accommodant (Fed en-dessous de la regle) _(observation : 2026-09-25)_</t>
+          <t>**Regle taylor** — Taylor (2 termes, sans output gap)=6.03%, Fed reel=3.88%, ecart=-2.15pt -- accommodant (Fed en-dessous de la regle) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>**Chemin taux fed** — chemin de taux (pas des probabilites) : DFF=3.88%, prochaine reunion 2026-10-27 (11 a venir dans le calendrier) -- 0-1 mois: +16pb (hausse, confiance faible) | 1-3 mois: +46pb (hausse, confiance faible) | 3-6 mois: +54pb (hausse, confiance faible) | 6-12 mois: +79pb (hausse, confiance faible) _(observation : 2026-09-25)_</t>
+          <t>**Chemin taux fed** — chemin de taux (pas des probabilites) : DFF=3.88%, prochaine reunion 2026-10-27 (11 a venir dans le calendrier) -- 0-1 mois: +16pb (hausse, confiance faible) | 1-3 mois: +52pb (hausse, confiance faible) | 3-6 mois: +66pb (hausse, confiance faible) | 6-12 mois: +89pb (hausse, confiance faible) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>**Matieres premieres macro** — ratio cuivre/or stable -- pas de signal net sur la croissance (+3.1% sur 3 mois). Brent 95.9$ (+31.5% sur 3 mois, +41.1% sur 12 mois), gaz -8.0% sur 3 mois, ecart Brent-WTI +6.7$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-29)_</t>
+          <t>**Matieres premieres macro** — ratio cuivre/or stable -- pas de signal net sur la croissance (+3.0% sur 3 mois). Brent 95.7$ (+31.2% sur 3 mois, +40.8% sur 12 mois), gaz -8.0% sur 3 mois, ecart Brent-WTI +6.7$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -841,14 +841,14 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>**Taux reel us** — nominal=3.88%, inflation YoY=3.35%, reel=0.53% -- restrictif (taux reel positif et eleve) _(observation : 2026-09-25)_</t>
+          <t>**Taux reel us** — nominal=3.88%, inflation YoY=3.35%, reel=0.53% -- restrictif (taux reel positif et eleve) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>**Courbe taux us** — 10 ans=5.17%, 2 ans=4.81%, spread=+0.36pt -- normale (0 run(s) consecutif(s) dans l'historique accumule) _(observation : 2026-09-25)_</t>
+          <t>**Courbe taux us** — 10 ans=5.24%, 2 ans=4.92%, spread=+0.32pt -- normale (0 run(s) consecutif(s) dans l'historique accumule) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -862,7 +862,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>**Conditions financieres** — indice conditions financieres=+0.088 (3 composantes: {'taux_directeur': 0.5982151864455719, 'courbe_inversee': 0.17031877422284264, 'vix': -0.5039928815884913}) -- conditions proches de la normale _(observation : 2026-09-25)_</t>
+          <t>**Conditions financieres** — indice conditions financieres=+0.106 (3 composantes: {'taux_directeur': 0.5971439233898245, 'courbe_inversee': 0.23568763984021313, 'vix': -0.5151221380662802}) -- conditions proches de la normale _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -883,14 +883,14 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>**Stationnarite taux** — 1/5 series stationnaires (niveau, pas en difference) -- a garder en tete avant toute correlation/regression sur ces series telles quelles  _(sans synthese)_ _(observation : 2026-09-25)_</t>
+          <t>**Stationnarite taux** — 1/5 series stationnaires (niveau, pas en difference) -- a garder en tete avant toute correlation/regression sur ces series telles quelles  _(sans synthese)_ _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>**Cointegration taux** — 1/10 paires cointegrees  _(sans synthese)_ _(observation : 2026-09-25)_</t>
+          <t>**Cointegration taux** — 1/10 paires cointegrees  _(sans synthese)_ _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -904,7 +904,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>**Hp filter taux** — taux 10 ans observe=5.170%, tendance HP=4.983%, ecart cyclique=+0.187pt -- au-dessus de sa tendance locale _(observation : 2026-09-25)_</t>
+          <t>**Hp filter taux** — taux 10 ans observe=5.240%, tendance HP=5.011%, ecart cyclique=+0.229pt -- au-dessus de sa tendance locale _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -953,7 +953,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>**Differentiel taux change** — 8 paires testees sur variations a 21 jours -- le lien taux/change tient sur 6 paire(s) apres correction pour tests multiples : EURUSD, USDJPY, USDCAD, AUDUSD, USDSEK, EURJPY _(observation : 2026-09-24)_</t>
+          <t>**Differentiel taux change** — 8 paires testees sur variations a 21 jours -- le lien taux/change tient sur 5 paire(s) apres correction pour tests multiples : EURUSD, USDJPY, USDCAD, AUDUSD, EURJPY _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -981,7 +981,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>**Beta facteur macro** — beta SP500/DGS10 (60j) = -0.0794 (rendement SP500 pour +1pt de taux 10 ans, 57/60 jours avec variation reelle) -- sensibilite elevee au facteur macro (choc de +100pb extrapole = -7.6%) _(observation : 2026-09-25)_</t>
+          <t>**Beta facteur macro** — beta SP500/DGS10 (60j) = -0.0810 (rendement SP500 pour +1pt de taux 10 ans, 57/60 jours avec variation reelle) -- sensibilite elevee au facteur macro (choc de +100pb extrapole = -7.8%) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -995,21 +995,21 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>**Carry proxy** — Chine : 1.54% vs US 3.88% -- diff=-2.34pt (carry negatif (taux &lt; US))  _(sans synthese)_ _(observation : 2026-09-25)_</t>
+          <t>**Carry proxy** — Chine : 1.54% vs US 3.88% -- diff=-2.34pt (carry negatif (taux &lt; US))  _(sans synthese)_ _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>**Beta vol** — beta SP500/VIX (60j) = -0.00487 (rendement SP500 pour +1pt VIX) -- sensibilite normale, relation inverse attendue (normale) _(observation : 2026-09-29)_</t>
+          <t>**Beta vol** — beta SP500/VIX (60j) = -0.00486 (rendement SP500 pour +1pt VIX) -- sensibilite normale, relation inverse attendue (normale) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>**Rotation sectorielle** — classement momentum 3 mois (10 secteurs) : 1. Energie (XLE) : +15.89% | 2. Sante (XLV) : +7.61% | 3. Technologie (XLK) : +2.08% | 4. Finance (XLF) : +0.75% | 5. Consommation de base (XLP) : -1.48% _(observation : 2026-09-29)_</t>
+          <t>**Rotation sectorielle** — classement momentum 3 mois (10 secteurs) : 1. Energie (XLE) : +15.87% | 2. Sante (XLV) : +7.61% | 3. Technologie (XLK) : +2.09% | 4. Finance (XLF) : +0.75% | 5. Consommation de base (XLP) : -1.47% _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1030,14 +1030,14 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>**Low volatility** — tercile bas-vol ['XLF', 'XLRE', 'XLU'] Sharpe=-0.838 vs tercile haut-vol ['XLY', 'XLE', 'XLK'] Sharpe=0.040 -- anomalie low-vol non confirmee sur cet echantillon (puissance statistique faible, n petit -- limite assumee) _(observation : 2026-09-29)_</t>
+          <t>**Low volatility** — tercile bas-vol ['XLF', 'XLRE', 'XLU'] Sharpe=-0.842 vs tercile haut-vol ['XLY', 'XLE', 'XLK'] Sharpe=0.040 -- anomalie low-vol non confirmee sur cet echantillon (puissance statistique faible, n petit -- limite assumee) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>**Momentum cross sectional** — panier gagnant ['XLE', 'XLV', 'XLK'] (+8.53%) vs panier perdant ['XLY', 'XLI', 'XLU'] (-9.34%) -- spread momentum=+17.87pt _(observation : 2026-09-29)_</t>
+          <t>**Momentum cross sectional** — panier gagnant ['XLE', 'XLV', 'XLK'] (+8.52%) vs panier perdant ['XLY', 'XLI', 'XLU'] (-9.35%) -- spread momentum=+17.87pt _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>**Correlation facteurs** — correlation entre momentum 3m et beta-VIX, 10 secteurs : +0.360 (facteurs largement independants) _(observation : 2026-09-29)_</t>
+          <t>**Correlation facteurs** — correlation entre momentum 3m et beta-VIX, 10 secteurs : +0.361 (facteurs largement independants) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1191,14 +1191,14 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>**Vol cross asset** — 6 mesures de volatilite : Petrole (OVX) 86e pct, Or (GVZ) 85e pct, Taux US (MOVE) 58e pct, Nasdaq (VXN) 49e pct, Vol de la vol (VVIX) 34e pct, Actions US (VIX) 33e pct -- stress LOCALISE sur Petrole (OVX), Or (GVZ) pendant que le reste ne l'est pas -- episode propre a cette classe d'actifs, pas une aversion au risque d'ensemble _(observation : 2026-09-29)_</t>
+          <t>**Vol cross asset** — 6 mesures de volatilite : Petrole (OVX) 86e pct, Or (GVZ) 85e pct, Taux US (MOVE) 58e pct, Nasdaq (VXN) 48e pct, Vol de la vol (VVIX) 33e pct, Actions US (VIX) 32e pct -- stress LOCALISE sur Petrole (OVX), Or (GVZ) pendant que le reste ne l'est pas -- episode propre a cette classe d'actifs, pas une aversion au risque d'ensemble _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>**Volatilite ewma** — vol realisee 60j=0.11200610147428887, EWMA=0.1059 (tendance 10 runs: stable) _(observation : 2026-09-29)_</t>
+          <t>**Volatilite ewma** — vol realisee 60j=0.11200833249006233, EWMA=0.1059 (tendance 10 runs: stable) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1219,7 +1219,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>**Ornstein uhlenbeck vix** — VIX actuel=16.13, niveau moyen estime (mu)=20.20, demi-vie=28.8j, ecart actuel=-4.07 -- VIX actuel en-dessous de son niveau moyen de long terme _(observation : 2026-09-29)_</t>
+          <t>**Ornstein uhlenbeck vix** — VIX actuel=16.04, niveau moyen estime (mu)=20.20, demi-vie=28.8j, ecart actuel=-4.16 -- VIX actuel en-dessous de son niveau moyen de long terme _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1233,14 +1233,14 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>**Kalman niveau local** — VIX observe=16.13, filtre Kalman=16.10 (ecart-type=0.62), ratio signal/bruit=0.2051 -- le filtre lisse fortement le bruit, reagit lentement (ecart obs.-filtre=+0.03) _(observation : 2026-09-29)_</t>
+          <t>**Kalman niveau local** — VIX observe=16.04, filtre Kalman=16.02 (ecart-type=0.62), ratio signal/bruit=0.2052 -- le filtre lisse fortement le bruit, reagit lentement (ecart obs.-filtre=+0.02) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.37204216230183995 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.052351167944674745 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-29)_</t>
+          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.3726482026081239 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.05235096605723792 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1268,7 +1268,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>**Ratios performance** — Sharpe=1.090 (bon), Sortino=1.076 (bon), Calmar=1.558 (bon) -- lecture sur fenetre 252j (~1 an, echantillon limite), seuils academiques standards, taux sans risque suppose nul _(observation : 2026-09-29)_</t>
+          <t>**Ratios performance** — Sharpe=1.090 (bon), Sortino=1.076 (bon), Calmar=1.557 (bon) -- lecture sur fenetre 252j (~1 an, echantillon limite), seuils academiques standards, taux sans risque suppose nul _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1303,21 +1303,21 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>**Detection saut** — Z-stat BNS (fenetre 22j)=0.973 (seuil ±1.96) -- pas de saut isole detecte _(observation : 2026-09-29)_</t>
+          <t>**Detection saut** — Z-stat BNS (fenetre 22j)=0.970 (seuil ±1.96) -- pas de saut isole detecte _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>**Choc taux** — beta SP500/DGS10=-0.0794 -- choc +100pb : -7.94% (SP500 7743 -&gt; 7129) ; choc -100pb : +7.94% (-&gt; 8358) _(observation : 2026-09-25)_</t>
+          <t>**Choc taux** — beta SP500/DGS10=-0.0810 -- choc +100pb : -8.10% (SP500 7684 -&gt; 7061) ; choc -100pb : +8.10% (-&gt; 8306) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>**Qualite regime macro** — instabilite taux=0.0088, instabilite VIX=0.0681 -- score qualite du regime=-0.0384 (plus haut = regime plus stable/previsible) _(observation : 2026-09-25)_</t>
+          <t>**Qualite regime macro** — instabilite taux=0.0088, instabilite VIX=0.0681 -- score qualite du regime=-0.0384 (plus haut = regime plus stable/previsible) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1331,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>**Decomposition stl** — VIX : tendance=15.54, composante saisonniere (periode 5j)=+0.616, residu=-0.027 -- la saisonnalite explique 0.72% de la variance totale (negligeable) _(observation : 2026-09-29)_</t>
+          <t>**Decomposition stl** — VIX : tendance=15.52, composante saisonniere (periode 5j)=+0.586, residu=-0.064 -- la saisonnalite explique 0.72% de la variance totale (negligeable) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1387,7 +1387,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>**Anomalie multivariee** — distance de Mahalanobis=0.424 (seuil 3.0) -- jour ordinaire _(observation : 2026-09-29)_</t>
+          <t>**Anomalie multivariee** — distance de Mahalanobis=0.512 (seuil 3.0) -- jour ordinaire _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1408,7 +1408,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>**Kmeans regimes** — 2050 points, k=3 -- point actuel (VIX=14.9, spread=+0.36, taux=3.88%) -&gt; cluster 1 (tailles : {0: 357, 1: 1369, 2: 324}) -- regime calme (VIX du cluster en-dessous de la moyenne historique) _(observation : 2026-09-25)_</t>
+          <t>**Kmeans regimes** — 2048 points, k=3 -- point actuel (VIX=16.1, spread=+0.32, taux=3.88%) -&gt; cluster 1 (tailles : {0: 357, 1: 1367, 2: 324}) -- regime calme (VIX du cluster en-dessous de la moyenne historique) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1443,14 +1443,14 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>**Decomposition variance** — R² SP500~DGS10 (60j) = 0.2703 -- 27.0% de la variance des rendements SP500 expliquee par les variations du taux 10 ans (le reste = idiosyncratique/autres facteurs) _(observation : 2026-09-25)_</t>
+          <t>**Decomposition variance** — R² SP500~DGS10 (60j) = 0.2827 -- 28.3% de la variance des rendements SP500 expliquee par les variations du taux 10 ans (le reste = idiosyncratique/autres facteurs) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>**Test chow** — test de Chow (taux 10 ans, 1ere vs 2eme moitie des 12 derniers mois) : F=560.405, p=0.0000 -- RUPTURE structurelle significative _(observation : 2026-09-25)_</t>
+          <t>**Test chow** — test de Chow (taux 10 ans, 1ere vs 2eme moitie des 12 derniers mois) : F=547.278, p=0.0000 -- RUPTURE structurelle significative _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1493,7 +1493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2619,6 +2619,90 @@
         <v>3.88</v>
       </c>
       <c r="E53" t="n">
+        <v>-2.34</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Zone_euro</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D54" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="E54" t="n">
+        <v>-1.38</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Royaume-Uni</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>3.73</v>
+      </c>
+      <c r="D55" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="E55" t="n">
+        <v>-0.15</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Japon</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>0.977</v>
+      </c>
+      <c r="D56" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="E56" t="n">
+        <v>-2.903</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Chine</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="D57" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="E57" t="n">
         <v>-2.34</v>
       </c>
     </row>
@@ -3091,7 +3175,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F66"/>
+  <dimension ref="A1:F71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4949,6 +5033,146 @@
         <v>0.0002</v>
       </c>
       <c r="F66" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>DFF</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>-0.504</v>
+      </c>
+      <c r="E67" t="n">
+        <v>0.8912</v>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Zone_euro</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>ECBDFR</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>-0.5827</v>
+      </c>
+      <c r="E68" t="n">
+        <v>0.8748</v>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Royaume-Uni</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>IUDSOIA</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>-0.159</v>
+      </c>
+      <c r="E69" t="n">
+        <v>0.9432</v>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Japon</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>IRSTCI01JPM156N</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>-1.9195</v>
+      </c>
+      <c r="E70" t="n">
+        <v>0.3229</v>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Chine</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>IR3TIB01CNM156N</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>-4.4511</v>
+      </c>
+      <c r="E71" t="n">
+        <v>0.0002</v>
+      </c>
+      <c r="F71" t="inlineStr">
         <is>
           <t>True</t>
         </is>
@@ -5761,7 +5985,7 @@
         <v>-56.78</v>
       </c>
       <c r="F28" t="n">
-        <v>3315.79</v>
+        <v>3315.69</v>
       </c>
     </row>
     <row r="29">
@@ -5789,7 +6013,7 @@
         <v>-33.92</v>
       </c>
       <c r="F29" t="n">
-        <v>5068.66</v>
+        <v>5068.51</v>
       </c>
     </row>
   </sheetData>
@@ -5953,7 +6177,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6189,6 +6413,22 @@
         <v>3.353</v>
       </c>
       <c r="D14" t="n">
+        <v>0.527</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="C15" t="n">
+        <v>3.353</v>
+      </c>
+      <c r="D15" t="n">
         <v>0.527</v>
       </c>
     </row>
@@ -6203,7 +6443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6463,6 +6703,24 @@
         <v>0</v>
       </c>
       <c r="D14" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>547.278</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" t="inlineStr">
         <is>
           <t>True</t>
         </is>
@@ -8689,7 +8947,7 @@
         <v>10</v>
       </c>
       <c r="C15" t="n">
-        <v>0.37204</v>
+        <v>0.37265</v>
       </c>
       <c r="D15" t="n">
         <v>-0.052351</v>
@@ -8761,7 +9019,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>53.65</v>
+        <v>53.74</v>
       </c>
       <c r="D2" t="n">
         <v>85.90000000000001</v>
@@ -8787,10 +9045,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>24.27</v>
+        <v>24.37</v>
       </c>
       <c r="D3" t="n">
-        <v>84.8</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="E3" t="n">
         <v>1260</v>
@@ -8839,10 +9097,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>22.34</v>
+        <v>22.07</v>
       </c>
       <c r="D5" t="n">
-        <v>49.4</v>
+        <v>47.5</v>
       </c>
       <c r="E5" t="n">
         <v>1260</v>
@@ -8865,10 +9123,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>90.08</v>
+        <v>89.70999999999999</v>
       </c>
       <c r="D6" t="n">
-        <v>34.5</v>
+        <v>33.3</v>
       </c>
       <c r="E6" t="n">
         <v>1260</v>
@@ -8891,10 +9149,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>16.13</v>
+        <v>16.04</v>
       </c>
       <c r="D7" t="n">
-        <v>33.4</v>
+        <v>32.3</v>
       </c>
       <c r="E7" t="n">
         <v>1260</v>
@@ -9914,7 +10172,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J29"/>
+  <dimension ref="A1:J33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11269,6 +11527,190 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>0-1 mois</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" t="n">
+        <v>4.04</v>
+      </c>
+      <c r="F30" t="n">
+        <v>16</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>hausse</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>forward_treasury_proxy</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>mouvement net de fenetre; aucune probabilite isolee par reunion</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>1-3 mois</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>2026-12-28</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>2</v>
+      </c>
+      <c r="E31" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="F31" t="n">
+        <v>52</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>hausse</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>forward_treasury_proxy</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>mouvement net de fenetre; aucune probabilite isolee par reunion</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>3-6 mois</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>2027-03-29</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>5</v>
+      </c>
+      <c r="E32" t="n">
+        <v>4.54</v>
+      </c>
+      <c r="F32" t="n">
+        <v>66</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>hausse</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>forward_treasury_proxy</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>mouvement net de fenetre; aucune probabilite isolee par reunion</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>6-12 mois</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>2027-09-28</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>9</v>
+      </c>
+      <c r="E33" t="n">
+        <v>4.77</v>
+      </c>
+      <c r="F33" t="n">
+        <v>89</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>hausse</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>forward_treasury_proxy</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>mouvement net de fenetre; aucune probabilite isolee par reunion</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11280,7 +11722,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11652,6 +12094,31 @@
       </c>
       <c r="G14" t="n">
         <v>8358</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>-0.08103</v>
+      </c>
+      <c r="C15" t="n">
+        <v>7683.69</v>
+      </c>
+      <c r="D15" t="n">
+        <v>-8.1</v>
+      </c>
+      <c r="E15" t="n">
+        <v>7061.1</v>
+      </c>
+      <c r="F15" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="G15" t="n">
+        <v>8306.299999999999</v>
       </c>
     </row>
   </sheetData>
@@ -16841,10 +17308,10 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>-2.5118</v>
+        <v>-2.5102</v>
       </c>
       <c r="D132" t="n">
-        <v>0.2739</v>
+        <v>0.2746</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -16864,10 +17331,10 @@
         </is>
       </c>
       <c r="C133" t="n">
-        <v>-1.8329</v>
+        <v>-1.8331</v>
       </c>
       <c r="D133" t="n">
-        <v>0.6136</v>
+        <v>0.6135</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -16887,7 +17354,7 @@
         </is>
       </c>
       <c r="C134" t="n">
-        <v>-2.1418</v>
+        <v>-2.1416</v>
       </c>
       <c r="D134" t="n">
         <v>0.4546</v>
@@ -16933,10 +17400,10 @@
         </is>
       </c>
       <c r="C136" t="n">
-        <v>-1.4407</v>
+        <v>-1.4392</v>
       </c>
       <c r="D136" t="n">
-        <v>0.7832</v>
+        <v>0.7837</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -16956,10 +17423,10 @@
         </is>
       </c>
       <c r="C137" t="n">
-        <v>0.0391</v>
+        <v>0.0363</v>
       </c>
       <c r="D137" t="n">
-        <v>0.9868</v>
+        <v>0.9867</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -16979,10 +17446,10 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>-1.196</v>
+        <v>-1.1968</v>
       </c>
       <c r="D138" t="n">
-        <v>0.8589</v>
+        <v>0.8587</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -17002,10 +17469,10 @@
         </is>
       </c>
       <c r="C139" t="n">
-        <v>-0.7012</v>
+        <v>-0.698</v>
       </c>
       <c r="D139" t="n">
-        <v>0.9465</v>
+        <v>0.9469</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -17025,10 +17492,10 @@
         </is>
       </c>
       <c r="C140" t="n">
-        <v>-2.1228</v>
+        <v>-2.1262</v>
       </c>
       <c r="D140" t="n">
-        <v>0.4644</v>
+        <v>0.4627</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -17048,10 +17515,10 @@
         </is>
       </c>
       <c r="C141" t="n">
-        <v>-1.6207</v>
+        <v>-1.6182</v>
       </c>
       <c r="D141" t="n">
-        <v>0.7121</v>
+        <v>0.7131</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -17070,7 +17537,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F131"/>
+  <dimension ref="A1:F141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -20748,6 +21215,286 @@
         <v>0.7186</v>
       </c>
       <c r="F131" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Chine</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Japon</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>-3.6969</v>
+      </c>
+      <c r="E132" t="n">
+        <v>0.0185</v>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Chine</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Royaume-Uni</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>-2.417</v>
+      </c>
+      <c r="E133" t="n">
+        <v>0.3168</v>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Chine</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>-2.0335</v>
+      </c>
+      <c r="E134" t="n">
+        <v>0.5111</v>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Chine</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Zone_euro</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>-2.1259</v>
+      </c>
+      <c r="E135" t="n">
+        <v>0.4628</v>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Japon</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Royaume-Uni</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>-1.975</v>
+      </c>
+      <c r="E136" t="n">
+        <v>0.5415</v>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Japon</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>-0.3664</v>
+      </c>
+      <c r="E137" t="n">
+        <v>0.9726</v>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Japon</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Zone_euro</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>-0.7129</v>
+      </c>
+      <c r="E138" t="n">
+        <v>0.9452</v>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Royaume-Uni</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>-1.9872</v>
+      </c>
+      <c r="E139" t="n">
+        <v>0.5352</v>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Royaume-Uni</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Zone_euro</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>-2.2113</v>
+      </c>
+      <c r="E140" t="n">
+        <v>0.4185</v>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Zone_euro</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>-1.6087</v>
+      </c>
+      <c r="E141" t="n">
+        <v>0.7171999999999999</v>
+      </c>
+      <c r="F141" t="inlineStr">
         <is>
           <t>False</t>
         </is>
@@ -23565,7 +24312,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -23892,6 +24639,28 @@
       </c>
       <c r="F14" t="n">
         <v>-0.504</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0.1059</v>
+      </c>
+      <c r="C15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.5971</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.2357</v>
+      </c>
+      <c r="F15" t="n">
+        <v>-0.5151</v>
       </c>
     </row>
   </sheetData>
@@ -24179,7 +24948,7 @@
         <v>10</v>
       </c>
       <c r="C15" t="n">
-        <v>0.36</v>
+        <v>0.3607</v>
       </c>
     </row>
   </sheetData>
@@ -35819,7 +36588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -36124,6 +36893,27 @@
         <v>0.36</v>
       </c>
       <c r="E14" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>5.24</v>
+      </c>
+      <c r="C15" t="n">
+        <v>4.92</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="E15" t="inlineStr">
         <is>
           <t>False</t>
         </is>
@@ -36861,19 +37651,19 @@
         <v>2.2</v>
       </c>
       <c r="C14" t="n">
-        <v>428.56</v>
+        <v>428.43</v>
       </c>
       <c r="D14" t="n">
         <v>4</v>
       </c>
       <c r="E14" t="n">
-        <v>354.8</v>
+        <v>354.78</v>
       </c>
       <c r="F14" t="n">
         <v>5.4</v>
       </c>
       <c r="G14" t="n">
-        <v>351.77</v>
+        <v>351.67</v>
       </c>
     </row>
   </sheetData>
@@ -38319,13 +39109,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>15.541</v>
+        <v>15.519</v>
       </c>
       <c r="C14" t="n">
-        <v>0.616</v>
+        <v>0.586</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.027</v>
+        <v>-0.064</v>
       </c>
       <c r="E14" t="n">
         <v>0.72</v>
@@ -38342,7 +39132,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -38534,6 +39324,19 @@
       </c>
       <c r="C14" t="n">
         <v>27.03</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0.28274</v>
+      </c>
+      <c r="C15" t="n">
+        <v>28.27</v>
       </c>
     </row>
   </sheetData>
@@ -39181,7 +39984,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.973</v>
+        <v>0.97</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -39260,17 +40063,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>-1.641</v>
+        <v>-1.687</v>
       </c>
       <c r="D2" t="n">
-        <v>0.314</v>
+        <v>0.403</v>
       </c>
       <c r="E2" t="n">
-        <v>0.00054</v>
+        <v>1e-05</v>
       </c>
       <c r="F2" t="n">
         <v>118</v>
@@ -39296,7 +40099,7 @@
         <v>2.597</v>
       </c>
       <c r="D3" t="n">
-        <v>0.513</v>
+        <v>0.5590000000000001</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
@@ -39325,10 +40128,10 @@
         <v>-0.106</v>
       </c>
       <c r="D4" t="n">
-        <v>0.134</v>
+        <v>0.061</v>
       </c>
       <c r="E4" t="n">
-        <v>0.14953</v>
+        <v>0.51607</v>
       </c>
       <c r="F4" t="n">
         <v>117</v>
@@ -39347,14 +40150,14 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1.48</v>
+        <v>1.55</v>
       </c>
       <c r="D5" t="n">
-        <v>0.505</v>
+        <v>0.419</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
@@ -39383,10 +40186,10 @@
         <v>0.097</v>
       </c>
       <c r="D6" t="n">
-        <v>0.342</v>
+        <v>0.278</v>
       </c>
       <c r="E6" t="n">
-        <v>0.00017</v>
+        <v>0.00251</v>
       </c>
       <c r="F6" t="n">
         <v>116</v>
@@ -39405,24 +40208,24 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2.08</v>
+        <v>2.127</v>
       </c>
       <c r="D7" t="n">
-        <v>0.307</v>
+        <v>0.232</v>
       </c>
       <c r="E7" t="n">
-        <v>0.0008</v>
+        <v>0.0121</v>
       </c>
       <c r="F7" t="n">
         <v>116</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>oui</t>
+          <t>non</t>
         </is>
       </c>
     </row>
@@ -39812,13 +40615,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>-0.00164</v>
+        <v>-0.00167</v>
       </c>
       <c r="C15" t="n">
-        <v>0.06</v>
+        <v>-0.03</v>
       </c>
       <c r="D15" t="n">
-        <v>0.424</v>
+        <v>0.512</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -40131,13 +40934,13 @@
         <v>10</v>
       </c>
       <c r="C15" t="n">
-        <v>-1.269</v>
+        <v>-1.271</v>
       </c>
       <c r="D15" t="n">
         <v>7.921</v>
       </c>
       <c r="E15" t="n">
-        <v>28.287</v>
+        <v>28.29</v>
       </c>
     </row>
   </sheetData>
@@ -40468,7 +41271,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>-0.528</v>
+        <v>-0.531</v>
       </c>
       <c r="C15" t="n">
         <v>-133228</v>
@@ -50469,7 +51272,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>fred/DFF.csv</t>
+          <t>fred/IUDSOIA.csv</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -50498,7 +51301,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>fred/DFII10.csv</t>
+          <t>souverains/UK_10A.csv</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -50516,7 +51319,7 @@
         <v>42</v>
       </c>
       <c r="F188" t="n">
-        <v>3000</v>
+        <v>9284</v>
       </c>
       <c r="G188" t="inlineStr">
         <is>
@@ -50527,7 +51330,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>fred/DFII5.csv</t>
+          <t>souverains/UK_20A.csv</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -50545,7 +51348,7 @@
         <v>42</v>
       </c>
       <c r="F189" t="n">
-        <v>3000</v>
+        <v>6755</v>
       </c>
       <c r="G189" t="inlineStr">
         <is>
@@ -50556,7 +51359,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>fred/DGS1.csv</t>
+          <t>souverains/UK_5A.csv</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -50574,7 +51377,7 @@
         <v>42</v>
       </c>
       <c r="F190" t="n">
-        <v>3000</v>
+        <v>8292</v>
       </c>
       <c r="G190" t="inlineStr">
         <is>
@@ -50585,16 +51388,16 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>fred/DGS10.csv</t>
+          <t>fred/BAMLC0A0CM.csv</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C191" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D191" t="n">
         <v>1</v>
@@ -50603,7 +51406,7 @@
         <v>42</v>
       </c>
       <c r="F191" t="n">
-        <v>3000</v>
+        <v>793</v>
       </c>
       <c r="G191" t="inlineStr">
         <is>
@@ -50614,16 +51417,16 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>fred/DGS1MO.csv</t>
+          <t>fred/BAMLC0A0CMEY.csv</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C192" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D192" t="n">
         <v>1</v>
@@ -50632,7 +51435,7 @@
         <v>42</v>
       </c>
       <c r="F192" t="n">
-        <v>3000</v>
+        <v>793</v>
       </c>
       <c r="G192" t="inlineStr">
         <is>
@@ -50643,16 +51446,16 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>fred/DGS2.csv</t>
+          <t>fred/BAMLEMCBPIOAS.csv</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C193" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D193" t="n">
         <v>1</v>
@@ -50661,7 +51464,7 @@
         <v>42</v>
       </c>
       <c r="F193" t="n">
-        <v>3000</v>
+        <v>793</v>
       </c>
       <c r="G193" t="inlineStr">
         <is>
@@ -50672,16 +51475,16 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>fred/DGS30.csv</t>
+          <t>fred/BAMLEMFSFCRPIOAS.csv</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C194" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D194" t="n">
         <v>1</v>
@@ -50690,7 +51493,7 @@
         <v>42</v>
       </c>
       <c r="F194" t="n">
-        <v>3000</v>
+        <v>793</v>
       </c>
       <c r="G194" t="inlineStr">
         <is>
@@ -50701,16 +51504,16 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>fred/DGS3MO.csv</t>
+          <t>fred/BAMLEMHBHYCRPIOAS.csv</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C195" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D195" t="n">
         <v>1</v>
@@ -50719,7 +51522,7 @@
         <v>42</v>
       </c>
       <c r="F195" t="n">
-        <v>3000</v>
+        <v>793</v>
       </c>
       <c r="G195" t="inlineStr">
         <is>
@@ -50730,16 +51533,16 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>fred/DGS5.csv</t>
+          <t>fred/BAMLEMPBPUBSICRPIOAS.csv</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C196" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D196" t="n">
         <v>1</v>
@@ -50748,7 +51551,7 @@
         <v>42</v>
       </c>
       <c r="F196" t="n">
-        <v>3000</v>
+        <v>793</v>
       </c>
       <c r="G196" t="inlineStr">
         <is>
@@ -50759,16 +51562,16 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>fred/DGS6MO.csv</t>
+          <t>fred/BAMLH0A0HYM2.csv</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C197" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D197" t="n">
         <v>1</v>
@@ -50777,7 +51580,7 @@
         <v>42</v>
       </c>
       <c r="F197" t="n">
-        <v>3000</v>
+        <v>793</v>
       </c>
       <c r="G197" t="inlineStr">
         <is>
@@ -50788,16 +51591,16 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>fred/IUDSOIA.csv</t>
+          <t>fred/BAMLHE00EHYIEY.csv</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C198" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D198" t="n">
         <v>1</v>
@@ -50806,7 +51609,7 @@
         <v>42</v>
       </c>
       <c r="F198" t="n">
-        <v>3000</v>
+        <v>793</v>
       </c>
       <c r="G198" t="inlineStr">
         <is>
@@ -50817,16 +51620,16 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>souverains/UK_10A.csv</t>
+          <t>fred/BAMLHE00EHYIOAS.csv</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C199" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D199" t="n">
         <v>1</v>
@@ -50835,7 +51638,7 @@
         <v>42</v>
       </c>
       <c r="F199" t="n">
-        <v>9284</v>
+        <v>793</v>
       </c>
       <c r="G199" t="inlineStr">
         <is>
@@ -50846,16 +51649,16 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>souverains/UK_20A.csv</t>
+          <t>fred/DFF.csv</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C200" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D200" t="n">
         <v>1</v>
@@ -50864,7 +51667,7 @@
         <v>42</v>
       </c>
       <c r="F200" t="n">
-        <v>6755</v>
+        <v>3000</v>
       </c>
       <c r="G200" t="inlineStr">
         <is>
@@ -50875,16 +51678,16 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>souverains/UK_5A.csv</t>
+          <t>fred/DFII10.csv</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C201" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D201" t="n">
         <v>1</v>
@@ -50893,7 +51696,7 @@
         <v>42</v>
       </c>
       <c r="F201" t="n">
-        <v>8292</v>
+        <v>3000</v>
       </c>
       <c r="G201" t="inlineStr">
         <is>
@@ -50904,16 +51707,16 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>tresor_us/dette_quotidienne.csv</t>
+          <t>fred/DFII5.csv</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C202" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D202" t="n">
         <v>1</v>
@@ -50922,7 +51725,7 @@
         <v>42</v>
       </c>
       <c r="F202" t="n">
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="G202" t="inlineStr">
         <is>
@@ -50933,7 +51736,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>fred/BAMLC0A0CM.csv</t>
+          <t>fred/DGS1.csv</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -50951,7 +51754,7 @@
         <v>42</v>
       </c>
       <c r="F203" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G203" t="inlineStr">
         <is>
@@ -50962,7 +51765,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>fred/BAMLC0A0CMEY.csv</t>
+          <t>fred/DGS10.csv</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
@@ -50980,7 +51783,7 @@
         <v>42</v>
       </c>
       <c r="F204" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G204" t="inlineStr">
         <is>
@@ -50991,7 +51794,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>fred/BAMLEMCBPIOAS.csv</t>
+          <t>fred/DGS1MO.csv</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -51009,7 +51812,7 @@
         <v>42</v>
       </c>
       <c r="F205" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G205" t="inlineStr">
         <is>
@@ -51020,7 +51823,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>fred/BAMLEMFSFCRPIOAS.csv</t>
+          <t>fred/DGS2.csv</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -51038,7 +51841,7 @@
         <v>42</v>
       </c>
       <c r="F206" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G206" t="inlineStr">
         <is>
@@ -51049,7 +51852,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>fred/BAMLEMHBHYCRPIOAS.csv</t>
+          <t>fred/DGS30.csv</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -51067,7 +51870,7 @@
         <v>42</v>
       </c>
       <c r="F207" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G207" t="inlineStr">
         <is>
@@ -51078,7 +51881,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>fred/BAMLEMPBPUBSICRPIOAS.csv</t>
+          <t>fred/DGS3MO.csv</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -51096,7 +51899,7 @@
         <v>42</v>
       </c>
       <c r="F208" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G208" t="inlineStr">
         <is>
@@ -51107,7 +51910,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>fred/BAMLH0A0HYM2.csv</t>
+          <t>fred/DGS5.csv</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -51125,7 +51928,7 @@
         <v>42</v>
       </c>
       <c r="F209" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G209" t="inlineStr">
         <is>
@@ -51136,7 +51939,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>fred/BAMLHE00EHYIEY.csv</t>
+          <t>fred/DGS6MO.csv</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -51154,7 +51957,7 @@
         <v>42</v>
       </c>
       <c r="F210" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G210" t="inlineStr">
         <is>
@@ -51165,7 +51968,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>fred/BAMLHE00EHYIOAS.csv</t>
+          <t>marches/indices/HANGSENG.csv</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
@@ -51183,7 +51986,7 @@
         <v>42</v>
       </c>
       <c r="F211" t="n">
-        <v>793</v>
+        <v>3688</v>
       </c>
       <c r="G211" t="inlineStr">
         <is>
@@ -51194,7 +51997,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>fred/T10YIE.csv</t>
+          <t>marches/indices/KOSPI.csv</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -51212,7 +52015,7 @@
         <v>42</v>
       </c>
       <c r="F212" t="n">
-        <v>3000</v>
+        <v>3680</v>
       </c>
       <c r="G212" t="inlineStr">
         <is>
@@ -51223,7 +52026,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>marches/indices/HANGSENG.csv</t>
+          <t>marches/indices/NIKKEI225.csv</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -51241,7 +52044,7 @@
         <v>42</v>
       </c>
       <c r="F213" t="n">
-        <v>3688</v>
+        <v>3666</v>
       </c>
       <c r="G213" t="inlineStr">
         <is>
@@ -51252,7 +52055,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>marches/indices/KOSPI.csv</t>
+          <t>souverains/CANADA_10A.csv</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -51270,7 +52073,7 @@
         <v>42</v>
       </c>
       <c r="F214" t="n">
-        <v>3680</v>
+        <v>6437</v>
       </c>
       <c r="G214" t="inlineStr">
         <is>
@@ -51281,7 +52084,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>marches/indices/NIKKEI225.csv</t>
+          <t>souverains/CANADA_2A.csv</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -51299,7 +52102,7 @@
         <v>42</v>
       </c>
       <c r="F215" t="n">
-        <v>3666</v>
+        <v>6436</v>
       </c>
       <c r="G215" t="inlineStr">
         <is>
@@ -51310,7 +52113,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>souverains/CANADA_10A.csv</t>
+          <t>souverains/CANADA_5A.csv</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -51328,7 +52131,7 @@
         <v>42</v>
       </c>
       <c r="F216" t="n">
-        <v>6437</v>
+        <v>6436</v>
       </c>
       <c r="G216" t="inlineStr">
         <is>
@@ -51339,7 +52142,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>souverains/CANADA_2A.csv</t>
+          <t>souverains/CANADA_LONG.csv</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -51368,7 +52171,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>souverains/CANADA_5A.csv</t>
+          <t>souverains/SUEDE_10A.csv</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -51386,7 +52189,7 @@
         <v>42</v>
       </c>
       <c r="F218" t="n">
-        <v>6436</v>
+        <v>9203</v>
       </c>
       <c r="G218" t="inlineStr">
         <is>
@@ -51397,7 +52200,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>souverains/CANADA_LONG.csv</t>
+          <t>souverains/SUEDE_2A.csv</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -51415,7 +52218,7 @@
         <v>42</v>
       </c>
       <c r="F219" t="n">
-        <v>6436</v>
+        <v>9203</v>
       </c>
       <c r="G219" t="inlineStr">
         <is>
@@ -51426,7 +52229,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_10A.csv</t>
+          <t>souverains/SUEDE_5A.csv</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -51444,7 +52247,7 @@
         <v>42</v>
       </c>
       <c r="F220" t="n">
-        <v>9203</v>
+        <v>9205</v>
       </c>
       <c r="G220" t="inlineStr">
         <is>
@@ -51455,7 +52258,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_2A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -51473,7 +52276,7 @@
         <v>42</v>
       </c>
       <c r="F221" t="n">
-        <v>9203</v>
+        <v>5640</v>
       </c>
       <c r="G221" t="inlineStr">
         <is>
@@ -51484,7 +52287,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_5A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -51502,7 +52305,7 @@
         <v>42</v>
       </c>
       <c r="F222" t="n">
-        <v>9205</v>
+        <v>5640</v>
       </c>
       <c r="G222" t="inlineStr">
         <is>
@@ -51513,7 +52316,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -51542,7 +52345,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -51571,7 +52374,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
@@ -51600,7 +52403,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -51629,7 +52432,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -51658,7 +52461,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -51687,7 +52490,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
+          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -51716,7 +52519,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
+          <t>tresor_us/dette_quotidienne.csv</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -51734,7 +52537,7 @@
         <v>42</v>
       </c>
       <c r="F230" t="n">
-        <v>5640</v>
+        <v>2000</v>
       </c>
       <c r="G230" t="inlineStr">
         <is>
@@ -51745,7 +52548,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
+          <t>tresor_us/solde_tresorerie.csv</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -51763,7 +52566,7 @@
         <v>42</v>
       </c>
       <c r="F231" t="n">
-        <v>5640</v>
+        <v>500</v>
       </c>
       <c r="G231" t="inlineStr">
         <is>
@@ -51774,16 +52577,16 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>tresor_us/solde_tresorerie.csv</t>
+          <t>fred/ECBDFR.csv</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C232" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D232" t="n">
         <v>1</v>
@@ -51792,7 +52595,7 @@
         <v>42</v>
       </c>
       <c r="F232" t="n">
-        <v>500</v>
+        <v>3000</v>
       </c>
       <c r="G232" t="inlineStr">
         <is>
@@ -51803,7 +52606,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>fred/ECBDFR.csv</t>
+          <t>fred/RRPONTSYD.csv</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -51832,7 +52635,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>fred/RRPONTSYD.csv</t>
+          <t>fred/T10YIE.csv</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -53795,7 +54598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -54032,6 +54835,22 @@
       </c>
       <c r="D14" t="n">
         <v>0.1866</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>5.24</v>
+      </c>
+      <c r="C15" t="n">
+        <v>5.0108</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.2292</v>
       </c>
     </row>
   </sheetData>
@@ -54696,7 +55515,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>7671.07</v>
+        <v>7670.84</v>
       </c>
       <c r="D4" t="n">
         <v>2.29</v>
@@ -55481,10 +56300,10 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>16.129999</v>
+        <v>16.040001</v>
       </c>
       <c r="C14" t="n">
-        <v>16.097</v>
+        <v>16.02</v>
       </c>
       <c r="D14" t="n">
         <v>0.625</v>
@@ -55504,7 +56323,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -55856,6 +56675,30 @@
       <c r="F14" t="inlineStr">
         <is>
           <t>{0: 357, 1: 1369, 2: 324}</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>16.07</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="D15" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>{0: 357, 1: 1367, 2: 324}</t>
         </is>
       </c>
     </row>
@@ -56633,7 +57476,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>-0.838</v>
+        <v>-0.842</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -57002,25 +57845,25 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.001581</v>
+        <v>0.00158</v>
       </c>
       <c r="C12" t="n">
-        <v>3.09</v>
+        <v>3.02</v>
       </c>
       <c r="D12" t="n">
-        <v>95.90000000000001</v>
+        <v>95.67</v>
       </c>
       <c r="E12" t="n">
-        <v>31.51</v>
+        <v>31.2</v>
       </c>
       <c r="F12" t="n">
-        <v>41.09</v>
+        <v>40.75</v>
       </c>
       <c r="G12" t="n">
-        <v>-8.029999999999999</v>
+        <v>-7.97</v>
       </c>
       <c r="H12" t="n">
-        <v>6.7</v>
+        <v>6.73</v>
       </c>
     </row>
   </sheetData>
@@ -57865,7 +58708,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>8.526</v>
+        <v>8.523</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -57873,10 +58716,10 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>-9.34</v>
+        <v>-9.347</v>
       </c>
       <c r="F15" t="n">
-        <v>17.866</v>
+        <v>17.87</v>
       </c>
     </row>
   </sheetData>
@@ -57890,7 +58733,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -58081,6 +58924,19 @@
         <v>-0.07937</v>
       </c>
       <c r="C14" t="n">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>-0.08103</v>
+      </c>
+      <c r="C15" t="n">
         <v>57</v>
       </c>
     </row>
@@ -60810,16 +61666,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>-0.528</v>
+        <v>-0.531</v>
       </c>
       <c r="C15" t="n">
-        <v>2.29</v>
+        <v>2.287</v>
       </c>
       <c r="D15" t="n">
-        <v>17.501</v>
+        <v>17.497</v>
       </c>
       <c r="E15" t="n">
-        <v>15.16</v>
+        <v>15.157</v>
       </c>
       <c r="F15" t="n">
         <v>15.771</v>
@@ -61618,10 +62474,10 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>16.129999</v>
+        <v>16.040001</v>
       </c>
       <c r="C14" t="n">
-        <v>20.201</v>
+        <v>20.2</v>
       </c>
       <c r="D14" t="n">
         <v>0.02404</v>
@@ -61630,7 +62486,7 @@
         <v>28.8</v>
       </c>
       <c r="F14" t="n">
-        <v>-4.071</v>
+        <v>-4.16</v>
       </c>
     </row>
   </sheetData>
@@ -61849,26 +62705,26 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>4.81</v>
+        <v>4.92</v>
       </c>
       <c r="D3" t="n">
-        <v>5.17</v>
+        <v>5.24</v>
       </c>
       <c r="E3" t="n">
-        <v>0.36</v>
+        <v>0.32</v>
       </c>
       <c r="F3" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="G3" t="n">
-        <v>0.74</v>
+        <v>0.82</v>
       </c>
       <c r="H3" t="n">
-        <v>0.79</v>
+        <v>0.86</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -66904,7 +67760,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>-0.004866</v>
+        <v>-0.004863</v>
       </c>
     </row>
   </sheetData>
@@ -67801,7 +68657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -68038,6 +68894,22 @@
       </c>
       <c r="D14" t="n">
         <v>-0.03844</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0.00877</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0.06808</v>
+      </c>
+      <c r="D15" t="n">
+        <v>-0.03842</v>
       </c>
     </row>
   </sheetData>
@@ -71503,13 +72375,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1.0899</v>
+        <v>1.0897</v>
       </c>
       <c r="C15" t="n">
-        <v>1.0758</v>
+        <v>1.0756</v>
       </c>
       <c r="D15" t="n">
-        <v>1.5578</v>
+        <v>1.5574</v>
       </c>
     </row>
   </sheetData>
@@ -71581,7 +72453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G71"/>
+  <dimension ref="A1:G76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -73877,6 +74749,165 @@
         </is>
       </c>
     </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>stable</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>moyen</t>
+        </is>
+      </c>
+      <c r="F72" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>stable</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Zone euro</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>hausse</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>haut</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>non_couvert</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Royaume-Uni</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>3.73</v>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>stable</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>haut</t>
+        </is>
+      </c>
+      <c r="F74" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>stable</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Japon</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>0.977</v>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>stable</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>haut</t>
+        </is>
+      </c>
+      <c r="F75" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>stable</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Chine</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>stable</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>bas</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>non_couvert</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -73888,7 +74919,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -74238,6 +75269,30 @@
         <v>-2.15</v>
       </c>
       <c r="F14" t="inlineStr">
+        <is>
+          <t>2_termes_sans_output_gap</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>3.353</v>
+      </c>
+      <c r="C15" t="n">
+        <v>6.03</v>
+      </c>
+      <c r="D15" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="E15" t="n">
+        <v>-2.15</v>
+      </c>
+      <c r="F15" t="inlineStr">
         <is>
           <t>2_termes_sans_output_gap</t>
         </is>
@@ -78098,7 +79153,7 @@
         </is>
       </c>
       <c r="E132" t="n">
-        <v>15.892</v>
+        <v>15.873</v>
       </c>
     </row>
     <row r="133">
@@ -78144,7 +79199,7 @@
         </is>
       </c>
       <c r="E134" t="n">
-        <v>2.079</v>
+        <v>2.089</v>
       </c>
     </row>
     <row r="135">
@@ -78190,7 +79245,7 @@
         </is>
       </c>
       <c r="E136" t="n">
-        <v>-1.475</v>
+        <v>-1.469</v>
       </c>
     </row>
     <row r="137">
@@ -78213,7 +79268,7 @@
         </is>
       </c>
       <c r="E137" t="n">
-        <v>-3.433</v>
+        <v>-3.404</v>
       </c>
     </row>
     <row r="138">
@@ -78236,7 +79291,7 @@
         </is>
       </c>
       <c r="E138" t="n">
-        <v>-6.087</v>
+        <v>-6.109</v>
       </c>
     </row>
     <row r="139">
@@ -78259,7 +79314,7 @@
         </is>
       </c>
       <c r="E139" t="n">
-        <v>-6.945</v>
+        <v>-6.932</v>
       </c>
     </row>
     <row r="140">
@@ -78282,7 +79337,7 @@
         </is>
       </c>
       <c r="E140" t="n">
-        <v>-8.680999999999999</v>
+        <v>-8.692</v>
       </c>
     </row>
     <row r="141">
@@ -78305,7 +79360,7 @@
         </is>
       </c>
       <c r="E141" t="n">
-        <v>-12.395</v>
+        <v>-12.417</v>
       </c>
     </row>
   </sheetData>
@@ -81131,7 +82186,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>-0.1904</v>
+        <v>-0.1903</v>
       </c>
       <c r="C15" t="n">
         <v>1.0224</v>
@@ -81204,13 +82259,13 @@
         <v>13.8</v>
       </c>
       <c r="D2" t="n">
-        <v>5.17</v>
+        <v>5.24</v>
       </c>
       <c r="E2" t="n">
         <v>3.4</v>
       </c>
       <c r="F2" t="n">
-        <v>1.77</v>
+        <v>1.84</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-29T23:41Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-29 21:30 UTC</t>
+          <t>Genere le 2026-09-29 23:41 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-29 21:30 UTC</t>
+          <t>Rapport global — 2026-09-29 23:41 UTC</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>**Matieres premieres macro** — ratio cuivre/or stable -- pas de signal net sur la croissance (+3.0% sur 3 mois). Brent 95.7$ (+31.2% sur 3 mois, +40.8% sur 12 mois), gaz -8.0% sur 3 mois, ecart Brent-WTI +6.7$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-29)_</t>
+          <t>**Matieres premieres macro** — ratio cuivre/or stable -- pas de signal net sur la croissance (+3.1% sur 3 mois). Brent 96.1$ (+31.8% sur 3 mois, +41.4% sur 12 mois), gaz -7.6% sur 3 mois, ecart Brent-WTI +6.8$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -40244,10 +40244,10 @@
         <v>1.113</v>
       </c>
       <c r="D8" t="n">
-        <v>0.337</v>
+        <v>0.326</v>
       </c>
       <c r="E8" t="n">
-        <v>2e-05</v>
+        <v>5e-05</v>
       </c>
       <c r="F8" t="n">
         <v>150</v>
@@ -40273,10 +40273,10 @@
         <v>-1.581</v>
       </c>
       <c r="D9" t="n">
-        <v>0.09</v>
+        <v>0.065</v>
       </c>
       <c r="E9" t="n">
-        <v>0.26214</v>
+        <v>0.4176</v>
       </c>
       <c r="F9" t="n">
         <v>158</v>
@@ -51968,7 +51968,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>marches/indices/HANGSENG.csv</t>
+          <t>marches/fx/USDCNY.csv</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
@@ -51986,7 +51986,7 @@
         <v>42</v>
       </c>
       <c r="F211" t="n">
-        <v>3688</v>
+        <v>3903</v>
       </c>
       <c r="G211" t="inlineStr">
         <is>
@@ -51997,7 +51997,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>marches/indices/KOSPI.csv</t>
+          <t>marches/indices/DAX.csv</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -52015,7 +52015,7 @@
         <v>42</v>
       </c>
       <c r="F212" t="n">
-        <v>3680</v>
+        <v>3801</v>
       </c>
       <c r="G212" t="inlineStr">
         <is>
@@ -52026,7 +52026,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>marches/indices/NIKKEI225.csv</t>
+          <t>marches/indices/EUROSTOXX50.csv</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -52044,7 +52044,7 @@
         <v>42</v>
       </c>
       <c r="F213" t="n">
-        <v>3666</v>
+        <v>3758</v>
       </c>
       <c r="G213" t="inlineStr">
         <is>
@@ -52055,7 +52055,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>souverains/CANADA_10A.csv</t>
+          <t>marches/indices/FTSE100.csv</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -52073,7 +52073,7 @@
         <v>42</v>
       </c>
       <c r="F214" t="n">
-        <v>6437</v>
+        <v>3787</v>
       </c>
       <c r="G214" t="inlineStr">
         <is>
@@ -52084,7 +52084,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>souverains/CANADA_2A.csv</t>
+          <t>marches/indices/HANGSENG.csv</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -52102,7 +52102,7 @@
         <v>42</v>
       </c>
       <c r="F215" t="n">
-        <v>6436</v>
+        <v>3688</v>
       </c>
       <c r="G215" t="inlineStr">
         <is>
@@ -52113,7 +52113,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>souverains/CANADA_5A.csv</t>
+          <t>marches/indices/KOSPI.csv</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -52131,7 +52131,7 @@
         <v>42</v>
       </c>
       <c r="F216" t="n">
-        <v>6436</v>
+        <v>3680</v>
       </c>
       <c r="G216" t="inlineStr">
         <is>
@@ -52142,7 +52142,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>souverains/CANADA_LONG.csv</t>
+          <t>marches/indices/NIKKEI225.csv</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -52160,7 +52160,7 @@
         <v>42</v>
       </c>
       <c r="F217" t="n">
-        <v>6436</v>
+        <v>3666</v>
       </c>
       <c r="G217" t="inlineStr">
         <is>
@@ -52171,7 +52171,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_10A.csv</t>
+          <t>souverains/CANADA_10A.csv</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -52189,7 +52189,7 @@
         <v>42</v>
       </c>
       <c r="F218" t="n">
-        <v>9203</v>
+        <v>6437</v>
       </c>
       <c r="G218" t="inlineStr">
         <is>
@@ -52200,7 +52200,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_2A.csv</t>
+          <t>souverains/CANADA_2A.csv</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -52218,7 +52218,7 @@
         <v>42</v>
       </c>
       <c r="F219" t="n">
-        <v>9203</v>
+        <v>6436</v>
       </c>
       <c r="G219" t="inlineStr">
         <is>
@@ -52229,7 +52229,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_5A.csv</t>
+          <t>souverains/CANADA_5A.csv</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -52247,7 +52247,7 @@
         <v>42</v>
       </c>
       <c r="F220" t="n">
-        <v>9205</v>
+        <v>6436</v>
       </c>
       <c r="G220" t="inlineStr">
         <is>
@@ -52258,7 +52258,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
+          <t>souverains/CANADA_LONG.csv</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -52276,7 +52276,7 @@
         <v>42</v>
       </c>
       <c r="F221" t="n">
-        <v>5640</v>
+        <v>6436</v>
       </c>
       <c r="G221" t="inlineStr">
         <is>
@@ -52287,7 +52287,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
+          <t>souverains/SUEDE_10A.csv</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -52305,7 +52305,7 @@
         <v>42</v>
       </c>
       <c r="F222" t="n">
-        <v>5640</v>
+        <v>9203</v>
       </c>
       <c r="G222" t="inlineStr">
         <is>
@@ -52316,7 +52316,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
+          <t>souverains/SUEDE_2A.csv</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -52334,7 +52334,7 @@
         <v>42</v>
       </c>
       <c r="F223" t="n">
-        <v>5640</v>
+        <v>9203</v>
       </c>
       <c r="G223" t="inlineStr">
         <is>
@@ -52345,7 +52345,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
+          <t>souverains/SUEDE_5A.csv</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -52363,7 +52363,7 @@
         <v>42</v>
       </c>
       <c r="F224" t="n">
-        <v>5640</v>
+        <v>9205</v>
       </c>
       <c r="G224" t="inlineStr">
         <is>
@@ -52374,7 +52374,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
@@ -52403,7 +52403,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -52432,7 +52432,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -52461,7 +52461,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -52490,7 +52490,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -52519,7 +52519,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>tresor_us/dette_quotidienne.csv</t>
+          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -52537,7 +52537,7 @@
         <v>42</v>
       </c>
       <c r="F230" t="n">
-        <v>2000</v>
+        <v>5640</v>
       </c>
       <c r="G230" t="inlineStr">
         <is>
@@ -52548,7 +52548,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>tresor_us/solde_tresorerie.csv</t>
+          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -52566,7 +52566,7 @@
         <v>42</v>
       </c>
       <c r="F231" t="n">
-        <v>500</v>
+        <v>5640</v>
       </c>
       <c r="G231" t="inlineStr">
         <is>
@@ -52577,16 +52577,16 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>fred/ECBDFR.csv</t>
+          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C232" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D232" t="n">
         <v>1</v>
@@ -52595,7 +52595,7 @@
         <v>42</v>
       </c>
       <c r="F232" t="n">
-        <v>3000</v>
+        <v>5640</v>
       </c>
       <c r="G232" t="inlineStr">
         <is>
@@ -52606,16 +52606,16 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>fred/RRPONTSYD.csv</t>
+          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C233" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D233" t="n">
         <v>1</v>
@@ -52624,7 +52624,7 @@
         <v>42</v>
       </c>
       <c r="F233" t="n">
-        <v>3000</v>
+        <v>5640</v>
       </c>
       <c r="G233" t="inlineStr">
         <is>
@@ -52635,16 +52635,16 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>fred/T10YIE.csv</t>
+          <t>tresor_us/dette_quotidienne.csv</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C234" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D234" t="n">
         <v>1</v>
@@ -52653,7 +52653,7 @@
         <v>42</v>
       </c>
       <c r="F234" t="n">
-        <v>3000</v>
+        <v>2000</v>
       </c>
       <c r="G234" t="inlineStr">
         <is>
@@ -52664,16 +52664,16 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>marches/fx/AUDJPY.csv</t>
+          <t>tresor_us/solde_tresorerie.csv</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C235" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D235" t="n">
         <v>1</v>
@@ -52682,7 +52682,7 @@
         <v>42</v>
       </c>
       <c r="F235" t="n">
-        <v>3909</v>
+        <v>500</v>
       </c>
       <c r="G235" t="inlineStr">
         <is>
@@ -52693,7 +52693,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>marches/fx/AUDUSD.csv</t>
+          <t>fred/ECBDFR.csv</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -52711,7 +52711,7 @@
         <v>42</v>
       </c>
       <c r="F236" t="n">
-        <v>3905</v>
+        <v>3000</v>
       </c>
       <c r="G236" t="inlineStr">
         <is>
@@ -52722,7 +52722,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>marches/fx/DXY.csv</t>
+          <t>fred/RRPONTSYD.csv</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
@@ -52740,7 +52740,7 @@
         <v>42</v>
       </c>
       <c r="F237" t="n">
-        <v>3772</v>
+        <v>3000</v>
       </c>
       <c r="G237" t="inlineStr">
         <is>
@@ -52751,7 +52751,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>marches/fx/EURCHF.csv</t>
+          <t>fred/T10YIE.csv</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
@@ -52769,7 +52769,7 @@
         <v>42</v>
       </c>
       <c r="F238" t="n">
-        <v>3906</v>
+        <v>3000</v>
       </c>
       <c r="G238" t="inlineStr">
         <is>
@@ -52780,7 +52780,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>marches/fx/EURGBP.csv</t>
+          <t>marches/fx/AUDJPY.csv</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
@@ -52809,7 +52809,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>marches/fx/EURJPY.csv</t>
+          <t>marches/fx/AUDUSD.csv</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
@@ -52827,7 +52827,7 @@
         <v>42</v>
       </c>
       <c r="F240" t="n">
-        <v>3908</v>
+        <v>3904</v>
       </c>
       <c r="G240" t="inlineStr">
         <is>
@@ -52838,7 +52838,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>marches/fx/EURUSD.csv</t>
+          <t>marches/fx/DXY.csv</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
@@ -52856,7 +52856,7 @@
         <v>42</v>
       </c>
       <c r="F241" t="n">
-        <v>3905</v>
+        <v>3772</v>
       </c>
       <c r="G241" t="inlineStr">
         <is>
@@ -52867,7 +52867,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>marches/fx/GBPUSD.csv</t>
+          <t>marches/fx/EURCHF.csv</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
@@ -52885,7 +52885,7 @@
         <v>42</v>
       </c>
       <c r="F242" t="n">
-        <v>3906</v>
+        <v>3905</v>
       </c>
       <c r="G242" t="inlineStr">
         <is>
@@ -52896,7 +52896,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>marches/fx/NZDUSD.csv</t>
+          <t>marches/fx/EURGBP.csv</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
@@ -52914,7 +52914,7 @@
         <v>42</v>
       </c>
       <c r="F243" t="n">
-        <v>3906</v>
+        <v>3907</v>
       </c>
       <c r="G243" t="inlineStr">
         <is>
@@ -52925,7 +52925,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>marches/fx/USDCAD.csv</t>
+          <t>marches/fx/EURJPY.csv</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -52943,7 +52943,7 @@
         <v>42</v>
       </c>
       <c r="F244" t="n">
-        <v>3905</v>
+        <v>3907</v>
       </c>
       <c r="G244" t="inlineStr">
         <is>
@@ -52954,7 +52954,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>marches/fx/USDCHF.csv</t>
+          <t>marches/fx/EURUSD.csv</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -52972,7 +52972,7 @@
         <v>42</v>
       </c>
       <c r="F245" t="n">
-        <v>3903</v>
+        <v>3904</v>
       </c>
       <c r="G245" t="inlineStr">
         <is>
@@ -52983,7 +52983,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>marches/fx/USDCNY.csv</t>
+          <t>marches/fx/GBPUSD.csv</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -53012,7 +53012,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>marches/fx/USDJPY.csv</t>
+          <t>marches/fx/NZDUSD.csv</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
@@ -53030,7 +53030,7 @@
         <v>42</v>
       </c>
       <c r="F247" t="n">
-        <v>3906</v>
+        <v>3905</v>
       </c>
       <c r="G247" t="inlineStr">
         <is>
@@ -53041,7 +53041,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>marches/fx/USDKRW.csv</t>
+          <t>marches/fx/USDCAD.csv</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
@@ -53059,7 +53059,7 @@
         <v>42</v>
       </c>
       <c r="F248" t="n">
-        <v>3905</v>
+        <v>3904</v>
       </c>
       <c r="G248" t="inlineStr">
         <is>
@@ -53070,7 +53070,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>marches/fx/USDNOK.csv</t>
+          <t>marches/fx/USDCHF.csv</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
@@ -53088,7 +53088,7 @@
         <v>42</v>
       </c>
       <c r="F249" t="n">
-        <v>3906</v>
+        <v>3902</v>
       </c>
       <c r="G249" t="inlineStr">
         <is>
@@ -53099,7 +53099,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>marches/fx/USDSEK.csv</t>
+          <t>marches/fx/USDJPY.csv</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
@@ -53117,7 +53117,7 @@
         <v>42</v>
       </c>
       <c r="F250" t="n">
-        <v>3906</v>
+        <v>3905</v>
       </c>
       <c r="G250" t="inlineStr">
         <is>
@@ -53128,7 +53128,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>marches/indices/DAX.csv</t>
+          <t>marches/fx/USDKRW.csv</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
@@ -53146,7 +53146,7 @@
         <v>42</v>
       </c>
       <c r="F251" t="n">
-        <v>3802</v>
+        <v>3904</v>
       </c>
       <c r="G251" t="inlineStr">
         <is>
@@ -53157,7 +53157,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>marches/indices/EUROSTOXX50.csv</t>
+          <t>marches/fx/USDNOK.csv</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -53175,7 +53175,7 @@
         <v>42</v>
       </c>
       <c r="F252" t="n">
-        <v>3759</v>
+        <v>3905</v>
       </c>
       <c r="G252" t="inlineStr">
         <is>
@@ -53186,7 +53186,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>marches/indices/FTSE100.csv</t>
+          <t>marches/fx/USDSEK.csv</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -53204,7 +53204,7 @@
         <v>42</v>
       </c>
       <c r="F253" t="n">
-        <v>3788</v>
+        <v>3905</v>
       </c>
       <c r="G253" t="inlineStr">
         <is>
@@ -53320,7 +53320,7 @@
         <v>42</v>
       </c>
       <c r="F257" t="n">
-        <v>3770</v>
+        <v>3771</v>
       </c>
       <c r="G257" t="inlineStr">
         <is>
@@ -55527,43 +55527,43 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Zone euro (Euro Stoxx 50)</t>
+          <t>Royaume-Uni (FTSE 100)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>6320.26</v>
+        <v>10684.9</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.12</v>
+        <v>1.91</v>
       </c>
       <c r="E5" t="n">
-        <v>14.77</v>
+        <v>15.08</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Royaume-Uni (FTSE 100)</t>
+          <t>Zone euro (Euro Stoxx 50)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>10636.71</v>
+        <v>6301.28</v>
       </c>
       <c r="D6" t="n">
-        <v>1.33</v>
+        <v>1.12</v>
       </c>
       <c r="E6" t="n">
-        <v>14.38</v>
+        <v>14.57</v>
       </c>
     </row>
     <row r="7">
@@ -55574,17 +55574,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>25399.21</v>
+        <v>25374.42</v>
       </c>
       <c r="D7" t="n">
-        <v>1.61</v>
+        <v>3.04</v>
       </c>
       <c r="E7" t="n">
-        <v>6.97</v>
+        <v>6.89</v>
       </c>
     </row>
     <row r="8">
@@ -57845,25 +57845,25 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.00158</v>
+        <v>0.001581</v>
       </c>
       <c r="C12" t="n">
-        <v>3.02</v>
+        <v>3.12</v>
       </c>
       <c r="D12" t="n">
-        <v>95.67</v>
+        <v>96.11</v>
       </c>
       <c r="E12" t="n">
-        <v>31.2</v>
+        <v>31.8</v>
       </c>
       <c r="F12" t="n">
-        <v>40.75</v>
+        <v>41.4</v>
       </c>
       <c r="G12" t="n">
-        <v>-7.97</v>
+        <v>-7.63</v>
       </c>
       <c r="H12" t="n">
-        <v>6.73</v>
+        <v>6.75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-30T00:51Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-29 23:41 UTC</t>
+          <t>Genere le 2026-09-30 00:51 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-29 23:41 UTC</t>
+          <t>Rapport global — 2026-09-30 00:51 UTC</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>**Matieres premieres macro** — ratio cuivre/or stable -- pas de signal net sur la croissance (+3.1% sur 3 mois). Brent 96.1$ (+31.8% sur 3 mois, +41.4% sur 12 mois), gaz -7.6% sur 3 mois, ecart Brent-WTI +6.8$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-29)_</t>
+          <t>**Matieres premieres macro** — le ratio cuivre/or monte -- la croissance domine la peur (+5.3% sur 3 mois). Brent 96.0$ (+34.2% sur 3 mois, +43.3% sur 12 mois), gaz -6.2% sur 3 mois, ecart Brent-WTI +6.7$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -869,7 +869,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>**Emission tresor us** — 84 derniers jours, 7985 Mds$ offerts : court (moins d'un an) 6897 Mds$ (86%), intermediaire (2 a 10 ans) 969 Mds$ (12%), long (20 a 30 ans) 119 Mds$ (2%) -- financement concentre sur le court et l'intermediaire, part longue a 2% -- peu de pression par la duration _(observation : date non exposee)_</t>
+          <t>**Emission tresor us** — 84 derniers jours, 7785 Mds$ offerts : court (moins d'un an) 6755 Mds$ (87%), intermediaire (2 a 10 ans) 911 Mds$ (12%), long (20 a 30 ans) 119 Mds$ (2%) -- financement concentre sur le court et l'intermediaire, part longue a 2% -- peu de pression par la duration _(observation : date non exposee)_</t>
         </is>
       </c>
     </row>
@@ -960,7 +960,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>**Indices mondiaux** — 7 indices (devise locale) : Coree (KOSPI) +103.5% en tete sur 12 mois, Hong Kong (Hang Seng) -5.7% en queue -- ecart tres large entre blocs sur 12 mois (109pt) -- les cycles economiques ou les flux divergent nettement. ROTATION en cours : Coree (KOSPI) mene sur 12 mois mais Hong Kong (Hang Seng) a repris la tete sur 3 mois _(observation : 2026-09-29)_</t>
+          <t>**Indices mondiaux** — 7 indices (devise locale) : Coree (KOSPI) +102.5% en tete sur 12 mois, Hong Kong (Hang Seng) -5.7% en queue -- ecart tres large entre blocs sur 12 mois (108pt) -- les cycles economiques ou les flux divergent nettement. ROTATION en cours : Coree (KOSPI) mene sur 12 mois mais Hong Kong (Hang Seng) a repris la tete sur 3 mois _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1009,7 +1009,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>**Rotation sectorielle** — classement momentum 3 mois (10 secteurs) : 1. Energie (XLE) : +15.87% | 2. Sante (XLV) : +7.61% | 3. Technologie (XLK) : +2.09% | 4. Finance (XLF) : +0.75% | 5. Consommation de base (XLP) : -1.47% _(observation : 2026-09-29)_</t>
+          <t>**Rotation sectorielle** — classement momentum 3 mois (10 secteurs) : 1. Energie (XLE) : +15.90% | 2. Sante (XLV) : +6.54% | 3. Technologie (XLK) : +4.92% | 4. Finance (XLF) : +0.88% | 5. Materiaux (XLB) : -2.35% _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1023,21 +1023,21 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>**Dispersion sectorielle** — 10 secteurs, rendement moyen 3m=-1.27%, dispersion (ecart-type)=7.92pt, etendue=28.29pt -- dispersion intermediaire _(observation : 2026-09-29)_</t>
+          <t>**Dispersion sectorielle** — 10 secteurs, rendement moyen 3m=-1.38%, dispersion (ecart-type)=8.36pt, etendue=30.61pt -- dispersion intermediaire _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>**Low volatility** — tercile bas-vol ['XLF', 'XLRE', 'XLU'] Sharpe=-0.842 vs tercile haut-vol ['XLY', 'XLE', 'XLK'] Sharpe=0.040 -- anomalie low-vol non confirmee sur cet echantillon (puissance statistique faible, n petit -- limite assumee) _(observation : 2026-09-29)_</t>
+          <t>**Low volatility** — tercile bas-vol ['XLF', 'XLRE', 'XLU'] Sharpe=-0.720 vs tercile haut-vol ['XLY', 'XLE', 'XLK'] Sharpe=0.153 -- anomalie low-vol non confirmee sur cet echantillon (puissance statistique faible, n petit -- limite assumee) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>**Momentum cross sectional** — panier gagnant ['XLE', 'XLV', 'XLK'] (+8.52%) vs panier perdant ['XLY', 'XLI', 'XLU'] (-9.35%) -- spread momentum=+17.87pt _(observation : 2026-09-29)_</t>
+          <t>**Momentum cross sectional** — panier gagnant ['XLE', 'XLV', 'XLK'] (+9.12%) vs panier perdant ['XLI', 'XLRE', 'XLU'] (-10.10%) -- spread momentum=+19.22pt _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>**Correlation facteurs** — correlation entre momentum 3m et beta-VIX, 10 secteurs : +0.361 (facteurs largement independants) _(observation : 2026-09-29)_</t>
+          <t>**Correlation facteurs** — correlation entre momentum 3m et beta-VIX, 10 secteurs : +0.215 (facteurs largement independants) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -14217,7 +14217,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -17308,10 +17308,10 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>-2.5102</v>
+        <v>-2.5374</v>
       </c>
       <c r="D132" t="n">
-        <v>0.2746</v>
+        <v>0.2628</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -17331,10 +17331,10 @@
         </is>
       </c>
       <c r="C133" t="n">
-        <v>-1.8331</v>
+        <v>-1.8514</v>
       </c>
       <c r="D133" t="n">
-        <v>0.6135</v>
+        <v>0.6044</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -17354,10 +17354,10 @@
         </is>
       </c>
       <c r="C134" t="n">
-        <v>-2.1416</v>
+        <v>-2.1451</v>
       </c>
       <c r="D134" t="n">
-        <v>0.4546</v>
+        <v>0.4528</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -17377,10 +17377,10 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>-2.3975</v>
+        <v>-2.3952</v>
       </c>
       <c r="D135" t="n">
-        <v>0.326</v>
+        <v>0.3271</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -17400,10 +17400,10 @@
         </is>
       </c>
       <c r="C136" t="n">
-        <v>-1.4392</v>
+        <v>-1.3635</v>
       </c>
       <c r="D136" t="n">
-        <v>0.7837</v>
+        <v>0.8097</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -17423,10 +17423,10 @@
         </is>
       </c>
       <c r="C137" t="n">
-        <v>0.0363</v>
+        <v>0.0851</v>
       </c>
       <c r="D137" t="n">
-        <v>0.9867</v>
+        <v>0.9877</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -17446,10 +17446,10 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>-1.1968</v>
+        <v>-1.2195</v>
       </c>
       <c r="D138" t="n">
-        <v>0.8587</v>
+        <v>0.8527</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -17469,10 +17469,10 @@
         </is>
       </c>
       <c r="C139" t="n">
-        <v>-0.698</v>
+        <v>-0.5135999999999999</v>
       </c>
       <c r="D139" t="n">
-        <v>0.9469</v>
+        <v>0.9634</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -17492,10 +17492,10 @@
         </is>
       </c>
       <c r="C140" t="n">
-        <v>-2.1262</v>
+        <v>-2.1811</v>
       </c>
       <c r="D140" t="n">
-        <v>0.4627</v>
+        <v>0.4341</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -17515,10 +17515,10 @@
         </is>
       </c>
       <c r="C141" t="n">
-        <v>-1.6182</v>
+        <v>-1.6158</v>
       </c>
       <c r="D141" t="n">
-        <v>0.7131</v>
+        <v>0.7141999999999999</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -41960,13 +41960,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C2" t="n">
-        <v>6897</v>
+        <v>6755</v>
       </c>
       <c r="D2" t="n">
-        <v>86.40000000000001</v>
+        <v>86.8</v>
       </c>
       <c r="E2" t="n">
         <v>2.85</v>
@@ -41979,13 +41979,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C3" t="n">
-        <v>969</v>
+        <v>911</v>
       </c>
       <c r="D3" t="n">
-        <v>12.1</v>
+        <v>11.7</v>
       </c>
       <c r="E3" t="n">
         <v>2.59</v>
@@ -45916,7 +45916,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D2" t="n">
         <v>91.5</v>
@@ -45945,7 +45945,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D3" t="n">
         <v>91.5</v>
@@ -45974,7 +45974,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D4" t="n">
         <v>91.5</v>
@@ -46003,7 +46003,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D5" t="n">
         <v>91.5</v>
@@ -46032,7 +46032,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D6" t="n">
         <v>91.5</v>
@@ -46061,7 +46061,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D7" t="n">
         <v>91.5</v>
@@ -46090,7 +46090,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D8" t="n">
         <v>91.5</v>
@@ -46119,7 +46119,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D9" t="n">
         <v>91.5</v>
@@ -46148,7 +46148,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D10" t="n">
         <v>91.5</v>
@@ -46177,7 +46177,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D11" t="n">
         <v>91.5</v>
@@ -46206,7 +46206,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D12" t="n">
         <v>91.5</v>
@@ -46235,7 +46235,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D13" t="n">
         <v>91.5</v>
@@ -46264,7 +46264,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D14" t="n">
         <v>91.5</v>
@@ -46293,7 +46293,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D15" t="n">
         <v>91.5</v>
@@ -46322,7 +46322,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D16" t="n">
         <v>92</v>
@@ -46351,7 +46351,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D17" t="n">
         <v>91.5</v>
@@ -46380,7 +46380,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D18" t="n">
         <v>91.5</v>
@@ -46409,7 +46409,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D19" t="n">
         <v>91.5</v>
@@ -46438,7 +46438,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D20" t="n">
         <v>91.5</v>
@@ -46467,7 +46467,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D21" t="n">
         <v>91.5</v>
@@ -46496,7 +46496,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D22" t="n">
         <v>91.5</v>
@@ -46525,7 +46525,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D23" t="n">
         <v>91.5</v>
@@ -46554,7 +46554,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D24" t="n">
         <v>91.5</v>
@@ -46583,7 +46583,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="D25" t="n">
         <v>91</v>
@@ -46612,7 +46612,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D26" t="n">
         <v>31</v>
@@ -46641,7 +46641,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D27" t="n">
         <v>31</v>
@@ -46670,7 +46670,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D28" t="n">
         <v>31</v>
@@ -46699,7 +46699,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D29" t="n">
         <v>31</v>
@@ -46728,7 +46728,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D30" t="n">
         <v>31</v>
@@ -46757,7 +46757,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D31" t="n">
         <v>31</v>
@@ -46786,7 +46786,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D32" t="n">
         <v>31</v>
@@ -46815,7 +46815,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D33" t="n">
         <v>31</v>
@@ -46844,7 +46844,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D34" t="n">
         <v>31</v>
@@ -46873,7 +46873,7 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D35" t="n">
         <v>31</v>
@@ -46902,7 +46902,7 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D36" t="n">
         <v>31</v>
@@ -46931,7 +46931,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D37" t="n">
         <v>31</v>
@@ -46960,7 +46960,7 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D38" t="n">
         <v>31</v>
@@ -46989,7 +46989,7 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D39" t="n">
         <v>31</v>
@@ -47018,7 +47018,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D40" t="n">
         <v>31</v>
@@ -47047,7 +47047,7 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D41" t="n">
         <v>31</v>
@@ -47076,7 +47076,7 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D42" t="n">
         <v>31</v>
@@ -47105,7 +47105,7 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D43" t="n">
         <v>31</v>
@@ -47134,7 +47134,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D44" t="n">
         <v>31</v>
@@ -47163,7 +47163,7 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D45" t="n">
         <v>31</v>
@@ -47192,7 +47192,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D46" t="n">
         <v>31</v>
@@ -47221,7 +47221,7 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D47" t="n">
         <v>31</v>
@@ -47250,7 +47250,7 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D48" t="n">
         <v>31</v>
@@ -47279,7 +47279,7 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D49" t="n">
         <v>31</v>
@@ -47308,7 +47308,7 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D50" t="n">
         <v>31</v>
@@ -47337,7 +47337,7 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D51" t="n">
         <v>31</v>
@@ -47366,7 +47366,7 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D52" t="n">
         <v>31</v>
@@ -47395,7 +47395,7 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D53" t="n">
         <v>31</v>
@@ -47424,7 +47424,7 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D54" t="n">
         <v>31</v>
@@ -47453,7 +47453,7 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D55" t="n">
         <v>31</v>
@@ -47482,7 +47482,7 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D56" t="n">
         <v>31</v>
@@ -47511,7 +47511,7 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D57" t="n">
         <v>31</v>
@@ -47540,7 +47540,7 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D58" t="n">
         <v>31</v>
@@ -47569,7 +47569,7 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D59" t="n">
         <v>31</v>
@@ -47598,7 +47598,7 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D60" t="n">
         <v>31</v>
@@ -47627,7 +47627,7 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D61" t="n">
         <v>31</v>
@@ -47656,7 +47656,7 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D62" t="n">
         <v>31</v>
@@ -47685,7 +47685,7 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D63" t="n">
         <v>31</v>
@@ -47714,7 +47714,7 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D64" t="n">
         <v>31</v>
@@ -47743,7 +47743,7 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D65" t="n">
         <v>31</v>
@@ -47772,7 +47772,7 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D66" t="n">
         <v>31</v>
@@ -47801,7 +47801,7 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D67" t="n">
         <v>31</v>
@@ -47830,7 +47830,7 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D68" t="n">
         <v>31</v>
@@ -47859,7 +47859,7 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D69" t="n">
         <v>31</v>
@@ -47888,7 +47888,7 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D70" t="n">
         <v>31</v>
@@ -47917,7 +47917,7 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D71" t="n">
         <v>31</v>
@@ -47946,7 +47946,7 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D72" t="n">
         <v>31</v>
@@ -47975,7 +47975,7 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D73" t="n">
         <v>31</v>
@@ -48004,7 +48004,7 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D74" t="n">
         <v>31</v>
@@ -48033,7 +48033,7 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D75" t="n">
         <v>31</v>
@@ -48062,7 +48062,7 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D76" t="n">
         <v>31</v>
@@ -48091,7 +48091,7 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D77" t="n">
         <v>31</v>
@@ -48120,7 +48120,7 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D78" t="n">
         <v>31</v>
@@ -48149,7 +48149,7 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D79" t="n">
         <v>31</v>
@@ -48178,7 +48178,7 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D80" t="n">
         <v>31</v>
@@ -48207,7 +48207,7 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D81" t="n">
         <v>31</v>
@@ -48236,7 +48236,7 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D82" t="n">
         <v>31</v>
@@ -48265,7 +48265,7 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D83" t="n">
         <v>31</v>
@@ -48294,7 +48294,7 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D84" t="n">
         <v>31</v>
@@ -48323,7 +48323,7 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D85" t="n">
         <v>31</v>
@@ -48352,7 +48352,7 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D86" t="n">
         <v>31</v>
@@ -48381,7 +48381,7 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D87" t="n">
         <v>31</v>
@@ -48410,7 +48410,7 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D88" t="n">
         <v>31</v>
@@ -48439,7 +48439,7 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D89" t="n">
         <v>31</v>
@@ -48468,7 +48468,7 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D90" t="n">
         <v>1</v>
@@ -48497,7 +48497,7 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D91" t="n">
         <v>1</v>
@@ -48526,7 +48526,7 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D92" t="n">
         <v>1</v>
@@ -48555,7 +48555,7 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D93" t="n">
         <v>1</v>
@@ -48584,7 +48584,7 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D94" t="n">
         <v>1</v>
@@ -48613,7 +48613,7 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D95" t="n">
         <v>31</v>
@@ -48642,7 +48642,7 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D96" t="n">
         <v>31</v>
@@ -48671,7 +48671,7 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D97" t="n">
         <v>31</v>
@@ -48700,7 +48700,7 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D98" t="n">
         <v>31</v>
@@ -48729,7 +48729,7 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D99" t="n">
         <v>31</v>
@@ -48758,7 +48758,7 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D100" t="n">
         <v>31</v>
@@ -48787,7 +48787,7 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D101" t="n">
         <v>31</v>
@@ -48816,7 +48816,7 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D102" t="n">
         <v>1</v>
@@ -48845,7 +48845,7 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D103" t="n">
         <v>7</v>
@@ -48874,7 +48874,7 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D104" t="n">
         <v>1</v>
@@ -48903,7 +48903,7 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D105" t="n">
         <v>1</v>
@@ -48932,7 +48932,7 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D106" t="n">
         <v>7</v>
@@ -48961,7 +48961,7 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D107" t="n">
         <v>1</v>
@@ -48990,7 +48990,7 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D108" t="n">
         <v>7</v>
@@ -49019,7 +49019,7 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D109" t="n">
         <v>1</v>
@@ -49048,7 +49048,7 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D110" t="n">
         <v>1</v>
@@ -49077,7 +49077,7 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D111" t="n">
         <v>1</v>
@@ -49106,7 +49106,7 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D112" t="n">
         <v>1</v>
@@ -49135,7 +49135,7 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D113" t="n">
         <v>1</v>
@@ -49164,7 +49164,7 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D114" t="n">
         <v>1</v>
@@ -49193,7 +49193,7 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D115" t="n">
         <v>1</v>
@@ -49222,7 +49222,7 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D116" t="n">
         <v>7</v>
@@ -49251,7 +49251,7 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D117" t="n">
         <v>7</v>
@@ -49280,7 +49280,7 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D118" t="n">
         <v>7</v>
@@ -49309,7 +49309,7 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D119" t="n">
         <v>7</v>
@@ -49338,7 +49338,7 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D120" t="n">
         <v>7</v>
@@ -49367,7 +49367,7 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D121" t="n">
         <v>7</v>
@@ -49396,7 +49396,7 @@
         </is>
       </c>
       <c r="C122" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D122" t="n">
         <v>7</v>
@@ -49425,7 +49425,7 @@
         </is>
       </c>
       <c r="C123" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D123" t="n">
         <v>7</v>
@@ -49454,7 +49454,7 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D124" t="n">
         <v>7</v>
@@ -49483,7 +49483,7 @@
         </is>
       </c>
       <c r="C125" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D125" t="n">
         <v>7</v>
@@ -49512,7 +49512,7 @@
         </is>
       </c>
       <c r="C126" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D126" t="n">
         <v>7</v>
@@ -49541,7 +49541,7 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D127" t="n">
         <v>7</v>
@@ -49570,7 +49570,7 @@
         </is>
       </c>
       <c r="C128" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D128" t="n">
         <v>7</v>
@@ -49599,7 +49599,7 @@
         </is>
       </c>
       <c r="C129" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D129" t="n">
         <v>7</v>
@@ -49628,7 +49628,7 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D130" t="n">
         <v>7</v>
@@ -49657,7 +49657,7 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D131" t="n">
         <v>7</v>
@@ -49686,7 +49686,7 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D132" t="n">
         <v>7</v>
@@ -49715,7 +49715,7 @@
         </is>
       </c>
       <c r="C133" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D133" t="n">
         <v>7</v>
@@ -49744,7 +49744,7 @@
         </is>
       </c>
       <c r="C134" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D134" t="n">
         <v>7</v>
@@ -49773,7 +49773,7 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D135" t="n">
         <v>7</v>
@@ -49802,7 +49802,7 @@
         </is>
       </c>
       <c r="C136" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D136" t="n">
         <v>7</v>
@@ -49831,7 +49831,7 @@
         </is>
       </c>
       <c r="C137" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D137" t="n">
         <v>7</v>
@@ -49860,7 +49860,7 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D138" t="n">
         <v>7</v>
@@ -49889,7 +49889,7 @@
         </is>
       </c>
       <c r="C139" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D139" t="n">
         <v>7</v>
@@ -49918,7 +49918,7 @@
         </is>
       </c>
       <c r="C140" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D140" t="n">
         <v>7</v>
@@ -49947,7 +49947,7 @@
         </is>
       </c>
       <c r="C141" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D141" t="n">
         <v>7</v>
@@ -49976,7 +49976,7 @@
         </is>
       </c>
       <c r="C142" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D142" t="n">
         <v>7</v>
@@ -50005,7 +50005,7 @@
         </is>
       </c>
       <c r="C143" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D143" t="n">
         <v>7</v>
@@ -50034,7 +50034,7 @@
         </is>
       </c>
       <c r="C144" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D144" t="n">
         <v>7</v>
@@ -50063,7 +50063,7 @@
         </is>
       </c>
       <c r="C145" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D145" t="n">
         <v>7</v>
@@ -50092,7 +50092,7 @@
         </is>
       </c>
       <c r="C146" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D146" t="n">
         <v>7</v>
@@ -50121,7 +50121,7 @@
         </is>
       </c>
       <c r="C147" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D147" t="n">
         <v>7</v>
@@ -50150,7 +50150,7 @@
         </is>
       </c>
       <c r="C148" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D148" t="n">
         <v>7</v>
@@ -50179,7 +50179,7 @@
         </is>
       </c>
       <c r="C149" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D149" t="n">
         <v>7</v>
@@ -50208,7 +50208,7 @@
         </is>
       </c>
       <c r="C150" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D150" t="n">
         <v>7</v>
@@ -50237,7 +50237,7 @@
         </is>
       </c>
       <c r="C151" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D151" t="n">
         <v>7</v>
@@ -50266,7 +50266,7 @@
         </is>
       </c>
       <c r="C152" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D152" t="n">
         <v>7</v>
@@ -50295,7 +50295,7 @@
         </is>
       </c>
       <c r="C153" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D153" t="n">
         <v>7</v>
@@ -50324,7 +50324,7 @@
         </is>
       </c>
       <c r="C154" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D154" t="n">
         <v>7</v>
@@ -50353,7 +50353,7 @@
         </is>
       </c>
       <c r="C155" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D155" t="n">
         <v>7</v>
@@ -50382,7 +50382,7 @@
         </is>
       </c>
       <c r="C156" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D156" t="n">
         <v>7</v>
@@ -50411,7 +50411,7 @@
         </is>
       </c>
       <c r="C157" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D157" t="n">
         <v>7</v>
@@ -50440,7 +50440,7 @@
         </is>
       </c>
       <c r="C158" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D158" t="n">
         <v>7</v>
@@ -50469,7 +50469,7 @@
         </is>
       </c>
       <c r="C159" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D159" t="n">
         <v>7</v>
@@ -50498,7 +50498,7 @@
         </is>
       </c>
       <c r="C160" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D160" t="n">
         <v>7</v>
@@ -50527,7 +50527,7 @@
         </is>
       </c>
       <c r="C161" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D161" t="n">
         <v>7</v>
@@ -50556,7 +50556,7 @@
         </is>
       </c>
       <c r="C162" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D162" t="n">
         <v>7</v>
@@ -50585,7 +50585,7 @@
         </is>
       </c>
       <c r="C163" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D163" t="n">
         <v>7</v>
@@ -50614,7 +50614,7 @@
         </is>
       </c>
       <c r="C164" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D164" t="n">
         <v>7</v>
@@ -50643,7 +50643,7 @@
         </is>
       </c>
       <c r="C165" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D165" t="n">
         <v>7</v>
@@ -50672,7 +50672,7 @@
         </is>
       </c>
       <c r="C166" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D166" t="n">
         <v>7</v>
@@ -50701,7 +50701,7 @@
         </is>
       </c>
       <c r="C167" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D167" t="n">
         <v>7</v>
@@ -50730,7 +50730,7 @@
         </is>
       </c>
       <c r="C168" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D168" t="n">
         <v>7</v>
@@ -50759,7 +50759,7 @@
         </is>
       </c>
       <c r="C169" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D169" t="n">
         <v>7</v>
@@ -50788,7 +50788,7 @@
         </is>
       </c>
       <c r="C170" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D170" t="n">
         <v>7</v>
@@ -50817,7 +50817,7 @@
         </is>
       </c>
       <c r="C171" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D171" t="n">
         <v>7</v>
@@ -50846,7 +50846,7 @@
         </is>
       </c>
       <c r="C172" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D172" t="n">
         <v>7</v>
@@ -50875,7 +50875,7 @@
         </is>
       </c>
       <c r="C173" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D173" t="n">
         <v>7</v>
@@ -50904,7 +50904,7 @@
         </is>
       </c>
       <c r="C174" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D174" t="n">
         <v>7</v>
@@ -50933,7 +50933,7 @@
         </is>
       </c>
       <c r="C175" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D175" t="n">
         <v>7</v>
@@ -50962,7 +50962,7 @@
         </is>
       </c>
       <c r="C176" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D176" t="n">
         <v>7</v>
@@ -50991,7 +50991,7 @@
         </is>
       </c>
       <c r="C177" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D177" t="n">
         <v>7</v>
@@ -51020,7 +51020,7 @@
         </is>
       </c>
       <c r="C178" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D178" t="n">
         <v>7</v>
@@ -51049,7 +51049,7 @@
         </is>
       </c>
       <c r="C179" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D179" t="n">
         <v>7</v>
@@ -51078,7 +51078,7 @@
         </is>
       </c>
       <c r="C180" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D180" t="n">
         <v>7</v>
@@ -51107,7 +51107,7 @@
         </is>
       </c>
       <c r="C181" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D181" t="n">
         <v>7</v>
@@ -51136,7 +51136,7 @@
         </is>
       </c>
       <c r="C182" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D182" t="n">
         <v>7</v>
@@ -51165,7 +51165,7 @@
         </is>
       </c>
       <c r="C183" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D183" t="n">
         <v>1</v>
@@ -51194,7 +51194,7 @@
         </is>
       </c>
       <c r="C184" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D184" t="n">
         <v>1</v>
@@ -51223,7 +51223,7 @@
         </is>
       </c>
       <c r="C185" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D185" t="n">
         <v>1</v>
@@ -51252,7 +51252,7 @@
         </is>
       </c>
       <c r="C186" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D186" t="n">
         <v>7</v>
@@ -51281,7 +51281,7 @@
         </is>
       </c>
       <c r="C187" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D187" t="n">
         <v>1</v>
@@ -51310,7 +51310,7 @@
         </is>
       </c>
       <c r="C188" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D188" t="n">
         <v>1</v>
@@ -51339,7 +51339,7 @@
         </is>
       </c>
       <c r="C189" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D189" t="n">
         <v>1</v>
@@ -51368,7 +51368,7 @@
         </is>
       </c>
       <c r="C190" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D190" t="n">
         <v>1</v>
@@ -51397,7 +51397,7 @@
         </is>
       </c>
       <c r="C191" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D191" t="n">
         <v>1</v>
@@ -51426,7 +51426,7 @@
         </is>
       </c>
       <c r="C192" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D192" t="n">
         <v>1</v>
@@ -51455,7 +51455,7 @@
         </is>
       </c>
       <c r="C193" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D193" t="n">
         <v>1</v>
@@ -51484,7 +51484,7 @@
         </is>
       </c>
       <c r="C194" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D194" t="n">
         <v>1</v>
@@ -51513,7 +51513,7 @@
         </is>
       </c>
       <c r="C195" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D195" t="n">
         <v>1</v>
@@ -51542,7 +51542,7 @@
         </is>
       </c>
       <c r="C196" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D196" t="n">
         <v>1</v>
@@ -51571,7 +51571,7 @@
         </is>
       </c>
       <c r="C197" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D197" t="n">
         <v>1</v>
@@ -51600,7 +51600,7 @@
         </is>
       </c>
       <c r="C198" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D198" t="n">
         <v>1</v>
@@ -51629,7 +51629,7 @@
         </is>
       </c>
       <c r="C199" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D199" t="n">
         <v>1</v>
@@ -51658,7 +51658,7 @@
         </is>
       </c>
       <c r="C200" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D200" t="n">
         <v>1</v>
@@ -51687,7 +51687,7 @@
         </is>
       </c>
       <c r="C201" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D201" t="n">
         <v>1</v>
@@ -51716,7 +51716,7 @@
         </is>
       </c>
       <c r="C202" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D202" t="n">
         <v>1</v>
@@ -51745,7 +51745,7 @@
         </is>
       </c>
       <c r="C203" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D203" t="n">
         <v>1</v>
@@ -51774,7 +51774,7 @@
         </is>
       </c>
       <c r="C204" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D204" t="n">
         <v>1</v>
@@ -51803,7 +51803,7 @@
         </is>
       </c>
       <c r="C205" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D205" t="n">
         <v>1</v>
@@ -51832,7 +51832,7 @@
         </is>
       </c>
       <c r="C206" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D206" t="n">
         <v>1</v>
@@ -51861,7 +51861,7 @@
         </is>
       </c>
       <c r="C207" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D207" t="n">
         <v>1</v>
@@ -51890,7 +51890,7 @@
         </is>
       </c>
       <c r="C208" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D208" t="n">
         <v>1</v>
@@ -51919,7 +51919,7 @@
         </is>
       </c>
       <c r="C209" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D209" t="n">
         <v>1</v>
@@ -51948,7 +51948,7 @@
         </is>
       </c>
       <c r="C210" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D210" t="n">
         <v>1</v>
@@ -51968,7 +51968,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>marches/fx/USDCNY.csv</t>
+          <t>marches/indices/DAX.csv</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
@@ -51977,7 +51977,7 @@
         </is>
       </c>
       <c r="C211" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D211" t="n">
         <v>1</v>
@@ -51986,7 +51986,7 @@
         <v>42</v>
       </c>
       <c r="F211" t="n">
-        <v>3903</v>
+        <v>3801</v>
       </c>
       <c r="G211" t="inlineStr">
         <is>
@@ -51997,7 +51997,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>marches/indices/DAX.csv</t>
+          <t>marches/indices/EUROSTOXX50.csv</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -52006,7 +52006,7 @@
         </is>
       </c>
       <c r="C212" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D212" t="n">
         <v>1</v>
@@ -52015,7 +52015,7 @@
         <v>42</v>
       </c>
       <c r="F212" t="n">
-        <v>3801</v>
+        <v>3758</v>
       </c>
       <c r="G212" t="inlineStr">
         <is>
@@ -52026,7 +52026,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>marches/indices/EUROSTOXX50.csv</t>
+          <t>marches/indices/FTSE100.csv</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -52035,7 +52035,7 @@
         </is>
       </c>
       <c r="C213" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D213" t="n">
         <v>1</v>
@@ -52044,7 +52044,7 @@
         <v>42</v>
       </c>
       <c r="F213" t="n">
-        <v>3758</v>
+        <v>3787</v>
       </c>
       <c r="G213" t="inlineStr">
         <is>
@@ -52055,7 +52055,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>marches/indices/FTSE100.csv</t>
+          <t>marches/indices/HANGSENG.csv</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -52064,7 +52064,7 @@
         </is>
       </c>
       <c r="C214" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D214" t="n">
         <v>1</v>
@@ -52073,7 +52073,7 @@
         <v>42</v>
       </c>
       <c r="F214" t="n">
-        <v>3787</v>
+        <v>3688</v>
       </c>
       <c r="G214" t="inlineStr">
         <is>
@@ -52084,7 +52084,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>marches/indices/HANGSENG.csv</t>
+          <t>souverains/CANADA_10A.csv</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -52093,7 +52093,7 @@
         </is>
       </c>
       <c r="C215" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D215" t="n">
         <v>1</v>
@@ -52102,7 +52102,7 @@
         <v>42</v>
       </c>
       <c r="F215" t="n">
-        <v>3688</v>
+        <v>6437</v>
       </c>
       <c r="G215" t="inlineStr">
         <is>
@@ -52113,7 +52113,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>marches/indices/KOSPI.csv</t>
+          <t>souverains/CANADA_2A.csv</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -52122,7 +52122,7 @@
         </is>
       </c>
       <c r="C216" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D216" t="n">
         <v>1</v>
@@ -52131,7 +52131,7 @@
         <v>42</v>
       </c>
       <c r="F216" t="n">
-        <v>3680</v>
+        <v>6436</v>
       </c>
       <c r="G216" t="inlineStr">
         <is>
@@ -52142,7 +52142,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>marches/indices/NIKKEI225.csv</t>
+          <t>souverains/CANADA_5A.csv</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -52151,7 +52151,7 @@
         </is>
       </c>
       <c r="C217" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D217" t="n">
         <v>1</v>
@@ -52160,7 +52160,7 @@
         <v>42</v>
       </c>
       <c r="F217" t="n">
-        <v>3666</v>
+        <v>6436</v>
       </c>
       <c r="G217" t="inlineStr">
         <is>
@@ -52171,7 +52171,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>souverains/CANADA_10A.csv</t>
+          <t>souverains/CANADA_LONG.csv</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -52180,7 +52180,7 @@
         </is>
       </c>
       <c r="C218" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D218" t="n">
         <v>1</v>
@@ -52189,7 +52189,7 @@
         <v>42</v>
       </c>
       <c r="F218" t="n">
-        <v>6437</v>
+        <v>6436</v>
       </c>
       <c r="G218" t="inlineStr">
         <is>
@@ -52200,7 +52200,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>souverains/CANADA_2A.csv</t>
+          <t>souverains/SUEDE_10A.csv</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -52209,7 +52209,7 @@
         </is>
       </c>
       <c r="C219" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D219" t="n">
         <v>1</v>
@@ -52218,7 +52218,7 @@
         <v>42</v>
       </c>
       <c r="F219" t="n">
-        <v>6436</v>
+        <v>9203</v>
       </c>
       <c r="G219" t="inlineStr">
         <is>
@@ -52229,7 +52229,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>souverains/CANADA_5A.csv</t>
+          <t>souverains/SUEDE_2A.csv</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -52238,7 +52238,7 @@
         </is>
       </c>
       <c r="C220" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D220" t="n">
         <v>1</v>
@@ -52247,7 +52247,7 @@
         <v>42</v>
       </c>
       <c r="F220" t="n">
-        <v>6436</v>
+        <v>9203</v>
       </c>
       <c r="G220" t="inlineStr">
         <is>
@@ -52258,7 +52258,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>souverains/CANADA_LONG.csv</t>
+          <t>souverains/SUEDE_5A.csv</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -52267,7 +52267,7 @@
         </is>
       </c>
       <c r="C221" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D221" t="n">
         <v>1</v>
@@ -52276,7 +52276,7 @@
         <v>42</v>
       </c>
       <c r="F221" t="n">
-        <v>6436</v>
+        <v>9205</v>
       </c>
       <c r="G221" t="inlineStr">
         <is>
@@ -52287,7 +52287,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_10A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -52296,7 +52296,7 @@
         </is>
       </c>
       <c r="C222" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D222" t="n">
         <v>1</v>
@@ -52305,7 +52305,7 @@
         <v>42</v>
       </c>
       <c r="F222" t="n">
-        <v>9203</v>
+        <v>5640</v>
       </c>
       <c r="G222" t="inlineStr">
         <is>
@@ -52316,7 +52316,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_2A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -52325,7 +52325,7 @@
         </is>
       </c>
       <c r="C223" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D223" t="n">
         <v>1</v>
@@ -52334,7 +52334,7 @@
         <v>42</v>
       </c>
       <c r="F223" t="n">
-        <v>9203</v>
+        <v>5640</v>
       </c>
       <c r="G223" t="inlineStr">
         <is>
@@ -52345,7 +52345,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_5A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -52354,7 +52354,7 @@
         </is>
       </c>
       <c r="C224" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D224" t="n">
         <v>1</v>
@@ -52363,7 +52363,7 @@
         <v>42</v>
       </c>
       <c r="F224" t="n">
-        <v>9205</v>
+        <v>5640</v>
       </c>
       <c r="G224" t="inlineStr">
         <is>
@@ -52374,7 +52374,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
@@ -52383,7 +52383,7 @@
         </is>
       </c>
       <c r="C225" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D225" t="n">
         <v>1</v>
@@ -52403,7 +52403,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -52412,7 +52412,7 @@
         </is>
       </c>
       <c r="C226" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D226" t="n">
         <v>1</v>
@@ -52432,7 +52432,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -52441,7 +52441,7 @@
         </is>
       </c>
       <c r="C227" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D227" t="n">
         <v>1</v>
@@ -52461,7 +52461,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -52470,7 +52470,7 @@
         </is>
       </c>
       <c r="C228" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D228" t="n">
         <v>1</v>
@@ -52490,7 +52490,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -52499,7 +52499,7 @@
         </is>
       </c>
       <c r="C229" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D229" t="n">
         <v>1</v>
@@ -52519,7 +52519,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
+          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -52528,7 +52528,7 @@
         </is>
       </c>
       <c r="C230" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D230" t="n">
         <v>1</v>
@@ -52548,7 +52548,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
+          <t>tresor_us/dette_quotidienne.csv</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -52557,7 +52557,7 @@
         </is>
       </c>
       <c r="C231" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D231" t="n">
         <v>1</v>
@@ -52566,7 +52566,7 @@
         <v>42</v>
       </c>
       <c r="F231" t="n">
-        <v>5640</v>
+        <v>2000</v>
       </c>
       <c r="G231" t="inlineStr">
         <is>
@@ -52577,7 +52577,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
+          <t>tresor_us/solde_tresorerie.csv</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -52586,7 +52586,7 @@
         </is>
       </c>
       <c r="C232" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D232" t="n">
         <v>1</v>
@@ -52595,7 +52595,7 @@
         <v>42</v>
       </c>
       <c r="F232" t="n">
-        <v>5640</v>
+        <v>500</v>
       </c>
       <c r="G232" t="inlineStr">
         <is>
@@ -52606,7 +52606,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
+          <t>yfinance/XLB.csv</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -52615,7 +52615,7 @@
         </is>
       </c>
       <c r="C233" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D233" t="n">
         <v>1</v>
@@ -52624,7 +52624,7 @@
         <v>42</v>
       </c>
       <c r="F233" t="n">
-        <v>5640</v>
+        <v>500</v>
       </c>
       <c r="G233" t="inlineStr">
         <is>
@@ -52635,7 +52635,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>tresor_us/dette_quotidienne.csv</t>
+          <t>yfinance/XLE.csv</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -52644,7 +52644,7 @@
         </is>
       </c>
       <c r="C234" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D234" t="n">
         <v>1</v>
@@ -52653,7 +52653,7 @@
         <v>42</v>
       </c>
       <c r="F234" t="n">
-        <v>2000</v>
+        <v>500</v>
       </c>
       <c r="G234" t="inlineStr">
         <is>
@@ -52664,7 +52664,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>tresor_us/solde_tresorerie.csv</t>
+          <t>yfinance/XLF.csv</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -52673,7 +52673,7 @@
         </is>
       </c>
       <c r="C235" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D235" t="n">
         <v>1</v>
@@ -52693,16 +52693,16 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>fred/ECBDFR.csv</t>
+          <t>yfinance/XLI.csv</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C236" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D236" t="n">
         <v>1</v>
@@ -52711,7 +52711,7 @@
         <v>42</v>
       </c>
       <c r="F236" t="n">
-        <v>3000</v>
+        <v>500</v>
       </c>
       <c r="G236" t="inlineStr">
         <is>
@@ -52722,16 +52722,16 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>fred/RRPONTSYD.csv</t>
+          <t>yfinance/XLK.csv</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C237" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D237" t="n">
         <v>1</v>
@@ -52740,7 +52740,7 @@
         <v>42</v>
       </c>
       <c r="F237" t="n">
-        <v>3000</v>
+        <v>500</v>
       </c>
       <c r="G237" t="inlineStr">
         <is>
@@ -52751,16 +52751,16 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>fred/T10YIE.csv</t>
+          <t>yfinance/XLP.csv</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C238" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D238" t="n">
         <v>1</v>
@@ -52769,7 +52769,7 @@
         <v>42</v>
       </c>
       <c r="F238" t="n">
-        <v>3000</v>
+        <v>500</v>
       </c>
       <c r="G238" t="inlineStr">
         <is>
@@ -52780,16 +52780,16 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>marches/fx/AUDJPY.csv</t>
+          <t>yfinance/XLRE.csv</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C239" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D239" t="n">
         <v>1</v>
@@ -52798,7 +52798,7 @@
         <v>42</v>
       </c>
       <c r="F239" t="n">
-        <v>3908</v>
+        <v>500</v>
       </c>
       <c r="G239" t="inlineStr">
         <is>
@@ -52809,16 +52809,16 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>marches/fx/AUDUSD.csv</t>
+          <t>yfinance/XLU.csv</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C240" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D240" t="n">
         <v>1</v>
@@ -52827,7 +52827,7 @@
         <v>42</v>
       </c>
       <c r="F240" t="n">
-        <v>3904</v>
+        <v>500</v>
       </c>
       <c r="G240" t="inlineStr">
         <is>
@@ -52838,16 +52838,16 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>marches/fx/DXY.csv</t>
+          <t>yfinance/XLV.csv</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C241" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D241" t="n">
         <v>1</v>
@@ -52856,7 +52856,7 @@
         <v>42</v>
       </c>
       <c r="F241" t="n">
-        <v>3772</v>
+        <v>500</v>
       </c>
       <c r="G241" t="inlineStr">
         <is>
@@ -52867,16 +52867,16 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>marches/fx/EURCHF.csv</t>
+          <t>yfinance/XLY.csv</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C242" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D242" t="n">
         <v>1</v>
@@ -52885,7 +52885,7 @@
         <v>42</v>
       </c>
       <c r="F242" t="n">
-        <v>3905</v>
+        <v>500</v>
       </c>
       <c r="G242" t="inlineStr">
         <is>
@@ -52896,7 +52896,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>marches/fx/EURGBP.csv</t>
+          <t>fred/ECBDFR.csv</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
@@ -52905,7 +52905,7 @@
         </is>
       </c>
       <c r="C243" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D243" t="n">
         <v>1</v>
@@ -52914,7 +52914,7 @@
         <v>42</v>
       </c>
       <c r="F243" t="n">
-        <v>3907</v>
+        <v>3000</v>
       </c>
       <c r="G243" t="inlineStr">
         <is>
@@ -52925,7 +52925,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>marches/fx/EURJPY.csv</t>
+          <t>fred/RRPONTSYD.csv</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -52934,7 +52934,7 @@
         </is>
       </c>
       <c r="C244" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D244" t="n">
         <v>1</v>
@@ -52943,7 +52943,7 @@
         <v>42</v>
       </c>
       <c r="F244" t="n">
-        <v>3907</v>
+        <v>3000</v>
       </c>
       <c r="G244" t="inlineStr">
         <is>
@@ -52954,7 +52954,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>marches/fx/EURUSD.csv</t>
+          <t>fred/T10YIE.csv</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -52963,7 +52963,7 @@
         </is>
       </c>
       <c r="C245" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D245" t="n">
         <v>1</v>
@@ -52972,7 +52972,7 @@
         <v>42</v>
       </c>
       <c r="F245" t="n">
-        <v>3904</v>
+        <v>3000</v>
       </c>
       <c r="G245" t="inlineStr">
         <is>
@@ -52983,7 +52983,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>marches/fx/GBPUSD.csv</t>
+          <t>marches/volatilite/GVZ.csv</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -52992,7 +52992,7 @@
         </is>
       </c>
       <c r="C246" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D246" t="n">
         <v>1</v>
@@ -53001,7 +53001,7 @@
         <v>42</v>
       </c>
       <c r="F246" t="n">
-        <v>3905</v>
+        <v>3770</v>
       </c>
       <c r="G246" t="inlineStr">
         <is>
@@ -53012,7 +53012,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>marches/fx/NZDUSD.csv</t>
+          <t>marches/volatilite/MOVE.csv</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
@@ -53021,7 +53021,7 @@
         </is>
       </c>
       <c r="C247" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D247" t="n">
         <v>1</v>
@@ -53030,7 +53030,7 @@
         <v>42</v>
       </c>
       <c r="F247" t="n">
-        <v>3905</v>
+        <v>3689</v>
       </c>
       <c r="G247" t="inlineStr">
         <is>
@@ -53041,7 +53041,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>marches/fx/USDCAD.csv</t>
+          <t>marches/volatilite/OVX.csv</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
@@ -53050,7 +53050,7 @@
         </is>
       </c>
       <c r="C248" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D248" t="n">
         <v>1</v>
@@ -53059,7 +53059,7 @@
         <v>42</v>
       </c>
       <c r="F248" t="n">
-        <v>3904</v>
+        <v>3770</v>
       </c>
       <c r="G248" t="inlineStr">
         <is>
@@ -53070,7 +53070,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>marches/fx/USDCHF.csv</t>
+          <t>marches/volatilite/VVIX.csv</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
@@ -53079,7 +53079,7 @@
         </is>
       </c>
       <c r="C249" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D249" t="n">
         <v>1</v>
@@ -53088,7 +53088,7 @@
         <v>42</v>
       </c>
       <c r="F249" t="n">
-        <v>3902</v>
+        <v>3762</v>
       </c>
       <c r="G249" t="inlineStr">
         <is>
@@ -53099,7 +53099,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>marches/fx/USDJPY.csv</t>
+          <t>marches/volatilite/VXN.csv</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
@@ -53108,7 +53108,7 @@
         </is>
       </c>
       <c r="C250" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D250" t="n">
         <v>1</v>
@@ -53117,7 +53117,7 @@
         <v>42</v>
       </c>
       <c r="F250" t="n">
-        <v>3905</v>
+        <v>3770</v>
       </c>
       <c r="G250" t="inlineStr">
         <is>
@@ -53128,7 +53128,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>marches/fx/USDKRW.csv</t>
+          <t>yfinance/SP500.csv</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
@@ -53137,7 +53137,7 @@
         </is>
       </c>
       <c r="C251" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D251" t="n">
         <v>1</v>
@@ -53146,7 +53146,7 @@
         <v>42</v>
       </c>
       <c r="F251" t="n">
-        <v>3904</v>
+        <v>7547</v>
       </c>
       <c r="G251" t="inlineStr">
         <is>
@@ -53157,7 +53157,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>marches/fx/USDNOK.csv</t>
+          <t>yfinance/VIX.csv</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -53166,7 +53166,7 @@
         </is>
       </c>
       <c r="C252" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D252" t="n">
         <v>1</v>
@@ -53175,7 +53175,7 @@
         <v>42</v>
       </c>
       <c r="F252" t="n">
-        <v>3905</v>
+        <v>7549</v>
       </c>
       <c r="G252" t="inlineStr">
         <is>
@@ -53186,12 +53186,12 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>marches/fx/USDSEK.csv</t>
+          <t>marches/fx/AUDJPY.csv</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -53204,7 +53204,7 @@
         <v>42</v>
       </c>
       <c r="F253" t="n">
-        <v>3905</v>
+        <v>3908</v>
       </c>
       <c r="G253" t="inlineStr">
         <is>
@@ -53215,12 +53215,12 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>marches/matieres/BRENT.csv</t>
+          <t>marches/fx/AUDUSD.csv</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -53233,7 +53233,7 @@
         <v>42</v>
       </c>
       <c r="F254" t="n">
-        <v>3751</v>
+        <v>3904</v>
       </c>
       <c r="G254" t="inlineStr">
         <is>
@@ -53244,12 +53244,12 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>marches/matieres/CUIVRE.csv</t>
+          <t>marches/fx/DXY.csv</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -53262,7 +53262,7 @@
         <v>42</v>
       </c>
       <c r="F255" t="n">
-        <v>3771</v>
+        <v>3772</v>
       </c>
       <c r="G255" t="inlineStr">
         <is>
@@ -53273,12 +53273,12 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>marches/matieres/GAZ_HENRY_HUB.csv</t>
+          <t>marches/fx/EURCHF.csv</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -53291,7 +53291,7 @@
         <v>42</v>
       </c>
       <c r="F256" t="n">
-        <v>3772</v>
+        <v>3905</v>
       </c>
       <c r="G256" t="inlineStr">
         <is>
@@ -53302,12 +53302,12 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>marches/matieres/OR.csv</t>
+          <t>marches/fx/EURGBP.csv</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -53320,7 +53320,7 @@
         <v>42</v>
       </c>
       <c r="F257" t="n">
-        <v>3771</v>
+        <v>3907</v>
       </c>
       <c r="G257" t="inlineStr">
         <is>
@@ -53331,12 +53331,12 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>marches/matieres/WTI.csv</t>
+          <t>marches/fx/EURJPY.csv</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -53349,7 +53349,7 @@
         <v>42</v>
       </c>
       <c r="F258" t="n">
-        <v>3771</v>
+        <v>3907</v>
       </c>
       <c r="G258" t="inlineStr">
         <is>
@@ -53360,12 +53360,12 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>marches/taux_futures/FED_FUNDS_FRONT.csv</t>
+          <t>marches/fx/EURUSD.csv</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C259" t="n">
@@ -53378,7 +53378,7 @@
         <v>42</v>
       </c>
       <c r="F259" t="n">
-        <v>3772</v>
+        <v>3904</v>
       </c>
       <c r="G259" t="inlineStr">
         <is>
@@ -53389,12 +53389,12 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>marches/volatilite/GVZ.csv</t>
+          <t>marches/fx/GBPUSD.csv</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C260" t="n">
@@ -53407,7 +53407,7 @@
         <v>42</v>
       </c>
       <c r="F260" t="n">
-        <v>3770</v>
+        <v>3905</v>
       </c>
       <c r="G260" t="inlineStr">
         <is>
@@ -53418,12 +53418,12 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>marches/volatilite/MOVE.csv</t>
+          <t>marches/fx/NZDUSD.csv</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C261" t="n">
@@ -53436,7 +53436,7 @@
         <v>42</v>
       </c>
       <c r="F261" t="n">
-        <v>3689</v>
+        <v>3905</v>
       </c>
       <c r="G261" t="inlineStr">
         <is>
@@ -53447,12 +53447,12 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>marches/volatilite/OVX.csv</t>
+          <t>marches/fx/USDCAD.csv</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -53465,7 +53465,7 @@
         <v>42</v>
       </c>
       <c r="F262" t="n">
-        <v>3770</v>
+        <v>3904</v>
       </c>
       <c r="G262" t="inlineStr">
         <is>
@@ -53476,12 +53476,12 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>marches/volatilite/VVIX.csv</t>
+          <t>marches/fx/USDCHF.csv</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C263" t="n">
@@ -53494,7 +53494,7 @@
         <v>42</v>
       </c>
       <c r="F263" t="n">
-        <v>3762</v>
+        <v>3902</v>
       </c>
       <c r="G263" t="inlineStr">
         <is>
@@ -53505,12 +53505,12 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>marches/volatilite/VXN.csv</t>
+          <t>marches/fx/USDCNY.csv</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C264" t="n">
@@ -53523,7 +53523,7 @@
         <v>42</v>
       </c>
       <c r="F264" t="n">
-        <v>3770</v>
+        <v>3904</v>
       </c>
       <c r="G264" t="inlineStr">
         <is>
@@ -53534,12 +53534,12 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>yfinance/SP500.csv</t>
+          <t>marches/fx/USDJPY.csv</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -53552,7 +53552,7 @@
         <v>42</v>
       </c>
       <c r="F265" t="n">
-        <v>7547</v>
+        <v>3905</v>
       </c>
       <c r="G265" t="inlineStr">
         <is>
@@ -53563,12 +53563,12 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>yfinance/VIX.csv</t>
+          <t>marches/fx/USDKRW.csv</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C266" t="n">
@@ -53581,7 +53581,7 @@
         <v>42</v>
       </c>
       <c r="F266" t="n">
-        <v>7549</v>
+        <v>3904</v>
       </c>
       <c r="G266" t="inlineStr">
         <is>
@@ -53592,12 +53592,12 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>yfinance/XLB.csv</t>
+          <t>marches/fx/USDNOK.csv</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -53610,7 +53610,7 @@
         <v>42</v>
       </c>
       <c r="F267" t="n">
-        <v>501</v>
+        <v>3905</v>
       </c>
       <c r="G267" t="inlineStr">
         <is>
@@ -53621,12 +53621,12 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>yfinance/XLE.csv</t>
+          <t>marches/fx/USDSEK.csv</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -53639,7 +53639,7 @@
         <v>42</v>
       </c>
       <c r="F268" t="n">
-        <v>501</v>
+        <v>3905</v>
       </c>
       <c r="G268" t="inlineStr">
         <is>
@@ -53650,12 +53650,12 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>yfinance/XLF.csv</t>
+          <t>marches/indices/KOSPI.csv</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -53668,7 +53668,7 @@
         <v>42</v>
       </c>
       <c r="F269" t="n">
-        <v>501</v>
+        <v>3680</v>
       </c>
       <c r="G269" t="inlineStr">
         <is>
@@ -53679,12 +53679,12 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>yfinance/XLI.csv</t>
+          <t>marches/indices/NIKKEI225.csv</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -53697,7 +53697,7 @@
         <v>42</v>
       </c>
       <c r="F270" t="n">
-        <v>501</v>
+        <v>3666</v>
       </c>
       <c r="G270" t="inlineStr">
         <is>
@@ -53708,12 +53708,12 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>yfinance/XLK.csv</t>
+          <t>marches/matieres/BRENT.csv</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C271" t="n">
@@ -53726,7 +53726,7 @@
         <v>42</v>
       </c>
       <c r="F271" t="n">
-        <v>501</v>
+        <v>3751</v>
       </c>
       <c r="G271" t="inlineStr">
         <is>
@@ -53737,12 +53737,12 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>yfinance/XLP.csv</t>
+          <t>marches/matieres/CUIVRE.csv</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C272" t="n">
@@ -53755,7 +53755,7 @@
         <v>42</v>
       </c>
       <c r="F272" t="n">
-        <v>501</v>
+        <v>3771</v>
       </c>
       <c r="G272" t="inlineStr">
         <is>
@@ -53766,12 +53766,12 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>yfinance/XLRE.csv</t>
+          <t>marches/matieres/GAZ_HENRY_HUB.csv</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -53784,7 +53784,7 @@
         <v>42</v>
       </c>
       <c r="F273" t="n">
-        <v>501</v>
+        <v>3772</v>
       </c>
       <c r="G273" t="inlineStr">
         <is>
@@ -53795,12 +53795,12 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>yfinance/XLU.csv</t>
+          <t>marches/matieres/OR.csv</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C274" t="n">
@@ -53813,7 +53813,7 @@
         <v>42</v>
       </c>
       <c r="F274" t="n">
-        <v>501</v>
+        <v>3771</v>
       </c>
       <c r="G274" t="inlineStr">
         <is>
@@ -53824,12 +53824,12 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>yfinance/XLV.csv</t>
+          <t>marches/matieres/WTI.csv</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -53842,7 +53842,7 @@
         <v>42</v>
       </c>
       <c r="F275" t="n">
-        <v>501</v>
+        <v>3771</v>
       </c>
       <c r="G275" t="inlineStr">
         <is>
@@ -53853,12 +53853,12 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>yfinance/XLY.csv</t>
+          <t>marches/taux_futures/FED_FUNDS_FRONT.csv</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C276" t="n">
@@ -53871,7 +53871,7 @@
         <v>42</v>
       </c>
       <c r="F276" t="n">
-        <v>501</v>
+        <v>3772</v>
       </c>
       <c r="G276" t="inlineStr">
         <is>
@@ -53891,7 +53891,7 @@
         </is>
       </c>
       <c r="C277" t="n">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="D277" t="n">
         <v>2</v>
@@ -53920,7 +53920,7 @@
         </is>
       </c>
       <c r="C278" t="n">
-        <v>-434</v>
+        <v>-433</v>
       </c>
       <c r="D278" t="n">
         <v>42</v>
@@ -55469,17 +55469,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>6889.74</v>
+        <v>6934.3</v>
       </c>
       <c r="D2" t="n">
-        <v>-17.93</v>
+        <v>-16.49</v>
       </c>
       <c r="E2" t="n">
-        <v>103.47</v>
+        <v>102.48</v>
       </c>
     </row>
     <row r="3">
@@ -55490,17 +55490,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>65877.62</v>
+        <v>66476.69</v>
       </c>
       <c r="D3" t="n">
-        <v>-5.17</v>
+        <v>-5.67</v>
       </c>
       <c r="E3" t="n">
-        <v>45.25</v>
+        <v>47.95</v>
       </c>
     </row>
     <row r="4">
@@ -57503,7 +57503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -57864,6 +57864,34 @@
       </c>
       <c r="H12" t="n">
         <v>6.75</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.001579</v>
+      </c>
+      <c r="C13" t="n">
+        <v>5.26</v>
+      </c>
+      <c r="D13" t="n">
+        <v>96.02</v>
+      </c>
+      <c r="E13" t="n">
+        <v>34.16</v>
+      </c>
+      <c r="F13" t="n">
+        <v>43.27</v>
+      </c>
+      <c r="G13" t="n">
+        <v>-6.24</v>
+      </c>
+      <c r="H13" t="n">
+        <v>6.74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-30T02:25Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-30 00:51 UTC</t>
+          <t>Genere le 2026-09-30 02:25 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-30 00:51 UTC</t>
+          <t>Rapport global — 2026-09-30 02:25 UTC</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>**Matieres premieres macro** — le ratio cuivre/or monte -- la croissance domine la peur (+5.3% sur 3 mois). Brent 96.0$ (+34.2% sur 3 mois, +43.3% sur 12 mois), gaz -6.2% sur 3 mois, ecart Brent-WTI +6.7$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-30)_</t>
+          <t>**Matieres premieres macro** — le ratio cuivre/or monte -- la croissance domine la peur (+5.1% sur 3 mois). Brent 96.3$ (+34.6% sur 3 mois, +43.7% sur 12 mois), gaz -6.2% sur 3 mois, ecart Brent-WTI +6.8$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -960,7 +960,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>**Indices mondiaux** — 7 indices (devise locale) : Coree (KOSPI) +102.5% en tete sur 12 mois, Hong Kong (Hang Seng) -5.7% en queue -- ecart tres large entre blocs sur 12 mois (108pt) -- les cycles economiques ou les flux divergent nettement. ROTATION en cours : Coree (KOSPI) mene sur 12 mois mais Hong Kong (Hang Seng) a repris la tete sur 3 mois _(observation : 2026-09-30)_</t>
+          <t>**Indices mondiaux** — 7 indices (devise locale) : Coree (KOSPI) +101.7% en tete sur 12 mois, Hong Kong (Hang Seng) -9.0% en queue -- ecart tres large entre blocs sur 12 mois (111pt) -- les cycles economiques ou les flux divergent nettement. ROTATION en cours : Coree (KOSPI) mene sur 12 mois mais Hong Kong (Hang Seng) a repris la tete sur 3 mois _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1009,7 +1009,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>**Rotation sectorielle** — classement momentum 3 mois (10 secteurs) : 1. Energie (XLE) : +15.90% | 2. Sante (XLV) : +6.54% | 3. Technologie (XLK) : +4.92% | 4. Finance (XLF) : +0.88% | 5. Materiaux (XLB) : -2.35% _(observation : 2026-09-29)_</t>
+          <t>**Rotation sectorielle** — classement momentum 3 mois (10 secteurs) : 1. Energie (XLE) : +15.87% | 2. Sante (XLV) : +7.61% | 3. Technologie (XLK) : +2.09% | 4. Finance (XLF) : +0.75% | 5. Consommation de base (XLP) : -1.47% _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1023,21 +1023,21 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>**Dispersion sectorielle** — 10 secteurs, rendement moyen 3m=-1.38%, dispersion (ecart-type)=8.36pt, etendue=30.61pt -- dispersion intermediaire _(observation : 2026-09-29)_</t>
+          <t>**Dispersion sectorielle** — 10 secteurs, rendement moyen 3m=-1.27%, dispersion (ecart-type)=7.92pt, etendue=28.29pt -- dispersion intermediaire _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>**Low volatility** — tercile bas-vol ['XLF', 'XLRE', 'XLU'] Sharpe=-0.720 vs tercile haut-vol ['XLY', 'XLE', 'XLK'] Sharpe=0.153 -- anomalie low-vol non confirmee sur cet echantillon (puissance statistique faible, n petit -- limite assumee) _(observation : 2026-09-29)_</t>
+          <t>**Low volatility** — tercile bas-vol ['XLF', 'XLRE', 'XLU'] Sharpe=-0.842 vs tercile haut-vol ['XLY', 'XLE', 'XLK'] Sharpe=0.040 -- anomalie low-vol non confirmee sur cet echantillon (puissance statistique faible, n petit -- limite assumee) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>**Momentum cross sectional** — panier gagnant ['XLE', 'XLV', 'XLK'] (+9.12%) vs panier perdant ['XLI', 'XLRE', 'XLU'] (-10.10%) -- spread momentum=+19.22pt _(observation : 2026-09-29)_</t>
+          <t>**Momentum cross sectional** — panier gagnant ['XLE', 'XLV', 'XLK'] (+8.52%) vs panier perdant ['XLY', 'XLI', 'XLU'] (-9.35%) -- spread momentum=+17.87pt _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>**Correlation facteurs** — correlation entre momentum 3m et beta-VIX, 10 secteurs : +0.215 (facteurs largement independants) _(observation : 2026-09-29)_</t>
+          <t>**Correlation facteurs** — correlation entre momentum 3m et beta-VIX, 10 secteurs : +0.361 (facteurs largement independants) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -17308,10 +17308,10 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>-2.5374</v>
+        <v>-2.5102</v>
       </c>
       <c r="D132" t="n">
-        <v>0.2628</v>
+        <v>0.2746</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -17331,10 +17331,10 @@
         </is>
       </c>
       <c r="C133" t="n">
-        <v>-1.8514</v>
+        <v>-1.8331</v>
       </c>
       <c r="D133" t="n">
-        <v>0.6044</v>
+        <v>0.6135</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -17354,10 +17354,10 @@
         </is>
       </c>
       <c r="C134" t="n">
-        <v>-2.1451</v>
+        <v>-2.1416</v>
       </c>
       <c r="D134" t="n">
-        <v>0.4528</v>
+        <v>0.4546</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -17377,10 +17377,10 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>-2.3952</v>
+        <v>-2.3975</v>
       </c>
       <c r="D135" t="n">
-        <v>0.3271</v>
+        <v>0.326</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -17400,10 +17400,10 @@
         </is>
       </c>
       <c r="C136" t="n">
-        <v>-1.3635</v>
+        <v>-1.4392</v>
       </c>
       <c r="D136" t="n">
-        <v>0.8097</v>
+        <v>0.7837</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -17423,10 +17423,10 @@
         </is>
       </c>
       <c r="C137" t="n">
-        <v>0.0851</v>
+        <v>0.0363</v>
       </c>
       <c r="D137" t="n">
-        <v>0.9877</v>
+        <v>0.9867</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -17446,10 +17446,10 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>-1.2195</v>
+        <v>-1.1968</v>
       </c>
       <c r="D138" t="n">
-        <v>0.8527</v>
+        <v>0.8587</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -17469,10 +17469,10 @@
         </is>
       </c>
       <c r="C139" t="n">
-        <v>-0.5135999999999999</v>
+        <v>-0.698</v>
       </c>
       <c r="D139" t="n">
-        <v>0.9634</v>
+        <v>0.9469</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -17492,10 +17492,10 @@
         </is>
       </c>
       <c r="C140" t="n">
-        <v>-2.1811</v>
+        <v>-2.1262</v>
       </c>
       <c r="D140" t="n">
-        <v>0.4341</v>
+        <v>0.4627</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -17515,10 +17515,10 @@
         </is>
       </c>
       <c r="C141" t="n">
-        <v>-1.6158</v>
+        <v>-1.6182</v>
       </c>
       <c r="D141" t="n">
-        <v>0.7141999999999999</v>
+        <v>0.7131</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -51968,7 +51968,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>marches/indices/DAX.csv</t>
+          <t>souverains/CANADA_10A.csv</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
@@ -51986,7 +51986,7 @@
         <v>42</v>
       </c>
       <c r="F211" t="n">
-        <v>3801</v>
+        <v>6437</v>
       </c>
       <c r="G211" t="inlineStr">
         <is>
@@ -51997,7 +51997,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>marches/indices/EUROSTOXX50.csv</t>
+          <t>souverains/CANADA_2A.csv</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -52015,7 +52015,7 @@
         <v>42</v>
       </c>
       <c r="F212" t="n">
-        <v>3758</v>
+        <v>6436</v>
       </c>
       <c r="G212" t="inlineStr">
         <is>
@@ -52026,7 +52026,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>marches/indices/FTSE100.csv</t>
+          <t>souverains/CANADA_5A.csv</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -52044,7 +52044,7 @@
         <v>42</v>
       </c>
       <c r="F213" t="n">
-        <v>3787</v>
+        <v>6436</v>
       </c>
       <c r="G213" t="inlineStr">
         <is>
@@ -52055,7 +52055,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>marches/indices/HANGSENG.csv</t>
+          <t>souverains/CANADA_LONG.csv</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -52073,7 +52073,7 @@
         <v>42</v>
       </c>
       <c r="F214" t="n">
-        <v>3688</v>
+        <v>6436</v>
       </c>
       <c r="G214" t="inlineStr">
         <is>
@@ -52084,7 +52084,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>souverains/CANADA_10A.csv</t>
+          <t>souverains/SUEDE_10A.csv</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -52102,7 +52102,7 @@
         <v>42</v>
       </c>
       <c r="F215" t="n">
-        <v>6437</v>
+        <v>9203</v>
       </c>
       <c r="G215" t="inlineStr">
         <is>
@@ -52113,7 +52113,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>souverains/CANADA_2A.csv</t>
+          <t>souverains/SUEDE_2A.csv</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -52131,7 +52131,7 @@
         <v>42</v>
       </c>
       <c r="F216" t="n">
-        <v>6436</v>
+        <v>9203</v>
       </c>
       <c r="G216" t="inlineStr">
         <is>
@@ -52142,7 +52142,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>souverains/CANADA_5A.csv</t>
+          <t>souverains/SUEDE_5A.csv</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -52160,7 +52160,7 @@
         <v>42</v>
       </c>
       <c r="F217" t="n">
-        <v>6436</v>
+        <v>9205</v>
       </c>
       <c r="G217" t="inlineStr">
         <is>
@@ -52171,7 +52171,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>souverains/CANADA_LONG.csv</t>
+          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -52189,7 +52189,7 @@
         <v>42</v>
       </c>
       <c r="F218" t="n">
-        <v>6436</v>
+        <v>5640</v>
       </c>
       <c r="G218" t="inlineStr">
         <is>
@@ -52200,7 +52200,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_10A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -52218,7 +52218,7 @@
         <v>42</v>
       </c>
       <c r="F219" t="n">
-        <v>9203</v>
+        <v>5640</v>
       </c>
       <c r="G219" t="inlineStr">
         <is>
@@ -52229,7 +52229,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_2A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -52247,7 +52247,7 @@
         <v>42</v>
       </c>
       <c r="F220" t="n">
-        <v>9203</v>
+        <v>5640</v>
       </c>
       <c r="G220" t="inlineStr">
         <is>
@@ -52258,7 +52258,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_5A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -52276,7 +52276,7 @@
         <v>42</v>
       </c>
       <c r="F221" t="n">
-        <v>9205</v>
+        <v>5640</v>
       </c>
       <c r="G221" t="inlineStr">
         <is>
@@ -52287,7 +52287,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -52316,7 +52316,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -52345,7 +52345,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -52374,7 +52374,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
@@ -52403,7 +52403,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
+          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -52432,7 +52432,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
+          <t>tresor_us/dette_quotidienne.csv</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -52450,7 +52450,7 @@
         <v>42</v>
       </c>
       <c r="F227" t="n">
-        <v>5640</v>
+        <v>2000</v>
       </c>
       <c r="G227" t="inlineStr">
         <is>
@@ -52461,7 +52461,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
+          <t>tresor_us/solde_tresorerie.csv</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -52479,7 +52479,7 @@
         <v>42</v>
       </c>
       <c r="F228" t="n">
-        <v>5640</v>
+        <v>500</v>
       </c>
       <c r="G228" t="inlineStr">
         <is>
@@ -52490,16 +52490,16 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
+          <t>fred/ECBDFR.csv</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C229" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D229" t="n">
         <v>1</v>
@@ -52508,7 +52508,7 @@
         <v>42</v>
       </c>
       <c r="F229" t="n">
-        <v>5640</v>
+        <v>3000</v>
       </c>
       <c r="G229" t="inlineStr">
         <is>
@@ -52519,16 +52519,16 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
+          <t>fred/RRPONTSYD.csv</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C230" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D230" t="n">
         <v>1</v>
@@ -52537,7 +52537,7 @@
         <v>42</v>
       </c>
       <c r="F230" t="n">
-        <v>5640</v>
+        <v>3000</v>
       </c>
       <c r="G230" t="inlineStr">
         <is>
@@ -52548,16 +52548,16 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>tresor_us/dette_quotidienne.csv</t>
+          <t>fred/T10YIE.csv</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C231" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D231" t="n">
         <v>1</v>
@@ -52566,7 +52566,7 @@
         <v>42</v>
       </c>
       <c r="F231" t="n">
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="G231" t="inlineStr">
         <is>
@@ -52577,16 +52577,16 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>tresor_us/solde_tresorerie.csv</t>
+          <t>marches/indices/DAX.csv</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C232" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D232" t="n">
         <v>1</v>
@@ -52595,7 +52595,7 @@
         <v>42</v>
       </c>
       <c r="F232" t="n">
-        <v>500</v>
+        <v>3802</v>
       </c>
       <c r="G232" t="inlineStr">
         <is>
@@ -52606,16 +52606,16 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>yfinance/XLB.csv</t>
+          <t>marches/indices/EUROSTOXX50.csv</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C233" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D233" t="n">
         <v>1</v>
@@ -52624,7 +52624,7 @@
         <v>42</v>
       </c>
       <c r="F233" t="n">
-        <v>500</v>
+        <v>3759</v>
       </c>
       <c r="G233" t="inlineStr">
         <is>
@@ -52635,16 +52635,16 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>yfinance/XLE.csv</t>
+          <t>marches/indices/FTSE100.csv</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C234" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D234" t="n">
         <v>1</v>
@@ -52653,7 +52653,7 @@
         <v>42</v>
       </c>
       <c r="F234" t="n">
-        <v>500</v>
+        <v>3788</v>
       </c>
       <c r="G234" t="inlineStr">
         <is>
@@ -52664,16 +52664,16 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>yfinance/XLF.csv</t>
+          <t>marches/volatilite/GVZ.csv</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C235" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D235" t="n">
         <v>1</v>
@@ -52682,7 +52682,7 @@
         <v>42</v>
       </c>
       <c r="F235" t="n">
-        <v>500</v>
+        <v>3770</v>
       </c>
       <c r="G235" t="inlineStr">
         <is>
@@ -52693,16 +52693,16 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>yfinance/XLI.csv</t>
+          <t>marches/volatilite/MOVE.csv</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C236" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D236" t="n">
         <v>1</v>
@@ -52711,7 +52711,7 @@
         <v>42</v>
       </c>
       <c r="F236" t="n">
-        <v>500</v>
+        <v>3689</v>
       </c>
       <c r="G236" t="inlineStr">
         <is>
@@ -52722,16 +52722,16 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>yfinance/XLK.csv</t>
+          <t>marches/volatilite/OVX.csv</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C237" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D237" t="n">
         <v>1</v>
@@ -52740,7 +52740,7 @@
         <v>42</v>
       </c>
       <c r="F237" t="n">
-        <v>500</v>
+        <v>3770</v>
       </c>
       <c r="G237" t="inlineStr">
         <is>
@@ -52751,16 +52751,16 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>yfinance/XLP.csv</t>
+          <t>marches/volatilite/VVIX.csv</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C238" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D238" t="n">
         <v>1</v>
@@ -52769,7 +52769,7 @@
         <v>42</v>
       </c>
       <c r="F238" t="n">
-        <v>500</v>
+        <v>3762</v>
       </c>
       <c r="G238" t="inlineStr">
         <is>
@@ -52780,16 +52780,16 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>yfinance/XLRE.csv</t>
+          <t>marches/volatilite/VXN.csv</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C239" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D239" t="n">
         <v>1</v>
@@ -52798,7 +52798,7 @@
         <v>42</v>
       </c>
       <c r="F239" t="n">
-        <v>500</v>
+        <v>3770</v>
       </c>
       <c r="G239" t="inlineStr">
         <is>
@@ -52809,16 +52809,16 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>yfinance/XLU.csv</t>
+          <t>yfinance/SP500.csv</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C240" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D240" t="n">
         <v>1</v>
@@ -52827,7 +52827,7 @@
         <v>42</v>
       </c>
       <c r="F240" t="n">
-        <v>500</v>
+        <v>7547</v>
       </c>
       <c r="G240" t="inlineStr">
         <is>
@@ -52838,16 +52838,16 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>yfinance/XLV.csv</t>
+          <t>yfinance/VIX.csv</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C241" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D241" t="n">
         <v>1</v>
@@ -52856,7 +52856,7 @@
         <v>42</v>
       </c>
       <c r="F241" t="n">
-        <v>500</v>
+        <v>7549</v>
       </c>
       <c r="G241" t="inlineStr">
         <is>
@@ -52867,16 +52867,16 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>yfinance/XLY.csv</t>
+          <t>yfinance/XLB.csv</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C242" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D242" t="n">
         <v>1</v>
@@ -52885,7 +52885,7 @@
         <v>42</v>
       </c>
       <c r="F242" t="n">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="G242" t="inlineStr">
         <is>
@@ -52896,7 +52896,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>fred/ECBDFR.csv</t>
+          <t>yfinance/XLE.csv</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
@@ -52914,7 +52914,7 @@
         <v>42</v>
       </c>
       <c r="F243" t="n">
-        <v>3000</v>
+        <v>501</v>
       </c>
       <c r="G243" t="inlineStr">
         <is>
@@ -52925,7 +52925,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>fred/RRPONTSYD.csv</t>
+          <t>yfinance/XLF.csv</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -52943,7 +52943,7 @@
         <v>42</v>
       </c>
       <c r="F244" t="n">
-        <v>3000</v>
+        <v>501</v>
       </c>
       <c r="G244" t="inlineStr">
         <is>
@@ -52954,7 +52954,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>fred/T10YIE.csv</t>
+          <t>yfinance/XLI.csv</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -52972,7 +52972,7 @@
         <v>42</v>
       </c>
       <c r="F245" t="n">
-        <v>3000</v>
+        <v>501</v>
       </c>
       <c r="G245" t="inlineStr">
         <is>
@@ -52983,7 +52983,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>marches/volatilite/GVZ.csv</t>
+          <t>yfinance/XLK.csv</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -53001,7 +53001,7 @@
         <v>42</v>
       </c>
       <c r="F246" t="n">
-        <v>3770</v>
+        <v>501</v>
       </c>
       <c r="G246" t="inlineStr">
         <is>
@@ -53012,7 +53012,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>marches/volatilite/MOVE.csv</t>
+          <t>yfinance/XLP.csv</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
@@ -53030,7 +53030,7 @@
         <v>42</v>
       </c>
       <c r="F247" t="n">
-        <v>3689</v>
+        <v>501</v>
       </c>
       <c r="G247" t="inlineStr">
         <is>
@@ -53041,7 +53041,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>marches/volatilite/OVX.csv</t>
+          <t>yfinance/XLRE.csv</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
@@ -53059,7 +53059,7 @@
         <v>42</v>
       </c>
       <c r="F248" t="n">
-        <v>3770</v>
+        <v>501</v>
       </c>
       <c r="G248" t="inlineStr">
         <is>
@@ -53070,7 +53070,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>marches/volatilite/VVIX.csv</t>
+          <t>yfinance/XLU.csv</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
@@ -53088,7 +53088,7 @@
         <v>42</v>
       </c>
       <c r="F249" t="n">
-        <v>3762</v>
+        <v>501</v>
       </c>
       <c r="G249" t="inlineStr">
         <is>
@@ -53099,7 +53099,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>marches/volatilite/VXN.csv</t>
+          <t>yfinance/XLV.csv</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
@@ -53117,7 +53117,7 @@
         <v>42</v>
       </c>
       <c r="F250" t="n">
-        <v>3770</v>
+        <v>501</v>
       </c>
       <c r="G250" t="inlineStr">
         <is>
@@ -53128,7 +53128,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>yfinance/SP500.csv</t>
+          <t>yfinance/XLY.csv</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
@@ -53146,7 +53146,7 @@
         <v>42</v>
       </c>
       <c r="F251" t="n">
-        <v>7547</v>
+        <v>501</v>
       </c>
       <c r="G251" t="inlineStr">
         <is>
@@ -53157,16 +53157,16 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>yfinance/VIX.csv</t>
+          <t>marches/fx/AUDJPY.csv</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C252" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D252" t="n">
         <v>1</v>
@@ -53175,7 +53175,7 @@
         <v>42</v>
       </c>
       <c r="F252" t="n">
-        <v>7549</v>
+        <v>3908</v>
       </c>
       <c r="G252" t="inlineStr">
         <is>
@@ -53186,7 +53186,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>marches/fx/AUDJPY.csv</t>
+          <t>marches/fx/AUDUSD.csv</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -53204,7 +53204,7 @@
         <v>42</v>
       </c>
       <c r="F253" t="n">
-        <v>3908</v>
+        <v>3904</v>
       </c>
       <c r="G253" t="inlineStr">
         <is>
@@ -53215,7 +53215,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>marches/fx/AUDUSD.csv</t>
+          <t>marches/fx/DXY.csv</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
@@ -53233,7 +53233,7 @@
         <v>42</v>
       </c>
       <c r="F254" t="n">
-        <v>3904</v>
+        <v>3773</v>
       </c>
       <c r="G254" t="inlineStr">
         <is>
@@ -53244,7 +53244,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>marches/fx/DXY.csv</t>
+          <t>marches/fx/EURCHF.csv</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
@@ -53262,7 +53262,7 @@
         <v>42</v>
       </c>
       <c r="F255" t="n">
-        <v>3772</v>
+        <v>3905</v>
       </c>
       <c r="G255" t="inlineStr">
         <is>
@@ -53273,7 +53273,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>marches/fx/EURCHF.csv</t>
+          <t>marches/fx/EURGBP.csv</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
@@ -53291,7 +53291,7 @@
         <v>42</v>
       </c>
       <c r="F256" t="n">
-        <v>3905</v>
+        <v>3907</v>
       </c>
       <c r="G256" t="inlineStr">
         <is>
@@ -53302,7 +53302,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>marches/fx/EURGBP.csv</t>
+          <t>marches/fx/EURJPY.csv</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
@@ -53331,7 +53331,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>marches/fx/EURJPY.csv</t>
+          <t>marches/fx/EURUSD.csv</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
@@ -53349,7 +53349,7 @@
         <v>42</v>
       </c>
       <c r="F258" t="n">
-        <v>3907</v>
+        <v>3904</v>
       </c>
       <c r="G258" t="inlineStr">
         <is>
@@ -53360,7 +53360,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>marches/fx/EURUSD.csv</t>
+          <t>marches/fx/GBPUSD.csv</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
@@ -53378,7 +53378,7 @@
         <v>42</v>
       </c>
       <c r="F259" t="n">
-        <v>3904</v>
+        <v>3905</v>
       </c>
       <c r="G259" t="inlineStr">
         <is>
@@ -53389,7 +53389,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>marches/fx/GBPUSD.csv</t>
+          <t>marches/fx/NZDUSD.csv</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
@@ -53418,7 +53418,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>marches/fx/NZDUSD.csv</t>
+          <t>marches/fx/USDCAD.csv</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
@@ -53436,7 +53436,7 @@
         <v>42</v>
       </c>
       <c r="F261" t="n">
-        <v>3905</v>
+        <v>3904</v>
       </c>
       <c r="G261" t="inlineStr">
         <is>
@@ -53447,7 +53447,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>marches/fx/USDCAD.csv</t>
+          <t>marches/fx/USDCHF.csv</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
@@ -53465,7 +53465,7 @@
         <v>42</v>
       </c>
       <c r="F262" t="n">
-        <v>3904</v>
+        <v>3902</v>
       </c>
       <c r="G262" t="inlineStr">
         <is>
@@ -53476,7 +53476,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>marches/fx/USDCHF.csv</t>
+          <t>marches/fx/USDCNY.csv</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
@@ -53494,7 +53494,7 @@
         <v>42</v>
       </c>
       <c r="F263" t="n">
-        <v>3902</v>
+        <v>3904</v>
       </c>
       <c r="G263" t="inlineStr">
         <is>
@@ -53505,7 +53505,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>marches/fx/USDCNY.csv</t>
+          <t>marches/fx/USDJPY.csv</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
@@ -53523,7 +53523,7 @@
         <v>42</v>
       </c>
       <c r="F264" t="n">
-        <v>3904</v>
+        <v>3905</v>
       </c>
       <c r="G264" t="inlineStr">
         <is>
@@ -53534,7 +53534,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>marches/fx/USDJPY.csv</t>
+          <t>marches/fx/USDKRW.csv</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
@@ -53552,7 +53552,7 @@
         <v>42</v>
       </c>
       <c r="F265" t="n">
-        <v>3905</v>
+        <v>3904</v>
       </c>
       <c r="G265" t="inlineStr">
         <is>
@@ -53563,7 +53563,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>marches/fx/USDKRW.csv</t>
+          <t>marches/fx/USDNOK.csv</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
@@ -53581,7 +53581,7 @@
         <v>42</v>
       </c>
       <c r="F266" t="n">
-        <v>3904</v>
+        <v>3905</v>
       </c>
       <c r="G266" t="inlineStr">
         <is>
@@ -53592,7 +53592,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>marches/fx/USDNOK.csv</t>
+          <t>marches/fx/USDSEK.csv</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
@@ -53621,7 +53621,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>marches/fx/USDSEK.csv</t>
+          <t>marches/indices/HANGSENG.csv</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
@@ -53639,7 +53639,7 @@
         <v>42</v>
       </c>
       <c r="F268" t="n">
-        <v>3905</v>
+        <v>3690</v>
       </c>
       <c r="G268" t="inlineStr">
         <is>
@@ -53668,7 +53668,7 @@
         <v>42</v>
       </c>
       <c r="F269" t="n">
-        <v>3680</v>
+        <v>3681</v>
       </c>
       <c r="G269" t="inlineStr">
         <is>
@@ -53697,7 +53697,7 @@
         <v>42</v>
       </c>
       <c r="F270" t="n">
-        <v>3666</v>
+        <v>3667</v>
       </c>
       <c r="G270" t="inlineStr">
         <is>
@@ -53726,7 +53726,7 @@
         <v>42</v>
       </c>
       <c r="F271" t="n">
-        <v>3751</v>
+        <v>3752</v>
       </c>
       <c r="G271" t="inlineStr">
         <is>
@@ -53755,7 +53755,7 @@
         <v>42</v>
       </c>
       <c r="F272" t="n">
-        <v>3771</v>
+        <v>3772</v>
       </c>
       <c r="G272" t="inlineStr">
         <is>
@@ -53784,7 +53784,7 @@
         <v>42</v>
       </c>
       <c r="F273" t="n">
-        <v>3772</v>
+        <v>3773</v>
       </c>
       <c r="G273" t="inlineStr">
         <is>
@@ -53813,7 +53813,7 @@
         <v>42</v>
       </c>
       <c r="F274" t="n">
-        <v>3771</v>
+        <v>3772</v>
       </c>
       <c r="G274" t="inlineStr">
         <is>
@@ -53842,7 +53842,7 @@
         <v>42</v>
       </c>
       <c r="F275" t="n">
-        <v>3771</v>
+        <v>3772</v>
       </c>
       <c r="G275" t="inlineStr">
         <is>
@@ -53871,7 +53871,7 @@
         <v>42</v>
       </c>
       <c r="F276" t="n">
-        <v>3772</v>
+        <v>3773</v>
       </c>
       <c r="G276" t="inlineStr">
         <is>
@@ -55473,13 +55473,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>6934.3</v>
+        <v>6906.37</v>
       </c>
       <c r="D2" t="n">
-        <v>-16.49</v>
+        <v>-16.82</v>
       </c>
       <c r="E2" t="n">
-        <v>102.48</v>
+        <v>101.67</v>
       </c>
     </row>
     <row r="3">
@@ -55494,13 +55494,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>66476.69</v>
+        <v>66329.33</v>
       </c>
       <c r="D3" t="n">
-        <v>-5.67</v>
+        <v>-5.88</v>
       </c>
       <c r="E3" t="n">
-        <v>47.95</v>
+        <v>47.62</v>
       </c>
     </row>
     <row r="4">
@@ -55527,43 +55527,43 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Royaume-Uni (FTSE 100)</t>
+          <t>Zone euro (Euro Stoxx 50)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>10684.9</v>
+        <v>6320.26</v>
       </c>
       <c r="D5" t="n">
-        <v>1.91</v>
+        <v>-0.12</v>
       </c>
       <c r="E5" t="n">
-        <v>15.08</v>
+        <v>14.77</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Zone euro (Euro Stoxx 50)</t>
+          <t>Royaume-Uni (FTSE 100)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>6301.28</v>
+        <v>10636.7</v>
       </c>
       <c r="D6" t="n">
-        <v>1.12</v>
+        <v>1.33</v>
       </c>
       <c r="E6" t="n">
-        <v>14.57</v>
+        <v>14.38</v>
       </c>
     </row>
     <row r="7">
@@ -55574,17 +55574,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>25374.42</v>
+        <v>25399.21</v>
       </c>
       <c r="D7" t="n">
-        <v>3.04</v>
+        <v>1.61</v>
       </c>
       <c r="E7" t="n">
-        <v>6.89</v>
+        <v>6.97</v>
       </c>
     </row>
     <row r="8">
@@ -55595,17 +55595,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>24642.51</v>
+        <v>24432.07</v>
       </c>
       <c r="D8" t="n">
-        <v>7.02</v>
+        <v>6.78</v>
       </c>
       <c r="E8" t="n">
-        <v>-5.69</v>
+        <v>-9.02</v>
       </c>
     </row>
   </sheetData>
@@ -57873,25 +57873,25 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.001579</v>
+        <v>0.001576</v>
       </c>
       <c r="C13" t="n">
-        <v>5.26</v>
+        <v>5.07</v>
       </c>
       <c r="D13" t="n">
-        <v>96.02</v>
+        <v>96.31999999999999</v>
       </c>
       <c r="E13" t="n">
-        <v>34.16</v>
+        <v>34.58</v>
       </c>
       <c r="F13" t="n">
-        <v>43.27</v>
+        <v>43.72</v>
       </c>
       <c r="G13" t="n">
-        <v>-6.24</v>
+        <v>-6.21</v>
       </c>
       <c r="H13" t="n">
-        <v>6.74</v>
+        <v>6.82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-30T06:10Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-30 02:25 UTC</t>
+          <t>Genere le 2026-09-30 06:10 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-30 02:25 UTC</t>
+          <t>Rapport global — 2026-09-30 06:10 UTC</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>**Matieres premieres macro** — le ratio cuivre/or monte -- la croissance domine la peur (+5.1% sur 3 mois). Brent 96.3$ (+34.6% sur 3 mois, +43.7% sur 12 mois), gaz -6.2% sur 3 mois, ecart Brent-WTI +6.8$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-30)_</t>
+          <t>**Matieres premieres macro** — le ratio cuivre/or monte -- la croissance domine la peur (+5.1% sur 3 mois). Brent 96.4$ (+34.7% sur 3 mois, +43.9% sur 12 mois), gaz -6.0% sur 3 mois, ecart Brent-WTI +6.8$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -960,7 +960,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>**Indices mondiaux** — 7 indices (devise locale) : Coree (KOSPI) +101.7% en tete sur 12 mois, Hong Kong (Hang Seng) -9.0% en queue -- ecart tres large entre blocs sur 12 mois (111pt) -- les cycles economiques ou les flux divergent nettement. ROTATION en cours : Coree (KOSPI) mene sur 12 mois mais Hong Kong (Hang Seng) a repris la tete sur 3 mois _(observation : 2026-09-30)_</t>
+          <t>**Indices mondiaux** — 7 indices (devise locale) : Coree (KOSPI) +100.3% en tete sur 12 mois, Hong Kong (Hang Seng) -8.6% en queue -- ecart tres large entre blocs sur 12 mois (109pt) -- les cycles economiques ou les flux divergent nettement. ROTATION en cours : Coree (KOSPI) mene sur 12 mois mais Hong Kong (Hang Seng) a repris la tete sur 3 mois _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1240,7 +1240,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.3726482026081239 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.05235096605723792 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-29)_</t>
+          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.37264820260820386 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.05235096605723774 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -53233,7 +53233,7 @@
         <v>42</v>
       </c>
       <c r="F254" t="n">
-        <v>3773</v>
+        <v>3772</v>
       </c>
       <c r="G254" t="inlineStr">
         <is>
@@ -53726,7 +53726,7 @@
         <v>42</v>
       </c>
       <c r="F271" t="n">
-        <v>3752</v>
+        <v>3751</v>
       </c>
       <c r="G271" t="inlineStr">
         <is>
@@ -53755,7 +53755,7 @@
         <v>42</v>
       </c>
       <c r="F272" t="n">
-        <v>3772</v>
+        <v>3771</v>
       </c>
       <c r="G272" t="inlineStr">
         <is>
@@ -53784,7 +53784,7 @@
         <v>42</v>
       </c>
       <c r="F273" t="n">
-        <v>3773</v>
+        <v>3772</v>
       </c>
       <c r="G273" t="inlineStr">
         <is>
@@ -53813,7 +53813,7 @@
         <v>42</v>
       </c>
       <c r="F274" t="n">
-        <v>3772</v>
+        <v>3771</v>
       </c>
       <c r="G274" t="inlineStr">
         <is>
@@ -53842,7 +53842,7 @@
         <v>42</v>
       </c>
       <c r="F275" t="n">
-        <v>3772</v>
+        <v>3771</v>
       </c>
       <c r="G275" t="inlineStr">
         <is>
@@ -53871,7 +53871,7 @@
         <v>42</v>
       </c>
       <c r="F276" t="n">
-        <v>3773</v>
+        <v>3772</v>
       </c>
       <c r="G276" t="inlineStr">
         <is>
@@ -55473,13 +55473,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>6906.37</v>
+        <v>6861.3</v>
       </c>
       <c r="D2" t="n">
-        <v>-16.82</v>
+        <v>-17.37</v>
       </c>
       <c r="E2" t="n">
-        <v>101.67</v>
+        <v>100.35</v>
       </c>
     </row>
     <row r="3">
@@ -55494,13 +55494,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>66329.33</v>
+        <v>66842.02</v>
       </c>
       <c r="D3" t="n">
-        <v>-5.88</v>
+        <v>-5.15</v>
       </c>
       <c r="E3" t="n">
-        <v>47.62</v>
+        <v>48.76</v>
       </c>
     </row>
     <row r="4">
@@ -55599,13 +55599,13 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>24432.07</v>
+        <v>24537.31</v>
       </c>
       <c r="D8" t="n">
-        <v>6.78</v>
+        <v>7.24</v>
       </c>
       <c r="E8" t="n">
-        <v>-9.02</v>
+        <v>-8.630000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -57873,25 +57873,25 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.001576</v>
+        <v>0.001577</v>
       </c>
       <c r="C13" t="n">
-        <v>5.07</v>
+        <v>5.1</v>
       </c>
       <c r="D13" t="n">
-        <v>96.31999999999999</v>
+        <v>96.44</v>
       </c>
       <c r="E13" t="n">
-        <v>34.58</v>
+        <v>34.75</v>
       </c>
       <c r="F13" t="n">
-        <v>43.72</v>
+        <v>43.9</v>
       </c>
       <c r="G13" t="n">
-        <v>-6.21</v>
+        <v>-5.99</v>
       </c>
       <c r="H13" t="n">
-        <v>6.82</v>
+        <v>6.76</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-30T08:46Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-30 06:10 UTC</t>
+          <t>Genere le 2026-09-30 08:46 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-30 06:10 UTC</t>
+          <t>Rapport global — 2026-09-30 08:46 UTC</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>**Matieres premieres macro** — le ratio cuivre/or monte -- la croissance domine la peur (+5.1% sur 3 mois). Brent 96.4$ (+34.7% sur 3 mois, +43.9% sur 12 mois), gaz -6.0% sur 3 mois, ecart Brent-WTI +6.8$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-30)_</t>
+          <t>**Matieres premieres macro** — ratio cuivre/or stable -- pas de signal net sur la croissance (+4.8% sur 3 mois). Brent 96.8$ (+35.2% sur 3 mois, +44.4% sur 12 mois), gaz -6.0% sur 3 mois, ecart Brent-WTI +6.9$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -862,7 +862,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>**Conditions financieres** — indice conditions financieres=+0.106 (3 composantes: {'taux_directeur': 0.5971439233898245, 'courbe_inversee': 0.23568763984021313, 'vix': -0.5151221380662802}) -- conditions proches de la normale _(observation : 2026-09-28)_</t>
+          <t>**Conditions financieres** — indice conditions financieres=+0.101 (3 composantes: {'taux_directeur': 0.5971439233898245, 'courbe_inversee': 0.23568763984021313, 'vix': -0.5286824498400949}) -- conditions proches de la normale _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -876,7 +876,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>**Pentes courbes** — 7 courbes : pente de +0.30pt (Australie) a +1.20pt (Japon) -- aucune courbe inversee -- pas de signal recessif par la pente _(observation : 2026-09-28)_</t>
+          <t>**Pentes courbes** — 7 courbes : pente de +0.30pt (Australie) a +1.20pt (Japon) -- aucune courbe inversee -- pas de signal recessif par la pente _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -960,7 +960,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>**Indices mondiaux** — 7 indices (devise locale) : Coree (KOSPI) +100.3% en tete sur 12 mois, Hong Kong (Hang Seng) -8.6% en queue -- ecart tres large entre blocs sur 12 mois (109pt) -- les cycles economiques ou les flux divergent nettement. ROTATION en cours : Coree (KOSPI) mene sur 12 mois mais Hong Kong (Hang Seng) a repris la tete sur 3 mois _(observation : 2026-09-30)_</t>
+          <t>**Indices mondiaux** — 7 indices (devise locale) : Coree (KOSPI) +99.7% en tete sur 12 mois, Hong Kong (Hang Seng) -8.3% en queue -- ecart tres large entre blocs sur 12 mois (108pt) -- les cycles economiques ou les flux divergent nettement. ROTATION en cours : Coree (KOSPI) mene sur 12 mois mais Hong Kong (Hang Seng) a repris la tete sur 3 mois _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1191,7 +1191,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>**Vol cross asset** — 6 mesures de volatilite : Petrole (OVX) 86e pct, Or (GVZ) 85e pct, Taux US (MOVE) 58e pct, Nasdaq (VXN) 48e pct, Vol de la vol (VVIX) 33e pct, Actions US (VIX) 32e pct -- stress LOCALISE sur Petrole (OVX), Or (GVZ) pendant que le reste ne l'est pas -- episode propre a cette classe d'actifs, pas une aversion au risque d'ensemble _(observation : 2026-09-29)_</t>
+          <t>**Vol cross asset** — 6 mesures de volatilite : Petrole (OVX) 86e pct, Or (GVZ) 85e pct, Taux US (MOVE) 58e pct, Nasdaq (VXN) 48e pct, Vol de la vol (VVIX) 33e pct, Actions US (VIX) 31e pct -- stress LOCALISE sur Petrole (OVX), Or (GVZ) pendant que le reste ne l'est pas -- episode propre a cette classe d'actifs, pas une aversion au risque d'ensemble _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1219,7 +1219,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>**Ornstein uhlenbeck vix** — VIX actuel=16.04, niveau moyen estime (mu)=20.20, demi-vie=28.8j, ecart actuel=-4.16 -- VIX actuel en-dessous de son niveau moyen de long terme _(observation : 2026-09-29)_</t>
+          <t>**Ornstein uhlenbeck vix** — VIX actuel=15.93, niveau moyen estime (mu)=20.20, demi-vie=28.8j, ecart actuel=-4.27 -- VIX actuel en-dessous de son niveau moyen de long terme _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1233,7 +1233,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>**Kalman niveau local** — VIX observe=16.04, filtre Kalman=16.02 (ecart-type=0.62), ratio signal/bruit=0.2052 -- le filtre lisse fortement le bruit, reagit lentement (ecart obs.-filtre=+0.02) _(observation : 2026-09-29)_</t>
+          <t>**Kalman niveau local** — VIX observe=15.93, filtre Kalman=15.94 (ecart-type=0.62), ratio signal/bruit=0.2052 -- le filtre lisse fortement le bruit, reagit lentement (ecart obs.-filtre=-0.01) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1247,7 +1247,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>**Analyse spectrale** — 3 periodes dominantes (jours de bourse) : [2.2, 4.0, 5.4] -- cycle(s) connu(s) qui ressortent : 4.0j~hebdomadaire, 5.4j~hebdomadaire _(observation : 2026-09-29)_</t>
+          <t>**Analyse spectrale** — 3 periodes dominantes (jours de bourse) : [2.2, 4.0, 5.3] -- cycle(s) connu(s) qui ressortent : 4.0j~hebdomadaire, 5.3j~hebdomadaire _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1317,7 +1317,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>**Qualite regime macro** — instabilite taux=0.0088, instabilite VIX=0.0681 -- score qualite du regime=-0.0384 (plus haut = regime plus stable/previsible) _(observation : 2026-09-28)_</t>
+          <t>**Qualite regime macro** — instabilite taux=0.0088, instabilite VIX=0.0676 -- score qualite du regime=-0.0382 (plus haut = regime plus stable/previsible) _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1331,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>**Decomposition stl** — VIX : tendance=15.52, composante saisonniere (periode 5j)=+0.586, residu=-0.064 -- la saisonnalite explique 0.72% de la variance totale (negligeable) _(observation : 2026-09-29)_</t>
+          <t>**Decomposition stl** — VIX : tendance=15.56, composante saisonniere (periode 5j)=+0.363, residu=+0.010 -- la saisonnalite explique 0.68% de la variance totale (negligeable) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1457,7 +1457,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>**Arima** — ARIMA(1,1,1) sur 100 previsions 1-jour test : RMSE=2.319 vs baseline naive MSE=5.450 -- ARIMA bat la persistance simple _(observation : 2026-09-29)_</t>
+          <t>**Arima** — ARIMA(1,1,1) sur 100 previsions 1-jour test : RMSE=2.323 vs baseline naive MSE=5.451 -- ARIMA bat la persistance simple _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -9145,14 +9145,14 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>16.04</v>
+        <v>15.93</v>
       </c>
       <c r="D7" t="n">
-        <v>32.3</v>
+        <v>31</v>
       </c>
       <c r="E7" t="n">
         <v>1260</v>
@@ -24648,7 +24648,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.1059</v>
+        <v>0.1014</v>
       </c>
       <c r="C15" t="n">
         <v>3</v>
@@ -24660,7 +24660,7 @@
         <v>0.2357</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.5151</v>
+        <v>-0.5286999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -37292,7 +37292,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -37664,6 +37664,31 @@
       </c>
       <c r="G14" t="n">
         <v>351.67</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="C15" t="n">
+        <v>413.56</v>
+      </c>
+      <c r="D15" t="n">
+        <v>4</v>
+      </c>
+      <c r="E15" t="n">
+        <v>373.13</v>
+      </c>
+      <c r="F15" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="G15" t="n">
+        <v>323.93</v>
       </c>
     </row>
   </sheetData>
@@ -38837,7 +38862,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -39119,6 +39144,25 @@
       </c>
       <c r="E14" t="n">
         <v>0.72</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>15.558</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0.363</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.68</v>
       </c>
     </row>
   </sheetData>
@@ -40121,11 +40165,11 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>-0.106</v>
+        <v>-0.09</v>
       </c>
       <c r="D4" t="n">
         <v>0.061</v>
@@ -40266,11 +40310,11 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>-1.581</v>
+        <v>-1.591</v>
       </c>
       <c r="D9" t="n">
         <v>0.065</v>
@@ -45534,7 +45578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -45839,6 +45883,27 @@
         <v>5.4495</v>
       </c>
       <c r="E14" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>100</v>
+      </c>
+      <c r="C15" t="n">
+        <v>2.3232</v>
+      </c>
+      <c r="D15" t="n">
+        <v>5.4506</v>
+      </c>
+      <c r="E15" t="inlineStr">
         <is>
           <t>True</t>
         </is>
@@ -51301,16 +51366,16 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>souverains/UK_10A.csv</t>
+          <t>fred/BAMLC0A0CM.csv</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C188" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D188" t="n">
         <v>1</v>
@@ -51319,7 +51384,7 @@
         <v>42</v>
       </c>
       <c r="F188" t="n">
-        <v>9284</v>
+        <v>793</v>
       </c>
       <c r="G188" t="inlineStr">
         <is>
@@ -51330,16 +51395,16 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>souverains/UK_20A.csv</t>
+          <t>fred/BAMLC0A0CMEY.csv</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C189" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D189" t="n">
         <v>1</v>
@@ -51348,7 +51413,7 @@
         <v>42</v>
       </c>
       <c r="F189" t="n">
-        <v>6755</v>
+        <v>793</v>
       </c>
       <c r="G189" t="inlineStr">
         <is>
@@ -51359,16 +51424,16 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>souverains/UK_5A.csv</t>
+          <t>fred/BAMLEMCBPIOAS.csv</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C190" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D190" t="n">
         <v>1</v>
@@ -51377,7 +51442,7 @@
         <v>42</v>
       </c>
       <c r="F190" t="n">
-        <v>8292</v>
+        <v>793</v>
       </c>
       <c r="G190" t="inlineStr">
         <is>
@@ -51388,7 +51453,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>fred/BAMLC0A0CM.csv</t>
+          <t>fred/BAMLEMFSFCRPIOAS.csv</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -51417,7 +51482,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>fred/BAMLC0A0CMEY.csv</t>
+          <t>fred/BAMLEMHBHYCRPIOAS.csv</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -51446,7 +51511,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>fred/BAMLEMCBPIOAS.csv</t>
+          <t>fred/BAMLEMPBPUBSICRPIOAS.csv</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -51475,7 +51540,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>fred/BAMLEMFSFCRPIOAS.csv</t>
+          <t>fred/BAMLH0A0HYM2.csv</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -51504,7 +51569,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>fred/BAMLEMHBHYCRPIOAS.csv</t>
+          <t>fred/BAMLHE00EHYIEY.csv</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -51533,7 +51598,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>fred/BAMLEMPBPUBSICRPIOAS.csv</t>
+          <t>fred/BAMLHE00EHYIOAS.csv</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -51562,7 +51627,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>fred/BAMLH0A0HYM2.csv</t>
+          <t>fred/DFF.csv</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -51580,7 +51645,7 @@
         <v>42</v>
       </c>
       <c r="F197" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G197" t="inlineStr">
         <is>
@@ -51591,7 +51656,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>fred/BAMLHE00EHYIEY.csv</t>
+          <t>fred/DFII10.csv</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -51609,7 +51674,7 @@
         <v>42</v>
       </c>
       <c r="F198" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G198" t="inlineStr">
         <is>
@@ -51620,7 +51685,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>fred/BAMLHE00EHYIOAS.csv</t>
+          <t>fred/DFII5.csv</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -51638,7 +51703,7 @@
         <v>42</v>
       </c>
       <c r="F199" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G199" t="inlineStr">
         <is>
@@ -51649,7 +51714,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>fred/DFF.csv</t>
+          <t>fred/DGS1.csv</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -51678,7 +51743,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>fred/DFII10.csv</t>
+          <t>fred/DGS10.csv</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -51707,7 +51772,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>fred/DFII5.csv</t>
+          <t>fred/DGS1MO.csv</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -51736,7 +51801,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>fred/DGS1.csv</t>
+          <t>fred/DGS2.csv</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -51765,7 +51830,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>fred/DGS10.csv</t>
+          <t>fred/DGS30.csv</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
@@ -51794,7 +51859,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>fred/DGS1MO.csv</t>
+          <t>fred/DGS3MO.csv</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -51823,7 +51888,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>fred/DGS2.csv</t>
+          <t>fred/DGS5.csv</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -51852,7 +51917,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>fred/DGS30.csv</t>
+          <t>fred/DGS6MO.csv</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -51881,7 +51946,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>fred/DGS3MO.csv</t>
+          <t>souverains/CANADA_10A.csv</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -51899,7 +51964,7 @@
         <v>42</v>
       </c>
       <c r="F208" t="n">
-        <v>3000</v>
+        <v>6437</v>
       </c>
       <c r="G208" t="inlineStr">
         <is>
@@ -51910,7 +51975,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>fred/DGS5.csv</t>
+          <t>souverains/CANADA_2A.csv</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -51928,7 +51993,7 @@
         <v>42</v>
       </c>
       <c r="F209" t="n">
-        <v>3000</v>
+        <v>6436</v>
       </c>
       <c r="G209" t="inlineStr">
         <is>
@@ -51939,7 +52004,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>fred/DGS6MO.csv</t>
+          <t>souverains/CANADA_5A.csv</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -51957,7 +52022,7 @@
         <v>42</v>
       </c>
       <c r="F210" t="n">
-        <v>3000</v>
+        <v>6436</v>
       </c>
       <c r="G210" t="inlineStr">
         <is>
@@ -51968,7 +52033,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>souverains/CANADA_10A.csv</t>
+          <t>souverains/CANADA_LONG.csv</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
@@ -51986,7 +52051,7 @@
         <v>42</v>
       </c>
       <c r="F211" t="n">
-        <v>6437</v>
+        <v>6436</v>
       </c>
       <c r="G211" t="inlineStr">
         <is>
@@ -51997,7 +52062,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>souverains/CANADA_2A.csv</t>
+          <t>souverains/UK_10A.csv</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -52015,7 +52080,7 @@
         <v>42</v>
       </c>
       <c r="F212" t="n">
-        <v>6436</v>
+        <v>9285</v>
       </c>
       <c r="G212" t="inlineStr">
         <is>
@@ -52026,7 +52091,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>souverains/CANADA_5A.csv</t>
+          <t>souverains/UK_20A.csv</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -52044,7 +52109,7 @@
         <v>42</v>
       </c>
       <c r="F213" t="n">
-        <v>6436</v>
+        <v>6756</v>
       </c>
       <c r="G213" t="inlineStr">
         <is>
@@ -52055,7 +52120,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>souverains/CANADA_LONG.csv</t>
+          <t>souverains/UK_5A.csv</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -52073,7 +52138,7 @@
         <v>42</v>
       </c>
       <c r="F214" t="n">
-        <v>6436</v>
+        <v>8293</v>
       </c>
       <c r="G214" t="inlineStr">
         <is>
@@ -52084,7 +52149,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_10A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -52102,7 +52167,7 @@
         <v>42</v>
       </c>
       <c r="F215" t="n">
-        <v>9203</v>
+        <v>5640</v>
       </c>
       <c r="G215" t="inlineStr">
         <is>
@@ -52113,7 +52178,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_2A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -52131,7 +52196,7 @@
         <v>42</v>
       </c>
       <c r="F216" t="n">
-        <v>9203</v>
+        <v>5640</v>
       </c>
       <c r="G216" t="inlineStr">
         <is>
@@ -52142,7 +52207,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_5A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -52160,7 +52225,7 @@
         <v>42</v>
       </c>
       <c r="F217" t="n">
-        <v>9205</v>
+        <v>5640</v>
       </c>
       <c r="G217" t="inlineStr">
         <is>
@@ -52171,7 +52236,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -52200,7 +52265,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -52229,7 +52294,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -52258,7 +52323,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -52287,7 +52352,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -52316,7 +52381,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
+          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -52345,7 +52410,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
+          <t>tresor_us/dette_quotidienne.csv</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -52363,7 +52428,7 @@
         <v>42</v>
       </c>
       <c r="F224" t="n">
-        <v>5640</v>
+        <v>2000</v>
       </c>
       <c r="G224" t="inlineStr">
         <is>
@@ -52374,7 +52439,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
+          <t>tresor_us/solde_tresorerie.csv</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
@@ -52392,7 +52457,7 @@
         <v>42</v>
       </c>
       <c r="F225" t="n">
-        <v>5640</v>
+        <v>500</v>
       </c>
       <c r="G225" t="inlineStr">
         <is>
@@ -52403,16 +52468,16 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
+          <t>fred/ECBDFR.csv</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C226" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D226" t="n">
         <v>1</v>
@@ -52421,7 +52486,7 @@
         <v>42</v>
       </c>
       <c r="F226" t="n">
-        <v>5640</v>
+        <v>3000</v>
       </c>
       <c r="G226" t="inlineStr">
         <is>
@@ -52432,16 +52497,16 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>tresor_us/dette_quotidienne.csv</t>
+          <t>fred/RRPONTSYD.csv</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C227" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D227" t="n">
         <v>1</v>
@@ -52450,7 +52515,7 @@
         <v>42</v>
       </c>
       <c r="F227" t="n">
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="G227" t="inlineStr">
         <is>
@@ -52461,16 +52526,16 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>tresor_us/solde_tresorerie.csv</t>
+          <t>fred/T10YIE.csv</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C228" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D228" t="n">
         <v>1</v>
@@ -52479,7 +52544,7 @@
         <v>42</v>
       </c>
       <c r="F228" t="n">
-        <v>500</v>
+        <v>3000</v>
       </c>
       <c r="G228" t="inlineStr">
         <is>
@@ -52490,7 +52555,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>fred/ECBDFR.csv</t>
+          <t>marches/volatilite/GVZ.csv</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -52508,7 +52573,7 @@
         <v>42</v>
       </c>
       <c r="F229" t="n">
-        <v>3000</v>
+        <v>3770</v>
       </c>
       <c r="G229" t="inlineStr">
         <is>
@@ -52519,7 +52584,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>fred/RRPONTSYD.csv</t>
+          <t>marches/volatilite/MOVE.csv</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -52537,7 +52602,7 @@
         <v>42</v>
       </c>
       <c r="F230" t="n">
-        <v>3000</v>
+        <v>3689</v>
       </c>
       <c r="G230" t="inlineStr">
         <is>
@@ -52548,7 +52613,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>fred/T10YIE.csv</t>
+          <t>marches/volatilite/OVX.csv</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -52566,7 +52631,7 @@
         <v>42</v>
       </c>
       <c r="F231" t="n">
-        <v>3000</v>
+        <v>3770</v>
       </c>
       <c r="G231" t="inlineStr">
         <is>
@@ -52577,7 +52642,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>marches/indices/DAX.csv</t>
+          <t>marches/volatilite/VVIX.csv</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -52595,7 +52660,7 @@
         <v>42</v>
       </c>
       <c r="F232" t="n">
-        <v>3802</v>
+        <v>3762</v>
       </c>
       <c r="G232" t="inlineStr">
         <is>
@@ -52606,7 +52671,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>marches/indices/EUROSTOXX50.csv</t>
+          <t>marches/volatilite/VXN.csv</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -52624,7 +52689,7 @@
         <v>42</v>
       </c>
       <c r="F233" t="n">
-        <v>3759</v>
+        <v>3770</v>
       </c>
       <c r="G233" t="inlineStr">
         <is>
@@ -52635,7 +52700,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>marches/indices/FTSE100.csv</t>
+          <t>souverains/SUEDE_10A.csv</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -52653,7 +52718,7 @@
         <v>42</v>
       </c>
       <c r="F234" t="n">
-        <v>3788</v>
+        <v>9204</v>
       </c>
       <c r="G234" t="inlineStr">
         <is>
@@ -52664,7 +52729,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>marches/volatilite/GVZ.csv</t>
+          <t>souverains/SUEDE_2A.csv</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -52682,7 +52747,7 @@
         <v>42</v>
       </c>
       <c r="F235" t="n">
-        <v>3770</v>
+        <v>9204</v>
       </c>
       <c r="G235" t="inlineStr">
         <is>
@@ -52693,7 +52758,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>marches/volatilite/MOVE.csv</t>
+          <t>souverains/SUEDE_5A.csv</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -52711,7 +52776,7 @@
         <v>42</v>
       </c>
       <c r="F236" t="n">
-        <v>3689</v>
+        <v>9206</v>
       </c>
       <c r="G236" t="inlineStr">
         <is>
@@ -52722,7 +52787,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>marches/volatilite/OVX.csv</t>
+          <t>yfinance/SP500.csv</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
@@ -52740,7 +52805,7 @@
         <v>42</v>
       </c>
       <c r="F237" t="n">
-        <v>3770</v>
+        <v>7547</v>
       </c>
       <c r="G237" t="inlineStr">
         <is>
@@ -52751,7 +52816,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>marches/volatilite/VVIX.csv</t>
+          <t>yfinance/XLB.csv</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
@@ -52769,7 +52834,7 @@
         <v>42</v>
       </c>
       <c r="F238" t="n">
-        <v>3762</v>
+        <v>501</v>
       </c>
       <c r="G238" t="inlineStr">
         <is>
@@ -52780,7 +52845,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>marches/volatilite/VXN.csv</t>
+          <t>yfinance/XLE.csv</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
@@ -52798,7 +52863,7 @@
         <v>42</v>
       </c>
       <c r="F239" t="n">
-        <v>3770</v>
+        <v>501</v>
       </c>
       <c r="G239" t="inlineStr">
         <is>
@@ -52809,7 +52874,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>yfinance/SP500.csv</t>
+          <t>yfinance/XLF.csv</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
@@ -52827,7 +52892,7 @@
         <v>42</v>
       </c>
       <c r="F240" t="n">
-        <v>7547</v>
+        <v>501</v>
       </c>
       <c r="G240" t="inlineStr">
         <is>
@@ -52838,7 +52903,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>yfinance/VIX.csv</t>
+          <t>yfinance/XLI.csv</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
@@ -52856,7 +52921,7 @@
         <v>42</v>
       </c>
       <c r="F241" t="n">
-        <v>7549</v>
+        <v>501</v>
       </c>
       <c r="G241" t="inlineStr">
         <is>
@@ -52867,7 +52932,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>yfinance/XLB.csv</t>
+          <t>yfinance/XLK.csv</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
@@ -52896,7 +52961,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>yfinance/XLE.csv</t>
+          <t>yfinance/XLP.csv</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
@@ -52925,7 +52990,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>yfinance/XLF.csv</t>
+          <t>yfinance/XLRE.csv</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -52954,7 +53019,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>yfinance/XLI.csv</t>
+          <t>yfinance/XLU.csv</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -52983,7 +53048,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>yfinance/XLK.csv</t>
+          <t>yfinance/XLV.csv</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -53012,7 +53077,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>yfinance/XLP.csv</t>
+          <t>yfinance/XLY.csv</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
@@ -53041,16 +53106,16 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>yfinance/XLRE.csv</t>
+          <t>marches/fx/AUDJPY.csv</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C248" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D248" t="n">
         <v>1</v>
@@ -53059,7 +53124,7 @@
         <v>42</v>
       </c>
       <c r="F248" t="n">
-        <v>501</v>
+        <v>3908</v>
       </c>
       <c r="G248" t="inlineStr">
         <is>
@@ -53070,16 +53135,16 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>yfinance/XLU.csv</t>
+          <t>marches/fx/AUDUSD.csv</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C249" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D249" t="n">
         <v>1</v>
@@ -53088,7 +53153,7 @@
         <v>42</v>
       </c>
       <c r="F249" t="n">
-        <v>501</v>
+        <v>3904</v>
       </c>
       <c r="G249" t="inlineStr">
         <is>
@@ -53099,16 +53164,16 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>yfinance/XLV.csv</t>
+          <t>marches/fx/DXY.csv</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C250" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D250" t="n">
         <v>1</v>
@@ -53117,7 +53182,7 @@
         <v>42</v>
       </c>
       <c r="F250" t="n">
-        <v>501</v>
+        <v>3772</v>
       </c>
       <c r="G250" t="inlineStr">
         <is>
@@ -53128,16 +53193,16 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>yfinance/XLY.csv</t>
+          <t>marches/fx/EURCHF.csv</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C251" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D251" t="n">
         <v>1</v>
@@ -53146,7 +53211,7 @@
         <v>42</v>
       </c>
       <c r="F251" t="n">
-        <v>501</v>
+        <v>3905</v>
       </c>
       <c r="G251" t="inlineStr">
         <is>
@@ -53157,7 +53222,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>marches/fx/AUDJPY.csv</t>
+          <t>marches/fx/EURGBP.csv</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -53175,7 +53240,7 @@
         <v>42</v>
       </c>
       <c r="F252" t="n">
-        <v>3908</v>
+        <v>3907</v>
       </c>
       <c r="G252" t="inlineStr">
         <is>
@@ -53186,7 +53251,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>marches/fx/AUDUSD.csv</t>
+          <t>marches/fx/EURJPY.csv</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -53204,7 +53269,7 @@
         <v>42</v>
       </c>
       <c r="F253" t="n">
-        <v>3904</v>
+        <v>3907</v>
       </c>
       <c r="G253" t="inlineStr">
         <is>
@@ -53215,7 +53280,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>marches/fx/DXY.csv</t>
+          <t>marches/fx/EURUSD.csv</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
@@ -53233,7 +53298,7 @@
         <v>42</v>
       </c>
       <c r="F254" t="n">
-        <v>3772</v>
+        <v>3904</v>
       </c>
       <c r="G254" t="inlineStr">
         <is>
@@ -53244,7 +53309,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>marches/fx/EURCHF.csv</t>
+          <t>marches/fx/GBPUSD.csv</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
@@ -53273,7 +53338,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>marches/fx/EURGBP.csv</t>
+          <t>marches/fx/NZDUSD.csv</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
@@ -53291,7 +53356,7 @@
         <v>42</v>
       </c>
       <c r="F256" t="n">
-        <v>3907</v>
+        <v>3905</v>
       </c>
       <c r="G256" t="inlineStr">
         <is>
@@ -53302,7 +53367,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>marches/fx/EURJPY.csv</t>
+          <t>marches/fx/USDCAD.csv</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
@@ -53320,7 +53385,7 @@
         <v>42</v>
       </c>
       <c r="F257" t="n">
-        <v>3907</v>
+        <v>3904</v>
       </c>
       <c r="G257" t="inlineStr">
         <is>
@@ -53331,7 +53396,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>marches/fx/EURUSD.csv</t>
+          <t>marches/fx/USDCHF.csv</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
@@ -53349,7 +53414,7 @@
         <v>42</v>
       </c>
       <c r="F258" t="n">
-        <v>3904</v>
+        <v>3902</v>
       </c>
       <c r="G258" t="inlineStr">
         <is>
@@ -53360,7 +53425,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>marches/fx/GBPUSD.csv</t>
+          <t>marches/fx/USDCNY.csv</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
@@ -53378,7 +53443,7 @@
         <v>42</v>
       </c>
       <c r="F259" t="n">
-        <v>3905</v>
+        <v>3904</v>
       </c>
       <c r="G259" t="inlineStr">
         <is>
@@ -53389,7 +53454,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>marches/fx/NZDUSD.csv</t>
+          <t>marches/fx/USDJPY.csv</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
@@ -53418,7 +53483,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>marches/fx/USDCAD.csv</t>
+          <t>marches/fx/USDKRW.csv</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
@@ -53447,7 +53512,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>marches/fx/USDCHF.csv</t>
+          <t>marches/fx/USDNOK.csv</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
@@ -53465,7 +53530,7 @@
         <v>42</v>
       </c>
       <c r="F262" t="n">
-        <v>3902</v>
+        <v>3905</v>
       </c>
       <c r="G262" t="inlineStr">
         <is>
@@ -53476,7 +53541,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>marches/fx/USDCNY.csv</t>
+          <t>marches/fx/USDSEK.csv</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
@@ -53494,7 +53559,7 @@
         <v>42</v>
       </c>
       <c r="F263" t="n">
-        <v>3904</v>
+        <v>3905</v>
       </c>
       <c r="G263" t="inlineStr">
         <is>
@@ -53505,7 +53570,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>marches/fx/USDJPY.csv</t>
+          <t>marches/indices/DAX.csv</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
@@ -53523,7 +53588,7 @@
         <v>42</v>
       </c>
       <c r="F264" t="n">
-        <v>3905</v>
+        <v>3802</v>
       </c>
       <c r="G264" t="inlineStr">
         <is>
@@ -53534,7 +53599,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>marches/fx/USDKRW.csv</t>
+          <t>marches/indices/EUROSTOXX50.csv</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
@@ -53552,7 +53617,7 @@
         <v>42</v>
       </c>
       <c r="F265" t="n">
-        <v>3904</v>
+        <v>3759</v>
       </c>
       <c r="G265" t="inlineStr">
         <is>
@@ -53563,7 +53628,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>marches/fx/USDNOK.csv</t>
+          <t>marches/indices/FTSE100.csv</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
@@ -53581,7 +53646,7 @@
         <v>42</v>
       </c>
       <c r="F266" t="n">
-        <v>3905</v>
+        <v>3788</v>
       </c>
       <c r="G266" t="inlineStr">
         <is>
@@ -53592,7 +53657,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>marches/fx/USDSEK.csv</t>
+          <t>marches/indices/HANGSENG.csv</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
@@ -53610,7 +53675,7 @@
         <v>42</v>
       </c>
       <c r="F267" t="n">
-        <v>3905</v>
+        <v>3690</v>
       </c>
       <c r="G267" t="inlineStr">
         <is>
@@ -53621,7 +53686,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>marches/indices/HANGSENG.csv</t>
+          <t>marches/indices/KOSPI.csv</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
@@ -53639,7 +53704,7 @@
         <v>42</v>
       </c>
       <c r="F268" t="n">
-        <v>3690</v>
+        <v>3681</v>
       </c>
       <c r="G268" t="inlineStr">
         <is>
@@ -53650,7 +53715,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>marches/indices/KOSPI.csv</t>
+          <t>marches/indices/NIKKEI225.csv</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
@@ -53668,7 +53733,7 @@
         <v>42</v>
       </c>
       <c r="F269" t="n">
-        <v>3681</v>
+        <v>3667</v>
       </c>
       <c r="G269" t="inlineStr">
         <is>
@@ -53679,7 +53744,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>marches/indices/NIKKEI225.csv</t>
+          <t>marches/matieres/BRENT.csv</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
@@ -53697,7 +53762,7 @@
         <v>42</v>
       </c>
       <c r="F270" t="n">
-        <v>3667</v>
+        <v>3751</v>
       </c>
       <c r="G270" t="inlineStr">
         <is>
@@ -53708,7 +53773,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>marches/matieres/BRENT.csv</t>
+          <t>marches/matieres/CUIVRE.csv</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
@@ -53726,7 +53791,7 @@
         <v>42</v>
       </c>
       <c r="F271" t="n">
-        <v>3751</v>
+        <v>3771</v>
       </c>
       <c r="G271" t="inlineStr">
         <is>
@@ -53737,7 +53802,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>marches/matieres/CUIVRE.csv</t>
+          <t>marches/matieres/GAZ_HENRY_HUB.csv</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
@@ -53755,7 +53820,7 @@
         <v>42</v>
       </c>
       <c r="F272" t="n">
-        <v>3771</v>
+        <v>3772</v>
       </c>
       <c r="G272" t="inlineStr">
         <is>
@@ -53766,7 +53831,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>marches/matieres/GAZ_HENRY_HUB.csv</t>
+          <t>marches/matieres/OR.csv</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
@@ -53784,7 +53849,7 @@
         <v>42</v>
       </c>
       <c r="F273" t="n">
-        <v>3772</v>
+        <v>3771</v>
       </c>
       <c r="G273" t="inlineStr">
         <is>
@@ -53795,7 +53860,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>marches/matieres/OR.csv</t>
+          <t>marches/matieres/WTI.csv</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
@@ -53824,7 +53889,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>marches/matieres/WTI.csv</t>
+          <t>marches/taux_futures/FED_FUNDS_FRONT.csv</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
@@ -53842,7 +53907,7 @@
         <v>42</v>
       </c>
       <c r="F275" t="n">
-        <v>3771</v>
+        <v>3772</v>
       </c>
       <c r="G275" t="inlineStr">
         <is>
@@ -53853,7 +53918,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>marches/taux_futures/FED_FUNDS_FRONT.csv</t>
+          <t>yfinance/VIX.csv</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
@@ -53871,7 +53936,7 @@
         <v>42</v>
       </c>
       <c r="F276" t="n">
-        <v>3772</v>
+        <v>7550</v>
       </c>
       <c r="G276" t="inlineStr">
         <is>
@@ -55473,13 +55538,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>6861.3</v>
+        <v>6838.04</v>
       </c>
       <c r="D2" t="n">
-        <v>-17.37</v>
+        <v>-17.65</v>
       </c>
       <c r="E2" t="n">
-        <v>100.35</v>
+        <v>99.67</v>
       </c>
     </row>
     <row r="3">
@@ -55494,13 +55559,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>66842.02</v>
+        <v>66753.72</v>
       </c>
       <c r="D3" t="n">
-        <v>-5.15</v>
+        <v>-5.28</v>
       </c>
       <c r="E3" t="n">
-        <v>48.76</v>
+        <v>48.56</v>
       </c>
     </row>
     <row r="4">
@@ -55532,17 +55597,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>6320.26</v>
+        <v>6342.62</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.12</v>
+        <v>0.96</v>
       </c>
       <c r="E5" t="n">
-        <v>14.77</v>
+        <v>14.7</v>
       </c>
     </row>
     <row r="6">
@@ -55553,17 +55618,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>10636.7</v>
+        <v>10701.33</v>
       </c>
       <c r="D6" t="n">
-        <v>1.33</v>
+        <v>2.13</v>
       </c>
       <c r="E6" t="n">
-        <v>14.38</v>
+        <v>14.45</v>
       </c>
     </row>
     <row r="7">
@@ -55574,17 +55639,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>25399.21</v>
+        <v>25473.98</v>
       </c>
       <c r="D7" t="n">
-        <v>1.61</v>
+        <v>1.73</v>
       </c>
       <c r="E7" t="n">
-        <v>6.97</v>
+        <v>6.67</v>
       </c>
     </row>
     <row r="8">
@@ -55599,13 +55664,13 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>24537.31</v>
+        <v>24613.27</v>
       </c>
       <c r="D8" t="n">
-        <v>7.24</v>
+        <v>7.57</v>
       </c>
       <c r="E8" t="n">
-        <v>-8.630000000000001</v>
+        <v>-8.35</v>
       </c>
     </row>
   </sheetData>
@@ -56028,7 +56093,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -56310,6 +56375,25 @@
       </c>
       <c r="E14" t="n">
         <v>0.20515</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>15.93</v>
+      </c>
+      <c r="C15" t="n">
+        <v>15.943</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.624</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.20516</v>
       </c>
     </row>
   </sheetData>
@@ -57873,25 +57957,25 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.001577</v>
+        <v>0.001572</v>
       </c>
       <c r="C13" t="n">
-        <v>5.1</v>
+        <v>4.8</v>
       </c>
       <c r="D13" t="n">
-        <v>96.44</v>
+        <v>96.77</v>
       </c>
       <c r="E13" t="n">
-        <v>34.75</v>
+        <v>35.21</v>
       </c>
       <c r="F13" t="n">
-        <v>43.9</v>
+        <v>44.39</v>
       </c>
       <c r="G13" t="n">
-        <v>-5.99</v>
+        <v>-5.96</v>
       </c>
       <c r="H13" t="n">
-        <v>6.76</v>
+        <v>6.91</v>
       </c>
     </row>
   </sheetData>
@@ -62188,7 +62272,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -62515,6 +62599,28 @@
       </c>
       <c r="F14" t="n">
         <v>-4.16</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>15.93</v>
+      </c>
+      <c r="C15" t="n">
+        <v>20.199</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.02404</v>
+      </c>
+      <c r="E15" t="n">
+        <v>28.8</v>
+      </c>
+      <c r="F15" t="n">
+        <v>-4.269</v>
       </c>
     </row>
   </sheetData>
@@ -62813,26 +62919,26 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>4.916</v>
+        <v>4.97</v>
       </c>
       <c r="D5" t="n">
-        <v>5.384</v>
+        <v>5.412</v>
       </c>
       <c r="E5" t="n">
-        <v>0.468</v>
+        <v>0.443</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.079</v>
+        <v>-0.096</v>
       </c>
       <c r="G5" t="n">
-        <v>0.668</v>
+        <v>0.727</v>
       </c>
       <c r="H5" t="n">
-        <v>0.589</v>
+        <v>0.631</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -62853,26 +62959,26 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>2.793</v>
+        <v>2.778</v>
       </c>
       <c r="D6" t="n">
-        <v>3.285</v>
+        <v>3.25</v>
       </c>
       <c r="E6" t="n">
-        <v>0.492</v>
+        <v>0.472</v>
       </c>
       <c r="F6" t="n">
-        <v>-0.028</v>
+        <v>-0.06900000000000001</v>
       </c>
       <c r="G6" t="n">
-        <v>0.657</v>
+        <v>0.648</v>
       </c>
       <c r="H6" t="n">
-        <v>0.629</v>
+        <v>0.579</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -68934,10 +69040,10 @@
         <v>0.00877</v>
       </c>
       <c r="C15" t="n">
-        <v>0.06808</v>
+        <v>0.06761</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.03842</v>
+        <v>-0.03819</v>
       </c>
     </row>
   </sheetData>
@@ -82325,13 +82431,13 @@
         <v>12.9</v>
       </c>
       <c r="D4" t="n">
-        <v>5.38</v>
+        <v>5.41</v>
       </c>
       <c r="E4" t="n">
         <v>3.09</v>
       </c>
       <c r="F4" t="n">
-        <v>2.3</v>
+        <v>2.33</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-30T12:46Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-30 08:46 UTC</t>
+          <t>Genere le 2026-09-30 12:46 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-30 08:46 UTC</t>
+          <t>Rapport global — 2026-09-30 12:46 UTC</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>**Matieres premieres macro** — ratio cuivre/or stable -- pas de signal net sur la croissance (+4.8% sur 3 mois). Brent 96.8$ (+35.2% sur 3 mois, +44.4% sur 12 mois), gaz -6.0% sur 3 mois, ecart Brent-WTI +6.9$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-30)_</t>
+          <t>**Matieres premieres macro** — ratio cuivre/or stable -- pas de signal net sur la croissance (+4.6% sur 3 mois). Brent 97.6$ (+36.4% sur 3 mois, +45.7% sur 12 mois), gaz -6.2% sur 3 mois, ecart Brent-WTI +7.2$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -862,7 +862,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>**Conditions financieres** — indice conditions financieres=+0.101 (3 composantes: {'taux_directeur': 0.5971439233898245, 'courbe_inversee': 0.23568763984021313, 'vix': -0.5286824498400949}) -- conditions proches de la normale _(observation : 2026-09-28)_</t>
+          <t>**Conditions financieres** — indice conditions financieres=+0.109 (3 composantes: {'taux_directeur': 0.5971439233898245, 'courbe_inversee': 0.23568763984021313, 'vix': -0.505185598857439}) -- conditions proches de la normale _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -1191,7 +1191,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>**Vol cross asset** — 6 mesures de volatilite : Petrole (OVX) 86e pct, Or (GVZ) 85e pct, Taux US (MOVE) 58e pct, Nasdaq (VXN) 48e pct, Vol de la vol (VVIX) 33e pct, Actions US (VIX) 31e pct -- stress LOCALISE sur Petrole (OVX), Or (GVZ) pendant que le reste ne l'est pas -- episode propre a cette classe d'actifs, pas une aversion au risque d'ensemble _(observation : 2026-09-30)_</t>
+          <t>**Vol cross asset** — 6 mesures de volatilite : Petrole (OVX) 86e pct, Or (GVZ) 85e pct, Taux US (MOVE) 58e pct, Nasdaq (VXN) 48e pct, Actions US (VIX) 33e pct, Vol de la vol (VVIX) 33e pct -- stress LOCALISE sur Petrole (OVX), Or (GVZ) pendant que le reste ne l'est pas -- episode propre a cette classe d'actifs, pas une aversion au risque d'ensemble _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1219,7 +1219,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>**Ornstein uhlenbeck vix** — VIX actuel=15.93, niveau moyen estime (mu)=20.20, demi-vie=28.8j, ecart actuel=-4.27 -- VIX actuel en-dessous de son niveau moyen de long terme _(observation : 2026-09-30)_</t>
+          <t>**Ornstein uhlenbeck vix** — VIX actuel=16.12, niveau moyen estime (mu)=20.20, demi-vie=28.8j, ecart actuel=-4.08 -- VIX actuel en-dessous de son niveau moyen de long terme _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1233,14 +1233,14 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>**Kalman niveau local** — VIX observe=15.93, filtre Kalman=15.94 (ecart-type=0.62), ratio signal/bruit=0.2052 -- le filtre lisse fortement le bruit, reagit lentement (ecart obs.-filtre=-0.01) _(observation : 2026-09-30)_</t>
+          <t>**Kalman niveau local** — VIX observe=16.12, filtre Kalman=16.11 (ecart-type=0.62), ratio signal/bruit=0.2052 -- le filtre lisse fortement le bruit, reagit lentement (ecart obs.-filtre=+0.01) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.37264820260820386 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.05235096605723774 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-29)_</t>
+          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.3726482026081239 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.05235096605723792 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1331,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>**Decomposition stl** — VIX : tendance=15.56, composante saisonniere (periode 5j)=+0.363, residu=+0.010 -- la saisonnalite explique 0.68% de la variance totale (negligeable) _(observation : 2026-09-30)_</t>
+          <t>**Decomposition stl** — VIX : tendance=15.59, composante saisonniere (periode 5j)=+0.433, residu=+0.099 -- la saisonnalite explique 0.71% de la variance totale (negligeable) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>3.73</v>
+        <v>3.7302</v>
       </c>
       <c r="D55" t="n">
         <v>3.88</v>
@@ -5083,10 +5083,10 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>-0.5827</v>
+        <v>-0.5837</v>
       </c>
       <c r="E68" t="n">
-        <v>0.8748</v>
+        <v>0.8746</v>
       </c>
       <c r="F68" t="inlineStr">
         <is>
@@ -5111,10 +5111,10 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>-0.159</v>
+        <v>-0.1754</v>
       </c>
       <c r="E69" t="n">
-        <v>0.9432</v>
+        <v>0.9414</v>
       </c>
       <c r="F69" t="inlineStr">
         <is>
@@ -9114,16 +9114,16 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Vol de la vol (VVIX)</t>
+          <t>Actions US (VIX)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>89.70999999999999</v>
+        <v>16.12</v>
       </c>
       <c r="D6" t="n">
         <v>33.3</v>
@@ -9140,19 +9140,19 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Actions US (VIX)</t>
+          <t>Vol de la vol (VVIX)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>15.93</v>
+        <v>89.70999999999999</v>
       </c>
       <c r="D7" t="n">
-        <v>31</v>
+        <v>33.3</v>
       </c>
       <c r="E7" t="n">
         <v>1260</v>
@@ -21433,10 +21433,10 @@
         </is>
       </c>
       <c r="D139" t="n">
-        <v>-1.9872</v>
+        <v>-1.9877</v>
       </c>
       <c r="E139" t="n">
-        <v>0.5352</v>
+        <v>0.5349</v>
       </c>
       <c r="F139" t="inlineStr">
         <is>
@@ -21461,10 +21461,10 @@
         </is>
       </c>
       <c r="D140" t="n">
-        <v>-2.2113</v>
+        <v>-2.2118</v>
       </c>
       <c r="E140" t="n">
-        <v>0.4185</v>
+        <v>0.4183</v>
       </c>
       <c r="F140" t="inlineStr">
         <is>
@@ -21489,10 +21489,10 @@
         </is>
       </c>
       <c r="D141" t="n">
-        <v>-1.6087</v>
+        <v>-1.609</v>
       </c>
       <c r="E141" t="n">
-        <v>0.7171999999999999</v>
+        <v>0.7171</v>
       </c>
       <c r="F141" t="inlineStr">
         <is>
@@ -21735,14 +21735,14 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-07</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>98.40000000000001</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="E8" t="n">
-        <v>-2.38</v>
+        <v>-0.4</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -21763,14 +21763,14 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-07</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>109.7</v>
+        <v>108.6</v>
       </c>
       <c r="E9" t="n">
-        <v>3.39</v>
+        <v>1.59</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -21819,14 +21819,14 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-07</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>111.5</v>
+        <v>111.6</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.36</v>
+        <v>-0.45</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -24648,7 +24648,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.1014</v>
+        <v>0.1092</v>
       </c>
       <c r="C15" t="n">
         <v>3</v>
@@ -24660,7 +24660,7 @@
         <v>0.2357</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.5286999999999999</v>
+        <v>-0.5052</v>
       </c>
     </row>
   </sheetData>
@@ -37676,19 +37676,19 @@
         <v>2.2</v>
       </c>
       <c r="C15" t="n">
-        <v>413.56</v>
+        <v>413.81</v>
       </c>
       <c r="D15" t="n">
         <v>4</v>
       </c>
       <c r="E15" t="n">
-        <v>373.13</v>
+        <v>373.51</v>
       </c>
       <c r="F15" t="n">
         <v>5.3</v>
       </c>
       <c r="G15" t="n">
-        <v>323.93</v>
+        <v>323.82</v>
       </c>
     </row>
   </sheetData>
@@ -39153,16 +39153,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>15.558</v>
+        <v>15.588</v>
       </c>
       <c r="C15" t="n">
-        <v>0.363</v>
+        <v>0.433</v>
       </c>
       <c r="D15" t="n">
-        <v>0.01</v>
+        <v>0.099</v>
       </c>
       <c r="E15" t="n">
-        <v>0.68</v>
+        <v>0.71</v>
       </c>
     </row>
   </sheetData>
@@ -47103,7 +47103,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>eurostat/ventes_detail/DE.csv</t>
+          <t>eurostat/ventes_detail/EA21.csv</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -47121,7 +47121,7 @@
         <v>279</v>
       </c>
       <c r="F41" t="n">
-        <v>391</v>
+        <v>319</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
@@ -47132,7 +47132,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>eurostat/ventes_detail/EA21.csv</t>
+          <t>eurostat/ventes_detail/IT.csv</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -47161,7 +47161,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>eurostat/ventes_detail/ES.csv</t>
+          <t>fred/BOPGSTB.csv</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -47179,7 +47179,7 @@
         <v>279</v>
       </c>
       <c r="F43" t="n">
-        <v>319</v>
+        <v>415</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
@@ -47190,7 +47190,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>eurostat/ventes_detail/FR.csv</t>
+          <t>fred/IR3TIB01CNM156N.csv</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -47208,7 +47208,7 @@
         <v>279</v>
       </c>
       <c r="F44" t="n">
-        <v>331</v>
+        <v>350</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
@@ -47219,7 +47219,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>eurostat/ventes_detail/IT.csv</t>
+          <t>fred/LRHUTTTTAUM156S.csv</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -47237,7 +47237,7 @@
         <v>279</v>
       </c>
       <c r="F45" t="n">
-        <v>319</v>
+        <v>582</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -47248,7 +47248,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>fred/BOPGSTB.csv</t>
+          <t>fred/LRHUTTTTDEM156S.csv</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -47266,7 +47266,7 @@
         <v>279</v>
       </c>
       <c r="F46" t="n">
-        <v>415</v>
+        <v>427</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -47277,7 +47277,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>fred/IR3TIB01CNM156N.csv</t>
+          <t>fred/LRHUTTTTJPM156S.csv</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -47295,7 +47295,7 @@
         <v>279</v>
       </c>
       <c r="F47" t="n">
-        <v>350</v>
+        <v>859</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -47306,7 +47306,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>fred/LRHUTTTTAUM156S.csv</t>
+          <t>fred/LRHUTTTTKRM156S.csv</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -47324,7 +47324,7 @@
         <v>279</v>
       </c>
       <c r="F48" t="n">
-        <v>582</v>
+        <v>439</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -47335,7 +47335,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>fred/LRHUTTTTDEM156S.csv</t>
+          <t>fred/LRHUTTTTNOM156S.csv</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -47353,7 +47353,7 @@
         <v>279</v>
       </c>
       <c r="F49" t="n">
-        <v>427</v>
+        <v>451</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -47364,7 +47364,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>fred/LRHUTTTTJPM156S.csv</t>
+          <t>fred/LRHUTTTTSEM156S.csv</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -47382,7 +47382,7 @@
         <v>279</v>
       </c>
       <c r="F50" t="n">
-        <v>859</v>
+        <v>523</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -47393,7 +47393,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>fred/LRHUTTTTKRM156S.csv</t>
+          <t>fred/RBUSBIS.csv</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -47411,7 +47411,7 @@
         <v>279</v>
       </c>
       <c r="F51" t="n">
-        <v>439</v>
+        <v>391</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -47422,16 +47422,16 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>fred/LRHUTTTTNOM156S.csv</t>
+          <t>bis/cpi/CA.csv</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>91</v>
+        <v>60</v>
       </c>
       <c r="D52" t="n">
         <v>31</v>
@@ -47440,7 +47440,7 @@
         <v>279</v>
       </c>
       <c r="F52" t="n">
-        <v>451</v>
+        <v>1352</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -47451,16 +47451,16 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>fred/LRHUTTTTSEM156S.csv</t>
+          <t>bis/cpi/CH.csv</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>91</v>
+        <v>60</v>
       </c>
       <c r="D53" t="n">
         <v>31</v>
@@ -47469,7 +47469,7 @@
         <v>279</v>
       </c>
       <c r="F53" t="n">
-        <v>523</v>
+        <v>1268</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
@@ -47480,16 +47480,16 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>fred/RBUSBIS.csv</t>
+          <t>bis/cpi/CN.csv</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>91</v>
+        <v>60</v>
       </c>
       <c r="D54" t="n">
         <v>31</v>
@@ -47498,7 +47498,7 @@
         <v>279</v>
       </c>
       <c r="F54" t="n">
-        <v>391</v>
+        <v>380</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
@@ -47509,7 +47509,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>bis/cpi/CA.csv</t>
+          <t>bis/cpi/GB.csv</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -47527,7 +47527,7 @@
         <v>279</v>
       </c>
       <c r="F55" t="n">
-        <v>1352</v>
+        <v>1340</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
@@ -47538,7 +47538,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>bis/cpi/CH.csv</t>
+          <t>bis/cpi/NO.csv</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -47556,7 +47556,7 @@
         <v>279</v>
       </c>
       <c r="F56" t="n">
-        <v>1268</v>
+        <v>1278</v>
       </c>
       <c r="G56" t="inlineStr">
         <is>
@@ -47567,7 +47567,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>bis/cpi/CN.csv</t>
+          <t>bis/cpi/SE.csv</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -47585,7 +47585,7 @@
         <v>279</v>
       </c>
       <c r="F57" t="n">
-        <v>380</v>
+        <v>1302</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -47596,7 +47596,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>bis/cpi/GB.csv</t>
+          <t>bis/cpi/US.csv</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -47614,7 +47614,7 @@
         <v>279</v>
       </c>
       <c r="F58" t="n">
-        <v>1340</v>
+        <v>1364</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
@@ -47625,7 +47625,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>bis/cpi/NO.csv</t>
+          <t>bis/cpi/XM.csv</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -47643,7 +47643,7 @@
         <v>279</v>
       </c>
       <c r="F59" t="n">
-        <v>1278</v>
+        <v>440</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
@@ -47654,7 +47654,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>bis/cpi/SE.csv</t>
+          <t>eurostat/ventes_detail/DE.csv</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -47672,7 +47672,7 @@
         <v>279</v>
       </c>
       <c r="F60" t="n">
-        <v>1302</v>
+        <v>392</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
@@ -47683,7 +47683,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>bis/cpi/US.csv</t>
+          <t>eurostat/ventes_detail/ES.csv</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -47701,7 +47701,7 @@
         <v>279</v>
       </c>
       <c r="F61" t="n">
-        <v>1364</v>
+        <v>320</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
@@ -47712,7 +47712,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>bis/cpi/XM.csv</t>
+          <t>eurostat/ventes_detail/FR.csv</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -47730,7 +47730,7 @@
         <v>279</v>
       </c>
       <c r="F62" t="n">
-        <v>440</v>
+        <v>332</v>
       </c>
       <c r="G62" t="inlineStr">
         <is>
@@ -51337,16 +51337,16 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>fred/IUDSOIA.csv</t>
+          <t>fred/BAMLC0A0CM.csv</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C187" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D187" t="n">
         <v>1</v>
@@ -51355,7 +51355,7 @@
         <v>42</v>
       </c>
       <c r="F187" t="n">
-        <v>3000</v>
+        <v>793</v>
       </c>
       <c r="G187" t="inlineStr">
         <is>
@@ -51366,7 +51366,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>fred/BAMLC0A0CM.csv</t>
+          <t>fred/BAMLC0A0CMEY.csv</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -51395,7 +51395,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>fred/BAMLC0A0CMEY.csv</t>
+          <t>fred/BAMLEMCBPIOAS.csv</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -51424,7 +51424,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>fred/BAMLEMCBPIOAS.csv</t>
+          <t>fred/BAMLEMFSFCRPIOAS.csv</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -51453,7 +51453,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>fred/BAMLEMFSFCRPIOAS.csv</t>
+          <t>fred/BAMLEMHBHYCRPIOAS.csv</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -51482,7 +51482,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>fred/BAMLEMHBHYCRPIOAS.csv</t>
+          <t>fred/BAMLEMPBPUBSICRPIOAS.csv</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -51511,7 +51511,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>fred/BAMLEMPBPUBSICRPIOAS.csv</t>
+          <t>fred/BAMLH0A0HYM2.csv</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -51540,7 +51540,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>fred/BAMLH0A0HYM2.csv</t>
+          <t>fred/BAMLHE00EHYIEY.csv</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -51569,7 +51569,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>fred/BAMLHE00EHYIEY.csv</t>
+          <t>fred/BAMLHE00EHYIOAS.csv</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -51598,7 +51598,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>fred/BAMLHE00EHYIOAS.csv</t>
+          <t>fred/DFF.csv</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -51616,7 +51616,7 @@
         <v>42</v>
       </c>
       <c r="F196" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G196" t="inlineStr">
         <is>
@@ -51627,7 +51627,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>fred/DFF.csv</t>
+          <t>fred/DFII10.csv</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -51656,7 +51656,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>fred/DFII10.csv</t>
+          <t>fred/DFII5.csv</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -51685,7 +51685,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>fred/DFII5.csv</t>
+          <t>fred/DGS1.csv</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -51714,7 +51714,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>fred/DGS1.csv</t>
+          <t>fred/DGS10.csv</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -51743,7 +51743,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>fred/DGS10.csv</t>
+          <t>fred/DGS1MO.csv</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -51772,7 +51772,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>fred/DGS1MO.csv</t>
+          <t>fred/DGS2.csv</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -51801,7 +51801,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>fred/DGS2.csv</t>
+          <t>fred/DGS30.csv</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -51830,7 +51830,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>fred/DGS30.csv</t>
+          <t>fred/DGS3MO.csv</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
@@ -51859,7 +51859,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>fred/DGS3MO.csv</t>
+          <t>fred/DGS5.csv</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -51888,7 +51888,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>fred/DGS5.csv</t>
+          <t>fred/DGS6MO.csv</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -51917,7 +51917,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>fred/DGS6MO.csv</t>
+          <t>fred/IUDSOIA.csv</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -52149,7 +52149,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
+          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -52178,7 +52178,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
+          <t>tresor_us/dette_quotidienne.csv</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -52196,7 +52196,7 @@
         <v>42</v>
       </c>
       <c r="F216" t="n">
-        <v>5640</v>
+        <v>2000</v>
       </c>
       <c r="G216" t="inlineStr">
         <is>
@@ -52207,7 +52207,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
+          <t>tresor_us/solde_tresorerie.csv</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -52225,7 +52225,7 @@
         <v>42</v>
       </c>
       <c r="F217" t="n">
-        <v>5640</v>
+        <v>500</v>
       </c>
       <c r="G217" t="inlineStr">
         <is>
@@ -52236,16 +52236,16 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
+          <t>fred/RRPONTSYD.csv</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C218" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D218" t="n">
         <v>1</v>
@@ -52254,7 +52254,7 @@
         <v>42</v>
       </c>
       <c r="F218" t="n">
-        <v>5640</v>
+        <v>3000</v>
       </c>
       <c r="G218" t="inlineStr">
         <is>
@@ -52265,16 +52265,16 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
+          <t>fred/T10YIE.csv</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C219" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D219" t="n">
         <v>1</v>
@@ -52283,7 +52283,7 @@
         <v>42</v>
       </c>
       <c r="F219" t="n">
-        <v>5640</v>
+        <v>3000</v>
       </c>
       <c r="G219" t="inlineStr">
         <is>
@@ -52294,16 +52294,16 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
+          <t>marches/volatilite/GVZ.csv</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C220" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D220" t="n">
         <v>1</v>
@@ -52312,7 +52312,7 @@
         <v>42</v>
       </c>
       <c r="F220" t="n">
-        <v>5640</v>
+        <v>3770</v>
       </c>
       <c r="G220" t="inlineStr">
         <is>
@@ -52323,16 +52323,16 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
+          <t>marches/volatilite/MOVE.csv</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C221" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D221" t="n">
         <v>1</v>
@@ -52341,7 +52341,7 @@
         <v>42</v>
       </c>
       <c r="F221" t="n">
-        <v>5640</v>
+        <v>3689</v>
       </c>
       <c r="G221" t="inlineStr">
         <is>
@@ -52352,16 +52352,16 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
+          <t>marches/volatilite/OVX.csv</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C222" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D222" t="n">
         <v>1</v>
@@ -52370,7 +52370,7 @@
         <v>42</v>
       </c>
       <c r="F222" t="n">
-        <v>5640</v>
+        <v>3770</v>
       </c>
       <c r="G222" t="inlineStr">
         <is>
@@ -52381,16 +52381,16 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
+          <t>marches/volatilite/VVIX.csv</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C223" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D223" t="n">
         <v>1</v>
@@ -52399,7 +52399,7 @@
         <v>42</v>
       </c>
       <c r="F223" t="n">
-        <v>5640</v>
+        <v>3762</v>
       </c>
       <c r="G223" t="inlineStr">
         <is>
@@ -52410,16 +52410,16 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>tresor_us/dette_quotidienne.csv</t>
+          <t>marches/volatilite/VXN.csv</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C224" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D224" t="n">
         <v>1</v>
@@ -52428,7 +52428,7 @@
         <v>42</v>
       </c>
       <c r="F224" t="n">
-        <v>2000</v>
+        <v>3770</v>
       </c>
       <c r="G224" t="inlineStr">
         <is>
@@ -52439,16 +52439,16 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>tresor_us/solde_tresorerie.csv</t>
+          <t>souverains/SUEDE_10A.csv</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C225" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D225" t="n">
         <v>1</v>
@@ -52457,7 +52457,7 @@
         <v>42</v>
       </c>
       <c r="F225" t="n">
-        <v>500</v>
+        <v>9204</v>
       </c>
       <c r="G225" t="inlineStr">
         <is>
@@ -52468,7 +52468,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>fred/ECBDFR.csv</t>
+          <t>souverains/SUEDE_2A.csv</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -52486,7 +52486,7 @@
         <v>42</v>
       </c>
       <c r="F226" t="n">
-        <v>3000</v>
+        <v>9204</v>
       </c>
       <c r="G226" t="inlineStr">
         <is>
@@ -52497,7 +52497,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>fred/RRPONTSYD.csv</t>
+          <t>souverains/SUEDE_5A.csv</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -52515,7 +52515,7 @@
         <v>42</v>
       </c>
       <c r="F227" t="n">
-        <v>3000</v>
+        <v>9206</v>
       </c>
       <c r="G227" t="inlineStr">
         <is>
@@ -52526,7 +52526,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>fred/T10YIE.csv</t>
+          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -52544,7 +52544,7 @@
         <v>42</v>
       </c>
       <c r="F228" t="n">
-        <v>3000</v>
+        <v>5641</v>
       </c>
       <c r="G228" t="inlineStr">
         <is>
@@ -52555,7 +52555,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>marches/volatilite/GVZ.csv</t>
+          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -52573,7 +52573,7 @@
         <v>42</v>
       </c>
       <c r="F229" t="n">
-        <v>3770</v>
+        <v>5641</v>
       </c>
       <c r="G229" t="inlineStr">
         <is>
@@ -52584,7 +52584,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>marches/volatilite/MOVE.csv</t>
+          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -52602,7 +52602,7 @@
         <v>42</v>
       </c>
       <c r="F230" t="n">
-        <v>3689</v>
+        <v>5641</v>
       </c>
       <c r="G230" t="inlineStr">
         <is>
@@ -52613,7 +52613,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>marches/volatilite/OVX.csv</t>
+          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -52631,7 +52631,7 @@
         <v>42</v>
       </c>
       <c r="F231" t="n">
-        <v>3770</v>
+        <v>5641</v>
       </c>
       <c r="G231" t="inlineStr">
         <is>
@@ -52642,7 +52642,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>marches/volatilite/VVIX.csv</t>
+          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -52660,7 +52660,7 @@
         <v>42</v>
       </c>
       <c r="F232" t="n">
-        <v>3762</v>
+        <v>5641</v>
       </c>
       <c r="G232" t="inlineStr">
         <is>
@@ -52671,7 +52671,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>marches/volatilite/VXN.csv</t>
+          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -52689,7 +52689,7 @@
         <v>42</v>
       </c>
       <c r="F233" t="n">
-        <v>3770</v>
+        <v>5641</v>
       </c>
       <c r="G233" t="inlineStr">
         <is>
@@ -52700,7 +52700,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_10A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -52718,7 +52718,7 @@
         <v>42</v>
       </c>
       <c r="F234" t="n">
-        <v>9204</v>
+        <v>5641</v>
       </c>
       <c r="G234" t="inlineStr">
         <is>
@@ -52729,7 +52729,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_2A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -52747,7 +52747,7 @@
         <v>42</v>
       </c>
       <c r="F235" t="n">
-        <v>9204</v>
+        <v>5641</v>
       </c>
       <c r="G235" t="inlineStr">
         <is>
@@ -52758,7 +52758,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_5A.csv</t>
+          <t>yfinance/SP500.csv</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -52776,7 +52776,7 @@
         <v>42</v>
       </c>
       <c r="F236" t="n">
-        <v>9206</v>
+        <v>7547</v>
       </c>
       <c r="G236" t="inlineStr">
         <is>
@@ -52787,7 +52787,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>yfinance/SP500.csv</t>
+          <t>yfinance/XLB.csv</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
@@ -52805,7 +52805,7 @@
         <v>42</v>
       </c>
       <c r="F237" t="n">
-        <v>7547</v>
+        <v>501</v>
       </c>
       <c r="G237" t="inlineStr">
         <is>
@@ -52816,7 +52816,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>yfinance/XLB.csv</t>
+          <t>yfinance/XLE.csv</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
@@ -52845,7 +52845,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>yfinance/XLE.csv</t>
+          <t>yfinance/XLF.csv</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
@@ -52874,7 +52874,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>yfinance/XLF.csv</t>
+          <t>yfinance/XLI.csv</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
@@ -52903,7 +52903,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>yfinance/XLI.csv</t>
+          <t>yfinance/XLK.csv</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
@@ -52932,7 +52932,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>yfinance/XLK.csv</t>
+          <t>yfinance/XLP.csv</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
@@ -52961,7 +52961,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>yfinance/XLP.csv</t>
+          <t>yfinance/XLRE.csv</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
@@ -52990,7 +52990,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>yfinance/XLRE.csv</t>
+          <t>yfinance/XLU.csv</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -53019,7 +53019,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>yfinance/XLU.csv</t>
+          <t>yfinance/XLV.csv</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -53048,7 +53048,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>yfinance/XLV.csv</t>
+          <t>yfinance/XLY.csv</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -53077,16 +53077,16 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>yfinance/XLY.csv</t>
+          <t>fred/ECBDFR.csv</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C247" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D247" t="n">
         <v>1</v>
@@ -53095,7 +53095,7 @@
         <v>42</v>
       </c>
       <c r="F247" t="n">
-        <v>501</v>
+        <v>3000</v>
       </c>
       <c r="G247" t="inlineStr">
         <is>
@@ -55601,13 +55601,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>6342.62</v>
+        <v>6294.56</v>
       </c>
       <c r="D5" t="n">
-        <v>0.96</v>
+        <v>0.19</v>
       </c>
       <c r="E5" t="n">
-        <v>14.7</v>
+        <v>13.83</v>
       </c>
     </row>
     <row r="6">
@@ -55622,13 +55622,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>10701.33</v>
+        <v>10637.22</v>
       </c>
       <c r="D6" t="n">
-        <v>2.13</v>
+        <v>1.52</v>
       </c>
       <c r="E6" t="n">
-        <v>14.45</v>
+        <v>13.76</v>
       </c>
     </row>
     <row r="7">
@@ -55643,13 +55643,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>25473.98</v>
+        <v>25295.18</v>
       </c>
       <c r="D7" t="n">
-        <v>1.73</v>
+        <v>1.02</v>
       </c>
       <c r="E7" t="n">
-        <v>6.67</v>
+        <v>5.92</v>
       </c>
     </row>
     <row r="8">
@@ -56384,16 +56384,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>15.93</v>
+        <v>16.120001</v>
       </c>
       <c r="C15" t="n">
-        <v>15.943</v>
+        <v>16.105</v>
       </c>
       <c r="D15" t="n">
         <v>0.624</v>
       </c>
       <c r="E15" t="n">
-        <v>0.20516</v>
+        <v>0.20515</v>
       </c>
     </row>
   </sheetData>
@@ -57957,25 +57957,25 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.001572</v>
+        <v>0.001569</v>
       </c>
       <c r="C13" t="n">
-        <v>4.8</v>
+        <v>4.62</v>
       </c>
       <c r="D13" t="n">
-        <v>96.77</v>
+        <v>97.63</v>
       </c>
       <c r="E13" t="n">
-        <v>35.21</v>
+        <v>36.41</v>
       </c>
       <c r="F13" t="n">
-        <v>44.39</v>
+        <v>45.67</v>
       </c>
       <c r="G13" t="n">
-        <v>-5.96</v>
+        <v>-6.21</v>
       </c>
       <c r="H13" t="n">
-        <v>6.91</v>
+        <v>7.22</v>
       </c>
     </row>
   </sheetData>
@@ -62608,10 +62608,10 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>15.93</v>
+        <v>16.120001</v>
       </c>
       <c r="C15" t="n">
-        <v>20.199</v>
+        <v>20.2</v>
       </c>
       <c r="D15" t="n">
         <v>0.02404</v>
@@ -62620,7 +62620,7 @@
         <v>28.8</v>
       </c>
       <c r="F15" t="n">
-        <v>-4.269</v>
+        <v>-4.08</v>
       </c>
     </row>
   </sheetData>
@@ -62879,26 +62879,26 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>3.233</v>
+        <v>3.211</v>
       </c>
       <c r="D4" t="n">
-        <v>3.631</v>
+        <v>3.608</v>
       </c>
       <c r="E4" t="n">
-        <v>0.398</v>
+        <v>0.397</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.048</v>
+        <v>-0.051</v>
       </c>
       <c r="G4" t="n">
-        <v>0.756</v>
+        <v>0.735</v>
       </c>
       <c r="H4" t="n">
-        <v>0.708</v>
+        <v>0.6830000000000001</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -69040,10 +69040,10 @@
         <v>0.00877</v>
       </c>
       <c r="C15" t="n">
-        <v>0.06761</v>
+        <v>0.06759999999999999</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.03819</v>
+        <v>-0.03818</v>
       </c>
     </row>
   </sheetData>
@@ -74958,7 +74958,7 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>3.73</v>
+        <v>3.7302</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-30T15:21Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-30 12:46 UTC</t>
+          <t>Genere le 2026-09-30 15:21 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-30 12:46 UTC</t>
+          <t>Rapport global — 2026-09-30 15:21 UTC</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>**Matieres premieres macro** — ratio cuivre/or stable -- pas de signal net sur la croissance (+4.6% sur 3 mois). Brent 97.6$ (+36.4% sur 3 mois, +45.7% sur 12 mois), gaz -6.2% sur 3 mois, ecart Brent-WTI +7.2$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-30)_</t>
+          <t>**Matieres premieres macro** — le ratio cuivre/or monte -- la croissance domine la peur (+5.1% sur 3 mois). Brent 98.9$ (+38.2% sur 3 mois, +47.6% sur 12 mois), gaz -6.4% sur 3 mois, ecart Brent-WTI +7.3$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -862,7 +862,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>**Conditions financieres** — indice conditions financieres=+0.109 (3 composantes: {'taux_directeur': 0.5971439233898245, 'courbe_inversee': 0.23568763984021313, 'vix': -0.505185598857439}) -- conditions proches de la normale _(observation : 2026-09-28)_</t>
+          <t>**Conditions financieres** — indice conditions financieres=+0.098 (3 composantes: {'taux_directeur': 0.5971439233898245, 'courbe_inversee': 0.23568763984021313, 'vix': -0.5373391098837522}) -- conditions proches de la normale _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -911,21 +911,21 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>**Facteur qualite credit** — spread HY=3.02, IG=0.83, ecart=2.19pt (niveau contenu), variation 6m=-13.4% -- se resserre (risque credit percu en baisse) _(observation : 2026-09-28)_</t>
+          <t>**Facteur qualite credit** — spread HY=3.08, IG=0.84, ecart=2.24pt (niveau contenu), variation 6m=-5.9% -- se resserre (risque credit percu en baisse) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>**Ornstein uhlenbeck credit** — spread HY actuel=3.02, niveau moyen estime=3.03, demi-vie=40.0j, ecart actuel=-0.01 -- spread HY actuel en-dessous de son niveau moyen de long terme _(observation : 2026-09-28)_</t>
+          <t>**Ornstein uhlenbeck credit** — spread HY actuel=3.08, niveau moyen estime=3.03, demi-vie=38.4j, ecart actuel=+0.05 -- spread HY actuel au-dessus de son niveau moyen de long terme _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>**Momentum credit** — momentum credit 12-1 mois=-0.15pt -- spread qui se resserre (risque credit percu en baisse) _(observation : 2026-09-28)_</t>
+          <t>**Momentum credit** — momentum credit 12-1 mois=-0.14pt -- spread qui se resserre (risque credit percu en baisse) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -960,14 +960,14 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>**Indices mondiaux** — 7 indices (devise locale) : Coree (KOSPI) +99.7% en tete sur 12 mois, Hong Kong (Hang Seng) -8.3% en queue -- ecart tres large entre blocs sur 12 mois (108pt) -- les cycles economiques ou les flux divergent nettement. ROTATION en cours : Coree (KOSPI) mene sur 12 mois mais Hong Kong (Hang Seng) a repris la tete sur 3 mois _(observation : 2026-09-30)_</t>
+          <t>**Indices mondiaux** — 7 indices (devise locale) : Coree (KOSPI) +100.2% en tete sur 12 mois, Hong Kong (Hang Seng) -8.3% en queue -- ecart tres large entre blocs sur 12 mois (109pt) -- les cycles economiques ou les flux divergent nettement. ROTATION en cours : Coree (KOSPI) mene sur 12 mois mais Hong Kong (Hang Seng) a repris la tete sur 3 mois _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>**Correlation glissante** — correlation glissante 60j SP500/VIX = -0.759 (min=-0.955, max=-0.429 sur la fenetre d'historique disponible) -- dans la zone intermediaire de sa fourchette historique _(observation : 2026-09-29)_</t>
+          <t>**Correlation glissante** — correlation glissante 60j SP500/VIX = -0.757 (min=-0.955, max=-0.429 sur la fenetre d'historique disponible) -- dans la zone intermediaire de sa fourchette historique _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -988,7 +988,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>**Momentum prix** — SP500 momentum 12-1 mois = 15.77% -- haussier (momentum positif), detail 1/3/6/12m = [-0.53, 2.29, 17.5, 15.16] _(observation : 2026-09-29)_</t>
+          <t>**Momentum prix** — SP500 momentum 12-1 mois = 14.92% -- haussier (momentum positif), detail 1/3/6/12m = [0.41, 3.13, 17.37, 15.39] _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1002,56 +1002,56 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>**Beta vol** — beta SP500/VIX (60j) = -0.00486 (rendement SP500 pour +1pt VIX) -- sensibilite normale, relation inverse attendue (normale) _(observation : 2026-09-29)_</t>
+          <t>**Beta vol** — beta SP500/VIX (60j) = -0.00486 (rendement SP500 pour +1pt VIX) -- sensibilite normale, relation inverse attendue (normale) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>**Rotation sectorielle** — classement momentum 3 mois (10 secteurs) : 1. Energie (XLE) : +15.87% | 2. Sante (XLV) : +7.61% | 3. Technologie (XLK) : +2.09% | 4. Finance (XLF) : +0.75% | 5. Consommation de base (XLP) : -1.47% _(observation : 2026-09-29)_</t>
+          <t>**Rotation sectorielle** — classement momentum 3 mois (10 secteurs) : 1. Energie (XLE) : +17.15% | 2. Sante (XLV) : +6.59% | 3. Technologie (XLK) : +5.97% | 4. Finance (XLF) : -1.76% | 5. Consommation de base (XLP) : -2.25% _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>**Saisonnalite** — rendement journalier moyen ete=+0.0179%, hiver=+0.0465% (t=-1.03, p=0.3030) -- non significatif (attendu vu la faible puissance sur seulement ~2 ans) _(observation : 2026-09-29)_</t>
+          <t>**Saisonnalite** — rendement journalier moyen ete=+0.0181%, hiver=+0.0465% (t=-1.02, p=0.3056) -- non significatif (attendu vu la faible puissance sur seulement ~2 ans) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>**Dispersion sectorielle** — 10 secteurs, rendement moyen 3m=-1.27%, dispersion (ecart-type)=7.92pt, etendue=28.29pt -- dispersion intermediaire _(observation : 2026-09-29)_</t>
+          <t>**Dispersion sectorielle** — 10 secteurs, rendement moyen 3m=-1.16%, dispersion (ecart-type)=8.24pt, etendue=28.72pt -- dispersion intermediaire _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>**Low volatility** — tercile bas-vol ['XLF', 'XLRE', 'XLU'] Sharpe=-0.842 vs tercile haut-vol ['XLY', 'XLE', 'XLK'] Sharpe=0.040 -- anomalie low-vol non confirmee sur cet echantillon (puissance statistique faible, n petit -- limite assumee) _(observation : 2026-09-29)_</t>
+          <t>**Low volatility** — tercile bas-vol ['XLF', 'XLRE', 'XLU'] Sharpe=-1.005 vs tercile haut-vol ['XLY', 'XLE', 'XLK'] Sharpe=0.101 -- anomalie low-vol non confirmee sur cet echantillon (puissance statistique faible, n petit -- limite assumee) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>**Momentum cross sectional** — panier gagnant ['XLE', 'XLV', 'XLK'] (+8.52%) vs panier perdant ['XLY', 'XLI', 'XLU'] (-9.35%) -- spread momentum=+17.87pt _(observation : 2026-09-29)_</t>
+          <t>**Momentum cross sectional** — panier gagnant ['XLE', 'XLV', 'XLK'] (+9.90%) vs panier perdant ['XLY', 'XLI', 'XLU'] (-8.97%) -- spread momentum=+18.87pt _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>**Cointegration secteurs** — 0/10 secteurs cointegres avec SP500 -- decouples : ['XLK', 'XLF', 'XLE', 'XLV', 'XLI', 'XLY', 'XLP', 'XLU', 'XLB', 'XLRE']  _(sans synthese)_ _(observation : 2026-09-29)_</t>
+          <t>**Cointegration secteurs** — 0/10 secteurs cointegres avec SP500 -- decouples : ['XLK', 'XLF', 'XLE', 'XLV', 'XLI', 'XLY', 'XLP', 'XLU', 'XLB', 'XLRE']  _(sans synthese)_ _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>**Correlation facteurs** — correlation entre momentum 3m et beta-VIX, 10 secteurs : +0.361 (facteurs largement independants) _(observation : 2026-09-29)_</t>
+          <t>**Correlation facteurs** — correlation entre momentum 3m et beta-VIX, 10 secteurs : +0.267 (facteurs largement independants) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1107,7 +1107,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>**Divergence cot prix** — SP500 -0.53% sur 30j, COT net -10560 -&gt; -133228 -- pas de divergence _(observation : 2026-09-29)_</t>
+          <t>**Divergence cot prix** — SP500 +0.41% sur 30j, COT net -10560 -&gt; -133228 -- DIVERGENCE (prix monte, positionnement recule) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1191,56 +1191,56 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>**Vol cross asset** — 6 mesures de volatilite : Petrole (OVX) 86e pct, Or (GVZ) 85e pct, Taux US (MOVE) 58e pct, Nasdaq (VXN) 48e pct, Actions US (VIX) 33e pct, Vol de la vol (VVIX) 33e pct -- stress LOCALISE sur Petrole (OVX), Or (GVZ) pendant que le reste ne l'est pas -- episode propre a cette classe d'actifs, pas une aversion au risque d'ensemble _(observation : 2026-09-30)_</t>
+          <t>**Vol cross asset** — 6 mesures de volatilite : Petrole (OVX) 84e pct, Or (GVZ) 82e pct, Taux US (MOVE) 57e pct, Nasdaq (VXN) 49e pct, Vol de la vol (VVIX) 32e pct, Actions US (VIX) 31e pct -- stress LOCALISE sur Petrole (OVX), Or (GVZ) pendant que le reste ne l'est pas -- episode propre a cette classe d'actifs, pas une aversion au risque d'ensemble _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>**Volatilite ewma** — vol realisee 60j=0.11200833249006233, EWMA=0.1059 (tendance 10 runs: stable) _(observation : 2026-09-29)_</t>
+          <t>**Volatilite ewma** — vol realisee 60j=0.11218051553973624, EWMA=0.1054 (tendance 10 runs: stable) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>**Garch** — vol GARCH(1,1) annualisee=0.1224 (alpha=0.114, beta=0.868, persistance=0.983 -- tres proche de 1 -- chocs de volatilite tres durables) _(observation : 2026-09-29)_</t>
+          <t>**Garch** — vol GARCH(1,1) annualisee=0.1171 (alpha=0.114, beta=0.868, persistance=0.983 -- tres proche de 1 -- chocs de volatilite tres durables) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>**Hurst** — Hurst=0.5507 (R2 regression=1.000) -- persistant (tendanciel) _(observation : 2026-09-29)_</t>
+          <t>**Hurst** — Hurst=0.5507 (R2 regression=1.000) -- persistant (tendanciel) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>**Ornstein uhlenbeck vix** — VIX actuel=16.12, niveau moyen estime (mu)=20.20, demi-vie=28.8j, ecart actuel=-4.08 -- VIX actuel en-dessous de son niveau moyen de long terme _(observation : 2026-09-30)_</t>
+          <t>**Ornstein uhlenbeck vix** — VIX actuel=15.86, niveau moyen estime (mu)=20.20, demi-vie=28.8j, ecart actuel=-4.34 -- VIX actuel en-dessous de son niveau moyen de long terme _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>**Changepoint volatilite** — rupture detectee le 2011-12-21 -- vol avant=0.2130, vol apres=0.1666 (reduction SSE=0.5%) -- baisse de la vol au point de rupture (-21.8%) _(observation : 2026-09-29)_</t>
+          <t>**Changepoint volatilite** — rupture detectee le 2011-12-21 -- vol avant=0.2130, vol apres=0.1666 (reduction SSE=0.5%) -- baisse de la vol au point de rupture (-21.8%) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>**Kalman niveau local** — VIX observe=16.12, filtre Kalman=16.11 (ecart-type=0.62), ratio signal/bruit=0.2052 -- le filtre lisse fortement le bruit, reagit lentement (ecart obs.-filtre=+0.01) _(observation : 2026-09-30)_</t>
+          <t>**Kalman niveau local** — VIX observe=15.86, filtre Kalman=15.88 (ecart-type=0.62), ratio signal/bruit=0.2052 -- le filtre lisse fortement le bruit, reagit lentement (ecart obs.-filtre=-0.02) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.3726482026081239 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.05235096605723792 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-29)_</t>
+          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.3727962617538463 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.052375438187575216 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1254,42 +1254,42 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>**Var drawdown** — VaR95=-1.45% CVaR95=-1.80% VaR99=-2.08% CVaR99=-2.50% drawdown_max_252j=-9.10% -- soit l'equivalent de ~6 jours de VaR95 d'affilee _(observation : 2026-09-29)_</t>
+          <t>**Var drawdown** — VaR95=-1.45% CVaR95=-1.80% VaR99=-2.08% CVaR99=-2.50% drawdown_max_252j=-9.10% -- soit l'equivalent de ~6 jours de VaR95 d'affilee _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>**Skew kurtosis** — skewness=-0.190 (asymetrie negative (pertes extremes &gt; gains extremes)), kurtosis exces=+1.022 (queues epaisses (risque extreme sous-estime par une hypothese normale)) _(observation : 2026-09-29)_</t>
+          <t>**Skew kurtosis** — skewness=-0.194 (asymetrie negative (pertes extremes &gt; gains extremes)), kurtosis exces=+1.012 (queues epaisses (risque extreme sous-estime par une hypothese normale)) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>**Ratios performance** — Sharpe=1.090 (bon), Sortino=1.076 (bon), Calmar=1.557 (bon) -- lecture sur fenetre 252j (~1 an, echantillon limite), seuils academiques standards, taux sans risque suppose nul _(observation : 2026-09-29)_</t>
+          <t>**Ratios performance** — Sharpe=1.105 (bon), Sortino=1.091 (bon), Calmar=1.579 (bon) -- lecture sur fenetre 252j (~1 an, echantillon limite), seuils academiques standards, taux sans risque suppose nul _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>**Covar** — VaR95 inconditionnelle=-1.84%, VaR95|VIX detresse(&gt;=29.5)=-4.37%, VaR95|VIX normal=-1.52% -- DeltaCoVaR=-2.86pt (755 jours de detresse dans l'echantillon) -- contagion notable -- VaR 2.9x plus severe en detresse _(observation : 2026-09-29)_</t>
+          <t>**Covar** — VaR95 inconditionnelle=-1.84%, VaR95|VIX detresse(&gt;=29.5)=-4.37%, VaR95|VIX normal=-1.52% -- DeltaCoVaR=-2.86pt (755 jours de detresse dans l'echantillon) -- contagion notable -- VaR 2.9x plus severe en detresse _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>**Stress test historique** — COVID_2020 (2020-02-19 -&gt; 2020-03-23) : chute historique=-33.9% -- rejouee sur le niveau actuel (7671) -&gt; 5069  _(sans synthese)_ _(observation : 2026-09-29)_</t>
+          <t>**Stress test historique** — COVID_2020 (2020-02-19 -&gt; 2020-03-23) : chute historique=-33.9% -- rejouee sur le niveau actuel (7718) -&gt; 5099  _(sans synthese)_ _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>**Sizing robuste** — vol point estimate=0.1298, IC90%=[0.1174, 0.1411] (1000 tirages bootstrap) -- intervalle etroit (18% du point estimate) -- estimation relativement fiable _(observation : 2026-09-29)_</t>
+          <t>**Sizing robuste** — vol point estimate=0.1299, IC90%=[0.1176, 0.1415] (1000 tirages bootstrap) -- intervalle etroit (18% du point estimate) -- estimation relativement fiable _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1303,7 +1303,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>**Detection saut** — Z-stat BNS (fenetre 22j)=0.970 (seuil ±1.96) -- pas de saut isole detecte _(observation : 2026-09-29)_</t>
+          <t>**Detection saut** — Z-stat BNS (fenetre 22j)=1.172 (seuil ±1.96) -- pas de saut isole detecte _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1324,28 +1324,28 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>**Var conditionnelle regime** — regime VIX actuel=bas (rang percentile=33) -- VaR95 applicable maintenant=-1.14% (vs VaR95 globale non-conditionnelle=-1.84%) _(observation : 2026-09-29)_</t>
+          <t>**Var conditionnelle regime** — regime VIX actuel=bas (rang percentile=33) -- VaR95 applicable maintenant=-1.14% (vs VaR95 globale non-conditionnelle=-1.84%) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>**Decomposition stl** — VIX : tendance=15.59, composante saisonniere (periode 5j)=+0.433, residu=+0.099 -- la saisonnalite explique 0.71% de la variance totale (negligeable) _(observation : 2026-09-30)_</t>
+          <t>**Decomposition stl** — VIX : tendance=15.55, composante saisonniere (periode 5j)=+0.336, residu=-0.023 -- la saisonnalite explique 0.68% de la variance totale (negligeable) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>**Ratios conditionnels regime** — Sharpe regime haut-vol=-1.107, bas-vol=2.401, global=0.421 -- meilleur en regime calme, comme attendu _(observation : 2026-09-29)_</t>
+          <t>**Ratios conditionnels regime** — Sharpe regime haut-vol=-1.107, bas-vol=2.403, global=0.422 -- meilleur en regime calme, comme attendu _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>**Choc vol parametrique** — vol actuelle=12.98%, scenarios x1/x2/x3 calcules -- pire scenario (x3) = -3.98%/jour, soit 3.1x le scenario de base _(observation : 2026-09-29)_</t>
+          <t>**Choc vol parametrique** — vol actuelle=12.99%, scenarios x1/x2/x3 calcules -- pire scenario (x3) = -3.98%/jour, soit 3.1x le scenario de base _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1366,42 +1366,42 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>**Causalite granger** — causalite Granger detectee : SP500_cause_VIX (lag=5) _(observation : 2026-09-29)_</t>
+          <t>**Causalite granger** — causalite Granger detectee : SP500_cause_VIX (lag=5) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>**Dependance queue** — 518/7546 jours conjointement extremes (SP500 pire 10% ET VIX pire 10%), P observee=0.0686 vs P sous independance=0.0100 -- coefficient de dependance de queue=6.86 (dependance reelle) _(observation : 2026-09-29)_</t>
+          <t>**Dependance queue** — 518/7547 jours conjointement extremes (SP500 pire 10% ET VIX pire 10%), P observee=0.0686 vs P sous independance=0.0100 -- coefficient de dependance de queue=6.86 (dependance reelle) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>**Walkforward direction** — 7516 predictions walk-forward -- momentum 5j=0.4959 vs baseline majoritaire=0.5373 -- NE BAT PAS la baseline (resultat honnete, pas ajuste pour paraitre mieux) _(observation : 2026-09-29)_</t>
+          <t>**Walkforward direction** — 7517 predictions walk-forward -- momentum 5j=0.4958 vs baseline majoritaire=0.5373 -- NE BAT PAS la baseline (resultat honnete, pas ajuste pour paraitre mieux) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>**Anomalie multivariee** — distance de Mahalanobis=0.512 (seuil 3.0) -- jour ordinaire _(observation : 2026-09-29)_</t>
+          <t>**Anomalie multivariee** — distance de Mahalanobis=1.020 (seuil 3.0) -- jour ordinaire _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>**Test overfitting** — meilleure fenetre in-sample=23j (accuracy=0.5163) vs meme fenetre en walk-forward=0.5160 -- ecart=+0.0003 (ecart faible) _(observation : 2026-09-29)_</t>
+          <t>**Test overfitting** — meilleure fenetre in-sample=23j (accuracy=0.5162) vs meme fenetre en walk-forward=0.5159 -- ecart=+0.0003 (ecart faible) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>**Prevision vol regression** — regression AR(1) (a=0.000116, b=0.2096) MSE=2.9848e-07 vs baseline persistance MSE=3.8344e-07 -- BAT la baseline (resultat honnete, pas ajuste) _(observation : 2026-09-29)_</t>
+          <t>**Prevision vol regression** — regression AR(1) (a=0.000116, b=0.2096) MSE=2.9835e-07 vs baseline persistance MSE=3.8327e-07 -- BAT la baseline (resultat honnete, pas ajuste) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1415,28 +1415,28 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>**Ensemble signaux** — 7516 predictions -- momentum=0.4959, vix=0.4988, ensemble=0.4988, baseline=0.5373 -- ensemble NE BAT PAS la baseline _(observation : 2026-09-29)_</t>
+          <t>**Ensemble signaux** — 7517 predictions -- momentum=0.4958, vix=0.4989, ensemble=0.4989, baseline=0.5373 -- ensemble NE BAT PAS la baseline _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>**Screening features** — 2/4 features avec un lien univarie significatif (p&lt;0.05, sans correction multiple-testing ici -- seulement 4 tests)  _(sans synthese)_ _(observation : 2026-09-29)_</t>
+          <t>**Screening features** — 2/4 features avec un lien univarie significatif (p&lt;0.05, sans correction multiple-testing ici -- seulement 4 tests)  _(sans synthese)_ _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>**Couts transaction** — 7516 predictions, 1513 changements de position (5pb/changement) -- rendement cumule brut=-93.19%, cout total=53.08%, net=-96.80% -- les frais mangent une part importante du rendement (&gt;50% du brut) _(observation : 2026-09-29)_</t>
+          <t>**Couts transaction** — 7517 predictions, 1513 changements de position (5pb/changement) -- rendement cumule brut=-93.23%, cout total=53.08%, net=-96.82% -- les frais mangent une part importante du rendement (&gt;50% du brut) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>**Regression multifeatures** — coefs (intercept=0.00029, momentum5j=-0.0326, var_vix=0.00027) -- R2 out-of-sample=0.0103 (modele bat la moyenne) _(observation : 2026-09-29)_</t>
+          <t>**Regression multifeatures** — coefs (intercept=0.00029, momentum5j=-0.0326, var_vix=0.00027) -- R2 out-of-sample=0.0103 (modele bat la moyenne) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1464,21 +1464,21 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>**Stacking** — poids appris (momentum=-0.082, baseline=0.090, biais=0.090) -- accuracy stacking=0.5459 vs momentum seul=0.5024, baseline seule=0.5459 sur 2255 points test -- stacking NE BAT PAS la baseline, meilleur=stacking / baseline (ex-aequo) _(observation : 2026-09-29)_</t>
+          <t>**Stacking** — poids appris (momentum=-0.082, baseline=0.090, biais=0.090) -- accuracy stacking=0.5461 vs momentum seul=0.5022, baseline seule=0.5461 sur 2256 points test -- stacking NE BAT PAS la baseline, meilleur=stacking / baseline (ex-aequo) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>**Decision stump** — seuil appris=-1.530 (sens=False) -- accuracy stump=0.5455 vs baseline=0.5473 sur 2264 points test -- stump NE BAT PAS la baseline _(observation : 2026-09-29)_</t>
+          <t>**Decision stump** — seuil appris=-1.530 (sens=False) -- accuracy stump=0.5455 vs baseline=0.5473 sur 2264 points test -- stump NE BAT PAS la baseline _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>**Importance permutation** — R2 base=0.0103 -- importance momentum5j=0.00088, importance variation_vix=0.01377 -- VIX plus important _(observation : 2026-09-29)_</t>
+          <t>**Importance permutation** — R2 base=0.0103 -- importance momentum5j=0.00242, importance variation_vix=0.00882 -- VIX plus important _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -2717,7 +2717,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3162,6 +3162,34 @@
       </c>
       <c r="H15" t="n">
         <v>0.5459000000000001</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>-0.08160000000000001</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.08989999999999999</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.08989999999999999</v>
+      </c>
+      <c r="E16" t="n">
+        <v>2256</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.5461</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.5022</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0.5461</v>
       </c>
     </row>
   </sheetData>
@@ -5189,7 +5217,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6014,6 +6042,62 @@
       </c>
       <c r="F29" t="n">
         <v>5068.51</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>GFC_2008</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>2007-10-09</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>2009-03-09</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>-56.78</v>
+      </c>
+      <c r="F30" t="n">
+        <v>3335.92</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>COVID_2020</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>2020-02-19</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>2020-03-23</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>-33.92</v>
+      </c>
+      <c r="F31" t="n">
+        <v>5099.43</v>
       </c>
     </row>
   </sheetData>
@@ -6737,7 +6821,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7037,6 +7121,25 @@
         <v>0.516</v>
       </c>
       <c r="E15" t="n">
+        <v>0.0003</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>23</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.5162</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.5159</v>
+      </c>
+      <c r="E16" t="n">
         <v>0.0003</v>
       </c>
     </row>
@@ -7389,7 +7492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7642,6 +7745,22 @@
       </c>
       <c r="D15" t="n">
         <v>0.00416</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>5</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.07565</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.00415</v>
       </c>
     </row>
   </sheetData>
@@ -7898,7 +8017,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8325,6 +8444,33 @@
         <v>-1.141</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>bas</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>32.6</v>
+      </c>
+      <c r="D16" t="n">
+        <v>-2.847</v>
+      </c>
+      <c r="E16" t="n">
+        <v>-1.141</v>
+      </c>
+      <c r="F16" t="n">
+        <v>-1.845</v>
+      </c>
+      <c r="G16" t="n">
+        <v>-1.141</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8336,7 +8482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8687,6 +8833,28 @@
         <v>-9.098000000000001</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>-1.447</v>
+      </c>
+      <c r="C16" t="n">
+        <v>-1.803</v>
+      </c>
+      <c r="D16" t="n">
+        <v>-2.084</v>
+      </c>
+      <c r="E16" t="n">
+        <v>-2.504</v>
+      </c>
+      <c r="F16" t="n">
+        <v>-9.098000000000001</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8698,7 +8866,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8951,6 +9119,22 @@
       </c>
       <c r="D15" t="n">
         <v>-0.052351</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>10</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.3728</v>
+      </c>
+      <c r="D16" t="n">
+        <v>-0.052375</v>
       </c>
     </row>
   </sheetData>
@@ -9015,14 +9199,14 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>53.74</v>
+        <v>53.11</v>
       </c>
       <c r="D2" t="n">
-        <v>85.90000000000001</v>
+        <v>84.5</v>
       </c>
       <c r="E2" t="n">
         <v>1260</v>
@@ -9041,14 +9225,14 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>24.37</v>
+        <v>23.71</v>
       </c>
       <c r="D3" t="n">
-        <v>84.90000000000001</v>
+        <v>82.3</v>
       </c>
       <c r="E3" t="n">
         <v>1260</v>
@@ -9067,14 +9251,14 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>106.6</v>
+        <v>106.16</v>
       </c>
       <c r="D4" t="n">
-        <v>57.7</v>
+        <v>56.7</v>
       </c>
       <c r="E4" t="n">
         <v>1260</v>
@@ -9093,14 +9277,14 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>22.07</v>
+        <v>22.28</v>
       </c>
       <c r="D5" t="n">
-        <v>47.5</v>
+        <v>49</v>
       </c>
       <c r="E5" t="n">
         <v>1260</v>
@@ -9114,7 +9298,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Actions US (VIX)</t>
+          <t>Vol de la vol (VVIX)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -9123,10 +9307,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>16.12</v>
+        <v>89.09</v>
       </c>
       <c r="D6" t="n">
-        <v>33.3</v>
+        <v>31.7</v>
       </c>
       <c r="E6" t="n">
         <v>1260</v>
@@ -9140,19 +9324,19 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Vol de la vol (VVIX)</t>
+          <t>Actions US (VIX)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>89.70999999999999</v>
+        <v>15.86</v>
       </c>
       <c r="D7" t="n">
-        <v>33.3</v>
+        <v>30.6</v>
       </c>
       <c r="E7" t="n">
         <v>1260</v>
@@ -9174,7 +9358,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9477,6 +9661,25 @@
         <v>0.112</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.1054</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.0888</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.1094</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.1122</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9488,7 +9691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9819,6 +10022,27 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>7517</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.4958</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.5373</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9830,7 +10054,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10158,6 +10382,27 @@
         <v>0.1666</v>
       </c>
       <c r="E15" t="n">
+        <v>0.0048</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2011-12-21</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>0.213</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.1666</v>
+      </c>
+      <c r="E16" t="n">
         <v>0.0048</v>
       </c>
     </row>
@@ -12132,7 +12377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12433,6 +12678,25 @@
       </c>
       <c r="E15" t="n">
         <v>-3.978</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>12.988</v>
+      </c>
+      <c r="C16" t="n">
+        <v>-1.288</v>
+      </c>
+      <c r="D16" t="n">
+        <v>-2.633</v>
+      </c>
+      <c r="E16" t="n">
+        <v>-3.979</v>
       </c>
     </row>
   </sheetData>
@@ -14269,7 +14533,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E141"/>
+  <dimension ref="A1:E151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17521,6 +17785,236 @@
         <v>0.7131</v>
       </c>
       <c r="E141" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>XLK</t>
+        </is>
+      </c>
+      <c r="C142" t="n">
+        <v>-2.4931</v>
+      </c>
+      <c r="D142" t="n">
+        <v>0.2821</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>XLF</t>
+        </is>
+      </c>
+      <c r="C143" t="n">
+        <v>-1.7429</v>
+      </c>
+      <c r="D143" t="n">
+        <v>0.657</v>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>XLE</t>
+        </is>
+      </c>
+      <c r="C144" t="n">
+        <v>-2.139</v>
+      </c>
+      <c r="D144" t="n">
+        <v>0.456</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>XLV</t>
+        </is>
+      </c>
+      <c r="C145" t="n">
+        <v>-2.39</v>
+      </c>
+      <c r="D145" t="n">
+        <v>0.3296</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>XLI</t>
+        </is>
+      </c>
+      <c r="C146" t="n">
+        <v>-1.2558</v>
+      </c>
+      <c r="D146" t="n">
+        <v>0.8427</v>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>XLY</t>
+        </is>
+      </c>
+      <c r="C147" t="n">
+        <v>0.09710000000000001</v>
+      </c>
+      <c r="D147" t="n">
+        <v>0.9879</v>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>XLP</t>
+        </is>
+      </c>
+      <c r="C148" t="n">
+        <v>-1.1067</v>
+      </c>
+      <c r="D148" t="n">
+        <v>0.8807</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>XLU</t>
+        </is>
+      </c>
+      <c r="C149" t="n">
+        <v>-0.5633</v>
+      </c>
+      <c r="D149" t="n">
+        <v>0.9595</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>XLB</t>
+        </is>
+      </c>
+      <c r="C150" t="n">
+        <v>-2.0839</v>
+      </c>
+      <c r="D150" t="n">
+        <v>0.4848</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>XLRE</t>
+        </is>
+      </c>
+      <c r="C151" t="n">
+        <v>-1.5015</v>
+      </c>
+      <c r="D151" t="n">
+        <v>0.7606000000000001</v>
+      </c>
+      <c r="E151" t="inlineStr">
         <is>
           <t>False</t>
         </is>
@@ -24648,7 +25142,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.1092</v>
+        <v>0.0985</v>
       </c>
       <c r="C15" t="n">
         <v>3</v>
@@ -24660,7 +25154,7 @@
         <v>0.2357</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.5052</v>
+        <v>-0.5373</v>
       </c>
     </row>
   </sheetData>
@@ -24744,7 +25238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -24949,6 +25443,19 @@
       </c>
       <c r="C15" t="n">
         <v>0.3607</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>10</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.2665</v>
       </c>
     </row>
   </sheetData>
@@ -24962,7 +25469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -25119,6 +25626,16 @@
       </c>
       <c r="B15" t="n">
         <v>-0.7592</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>-0.7574</v>
       </c>
     </row>
   </sheetData>
@@ -36930,7 +37447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -37279,6 +37796,28 @@
       </c>
       <c r="F15" t="n">
         <v>-96.8</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>7517</v>
+      </c>
+      <c r="C16" t="n">
+        <v>1513</v>
+      </c>
+      <c r="D16" t="n">
+        <v>53.08</v>
+      </c>
+      <c r="E16" t="n">
+        <v>-93.23</v>
+      </c>
+      <c r="F16" t="n">
+        <v>-96.81999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -37676,19 +38215,19 @@
         <v>2.2</v>
       </c>
       <c r="C15" t="n">
-        <v>413.81</v>
+        <v>413.47</v>
       </c>
       <c r="D15" t="n">
         <v>4</v>
       </c>
       <c r="E15" t="n">
-        <v>373.51</v>
+        <v>372.99</v>
       </c>
       <c r="F15" t="n">
         <v>5.3</v>
       </c>
       <c r="G15" t="n">
-        <v>323.82</v>
+        <v>323.97</v>
       </c>
     </row>
   </sheetData>
@@ -37702,7 +38241,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -38098,6 +38637,31 @@
         <v>-2.858</v>
       </c>
       <c r="G15" t="n">
+        <v>755</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>29.55</v>
+      </c>
+      <c r="C16" t="n">
+        <v>-1.845</v>
+      </c>
+      <c r="D16" t="n">
+        <v>-4.373</v>
+      </c>
+      <c r="E16" t="n">
+        <v>-1.515</v>
+      </c>
+      <c r="F16" t="n">
+        <v>-2.858</v>
+      </c>
+      <c r="G16" t="n">
         <v>755</v>
       </c>
     </row>
@@ -38472,7 +39036,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -38848,6 +39412,30 @@
         <v>0.5455</v>
       </c>
       <c r="F15" t="n">
+        <v>0.5473</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>-1.53</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>2264</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.5455</v>
+      </c>
+      <c r="F16" t="n">
         <v>0.5473</v>
       </c>
     </row>
@@ -39153,16 +39741,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>15.588</v>
+        <v>15.547</v>
       </c>
       <c r="C15" t="n">
-        <v>0.433</v>
+        <v>0.336</v>
       </c>
       <c r="D15" t="n">
-        <v>0.099</v>
+        <v>-0.023</v>
       </c>
       <c r="E15" t="n">
-        <v>0.71</v>
+        <v>0.68</v>
       </c>
     </row>
   </sheetData>
@@ -39394,7 +39982,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -39745,6 +40333,28 @@
         <v>6.86</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>7547</v>
+      </c>
+      <c r="C16" t="n">
+        <v>518</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.06864000000000001</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F16" t="n">
+        <v>6.86</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -39756,7 +40366,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -40036,6 +40646,24 @@
         </is>
       </c>
       <c r="D15" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1.172</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
         <v>22</v>
       </c>
     </row>
@@ -40342,7 +40970,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -40673,6 +41301,27 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.00608</v>
+      </c>
+      <c r="C16" t="n">
+        <v>-0.18</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -40684,7 +41333,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -40987,6 +41636,25 @@
         <v>28.29</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>10</v>
+      </c>
+      <c r="C16" t="n">
+        <v>-1.164</v>
+      </c>
+      <c r="D16" t="n">
+        <v>8.24</v>
+      </c>
+      <c r="E16" t="n">
+        <v>28.717</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -40998,7 +41666,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -41326,6 +41994,27 @@
       <c r="E15" t="inlineStr">
         <is>
           <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="C16" t="n">
+        <v>-133228</v>
+      </c>
+      <c r="D16" t="n">
+        <v>-10560</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>True</t>
         </is>
       </c>
     </row>
@@ -42065,7 +42754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -42413,6 +43102,28 @@
         <v>0.4988</v>
       </c>
       <c r="F15" t="n">
+        <v>0.5373</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>7517</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.4958</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.4989</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.4989</v>
+      </c>
+      <c r="F16" t="n">
         <v>0.5373</v>
       </c>
     </row>
@@ -45264,7 +45975,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -45565,6 +46276,25 @@
       </c>
       <c r="E15" t="n">
         <v>-13.4</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>3.08</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="D16" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="E16" t="n">
+        <v>-5.9</v>
       </c>
     </row>
   </sheetData>
@@ -51337,7 +52067,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>fred/BAMLC0A0CM.csv</t>
+          <t>fred/DFF.csv</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -51355,7 +52085,7 @@
         <v>42</v>
       </c>
       <c r="F187" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G187" t="inlineStr">
         <is>
@@ -51366,7 +52096,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>fred/BAMLC0A0CMEY.csv</t>
+          <t>fred/DFII10.csv</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -51384,7 +52114,7 @@
         <v>42</v>
       </c>
       <c r="F188" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G188" t="inlineStr">
         <is>
@@ -51395,7 +52125,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>fred/BAMLEMCBPIOAS.csv</t>
+          <t>fred/DFII5.csv</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -51413,7 +52143,7 @@
         <v>42</v>
       </c>
       <c r="F189" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G189" t="inlineStr">
         <is>
@@ -51424,7 +52154,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>fred/BAMLEMFSFCRPIOAS.csv</t>
+          <t>fred/DGS1.csv</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -51442,7 +52172,7 @@
         <v>42</v>
       </c>
       <c r="F190" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G190" t="inlineStr">
         <is>
@@ -51453,7 +52183,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>fred/BAMLEMHBHYCRPIOAS.csv</t>
+          <t>fred/DGS10.csv</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -51471,7 +52201,7 @@
         <v>42</v>
       </c>
       <c r="F191" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G191" t="inlineStr">
         <is>
@@ -51482,7 +52212,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>fred/BAMLEMPBPUBSICRPIOAS.csv</t>
+          <t>fred/DGS1MO.csv</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -51500,7 +52230,7 @@
         <v>42</v>
       </c>
       <c r="F192" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G192" t="inlineStr">
         <is>
@@ -51511,7 +52241,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>fred/BAMLH0A0HYM2.csv</t>
+          <t>fred/DGS2.csv</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -51529,7 +52259,7 @@
         <v>42</v>
       </c>
       <c r="F193" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G193" t="inlineStr">
         <is>
@@ -51540,7 +52270,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>fred/BAMLHE00EHYIEY.csv</t>
+          <t>fred/DGS30.csv</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -51558,7 +52288,7 @@
         <v>42</v>
       </c>
       <c r="F194" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G194" t="inlineStr">
         <is>
@@ -51569,7 +52299,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>fred/BAMLHE00EHYIOAS.csv</t>
+          <t>fred/DGS3MO.csv</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -51587,7 +52317,7 @@
         <v>42</v>
       </c>
       <c r="F195" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G195" t="inlineStr">
         <is>
@@ -51598,7 +52328,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>fred/DFF.csv</t>
+          <t>fred/DGS5.csv</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -51627,7 +52357,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>fred/DFII10.csv</t>
+          <t>fred/DGS6MO.csv</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -51656,7 +52386,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>fred/DFII5.csv</t>
+          <t>fred/IUDSOIA.csv</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -51685,7 +52415,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>fred/DGS1.csv</t>
+          <t>souverains/CANADA_10A.csv</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -51703,7 +52433,7 @@
         <v>42</v>
       </c>
       <c r="F199" t="n">
-        <v>3000</v>
+        <v>6437</v>
       </c>
       <c r="G199" t="inlineStr">
         <is>
@@ -51714,7 +52444,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>fred/DGS10.csv</t>
+          <t>souverains/CANADA_2A.csv</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -51732,7 +52462,7 @@
         <v>42</v>
       </c>
       <c r="F200" t="n">
-        <v>3000</v>
+        <v>6436</v>
       </c>
       <c r="G200" t="inlineStr">
         <is>
@@ -51743,7 +52473,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>fred/DGS1MO.csv</t>
+          <t>souverains/CANADA_5A.csv</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -51761,7 +52491,7 @@
         <v>42</v>
       </c>
       <c r="F201" t="n">
-        <v>3000</v>
+        <v>6436</v>
       </c>
       <c r="G201" t="inlineStr">
         <is>
@@ -51772,7 +52502,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>fred/DGS2.csv</t>
+          <t>souverains/CANADA_LONG.csv</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -51790,7 +52520,7 @@
         <v>42</v>
       </c>
       <c r="F202" t="n">
-        <v>3000</v>
+        <v>6436</v>
       </c>
       <c r="G202" t="inlineStr">
         <is>
@@ -51801,7 +52531,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>fred/DGS30.csv</t>
+          <t>souverains/UK_10A.csv</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -51819,7 +52549,7 @@
         <v>42</v>
       </c>
       <c r="F203" t="n">
-        <v>3000</v>
+        <v>9285</v>
       </c>
       <c r="G203" t="inlineStr">
         <is>
@@ -51830,7 +52560,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>fred/DGS3MO.csv</t>
+          <t>souverains/UK_20A.csv</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
@@ -51848,7 +52578,7 @@
         <v>42</v>
       </c>
       <c r="F204" t="n">
-        <v>3000</v>
+        <v>6756</v>
       </c>
       <c r="G204" t="inlineStr">
         <is>
@@ -51859,7 +52589,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>fred/DGS5.csv</t>
+          <t>souverains/UK_5A.csv</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -51877,7 +52607,7 @@
         <v>42</v>
       </c>
       <c r="F205" t="n">
-        <v>3000</v>
+        <v>8293</v>
       </c>
       <c r="G205" t="inlineStr">
         <is>
@@ -51888,7 +52618,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>fred/DGS6MO.csv</t>
+          <t>tresor_us/dette_quotidienne.csv</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -51906,7 +52636,7 @@
         <v>42</v>
       </c>
       <c r="F206" t="n">
-        <v>3000</v>
+        <v>2000</v>
       </c>
       <c r="G206" t="inlineStr">
         <is>
@@ -51917,7 +52647,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>fred/IUDSOIA.csv</t>
+          <t>tresor_us/solde_tresorerie.csv</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -51935,7 +52665,7 @@
         <v>42</v>
       </c>
       <c r="F207" t="n">
-        <v>3000</v>
+        <v>500</v>
       </c>
       <c r="G207" t="inlineStr">
         <is>
@@ -51946,16 +52676,16 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>souverains/CANADA_10A.csv</t>
+          <t>fred/BAMLC0A0CM.csv</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C208" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D208" t="n">
         <v>1</v>
@@ -51964,7 +52694,7 @@
         <v>42</v>
       </c>
       <c r="F208" t="n">
-        <v>6437</v>
+        <v>793</v>
       </c>
       <c r="G208" t="inlineStr">
         <is>
@@ -51975,16 +52705,16 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>souverains/CANADA_2A.csv</t>
+          <t>fred/BAMLC0A0CMEY.csv</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C209" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D209" t="n">
         <v>1</v>
@@ -51993,7 +52723,7 @@
         <v>42</v>
       </c>
       <c r="F209" t="n">
-        <v>6436</v>
+        <v>793</v>
       </c>
       <c r="G209" t="inlineStr">
         <is>
@@ -52004,16 +52734,16 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>souverains/CANADA_5A.csv</t>
+          <t>fred/BAMLEMCBPIOAS.csv</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C210" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D210" t="n">
         <v>1</v>
@@ -52022,7 +52752,7 @@
         <v>42</v>
       </c>
       <c r="F210" t="n">
-        <v>6436</v>
+        <v>793</v>
       </c>
       <c r="G210" t="inlineStr">
         <is>
@@ -52033,16 +52763,16 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>souverains/CANADA_LONG.csv</t>
+          <t>fred/BAMLEMFSFCRPIOAS.csv</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C211" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D211" t="n">
         <v>1</v>
@@ -52051,7 +52781,7 @@
         <v>42</v>
       </c>
       <c r="F211" t="n">
-        <v>6436</v>
+        <v>793</v>
       </c>
       <c r="G211" t="inlineStr">
         <is>
@@ -52062,16 +52792,16 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>souverains/UK_10A.csv</t>
+          <t>fred/BAMLEMHBHYCRPIOAS.csv</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C212" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D212" t="n">
         <v>1</v>
@@ -52080,7 +52810,7 @@
         <v>42</v>
       </c>
       <c r="F212" t="n">
-        <v>9285</v>
+        <v>793</v>
       </c>
       <c r="G212" t="inlineStr">
         <is>
@@ -52091,16 +52821,16 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>souverains/UK_20A.csv</t>
+          <t>fred/BAMLEMPBPUBSICRPIOAS.csv</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C213" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D213" t="n">
         <v>1</v>
@@ -52109,7 +52839,7 @@
         <v>42</v>
       </c>
       <c r="F213" t="n">
-        <v>6756</v>
+        <v>793</v>
       </c>
       <c r="G213" t="inlineStr">
         <is>
@@ -52120,16 +52850,16 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>souverains/UK_5A.csv</t>
+          <t>fred/BAMLH0A0HYM2.csv</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C214" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D214" t="n">
         <v>1</v>
@@ -52138,7 +52868,7 @@
         <v>42</v>
       </c>
       <c r="F214" t="n">
-        <v>8293</v>
+        <v>793</v>
       </c>
       <c r="G214" t="inlineStr">
         <is>
@@ -52149,16 +52879,16 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
+          <t>fred/BAMLHE00EHYIEY.csv</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C215" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D215" t="n">
         <v>1</v>
@@ -52167,7 +52897,7 @@
         <v>42</v>
       </c>
       <c r="F215" t="n">
-        <v>5640</v>
+        <v>793</v>
       </c>
       <c r="G215" t="inlineStr">
         <is>
@@ -52178,16 +52908,16 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>tresor_us/dette_quotidienne.csv</t>
+          <t>fred/BAMLHE00EHYIOAS.csv</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C216" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D216" t="n">
         <v>1</v>
@@ -52196,7 +52926,7 @@
         <v>42</v>
       </c>
       <c r="F216" t="n">
-        <v>2000</v>
+        <v>793</v>
       </c>
       <c r="G216" t="inlineStr">
         <is>
@@ -52207,16 +52937,16 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>tresor_us/solde_tresorerie.csv</t>
+          <t>fred/RRPONTSYD.csv</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C217" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D217" t="n">
         <v>1</v>
@@ -52225,7 +52955,7 @@
         <v>42</v>
       </c>
       <c r="F217" t="n">
-        <v>500</v>
+        <v>3000</v>
       </c>
       <c r="G217" t="inlineStr">
         <is>
@@ -52236,7 +52966,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>fred/RRPONTSYD.csv</t>
+          <t>fred/T10YIE.csv</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -52265,7 +52995,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>fred/T10YIE.csv</t>
+          <t>marches/indices/KOSPI.csv</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -52283,7 +53013,7 @@
         <v>42</v>
       </c>
       <c r="F219" t="n">
-        <v>3000</v>
+        <v>3680</v>
       </c>
       <c r="G219" t="inlineStr">
         <is>
@@ -52294,7 +53024,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>marches/volatilite/GVZ.csv</t>
+          <t>marches/indices/NIKKEI225.csv</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -52312,7 +53042,7 @@
         <v>42</v>
       </c>
       <c r="F220" t="n">
-        <v>3770</v>
+        <v>3666</v>
       </c>
       <c r="G220" t="inlineStr">
         <is>
@@ -52323,7 +53053,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>marches/volatilite/MOVE.csv</t>
+          <t>souverains/SUEDE_10A.csv</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -52341,7 +53071,7 @@
         <v>42</v>
       </c>
       <c r="F221" t="n">
-        <v>3689</v>
+        <v>9204</v>
       </c>
       <c r="G221" t="inlineStr">
         <is>
@@ -52352,7 +53082,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>marches/volatilite/OVX.csv</t>
+          <t>souverains/SUEDE_2A.csv</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -52370,7 +53100,7 @@
         <v>42</v>
       </c>
       <c r="F222" t="n">
-        <v>3770</v>
+        <v>9204</v>
       </c>
       <c r="G222" t="inlineStr">
         <is>
@@ -52381,7 +53111,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>marches/volatilite/VVIX.csv</t>
+          <t>souverains/SUEDE_5A.csv</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -52399,7 +53129,7 @@
         <v>42</v>
       </c>
       <c r="F223" t="n">
-        <v>3762</v>
+        <v>9206</v>
       </c>
       <c r="G223" t="inlineStr">
         <is>
@@ -52410,7 +53140,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>marches/volatilite/VXN.csv</t>
+          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -52428,7 +53158,7 @@
         <v>42</v>
       </c>
       <c r="F224" t="n">
-        <v>3770</v>
+        <v>5641</v>
       </c>
       <c r="G224" t="inlineStr">
         <is>
@@ -52439,7 +53169,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_10A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
@@ -52457,7 +53187,7 @@
         <v>42</v>
       </c>
       <c r="F225" t="n">
-        <v>9204</v>
+        <v>5641</v>
       </c>
       <c r="G225" t="inlineStr">
         <is>
@@ -52468,7 +53198,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_2A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -52486,7 +53216,7 @@
         <v>42</v>
       </c>
       <c r="F226" t="n">
-        <v>9204</v>
+        <v>5641</v>
       </c>
       <c r="G226" t="inlineStr">
         <is>
@@ -52497,7 +53227,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_5A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -52515,7 +53245,7 @@
         <v>42</v>
       </c>
       <c r="F227" t="n">
-        <v>9206</v>
+        <v>5641</v>
       </c>
       <c r="G227" t="inlineStr">
         <is>
@@ -52526,7 +53256,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -52555,7 +53285,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -52584,7 +53314,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -52613,7 +53343,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -52642,7 +53372,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
+          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -52671,16 +53401,16 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
+          <t>fred/ECBDFR.csv</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C233" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D233" t="n">
         <v>1</v>
@@ -52689,7 +53419,7 @@
         <v>42</v>
       </c>
       <c r="F233" t="n">
-        <v>5641</v>
+        <v>3000</v>
       </c>
       <c r="G233" t="inlineStr">
         <is>
@@ -52700,16 +53430,16 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
+          <t>marches/fx/AUDJPY.csv</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C234" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D234" t="n">
         <v>1</v>
@@ -52718,7 +53448,7 @@
         <v>42</v>
       </c>
       <c r="F234" t="n">
-        <v>5641</v>
+        <v>3908</v>
       </c>
       <c r="G234" t="inlineStr">
         <is>
@@ -52729,16 +53459,16 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
+          <t>marches/fx/AUDUSD.csv</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C235" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D235" t="n">
         <v>1</v>
@@ -52747,7 +53477,7 @@
         <v>42</v>
       </c>
       <c r="F235" t="n">
-        <v>5641</v>
+        <v>3904</v>
       </c>
       <c r="G235" t="inlineStr">
         <is>
@@ -52758,16 +53488,16 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>yfinance/SP500.csv</t>
+          <t>marches/fx/DXY.csv</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C236" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D236" t="n">
         <v>1</v>
@@ -52776,7 +53506,7 @@
         <v>42</v>
       </c>
       <c r="F236" t="n">
-        <v>7547</v>
+        <v>3772</v>
       </c>
       <c r="G236" t="inlineStr">
         <is>
@@ -52787,16 +53517,16 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>yfinance/XLB.csv</t>
+          <t>marches/fx/EURCHF.csv</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C237" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D237" t="n">
         <v>1</v>
@@ -52805,7 +53535,7 @@
         <v>42</v>
       </c>
       <c r="F237" t="n">
-        <v>501</v>
+        <v>3905</v>
       </c>
       <c r="G237" t="inlineStr">
         <is>
@@ -52816,16 +53546,16 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>yfinance/XLE.csv</t>
+          <t>marches/fx/EURGBP.csv</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C238" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D238" t="n">
         <v>1</v>
@@ -52834,7 +53564,7 @@
         <v>42</v>
       </c>
       <c r="F238" t="n">
-        <v>501</v>
+        <v>3907</v>
       </c>
       <c r="G238" t="inlineStr">
         <is>
@@ -52845,16 +53575,16 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>yfinance/XLF.csv</t>
+          <t>marches/fx/EURJPY.csv</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C239" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D239" t="n">
         <v>1</v>
@@ -52863,7 +53593,7 @@
         <v>42</v>
       </c>
       <c r="F239" t="n">
-        <v>501</v>
+        <v>3907</v>
       </c>
       <c r="G239" t="inlineStr">
         <is>
@@ -52874,16 +53604,16 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>yfinance/XLI.csv</t>
+          <t>marches/fx/EURUSD.csv</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C240" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D240" t="n">
         <v>1</v>
@@ -52892,7 +53622,7 @@
         <v>42</v>
       </c>
       <c r="F240" t="n">
-        <v>501</v>
+        <v>3904</v>
       </c>
       <c r="G240" t="inlineStr">
         <is>
@@ -52903,16 +53633,16 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>yfinance/XLK.csv</t>
+          <t>marches/fx/GBPUSD.csv</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C241" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D241" t="n">
         <v>1</v>
@@ -52921,7 +53651,7 @@
         <v>42</v>
       </c>
       <c r="F241" t="n">
-        <v>501</v>
+        <v>3905</v>
       </c>
       <c r="G241" t="inlineStr">
         <is>
@@ -52932,16 +53662,16 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>yfinance/XLP.csv</t>
+          <t>marches/fx/NZDUSD.csv</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C242" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D242" t="n">
         <v>1</v>
@@ -52950,7 +53680,7 @@
         <v>42</v>
       </c>
       <c r="F242" t="n">
-        <v>501</v>
+        <v>3905</v>
       </c>
       <c r="G242" t="inlineStr">
         <is>
@@ -52961,16 +53691,16 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>yfinance/XLRE.csv</t>
+          <t>marches/fx/USDCAD.csv</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C243" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D243" t="n">
         <v>1</v>
@@ -52979,7 +53709,7 @@
         <v>42</v>
       </c>
       <c r="F243" t="n">
-        <v>501</v>
+        <v>3904</v>
       </c>
       <c r="G243" t="inlineStr">
         <is>
@@ -52990,16 +53720,16 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>yfinance/XLU.csv</t>
+          <t>marches/fx/USDCHF.csv</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C244" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D244" t="n">
         <v>1</v>
@@ -53008,7 +53738,7 @@
         <v>42</v>
       </c>
       <c r="F244" t="n">
-        <v>501</v>
+        <v>3902</v>
       </c>
       <c r="G244" t="inlineStr">
         <is>
@@ -53019,16 +53749,16 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>yfinance/XLV.csv</t>
+          <t>marches/fx/USDCNY.csv</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C245" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D245" t="n">
         <v>1</v>
@@ -53037,7 +53767,7 @@
         <v>42</v>
       </c>
       <c r="F245" t="n">
-        <v>501</v>
+        <v>3904</v>
       </c>
       <c r="G245" t="inlineStr">
         <is>
@@ -53048,16 +53778,16 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>yfinance/XLY.csv</t>
+          <t>marches/fx/USDJPY.csv</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C246" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D246" t="n">
         <v>1</v>
@@ -53066,7 +53796,7 @@
         <v>42</v>
       </c>
       <c r="F246" t="n">
-        <v>501</v>
+        <v>3905</v>
       </c>
       <c r="G246" t="inlineStr">
         <is>
@@ -53077,7 +53807,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>fred/ECBDFR.csv</t>
+          <t>marches/fx/USDKRW.csv</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
@@ -53095,7 +53825,7 @@
         <v>42</v>
       </c>
       <c r="F247" t="n">
-        <v>3000</v>
+        <v>3904</v>
       </c>
       <c r="G247" t="inlineStr">
         <is>
@@ -53106,7 +53836,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>marches/fx/AUDJPY.csv</t>
+          <t>marches/fx/USDNOK.csv</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
@@ -53124,7 +53854,7 @@
         <v>42</v>
       </c>
       <c r="F248" t="n">
-        <v>3908</v>
+        <v>3905</v>
       </c>
       <c r="G248" t="inlineStr">
         <is>
@@ -53135,7 +53865,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>marches/fx/AUDUSD.csv</t>
+          <t>marches/fx/USDSEK.csv</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
@@ -53153,7 +53883,7 @@
         <v>42</v>
       </c>
       <c r="F249" t="n">
-        <v>3904</v>
+        <v>3905</v>
       </c>
       <c r="G249" t="inlineStr">
         <is>
@@ -53164,7 +53894,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>marches/fx/DXY.csv</t>
+          <t>marches/indices/DAX.csv</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
@@ -53182,7 +53912,7 @@
         <v>42</v>
       </c>
       <c r="F250" t="n">
-        <v>3772</v>
+        <v>3802</v>
       </c>
       <c r="G250" t="inlineStr">
         <is>
@@ -53193,7 +53923,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>marches/fx/EURCHF.csv</t>
+          <t>marches/indices/EUROSTOXX50.csv</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
@@ -53211,7 +53941,7 @@
         <v>42</v>
       </c>
       <c r="F251" t="n">
-        <v>3905</v>
+        <v>3759</v>
       </c>
       <c r="G251" t="inlineStr">
         <is>
@@ -53222,7 +53952,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>marches/fx/EURGBP.csv</t>
+          <t>marches/indices/FTSE100.csv</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -53240,7 +53970,7 @@
         <v>42</v>
       </c>
       <c r="F252" t="n">
-        <v>3907</v>
+        <v>3788</v>
       </c>
       <c r="G252" t="inlineStr">
         <is>
@@ -53251,7 +53981,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>marches/fx/EURJPY.csv</t>
+          <t>marches/indices/HANGSENG.csv</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -53269,7 +53999,7 @@
         <v>42</v>
       </c>
       <c r="F253" t="n">
-        <v>3907</v>
+        <v>3690</v>
       </c>
       <c r="G253" t="inlineStr">
         <is>
@@ -53280,7 +54010,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>marches/fx/EURUSD.csv</t>
+          <t>marches/matieres/BRENT.csv</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
@@ -53298,7 +54028,7 @@
         <v>42</v>
       </c>
       <c r="F254" t="n">
-        <v>3904</v>
+        <v>3751</v>
       </c>
       <c r="G254" t="inlineStr">
         <is>
@@ -53309,7 +54039,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>marches/fx/GBPUSD.csv</t>
+          <t>marches/matieres/CUIVRE.csv</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
@@ -53327,7 +54057,7 @@
         <v>42</v>
       </c>
       <c r="F255" t="n">
-        <v>3905</v>
+        <v>3771</v>
       </c>
       <c r="G255" t="inlineStr">
         <is>
@@ -53338,7 +54068,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>marches/fx/NZDUSD.csv</t>
+          <t>marches/matieres/GAZ_HENRY_HUB.csv</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
@@ -53356,7 +54086,7 @@
         <v>42</v>
       </c>
       <c r="F256" t="n">
-        <v>3905</v>
+        <v>3772</v>
       </c>
       <c r="G256" t="inlineStr">
         <is>
@@ -53367,7 +54097,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>marches/fx/USDCAD.csv</t>
+          <t>marches/matieres/OR.csv</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
@@ -53385,7 +54115,7 @@
         <v>42</v>
       </c>
       <c r="F257" t="n">
-        <v>3904</v>
+        <v>3771</v>
       </c>
       <c r="G257" t="inlineStr">
         <is>
@@ -53396,7 +54126,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>marches/fx/USDCHF.csv</t>
+          <t>marches/matieres/WTI.csv</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
@@ -53414,7 +54144,7 @@
         <v>42</v>
       </c>
       <c r="F258" t="n">
-        <v>3902</v>
+        <v>3771</v>
       </c>
       <c r="G258" t="inlineStr">
         <is>
@@ -53425,7 +54155,7 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>marches/fx/USDCNY.csv</t>
+          <t>marches/taux_futures/FED_FUNDS_FRONT.csv</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
@@ -53443,7 +54173,7 @@
         <v>42</v>
       </c>
       <c r="F259" t="n">
-        <v>3904</v>
+        <v>3772</v>
       </c>
       <c r="G259" t="inlineStr">
         <is>
@@ -53454,7 +54184,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>marches/fx/USDJPY.csv</t>
+          <t>marches/volatilite/GVZ.csv</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
@@ -53472,7 +54202,7 @@
         <v>42</v>
       </c>
       <c r="F260" t="n">
-        <v>3905</v>
+        <v>3771</v>
       </c>
       <c r="G260" t="inlineStr">
         <is>
@@ -53483,7 +54213,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>marches/fx/USDKRW.csv</t>
+          <t>marches/volatilite/MOVE.csv</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
@@ -53501,7 +54231,7 @@
         <v>42</v>
       </c>
       <c r="F261" t="n">
-        <v>3904</v>
+        <v>3690</v>
       </c>
       <c r="G261" t="inlineStr">
         <is>
@@ -53512,7 +54242,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>marches/fx/USDNOK.csv</t>
+          <t>marches/volatilite/OVX.csv</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
@@ -53530,7 +54260,7 @@
         <v>42</v>
       </c>
       <c r="F262" t="n">
-        <v>3905</v>
+        <v>3771</v>
       </c>
       <c r="G262" t="inlineStr">
         <is>
@@ -53541,7 +54271,7 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>marches/fx/USDSEK.csv</t>
+          <t>marches/volatilite/VVIX.csv</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
@@ -53559,7 +54289,7 @@
         <v>42</v>
       </c>
       <c r="F263" t="n">
-        <v>3905</v>
+        <v>3763</v>
       </c>
       <c r="G263" t="inlineStr">
         <is>
@@ -53570,7 +54300,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>marches/indices/DAX.csv</t>
+          <t>marches/volatilite/VXN.csv</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
@@ -53588,7 +54318,7 @@
         <v>42</v>
       </c>
       <c r="F264" t="n">
-        <v>3802</v>
+        <v>3771</v>
       </c>
       <c r="G264" t="inlineStr">
         <is>
@@ -53599,7 +54329,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>marches/indices/EUROSTOXX50.csv</t>
+          <t>yfinance/SP500.csv</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
@@ -53617,7 +54347,7 @@
         <v>42</v>
       </c>
       <c r="F265" t="n">
-        <v>3759</v>
+        <v>7548</v>
       </c>
       <c r="G265" t="inlineStr">
         <is>
@@ -53628,7 +54358,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>marches/indices/FTSE100.csv</t>
+          <t>yfinance/VIX.csv</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
@@ -53646,7 +54376,7 @@
         <v>42</v>
       </c>
       <c r="F266" t="n">
-        <v>3788</v>
+        <v>7550</v>
       </c>
       <c r="G266" t="inlineStr">
         <is>
@@ -53657,7 +54387,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>marches/indices/HANGSENG.csv</t>
+          <t>yfinance/XLB.csv</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
@@ -53675,7 +54405,7 @@
         <v>42</v>
       </c>
       <c r="F267" t="n">
-        <v>3690</v>
+        <v>502</v>
       </c>
       <c r="G267" t="inlineStr">
         <is>
@@ -53686,7 +54416,7 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>marches/indices/KOSPI.csv</t>
+          <t>yfinance/XLE.csv</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
@@ -53704,7 +54434,7 @@
         <v>42</v>
       </c>
       <c r="F268" t="n">
-        <v>3681</v>
+        <v>502</v>
       </c>
       <c r="G268" t="inlineStr">
         <is>
@@ -53715,7 +54445,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>marches/indices/NIKKEI225.csv</t>
+          <t>yfinance/XLF.csv</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
@@ -53733,7 +54463,7 @@
         <v>42</v>
       </c>
       <c r="F269" t="n">
-        <v>3667</v>
+        <v>502</v>
       </c>
       <c r="G269" t="inlineStr">
         <is>
@@ -53744,7 +54474,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>marches/matieres/BRENT.csv</t>
+          <t>yfinance/XLI.csv</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
@@ -53762,7 +54492,7 @@
         <v>42</v>
       </c>
       <c r="F270" t="n">
-        <v>3751</v>
+        <v>502</v>
       </c>
       <c r="G270" t="inlineStr">
         <is>
@@ -53773,7 +54503,7 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>marches/matieres/CUIVRE.csv</t>
+          <t>yfinance/XLK.csv</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
@@ -53791,7 +54521,7 @@
         <v>42</v>
       </c>
       <c r="F271" t="n">
-        <v>3771</v>
+        <v>502</v>
       </c>
       <c r="G271" t="inlineStr">
         <is>
@@ -53802,7 +54532,7 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>marches/matieres/GAZ_HENRY_HUB.csv</t>
+          <t>yfinance/XLP.csv</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
@@ -53820,7 +54550,7 @@
         <v>42</v>
       </c>
       <c r="F272" t="n">
-        <v>3772</v>
+        <v>502</v>
       </c>
       <c r="G272" t="inlineStr">
         <is>
@@ -53831,7 +54561,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>marches/matieres/OR.csv</t>
+          <t>yfinance/XLRE.csv</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
@@ -53849,7 +54579,7 @@
         <v>42</v>
       </c>
       <c r="F273" t="n">
-        <v>3771</v>
+        <v>502</v>
       </c>
       <c r="G273" t="inlineStr">
         <is>
@@ -53860,7 +54590,7 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>marches/matieres/WTI.csv</t>
+          <t>yfinance/XLU.csv</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
@@ -53878,7 +54608,7 @@
         <v>42</v>
       </c>
       <c r="F274" t="n">
-        <v>3771</v>
+        <v>502</v>
       </c>
       <c r="G274" t="inlineStr">
         <is>
@@ -53889,7 +54619,7 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>marches/taux_futures/FED_FUNDS_FRONT.csv</t>
+          <t>yfinance/XLV.csv</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
@@ -53907,7 +54637,7 @@
         <v>42</v>
       </c>
       <c r="F275" t="n">
-        <v>3772</v>
+        <v>502</v>
       </c>
       <c r="G275" t="inlineStr">
         <is>
@@ -53918,7 +54648,7 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>yfinance/VIX.csv</t>
+          <t>yfinance/XLY.csv</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
@@ -53936,7 +54666,7 @@
         <v>42</v>
       </c>
       <c r="F276" t="n">
-        <v>7550</v>
+        <v>502</v>
       </c>
       <c r="G276" t="inlineStr">
         <is>
@@ -54349,7 +55079,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -54649,6 +55379,25 @@
         <v>0.8685</v>
       </c>
       <c r="E15" t="n">
+        <v>0.9826</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.1171</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.1141</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.8685</v>
+      </c>
+      <c r="E16" t="n">
         <v>0.9826</v>
       </c>
     </row>
@@ -54929,7 +55678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -55207,6 +55956,24 @@
         <v>0.9996</v>
       </c>
       <c r="D15" t="inlineStr">
+        <is>
+          <t>persistant (tendanciel)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.5507</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.9996</v>
+      </c>
+      <c r="D16" t="inlineStr">
         <is>
           <t>persistant (tendanciel)</t>
         </is>
@@ -55223,7 +55990,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -55476,6 +56243,22 @@
       </c>
       <c r="D15" t="n">
         <v>0.01377</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.01027</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.00242</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.00882</v>
       </c>
     </row>
   </sheetData>
@@ -55534,17 +56317,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>6838.04</v>
+        <v>6870.81</v>
       </c>
       <c r="D2" t="n">
-        <v>-17.65</v>
+        <v>-18.94</v>
       </c>
       <c r="E2" t="n">
-        <v>99.67</v>
+        <v>100.24</v>
       </c>
     </row>
     <row r="3">
@@ -55555,17 +56338,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>66753.72</v>
+        <v>65481.27</v>
       </c>
       <c r="D3" t="n">
-        <v>-5.28</v>
+        <v>-6.54</v>
       </c>
       <c r="E3" t="n">
-        <v>48.56</v>
+        <v>45.37</v>
       </c>
     </row>
     <row r="4">
@@ -55576,23 +56359,23 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>7670.84</v>
+        <v>7717.64</v>
       </c>
       <c r="D4" t="n">
-        <v>2.29</v>
+        <v>3.13</v>
       </c>
       <c r="E4" t="n">
-        <v>15.16</v>
+        <v>15.39</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Zone euro (Euro Stoxx 50)</t>
+          <t>Royaume-Uni (FTSE 100)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -55601,19 +56384,19 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>6294.56</v>
+        <v>10609.71</v>
       </c>
       <c r="D5" t="n">
-        <v>0.19</v>
+        <v>1.25</v>
       </c>
       <c r="E5" t="n">
-        <v>13.83</v>
+        <v>13.47</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Royaume-Uni (FTSE 100)</t>
+          <t>Zone euro (Euro Stoxx 50)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -55622,13 +56405,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>10637.22</v>
+        <v>6269.95</v>
       </c>
       <c r="D6" t="n">
-        <v>1.52</v>
+        <v>-0.2</v>
       </c>
       <c r="E6" t="n">
-        <v>13.76</v>
+        <v>13.38</v>
       </c>
     </row>
     <row r="7">
@@ -55643,13 +56426,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>25295.18</v>
+        <v>25200.04</v>
       </c>
       <c r="D7" t="n">
-        <v>1.02</v>
+        <v>0.64</v>
       </c>
       <c r="E7" t="n">
-        <v>5.92</v>
+        <v>5.52</v>
       </c>
     </row>
     <row r="8">
@@ -56384,16 +57167,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>16.120001</v>
+        <v>15.86</v>
       </c>
       <c r="C15" t="n">
-        <v>16.105</v>
+        <v>15.884</v>
       </c>
       <c r="D15" t="n">
         <v>0.624</v>
       </c>
       <c r="E15" t="n">
-        <v>0.20515</v>
+        <v>0.20516</v>
       </c>
     </row>
   </sheetData>
@@ -57093,7 +57876,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -57571,6 +58354,37 @@
         <v>0.04</v>
       </c>
       <c r="G15" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>10</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>XLF;XLRE;XLU</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>-1.005</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>XLY;XLE;XLK</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>0.101</v>
+      </c>
+      <c r="G16" t="inlineStr">
         <is>
           <t>False</t>
         </is>
@@ -57957,25 +58771,25 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.001569</v>
+        <v>0.001576</v>
       </c>
       <c r="C13" t="n">
-        <v>4.62</v>
+        <v>5.08</v>
       </c>
       <c r="D13" t="n">
-        <v>97.63</v>
+        <v>98.89</v>
       </c>
       <c r="E13" t="n">
-        <v>36.41</v>
+        <v>38.17</v>
       </c>
       <c r="F13" t="n">
-        <v>45.67</v>
+        <v>47.55</v>
       </c>
       <c r="G13" t="n">
-        <v>-6.21</v>
+        <v>-6.4</v>
       </c>
       <c r="H13" t="n">
-        <v>7.22</v>
+        <v>7.33</v>
       </c>
     </row>
   </sheetData>
@@ -58113,7 +58927,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -58416,6 +59230,25 @@
         <v>0.27</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>3.08</v>
+      </c>
+      <c r="C16" t="n">
+        <v>2.74</v>
+      </c>
+      <c r="D16" t="n">
+        <v>-0.14</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.34</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -58427,7 +59260,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -58832,6 +59665,32 @@
       </c>
       <c r="F15" t="n">
         <v>17.87</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>XLE;XLV;XLK</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>9.901</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>XLY;XLI;XLU</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>-8.970000000000001</v>
+      </c>
+      <c r="F16" t="n">
+        <v>18.871</v>
       </c>
     </row>
   </sheetData>
@@ -61442,7 +62301,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -61791,6 +62650,28 @@
       </c>
       <c r="F15" t="n">
         <v>15.771</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="C16" t="n">
+        <v>3.132</v>
+      </c>
+      <c r="D16" t="n">
+        <v>17.373</v>
+      </c>
+      <c r="E16" t="n">
+        <v>15.387</v>
+      </c>
+      <c r="F16" t="n">
+        <v>14.916</v>
       </c>
     </row>
   </sheetData>
@@ -61910,7 +62791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -62259,6 +63140,28 @@
       </c>
       <c r="F15" t="n">
         <v>-0.011</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>3.08</v>
+      </c>
+      <c r="C16" t="n">
+        <v>3.031</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.018062</v>
+      </c>
+      <c r="E16" t="n">
+        <v>38.4</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.049</v>
       </c>
     </row>
   </sheetData>
@@ -62608,10 +63511,10 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>16.120001</v>
+        <v>15.86</v>
       </c>
       <c r="C15" t="n">
-        <v>20.2</v>
+        <v>20.199</v>
       </c>
       <c r="D15" t="n">
         <v>0.02404</v>
@@ -62620,7 +63523,7 @@
         <v>28.8</v>
       </c>
       <c r="F15" t="n">
-        <v>-4.08</v>
+        <v>-4.339</v>
       </c>
     </row>
   </sheetData>
@@ -67738,7 +68641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -67895,6 +68798,16 @@
       </c>
       <c r="B15" t="n">
         <v>-0.004863</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>-0.004859</v>
       </c>
     </row>
   </sheetData>
@@ -68305,7 +69218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -68775,6 +69688,36 @@
         <v>3.834e-07</v>
       </c>
       <c r="H15" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>5282</v>
+      </c>
+      <c r="C16" t="n">
+        <v>2265</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.00011626</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.20964</v>
+      </c>
+      <c r="F16" t="n">
+        <v>2.983e-07</v>
+      </c>
+      <c r="G16" t="n">
+        <v>3.833e-07</v>
+      </c>
+      <c r="H16" t="inlineStr">
         <is>
           <t>True</t>
         </is>
@@ -69040,10 +69983,10 @@
         <v>0.00877</v>
       </c>
       <c r="C15" t="n">
-        <v>0.06759999999999999</v>
+        <v>0.06763</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.03818</v>
+        <v>-0.0382</v>
       </c>
     </row>
   </sheetData>
@@ -71997,7 +72940,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -72250,6 +73193,22 @@
       </c>
       <c r="D15" t="n">
         <v>0.421</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>-1.107</v>
+      </c>
+      <c r="C16" t="n">
+        <v>2.403</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.422</v>
       </c>
     </row>
   </sheetData>
@@ -72263,7 +73222,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -72516,6 +73475,22 @@
       </c>
       <c r="D15" t="n">
         <v>1.5574</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1.1045</v>
+      </c>
+      <c r="C16" t="n">
+        <v>1.0908</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1.5795</v>
       </c>
     </row>
   </sheetData>
@@ -75443,7 +76418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -75839,6 +76814,31 @@
         <v>2263</v>
       </c>
       <c r="G15" t="n">
+        <v>0.01027</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.000291</v>
+      </c>
+      <c r="C16" t="n">
+        <v>-0.032603</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.000269</v>
+      </c>
+      <c r="E16" t="n">
+        <v>5279</v>
+      </c>
+      <c r="F16" t="n">
+        <v>2263</v>
+      </c>
+      <c r="G16" t="n">
         <v>0.01027</v>
       </c>
     </row>
@@ -76240,7 +77240,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E141"/>
+  <dimension ref="A1:E151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -79495,6 +80495,236 @@
       </c>
       <c r="E141" t="n">
         <v>-12.417</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B142" t="n">
+        <v>1</v>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>XLE</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Energie</t>
+        </is>
+      </c>
+      <c r="E142" t="n">
+        <v>17.146</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B143" t="n">
+        <v>2</v>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>XLV</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Sante</t>
+        </is>
+      </c>
+      <c r="E143" t="n">
+        <v>6.589</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B144" t="n">
+        <v>3</v>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>XLK</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Technologie</t>
+        </is>
+      </c>
+      <c r="E144" t="n">
+        <v>5.969</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B145" t="n">
+        <v>4</v>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>XLF</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="E145" t="n">
+        <v>-1.762</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B146" t="n">
+        <v>5</v>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>XLP</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Consommation de base</t>
+        </is>
+      </c>
+      <c r="E146" t="n">
+        <v>-2.245</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B147" t="n">
+        <v>6</v>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>XLB</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Materiaux</t>
+        </is>
+      </c>
+      <c r="E147" t="n">
+        <v>-3.606</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B148" t="n">
+        <v>7</v>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>XLRE</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Immobilier</t>
+        </is>
+      </c>
+      <c r="E148" t="n">
+        <v>-6.824</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B149" t="n">
+        <v>8</v>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>XLY</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Consommation discretionnaire</t>
+        </is>
+      </c>
+      <c r="E149" t="n">
+        <v>-7.316</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B150" t="n">
+        <v>9</v>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>XLI</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Industrie</t>
+        </is>
+      </c>
+      <c r="E150" t="n">
+        <v>-8.022</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B151" t="n">
+        <v>10</v>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>XLU</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Services collectifs</t>
+        </is>
+      </c>
+      <c r="E151" t="n">
+        <v>-11.57</v>
       </c>
     </row>
   </sheetData>
@@ -79900,7 +81130,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -80375,6 +81605,36 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>3842</v>
+      </c>
+      <c r="C16" t="n">
+        <v>3705</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.01806</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.04655</v>
+      </c>
+      <c r="F16" t="n">
+        <v>-1.025</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.3056</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -80386,7 +81646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E57"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -81706,6 +82966,98 @@
         <v>0.008200000000000001</v>
       </c>
       <c r="E57" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>momentum_5j</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>-0.0295</v>
+      </c>
+      <c r="D58" t="n">
+        <v>0.0104</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>momentum_20j</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>-0.0112</v>
+      </c>
+      <c r="D59" t="n">
+        <v>0.3298</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>niveau_vix</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>-0.0036</v>
+      </c>
+      <c r="D60" t="n">
+        <v>0.7522</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>variation_vix</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>0.0304</v>
+      </c>
+      <c r="D61" t="n">
+        <v>0.008200000000000001</v>
+      </c>
+      <c r="E61" t="inlineStr">
         <is>
           <t>True</t>
         </is>
@@ -81805,7 +83157,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -82108,6 +83460,25 @@
         <v>1000</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.1299</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.1176</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.1415</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1000</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -82119,7 +83490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -82324,6 +83695,19 @@
       </c>
       <c r="C15" t="n">
         <v>1.0224</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>-0.1937</v>
+      </c>
+      <c r="C16" t="n">
+        <v>1.012</v>
       </c>
     </row>
   </sheetData>
@@ -82412,13 +83796,13 @@
         <v>89.40000000000001</v>
       </c>
       <c r="D3" t="n">
-        <v>4.13</v>
+        <v>4.14</v>
       </c>
       <c r="E3" t="n">
         <v>3.25</v>
       </c>
       <c r="F3" t="n">
-        <v>0.88</v>
+        <v>0.89</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-30T18:14Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-30 15:21 UTC</t>
+          <t>Genere le 2026-09-30 18:14 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-30 15:21 UTC</t>
+          <t>Rapport global — 2026-09-30 18:14 UTC</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>**Bilans banques centrales** — 9 bilans suivis sur 12 mois : de -19.2% (RBA -- titres locaux) a +8.5% (Fed -- titres du Tresor) -- regimes OPPOSES -- 5 bilan(s) en reduction pendant que 4 s'etendent, la liquidite mondiale ne va pas dans un sens unique _(observation : 2026-09-23)_</t>
+          <t>**Bilans banques centrales** — 9 bilans suivis sur 12 mois : de -19.2% (RBA -- titres locaux) a +8.5% (Fed -- titres du Tresor) -- regimes OPPOSES -- 5 bilan(s) en reduction pendant que 4 s'etendent, la liquidite mondiale ne va pas dans un sens unique _(observation : 2026-09-25)_</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>**Matieres premieres macro** — le ratio cuivre/or monte -- la croissance domine la peur (+5.1% sur 3 mois). Brent 98.9$ (+38.2% sur 3 mois, +47.6% sur 12 mois), gaz -6.4% sur 3 mois, ecart Brent-WTI +7.3$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-30)_</t>
+          <t>**Matieres premieres macro** — le ratio cuivre/or monte -- la croissance domine la peur (+5.5% sur 3 mois). Brent 98.3$ (+37.3% sur 3 mois, +46.7% sur 12 mois), gaz -6.5% sur 3 mois, ecart Brent-WTI +7.6$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -862,7 +862,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>**Conditions financieres** — indice conditions financieres=+0.098 (3 composantes: {'taux_directeur': 0.5971439233898245, 'courbe_inversee': 0.23568763984021313, 'vix': -0.5373391098837522}) -- conditions proches de la normale _(observation : 2026-09-28)_</t>
+          <t>**Conditions financieres** — indice conditions financieres=+0.097 (3 composantes: {'taux_directeur': 0.5971439233898245, 'courbe_inversee': 0.23568763984021313, 'vix': -0.5410491021615241}) -- conditions proches de la normale _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -960,7 +960,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>**Indices mondiaux** — 7 indices (devise locale) : Coree (KOSPI) +100.2% en tete sur 12 mois, Hong Kong (Hang Seng) -8.3% en queue -- ecart tres large entre blocs sur 12 mois (109pt) -- les cycles economiques ou les flux divergent nettement. ROTATION en cours : Coree (KOSPI) mene sur 12 mois mais Hong Kong (Hang Seng) a repris la tete sur 3 mois _(observation : 2026-09-30)_</t>
+          <t>**Indices mondiaux** — 7 indices (devise locale) : Coree (KOSPI) +100.2% en tete sur 12 mois, Hong Kong (Hang Seng) -7.9% en queue -- ecart tres large entre blocs sur 12 mois (108pt) -- les cycles economiques ou les flux divergent nettement. ROTATION en cours : Coree (KOSPI) mene sur 12 mois mais Hong Kong (Hang Seng) a repris la tete sur 3 mois _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -988,7 +988,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>**Momentum prix** — SP500 momentum 12-1 mois = 14.92% -- haussier (momentum positif), detail 1/3/6/12m = [0.41, 3.13, 17.37, 15.39] _(observation : 2026-09-30)_</t>
+          <t>**Momentum prix** — SP500 momentum 12-1 mois = 14.92% -- haussier (momentum positif), detail 1/3/6/12m = [0.18, 2.9, 17.1, 15.12] _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1002,42 +1002,42 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>**Beta vol** — beta SP500/VIX (60j) = -0.00486 (rendement SP500 pour +1pt VIX) -- sensibilite normale, relation inverse attendue (normale) _(observation : 2026-09-30)_</t>
+          <t>**Beta vol** — beta SP500/VIX (60j) = -0.00485 (rendement SP500 pour +1pt VIX) -- sensibilite normale, relation inverse attendue (normale) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>**Rotation sectorielle** — classement momentum 3 mois (10 secteurs) : 1. Energie (XLE) : +17.15% | 2. Sante (XLV) : +6.59% | 3. Technologie (XLK) : +5.97% | 4. Finance (XLF) : -1.76% | 5. Consommation de base (XLP) : -2.25% _(observation : 2026-09-30)_</t>
+          <t>**Rotation sectorielle** — classement momentum 3 mois (10 secteurs) : 1. Energie (XLE) : +17.45% | 2. Sante (XLV) : +6.38% | 3. Technologie (XLK) : +5.86% | 4. Finance (XLF) : -2.18% | 5. Consommation de base (XLP) : -2.59% _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>**Saisonnalite** — rendement journalier moyen ete=+0.0181%, hiver=+0.0465% (t=-1.02, p=0.3056) -- non significatif (attendu vu la faible puissance sur seulement ~2 ans) _(observation : 2026-09-30)_</t>
+          <t>**Saisonnalite** — rendement journalier moyen ete=+0.0180%, hiver=+0.0465% (t=-1.03, p=0.3045) -- non significatif (attendu vu la faible puissance sur seulement ~2 ans) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>**Dispersion sectorielle** — 10 secteurs, rendement moyen 3m=-1.16%, dispersion (ecart-type)=8.24pt, etendue=28.72pt -- dispersion intermediaire _(observation : 2026-09-30)_</t>
+          <t>**Dispersion sectorielle** — 10 secteurs, rendement moyen 3m=-1.34%, dispersion (ecart-type)=8.36pt, etendue=28.98pt -- dispersion intermediaire _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>**Low volatility** — tercile bas-vol ['XLF', 'XLRE', 'XLU'] Sharpe=-1.005 vs tercile haut-vol ['XLY', 'XLE', 'XLK'] Sharpe=0.101 -- anomalie low-vol non confirmee sur cet echantillon (puissance statistique faible, n petit -- limite assumee) _(observation : 2026-09-30)_</t>
+          <t>**Low volatility** — tercile bas-vol ['XLF', 'XLRE', 'XLU'] Sharpe=-1.047 vs tercile haut-vol ['XLY', 'XLE', 'XLK'] Sharpe=0.094 -- anomalie low-vol non confirmee sur cet echantillon (puissance statistique faible, n petit -- limite assumee) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>**Momentum cross sectional** — panier gagnant ['XLE', 'XLV', 'XLK'] (+9.90%) vs panier perdant ['XLY', 'XLI', 'XLU'] (-8.97%) -- spread momentum=+18.87pt _(observation : 2026-09-30)_</t>
+          <t>**Momentum cross sectional** — panier gagnant ['XLE', 'XLV', 'XLK'] (+9.90%) vs panier perdant ['XLY', 'XLI', 'XLU'] (-9.19%) -- spread momentum=+19.08pt _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>**Correlation facteurs** — correlation entre momentum 3m et beta-VIX, 10 secteurs : +0.267 (facteurs largement independants) _(observation : 2026-09-30)_</t>
+          <t>**Correlation facteurs** — correlation entre momentum 3m et beta-VIX, 10 secteurs : +0.271 (facteurs largement independants) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1107,7 +1107,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>**Divergence cot prix** — SP500 +0.41% sur 30j, COT net -10560 -&gt; -133228 -- DIVERGENCE (prix monte, positionnement recule) _(observation : 2026-09-30)_</t>
+          <t>**Divergence cot prix** — SP500 +0.18% sur 30j, COT net -10560 -&gt; -133228 -- DIVERGENCE (prix monte, positionnement recule) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1191,14 +1191,14 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>**Vol cross asset** — 6 mesures de volatilite : Petrole (OVX) 84e pct, Or (GVZ) 82e pct, Taux US (MOVE) 57e pct, Nasdaq (VXN) 49e pct, Vol de la vol (VVIX) 32e pct, Actions US (VIX) 31e pct -- stress LOCALISE sur Petrole (OVX), Or (GVZ) pendant que le reste ne l'est pas -- episode propre a cette classe d'actifs, pas une aversion au risque d'ensemble _(observation : 2026-09-30)_</t>
+          <t>**Vol cross asset** — 6 mesures de volatilite : Or (GVZ) 84e pct, Petrole (OVX) 83e pct, Taux US (MOVE) 62e pct, Nasdaq (VXN) 48e pct, Vol de la vol (VVIX) 30e pct, Actions US (VIX) 30e pct -- stress LOCALISE sur Or (GVZ), Petrole (OVX) pendant que le reste ne l'est pas -- episode propre a cette classe d'actifs, pas une aversion au risque d'ensemble _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>**Volatilite ewma** — vol realisee 60j=0.11218051553973624, EWMA=0.1054 (tendance 10 runs: stable) _(observation : 2026-09-30)_</t>
+          <t>**Volatilite ewma** — vol realisee 60j=0.11178654130535158, EWMA=0.1037 (tendance 10 runs: stable) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1219,7 +1219,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>**Ornstein uhlenbeck vix** — VIX actuel=15.86, niveau moyen estime (mu)=20.20, demi-vie=28.8j, ecart actuel=-4.34 -- VIX actuel en-dessous de son niveau moyen de long terme _(observation : 2026-09-30)_</t>
+          <t>**Ornstein uhlenbeck vix** — VIX actuel=15.83, niveau moyen estime (mu)=20.20, demi-vie=28.8j, ecart actuel=-4.37 -- VIX actuel en-dessous de son niveau moyen de long terme _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1233,14 +1233,14 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>**Kalman niveau local** — VIX observe=15.86, filtre Kalman=15.88 (ecart-type=0.62), ratio signal/bruit=0.2052 -- le filtre lisse fortement le bruit, reagit lentement (ecart obs.-filtre=-0.02) _(observation : 2026-09-30)_</t>
+          <t>**Kalman niveau local** — VIX observe=15.83, filtre Kalman=15.86 (ecart-type=0.62), ratio signal/bruit=0.2052 -- le filtre lisse fortement le bruit, reagit lentement (ecart obs.-filtre=-0.03) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.3727962617538463 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.052375438187575216 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-30)_</t>
+          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.3729361339989534 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.05236469052186711 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1261,14 +1261,14 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>**Skew kurtosis** — skewness=-0.194 (asymetrie negative (pertes extremes &gt; gains extremes)), kurtosis exces=+1.012 (queues epaisses (risque extreme sous-estime par une hypothese normale)) _(observation : 2026-09-30)_</t>
+          <t>**Skew kurtosis** — skewness=-0.192 (asymetrie negative (pertes extremes &gt; gains extremes)), kurtosis exces=+1.020 (queues epaisses (risque extreme sous-estime par une hypothese normale)) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>**Ratios performance** — Sharpe=1.105 (bon), Sortino=1.091 (bon), Calmar=1.579 (bon) -- lecture sur fenetre 252j (~1 an, echantillon limite), seuils academiques standards, taux sans risque suppose nul _(observation : 2026-09-30)_</t>
+          <t>**Ratios performance** — Sharpe=1.087 (bon), Sortino=1.073 (bon), Calmar=1.554 (bon) -- lecture sur fenetre 252j (~1 an, echantillon limite), seuils academiques standards, taux sans risque suppose nul _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1282,14 +1282,14 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>**Stress test historique** — COVID_2020 (2020-02-19 -&gt; 2020-03-23) : chute historique=-33.9% -- rejouee sur le niveau actuel (7718) -&gt; 5099  _(sans synthese)_ _(observation : 2026-09-30)_</t>
+          <t>**Stress test historique** — COVID_2020 (2020-02-19 -&gt; 2020-03-23) : chute historique=-33.9% -- rejouee sur le niveau actuel (7700) -&gt; 5088  _(sans synthese)_ _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>**Sizing robuste** — vol point estimate=0.1299, IC90%=[0.1176, 0.1415] (1000 tirages bootstrap) -- intervalle etroit (18% du point estimate) -- estimation relativement fiable _(observation : 2026-09-30)_</t>
+          <t>**Sizing robuste** — vol point estimate=0.1298, IC90%=[0.1175, 0.1414] (1000 tirages bootstrap) -- intervalle etroit (18% du point estimate) -- estimation relativement fiable _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1303,7 +1303,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>**Detection saut** — Z-stat BNS (fenetre 22j)=1.172 (seuil ±1.96) -- pas de saut isole detecte _(observation : 2026-09-30)_</t>
+          <t>**Detection saut** — Z-stat BNS (fenetre 22j)=1.057 (seuil ±1.96) -- pas de saut isole detecte _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1331,21 +1331,21 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>**Decomposition stl** — VIX : tendance=15.55, composante saisonniere (periode 5j)=+0.336, residu=-0.023 -- la saisonnalite explique 0.68% de la variance totale (negligeable) _(observation : 2026-09-30)_</t>
+          <t>**Decomposition stl** — VIX : tendance=15.54, composante saisonniere (periode 5j)=+0.325, residu=-0.037 -- la saisonnalite explique 0.68% de la variance totale (negligeable) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>**Ratios conditionnels regime** — Sharpe regime haut-vol=-1.107, bas-vol=2.403, global=0.422 -- meilleur en regime calme, comme attendu _(observation : 2026-09-30)_</t>
+          <t>**Ratios conditionnels regime** — Sharpe regime haut-vol=-1.107, bas-vol=2.402, global=0.421 -- meilleur en regime calme, comme attendu _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>**Choc vol parametrique** — vol actuelle=12.99%, scenarios x1/x2/x3 calcules -- pire scenario (x3) = -3.98%/jour, soit 3.1x le scenario de base _(observation : 2026-09-30)_</t>
+          <t>**Choc vol parametrique** — vol actuelle=12.98%, scenarios x1/x2/x3 calcules -- pire scenario (x3) = -3.98%/jour, soit 3.1x le scenario de base _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1387,7 +1387,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>**Anomalie multivariee** — distance de Mahalanobis=1.020 (seuil 3.0) -- jour ordinaire _(observation : 2026-09-30)_</t>
+          <t>**Anomalie multivariee** — distance de Mahalanobis=0.512 (seuil 3.0) -- jour ordinaire _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>**Couts transaction** — 7517 predictions, 1513 changements de position (5pb/changement) -- rendement cumule brut=-93.23%, cout total=53.08%, net=-96.82% -- les frais mangent une part importante du rendement (&gt;50% du brut) _(observation : 2026-09-30)_</t>
+          <t>**Couts transaction** — 7517 predictions, 1513 changements de position (5pb/changement) -- rendement cumule brut=-93.22%, cout total=53.08%, net=-96.82% -- les frais mangent une part importante du rendement (&gt;50% du brut) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1478,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>**Importance permutation** — R2 base=0.0103 -- importance momentum5j=0.00242, importance variation_vix=0.00882 -- VIX plus important _(observation : 2026-09-30)_</t>
+          <t>**Importance permutation** — R2 base=0.0103 -- importance momentum5j=0.00242, importance variation_vix=0.00883 -- VIX plus important _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -6069,7 +6069,7 @@
         <v>-56.78</v>
       </c>
       <c r="F30" t="n">
-        <v>3335.92</v>
+        <v>3328.24</v>
       </c>
     </row>
     <row r="31">
@@ -6097,7 +6097,7 @@
         <v>-33.92</v>
       </c>
       <c r="F31" t="n">
-        <v>5099.43</v>
+        <v>5087.69</v>
       </c>
     </row>
   </sheetData>
@@ -7757,7 +7757,7 @@
         <v>5</v>
       </c>
       <c r="C16" t="n">
-        <v>0.07565</v>
+        <v>0.0756</v>
       </c>
       <c r="D16" t="n">
         <v>0.00415</v>
@@ -9131,10 +9131,10 @@
         <v>10</v>
       </c>
       <c r="C16" t="n">
-        <v>0.3728</v>
+        <v>0.37294</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.052375</v>
+        <v>-0.052365</v>
       </c>
     </row>
   </sheetData>
@@ -9194,7 +9194,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Petrole (OVX)</t>
+          <t>Or (GVZ)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -9203,10 +9203,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>53.11</v>
+        <v>24.01</v>
       </c>
       <c r="D2" t="n">
-        <v>84.5</v>
+        <v>83.8</v>
       </c>
       <c r="E2" t="n">
         <v>1260</v>
@@ -9220,7 +9220,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Or (GVZ)</t>
+          <t>Petrole (OVX)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -9229,10 +9229,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>23.71</v>
+        <v>51.98</v>
       </c>
       <c r="D3" t="n">
-        <v>82.3</v>
+        <v>82.7</v>
       </c>
       <c r="E3" t="n">
         <v>1260</v>
@@ -9255,10 +9255,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>106.16</v>
+        <v>109.19</v>
       </c>
       <c r="D4" t="n">
-        <v>56.7</v>
+        <v>61.7</v>
       </c>
       <c r="E4" t="n">
         <v>1260</v>
@@ -9281,10 +9281,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>22.28</v>
+        <v>22.16</v>
       </c>
       <c r="D5" t="n">
-        <v>49</v>
+        <v>48.2</v>
       </c>
       <c r="E5" t="n">
         <v>1260</v>
@@ -9307,10 +9307,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>89.09</v>
+        <v>88.72</v>
       </c>
       <c r="D6" t="n">
-        <v>31.7</v>
+        <v>30.3</v>
       </c>
       <c r="E6" t="n">
         <v>1260</v>
@@ -9333,10 +9333,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>15.86</v>
+        <v>15.83</v>
       </c>
       <c r="D7" t="n">
-        <v>30.6</v>
+        <v>29.7</v>
       </c>
       <c r="E7" t="n">
         <v>1260</v>
@@ -9668,16 +9668,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.1054</v>
+        <v>0.1037</v>
       </c>
       <c r="C16" t="n">
-        <v>0.0888</v>
+        <v>0.0805</v>
       </c>
       <c r="D16" t="n">
-        <v>0.1094</v>
+        <v>0.1082</v>
       </c>
       <c r="E16" t="n">
-        <v>0.1122</v>
+        <v>0.1118</v>
       </c>
     </row>
   </sheetData>
@@ -12687,7 +12687,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>12.988</v>
+        <v>12.981</v>
       </c>
       <c r="C16" t="n">
         <v>-1.288</v>
@@ -12696,7 +12696,7 @@
         <v>-2.633</v>
       </c>
       <c r="E16" t="n">
-        <v>-3.979</v>
+        <v>-3.978</v>
       </c>
     </row>
   </sheetData>
@@ -17802,10 +17802,10 @@
         </is>
       </c>
       <c r="C142" t="n">
-        <v>-2.4931</v>
+        <v>-2.4626</v>
       </c>
       <c r="D142" t="n">
-        <v>0.2821</v>
+        <v>0.2958</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -17825,10 +17825,10 @@
         </is>
       </c>
       <c r="C143" t="n">
-        <v>-1.7429</v>
+        <v>-1.7131</v>
       </c>
       <c r="D143" t="n">
-        <v>0.657</v>
+        <v>0.6709000000000001</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -17848,10 +17848,10 @@
         </is>
       </c>
       <c r="C144" t="n">
-        <v>-2.139</v>
+        <v>-2.1465</v>
       </c>
       <c r="D144" t="n">
-        <v>0.456</v>
+        <v>0.4521</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -17871,10 +17871,10 @@
         </is>
       </c>
       <c r="C145" t="n">
-        <v>-2.39</v>
+        <v>-2.3904</v>
       </c>
       <c r="D145" t="n">
-        <v>0.3296</v>
+        <v>0.3294</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -17894,10 +17894,10 @@
         </is>
       </c>
       <c r="C146" t="n">
-        <v>-1.2558</v>
+        <v>-1.2267</v>
       </c>
       <c r="D146" t="n">
-        <v>0.8427</v>
+        <v>0.8508</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -17917,10 +17917,10 @@
         </is>
       </c>
       <c r="C147" t="n">
-        <v>0.09710000000000001</v>
+        <v>0.1087</v>
       </c>
       <c r="D147" t="n">
-        <v>0.9879</v>
+        <v>0.9881</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -17940,10 +17940,10 @@
         </is>
       </c>
       <c r="C148" t="n">
-        <v>-1.1067</v>
+        <v>-1.0933</v>
       </c>
       <c r="D148" t="n">
-        <v>0.8807</v>
+        <v>0.8837</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -17963,10 +17963,10 @@
         </is>
       </c>
       <c r="C149" t="n">
-        <v>-0.5633</v>
+        <v>-0.6028</v>
       </c>
       <c r="D149" t="n">
-        <v>0.9595</v>
+        <v>0.9562</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -17986,10 +17986,10 @@
         </is>
       </c>
       <c r="C150" t="n">
-        <v>-2.0839</v>
+        <v>-2.0927</v>
       </c>
       <c r="D150" t="n">
-        <v>0.4848</v>
+        <v>0.4802</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -18009,10 +18009,10 @@
         </is>
       </c>
       <c r="C151" t="n">
-        <v>-1.5015</v>
+        <v>-1.4984</v>
       </c>
       <c r="D151" t="n">
-        <v>0.7606000000000001</v>
+        <v>0.7618</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -25142,7 +25142,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.0985</v>
+        <v>0.0973</v>
       </c>
       <c r="C15" t="n">
         <v>3</v>
@@ -25154,7 +25154,7 @@
         <v>0.2357</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.5373</v>
+        <v>-0.541</v>
       </c>
     </row>
   </sheetData>
@@ -25455,7 +25455,7 @@
         <v>10</v>
       </c>
       <c r="C16" t="n">
-        <v>0.2665</v>
+        <v>0.2711</v>
       </c>
     </row>
   </sheetData>
@@ -37814,7 +37814,7 @@
         <v>53.08</v>
       </c>
       <c r="E16" t="n">
-        <v>-93.23</v>
+        <v>-93.22</v>
       </c>
       <c r="F16" t="n">
         <v>-96.81999999999999</v>
@@ -38215,19 +38215,19 @@
         <v>2.2</v>
       </c>
       <c r="C15" t="n">
-        <v>413.47</v>
+        <v>413.44</v>
       </c>
       <c r="D15" t="n">
         <v>4</v>
       </c>
       <c r="E15" t="n">
-        <v>372.99</v>
+        <v>372.92</v>
       </c>
       <c r="F15" t="n">
         <v>5.3</v>
       </c>
       <c r="G15" t="n">
-        <v>323.97</v>
+        <v>323.99</v>
       </c>
     </row>
   </sheetData>
@@ -39741,13 +39741,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>15.547</v>
+        <v>15.542</v>
       </c>
       <c r="C15" t="n">
-        <v>0.336</v>
+        <v>0.325</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.023</v>
+        <v>-0.037</v>
       </c>
       <c r="E15" t="n">
         <v>0.68</v>
@@ -40656,7 +40656,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1.172</v>
+        <v>1.057</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -41308,13 +41308,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.00608</v>
+        <v>0.00378</v>
       </c>
       <c r="C16" t="n">
-        <v>-0.18</v>
+        <v>-0.21</v>
       </c>
       <c r="D16" t="n">
-        <v>1.02</v>
+        <v>0.512</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -41646,13 +41646,13 @@
         <v>10</v>
       </c>
       <c r="C16" t="n">
-        <v>-1.164</v>
+        <v>-1.344</v>
       </c>
       <c r="D16" t="n">
-        <v>8.24</v>
+        <v>8.356</v>
       </c>
       <c r="E16" t="n">
-        <v>28.717</v>
+        <v>28.977</v>
       </c>
     </row>
   </sheetData>
@@ -42004,7 +42004,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.41</v>
+        <v>0.179</v>
       </c>
       <c r="C16" t="n">
         <v>-133228</v>
@@ -49718,25 +49718,25 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>fred/ECBASSETSW.csv</t>
+          <t>bis/taux_directeurs/CN.csv</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D106" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E106" t="n">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="F106" t="n">
-        <v>1447</v>
+        <v>10949</v>
       </c>
       <c r="G106" t="inlineStr">
         <is>
@@ -49747,25 +49747,25 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>bis/taux_directeurs/CN.csv</t>
+          <t>bilans/BCE_AVOIRS_DE_RESERVE.csv</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D107" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E107" t="n">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="F107" t="n">
-        <v>10949</v>
+        <v>1448</v>
       </c>
       <c r="G107" t="inlineStr">
         <is>
@@ -49776,7 +49776,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>bilans/BCE_AVOIRS_DE_RESERVE.csv</t>
+          <t>bis/taux_directeurs/CA.csv</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -49788,13 +49788,13 @@
         <v>9</v>
       </c>
       <c r="D108" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E108" t="n">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="F108" t="n">
-        <v>1448</v>
+        <v>23147</v>
       </c>
       <c r="G108" t="inlineStr">
         <is>
@@ -49805,7 +49805,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>bis/taux_directeurs/CA.csv</t>
+          <t>bis/taux_directeurs/GB.csv</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -49823,7 +49823,7 @@
         <v>42</v>
       </c>
       <c r="F109" t="n">
-        <v>23147</v>
+        <v>23865</v>
       </c>
       <c r="G109" t="inlineStr">
         <is>
@@ -49834,16 +49834,16 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>bis/taux_directeurs/GB.csv</t>
+          <t>bis/taux_directeurs/CH.csv</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D110" t="n">
         <v>1</v>
@@ -49852,7 +49852,7 @@
         <v>42</v>
       </c>
       <c r="F110" t="n">
-        <v>23865</v>
+        <v>21061</v>
       </c>
       <c r="G110" t="inlineStr">
         <is>
@@ -49863,7 +49863,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>bis/taux_directeurs/CH.csv</t>
+          <t>bis/taux_directeurs/JP.csv</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -49881,7 +49881,7 @@
         <v>42</v>
       </c>
       <c r="F111" t="n">
-        <v>21061</v>
+        <v>24889</v>
       </c>
       <c r="G111" t="inlineStr">
         <is>
@@ -49892,7 +49892,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>bis/taux_directeurs/JP.csv</t>
+          <t>bis/taux_directeurs/SE.csv</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -49910,7 +49910,7 @@
         <v>42</v>
       </c>
       <c r="F112" t="n">
-        <v>24889</v>
+        <v>22804</v>
       </c>
       <c r="G112" t="inlineStr">
         <is>
@@ -49921,7 +49921,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>bis/taux_directeurs/SE.csv</t>
+          <t>bis/taux_directeurs/US.csv</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -49939,7 +49939,7 @@
         <v>42</v>
       </c>
       <c r="F113" t="n">
-        <v>22804</v>
+        <v>26381</v>
       </c>
       <c r="G113" t="inlineStr">
         <is>
@@ -49950,7 +49950,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>bis/taux_directeurs/US.csv</t>
+          <t>bis/taux_directeurs/XM.csv</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -49968,7 +49968,7 @@
         <v>42</v>
       </c>
       <c r="F114" t="n">
-        <v>26381</v>
+        <v>10127</v>
       </c>
       <c r="G114" t="inlineStr">
         <is>
@@ -49979,7 +49979,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>bis/taux_directeurs/XM.csv</t>
+          <t>cftc/AUD_FX.csv</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -49991,13 +49991,13 @@
         <v>8</v>
       </c>
       <c r="D115" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E115" t="n">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="F115" t="n">
-        <v>10127</v>
+        <v>1000</v>
       </c>
       <c r="G115" t="inlineStr">
         <is>
@@ -50008,7 +50008,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>cftc/AUD_FX.csv</t>
+          <t>cftc/BRENT_CRUDE.csv</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -50026,7 +50026,7 @@
         <v>63</v>
       </c>
       <c r="F116" t="n">
-        <v>1000</v>
+        <v>242</v>
       </c>
       <c r="G116" t="inlineStr">
         <is>
@@ -50037,7 +50037,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>cftc/BRENT_CRUDE.csv</t>
+          <t>cftc/CAD_FX.csv</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -50055,7 +50055,7 @@
         <v>63</v>
       </c>
       <c r="F117" t="n">
-        <v>242</v>
+        <v>1000</v>
       </c>
       <c r="G117" t="inlineStr">
         <is>
@@ -50066,7 +50066,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>cftc/CAD_FX.csv</t>
+          <t>cftc/CHF_FX.csv</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -50095,7 +50095,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>cftc/CHF_FX.csv</t>
+          <t>cftc/COPPER.csv</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -50113,7 +50113,7 @@
         <v>63</v>
       </c>
       <c r="F119" t="n">
-        <v>1000</v>
+        <v>242</v>
       </c>
       <c r="G119" t="inlineStr">
         <is>
@@ -50124,7 +50124,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>cftc/COPPER.csv</t>
+          <t>cftc/CORN.csv</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -50142,7 +50142,7 @@
         <v>63</v>
       </c>
       <c r="F120" t="n">
-        <v>242</v>
+        <v>1000</v>
       </c>
       <c r="G120" t="inlineStr">
         <is>
@@ -50153,7 +50153,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>cftc/CORN.csv</t>
+          <t>cftc/EUR_FX.csv</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -50182,7 +50182,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>cftc/EUR_FX.csv</t>
+          <t>cftc/FED_FUNDS.csv</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -50200,7 +50200,7 @@
         <v>63</v>
       </c>
       <c r="F122" t="n">
-        <v>1000</v>
+        <v>242</v>
       </c>
       <c r="G122" t="inlineStr">
         <is>
@@ -50211,7 +50211,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>cftc/FED_FUNDS.csv</t>
+          <t>cftc/GBP_FX.csv</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -50240,7 +50240,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>cftc/GBP_FX.csv</t>
+          <t>cftc/GOLD.csv</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -50258,7 +50258,7 @@
         <v>63</v>
       </c>
       <c r="F124" t="n">
-        <v>242</v>
+        <v>1000</v>
       </c>
       <c r="G124" t="inlineStr">
         <is>
@@ -50269,7 +50269,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>cftc/GOLD.csv</t>
+          <t>cftc/JPY_FX.csv</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -50298,7 +50298,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>cftc/JPY_FX.csv</t>
+          <t>cftc/MXN_FX.csv</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -50327,7 +50327,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>cftc/MXN_FX.csv</t>
+          <t>cftc/NASDAQ_MINI.csv</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -50345,7 +50345,7 @@
         <v>63</v>
       </c>
       <c r="F127" t="n">
-        <v>1000</v>
+        <v>242</v>
       </c>
       <c r="G127" t="inlineStr">
         <is>
@@ -50356,7 +50356,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>cftc/NASDAQ_MINI.csv</t>
+          <t>cftc/NAT_GAS.csv</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -50385,7 +50385,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>cftc/NAT_GAS.csv</t>
+          <t>cftc/NZD_FX.csv</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -50414,7 +50414,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>cftc/NZD_FX.csv</t>
+          <t>cftc/PALLADIUM.csv</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -50432,7 +50432,7 @@
         <v>63</v>
       </c>
       <c r="F130" t="n">
-        <v>242</v>
+        <v>1000</v>
       </c>
       <c r="G130" t="inlineStr">
         <is>
@@ -50443,7 +50443,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>cftc/PALLADIUM.csv</t>
+          <t>cftc/PLATINUM.csv</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -50472,7 +50472,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>cftc/PLATINUM.csv</t>
+          <t>cftc/RUSSELL_MINI.csv</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -50490,7 +50490,7 @@
         <v>63</v>
       </c>
       <c r="F132" t="n">
-        <v>1000</v>
+        <v>242</v>
       </c>
       <c r="G132" t="inlineStr">
         <is>
@@ -50501,7 +50501,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>cftc/RUSSELL_MINI.csv</t>
+          <t>cftc/SILVER.csv</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -50519,7 +50519,7 @@
         <v>63</v>
       </c>
       <c r="F133" t="n">
-        <v>242</v>
+        <v>1000</v>
       </c>
       <c r="G133" t="inlineStr">
         <is>
@@ -50530,7 +50530,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>cftc/SILVER.csv</t>
+          <t>cftc/SOFR_3M.csv</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -50548,7 +50548,7 @@
         <v>63</v>
       </c>
       <c r="F134" t="n">
-        <v>1000</v>
+        <v>242</v>
       </c>
       <c r="G134" t="inlineStr">
         <is>
@@ -50559,7 +50559,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>cftc/SOFR_3M.csv</t>
+          <t>cftc/SOYBEANS.csv</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -50577,7 +50577,7 @@
         <v>63</v>
       </c>
       <c r="F135" t="n">
-        <v>242</v>
+        <v>1000</v>
       </c>
       <c r="G135" t="inlineStr">
         <is>
@@ -50588,7 +50588,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>cftc/SOYBEANS.csv</t>
+          <t>cftc/SP500_EMINI.csv</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -50606,7 +50606,7 @@
         <v>63</v>
       </c>
       <c r="F136" t="n">
-        <v>1000</v>
+        <v>242</v>
       </c>
       <c r="G136" t="inlineStr">
         <is>
@@ -50617,7 +50617,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>cftc/SP500_EMINI.csv</t>
+          <t>cftc/USD_INDEX.csv</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -50646,7 +50646,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>cftc/USD_INDEX.csv</t>
+          <t>cftc/UST_10Y.csv</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -50675,7 +50675,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>cftc/UST_10Y.csv</t>
+          <t>cftc/UST_2Y.csv</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -50704,7 +50704,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>cftc/UST_2Y.csv</t>
+          <t>cftc/UST_5Y.csv</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -50733,7 +50733,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>cftc/UST_5Y.csv</t>
+          <t>cftc/UST_BOND.csv</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -50762,7 +50762,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>cftc/UST_BOND.csv</t>
+          <t>cftc/UST_ULTRA_10Y.csv</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -50791,7 +50791,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>cftc/UST_ULTRA_10Y.csv</t>
+          <t>cftc/UST_ULTRA_BOND.csv</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -50809,7 +50809,7 @@
         <v>63</v>
       </c>
       <c r="F143" t="n">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="G143" t="inlineStr">
         <is>
@@ -50820,7 +50820,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>cftc/UST_ULTRA_BOND.csv</t>
+          <t>cftc/VIX_FUT.csv</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -50838,7 +50838,7 @@
         <v>63</v>
       </c>
       <c r="F144" t="n">
-        <v>240</v>
+        <v>1000</v>
       </c>
       <c r="G144" t="inlineStr">
         <is>
@@ -50849,7 +50849,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>cftc/VIX_FUT.csv</t>
+          <t>cftc/WHEAT.csv</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -50867,7 +50867,7 @@
         <v>63</v>
       </c>
       <c r="F145" t="n">
-        <v>1000</v>
+        <v>667</v>
       </c>
       <c r="G145" t="inlineStr">
         <is>
@@ -50878,7 +50878,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>cftc/WHEAT.csv</t>
+          <t>cftc/WTI_CRUDE.csv</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -50896,7 +50896,7 @@
         <v>63</v>
       </c>
       <c r="F146" t="n">
-        <v>667</v>
+        <v>242</v>
       </c>
       <c r="G146" t="inlineStr">
         <is>
@@ -50907,16 +50907,16 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>cftc/WTI_CRUDE.csv</t>
+          <t>bilans/BOC_V1038114416.csv</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D147" t="n">
         <v>7</v>
@@ -50925,7 +50925,7 @@
         <v>63</v>
       </c>
       <c r="F147" t="n">
-        <v>242</v>
+        <v>405</v>
       </c>
       <c r="G147" t="inlineStr">
         <is>
@@ -50936,7 +50936,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>bilans/BOC_V1038114416.csv</t>
+          <t>bilans/BOC_V1146067261.csv</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -50954,7 +50954,7 @@
         <v>63</v>
       </c>
       <c r="F148" t="n">
-        <v>405</v>
+        <v>340</v>
       </c>
       <c r="G148" t="inlineStr">
         <is>
@@ -50965,7 +50965,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>bilans/BOC_V1146067261.csv</t>
+          <t>bilans/BOC_V1146067262.csv</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -50994,7 +50994,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>bilans/BOC_V1146067262.csv</t>
+          <t>bilans/BOC_V1146067263.csv</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -51012,7 +51012,7 @@
         <v>63</v>
       </c>
       <c r="F150" t="n">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="G150" t="inlineStr">
         <is>
@@ -51023,7 +51023,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>bilans/BOC_V1146067263.csv</t>
+          <t>bilans/BOC_V1146067264.csv</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -51041,7 +51041,7 @@
         <v>63</v>
       </c>
       <c r="F151" t="n">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="G151" t="inlineStr">
         <is>
@@ -51052,7 +51052,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>bilans/BOC_V1146067264.csv</t>
+          <t>bilans/BOC_V1154426989.csv</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -51070,7 +51070,7 @@
         <v>63</v>
       </c>
       <c r="F152" t="n">
-        <v>340</v>
+        <v>333</v>
       </c>
       <c r="G152" t="inlineStr">
         <is>
@@ -51081,7 +51081,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>bilans/BOC_V1154426989.csv</t>
+          <t>bilans/BOC_V1154426990.csv</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -51099,7 +51099,7 @@
         <v>63</v>
       </c>
       <c r="F153" t="n">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="G153" t="inlineStr">
         <is>
@@ -51110,7 +51110,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>bilans/BOC_V1154426990.csv</t>
+          <t>bilans/BOC_V1154426991.csv</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -51128,7 +51128,7 @@
         <v>63</v>
       </c>
       <c r="F154" t="n">
-        <v>330</v>
+        <v>308</v>
       </c>
       <c r="G154" t="inlineStr">
         <is>
@@ -51139,7 +51139,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>bilans/BOC_V1154426991.csv</t>
+          <t>bilans/BOC_V1160788296.csv</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -51157,7 +51157,7 @@
         <v>63</v>
       </c>
       <c r="F155" t="n">
-        <v>308</v>
+        <v>330</v>
       </c>
       <c r="G155" t="inlineStr">
         <is>
@@ -51168,7 +51168,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>bilans/BOC_V1160788296.csv</t>
+          <t>bilans/BOC_V1203435186.csv</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -51186,7 +51186,7 @@
         <v>63</v>
       </c>
       <c r="F156" t="n">
-        <v>330</v>
+        <v>322</v>
       </c>
       <c r="G156" t="inlineStr">
         <is>
@@ -51197,7 +51197,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>bilans/BOC_V1203435186.csv</t>
+          <t>bilans/BOC_V1210798115.csv</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -51215,7 +51215,7 @@
         <v>63</v>
       </c>
       <c r="F157" t="n">
-        <v>322</v>
+        <v>326</v>
       </c>
       <c r="G157" t="inlineStr">
         <is>
@@ -51226,7 +51226,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>bilans/BOC_V1210798115.csv</t>
+          <t>bilans/BOC_V1490410223.csv</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -51244,7 +51244,7 @@
         <v>63</v>
       </c>
       <c r="F158" t="n">
-        <v>326</v>
+        <v>195</v>
       </c>
       <c r="G158" t="inlineStr">
         <is>
@@ -51255,7 +51255,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>bilans/BOC_V1490410223.csv</t>
+          <t>bilans/BOC_V1490410224.csv</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -51284,7 +51284,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>bilans/BOC_V1490410224.csv</t>
+          <t>bilans/BOC_V36610.csv</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -51302,7 +51302,7 @@
         <v>63</v>
       </c>
       <c r="F160" t="n">
-        <v>195</v>
+        <v>1917</v>
       </c>
       <c r="G160" t="inlineStr">
         <is>
@@ -51313,7 +51313,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>bilans/BOC_V36610.csv</t>
+          <t>bilans/BOC_V36612.csv</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -51342,7 +51342,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>bilans/BOC_V36612.csv</t>
+          <t>bilans/BOC_V36613.csv</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -51371,7 +51371,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>bilans/BOC_V36613.csv</t>
+          <t>bilans/BOC_V36624.csv</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -51400,7 +51400,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>bilans/BOC_V36624.csv</t>
+          <t>bilans/BOC_V36625.csv</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -51429,7 +51429,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>bilans/BOC_V36625.csv</t>
+          <t>bilans/BOC_V36628.csv</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
@@ -51458,7 +51458,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>bilans/BOC_V36628.csv</t>
+          <t>bilans/BOC_V36634.csv</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -51487,7 +51487,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>bilans/BOC_V36634.csv</t>
+          <t>bilans/BOC_V36635.csv</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -51516,7 +51516,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>bilans/BOC_V36635.csv</t>
+          <t>bilans/BOC_V36636.csv</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -51545,7 +51545,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>bilans/BOC_V36636.csv</t>
+          <t>bilans/BOC_V44201362.csv</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
@@ -51563,7 +51563,7 @@
         <v>63</v>
       </c>
       <c r="F169" t="n">
-        <v>1917</v>
+        <v>991</v>
       </c>
       <c r="G169" t="inlineStr">
         <is>
@@ -51574,7 +51574,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>bilans/BOC_V44201362.csv</t>
+          <t>bilans/BOE_BILAN_TOTAL.csv</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -51592,7 +51592,7 @@
         <v>63</v>
       </c>
       <c r="F170" t="n">
-        <v>991</v>
+        <v>1610</v>
       </c>
       <c r="G170" t="inlineStr">
         <is>
@@ -51603,7 +51603,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>bilans/BOE_BILAN_TOTAL.csv</t>
+          <t>bilans/RBA_BILAN_TOTAL.csv</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -51621,7 +51621,7 @@
         <v>63</v>
       </c>
       <c r="F171" t="n">
-        <v>1610</v>
+        <v>691</v>
       </c>
       <c r="G171" t="inlineStr">
         <is>
@@ -51632,7 +51632,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>bilans/RBA_BILAN_TOTAL.csv</t>
+          <t>bilans/RBA_OR_ET_DEVISES.csv</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -51661,7 +51661,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>bilans/RBA_OR_ET_DEVISES.csv</t>
+          <t>bilans/RBA_TITRES_LOCAUX.csv</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -51690,7 +51690,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>bilans/RBA_TITRES_LOCAUX.csv</t>
+          <t>fred/RESPPLLOPNWW.csv</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -51708,7 +51708,7 @@
         <v>63</v>
       </c>
       <c r="F174" t="n">
-        <v>691</v>
+        <v>1241</v>
       </c>
       <c r="G174" t="inlineStr">
         <is>
@@ -51719,7 +51719,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>fred/RESPPLLOPNWW.csv</t>
+          <t>fred/TREAST.csv</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -51748,7 +51748,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>fred/TREAST.csv</t>
+          <t>fred/WALCL.csv</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -51777,7 +51777,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>fred/WALCL.csv</t>
+          <t>fred/WLRRAL.csv</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
@@ -51806,7 +51806,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>fred/WLRRAL.csv</t>
+          <t>fred/WRESBAL.csv</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -51824,7 +51824,7 @@
         <v>63</v>
       </c>
       <c r="F178" t="n">
-        <v>1241</v>
+        <v>2230</v>
       </c>
       <c r="G178" t="inlineStr">
         <is>
@@ -51835,7 +51835,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>fred/WRESBAL.csv</t>
+          <t>fred/WSHOMCB.csv</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -51853,7 +51853,7 @@
         <v>63</v>
       </c>
       <c r="F179" t="n">
-        <v>2230</v>
+        <v>1241</v>
       </c>
       <c r="G179" t="inlineStr">
         <is>
@@ -51864,7 +51864,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>fred/WSHOMCB.csv</t>
+          <t>fred/WSHOSHO.csv</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -51893,7 +51893,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>fred/WSHOSHO.csv</t>
+          <t>fred/WTREGEN.csv</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -51911,7 +51911,7 @@
         <v>63</v>
       </c>
       <c r="F181" t="n">
-        <v>1241</v>
+        <v>2125</v>
       </c>
       <c r="G181" t="inlineStr">
         <is>
@@ -51922,7 +51922,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>fred/WTREGEN.csv</t>
+          <t>souverains/AUSTRALIE_10A.csv</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
@@ -51934,13 +51934,13 @@
         <v>7</v>
       </c>
       <c r="D182" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E182" t="n">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="F182" t="n">
-        <v>2125</v>
+        <v>3361</v>
       </c>
       <c r="G182" t="inlineStr">
         <is>
@@ -51951,7 +51951,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>souverains/AUSTRALIE_10A.csv</t>
+          <t>souverains/AUSTRALIE_2A.csv</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -51969,7 +51969,7 @@
         <v>42</v>
       </c>
       <c r="F183" t="n">
-        <v>3361</v>
+        <v>3283</v>
       </c>
       <c r="G183" t="inlineStr">
         <is>
@@ -51980,7 +51980,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>souverains/AUSTRALIE_2A.csv</t>
+          <t>souverains/AUSTRALIE_5A.csv</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -52009,25 +52009,25 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>souverains/AUSTRALIE_5A.csv</t>
+          <t>fred/MORTGAGE30US.csv</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="C185" t="n">
+        <v>6</v>
+      </c>
+      <c r="D185" t="n">
         <v>7</v>
       </c>
-      <c r="D185" t="n">
-        <v>1</v>
-      </c>
       <c r="E185" t="n">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="F185" t="n">
-        <v>3283</v>
+        <v>2896</v>
       </c>
       <c r="G185" t="inlineStr">
         <is>
@@ -52038,16 +52038,16 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>fred/MORTGAGE30US.csv</t>
+          <t>fred/ECBASSETSW.csv</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C186" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D186" t="n">
         <v>7</v>
@@ -52056,7 +52056,7 @@
         <v>63</v>
       </c>
       <c r="F186" t="n">
-        <v>2896</v>
+        <v>1448</v>
       </c>
       <c r="G186" t="inlineStr">
         <is>
@@ -52937,7 +52937,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>fred/RRPONTSYD.csv</t>
+          <t>fred/T10YIE.csv</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -52966,7 +52966,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>fred/T10YIE.csv</t>
+          <t>marches/indices/HANGSENG.csv</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -52984,7 +52984,7 @@
         <v>42</v>
       </c>
       <c r="F218" t="n">
-        <v>3000</v>
+        <v>3689</v>
       </c>
       <c r="G218" t="inlineStr">
         <is>
@@ -53430,7 +53430,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>marches/fx/AUDJPY.csv</t>
+          <t>fred/RRPONTSYD.csv</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -53448,7 +53448,7 @@
         <v>42</v>
       </c>
       <c r="F234" t="n">
-        <v>3908</v>
+        <v>3000</v>
       </c>
       <c r="G234" t="inlineStr">
         <is>
@@ -53459,7 +53459,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>marches/fx/AUDUSD.csv</t>
+          <t>marches/fx/AUDJPY.csv</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -53477,7 +53477,7 @@
         <v>42</v>
       </c>
       <c r="F235" t="n">
-        <v>3904</v>
+        <v>3908</v>
       </c>
       <c r="G235" t="inlineStr">
         <is>
@@ -53488,7 +53488,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>marches/fx/DXY.csv</t>
+          <t>marches/fx/AUDUSD.csv</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -53506,7 +53506,7 @@
         <v>42</v>
       </c>
       <c r="F236" t="n">
-        <v>3772</v>
+        <v>3904</v>
       </c>
       <c r="G236" t="inlineStr">
         <is>
@@ -53517,7 +53517,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>marches/fx/EURCHF.csv</t>
+          <t>marches/fx/DXY.csv</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
@@ -53535,7 +53535,7 @@
         <v>42</v>
       </c>
       <c r="F237" t="n">
-        <v>3905</v>
+        <v>3772</v>
       </c>
       <c r="G237" t="inlineStr">
         <is>
@@ -53546,7 +53546,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>marches/fx/EURGBP.csv</t>
+          <t>marches/fx/EURCHF.csv</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
@@ -53564,7 +53564,7 @@
         <v>42</v>
       </c>
       <c r="F238" t="n">
-        <v>3907</v>
+        <v>3905</v>
       </c>
       <c r="G238" t="inlineStr">
         <is>
@@ -53575,7 +53575,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>marches/fx/EURJPY.csv</t>
+          <t>marches/fx/EURGBP.csv</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
@@ -53604,7 +53604,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>marches/fx/EURUSD.csv</t>
+          <t>marches/fx/EURJPY.csv</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
@@ -53622,7 +53622,7 @@
         <v>42</v>
       </c>
       <c r="F240" t="n">
-        <v>3904</v>
+        <v>3907</v>
       </c>
       <c r="G240" t="inlineStr">
         <is>
@@ -53633,7 +53633,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>marches/fx/GBPUSD.csv</t>
+          <t>marches/fx/EURUSD.csv</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
@@ -53651,7 +53651,7 @@
         <v>42</v>
       </c>
       <c r="F241" t="n">
-        <v>3905</v>
+        <v>3904</v>
       </c>
       <c r="G241" t="inlineStr">
         <is>
@@ -53662,7 +53662,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>marches/fx/NZDUSD.csv</t>
+          <t>marches/fx/GBPUSD.csv</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
@@ -53691,7 +53691,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>marches/fx/USDCAD.csv</t>
+          <t>marches/fx/NZDUSD.csv</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
@@ -53709,7 +53709,7 @@
         <v>42</v>
       </c>
       <c r="F243" t="n">
-        <v>3904</v>
+        <v>3905</v>
       </c>
       <c r="G243" t="inlineStr">
         <is>
@@ -53720,7 +53720,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>marches/fx/USDCHF.csv</t>
+          <t>marches/fx/USDCAD.csv</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -53738,7 +53738,7 @@
         <v>42</v>
       </c>
       <c r="F244" t="n">
-        <v>3902</v>
+        <v>3904</v>
       </c>
       <c r="G244" t="inlineStr">
         <is>
@@ -53749,7 +53749,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>marches/fx/USDCNY.csv</t>
+          <t>marches/fx/USDCHF.csv</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -53767,7 +53767,7 @@
         <v>42</v>
       </c>
       <c r="F245" t="n">
-        <v>3904</v>
+        <v>3902</v>
       </c>
       <c r="G245" t="inlineStr">
         <is>
@@ -53778,7 +53778,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>marches/fx/USDJPY.csv</t>
+          <t>marches/fx/USDCNY.csv</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -53796,7 +53796,7 @@
         <v>42</v>
       </c>
       <c r="F246" t="n">
-        <v>3905</v>
+        <v>3904</v>
       </c>
       <c r="G246" t="inlineStr">
         <is>
@@ -53807,7 +53807,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>marches/fx/USDKRW.csv</t>
+          <t>marches/fx/USDJPY.csv</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
@@ -53825,7 +53825,7 @@
         <v>42</v>
       </c>
       <c r="F247" t="n">
-        <v>3904</v>
+        <v>3905</v>
       </c>
       <c r="G247" t="inlineStr">
         <is>
@@ -53836,7 +53836,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>marches/fx/USDNOK.csv</t>
+          <t>marches/fx/USDKRW.csv</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
@@ -53854,7 +53854,7 @@
         <v>42</v>
       </c>
       <c r="F248" t="n">
-        <v>3905</v>
+        <v>3904</v>
       </c>
       <c r="G248" t="inlineStr">
         <is>
@@ -53865,7 +53865,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>marches/fx/USDSEK.csv</t>
+          <t>marches/fx/USDNOK.csv</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
@@ -53894,7 +53894,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>marches/indices/DAX.csv</t>
+          <t>marches/fx/USDSEK.csv</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
@@ -53912,7 +53912,7 @@
         <v>42</v>
       </c>
       <c r="F250" t="n">
-        <v>3802</v>
+        <v>3905</v>
       </c>
       <c r="G250" t="inlineStr">
         <is>
@@ -53923,7 +53923,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>marches/indices/EUROSTOXX50.csv</t>
+          <t>marches/indices/DAX.csv</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
@@ -53941,7 +53941,7 @@
         <v>42</v>
       </c>
       <c r="F251" t="n">
-        <v>3759</v>
+        <v>3802</v>
       </c>
       <c r="G251" t="inlineStr">
         <is>
@@ -53952,7 +53952,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>marches/indices/FTSE100.csv</t>
+          <t>marches/indices/EUROSTOXX50.csv</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -53970,7 +53970,7 @@
         <v>42</v>
       </c>
       <c r="F252" t="n">
-        <v>3788</v>
+        <v>3759</v>
       </c>
       <c r="G252" t="inlineStr">
         <is>
@@ -53981,7 +53981,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>marches/indices/HANGSENG.csv</t>
+          <t>marches/indices/FTSE100.csv</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -53999,7 +53999,7 @@
         <v>42</v>
       </c>
       <c r="F253" t="n">
-        <v>3690</v>
+        <v>3788</v>
       </c>
       <c r="G253" t="inlineStr">
         <is>
@@ -56258,7 +56258,7 @@
         <v>0.00242</v>
       </c>
       <c r="D16" t="n">
-        <v>0.00882</v>
+        <v>0.008829999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -56363,13 +56363,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>7717.64</v>
+        <v>7699.87</v>
       </c>
       <c r="D4" t="n">
-        <v>3.13</v>
+        <v>2.9</v>
       </c>
       <c r="E4" t="n">
-        <v>15.39</v>
+        <v>15.12</v>
       </c>
     </row>
     <row r="5">
@@ -56384,13 +56384,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>10609.71</v>
+        <v>10606</v>
       </c>
       <c r="D5" t="n">
-        <v>1.25</v>
+        <v>1.22</v>
       </c>
       <c r="E5" t="n">
-        <v>13.47</v>
+        <v>13.43</v>
       </c>
     </row>
     <row r="6">
@@ -56405,13 +56405,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>6269.95</v>
+        <v>6269.02</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.2</v>
+        <v>-0.21</v>
       </c>
       <c r="E6" t="n">
-        <v>13.38</v>
+        <v>13.36</v>
       </c>
     </row>
     <row r="7">
@@ -56426,10 +56426,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>25200.04</v>
+        <v>25199.19</v>
       </c>
       <c r="D7" t="n">
-        <v>0.64</v>
+        <v>0.63</v>
       </c>
       <c r="E7" t="n">
         <v>5.52</v>
@@ -56443,17 +56443,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>24613.27</v>
+        <v>24523.57</v>
       </c>
       <c r="D8" t="n">
-        <v>7.57</v>
+        <v>7.18</v>
       </c>
       <c r="E8" t="n">
-        <v>-8.35</v>
+        <v>-7.89</v>
       </c>
     </row>
   </sheetData>
@@ -57167,10 +57167,10 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>15.86</v>
+        <v>15.83</v>
       </c>
       <c r="C15" t="n">
-        <v>15.884</v>
+        <v>15.858</v>
       </c>
       <c r="D15" t="n">
         <v>0.624</v>
@@ -58374,7 +58374,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>-1.005</v>
+        <v>-1.047</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -58382,7 +58382,7 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>0.101</v>
+        <v>0.094</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -58771,25 +58771,25 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.001576</v>
+        <v>0.001582</v>
       </c>
       <c r="C13" t="n">
-        <v>5.08</v>
+        <v>5.47</v>
       </c>
       <c r="D13" t="n">
-        <v>98.89</v>
+        <v>98.29000000000001</v>
       </c>
       <c r="E13" t="n">
-        <v>38.17</v>
+        <v>37.33</v>
       </c>
       <c r="F13" t="n">
-        <v>47.55</v>
+        <v>46.66</v>
       </c>
       <c r="G13" t="n">
-        <v>-6.4</v>
+        <v>-6.49</v>
       </c>
       <c r="H13" t="n">
-        <v>7.33</v>
+        <v>7.61</v>
       </c>
     </row>
   </sheetData>
@@ -59679,7 +59679,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>9.901</v>
+        <v>9.896000000000001</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -59687,10 +59687,10 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>-8.970000000000001</v>
+        <v>-9.186999999999999</v>
       </c>
       <c r="F16" t="n">
-        <v>18.871</v>
+        <v>19.082</v>
       </c>
     </row>
   </sheetData>
@@ -62659,16 +62659,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.41</v>
+        <v>0.179</v>
       </c>
       <c r="C16" t="n">
-        <v>3.132</v>
+        <v>2.895</v>
       </c>
       <c r="D16" t="n">
-        <v>17.373</v>
+        <v>17.103</v>
       </c>
       <c r="E16" t="n">
-        <v>15.387</v>
+        <v>15.122</v>
       </c>
       <c r="F16" t="n">
         <v>14.916</v>
@@ -63511,7 +63511,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>15.86</v>
+        <v>15.83</v>
       </c>
       <c r="C15" t="n">
         <v>20.199</v>
@@ -63523,7 +63523,7 @@
         <v>28.8</v>
       </c>
       <c r="F15" t="n">
-        <v>-4.339</v>
+        <v>-4.369</v>
       </c>
     </row>
   </sheetData>
@@ -68807,7 +68807,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>-0.004859</v>
+        <v>-0.004854</v>
       </c>
     </row>
   </sheetData>
@@ -69712,7 +69712,7 @@
         <v>0.20964</v>
       </c>
       <c r="F16" t="n">
-        <v>2.983e-07</v>
+        <v>2.984e-07</v>
       </c>
       <c r="G16" t="n">
         <v>3.833e-07</v>
@@ -69983,7 +69983,7 @@
         <v>0.00877</v>
       </c>
       <c r="C15" t="n">
-        <v>0.06763</v>
+        <v>0.06764000000000001</v>
       </c>
       <c r="D15" t="n">
         <v>-0.0382</v>
@@ -73205,10 +73205,10 @@
         <v>-1.107</v>
       </c>
       <c r="C16" t="n">
-        <v>2.403</v>
+        <v>2.402</v>
       </c>
       <c r="D16" t="n">
-        <v>0.422</v>
+        <v>0.421</v>
       </c>
     </row>
   </sheetData>
@@ -73484,13 +73484,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1.1045</v>
+        <v>1.0874</v>
       </c>
       <c r="C16" t="n">
-        <v>1.0908</v>
+        <v>1.0733</v>
       </c>
       <c r="D16" t="n">
-        <v>1.5795</v>
+        <v>1.5541</v>
       </c>
     </row>
   </sheetData>
@@ -76990,14 +76990,14 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>-3.62</v>
+        <v>-3.6</v>
       </c>
       <c r="D6" t="n">
-        <v>-3.04</v>
+        <v>-2.85</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -80517,7 +80517,7 @@
         </is>
       </c>
       <c r="E142" t="n">
-        <v>17.146</v>
+        <v>17.451</v>
       </c>
     </row>
     <row r="143">
@@ -80540,7 +80540,7 @@
         </is>
       </c>
       <c r="E143" t="n">
-        <v>6.589</v>
+        <v>6.375</v>
       </c>
     </row>
     <row r="144">
@@ -80563,7 +80563,7 @@
         </is>
       </c>
       <c r="E144" t="n">
-        <v>5.969</v>
+        <v>5.861</v>
       </c>
     </row>
     <row r="145">
@@ -80586,7 +80586,7 @@
         </is>
       </c>
       <c r="E145" t="n">
-        <v>-1.762</v>
+        <v>-2.181</v>
       </c>
     </row>
     <row r="146">
@@ -80609,7 +80609,7 @@
         </is>
       </c>
       <c r="E146" t="n">
-        <v>-2.245</v>
+        <v>-2.593</v>
       </c>
     </row>
     <row r="147">
@@ -80632,7 +80632,7 @@
         </is>
       </c>
       <c r="E147" t="n">
-        <v>-3.606</v>
+        <v>-3.763</v>
       </c>
     </row>
     <row r="148">
@@ -80655,7 +80655,7 @@
         </is>
       </c>
       <c r="E148" t="n">
-        <v>-6.824</v>
+        <v>-7.028</v>
       </c>
     </row>
     <row r="149">
@@ -80678,7 +80678,7 @@
         </is>
       </c>
       <c r="E149" t="n">
-        <v>-7.316</v>
+        <v>-7.609</v>
       </c>
     </row>
     <row r="150">
@@ -80701,7 +80701,7 @@
         </is>
       </c>
       <c r="E150" t="n">
-        <v>-8.022</v>
+        <v>-8.426</v>
       </c>
     </row>
     <row r="151">
@@ -80724,7 +80724,7 @@
         </is>
       </c>
       <c r="E151" t="n">
-        <v>-11.57</v>
+        <v>-11.526</v>
       </c>
     </row>
   </sheetData>
@@ -81618,16 +81618,16 @@
         <v>3705</v>
       </c>
       <c r="D16" t="n">
-        <v>0.01806</v>
+        <v>0.018</v>
       </c>
       <c r="E16" t="n">
         <v>0.04655</v>
       </c>
       <c r="F16" t="n">
-        <v>-1.025</v>
+        <v>-1.027</v>
       </c>
       <c r="G16" t="n">
-        <v>0.3056</v>
+        <v>0.3045</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -83467,13 +83467,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.1299</v>
+        <v>0.1298</v>
       </c>
       <c r="C16" t="n">
-        <v>0.1176</v>
+        <v>0.1175</v>
       </c>
       <c r="D16" t="n">
-        <v>0.1415</v>
+        <v>0.1414</v>
       </c>
       <c r="E16" t="n">
         <v>1000</v>
@@ -83704,10 +83704,10 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>-0.1937</v>
+        <v>-0.1917</v>
       </c>
       <c r="C16" t="n">
-        <v>1.012</v>
+        <v>1.02</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-30T20:08Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-30 18:14 UTC</t>
+          <t>Genere le 2026-09-30 20:08 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-30 18:14 UTC</t>
+          <t>Rapport global — 2026-09-30 20:08 UTC</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>**Matieres premieres macro** — le ratio cuivre/or monte -- la croissance domine la peur (+5.5% sur 3 mois). Brent 98.3$ (+37.3% sur 3 mois, +46.7% sur 12 mois), gaz -6.5% sur 3 mois, ecart Brent-WTI +7.6$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-30)_</t>
+          <t>**Matieres premieres macro** — le ratio cuivre/or monte -- la croissance domine la peur (+5.5% sur 3 mois). Brent 98.1$ (+37.0% sur 3 mois, +46.3% sur 12 mois), gaz -6.3% sur 3 mois, ecart Brent-WTI +7.6$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -862,7 +862,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>**Conditions financieres** — indice conditions financieres=+0.097 (3 composantes: {'taux_directeur': 0.5971439233898245, 'courbe_inversee': 0.23568763984021313, 'vix': -0.5410491021615241}) -- conditions proches de la normale _(observation : 2026-09-28)_</t>
+          <t>**Conditions financieres** — indice conditions financieres=+0.113 (3 composantes: {'taux_directeur': 0.5971439233898245, 'courbe_inversee': 0.23568763984021313, 'vix': -0.49281910275629404}) -- conditions proches de la normale _(observation : 2026-09-28)_</t>
         </is>
       </c>
     </row>
@@ -988,7 +988,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>**Momentum prix** — SP500 momentum 12-1 mois = 14.92% -- haussier (momentum positif), detail 1/3/6/12m = [0.18, 2.9, 17.1, 15.12] _(observation : 2026-09-30)_</t>
+          <t>**Momentum prix** — SP500 momentum 12-1 mois = 14.92% -- haussier (momentum positif), detail 1/3/6/12m = [-0.44, 2.25, 16.37, 14.41] _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1009,35 +1009,35 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>**Rotation sectorielle** — classement momentum 3 mois (10 secteurs) : 1. Energie (XLE) : +17.45% | 2. Sante (XLV) : +6.38% | 3. Technologie (XLK) : +5.86% | 4. Finance (XLF) : -2.18% | 5. Consommation de base (XLP) : -2.59% _(observation : 2026-09-30)_</t>
+          <t>**Rotation sectorielle** — classement momentum 3 mois (10 secteurs) : 1. Energie (XLE) : +16.45% | 2. Sante (XLV) : +5.56% | 3. Technologie (XLK) : +5.46% | 4. Finance (XLF) : -2.55% | 5. Consommation de base (XLP) : -3.26% _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>**Saisonnalite** — rendement journalier moyen ete=+0.0180%, hiver=+0.0465% (t=-1.03, p=0.3045) -- non significatif (attendu vu la faible puissance sur seulement ~2 ans) _(observation : 2026-09-30)_</t>
+          <t>**Saisonnalite** — rendement journalier moyen ete=+0.0178%, hiver=+0.0465% (t=-1.03, p=0.3008) -- non significatif (attendu vu la faible puissance sur seulement ~2 ans) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>**Dispersion sectorielle** — 10 secteurs, rendement moyen 3m=-1.34%, dispersion (ecart-type)=8.36pt, etendue=28.98pt -- dispersion intermediaire _(observation : 2026-09-30)_</t>
+          <t>**Dispersion sectorielle** — 10 secteurs, rendement moyen 3m=-1.90%, dispersion (ecart-type)=8.20pt, etendue=28.38pt -- dispersion intermediaire _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>**Low volatility** — tercile bas-vol ['XLF', 'XLRE', 'XLU'] Sharpe=-1.047 vs tercile haut-vol ['XLY', 'XLE', 'XLK'] Sharpe=0.094 -- anomalie low-vol non confirmee sur cet echantillon (puissance statistique faible, n petit -- limite assumee) _(observation : 2026-09-30)_</t>
+          <t>**Low volatility** — tercile bas-vol ['XLF', 'XLRE', 'XLU'] Sharpe=-1.125 vs tercile haut-vol ['XLY', 'XLE', 'XLK'] Sharpe=0.037 -- anomalie low-vol non confirmee sur cet echantillon (puissance statistique faible, n petit -- limite assumee) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>**Momentum cross sectional** — panier gagnant ['XLE', 'XLV', 'XLK'] (+9.90%) vs panier perdant ['XLY', 'XLI', 'XLU'] (-9.19%) -- spread momentum=+19.08pt _(observation : 2026-09-30)_</t>
+          <t>**Momentum cross sectional** — panier gagnant ['XLE', 'XLV', 'XLK'] (+9.16%) vs panier perdant ['XLY', 'XLI', 'XLU'] (-9.57%) -- spread momentum=+18.72pt _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>**Correlation facteurs** — correlation entre momentum 3m et beta-VIX, 10 secteurs : +0.271 (facteurs largement independants) _(observation : 2026-09-30)_</t>
+          <t>**Correlation facteurs** — correlation entre momentum 3m et beta-VIX, 10 secteurs : +0.263 (facteurs largement independants) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1107,7 +1107,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>**Divergence cot prix** — SP500 +0.18% sur 30j, COT net -10560 -&gt; -133228 -- DIVERGENCE (prix monte, positionnement recule) _(observation : 2026-09-30)_</t>
+          <t>**Divergence cot prix** — SP500 -0.44% sur 30j, COT net -10560 -&gt; -133228 -- pas de divergence _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1191,35 +1191,35 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>**Vol cross asset** — 6 mesures de volatilite : Or (GVZ) 84e pct, Petrole (OVX) 83e pct, Taux US (MOVE) 62e pct, Nasdaq (VXN) 48e pct, Vol de la vol (VVIX) 30e pct, Actions US (VIX) 30e pct -- stress LOCALISE sur Or (GVZ), Petrole (OVX) pendant que le reste ne l'est pas -- episode propre a cette classe d'actifs, pas une aversion au risque d'ensemble _(observation : 2026-09-30)_</t>
+          <t>**Vol cross asset** — 6 mesures de volatilite : Petrole (OVX) 84e pct, Or (GVZ) 83e pct, Taux US (MOVE) 64e pct, Nasdaq (VXN) 50e pct, Actions US (VIX) 34e pct, Vol de la vol (VVIX) 31e pct -- stress LOCALISE sur Petrole (OVX), Or (GVZ) pendant que le reste ne l'est pas -- episode propre a cette classe d'actifs, pas une aversion au risque d'ensemble _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>**Volatilite ewma** — vol realisee 60j=0.11178654130535158, EWMA=0.1037 (tendance 10 runs: stable) _(observation : 2026-09-30)_</t>
+          <t>**Volatilite ewma** — vol realisee 60j=0.11172032117323961, EWMA=0.1031 (tendance 10 runs: stable) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>**Garch** — vol GARCH(1,1) annualisee=0.1171 (alpha=0.114, beta=0.868, persistance=0.983 -- tres proche de 1 -- chocs de volatilite tres durables) _(observation : 2026-09-30)_</t>
+          <t>**Garch** — vol GARCH(1,1) annualisee=0.1170 (alpha=0.114, beta=0.868, persistance=0.983 -- tres proche de 1 -- chocs de volatilite tres durables) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>**Hurst** — Hurst=0.5507 (R2 regression=1.000) -- persistant (tendanciel) _(observation : 2026-09-30)_</t>
+          <t>**Hurst** — Hurst=0.5517 (R2 regression=1.000) -- persistant (tendanciel) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>**Ornstein uhlenbeck vix** — VIX actuel=15.83, niveau moyen estime (mu)=20.20, demi-vie=28.8j, ecart actuel=-4.37 -- VIX actuel en-dessous de son niveau moyen de long terme _(observation : 2026-09-30)_</t>
+          <t>**Ornstein uhlenbeck vix** — VIX actuel=16.22, niveau moyen estime (mu)=20.20, demi-vie=28.8j, ecart actuel=-3.98 -- VIX actuel en-dessous de son niveau moyen de long terme _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1233,14 +1233,14 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>**Kalman niveau local** — VIX observe=15.83, filtre Kalman=15.86 (ecart-type=0.62), ratio signal/bruit=0.2052 -- le filtre lisse fortement le bruit, reagit lentement (ecart obs.-filtre=-0.03) _(observation : 2026-09-30)_</t>
+          <t>**Kalman niveau local** — VIX observe=16.22, filtre Kalman=16.19 (ecart-type=0.62), ratio signal/bruit=0.2051 -- le filtre lisse fortement le bruit, reagit lentement (ecart obs.-filtre=+0.03) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.3729361339989534 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.05236469052186711 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-30)_</t>
+          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.3658803288447583 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.0523166004347603 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1261,14 +1261,14 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>**Skew kurtosis** — skewness=-0.192 (asymetrie negative (pertes extremes &gt; gains extremes)), kurtosis exces=+1.020 (queues epaisses (risque extreme sous-estime par une hypothese normale)) _(observation : 2026-09-30)_</t>
+          <t>**Skew kurtosis** — skewness=-0.183 (asymetrie negative (pertes extremes &gt; gains extremes)), kurtosis exces=+1.018 (queues epaisses (risque extreme sous-estime par une hypothese normale)) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>**Ratios performance** — Sharpe=1.087 (bon), Sortino=1.073 (bon), Calmar=1.554 (bon) -- lecture sur fenetre 252j (~1 an, echantillon limite), seuils academiques standards, taux sans risque suppose nul _(observation : 2026-09-30)_</t>
+          <t>**Ratios performance** — Sharpe=1.039 (bon), Sortino=1.030 (bon), Calmar=1.485 (bon) -- lecture sur fenetre 252j (~1 an, echantillon limite), seuils academiques standards, taux sans risque suppose nul _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1282,7 +1282,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>**Stress test historique** — COVID_2020 (2020-02-19 -&gt; 2020-03-23) : chute historique=-33.9% -- rejouee sur le niveau actuel (7700) -&gt; 5088  _(sans synthese)_ _(observation : 2026-09-30)_</t>
+          <t>**Stress test historique** — COVID_2020 (2020-02-19 -&gt; 2020-03-23) : chute historique=-33.9% -- rejouee sur le niveau actuel (7652) -&gt; 5056  _(sans synthese)_ _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1303,7 +1303,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>**Detection saut** — Z-stat BNS (fenetre 22j)=1.057 (seuil ±1.96) -- pas de saut isole detecte _(observation : 2026-09-30)_</t>
+          <t>**Detection saut** — Z-stat BNS (fenetre 22j)=1.026 (seuil ±1.96) -- pas de saut isole detecte _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1331,14 +1331,14 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>**Decomposition stl** — VIX : tendance=15.54, composante saisonniere (periode 5j)=+0.325, residu=-0.037 -- la saisonnalite explique 0.68% de la variance totale (negligeable) _(observation : 2026-09-30)_</t>
+          <t>**Decomposition stl** — VIX : tendance=15.61, composante saisonniere (periode 5j)=+0.469, residu=+0.146 -- la saisonnalite explique 0.72% de la variance totale (negligeable) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>**Ratios conditionnels regime** — Sharpe regime haut-vol=-1.107, bas-vol=2.402, global=0.421 -- meilleur en regime calme, comme attendu _(observation : 2026-09-30)_</t>
+          <t>**Ratios conditionnels regime** — Sharpe regime haut-vol=-1.107, bas-vol=2.398, global=0.420 -- meilleur en regime calme, comme attendu _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1373,35 +1373,35 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>**Dependance queue** — 518/7547 jours conjointement extremes (SP500 pire 10% ET VIX pire 10%), P observee=0.0686 vs P sous independance=0.0100 -- coefficient de dependance de queue=6.86 (dependance reelle) _(observation : 2026-09-30)_</t>
+          <t>**Dependance queue** — 518/7546 jours conjointement extremes (SP500 pire 10% ET VIX pire 10%), P observee=0.0686 vs P sous independance=0.0100 -- coefficient de dependance de queue=6.86 (dependance reelle) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>**Walkforward direction** — 7517 predictions walk-forward -- momentum 5j=0.4958 vs baseline majoritaire=0.5373 -- NE BAT PAS la baseline (resultat honnete, pas ajuste pour paraitre mieux) _(observation : 2026-09-30)_</t>
+          <t>**Walkforward direction** — 7516 predictions walk-forward -- momentum 5j=0.4960 vs baseline majoritaire=0.5371 -- NE BAT PAS la baseline (resultat honnete, pas ajuste pour paraitre mieux) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>**Anomalie multivariee** — distance de Mahalanobis=0.512 (seuil 3.0) -- jour ordinaire _(observation : 2026-09-30)_</t>
+          <t>**Anomalie multivariee** — distance de Mahalanobis=0.495 (seuil 3.0) -- jour ordinaire _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>**Test overfitting** — meilleure fenetre in-sample=23j (accuracy=0.5162) vs meme fenetre en walk-forward=0.5159 -- ecart=+0.0003 (ecart faible) _(observation : 2026-09-30)_</t>
+          <t>**Test overfitting** — meilleure fenetre in-sample=23j (accuracy=0.5164) vs meme fenetre en walk-forward=0.5161 -- ecart=+0.0003 (ecart faible) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>**Prevision vol regression** — regression AR(1) (a=0.000116, b=0.2096) MSE=2.9835e-07 vs baseline persistance MSE=3.8327e-07 -- BAT la baseline (resultat honnete, pas ajuste) _(observation : 2026-09-30)_</t>
+          <t>**Prevision vol regression** — regression AR(1) (a=0.000116, b=0.2096) MSE=2.9848e-07 vs baseline persistance MSE=3.8344e-07 -- BAT la baseline (resultat honnete, pas ajuste) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1415,7 +1415,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>**Ensemble signaux** — 7517 predictions -- momentum=0.4958, vix=0.4989, ensemble=0.4989, baseline=0.5373 -- ensemble NE BAT PAS la baseline _(observation : 2026-09-30)_</t>
+          <t>**Ensemble signaux** — 7516 predictions -- momentum=0.4960, vix=0.4988, ensemble=0.4988, baseline=0.5371 -- ensemble NE BAT PAS la baseline _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>**Couts transaction** — 7517 predictions, 1513 changements de position (5pb/changement) -- rendement cumule brut=-93.22%, cout total=53.08%, net=-96.82% -- les frais mangent une part importante du rendement (&gt;50% du brut) _(observation : 2026-09-30)_</t>
+          <t>**Couts transaction** — 7516 predictions, 1513 changements de position (5pb/changement) -- rendement cumule brut=-93.15%, cout total=53.08%, net=-96.79% -- les frais mangent une part importante du rendement (&gt;50% du brut) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1464,21 +1464,21 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>**Stacking** — poids appris (momentum=-0.082, baseline=0.090, biais=0.090) -- accuracy stacking=0.5461 vs momentum seul=0.5022, baseline seule=0.5461 sur 2256 points test -- stacking NE BAT PAS la baseline, meilleur=stacking / baseline (ex-aequo) _(observation : 2026-09-30)_</t>
+          <t>**Stacking** — poids appris (momentum=-0.081, baseline=0.087, biais=0.092) -- accuracy stacking=0.5459 vs momentum seul=0.5029, baseline seule=0.5459 sur 2255 points test -- stacking NE BAT PAS la baseline, meilleur=stacking / baseline (ex-aequo) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>**Decision stump** — seuil appris=-1.530 (sens=False) -- accuracy stump=0.5455 vs baseline=0.5473 sur 2264 points test -- stump NE BAT PAS la baseline _(observation : 2026-09-30)_</t>
+          <t>**Decision stump** — seuil appris=-1.530 (sens=False) -- accuracy stump=0.5451 vs baseline=0.5468 sur 2264 points test -- stump NE BAT PAS la baseline _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>**Importance permutation** — R2 base=0.0103 -- importance momentum5j=0.00242, importance variation_vix=0.00883 -- VIX plus important _(observation : 2026-09-30)_</t>
+          <t>**Importance permutation** — R2 base=0.0103 -- importance momentum5j=0.00240, importance variation_vix=0.00888 -- VIX plus important _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -3171,25 +3171,25 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>-0.08160000000000001</v>
+        <v>-0.08119999999999999</v>
       </c>
       <c r="C16" t="n">
-        <v>0.08989999999999999</v>
+        <v>0.08740000000000001</v>
       </c>
       <c r="D16" t="n">
-        <v>0.08989999999999999</v>
+        <v>0.092</v>
       </c>
       <c r="E16" t="n">
-        <v>2256</v>
+        <v>2255</v>
       </c>
       <c r="F16" t="n">
-        <v>0.5461</v>
+        <v>0.5459000000000001</v>
       </c>
       <c r="G16" t="n">
-        <v>0.5022</v>
+        <v>0.5029</v>
       </c>
       <c r="H16" t="n">
-        <v>0.5461</v>
+        <v>0.5459000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -6069,7 +6069,7 @@
         <v>-56.78</v>
       </c>
       <c r="F30" t="n">
-        <v>3328.24</v>
+        <v>3307.52</v>
       </c>
     </row>
     <row r="31">
@@ -6097,7 +6097,7 @@
         <v>-33.92</v>
       </c>
       <c r="F31" t="n">
-        <v>5087.69</v>
+        <v>5056.02</v>
       </c>
     </row>
   </sheetData>
@@ -7134,10 +7134,10 @@
         <v>23</v>
       </c>
       <c r="C16" t="n">
-        <v>0.5162</v>
+        <v>0.5164</v>
       </c>
       <c r="D16" t="n">
-        <v>0.5159</v>
+        <v>0.5161</v>
       </c>
       <c r="E16" t="n">
         <v>0.0003</v>
@@ -7757,10 +7757,10 @@
         <v>5</v>
       </c>
       <c r="C16" t="n">
-        <v>0.0756</v>
+        <v>0.07518</v>
       </c>
       <c r="D16" t="n">
-        <v>0.00415</v>
+        <v>0.00418</v>
       </c>
     </row>
   </sheetData>
@@ -8456,7 +8456,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>32.6</v>
+        <v>32.7</v>
       </c>
       <c r="D16" t="n">
         <v>-2.847</v>
@@ -9131,10 +9131,10 @@
         <v>10</v>
       </c>
       <c r="C16" t="n">
-        <v>0.37294</v>
+        <v>0.36588</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.052365</v>
+        <v>-0.052317</v>
       </c>
     </row>
   </sheetData>
@@ -9194,7 +9194,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Or (GVZ)</t>
+          <t>Petrole (OVX)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -9203,10 +9203,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>24.01</v>
+        <v>52.58</v>
       </c>
       <c r="D2" t="n">
-        <v>83.8</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="E2" t="n">
         <v>1260</v>
@@ -9220,7 +9220,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Petrole (OVX)</t>
+          <t>Or (GVZ)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -9229,10 +9229,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>51.98</v>
+        <v>23.84</v>
       </c>
       <c r="D3" t="n">
-        <v>82.7</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="E3" t="n">
         <v>1260</v>
@@ -9255,10 +9255,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>109.19</v>
+        <v>110.49</v>
       </c>
       <c r="D4" t="n">
-        <v>61.7</v>
+        <v>63.7</v>
       </c>
       <c r="E4" t="n">
         <v>1260</v>
@@ -9281,10 +9281,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>22.16</v>
+        <v>22.4</v>
       </c>
       <c r="D5" t="n">
-        <v>48.2</v>
+        <v>49.8</v>
       </c>
       <c r="E5" t="n">
         <v>1260</v>
@@ -9298,7 +9298,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Vol de la vol (VVIX)</t>
+          <t>Actions US (VIX)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -9307,10 +9307,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>88.72</v>
+        <v>16.22</v>
       </c>
       <c r="D6" t="n">
-        <v>30.3</v>
+        <v>34.1</v>
       </c>
       <c r="E6" t="n">
         <v>1260</v>
@@ -9324,7 +9324,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Actions US (VIX)</t>
+          <t>Vol de la vol (VVIX)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -9333,10 +9333,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>15.83</v>
+        <v>88.88</v>
       </c>
       <c r="D7" t="n">
-        <v>29.7</v>
+        <v>31</v>
       </c>
       <c r="E7" t="n">
         <v>1260</v>
@@ -9668,16 +9668,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.1037</v>
+        <v>0.1031</v>
       </c>
       <c r="C16" t="n">
-        <v>0.0805</v>
+        <v>0.0731</v>
       </c>
       <c r="D16" t="n">
-        <v>0.1082</v>
+        <v>0.1079</v>
       </c>
       <c r="E16" t="n">
-        <v>0.1118</v>
+        <v>0.1117</v>
       </c>
     </row>
   </sheetData>
@@ -10029,13 +10029,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>7517</v>
+        <v>7516</v>
       </c>
       <c r="C16" t="n">
-        <v>0.4958</v>
+        <v>0.496</v>
       </c>
       <c r="D16" t="n">
-        <v>0.5373</v>
+        <v>0.5371</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -12687,16 +12687,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>12.981</v>
+        <v>12.98</v>
       </c>
       <c r="C16" t="n">
-        <v>-1.288</v>
+        <v>-1.29</v>
       </c>
       <c r="D16" t="n">
-        <v>-2.633</v>
+        <v>-2.635</v>
       </c>
       <c r="E16" t="n">
-        <v>-3.978</v>
+        <v>-3.98</v>
       </c>
     </row>
   </sheetData>
@@ -17802,10 +17802,10 @@
         </is>
       </c>
       <c r="C142" t="n">
-        <v>-2.4626</v>
+        <v>-2.373</v>
       </c>
       <c r="D142" t="n">
-        <v>0.2958</v>
+        <v>0.3377</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -17825,10 +17825,10 @@
         </is>
       </c>
       <c r="C143" t="n">
-        <v>-1.7131</v>
+        <v>-1.7321</v>
       </c>
       <c r="D143" t="n">
-        <v>0.6709000000000001</v>
+        <v>0.6621</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -17848,10 +17848,10 @@
         </is>
       </c>
       <c r="C144" t="n">
-        <v>-2.1465</v>
+        <v>-2.2349</v>
       </c>
       <c r="D144" t="n">
-        <v>0.4521</v>
+        <v>0.4065</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -17871,10 +17871,10 @@
         </is>
       </c>
       <c r="C145" t="n">
-        <v>-2.3904</v>
+        <v>-2.4302</v>
       </c>
       <c r="D145" t="n">
-        <v>0.3294</v>
+        <v>0.3107</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -17894,10 +17894,10 @@
         </is>
       </c>
       <c r="C146" t="n">
-        <v>-1.2267</v>
+        <v>-1.285</v>
       </c>
       <c r="D146" t="n">
-        <v>0.8508</v>
+        <v>0.8342000000000001</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -17917,10 +17917,10 @@
         </is>
       </c>
       <c r="C147" t="n">
-        <v>0.1087</v>
+        <v>0.0406</v>
       </c>
       <c r="D147" t="n">
-        <v>0.9881</v>
+        <v>0.9868</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -17940,10 +17940,10 @@
         </is>
       </c>
       <c r="C148" t="n">
-        <v>-1.0933</v>
+        <v>-1.0663</v>
       </c>
       <c r="D148" t="n">
-        <v>0.8837</v>
+        <v>0.8895</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -17963,10 +17963,10 @@
         </is>
       </c>
       <c r="C149" t="n">
-        <v>-0.6028</v>
+        <v>-0.6891</v>
       </c>
       <c r="D149" t="n">
-        <v>0.9562</v>
+        <v>0.9478</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -17986,10 +17986,10 @@
         </is>
       </c>
       <c r="C150" t="n">
-        <v>-2.0927</v>
+        <v>-2.0399</v>
       </c>
       <c r="D150" t="n">
-        <v>0.4802</v>
+        <v>0.5078</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -18009,10 +18009,10 @@
         </is>
       </c>
       <c r="C151" t="n">
-        <v>-1.4984</v>
+        <v>-1.5365</v>
       </c>
       <c r="D151" t="n">
-        <v>0.7618</v>
+        <v>0.7469</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -25142,7 +25142,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.0973</v>
+        <v>0.1133</v>
       </c>
       <c r="C15" t="n">
         <v>3</v>
@@ -25154,7 +25154,7 @@
         <v>0.2357</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.541</v>
+        <v>-0.4928</v>
       </c>
     </row>
   </sheetData>
@@ -25455,7 +25455,7 @@
         <v>10</v>
       </c>
       <c r="C16" t="n">
-        <v>0.2711</v>
+        <v>0.2626</v>
       </c>
     </row>
   </sheetData>
@@ -37805,7 +37805,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>7517</v>
+        <v>7516</v>
       </c>
       <c r="C16" t="n">
         <v>1513</v>
@@ -37814,10 +37814,10 @@
         <v>53.08</v>
       </c>
       <c r="E16" t="n">
-        <v>-93.22</v>
+        <v>-93.15000000000001</v>
       </c>
       <c r="F16" t="n">
-        <v>-96.81999999999999</v>
+        <v>-96.79000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -38215,19 +38215,19 @@
         <v>2.2</v>
       </c>
       <c r="C15" t="n">
-        <v>413.44</v>
+        <v>413.94</v>
       </c>
       <c r="D15" t="n">
         <v>4</v>
       </c>
       <c r="E15" t="n">
-        <v>372.92</v>
+        <v>373.71</v>
       </c>
       <c r="F15" t="n">
         <v>5.3</v>
       </c>
       <c r="G15" t="n">
-        <v>323.99</v>
+        <v>323.76</v>
       </c>
     </row>
   </sheetData>
@@ -39433,10 +39433,10 @@
         <v>2264</v>
       </c>
       <c r="E16" t="n">
-        <v>0.5455</v>
+        <v>0.5451</v>
       </c>
       <c r="F16" t="n">
-        <v>0.5473</v>
+        <v>0.5468</v>
       </c>
     </row>
   </sheetData>
@@ -39741,16 +39741,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>15.542</v>
+        <v>15.606</v>
       </c>
       <c r="C15" t="n">
-        <v>0.325</v>
+        <v>0.469</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.037</v>
+        <v>0.146</v>
       </c>
       <c r="E15" t="n">
-        <v>0.68</v>
+        <v>0.72</v>
       </c>
     </row>
   </sheetData>
@@ -40340,13 +40340,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>7547</v>
+        <v>7546</v>
       </c>
       <c r="C16" t="n">
         <v>518</v>
       </c>
       <c r="D16" t="n">
-        <v>0.06864000000000001</v>
+        <v>0.06865</v>
       </c>
       <c r="E16" t="n">
         <v>0.01</v>
@@ -40656,7 +40656,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1.057</v>
+        <v>1.026</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -41308,13 +41308,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.00378</v>
+        <v>-0.00247</v>
       </c>
       <c r="C16" t="n">
-        <v>-0.21</v>
+        <v>0.18</v>
       </c>
       <c r="D16" t="n">
-        <v>0.512</v>
+        <v>0.495</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -41646,13 +41646,13 @@
         <v>10</v>
       </c>
       <c r="C16" t="n">
-        <v>-1.344</v>
+        <v>-1.901</v>
       </c>
       <c r="D16" t="n">
-        <v>8.356</v>
+        <v>8.196</v>
       </c>
       <c r="E16" t="n">
-        <v>28.977</v>
+        <v>28.383</v>
       </c>
     </row>
   </sheetData>
@@ -42004,7 +42004,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.179</v>
+        <v>-0.445</v>
       </c>
       <c r="C16" t="n">
         <v>-133228</v>
@@ -42014,7 +42014,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
@@ -43112,19 +43112,19 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>7517</v>
+        <v>7516</v>
       </c>
       <c r="C16" t="n">
-        <v>0.4958</v>
+        <v>0.496</v>
       </c>
       <c r="D16" t="n">
-        <v>0.4989</v>
+        <v>0.4988</v>
       </c>
       <c r="E16" t="n">
-        <v>0.4989</v>
+        <v>0.4988</v>
       </c>
       <c r="F16" t="n">
-        <v>0.5373</v>
+        <v>0.5371</v>
       </c>
     </row>
   </sheetData>
@@ -52647,16 +52647,16 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>tresor_us/solde_tresorerie.csv</t>
+          <t>fred/BAMLC0A0CM.csv</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C207" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D207" t="n">
         <v>1</v>
@@ -52665,7 +52665,7 @@
         <v>42</v>
       </c>
       <c r="F207" t="n">
-        <v>500</v>
+        <v>793</v>
       </c>
       <c r="G207" t="inlineStr">
         <is>
@@ -52676,7 +52676,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>fred/BAMLC0A0CM.csv</t>
+          <t>fred/BAMLC0A0CMEY.csv</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -52705,7 +52705,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>fred/BAMLC0A0CMEY.csv</t>
+          <t>fred/BAMLEMCBPIOAS.csv</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -52734,7 +52734,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>fred/BAMLEMCBPIOAS.csv</t>
+          <t>fred/BAMLEMFSFCRPIOAS.csv</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -52763,7 +52763,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>fred/BAMLEMFSFCRPIOAS.csv</t>
+          <t>fred/BAMLEMHBHYCRPIOAS.csv</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
@@ -52792,7 +52792,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>fred/BAMLEMHBHYCRPIOAS.csv</t>
+          <t>fred/BAMLEMPBPUBSICRPIOAS.csv</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -52821,7 +52821,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>fred/BAMLEMPBPUBSICRPIOAS.csv</t>
+          <t>fred/BAMLH0A0HYM2.csv</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -52850,7 +52850,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>fred/BAMLH0A0HYM2.csv</t>
+          <t>fred/BAMLHE00EHYIEY.csv</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -52879,7 +52879,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>fred/BAMLHE00EHYIEY.csv</t>
+          <t>fred/BAMLHE00EHYIOAS.csv</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -52908,7 +52908,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>fred/BAMLHE00EHYIOAS.csv</t>
+          <t>fred/T10YIE.csv</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -52926,7 +52926,7 @@
         <v>42</v>
       </c>
       <c r="F216" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G216" t="inlineStr">
         <is>
@@ -52937,7 +52937,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>fred/T10YIE.csv</t>
+          <t>marches/indices/HANGSENG.csv</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -52955,7 +52955,7 @@
         <v>42</v>
       </c>
       <c r="F217" t="n">
-        <v>3000</v>
+        <v>3689</v>
       </c>
       <c r="G217" t="inlineStr">
         <is>
@@ -52966,7 +52966,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>marches/indices/HANGSENG.csv</t>
+          <t>marches/indices/KOSPI.csv</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -52984,7 +52984,7 @@
         <v>42</v>
       </c>
       <c r="F218" t="n">
-        <v>3689</v>
+        <v>3680</v>
       </c>
       <c r="G218" t="inlineStr">
         <is>
@@ -52995,7 +52995,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>marches/indices/KOSPI.csv</t>
+          <t>marches/indices/NIKKEI225.csv</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -53013,7 +53013,7 @@
         <v>42</v>
       </c>
       <c r="F219" t="n">
-        <v>3680</v>
+        <v>3666</v>
       </c>
       <c r="G219" t="inlineStr">
         <is>
@@ -53024,7 +53024,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>marches/indices/NIKKEI225.csv</t>
+          <t>souverains/SUEDE_10A.csv</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -53042,7 +53042,7 @@
         <v>42</v>
       </c>
       <c r="F220" t="n">
-        <v>3666</v>
+        <v>9204</v>
       </c>
       <c r="G220" t="inlineStr">
         <is>
@@ -53053,7 +53053,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_10A.csv</t>
+          <t>souverains/SUEDE_2A.csv</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -53082,7 +53082,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_2A.csv</t>
+          <t>souverains/SUEDE_5A.csv</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -53100,7 +53100,7 @@
         <v>42</v>
       </c>
       <c r="F222" t="n">
-        <v>9204</v>
+        <v>9206</v>
       </c>
       <c r="G222" t="inlineStr">
         <is>
@@ -53111,7 +53111,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_5A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -53129,7 +53129,7 @@
         <v>42</v>
       </c>
       <c r="F223" t="n">
-        <v>9206</v>
+        <v>5641</v>
       </c>
       <c r="G223" t="inlineStr">
         <is>
@@ -53140,7 +53140,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -53169,7 +53169,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
@@ -53198,7 +53198,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -53227,7 +53227,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -53256,7 +53256,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -53285,7 +53285,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -53314,7 +53314,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -53343,7 +53343,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
+          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -53372,7 +53372,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
+          <t>tresor_us/solde_tresorerie.csv</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -53390,7 +53390,7 @@
         <v>42</v>
       </c>
       <c r="F232" t="n">
-        <v>5641</v>
+        <v>500</v>
       </c>
       <c r="G232" t="inlineStr">
         <is>
@@ -53477,7 +53477,7 @@
         <v>42</v>
       </c>
       <c r="F235" t="n">
-        <v>3908</v>
+        <v>3909</v>
       </c>
       <c r="G235" t="inlineStr">
         <is>
@@ -53506,7 +53506,7 @@
         <v>42</v>
       </c>
       <c r="F236" t="n">
-        <v>3904</v>
+        <v>3905</v>
       </c>
       <c r="G236" t="inlineStr">
         <is>
@@ -53564,7 +53564,7 @@
         <v>42</v>
       </c>
       <c r="F238" t="n">
-        <v>3905</v>
+        <v>3906</v>
       </c>
       <c r="G238" t="inlineStr">
         <is>
@@ -53593,7 +53593,7 @@
         <v>42</v>
       </c>
       <c r="F239" t="n">
-        <v>3907</v>
+        <v>3908</v>
       </c>
       <c r="G239" t="inlineStr">
         <is>
@@ -53622,7 +53622,7 @@
         <v>42</v>
       </c>
       <c r="F240" t="n">
-        <v>3907</v>
+        <v>3908</v>
       </c>
       <c r="G240" t="inlineStr">
         <is>
@@ -53651,7 +53651,7 @@
         <v>42</v>
       </c>
       <c r="F241" t="n">
-        <v>3904</v>
+        <v>3905</v>
       </c>
       <c r="G241" t="inlineStr">
         <is>
@@ -53680,7 +53680,7 @@
         <v>42</v>
       </c>
       <c r="F242" t="n">
-        <v>3905</v>
+        <v>3906</v>
       </c>
       <c r="G242" t="inlineStr">
         <is>
@@ -53709,7 +53709,7 @@
         <v>42</v>
       </c>
       <c r="F243" t="n">
-        <v>3905</v>
+        <v>3906</v>
       </c>
       <c r="G243" t="inlineStr">
         <is>
@@ -53738,7 +53738,7 @@
         <v>42</v>
       </c>
       <c r="F244" t="n">
-        <v>3904</v>
+        <v>3905</v>
       </c>
       <c r="G244" t="inlineStr">
         <is>
@@ -53767,7 +53767,7 @@
         <v>42</v>
       </c>
       <c r="F245" t="n">
-        <v>3902</v>
+        <v>3903</v>
       </c>
       <c r="G245" t="inlineStr">
         <is>
@@ -53796,7 +53796,7 @@
         <v>42</v>
       </c>
       <c r="F246" t="n">
-        <v>3904</v>
+        <v>3905</v>
       </c>
       <c r="G246" t="inlineStr">
         <is>
@@ -53825,7 +53825,7 @@
         <v>42</v>
       </c>
       <c r="F247" t="n">
-        <v>3905</v>
+        <v>3906</v>
       </c>
       <c r="G247" t="inlineStr">
         <is>
@@ -53854,7 +53854,7 @@
         <v>42</v>
       </c>
       <c r="F248" t="n">
-        <v>3904</v>
+        <v>3905</v>
       </c>
       <c r="G248" t="inlineStr">
         <is>
@@ -53883,7 +53883,7 @@
         <v>42</v>
       </c>
       <c r="F249" t="n">
-        <v>3905</v>
+        <v>3906</v>
       </c>
       <c r="G249" t="inlineStr">
         <is>
@@ -53912,7 +53912,7 @@
         <v>42</v>
       </c>
       <c r="F250" t="n">
-        <v>3905</v>
+        <v>3906</v>
       </c>
       <c r="G250" t="inlineStr">
         <is>
@@ -54202,7 +54202,7 @@
         <v>42</v>
       </c>
       <c r="F260" t="n">
-        <v>3771</v>
+        <v>3770</v>
       </c>
       <c r="G260" t="inlineStr">
         <is>
@@ -54231,7 +54231,7 @@
         <v>42</v>
       </c>
       <c r="F261" t="n">
-        <v>3690</v>
+        <v>3689</v>
       </c>
       <c r="G261" t="inlineStr">
         <is>
@@ -54260,7 +54260,7 @@
         <v>42</v>
       </c>
       <c r="F262" t="n">
-        <v>3771</v>
+        <v>3770</v>
       </c>
       <c r="G262" t="inlineStr">
         <is>
@@ -54289,7 +54289,7 @@
         <v>42</v>
       </c>
       <c r="F263" t="n">
-        <v>3763</v>
+        <v>3762</v>
       </c>
       <c r="G263" t="inlineStr">
         <is>
@@ -54318,7 +54318,7 @@
         <v>42</v>
       </c>
       <c r="F264" t="n">
-        <v>3771</v>
+        <v>3770</v>
       </c>
       <c r="G264" t="inlineStr">
         <is>
@@ -54347,7 +54347,7 @@
         <v>42</v>
       </c>
       <c r="F265" t="n">
-        <v>7548</v>
+        <v>7547</v>
       </c>
       <c r="G265" t="inlineStr">
         <is>
@@ -54405,7 +54405,7 @@
         <v>42</v>
       </c>
       <c r="F267" t="n">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="G267" t="inlineStr">
         <is>
@@ -54434,7 +54434,7 @@
         <v>42</v>
       </c>
       <c r="F268" t="n">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="G268" t="inlineStr">
         <is>
@@ -54463,7 +54463,7 @@
         <v>42</v>
       </c>
       <c r="F269" t="n">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="G269" t="inlineStr">
         <is>
@@ -54492,7 +54492,7 @@
         <v>42</v>
       </c>
       <c r="F270" t="n">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="G270" t="inlineStr">
         <is>
@@ -54521,7 +54521,7 @@
         <v>42</v>
       </c>
       <c r="F271" t="n">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="G271" t="inlineStr">
         <is>
@@ -54550,7 +54550,7 @@
         <v>42</v>
       </c>
       <c r="F272" t="n">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="G272" t="inlineStr">
         <is>
@@ -54579,7 +54579,7 @@
         <v>42</v>
       </c>
       <c r="F273" t="n">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="G273" t="inlineStr">
         <is>
@@ -54608,7 +54608,7 @@
         <v>42</v>
       </c>
       <c r="F274" t="n">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="G274" t="inlineStr">
         <is>
@@ -54637,7 +54637,7 @@
         <v>42</v>
       </c>
       <c r="F275" t="n">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="G275" t="inlineStr">
         <is>
@@ -54666,7 +54666,7 @@
         <v>42</v>
       </c>
       <c r="F276" t="n">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="G276" t="inlineStr">
         <is>
@@ -55389,13 +55389,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.1171</v>
+        <v>0.117</v>
       </c>
       <c r="C16" t="n">
         <v>0.1141</v>
       </c>
       <c r="D16" t="n">
-        <v>0.8685</v>
+        <v>0.8683999999999999</v>
       </c>
       <c r="E16" t="n">
         <v>0.9826</v>
@@ -55968,10 +55968,10 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.5507</v>
+        <v>0.5517</v>
       </c>
       <c r="C16" t="n">
-        <v>0.9996</v>
+        <v>0.9995000000000001</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -56252,13 +56252,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.01027</v>
+        <v>0.01028</v>
       </c>
       <c r="C16" t="n">
-        <v>0.00242</v>
+        <v>0.0024</v>
       </c>
       <c r="D16" t="n">
-        <v>0.008829999999999999</v>
+        <v>0.008880000000000001</v>
       </c>
     </row>
   </sheetData>
@@ -56363,13 +56363,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>7699.87</v>
+        <v>7651.94</v>
       </c>
       <c r="D4" t="n">
-        <v>2.9</v>
+        <v>2.25</v>
       </c>
       <c r="E4" t="n">
-        <v>15.12</v>
+        <v>14.41</v>
       </c>
     </row>
     <row r="5">
@@ -57167,16 +57167,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>15.83</v>
+        <v>16.219999</v>
       </c>
       <c r="C15" t="n">
-        <v>15.858</v>
+        <v>16.19</v>
       </c>
       <c r="D15" t="n">
         <v>0.624</v>
       </c>
       <c r="E15" t="n">
-        <v>0.20516</v>
+        <v>0.20515</v>
       </c>
     </row>
   </sheetData>
@@ -58374,7 +58374,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>-1.047</v>
+        <v>-1.125</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -58382,7 +58382,7 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>0.094</v>
+        <v>0.037</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -58774,22 +58774,22 @@
         <v>0.001582</v>
       </c>
       <c r="C13" t="n">
-        <v>5.47</v>
+        <v>5.48</v>
       </c>
       <c r="D13" t="n">
-        <v>98.29000000000001</v>
+        <v>98.08</v>
       </c>
       <c r="E13" t="n">
-        <v>37.33</v>
+        <v>37.04</v>
       </c>
       <c r="F13" t="n">
-        <v>46.66</v>
+        <v>46.34</v>
       </c>
       <c r="G13" t="n">
-        <v>-6.49</v>
+        <v>-6.34</v>
       </c>
       <c r="H13" t="n">
-        <v>7.61</v>
+        <v>7.58</v>
       </c>
     </row>
   </sheetData>
@@ -59679,7 +59679,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>9.896000000000001</v>
+        <v>9.157</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -59687,10 +59687,10 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>-9.186999999999999</v>
+        <v>-9.566000000000001</v>
       </c>
       <c r="F16" t="n">
-        <v>19.082</v>
+        <v>18.723</v>
       </c>
     </row>
   </sheetData>
@@ -62659,16 +62659,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.179</v>
+        <v>-0.445</v>
       </c>
       <c r="C16" t="n">
-        <v>2.895</v>
+        <v>2.255</v>
       </c>
       <c r="D16" t="n">
-        <v>17.103</v>
+        <v>16.374</v>
       </c>
       <c r="E16" t="n">
-        <v>15.122</v>
+        <v>14.405</v>
       </c>
       <c r="F16" t="n">
         <v>14.916</v>
@@ -63511,10 +63511,10 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>15.83</v>
+        <v>16.219999</v>
       </c>
       <c r="C15" t="n">
-        <v>20.199</v>
+        <v>20.201</v>
       </c>
       <c r="D15" t="n">
         <v>0.02404</v>
@@ -63523,7 +63523,7 @@
         <v>28.8</v>
       </c>
       <c r="F15" t="n">
-        <v>-4.369</v>
+        <v>-3.981</v>
       </c>
     </row>
   </sheetData>
@@ -68807,7 +68807,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>-0.004854</v>
+        <v>-0.004852</v>
       </c>
     </row>
   </sheetData>
@@ -69703,19 +69703,19 @@
         <v>5282</v>
       </c>
       <c r="C16" t="n">
-        <v>2265</v>
+        <v>2264</v>
       </c>
       <c r="D16" t="n">
-        <v>0.00011626</v>
+        <v>0.00011625</v>
       </c>
       <c r="E16" t="n">
-        <v>0.20964</v>
+        <v>0.20965</v>
       </c>
       <c r="F16" t="n">
-        <v>2.984e-07</v>
+        <v>2.985e-07</v>
       </c>
       <c r="G16" t="n">
-        <v>3.833e-07</v>
+        <v>3.834e-07</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -69983,10 +69983,10 @@
         <v>0.00877</v>
       </c>
       <c r="C15" t="n">
-        <v>0.06764000000000001</v>
+        <v>0.06759999999999999</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.0382</v>
+        <v>-0.03819</v>
       </c>
     </row>
   </sheetData>
@@ -73205,10 +73205,10 @@
         <v>-1.107</v>
       </c>
       <c r="C16" t="n">
-        <v>2.402</v>
+        <v>2.398</v>
       </c>
       <c r="D16" t="n">
-        <v>0.421</v>
+        <v>0.42</v>
       </c>
     </row>
   </sheetData>
@@ -73484,13 +73484,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1.0874</v>
+        <v>1.0392</v>
       </c>
       <c r="C16" t="n">
-        <v>1.0733</v>
+        <v>1.0297</v>
       </c>
       <c r="D16" t="n">
-        <v>1.5541</v>
+        <v>1.4851</v>
       </c>
     </row>
   </sheetData>
@@ -76827,19 +76827,19 @@
         <v>0.000291</v>
       </c>
       <c r="C16" t="n">
-        <v>-0.032603</v>
+        <v>-0.032576</v>
       </c>
       <c r="D16" t="n">
         <v>0.000269</v>
       </c>
       <c r="E16" t="n">
-        <v>5279</v>
+        <v>5278</v>
       </c>
       <c r="F16" t="n">
         <v>2263</v>
       </c>
       <c r="G16" t="n">
-        <v>0.01027</v>
+        <v>0.01028</v>
       </c>
     </row>
   </sheetData>
@@ -80517,7 +80517,7 @@
         </is>
       </c>
       <c r="E142" t="n">
-        <v>17.451</v>
+        <v>16.455</v>
       </c>
     </row>
     <row r="143">
@@ -80540,7 +80540,7 @@
         </is>
       </c>
       <c r="E143" t="n">
-        <v>6.375</v>
+        <v>5.56</v>
       </c>
     </row>
     <row r="144">
@@ -80563,7 +80563,7 @@
         </is>
       </c>
       <c r="E144" t="n">
-        <v>5.861</v>
+        <v>5.457</v>
       </c>
     </row>
     <row r="145">
@@ -80586,7 +80586,7 @@
         </is>
       </c>
       <c r="E145" t="n">
-        <v>-2.181</v>
+        <v>-2.552</v>
       </c>
     </row>
     <row r="146">
@@ -80609,7 +80609,7 @@
         </is>
       </c>
       <c r="E146" t="n">
-        <v>-2.593</v>
+        <v>-3.263</v>
       </c>
     </row>
     <row r="147">
@@ -80632,7 +80632,7 @@
         </is>
       </c>
       <c r="E147" t="n">
-        <v>-3.763</v>
+        <v>-4.567</v>
       </c>
     </row>
     <row r="148">
@@ -80655,7 +80655,7 @@
         </is>
       </c>
       <c r="E148" t="n">
-        <v>-7.028</v>
+        <v>-7.404</v>
       </c>
     </row>
     <row r="149">
@@ -80678,7 +80678,7 @@
         </is>
       </c>
       <c r="E149" t="n">
-        <v>-7.609</v>
+        <v>-7.82</v>
       </c>
     </row>
     <row r="150">
@@ -80701,7 +80701,7 @@
         </is>
       </c>
       <c r="E150" t="n">
-        <v>-8.426</v>
+        <v>-8.949999999999999</v>
       </c>
     </row>
     <row r="151">
@@ -80724,7 +80724,7 @@
         </is>
       </c>
       <c r="E151" t="n">
-        <v>-11.526</v>
+        <v>-11.928</v>
       </c>
     </row>
   </sheetData>
@@ -81612,22 +81612,22 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>3842</v>
+        <v>3841</v>
       </c>
       <c r="C16" t="n">
         <v>3705</v>
       </c>
       <c r="D16" t="n">
-        <v>0.018</v>
+        <v>0.01778</v>
       </c>
       <c r="E16" t="n">
         <v>0.04655</v>
       </c>
       <c r="F16" t="n">
-        <v>-1.027</v>
+        <v>-1.035</v>
       </c>
       <c r="G16" t="n">
-        <v>0.3045</v>
+        <v>0.3008</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -82983,10 +82983,10 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>-0.0295</v>
+        <v>-0.0292</v>
       </c>
       <c r="D58" t="n">
-        <v>0.0104</v>
+        <v>0.0112</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -83009,7 +83009,7 @@
         <v>-0.0112</v>
       </c>
       <c r="D59" t="n">
-        <v>0.3298</v>
+        <v>0.3314</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -83029,10 +83029,10 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>-0.0036</v>
+        <v>-0.0034</v>
       </c>
       <c r="D60" t="n">
-        <v>0.7522</v>
+        <v>0.7645</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -83704,10 +83704,10 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>-0.1917</v>
+        <v>-0.1831</v>
       </c>
       <c r="C16" t="n">
-        <v>1.02</v>
+        <v>1.0182</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-30T22:24Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-30 20:08 UTC</t>
+          <t>Genere le 2026-09-30 22:24 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-30 20:08 UTC</t>
+          <t>Rapport global — 2026-09-30 22:24 UTC</t>
         </is>
       </c>
     </row>
@@ -617,21 +617,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>**Regime monetaire emploi** — Chine : taux 1.54% (stable, niveau bas) -- chomage non_couvert  _(sans synthese)_ _(observation : 2026-09-28)_</t>
+          <t>**Regime monetaire emploi** — Chine : taux 1.54% (stable, niveau bas) -- chomage non_couvert  _(sans synthese)_ _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>**Regle taylor** — Taylor (2 termes, sans output gap)=6.03%, Fed reel=3.88%, ecart=-2.15pt -- accommodant (Fed en-dessous de la regle) _(observation : 2026-09-28)_</t>
+          <t>**Regle taylor** — Taylor (2 termes, sans output gap)=6.03%, Fed reel=3.88%, ecart=-2.15pt -- accommodant (Fed en-dessous de la regle) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>**Chemin taux fed** — chemin de taux (pas des probabilites) : DFF=3.88%, prochaine reunion 2026-10-27 (11 a venir dans le calendrier) -- 0-1 mois: +16pb (hausse, confiance faible) | 1-3 mois: +52pb (hausse, confiance faible) | 3-6 mois: +66pb (hausse, confiance faible) | 6-12 mois: +89pb (hausse, confiance faible) _(observation : 2026-09-28)_</t>
+          <t>**Chemin taux fed** — chemin de taux (pas des probabilites) : DFF=3.88%, prochaine reunion 2026-10-27 (11 a venir dans le calendrier) -- 0-1 mois: +16pb (hausse, confiance faible) | 1-3 mois: +48pb (hausse, confiance faible) | 3-6 mois: +59pb (hausse, confiance faible) | 6-12 mois: +92pb (hausse, confiance faible) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -792,14 +792,14 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>**Soutenabilite dette** — 8 pays. charge la plus lourde : Canada a 25.5% du revenu. taux 10 ans AU-DESSUS de l'inflation dans 5 pays -- Royaume-Uni (+2.3pt), Etats-Unis (+1.8pt), Japon (+1.0pt), Canada (+0.9pt), Zone euro (+0.9pt). Configuration ou le ratio d'endettement monte meme a budget primaire equilibre (approximation : croissance nominale reduite a l'inflation) _(observation : date non exposee)_</t>
+          <t>**Soutenabilite dette** — 8 pays. charge la plus lourde : Canada a 25.5% du revenu. taux 10 ans AU-DESSUS de l'inflation dans 5 pays -- Royaume-Uni (+2.3pt), Etats-Unis (+1.9pt), Japon (+1.0pt), Canada (+0.9pt), Zone euro (+0.9pt). Configuration ou le ratio d'endettement monte meme a budget primaire equilibre (approximation : croissance nominale reduite a l'inflation) _(observation : date non exposee)_</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>**Matieres premieres macro** — le ratio cuivre/or monte -- la croissance domine la peur (+5.5% sur 3 mois). Brent 98.1$ (+37.0% sur 3 mois, +46.3% sur 12 mois), gaz -6.3% sur 3 mois, ecart Brent-WTI +7.6$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-30)_</t>
+          <t>**Matieres premieres macro** — le ratio cuivre/or monte -- la croissance domine la peur (+5.6% sur 3 mois). Brent 97.7$ (+36.6% sur 3 mois, +45.8% sur 12 mois), gaz -6.6% sur 3 mois, ecart Brent-WTI +7.5$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -841,14 +841,14 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>**Taux reel us** — nominal=3.88%, inflation YoY=3.35%, reel=0.53% -- restrictif (taux reel positif et eleve) _(observation : 2026-09-28)_</t>
+          <t>**Taux reel us** — nominal=3.88%, inflation YoY=3.35%, reel=0.53% -- restrictif (taux reel positif et eleve) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>**Courbe taux us** — 10 ans=5.24%, 2 ans=4.92%, spread=+0.32pt -- normale (0 run(s) consecutif(s) dans l'historique accumule) _(observation : 2026-09-28)_</t>
+          <t>**Courbe taux us** — 10 ans=5.26%, 2 ans=4.89%, spread=+0.37pt -- normale (0 run(s) consecutif(s) dans l'historique accumule) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -862,7 +862,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>**Conditions financieres** — indice conditions financieres=+0.113 (3 composantes: {'taux_directeur': 0.5971439233898245, 'courbe_inversee': 0.23568763984021313, 'vix': -0.49281910275629404}) -- conditions proches de la normale _(observation : 2026-09-28)_</t>
+          <t>**Conditions financieres** — indice conditions financieres=+0.091 (3 composantes: {'taux_directeur': 0.5967870171242431, 'courbe_inversee': 0.15278119545281305, 'vix': -0.4779788474932477}) -- conditions proches de la normale _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -883,14 +883,14 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>**Stationnarite taux** — 1/5 series stationnaires (niveau, pas en difference) -- a garder en tete avant toute correlation/regression sur ces series telles quelles  _(sans synthese)_ _(observation : 2026-09-28)_</t>
+          <t>**Stationnarite taux** — 1/5 series stationnaires (niveau, pas en difference) -- a garder en tete avant toute correlation/regression sur ces series telles quelles  _(sans synthese)_ _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>**Cointegration taux** — 1/10 paires cointegrees  _(sans synthese)_ _(observation : 2026-09-28)_</t>
+          <t>**Cointegration taux** — 1/10 paires cointegrees  _(sans synthese)_ _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -904,7 +904,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>**Hp filter taux** — taux 10 ans observe=5.240%, tendance HP=5.011%, ecart cyclique=+0.229pt -- au-dessus de sa tendance locale _(observation : 2026-09-28)_</t>
+          <t>**Hp filter taux** — taux 10 ans observe=5.260%, tendance HP=5.038%, ecart cyclique=+0.222pt -- au-dessus de sa tendance locale _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -953,7 +953,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>**Differentiel taux change** — 8 paires testees sur variations a 21 jours -- le lien taux/change tient sur 5 paire(s) apres correction pour tests multiples : EURUSD, USDJPY, USDCAD, AUDUSD, EURJPY _(observation : 2026-09-28)_</t>
+          <t>**Differentiel taux change** — 8 paires testees sur variations a 21 jours -- le lien taux/change tient sur 4 paire(s) apres correction pour tests multiples : EURUSD, USDJPY, USDCAD, EURJPY _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -981,21 +981,21 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>**Beta facteur macro** — beta SP500/DGS10 (60j) = -0.0810 (rendement SP500 pour +1pt de taux 10 ans, 57/60 jours avec variation reelle) -- sensibilite elevee au facteur macro (choc de +100pb extrapole = -7.8%) _(observation : 2026-09-28)_</t>
+          <t>**Beta facteur macro** — beta SP500/DGS10 (60j) = -0.0802 (rendement SP500 pour +1pt de taux 10 ans, 57/60 jours avec variation reelle) -- sensibilite elevee au facteur macro (choc de +100pb extrapole = -7.7%) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>**Momentum prix** — SP500 momentum 12-1 mois = 14.92% -- haussier (momentum positif), detail 1/3/6/12m = [-0.44, 2.25, 16.37, 14.41] _(observation : 2026-09-30)_</t>
+          <t>**Momentum prix** — SP500 momentum 12-1 mois = 14.92% -- haussier (momentum positif), detail 1/3/6/12m = [-0.45, 2.25, 16.37, 14.4] _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>**Carry proxy** — Chine : 1.54% vs US 3.88% -- diff=-2.34pt (carry negatif (taux &lt; US))  _(sans synthese)_ _(observation : 2026-09-28)_</t>
+          <t>**Carry proxy** — Chine : 1.54% vs US 3.88% -- diff=-2.34pt (carry negatif (taux &lt; US))  _(sans synthese)_ _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1009,7 +1009,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>**Rotation sectorielle** — classement momentum 3 mois (10 secteurs) : 1. Energie (XLE) : +16.45% | 2. Sante (XLV) : +5.56% | 3. Technologie (XLK) : +5.46% | 4. Finance (XLF) : -2.55% | 5. Consommation de base (XLP) : -3.26% _(observation : 2026-09-30)_</t>
+          <t>**Rotation sectorielle** — classement momentum 3 mois (10 secteurs) : 1. Energie (XLE) : +16.45% | 2. Sante (XLV) : +5.57% | 3. Technologie (XLK) : +5.46% | 4. Finance (XLF) : -2.52% | 5. Consommation de base (XLP) : -3.24% _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1023,21 +1023,21 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>**Dispersion sectorielle** — 10 secteurs, rendement moyen 3m=-1.90%, dispersion (ecart-type)=8.20pt, etendue=28.38pt -- dispersion intermediaire _(observation : 2026-09-30)_</t>
+          <t>**Dispersion sectorielle** — 10 secteurs, rendement moyen 3m=-1.89%, dispersion (ecart-type)=8.19pt, etendue=28.36pt -- dispersion intermediaire _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>**Low volatility** — tercile bas-vol ['XLF', 'XLRE', 'XLU'] Sharpe=-1.125 vs tercile haut-vol ['XLY', 'XLE', 'XLK'] Sharpe=0.037 -- anomalie low-vol non confirmee sur cet echantillon (puissance statistique faible, n petit -- limite assumee) _(observation : 2026-09-30)_</t>
+          <t>**Low volatility** — tercile bas-vol ['XLF', 'XLRE', 'XLU'] Sharpe=-1.121 vs tercile haut-vol ['XLY', 'XLE', 'XLK'] Sharpe=0.036 -- anomalie low-vol non confirmee sur cet echantillon (puissance statistique faible, n petit -- limite assumee) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>**Momentum cross sectional** — panier gagnant ['XLE', 'XLV', 'XLK'] (+9.16%) vs panier perdant ['XLY', 'XLI', 'XLU'] (-9.57%) -- spread momentum=+18.72pt _(observation : 2026-09-30)_</t>
+          <t>**Momentum cross sectional** — panier gagnant ['XLE', 'XLV', 'XLK'] (+9.16%) vs panier perdant ['XLY', 'XLI', 'XLU'] (-9.56%) -- spread momentum=+18.72pt _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1051,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>**Correlation facteurs** — correlation entre momentum 3m et beta-VIX, 10 secteurs : +0.263 (facteurs largement independants) _(observation : 2026-09-30)_</t>
+          <t>**Correlation facteurs** — correlation entre momentum 3m et beta-VIX, 10 secteurs : +0.264 (facteurs largement independants) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1107,7 +1107,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>**Divergence cot prix** — SP500 -0.44% sur 30j, COT net -10560 -&gt; -133228 -- pas de divergence _(observation : 2026-09-30)_</t>
+          <t>**Divergence cot prix** — SP500 -0.45% sur 30j, COT net -10560 -&gt; -133228 -- pas de divergence _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1191,14 +1191,14 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>**Vol cross asset** — 6 mesures de volatilite : Petrole (OVX) 84e pct, Or (GVZ) 83e pct, Taux US (MOVE) 64e pct, Nasdaq (VXN) 50e pct, Actions US (VIX) 34e pct, Vol de la vol (VVIX) 31e pct -- stress LOCALISE sur Petrole (OVX), Or (GVZ) pendant que le reste ne l'est pas -- episode propre a cette classe d'actifs, pas une aversion au risque d'ensemble _(observation : 2026-09-30)_</t>
+          <t>**Vol cross asset** — 6 mesures de volatilite : Petrole (OVX) 83e pct, Or (GVZ) 82e pct, Taux US (MOVE) 64e pct, Nasdaq (VXN) 50e pct, Actions US (VIX) 35e pct, Vol de la vol (VVIX) 32e pct -- stress LOCALISE sur Petrole (OVX), Or (GVZ) pendant que le reste ne l'est pas -- episode propre a cette classe d'actifs, pas une aversion au risque d'ensemble _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>**Volatilite ewma** — vol realisee 60j=0.11172032117323961, EWMA=0.1031 (tendance 10 runs: stable) _(observation : 2026-09-30)_</t>
+          <t>**Volatilite ewma** — vol realisee 60j=0.11172595221123988, EWMA=0.1031 (tendance 10 runs: stable) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1219,7 +1219,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>**Ornstein uhlenbeck vix** — VIX actuel=16.22, niveau moyen estime (mu)=20.20, demi-vie=28.8j, ecart actuel=-3.98 -- VIX actuel en-dessous de son niveau moyen de long terme _(observation : 2026-09-30)_</t>
+          <t>**Ornstein uhlenbeck vix** — VIX actuel=16.34, niveau moyen estime (mu)=20.20, demi-vie=28.8j, ecart actuel=-3.86 -- VIX actuel en-dessous de son niveau moyen de long terme _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1233,14 +1233,14 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>**Kalman niveau local** — VIX observe=16.22, filtre Kalman=16.19 (ecart-type=0.62), ratio signal/bruit=0.2051 -- le filtre lisse fortement le bruit, reagit lentement (ecart obs.-filtre=+0.03) _(observation : 2026-09-30)_</t>
+          <t>**Kalman niveau local** — VIX observe=16.34, filtre Kalman=16.29 (ecart-type=0.62), ratio signal/bruit=0.2051 -- le filtre lisse fortement le bruit, reagit lentement (ecart obs.-filtre=+0.05) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.3658803288447583 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.0523166004347603 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-30)_</t>
+          <t>**Var sp500 vix** — VAR ordre choisi par AIC=10 -- coef SP500(t-1)-&gt;VIX(t)=0.3653209340540666 (SP500(t-1) en hausse -&gt; VIX(t) tend aussi a monter), coef VIX(t-1)-&gt;SP500(t)=-0.05231635680691482 (VIX(t-1) en hausse -&gt; SP500(t) tend a baisser) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1268,7 +1268,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>**Ratios performance** — Sharpe=1.039 (bon), Sortino=1.030 (bon), Calmar=1.485 (bon) -- lecture sur fenetre 252j (~1 an, echantillon limite), seuils academiques standards, taux sans risque suppose nul _(observation : 2026-09-30)_</t>
+          <t>**Ratios performance** — Sharpe=1.039 (bon), Sortino=1.029 (bon), Calmar=1.485 (bon) -- lecture sur fenetre 252j (~1 an, echantillon limite), seuils academiques standards, taux sans risque suppose nul _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1303,21 +1303,21 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>**Detection saut** — Z-stat BNS (fenetre 22j)=1.026 (seuil ±1.96) -- pas de saut isole detecte _(observation : 2026-09-30)_</t>
+          <t>**Detection saut** — Z-stat BNS (fenetre 22j)=1.027 (seuil ±1.96) -- pas de saut isole detecte _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>**Choc taux** — beta SP500/DGS10=-0.0810 -- choc +100pb : -8.10% (SP500 7684 -&gt; 7061) ; choc -100pb : +8.10% (-&gt; 8306) _(observation : 2026-09-28)_</t>
+          <t>**Choc taux** — beta SP500/DGS10=-0.0802 -- choc +100pb : -8.02% (SP500 7671 -&gt; 7055) ; choc -100pb : +8.02% (-&gt; 8286) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>**Qualite regime macro** — instabilite taux=0.0088, instabilite VIX=0.0676 -- score qualite du regime=-0.0382 (plus haut = regime plus stable/previsible) _(observation : 2026-09-28)_</t>
+          <t>**Qualite regime macro** — instabilite taux=0.0088, instabilite VIX=0.0676 -- score qualite du regime=-0.0382 (plus haut = regime plus stable/previsible) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1331,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>**Decomposition stl** — VIX : tendance=15.61, composante saisonniere (periode 5j)=+0.469, residu=+0.146 -- la saisonnalite explique 0.72% de la variance totale (negligeable) _(observation : 2026-09-30)_</t>
+          <t>**Decomposition stl** — VIX : tendance=15.63, composante saisonniere (periode 5j)=+0.508, residu=+0.205 -- la saisonnalite explique 0.72% de la variance totale (negligeable) _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1387,7 +1387,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>**Anomalie multivariee** — distance de Mahalanobis=0.495 (seuil 3.0) -- jour ordinaire _(observation : 2026-09-30)_</t>
+          <t>**Anomalie multivariee** — distance de Mahalanobis=0.428 (seuil 3.0) -- jour ordinaire _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -1408,7 +1408,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>**Kmeans regimes** — 2048 points, k=3 -- point actuel (VIX=16.1, spread=+0.32, taux=3.88%) -&gt; cluster 1 (tailles : {0: 357, 1: 1367, 2: 324}) -- regime calme (VIX du cluster en-dessous de la moyenne historique) _(observation : 2026-09-28)_</t>
+          <t>**Kmeans regimes** — 2048 points, k=3 -- point actuel (VIX=16.0, spread=+0.37, taux=3.88%) -&gt; cluster 1 (tailles : {0: 357, 1: 1367, 2: 324}) -- regime calme (VIX du cluster en-dessous de la moyenne historique) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1443,14 +1443,14 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>**Decomposition variance** — R² SP500~DGS10 (60j) = 0.2827 -- 28.3% de la variance des rendements SP500 expliquee par les variations du taux 10 ans (le reste = idiosyncratique/autres facteurs) _(observation : 2026-09-28)_</t>
+          <t>**Decomposition variance** — R² SP500~DGS10 (60j) = 0.2801 -- 28.0% de la variance des rendements SP500 expliquee par les variations du taux 10 ans (le reste = idiosyncratique/autres facteurs) _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>**Test chow** — test de Chow (taux 10 ans, 1ere vs 2eme moitie des 12 derniers mois) : F=547.278, p=0.0000 -- RUPTURE structurelle significative _(observation : 2026-09-28)_</t>
+          <t>**Test chow** — test de Chow (taux 10 ans, 1ere vs 2eme moitie des 12 derniers mois) : F=538.154, p=0.0000 -- RUPTURE structurelle significative _(observation : 2026-09-29)_</t>
         </is>
       </c>
     </row>
@@ -1493,7 +1493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E57"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2703,6 +2703,90 @@
         <v>3.88</v>
       </c>
       <c r="E57" t="n">
+        <v>-2.34</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Zone_euro</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D58" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="E58" t="n">
+        <v>-1.38</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Royaume-Uni</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>3.7302</v>
+      </c>
+      <c r="D59" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="E59" t="n">
+        <v>-0.15</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Japon</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>0.977</v>
+      </c>
+      <c r="D60" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="E60" t="n">
+        <v>-2.903</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Chine</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="D61" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="E61" t="n">
         <v>-2.34</v>
       </c>
     </row>
@@ -3203,7 +3287,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F71"/>
+  <dimension ref="A1:F76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5201,6 +5285,146 @@
         <v>0.0002</v>
       </c>
       <c r="F71" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>DFF</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>-0.5043</v>
+      </c>
+      <c r="E72" t="n">
+        <v>0.8912</v>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Zone_euro</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>ECBDFR</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>-0.5837</v>
+      </c>
+      <c r="E73" t="n">
+        <v>0.8746</v>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Royaume-Uni</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>IUDSOIA</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>-0.1754</v>
+      </c>
+      <c r="E74" t="n">
+        <v>0.9414</v>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Japon</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>IRSTCI01JPM156N</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>-1.9195</v>
+      </c>
+      <c r="E75" t="n">
+        <v>0.3229</v>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Chine</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>IR3TIB01CNM156N</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>-4.4511</v>
+      </c>
+      <c r="E76" t="n">
+        <v>0.0002</v>
+      </c>
+      <c r="F76" t="inlineStr">
         <is>
           <t>True</t>
         </is>
@@ -6069,7 +6293,7 @@
         <v>-56.78</v>
       </c>
       <c r="F30" t="n">
-        <v>3307.52</v>
+        <v>3307.35</v>
       </c>
     </row>
     <row r="31">
@@ -6097,7 +6321,7 @@
         <v>-33.92</v>
       </c>
       <c r="F31" t="n">
-        <v>5056.02</v>
+        <v>5055.76</v>
       </c>
     </row>
   </sheetData>
@@ -6261,7 +6485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6513,6 +6737,22 @@
         <v>3.353</v>
       </c>
       <c r="D15" t="n">
+        <v>0.527</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="C16" t="n">
+        <v>3.353</v>
+      </c>
+      <c r="D16" t="n">
         <v>0.527</v>
       </c>
     </row>
@@ -6527,7 +6767,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6805,6 +7045,24 @@
         <v>0</v>
       </c>
       <c r="D15" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>538.154</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" t="inlineStr">
         <is>
           <t>True</t>
         </is>
@@ -8456,7 +8714,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>32.7</v>
+        <v>32.8</v>
       </c>
       <c r="D16" t="n">
         <v>-2.847</v>
@@ -9131,10 +9389,10 @@
         <v>10</v>
       </c>
       <c r="C16" t="n">
-        <v>0.36588</v>
+        <v>0.36532</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.052317</v>
+        <v>-0.052316</v>
       </c>
     </row>
   </sheetData>
@@ -9203,10 +9461,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>52.58</v>
+        <v>52.24</v>
       </c>
       <c r="D2" t="n">
-        <v>83.59999999999999</v>
+        <v>83.09999999999999</v>
       </c>
       <c r="E2" t="n">
         <v>1260</v>
@@ -9229,10 +9487,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>23.84</v>
+        <v>23.74</v>
       </c>
       <c r="D3" t="n">
-        <v>82.90000000000001</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="E3" t="n">
         <v>1260</v>
@@ -9255,7 +9513,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>110.49</v>
+        <v>110.45</v>
       </c>
       <c r="D4" t="n">
         <v>63.7</v>
@@ -9281,10 +9539,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>22.4</v>
+        <v>22.46</v>
       </c>
       <c r="D5" t="n">
-        <v>49.8</v>
+        <v>50.4</v>
       </c>
       <c r="E5" t="n">
         <v>1260</v>
@@ -9307,10 +9565,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>16.22</v>
+        <v>16.34</v>
       </c>
       <c r="D6" t="n">
-        <v>34.1</v>
+        <v>35.3</v>
       </c>
       <c r="E6" t="n">
         <v>1260</v>
@@ -9333,10 +9591,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>88.88</v>
+        <v>89.48</v>
       </c>
       <c r="D7" t="n">
-        <v>31</v>
+        <v>32.5</v>
       </c>
       <c r="E7" t="n">
         <v>1260</v>
@@ -9671,7 +9929,7 @@
         <v>0.1031</v>
       </c>
       <c r="C16" t="n">
-        <v>0.0731</v>
+        <v>0.0732</v>
       </c>
       <c r="D16" t="n">
         <v>0.1079</v>
@@ -10417,7 +10675,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J33"/>
+  <dimension ref="A1:J37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11956,6 +12214,190 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>0-1 mois</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" t="n">
+        <v>4.04</v>
+      </c>
+      <c r="F34" t="n">
+        <v>16</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>hausse</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>forward_treasury_proxy</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>mouvement net de fenetre; aucune probabilite isolee par reunion</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>1-3 mois</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>2026-12-29</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>2</v>
+      </c>
+      <c r="E35" t="n">
+        <v>4.355</v>
+      </c>
+      <c r="F35" t="n">
+        <v>47.5</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>hausse</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>forward_treasury_proxy</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>mouvement net de fenetre; aucune probabilite isolee par reunion</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>3-6 mois</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>2027-03-30</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>5</v>
+      </c>
+      <c r="E36" t="n">
+        <v>4.47</v>
+      </c>
+      <c r="F36" t="n">
+        <v>59</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>hausse</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>forward_treasury_proxy</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>mouvement net de fenetre; aucune probabilite isolee par reunion</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>6-12 mois</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>2027-09-29</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>9</v>
+      </c>
+      <c r="E37" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F37" t="n">
+        <v>92</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>hausse</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>forward_treasury_proxy</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>faible</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>mouvement net de fenetre; aucune probabilite isolee par reunion</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11967,7 +12409,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12364,6 +12806,31 @@
       </c>
       <c r="G15" t="n">
         <v>8306.299999999999</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>-0.08022</v>
+      </c>
+      <c r="C16" t="n">
+        <v>7670.84</v>
+      </c>
+      <c r="D16" t="n">
+        <v>-8.02</v>
+      </c>
+      <c r="E16" t="n">
+        <v>7055.5</v>
+      </c>
+      <c r="F16" t="n">
+        <v>8.02</v>
+      </c>
+      <c r="G16" t="n">
+        <v>8286.200000000001</v>
       </c>
     </row>
   </sheetData>
@@ -17802,10 +18269,10 @@
         </is>
       </c>
       <c r="C142" t="n">
-        <v>-2.373</v>
+        <v>-2.372</v>
       </c>
       <c r="D142" t="n">
-        <v>0.3377</v>
+        <v>0.3382</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -17825,10 +18292,10 @@
         </is>
       </c>
       <c r="C143" t="n">
-        <v>-1.7321</v>
+        <v>-1.7365</v>
       </c>
       <c r="D143" t="n">
-        <v>0.6621</v>
+        <v>0.66</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -17848,10 +18315,10 @@
         </is>
       </c>
       <c r="C144" t="n">
-        <v>-2.2349</v>
+        <v>-2.235</v>
       </c>
       <c r="D144" t="n">
-        <v>0.4065</v>
+        <v>0.4064</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -17871,10 +18338,10 @@
         </is>
       </c>
       <c r="C145" t="n">
-        <v>-2.4302</v>
+        <v>-2.4303</v>
       </c>
       <c r="D145" t="n">
-        <v>0.3107</v>
+        <v>0.3106</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -17894,10 +18361,10 @@
         </is>
       </c>
       <c r="C146" t="n">
-        <v>-1.285</v>
+        <v>-1.2894</v>
       </c>
       <c r="D146" t="n">
-        <v>0.8342000000000001</v>
+        <v>0.8329</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -17917,7 +18384,7 @@
         </is>
       </c>
       <c r="C147" t="n">
-        <v>0.0406</v>
+        <v>0.0419</v>
       </c>
       <c r="D147" t="n">
         <v>0.9868</v>
@@ -17940,10 +18407,10 @@
         </is>
       </c>
       <c r="C148" t="n">
-        <v>-1.0663</v>
+        <v>-1.0685</v>
       </c>
       <c r="D148" t="n">
-        <v>0.8895</v>
+        <v>0.8891</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -17963,10 +18430,10 @@
         </is>
       </c>
       <c r="C149" t="n">
-        <v>-0.6891</v>
+        <v>-0.6932</v>
       </c>
       <c r="D149" t="n">
-        <v>0.9478</v>
+        <v>0.9474</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -17986,10 +18453,10 @@
         </is>
       </c>
       <c r="C150" t="n">
-        <v>-2.0399</v>
+        <v>-2.0425</v>
       </c>
       <c r="D150" t="n">
-        <v>0.5078</v>
+        <v>0.5064</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -18009,10 +18476,10 @@
         </is>
       </c>
       <c r="C151" t="n">
-        <v>-1.5365</v>
+        <v>-1.5373</v>
       </c>
       <c r="D151" t="n">
-        <v>0.7469</v>
+        <v>0.7466</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -18031,7 +18498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F141"/>
+  <dimension ref="A1:F151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -21989,6 +22456,286 @@
         <v>0.7171</v>
       </c>
       <c r="F141" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Chine</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Japon</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>-3.6969</v>
+      </c>
+      <c r="E142" t="n">
+        <v>0.0185</v>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>True</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Chine</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Royaume-Uni</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>-2.417</v>
+      </c>
+      <c r="E143" t="n">
+        <v>0.3168</v>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Chine</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>-2.0335</v>
+      </c>
+      <c r="E144" t="n">
+        <v>0.5111</v>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Chine</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Zone_euro</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>-2.1259</v>
+      </c>
+      <c r="E145" t="n">
+        <v>0.4628</v>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Japon</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Royaume-Uni</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>-1.975</v>
+      </c>
+      <c r="E146" t="n">
+        <v>0.5415</v>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Japon</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>-0.3664</v>
+      </c>
+      <c r="E147" t="n">
+        <v>0.9726</v>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Japon</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Zone_euro</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>-0.7129</v>
+      </c>
+      <c r="E148" t="n">
+        <v>0.9452</v>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Royaume-Uni</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>-1.9904</v>
+      </c>
+      <c r="E149" t="n">
+        <v>0.5336</v>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Royaume-Uni</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Zone_euro</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>-2.2118</v>
+      </c>
+      <c r="E150" t="n">
+        <v>0.4183</v>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Zone_euro</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>-1.6072</v>
+      </c>
+      <c r="E151" t="n">
+        <v>0.7178</v>
+      </c>
+      <c r="F151" t="inlineStr">
         <is>
           <t>False</t>
         </is>
@@ -24806,7 +25553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -25155,6 +25902,28 @@
       </c>
       <c r="F15" t="n">
         <v>-0.4928</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.0905</v>
+      </c>
+      <c r="C16" t="n">
+        <v>3</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.5968</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.1528</v>
+      </c>
+      <c r="F16" t="n">
+        <v>-0.478</v>
       </c>
     </row>
   </sheetData>
@@ -25455,7 +26224,7 @@
         <v>10</v>
       </c>
       <c r="C16" t="n">
-        <v>0.2626</v>
+        <v>0.2642</v>
       </c>
     </row>
   </sheetData>
@@ -37105,7 +37874,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -37431,6 +38200,27 @@
         <v>0.32</v>
       </c>
       <c r="E15" t="inlineStr">
+        <is>
+          <t>False</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>5.26</v>
+      </c>
+      <c r="C16" t="n">
+        <v>4.89</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="E16" t="inlineStr">
         <is>
           <t>False</t>
         </is>
@@ -38215,19 +39005,19 @@
         <v>2.2</v>
       </c>
       <c r="C15" t="n">
-        <v>413.94</v>
+        <v>414.09</v>
       </c>
       <c r="D15" t="n">
         <v>4</v>
       </c>
       <c r="E15" t="n">
-        <v>373.71</v>
+        <v>373.95</v>
       </c>
       <c r="F15" t="n">
         <v>5.3</v>
       </c>
       <c r="G15" t="n">
-        <v>323.76</v>
+        <v>323.7</v>
       </c>
     </row>
   </sheetData>
@@ -39741,13 +40531,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>15.606</v>
+        <v>15.627</v>
       </c>
       <c r="C15" t="n">
-        <v>0.469</v>
+        <v>0.508</v>
       </c>
       <c r="D15" t="n">
-        <v>0.146</v>
+        <v>0.205</v>
       </c>
       <c r="E15" t="n">
         <v>0.72</v>
@@ -39764,7 +40554,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -39969,6 +40759,19 @@
       </c>
       <c r="C15" t="n">
         <v>28.27</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.28015</v>
+      </c>
+      <c r="C16" t="n">
+        <v>28.01</v>
       </c>
     </row>
   </sheetData>
@@ -40656,7 +41459,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1.026</v>
+        <v>1.027</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -40735,17 +41538,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>-1.687</v>
+        <v>-1.679</v>
       </c>
       <c r="D2" t="n">
-        <v>0.403</v>
+        <v>0.409</v>
       </c>
       <c r="E2" t="n">
-        <v>1e-05</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
         <v>118</v>
@@ -40771,7 +41574,7 @@
         <v>2.597</v>
       </c>
       <c r="D3" t="n">
-        <v>0.5590000000000001</v>
+        <v>0.525</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
@@ -40800,10 +41603,10 @@
         <v>-0.09</v>
       </c>
       <c r="D4" t="n">
-        <v>0.061</v>
+        <v>0.115</v>
       </c>
       <c r="E4" t="n">
-        <v>0.51607</v>
+        <v>0.21536</v>
       </c>
       <c r="F4" t="n">
         <v>117</v>
@@ -40829,10 +41632,10 @@
         <v>1.55</v>
       </c>
       <c r="D5" t="n">
-        <v>0.419</v>
+        <v>0.385</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>2e-05</v>
       </c>
       <c r="F5" t="n">
         <v>117</v>
@@ -40858,17 +41661,17 @@
         <v>0.097</v>
       </c>
       <c r="D6" t="n">
-        <v>0.278</v>
+        <v>0.235</v>
       </c>
       <c r="E6" t="n">
-        <v>0.00251</v>
+        <v>0.01127</v>
       </c>
       <c r="F6" t="n">
         <v>116</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>oui</t>
+          <t>non</t>
         </is>
       </c>
     </row>
@@ -40880,17 +41683,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2.127</v>
+        <v>2.112</v>
       </c>
       <c r="D7" t="n">
-        <v>0.232</v>
+        <v>0.248</v>
       </c>
       <c r="E7" t="n">
-        <v>0.0121</v>
+        <v>0.00733</v>
       </c>
       <c r="F7" t="n">
         <v>116</v>
@@ -41308,13 +42111,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>-0.00247</v>
+        <v>-0.00252</v>
       </c>
       <c r="C16" t="n">
-        <v>0.18</v>
+        <v>0.3</v>
       </c>
       <c r="D16" t="n">
-        <v>0.495</v>
+        <v>0.428</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -41646,13 +42449,13 @@
         <v>10</v>
       </c>
       <c r="C16" t="n">
-        <v>-1.901</v>
+        <v>-1.89</v>
       </c>
       <c r="D16" t="n">
-        <v>8.196</v>
+        <v>8.192</v>
       </c>
       <c r="E16" t="n">
-        <v>28.383</v>
+        <v>28.361</v>
       </c>
     </row>
   </sheetData>
@@ -42004,7 +42807,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>-0.445</v>
+        <v>-0.45</v>
       </c>
       <c r="C16" t="n">
         <v>-133228</v>
@@ -52067,7 +52870,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>fred/DFF.csv</t>
+          <t>fred/IUDSOIA.csv</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -52096,7 +52899,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>fred/DFII10.csv</t>
+          <t>souverains/CANADA_10A.csv</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -52114,7 +52917,7 @@
         <v>42</v>
       </c>
       <c r="F188" t="n">
-        <v>3000</v>
+        <v>6437</v>
       </c>
       <c r="G188" t="inlineStr">
         <is>
@@ -52125,7 +52928,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>fred/DFII5.csv</t>
+          <t>souverains/CANADA_2A.csv</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -52143,7 +52946,7 @@
         <v>42</v>
       </c>
       <c r="F189" t="n">
-        <v>3000</v>
+        <v>6436</v>
       </c>
       <c r="G189" t="inlineStr">
         <is>
@@ -52154,7 +52957,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>fred/DGS1.csv</t>
+          <t>souverains/CANADA_5A.csv</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -52172,7 +52975,7 @@
         <v>42</v>
       </c>
       <c r="F190" t="n">
-        <v>3000</v>
+        <v>6436</v>
       </c>
       <c r="G190" t="inlineStr">
         <is>
@@ -52183,7 +52986,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>fred/DGS10.csv</t>
+          <t>souverains/CANADA_LONG.csv</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -52201,7 +53004,7 @@
         <v>42</v>
       </c>
       <c r="F191" t="n">
-        <v>3000</v>
+        <v>6436</v>
       </c>
       <c r="G191" t="inlineStr">
         <is>
@@ -52212,7 +53015,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>fred/DGS1MO.csv</t>
+          <t>souverains/UK_10A.csv</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -52230,7 +53033,7 @@
         <v>42</v>
       </c>
       <c r="F192" t="n">
-        <v>3000</v>
+        <v>9285</v>
       </c>
       <c r="G192" t="inlineStr">
         <is>
@@ -52241,7 +53044,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>fred/DGS2.csv</t>
+          <t>souverains/UK_20A.csv</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -52259,7 +53062,7 @@
         <v>42</v>
       </c>
       <c r="F193" t="n">
-        <v>3000</v>
+        <v>6756</v>
       </c>
       <c r="G193" t="inlineStr">
         <is>
@@ -52270,7 +53073,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>fred/DGS30.csv</t>
+          <t>souverains/UK_5A.csv</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -52288,7 +53091,7 @@
         <v>42</v>
       </c>
       <c r="F194" t="n">
-        <v>3000</v>
+        <v>8293</v>
       </c>
       <c r="G194" t="inlineStr">
         <is>
@@ -52299,16 +53102,16 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>fred/DGS3MO.csv</t>
+          <t>fred/BAMLC0A0CM.csv</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C195" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D195" t="n">
         <v>1</v>
@@ -52317,7 +53120,7 @@
         <v>42</v>
       </c>
       <c r="F195" t="n">
-        <v>3000</v>
+        <v>793</v>
       </c>
       <c r="G195" t="inlineStr">
         <is>
@@ -52328,16 +53131,16 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>fred/DGS5.csv</t>
+          <t>fred/BAMLC0A0CMEY.csv</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C196" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D196" t="n">
         <v>1</v>
@@ -52346,7 +53149,7 @@
         <v>42</v>
       </c>
       <c r="F196" t="n">
-        <v>3000</v>
+        <v>793</v>
       </c>
       <c r="G196" t="inlineStr">
         <is>
@@ -52357,16 +53160,16 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>fred/DGS6MO.csv</t>
+          <t>fred/BAMLEMCBPIOAS.csv</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C197" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D197" t="n">
         <v>1</v>
@@ -52375,7 +53178,7 @@
         <v>42</v>
       </c>
       <c r="F197" t="n">
-        <v>3000</v>
+        <v>793</v>
       </c>
       <c r="G197" t="inlineStr">
         <is>
@@ -52386,16 +53189,16 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>fred/IUDSOIA.csv</t>
+          <t>fred/BAMLEMFSFCRPIOAS.csv</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C198" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D198" t="n">
         <v>1</v>
@@ -52404,7 +53207,7 @@
         <v>42</v>
       </c>
       <c r="F198" t="n">
-        <v>3000</v>
+        <v>793</v>
       </c>
       <c r="G198" t="inlineStr">
         <is>
@@ -52415,16 +53218,16 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>souverains/CANADA_10A.csv</t>
+          <t>fred/BAMLEMHBHYCRPIOAS.csv</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C199" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D199" t="n">
         <v>1</v>
@@ -52433,7 +53236,7 @@
         <v>42</v>
       </c>
       <c r="F199" t="n">
-        <v>6437</v>
+        <v>793</v>
       </c>
       <c r="G199" t="inlineStr">
         <is>
@@ -52444,16 +53247,16 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>souverains/CANADA_2A.csv</t>
+          <t>fred/BAMLEMPBPUBSICRPIOAS.csv</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C200" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D200" t="n">
         <v>1</v>
@@ -52462,7 +53265,7 @@
         <v>42</v>
       </c>
       <c r="F200" t="n">
-        <v>6436</v>
+        <v>793</v>
       </c>
       <c r="G200" t="inlineStr">
         <is>
@@ -52473,16 +53276,16 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>souverains/CANADA_5A.csv</t>
+          <t>fred/BAMLH0A0HYM2.csv</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C201" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D201" t="n">
         <v>1</v>
@@ -52491,7 +53294,7 @@
         <v>42</v>
       </c>
       <c r="F201" t="n">
-        <v>6436</v>
+        <v>793</v>
       </c>
       <c r="G201" t="inlineStr">
         <is>
@@ -52502,16 +53305,16 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>souverains/CANADA_LONG.csv</t>
+          <t>fred/BAMLHE00EHYIEY.csv</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C202" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D202" t="n">
         <v>1</v>
@@ -52520,7 +53323,7 @@
         <v>42</v>
       </c>
       <c r="F202" t="n">
-        <v>6436</v>
+        <v>793</v>
       </c>
       <c r="G202" t="inlineStr">
         <is>
@@ -52531,16 +53334,16 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>souverains/UK_10A.csv</t>
+          <t>fred/BAMLHE00EHYIOAS.csv</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C203" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D203" t="n">
         <v>1</v>
@@ -52549,7 +53352,7 @@
         <v>42</v>
       </c>
       <c r="F203" t="n">
-        <v>9285</v>
+        <v>793</v>
       </c>
       <c r="G203" t="inlineStr">
         <is>
@@ -52560,16 +53363,16 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>souverains/UK_20A.csv</t>
+          <t>fred/DFF.csv</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C204" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D204" t="n">
         <v>1</v>
@@ -52578,7 +53381,7 @@
         <v>42</v>
       </c>
       <c r="F204" t="n">
-        <v>6756</v>
+        <v>3000</v>
       </c>
       <c r="G204" t="inlineStr">
         <is>
@@ -52589,16 +53392,16 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>souverains/UK_5A.csv</t>
+          <t>fred/DFII10.csv</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C205" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D205" t="n">
         <v>1</v>
@@ -52607,7 +53410,7 @@
         <v>42</v>
       </c>
       <c r="F205" t="n">
-        <v>8293</v>
+        <v>3000</v>
       </c>
       <c r="G205" t="inlineStr">
         <is>
@@ -52618,16 +53421,16 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>tresor_us/dette_quotidienne.csv</t>
+          <t>fred/DFII5.csv</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C206" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D206" t="n">
         <v>1</v>
@@ -52636,7 +53439,7 @@
         <v>42</v>
       </c>
       <c r="F206" t="n">
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="G206" t="inlineStr">
         <is>
@@ -52647,7 +53450,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>fred/BAMLC0A0CM.csv</t>
+          <t>fred/DGS1.csv</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -52665,7 +53468,7 @@
         <v>42</v>
       </c>
       <c r="F207" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G207" t="inlineStr">
         <is>
@@ -52676,7 +53479,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>fred/BAMLC0A0CMEY.csv</t>
+          <t>fred/DGS10.csv</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -52694,7 +53497,7 @@
         <v>42</v>
       </c>
       <c r="F208" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G208" t="inlineStr">
         <is>
@@ -52705,7 +53508,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>fred/BAMLEMCBPIOAS.csv</t>
+          <t>fred/DGS1MO.csv</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -52723,7 +53526,7 @@
         <v>42</v>
       </c>
       <c r="F209" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G209" t="inlineStr">
         <is>
@@ -52734,7 +53537,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>fred/BAMLEMFSFCRPIOAS.csv</t>
+          <t>fred/DGS2.csv</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -52752,7 +53555,7 @@
         <v>42</v>
       </c>
       <c r="F210" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G210" t="inlineStr">
         <is>
@@ -52763,7 +53566,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>fred/BAMLEMHBHYCRPIOAS.csv</t>
+          <t>fred/DGS30.csv</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
@@ -52781,7 +53584,7 @@
         <v>42</v>
       </c>
       <c r="F211" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G211" t="inlineStr">
         <is>
@@ -52792,7 +53595,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>fred/BAMLEMPBPUBSICRPIOAS.csv</t>
+          <t>fred/DGS3MO.csv</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -52810,7 +53613,7 @@
         <v>42</v>
       </c>
       <c r="F212" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G212" t="inlineStr">
         <is>
@@ -52821,7 +53624,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>fred/BAMLH0A0HYM2.csv</t>
+          <t>fred/DGS5.csv</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -52839,7 +53642,7 @@
         <v>42</v>
       </c>
       <c r="F213" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G213" t="inlineStr">
         <is>
@@ -52850,7 +53653,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>fred/BAMLHE00EHYIEY.csv</t>
+          <t>fred/DGS6MO.csv</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -52868,7 +53671,7 @@
         <v>42</v>
       </c>
       <c r="F214" t="n">
-        <v>793</v>
+        <v>3000</v>
       </c>
       <c r="G214" t="inlineStr">
         <is>
@@ -52879,7 +53682,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>fred/BAMLHE00EHYIOAS.csv</t>
+          <t>marches/indices/DAX.csv</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -52897,7 +53700,7 @@
         <v>42</v>
       </c>
       <c r="F215" t="n">
-        <v>793</v>
+        <v>3801</v>
       </c>
       <c r="G215" t="inlineStr">
         <is>
@@ -52908,7 +53711,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>fred/T10YIE.csv</t>
+          <t>marches/indices/EUROSTOXX50.csv</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -52926,7 +53729,7 @@
         <v>42</v>
       </c>
       <c r="F216" t="n">
-        <v>3000</v>
+        <v>3758</v>
       </c>
       <c r="G216" t="inlineStr">
         <is>
@@ -53372,7 +54175,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>tresor_us/solde_tresorerie.csv</t>
+          <t>tresor_us/dette_quotidienne.csv</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -53390,7 +54193,7 @@
         <v>42</v>
       </c>
       <c r="F232" t="n">
-        <v>500</v>
+        <v>2000</v>
       </c>
       <c r="G232" t="inlineStr">
         <is>
@@ -53401,16 +54204,16 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>fred/ECBDFR.csv</t>
+          <t>tresor_us/solde_tresorerie.csv</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C233" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D233" t="n">
         <v>1</v>
@@ -53419,7 +54222,7 @@
         <v>42</v>
       </c>
       <c r="F233" t="n">
-        <v>3000</v>
+        <v>500</v>
       </c>
       <c r="G233" t="inlineStr">
         <is>
@@ -53430,7 +54233,7 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>fred/RRPONTSYD.csv</t>
+          <t>fred/ECBDFR.csv</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
@@ -53459,7 +54262,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>marches/fx/AUDJPY.csv</t>
+          <t>fred/RRPONTSYD.csv</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -53477,7 +54280,7 @@
         <v>42</v>
       </c>
       <c r="F235" t="n">
-        <v>3909</v>
+        <v>3000</v>
       </c>
       <c r="G235" t="inlineStr">
         <is>
@@ -53488,7 +54291,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>marches/fx/AUDUSD.csv</t>
+          <t>fred/T10YIE.csv</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -53506,7 +54309,7 @@
         <v>42</v>
       </c>
       <c r="F236" t="n">
-        <v>3905</v>
+        <v>3000</v>
       </c>
       <c r="G236" t="inlineStr">
         <is>
@@ -53517,7 +54320,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>marches/fx/DXY.csv</t>
+          <t>marches/fx/AUDJPY.csv</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
@@ -53535,7 +54338,7 @@
         <v>42</v>
       </c>
       <c r="F237" t="n">
-        <v>3772</v>
+        <v>3909</v>
       </c>
       <c r="G237" t="inlineStr">
         <is>
@@ -53546,7 +54349,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>marches/fx/EURCHF.csv</t>
+          <t>marches/fx/AUDUSD.csv</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
@@ -53564,7 +54367,7 @@
         <v>42</v>
       </c>
       <c r="F238" t="n">
-        <v>3906</v>
+        <v>3905</v>
       </c>
       <c r="G238" t="inlineStr">
         <is>
@@ -53575,7 +54378,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>marches/fx/EURGBP.csv</t>
+          <t>marches/fx/DXY.csv</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
@@ -53593,7 +54396,7 @@
         <v>42</v>
       </c>
       <c r="F239" t="n">
-        <v>3908</v>
+        <v>3772</v>
       </c>
       <c r="G239" t="inlineStr">
         <is>
@@ -53604,7 +54407,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>marches/fx/EURJPY.csv</t>
+          <t>marches/fx/EURCHF.csv</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
@@ -53622,7 +54425,7 @@
         <v>42</v>
       </c>
       <c r="F240" t="n">
-        <v>3908</v>
+        <v>3906</v>
       </c>
       <c r="G240" t="inlineStr">
         <is>
@@ -53633,7 +54436,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>marches/fx/EURUSD.csv</t>
+          <t>marches/fx/EURGBP.csv</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
@@ -53651,7 +54454,7 @@
         <v>42</v>
       </c>
       <c r="F241" t="n">
-        <v>3905</v>
+        <v>3908</v>
       </c>
       <c r="G241" t="inlineStr">
         <is>
@@ -53662,7 +54465,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>marches/fx/GBPUSD.csv</t>
+          <t>marches/fx/EURJPY.csv</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
@@ -53680,7 +54483,7 @@
         <v>42</v>
       </c>
       <c r="F242" t="n">
-        <v>3906</v>
+        <v>3908</v>
       </c>
       <c r="G242" t="inlineStr">
         <is>
@@ -53691,7 +54494,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>marches/fx/NZDUSD.csv</t>
+          <t>marches/fx/EURUSD.csv</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
@@ -53709,7 +54512,7 @@
         <v>42</v>
       </c>
       <c r="F243" t="n">
-        <v>3906</v>
+        <v>3905</v>
       </c>
       <c r="G243" t="inlineStr">
         <is>
@@ -53720,7 +54523,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>marches/fx/USDCAD.csv</t>
+          <t>marches/fx/GBPUSD.csv</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -53738,7 +54541,7 @@
         <v>42</v>
       </c>
       <c r="F244" t="n">
-        <v>3905</v>
+        <v>3906</v>
       </c>
       <c r="G244" t="inlineStr">
         <is>
@@ -53749,7 +54552,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>marches/fx/USDCHF.csv</t>
+          <t>marches/fx/NZDUSD.csv</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -53767,7 +54570,7 @@
         <v>42</v>
       </c>
       <c r="F245" t="n">
-        <v>3903</v>
+        <v>3906</v>
       </c>
       <c r="G245" t="inlineStr">
         <is>
@@ -53778,7 +54581,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>marches/fx/USDCNY.csv</t>
+          <t>marches/fx/USDCAD.csv</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -53807,7 +54610,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>marches/fx/USDJPY.csv</t>
+          <t>marches/fx/USDCHF.csv</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
@@ -53825,7 +54628,7 @@
         <v>42</v>
       </c>
       <c r="F247" t="n">
-        <v>3906</v>
+        <v>3903</v>
       </c>
       <c r="G247" t="inlineStr">
         <is>
@@ -53836,7 +54639,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>marches/fx/USDKRW.csv</t>
+          <t>marches/fx/USDCNY.csv</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
@@ -53865,7 +54668,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>marches/fx/USDNOK.csv</t>
+          <t>marches/fx/USDJPY.csv</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
@@ -53894,7 +54697,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>marches/fx/USDSEK.csv</t>
+          <t>marches/fx/USDKRW.csv</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
@@ -53912,7 +54715,7 @@
         <v>42</v>
       </c>
       <c r="F250" t="n">
-        <v>3906</v>
+        <v>3905</v>
       </c>
       <c r="G250" t="inlineStr">
         <is>
@@ -53923,7 +54726,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>marches/indices/DAX.csv</t>
+          <t>marches/fx/USDNOK.csv</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
@@ -53941,7 +54744,7 @@
         <v>42</v>
       </c>
       <c r="F251" t="n">
-        <v>3802</v>
+        <v>3906</v>
       </c>
       <c r="G251" t="inlineStr">
         <is>
@@ -53952,7 +54755,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>marches/indices/EUROSTOXX50.csv</t>
+          <t>marches/fx/USDSEK.csv</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -53970,7 +54773,7 @@
         <v>42</v>
       </c>
       <c r="F252" t="n">
-        <v>3759</v>
+        <v>3906</v>
       </c>
       <c r="G252" t="inlineStr">
         <is>
@@ -55412,7 +56215,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -55665,6 +56468,22 @@
       </c>
       <c r="D15" t="n">
         <v>0.2292</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>5.26</v>
+      </c>
+      <c r="C16" t="n">
+        <v>5.0382</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.2218</v>
       </c>
     </row>
   </sheetData>
@@ -56354,28 +57173,28 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Etats-Unis (S&amp;P 500)</t>
+          <t>Zone euro (Euro Stoxx 50)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>7651.94</v>
+        <v>6320.26</v>
       </c>
       <c r="D4" t="n">
-        <v>2.25</v>
+        <v>-0.12</v>
       </c>
       <c r="E4" t="n">
-        <v>14.41</v>
+        <v>14.77</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Royaume-Uni (FTSE 100)</t>
+          <t>Etats-Unis (S&amp;P 500)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -56384,19 +57203,19 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>10606</v>
+        <v>7651.54</v>
       </c>
       <c r="D5" t="n">
-        <v>1.22</v>
+        <v>2.25</v>
       </c>
       <c r="E5" t="n">
-        <v>13.43</v>
+        <v>14.4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Zone euro (Euro Stoxx 50)</t>
+          <t>Royaume-Uni (FTSE 100)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -56405,13 +57224,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>6269.02</v>
+        <v>10606</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.21</v>
+        <v>1.22</v>
       </c>
       <c r="E6" t="n">
-        <v>13.36</v>
+        <v>13.43</v>
       </c>
     </row>
     <row r="7">
@@ -56422,17 +57241,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>25199.19</v>
+        <v>25399.21</v>
       </c>
       <c r="D7" t="n">
-        <v>0.63</v>
+        <v>1.61</v>
       </c>
       <c r="E7" t="n">
-        <v>5.52</v>
+        <v>6.97</v>
       </c>
     </row>
     <row r="8">
@@ -57167,10 +57986,10 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>16.219999</v>
+        <v>16.34</v>
       </c>
       <c r="C15" t="n">
-        <v>16.19</v>
+        <v>16.292</v>
       </c>
       <c r="D15" t="n">
         <v>0.624</v>
@@ -57190,7 +58009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -57564,6 +58383,30 @@
         <v>1</v>
       </c>
       <c r="F15" t="inlineStr">
+        <is>
+          <t>{0: 357, 1: 1367, 2: 324}</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>16.040001</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="D16" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" t="inlineStr">
         <is>
           <t>{0: 357, 1: 1367, 2: 324}</t>
         </is>
@@ -58374,7 +59217,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>-1.125</v>
+        <v>-1.121</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -58382,7 +59225,7 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>0.037</v>
+        <v>0.036</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -58771,25 +59614,25 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.001582</v>
+        <v>0.001583</v>
       </c>
       <c r="C13" t="n">
-        <v>5.48</v>
+        <v>5.56</v>
       </c>
       <c r="D13" t="n">
-        <v>98.08</v>
+        <v>97.73999999999999</v>
       </c>
       <c r="E13" t="n">
-        <v>37.04</v>
+        <v>36.57</v>
       </c>
       <c r="F13" t="n">
-        <v>46.34</v>
+        <v>45.84</v>
       </c>
       <c r="G13" t="n">
-        <v>-6.34</v>
+        <v>-6.55</v>
       </c>
       <c r="H13" t="n">
-        <v>7.58</v>
+        <v>7.51</v>
       </c>
     </row>
   </sheetData>
@@ -59679,7 +60522,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>9.157</v>
+        <v>9.16</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -59687,10 +60530,10 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>-9.566000000000001</v>
+        <v>-9.557</v>
       </c>
       <c r="F16" t="n">
-        <v>18.723</v>
+        <v>18.717</v>
       </c>
     </row>
   </sheetData>
@@ -59704,7 +60547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -59908,6 +60751,19 @@
         <v>-0.08103</v>
       </c>
       <c r="C15" t="n">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>-0.08022</v>
+      </c>
+      <c r="C16" t="n">
         <v>57</v>
       </c>
     </row>
@@ -62659,16 +63515,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>-0.445</v>
+        <v>-0.45</v>
       </c>
       <c r="C16" t="n">
-        <v>2.255</v>
+        <v>2.249</v>
       </c>
       <c r="D16" t="n">
-        <v>16.374</v>
+        <v>16.368</v>
       </c>
       <c r="E16" t="n">
-        <v>14.405</v>
+        <v>14.399</v>
       </c>
       <c r="F16" t="n">
         <v>14.916</v>
@@ -63511,19 +64367,19 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>16.219999</v>
+        <v>16.34</v>
       </c>
       <c r="C15" t="n">
-        <v>20.201</v>
+        <v>20.202</v>
       </c>
       <c r="D15" t="n">
-        <v>0.02404</v>
+        <v>0.02405</v>
       </c>
       <c r="E15" t="n">
         <v>28.8</v>
       </c>
       <c r="F15" t="n">
-        <v>-3.981</v>
+        <v>-3.862</v>
       </c>
     </row>
   </sheetData>
@@ -63742,26 +64598,26 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>4.92</v>
+        <v>4.89</v>
       </c>
       <c r="D3" t="n">
-        <v>5.24</v>
+        <v>5.26</v>
       </c>
       <c r="E3" t="n">
-        <v>0.32</v>
+        <v>0.37</v>
       </c>
       <c r="F3" t="n">
-        <v>0.04</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="G3" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H3" t="n">
         <v>0.82</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0.86</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -68807,7 +69663,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>-0.004852</v>
+        <v>-0.004853</v>
       </c>
     </row>
   </sheetData>
@@ -69734,7 +70590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -69986,6 +70842,22 @@
         <v>0.06759999999999999</v>
       </c>
       <c r="D15" t="n">
+        <v>-0.03819</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.00876</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.06762</v>
+      </c>
+      <c r="D16" t="n">
         <v>-0.03819</v>
       </c>
     </row>
@@ -73484,13 +74356,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1.0392</v>
+        <v>1.0388</v>
       </c>
       <c r="C16" t="n">
-        <v>1.0297</v>
+        <v>1.0293</v>
       </c>
       <c r="D16" t="n">
-        <v>1.4851</v>
+        <v>1.4846</v>
       </c>
     </row>
   </sheetData>
@@ -73562,7 +74434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G76"/>
+  <dimension ref="A1:G81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -76017,6 +76889,165 @@
         </is>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>stable</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>moyen</t>
+        </is>
+      </c>
+      <c r="F77" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>stable</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Zone euro</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>hausse</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>haut</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>non_couvert</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Royaume-Uni</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>3.7302</v>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>stable</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>haut</t>
+        </is>
+      </c>
+      <c r="F79" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>stable</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Japon</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>0.977</v>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>stable</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>haut</t>
+        </is>
+      </c>
+      <c r="F80" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>stable</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Chine</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>1.54</v>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>stable</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>bas</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>non_couvert</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -76028,7 +77059,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -76402,6 +77433,30 @@
         <v>-2.15</v>
       </c>
       <c r="F15" t="inlineStr">
+        <is>
+          <t>2_termes_sans_output_gap</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>3.353</v>
+      </c>
+      <c r="C16" t="n">
+        <v>6.03</v>
+      </c>
+      <c r="D16" t="n">
+        <v>3.88</v>
+      </c>
+      <c r="E16" t="n">
+        <v>-2.15</v>
+      </c>
+      <c r="F16" t="inlineStr">
         <is>
           <t>2_termes_sans_output_gap</t>
         </is>
@@ -80540,7 +81595,7 @@
         </is>
       </c>
       <c r="E143" t="n">
-        <v>5.56</v>
+        <v>5.566</v>
       </c>
     </row>
     <row r="144">
@@ -80586,7 +81641,7 @@
         </is>
       </c>
       <c r="E145" t="n">
-        <v>-2.552</v>
+        <v>-2.519</v>
       </c>
     </row>
     <row r="146">
@@ -80609,7 +81664,7 @@
         </is>
       </c>
       <c r="E146" t="n">
-        <v>-3.263</v>
+        <v>-3.241</v>
       </c>
     </row>
     <row r="147">
@@ -80632,7 +81687,7 @@
         </is>
       </c>
       <c r="E147" t="n">
-        <v>-4.567</v>
+        <v>-4.547</v>
       </c>
     </row>
     <row r="148">
@@ -80655,7 +81710,7 @@
         </is>
       </c>
       <c r="E148" t="n">
-        <v>-7.404</v>
+        <v>-7.402</v>
       </c>
     </row>
     <row r="149">
@@ -80678,7 +81733,7 @@
         </is>
       </c>
       <c r="E149" t="n">
-        <v>-7.82</v>
+        <v>-7.833</v>
       </c>
     </row>
     <row r="150">
@@ -80701,7 +81756,7 @@
         </is>
       </c>
       <c r="E150" t="n">
-        <v>-8.949999999999999</v>
+        <v>-8.933</v>
       </c>
     </row>
     <row r="151">
@@ -80724,7 +81779,7 @@
         </is>
       </c>
       <c r="E151" t="n">
-        <v>-11.928</v>
+        <v>-11.905</v>
       </c>
     </row>
   </sheetData>
@@ -81618,7 +82673,7 @@
         <v>3705</v>
       </c>
       <c r="D16" t="n">
-        <v>0.01778</v>
+        <v>0.01777</v>
       </c>
       <c r="E16" t="n">
         <v>0.04655</v>
@@ -83704,10 +84759,10 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>-0.1831</v>
+        <v>-0.183</v>
       </c>
       <c r="C16" t="n">
-        <v>1.0182</v>
+        <v>1.0181</v>
       </c>
     </row>
   </sheetData>
@@ -83777,13 +84832,13 @@
         <v>13.8</v>
       </c>
       <c r="D2" t="n">
-        <v>5.24</v>
+        <v>5.26</v>
       </c>
       <c r="E2" t="n">
         <v>3.4</v>
       </c>
       <c r="F2" t="n">
-        <v>1.84</v>
+        <v>1.86</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-09-30T23:43Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-30 22:24 UTC</t>
+          <t>Genere le 2026-09-30 23:43 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-30 22:24 UTC</t>
+          <t>Rapport global — 2026-09-30 23:43 UTC</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>**Matieres premieres macro** — le ratio cuivre/or monte -- la croissance domine la peur (+5.6% sur 3 mois). Brent 97.7$ (+36.6% sur 3 mois, +45.8% sur 12 mois), gaz -6.6% sur 3 mois, ecart Brent-WTI +7.5$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-30)_</t>
+          <t>**Matieres premieres macro** — le ratio cuivre/or monte -- la croissance domine la peur (+5.6% sur 3 mois). Brent 97.7$ (+36.5% sur 3 mois, +45.7% sur 12 mois), gaz -6.6% sur 3 mois, ecart Brent-WTI +7.6$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-30)_</t>
         </is>
       </c>
     </row>
@@ -41719,10 +41719,10 @@
         <v>1.113</v>
       </c>
       <c r="D8" t="n">
-        <v>0.326</v>
+        <v>0.405</v>
       </c>
       <c r="E8" t="n">
-        <v>5e-05</v>
+        <v>0</v>
       </c>
       <c r="F8" t="n">
         <v>150</v>
@@ -41748,10 +41748,10 @@
         <v>-1.591</v>
       </c>
       <c r="D9" t="n">
-        <v>0.065</v>
+        <v>0.14</v>
       </c>
       <c r="E9" t="n">
-        <v>0.4176</v>
+        <v>0.07877000000000001</v>
       </c>
       <c r="F9" t="n">
         <v>158</v>
@@ -53682,7 +53682,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>marches/indices/DAX.csv</t>
+          <t>marches/fx/USDCNY.csv</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -53700,7 +53700,7 @@
         <v>42</v>
       </c>
       <c r="F215" t="n">
-        <v>3801</v>
+        <v>3903</v>
       </c>
       <c r="G215" t="inlineStr">
         <is>
@@ -53711,7 +53711,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>marches/indices/EUROSTOXX50.csv</t>
+          <t>marches/indices/DAX.csv</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -53729,7 +53729,7 @@
         <v>42</v>
       </c>
       <c r="F216" t="n">
-        <v>3758</v>
+        <v>3801</v>
       </c>
       <c r="G216" t="inlineStr">
         <is>
@@ -53740,7 +53740,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>marches/indices/HANGSENG.csv</t>
+          <t>marches/indices/EUROSTOXX50.csv</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -53758,7 +53758,7 @@
         <v>42</v>
       </c>
       <c r="F217" t="n">
-        <v>3689</v>
+        <v>3758</v>
       </c>
       <c r="G217" t="inlineStr">
         <is>
@@ -53769,7 +53769,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>marches/indices/KOSPI.csv</t>
+          <t>marches/indices/FTSE100.csv</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -53787,7 +53787,7 @@
         <v>42</v>
       </c>
       <c r="F218" t="n">
-        <v>3680</v>
+        <v>3787</v>
       </c>
       <c r="G218" t="inlineStr">
         <is>
@@ -53798,7 +53798,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>marches/indices/NIKKEI225.csv</t>
+          <t>marches/indices/HANGSENG.csv</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -53816,7 +53816,7 @@
         <v>42</v>
       </c>
       <c r="F219" t="n">
-        <v>3666</v>
+        <v>3689</v>
       </c>
       <c r="G219" t="inlineStr">
         <is>
@@ -53827,7 +53827,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_10A.csv</t>
+          <t>marches/indices/KOSPI.csv</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -53845,7 +53845,7 @@
         <v>42</v>
       </c>
       <c r="F220" t="n">
-        <v>9204</v>
+        <v>3680</v>
       </c>
       <c r="G220" t="inlineStr">
         <is>
@@ -53856,7 +53856,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_2A.csv</t>
+          <t>marches/indices/NIKKEI225.csv</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -53874,7 +53874,7 @@
         <v>42</v>
       </c>
       <c r="F221" t="n">
-        <v>9204</v>
+        <v>3666</v>
       </c>
       <c r="G221" t="inlineStr">
         <is>
@@ -53885,7 +53885,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_5A.csv</t>
+          <t>souverains/SUEDE_10A.csv</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -53903,7 +53903,7 @@
         <v>42</v>
       </c>
       <c r="F222" t="n">
-        <v>9206</v>
+        <v>9204</v>
       </c>
       <c r="G222" t="inlineStr">
         <is>
@@ -53914,7 +53914,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
+          <t>souverains/SUEDE_2A.csv</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -53932,7 +53932,7 @@
         <v>42</v>
       </c>
       <c r="F223" t="n">
-        <v>5641</v>
+        <v>9204</v>
       </c>
       <c r="G223" t="inlineStr">
         <is>
@@ -53943,7 +53943,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
+          <t>souverains/SUEDE_5A.csv</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -53961,7 +53961,7 @@
         <v>42</v>
       </c>
       <c r="F224" t="n">
-        <v>5641</v>
+        <v>9206</v>
       </c>
       <c r="G224" t="inlineStr">
         <is>
@@ -53972,7 +53972,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
@@ -54001,7 +54001,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -54030,7 +54030,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -54059,7 +54059,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -54088,7 +54088,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -54117,7 +54117,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -54146,7 +54146,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -54175,7 +54175,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>tresor_us/dette_quotidienne.csv</t>
+          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
@@ -54193,7 +54193,7 @@
         <v>42</v>
       </c>
       <c r="F232" t="n">
-        <v>2000</v>
+        <v>5641</v>
       </c>
       <c r="G232" t="inlineStr">
         <is>
@@ -54204,7 +54204,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>tresor_us/solde_tresorerie.csv</t>
+          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
@@ -54222,7 +54222,7 @@
         <v>42</v>
       </c>
       <c r="F233" t="n">
-        <v>500</v>
+        <v>5641</v>
       </c>
       <c r="G233" t="inlineStr">
         <is>
@@ -54233,16 +54233,16 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>fred/ECBDFR.csv</t>
+          <t>tresor_us/dette_quotidienne.csv</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C234" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D234" t="n">
         <v>1</v>
@@ -54251,7 +54251,7 @@
         <v>42</v>
       </c>
       <c r="F234" t="n">
-        <v>3000</v>
+        <v>2000</v>
       </c>
       <c r="G234" t="inlineStr">
         <is>
@@ -54262,16 +54262,16 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>fred/RRPONTSYD.csv</t>
+          <t>tresor_us/solde_tresorerie.csv</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C235" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D235" t="n">
         <v>1</v>
@@ -54280,7 +54280,7 @@
         <v>42</v>
       </c>
       <c r="F235" t="n">
-        <v>3000</v>
+        <v>500</v>
       </c>
       <c r="G235" t="inlineStr">
         <is>
@@ -54291,7 +54291,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>fred/T10YIE.csv</t>
+          <t>fred/ECBDFR.csv</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -54320,7 +54320,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>marches/fx/AUDJPY.csv</t>
+          <t>fred/RRPONTSYD.csv</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
@@ -54338,7 +54338,7 @@
         <v>42</v>
       </c>
       <c r="F237" t="n">
-        <v>3909</v>
+        <v>3000</v>
       </c>
       <c r="G237" t="inlineStr">
         <is>
@@ -54349,7 +54349,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>marches/fx/AUDUSD.csv</t>
+          <t>fred/T10YIE.csv</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
@@ -54367,7 +54367,7 @@
         <v>42</v>
       </c>
       <c r="F238" t="n">
-        <v>3905</v>
+        <v>3000</v>
       </c>
       <c r="G238" t="inlineStr">
         <is>
@@ -54378,7 +54378,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>marches/fx/DXY.csv</t>
+          <t>marches/fx/AUDJPY.csv</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
@@ -54396,7 +54396,7 @@
         <v>42</v>
       </c>
       <c r="F239" t="n">
-        <v>3772</v>
+        <v>3908</v>
       </c>
       <c r="G239" t="inlineStr">
         <is>
@@ -54407,7 +54407,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>marches/fx/EURCHF.csv</t>
+          <t>marches/fx/AUDUSD.csv</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
@@ -54425,7 +54425,7 @@
         <v>42</v>
       </c>
       <c r="F240" t="n">
-        <v>3906</v>
+        <v>3904</v>
       </c>
       <c r="G240" t="inlineStr">
         <is>
@@ -54436,7 +54436,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>marches/fx/EURGBP.csv</t>
+          <t>marches/fx/DXY.csv</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
@@ -54454,7 +54454,7 @@
         <v>42</v>
       </c>
       <c r="F241" t="n">
-        <v>3908</v>
+        <v>3772</v>
       </c>
       <c r="G241" t="inlineStr">
         <is>
@@ -54465,7 +54465,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>marches/fx/EURJPY.csv</t>
+          <t>marches/fx/EURCHF.csv</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
@@ -54483,7 +54483,7 @@
         <v>42</v>
       </c>
       <c r="F242" t="n">
-        <v>3908</v>
+        <v>3905</v>
       </c>
       <c r="G242" t="inlineStr">
         <is>
@@ -54494,7 +54494,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>marches/fx/EURUSD.csv</t>
+          <t>marches/fx/EURGBP.csv</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
@@ -54512,7 +54512,7 @@
         <v>42</v>
       </c>
       <c r="F243" t="n">
-        <v>3905</v>
+        <v>3907</v>
       </c>
       <c r="G243" t="inlineStr">
         <is>
@@ -54523,7 +54523,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>marches/fx/GBPUSD.csv</t>
+          <t>marches/fx/EURJPY.csv</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -54541,7 +54541,7 @@
         <v>42</v>
       </c>
       <c r="F244" t="n">
-        <v>3906</v>
+        <v>3907</v>
       </c>
       <c r="G244" t="inlineStr">
         <is>
@@ -54552,7 +54552,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>marches/fx/NZDUSD.csv</t>
+          <t>marches/fx/EURUSD.csv</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -54570,7 +54570,7 @@
         <v>42</v>
       </c>
       <c r="F245" t="n">
-        <v>3906</v>
+        <v>3904</v>
       </c>
       <c r="G245" t="inlineStr">
         <is>
@@ -54581,7 +54581,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>marches/fx/USDCAD.csv</t>
+          <t>marches/fx/GBPUSD.csv</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -54610,7 +54610,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>marches/fx/USDCHF.csv</t>
+          <t>marches/fx/NZDUSD.csv</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
@@ -54628,7 +54628,7 @@
         <v>42</v>
       </c>
       <c r="F247" t="n">
-        <v>3903</v>
+        <v>3905</v>
       </c>
       <c r="G247" t="inlineStr">
         <is>
@@ -54639,7 +54639,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>marches/fx/USDCNY.csv</t>
+          <t>marches/fx/USDCAD.csv</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
@@ -54657,7 +54657,7 @@
         <v>42</v>
       </c>
       <c r="F248" t="n">
-        <v>3905</v>
+        <v>3904</v>
       </c>
       <c r="G248" t="inlineStr">
         <is>
@@ -54668,7 +54668,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>marches/fx/USDJPY.csv</t>
+          <t>marches/fx/USDCHF.csv</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
@@ -54686,7 +54686,7 @@
         <v>42</v>
       </c>
       <c r="F249" t="n">
-        <v>3906</v>
+        <v>3902</v>
       </c>
       <c r="G249" t="inlineStr">
         <is>
@@ -54697,7 +54697,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>marches/fx/USDKRW.csv</t>
+          <t>marches/fx/USDJPY.csv</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
@@ -54726,7 +54726,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>marches/fx/USDNOK.csv</t>
+          <t>marches/fx/USDKRW.csv</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
@@ -54744,7 +54744,7 @@
         <v>42</v>
       </c>
       <c r="F251" t="n">
-        <v>3906</v>
+        <v>3904</v>
       </c>
       <c r="G251" t="inlineStr">
         <is>
@@ -54755,7 +54755,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>marches/fx/USDSEK.csv</t>
+          <t>marches/fx/USDNOK.csv</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -54773,7 +54773,7 @@
         <v>42</v>
       </c>
       <c r="F252" t="n">
-        <v>3906</v>
+        <v>3905</v>
       </c>
       <c r="G252" t="inlineStr">
         <is>
@@ -54784,7 +54784,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>marches/indices/FTSE100.csv</t>
+          <t>marches/fx/USDSEK.csv</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -54802,7 +54802,7 @@
         <v>42</v>
       </c>
       <c r="F253" t="n">
-        <v>3788</v>
+        <v>3905</v>
       </c>
       <c r="G253" t="inlineStr">
         <is>
@@ -57220,17 +57220,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>10606</v>
+        <v>10636.7</v>
       </c>
       <c r="D6" t="n">
-        <v>1.22</v>
+        <v>1.33</v>
       </c>
       <c r="E6" t="n">
-        <v>13.43</v>
+        <v>14.38</v>
       </c>
     </row>
     <row r="7">
@@ -59617,22 +59617,22 @@
         <v>0.001583</v>
       </c>
       <c r="C13" t="n">
-        <v>5.56</v>
+        <v>5.57</v>
       </c>
       <c r="D13" t="n">
-        <v>97.73999999999999</v>
+        <v>97.67</v>
       </c>
       <c r="E13" t="n">
-        <v>36.57</v>
+        <v>36.47</v>
       </c>
       <c r="F13" t="n">
-        <v>45.84</v>
+        <v>45.73</v>
       </c>
       <c r="G13" t="n">
-        <v>-6.55</v>
+        <v>-6.65</v>
       </c>
       <c r="H13" t="n">
-        <v>7.51</v>
+        <v>7.58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Recherche - mise a jour complete 2026-10-01T01:41Z
</commit_message>
<xml_diff>
--- a/rapports/etat-recherche.xlsx
+++ b/rapports/etat-recherche.xlsx
@@ -554,7 +554,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Genere le 2026-09-30 23:43 UTC</t>
+          <t>Genere le 2026-10-01 01:41 UTC</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Rapport global — 2026-09-30 23:43 UTC</t>
+          <t>Rapport global — 2026-10-01 01:41 UTC</t>
         </is>
       </c>
     </row>
@@ -799,7 +799,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>**Matieres premieres macro** — le ratio cuivre/or monte -- la croissance domine la peur (+5.6% sur 3 mois). Brent 97.7$ (+36.5% sur 3 mois, +45.7% sur 12 mois), gaz -6.6% sur 3 mois, ecart Brent-WTI +7.6$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-09-30)_</t>
+          <t>**Matieres premieres macro** — le ratio cuivre/or monte -- la croissance domine la peur (+6.6% sur 3 mois). Brent 97.9$ (+36.4% sur 3 mois, +49.8% sur 12 mois), gaz -6.3% sur 3 mois, ecart Brent-WTI +7.8$ -- energie nettement plus chere sur un an -- pression inflationniste a venir que les prix a la consommation ne montrent pas encore _(observation : 2026-10-01)_</t>
         </is>
       </c>
     </row>
@@ -869,7 +869,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>**Emission tresor us** — 84 derniers jours, 7785 Mds$ offerts : court (moins d'un an) 6755 Mds$ (87%), intermediaire (2 a 10 ans) 911 Mds$ (12%), long (20 a 30 ans) 119 Mds$ (2%) -- financement concentre sur le court et l'intermediaire, part longue a 2% -- peu de pression par la duration _(observation : date non exposee)_</t>
+          <t>**Emission tresor us** — 84 derniers jours, 7674 Mds$ offerts : court (moins d'un an) 6683 Mds$ (87%), intermediaire (2 a 10 ans) 872 Mds$ (11%), long (20 a 30 ans) 119 Mds$ (2%) -- financement concentre sur le court et l'intermediaire, part longue a 2% -- peu de pression par la duration _(observation : date non exposee)_</t>
         </is>
       </c>
     </row>
@@ -960,7 +960,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>**Indices mondiaux** — 7 indices (devise locale) : Coree (KOSPI) +100.2% en tete sur 12 mois, Hong Kong (Hang Seng) -7.9% en queue -- ecart tres large entre blocs sur 12 mois (108pt) -- les cycles economiques ou les flux divergent nettement. ROTATION en cours : Coree (KOSPI) mene sur 12 mois mais Hong Kong (Hang Seng) a repris la tete sur 3 mois _(observation : 2026-09-30)_</t>
+          <t>**Indices mondiaux** — 7 indices (devise locale) : Coree (KOSPI) +97.7% en tete sur 12 mois, Hong Kong (Hang Seng) -8.3% en queue -- ecart tres large entre blocs sur 12 mois (106pt) -- les cycles economiques ou les flux divergent nettement. ROTATION en cours : Coree (KOSPI) mene sur 12 mois mais Hong Kong (Hang Seng) a repris la tete sur 3 mois _(observation : 2026-10-01)_</t>
         </is>
       </c>
     </row>
@@ -14948,7 +14948,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -43496,13 +43496,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C2" t="n">
-        <v>6755</v>
+        <v>6683</v>
       </c>
       <c r="D2" t="n">
-        <v>86.8</v>
+        <v>87.09999999999999</v>
       </c>
       <c r="E2" t="n">
         <v>2.85</v>
@@ -43515,16 +43515,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C3" t="n">
-        <v>911</v>
+        <v>872</v>
       </c>
       <c r="D3" t="n">
-        <v>11.7</v>
+        <v>11.4</v>
       </c>
       <c r="E3" t="n">
-        <v>2.59</v>
+        <v>2.56</v>
       </c>
     </row>
     <row r="4">
@@ -43540,7 +43540,7 @@
         <v>119</v>
       </c>
       <c r="D4" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="E4" t="n">
         <v>2.57</v>
@@ -47514,7 +47514,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D2" t="n">
         <v>91.5</v>
@@ -47543,7 +47543,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D3" t="n">
         <v>91.5</v>
@@ -47572,7 +47572,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D4" t="n">
         <v>91.5</v>
@@ -47601,7 +47601,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D5" t="n">
         <v>91.5</v>
@@ -47630,7 +47630,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D6" t="n">
         <v>91.5</v>
@@ -47659,7 +47659,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D7" t="n">
         <v>91.5</v>
@@ -47688,7 +47688,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D8" t="n">
         <v>91.5</v>
@@ -47717,7 +47717,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D9" t="n">
         <v>91.5</v>
@@ -47746,7 +47746,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D10" t="n">
         <v>91.5</v>
@@ -47775,7 +47775,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D11" t="n">
         <v>91.5</v>
@@ -47804,7 +47804,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D12" t="n">
         <v>91.5</v>
@@ -47833,7 +47833,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D13" t="n">
         <v>91.5</v>
@@ -47862,7 +47862,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D14" t="n">
         <v>91.5</v>
@@ -47891,7 +47891,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D15" t="n">
         <v>91.5</v>
@@ -47920,7 +47920,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D16" t="n">
         <v>92</v>
@@ -47949,7 +47949,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D17" t="n">
         <v>91.5</v>
@@ -47978,7 +47978,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D18" t="n">
         <v>91.5</v>
@@ -48007,7 +48007,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D19" t="n">
         <v>91.5</v>
@@ -48036,7 +48036,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D20" t="n">
         <v>91.5</v>
@@ -48065,7 +48065,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D21" t="n">
         <v>91.5</v>
@@ -48094,7 +48094,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D22" t="n">
         <v>91.5</v>
@@ -48123,7 +48123,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D23" t="n">
         <v>91.5</v>
@@ -48152,7 +48152,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D24" t="n">
         <v>91.5</v>
@@ -48181,7 +48181,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D25" t="n">
         <v>91</v>
@@ -48210,7 +48210,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D26" t="n">
         <v>31</v>
@@ -48239,7 +48239,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D27" t="n">
         <v>31</v>
@@ -48268,7 +48268,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D28" t="n">
         <v>31</v>
@@ -48297,7 +48297,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D29" t="n">
         <v>31</v>
@@ -48326,7 +48326,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D30" t="n">
         <v>31</v>
@@ -48355,7 +48355,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D31" t="n">
         <v>31</v>
@@ -48384,7 +48384,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D32" t="n">
         <v>31</v>
@@ -48413,7 +48413,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D33" t="n">
         <v>31</v>
@@ -48442,7 +48442,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D34" t="n">
         <v>31</v>
@@ -48471,7 +48471,7 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D35" t="n">
         <v>31</v>
@@ -48500,7 +48500,7 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D36" t="n">
         <v>31</v>
@@ -48529,7 +48529,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D37" t="n">
         <v>31</v>
@@ -48558,7 +48558,7 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D38" t="n">
         <v>31</v>
@@ -48587,7 +48587,7 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D39" t="n">
         <v>31</v>
@@ -48616,7 +48616,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D40" t="n">
         <v>31</v>
@@ -48645,7 +48645,7 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D41" t="n">
         <v>31</v>
@@ -48674,7 +48674,7 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D42" t="n">
         <v>31</v>
@@ -48703,7 +48703,7 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D43" t="n">
         <v>31</v>
@@ -48732,7 +48732,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D44" t="n">
         <v>31</v>
@@ -48761,7 +48761,7 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D45" t="n">
         <v>31</v>
@@ -48790,7 +48790,7 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D46" t="n">
         <v>31</v>
@@ -48819,7 +48819,7 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D47" t="n">
         <v>31</v>
@@ -48848,7 +48848,7 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D48" t="n">
         <v>31</v>
@@ -48877,7 +48877,7 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D49" t="n">
         <v>31</v>
@@ -48906,7 +48906,7 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D50" t="n">
         <v>31</v>
@@ -48935,7 +48935,7 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D51" t="n">
         <v>31</v>
@@ -48964,7 +48964,7 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D52" t="n">
         <v>31</v>
@@ -48993,7 +48993,7 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D53" t="n">
         <v>31</v>
@@ -49022,7 +49022,7 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D54" t="n">
         <v>31</v>
@@ -49051,7 +49051,7 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D55" t="n">
         <v>31</v>
@@ -49080,7 +49080,7 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D56" t="n">
         <v>31</v>
@@ -49109,7 +49109,7 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D57" t="n">
         <v>31</v>
@@ -49138,7 +49138,7 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D58" t="n">
         <v>31</v>
@@ -49167,7 +49167,7 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D59" t="n">
         <v>31</v>
@@ -49196,7 +49196,7 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D60" t="n">
         <v>31</v>
@@ -49225,7 +49225,7 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D61" t="n">
         <v>31</v>
@@ -49254,7 +49254,7 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D62" t="n">
         <v>31</v>
@@ -49283,7 +49283,7 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D63" t="n">
         <v>31</v>
@@ -49312,7 +49312,7 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D64" t="n">
         <v>31</v>
@@ -49341,7 +49341,7 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D65" t="n">
         <v>31</v>
@@ -49370,7 +49370,7 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D66" t="n">
         <v>31</v>
@@ -49399,7 +49399,7 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D67" t="n">
         <v>31</v>
@@ -49428,7 +49428,7 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D68" t="n">
         <v>31</v>
@@ -49457,7 +49457,7 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D69" t="n">
         <v>31</v>
@@ -49486,7 +49486,7 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D70" t="n">
         <v>31</v>
@@ -49515,7 +49515,7 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D71" t="n">
         <v>31</v>
@@ -49544,7 +49544,7 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D72" t="n">
         <v>31</v>
@@ -49573,7 +49573,7 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D73" t="n">
         <v>31</v>
@@ -49602,7 +49602,7 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D74" t="n">
         <v>31</v>
@@ -49631,7 +49631,7 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D75" t="n">
         <v>31</v>
@@ -49660,7 +49660,7 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D76" t="n">
         <v>31</v>
@@ -49689,7 +49689,7 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D77" t="n">
         <v>31</v>
@@ -49718,7 +49718,7 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D78" t="n">
         <v>31</v>
@@ -49747,7 +49747,7 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D79" t="n">
         <v>31</v>
@@ -49776,7 +49776,7 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D80" t="n">
         <v>31</v>
@@ -49805,7 +49805,7 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D81" t="n">
         <v>31</v>
@@ -49834,7 +49834,7 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D82" t="n">
         <v>31</v>
@@ -49863,7 +49863,7 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D83" t="n">
         <v>31</v>
@@ -49892,7 +49892,7 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D84" t="n">
         <v>31</v>
@@ -49921,7 +49921,7 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D85" t="n">
         <v>31</v>
@@ -49950,7 +49950,7 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D86" t="n">
         <v>31</v>
@@ -49979,7 +49979,7 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D87" t="n">
         <v>31</v>
@@ -50008,7 +50008,7 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D88" t="n">
         <v>31</v>
@@ -50037,7 +50037,7 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D89" t="n">
         <v>31</v>
@@ -50066,7 +50066,7 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D90" t="n">
         <v>1</v>
@@ -50095,7 +50095,7 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D91" t="n">
         <v>1</v>
@@ -50124,7 +50124,7 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D92" t="n">
         <v>1</v>
@@ -50153,7 +50153,7 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D93" t="n">
         <v>1</v>
@@ -50182,7 +50182,7 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D94" t="n">
         <v>1</v>
@@ -50211,7 +50211,7 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D95" t="n">
         <v>31</v>
@@ -50240,7 +50240,7 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D96" t="n">
         <v>31</v>
@@ -50269,7 +50269,7 @@
         </is>
       </c>
       <c r="C97" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D97" t="n">
         <v>31</v>
@@ -50298,7 +50298,7 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D98" t="n">
         <v>31</v>
@@ -50327,7 +50327,7 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D99" t="n">
         <v>31</v>
@@ -50356,7 +50356,7 @@
         </is>
       </c>
       <c r="C100" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D100" t="n">
         <v>31</v>
@@ -50385,7 +50385,7 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D101" t="n">
         <v>31</v>
@@ -50414,7 +50414,7 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D102" t="n">
         <v>1</v>
@@ -50443,7 +50443,7 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D103" t="n">
         <v>7</v>
@@ -50472,7 +50472,7 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D104" t="n">
         <v>1</v>
@@ -50501,7 +50501,7 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D105" t="n">
         <v>1</v>
@@ -50530,7 +50530,7 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D106" t="n">
         <v>1</v>
@@ -50559,7 +50559,7 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D107" t="n">
         <v>7</v>
@@ -50588,7 +50588,7 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D108" t="n">
         <v>1</v>
@@ -50617,7 +50617,7 @@
         </is>
       </c>
       <c r="C109" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D109" t="n">
         <v>1</v>
@@ -50646,7 +50646,7 @@
         </is>
       </c>
       <c r="C110" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D110" t="n">
         <v>1</v>
@@ -50675,7 +50675,7 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D111" t="n">
         <v>1</v>
@@ -50704,7 +50704,7 @@
         </is>
       </c>
       <c r="C112" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D112" t="n">
         <v>1</v>
@@ -50733,7 +50733,7 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D113" t="n">
         <v>1</v>
@@ -50762,7 +50762,7 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D114" t="n">
         <v>1</v>
@@ -50791,7 +50791,7 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D115" t="n">
         <v>7</v>
@@ -50820,7 +50820,7 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D116" t="n">
         <v>7</v>
@@ -50849,7 +50849,7 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D117" t="n">
         <v>7</v>
@@ -50878,7 +50878,7 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D118" t="n">
         <v>7</v>
@@ -50907,7 +50907,7 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D119" t="n">
         <v>7</v>
@@ -50936,7 +50936,7 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D120" t="n">
         <v>7</v>
@@ -50965,7 +50965,7 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D121" t="n">
         <v>7</v>
@@ -50994,7 +50994,7 @@
         </is>
       </c>
       <c r="C122" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D122" t="n">
         <v>7</v>
@@ -51023,7 +51023,7 @@
         </is>
       </c>
       <c r="C123" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D123" t="n">
         <v>7</v>
@@ -51052,7 +51052,7 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D124" t="n">
         <v>7</v>
@@ -51081,7 +51081,7 @@
         </is>
       </c>
       <c r="C125" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D125" t="n">
         <v>7</v>
@@ -51110,7 +51110,7 @@
         </is>
       </c>
       <c r="C126" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D126" t="n">
         <v>7</v>
@@ -51139,7 +51139,7 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D127" t="n">
         <v>7</v>
@@ -51168,7 +51168,7 @@
         </is>
       </c>
       <c r="C128" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D128" t="n">
         <v>7</v>
@@ -51197,7 +51197,7 @@
         </is>
       </c>
       <c r="C129" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D129" t="n">
         <v>7</v>
@@ -51226,7 +51226,7 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D130" t="n">
         <v>7</v>
@@ -51255,7 +51255,7 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D131" t="n">
         <v>7</v>
@@ -51284,7 +51284,7 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D132" t="n">
         <v>7</v>
@@ -51313,7 +51313,7 @@
         </is>
       </c>
       <c r="C133" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D133" t="n">
         <v>7</v>
@@ -51342,7 +51342,7 @@
         </is>
       </c>
       <c r="C134" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D134" t="n">
         <v>7</v>
@@ -51371,7 +51371,7 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D135" t="n">
         <v>7</v>
@@ -51400,7 +51400,7 @@
         </is>
       </c>
       <c r="C136" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D136" t="n">
         <v>7</v>
@@ -51429,7 +51429,7 @@
         </is>
       </c>
       <c r="C137" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D137" t="n">
         <v>7</v>
@@ -51458,7 +51458,7 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D138" t="n">
         <v>7</v>
@@ -51487,7 +51487,7 @@
         </is>
       </c>
       <c r="C139" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D139" t="n">
         <v>7</v>
@@ -51516,7 +51516,7 @@
         </is>
       </c>
       <c r="C140" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D140" t="n">
         <v>7</v>
@@ -51545,7 +51545,7 @@
         </is>
       </c>
       <c r="C141" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D141" t="n">
         <v>7</v>
@@ -51574,7 +51574,7 @@
         </is>
       </c>
       <c r="C142" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D142" t="n">
         <v>7</v>
@@ -51603,7 +51603,7 @@
         </is>
       </c>
       <c r="C143" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D143" t="n">
         <v>7</v>
@@ -51632,7 +51632,7 @@
         </is>
       </c>
       <c r="C144" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D144" t="n">
         <v>7</v>
@@ -51661,7 +51661,7 @@
         </is>
       </c>
       <c r="C145" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D145" t="n">
         <v>7</v>
@@ -51690,7 +51690,7 @@
         </is>
       </c>
       <c r="C146" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D146" t="n">
         <v>7</v>
@@ -51719,7 +51719,7 @@
         </is>
       </c>
       <c r="C147" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D147" t="n">
         <v>7</v>
@@ -51748,7 +51748,7 @@
         </is>
       </c>
       <c r="C148" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D148" t="n">
         <v>7</v>
@@ -51777,7 +51777,7 @@
         </is>
       </c>
       <c r="C149" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D149" t="n">
         <v>7</v>
@@ -51806,7 +51806,7 @@
         </is>
       </c>
       <c r="C150" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D150" t="n">
         <v>7</v>
@@ -51835,7 +51835,7 @@
         </is>
       </c>
       <c r="C151" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D151" t="n">
         <v>7</v>
@@ -51864,7 +51864,7 @@
         </is>
       </c>
       <c r="C152" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D152" t="n">
         <v>7</v>
@@ -51893,7 +51893,7 @@
         </is>
       </c>
       <c r="C153" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D153" t="n">
         <v>7</v>
@@ -51922,7 +51922,7 @@
         </is>
       </c>
       <c r="C154" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D154" t="n">
         <v>7</v>
@@ -51951,7 +51951,7 @@
         </is>
       </c>
       <c r="C155" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D155" t="n">
         <v>7</v>
@@ -51980,7 +51980,7 @@
         </is>
       </c>
       <c r="C156" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D156" t="n">
         <v>7</v>
@@ -52009,7 +52009,7 @@
         </is>
       </c>
       <c r="C157" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D157" t="n">
         <v>7</v>
@@ -52038,7 +52038,7 @@
         </is>
       </c>
       <c r="C158" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D158" t="n">
         <v>7</v>
@@ -52067,7 +52067,7 @@
         </is>
       </c>
       <c r="C159" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D159" t="n">
         <v>7</v>
@@ -52096,7 +52096,7 @@
         </is>
       </c>
       <c r="C160" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D160" t="n">
         <v>7</v>
@@ -52125,7 +52125,7 @@
         </is>
       </c>
       <c r="C161" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D161" t="n">
         <v>7</v>
@@ -52154,7 +52154,7 @@
         </is>
       </c>
       <c r="C162" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D162" t="n">
         <v>7</v>
@@ -52183,7 +52183,7 @@
         </is>
       </c>
       <c r="C163" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D163" t="n">
         <v>7</v>
@@ -52212,7 +52212,7 @@
         </is>
       </c>
       <c r="C164" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D164" t="n">
         <v>7</v>
@@ -52241,7 +52241,7 @@
         </is>
       </c>
       <c r="C165" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D165" t="n">
         <v>7</v>
@@ -52270,7 +52270,7 @@
         </is>
       </c>
       <c r="C166" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D166" t="n">
         <v>7</v>
@@ -52299,7 +52299,7 @@
         </is>
       </c>
       <c r="C167" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D167" t="n">
         <v>7</v>
@@ -52328,7 +52328,7 @@
         </is>
       </c>
       <c r="C168" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D168" t="n">
         <v>7</v>
@@ -52357,7 +52357,7 @@
         </is>
       </c>
       <c r="C169" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D169" t="n">
         <v>7</v>
@@ -52386,7 +52386,7 @@
         </is>
       </c>
       <c r="C170" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D170" t="n">
         <v>7</v>
@@ -52415,7 +52415,7 @@
         </is>
       </c>
       <c r="C171" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D171" t="n">
         <v>7</v>
@@ -52444,7 +52444,7 @@
         </is>
       </c>
       <c r="C172" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D172" t="n">
         <v>7</v>
@@ -52473,7 +52473,7 @@
         </is>
       </c>
       <c r="C173" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D173" t="n">
         <v>7</v>
@@ -52502,7 +52502,7 @@
         </is>
       </c>
       <c r="C174" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D174" t="n">
         <v>7</v>
@@ -52531,7 +52531,7 @@
         </is>
       </c>
       <c r="C175" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D175" t="n">
         <v>7</v>
@@ -52560,7 +52560,7 @@
         </is>
       </c>
       <c r="C176" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D176" t="n">
         <v>7</v>
@@ -52589,7 +52589,7 @@
         </is>
       </c>
       <c r="C177" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D177" t="n">
         <v>7</v>
@@ -52618,7 +52618,7 @@
         </is>
       </c>
       <c r="C178" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D178" t="n">
         <v>7</v>
@@ -52647,7 +52647,7 @@
         </is>
       </c>
       <c r="C179" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D179" t="n">
         <v>7</v>
@@ -52676,7 +52676,7 @@
         </is>
       </c>
       <c r="C180" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D180" t="n">
         <v>7</v>
@@ -52705,7 +52705,7 @@
         </is>
       </c>
       <c r="C181" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D181" t="n">
         <v>7</v>
@@ -52734,7 +52734,7 @@
         </is>
       </c>
       <c r="C182" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D182" t="n">
         <v>1</v>
@@ -52763,7 +52763,7 @@
         </is>
       </c>
       <c r="C183" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D183" t="n">
         <v>1</v>
@@ -52792,7 +52792,7 @@
         </is>
       </c>
       <c r="C184" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D184" t="n">
         <v>1</v>
@@ -52821,7 +52821,7 @@
         </is>
       </c>
       <c r="C185" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D185" t="n">
         <v>7</v>
@@ -52850,7 +52850,7 @@
         </is>
       </c>
       <c r="C186" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D186" t="n">
         <v>7</v>
@@ -52879,7 +52879,7 @@
         </is>
       </c>
       <c r="C187" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D187" t="n">
         <v>1</v>
@@ -52908,7 +52908,7 @@
         </is>
       </c>
       <c r="C188" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D188" t="n">
         <v>1</v>
@@ -52937,7 +52937,7 @@
         </is>
       </c>
       <c r="C189" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D189" t="n">
         <v>1</v>
@@ -52966,7 +52966,7 @@
         </is>
       </c>
       <c r="C190" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D190" t="n">
         <v>1</v>
@@ -52995,7 +52995,7 @@
         </is>
       </c>
       <c r="C191" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D191" t="n">
         <v>1</v>
@@ -53024,7 +53024,7 @@
         </is>
       </c>
       <c r="C192" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D192" t="n">
         <v>1</v>
@@ -53053,7 +53053,7 @@
         </is>
       </c>
       <c r="C193" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D193" t="n">
         <v>1</v>
@@ -53082,7 +53082,7 @@
         </is>
       </c>
       <c r="C194" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D194" t="n">
         <v>1</v>
@@ -53111,7 +53111,7 @@
         </is>
       </c>
       <c r="C195" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D195" t="n">
         <v>1</v>
@@ -53140,7 +53140,7 @@
         </is>
       </c>
       <c r="C196" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D196" t="n">
         <v>1</v>
@@ -53169,7 +53169,7 @@
         </is>
       </c>
       <c r="C197" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D197" t="n">
         <v>1</v>
@@ -53198,7 +53198,7 @@
         </is>
       </c>
       <c r="C198" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D198" t="n">
         <v>1</v>
@@ -53227,7 +53227,7 @@
         </is>
       </c>
       <c r="C199" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D199" t="n">
         <v>1</v>
@@ -53256,7 +53256,7 @@
         </is>
       </c>
       <c r="C200" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D200" t="n">
         <v>1</v>
@@ -53285,7 +53285,7 @@
         </is>
       </c>
       <c r="C201" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D201" t="n">
         <v>1</v>
@@ -53314,7 +53314,7 @@
         </is>
       </c>
       <c r="C202" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D202" t="n">
         <v>1</v>
@@ -53343,7 +53343,7 @@
         </is>
       </c>
       <c r="C203" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D203" t="n">
         <v>1</v>
@@ -53372,7 +53372,7 @@
         </is>
       </c>
       <c r="C204" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D204" t="n">
         <v>1</v>
@@ -53401,7 +53401,7 @@
         </is>
       </c>
       <c r="C205" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D205" t="n">
         <v>1</v>
@@ -53430,7 +53430,7 @@
         </is>
       </c>
       <c r="C206" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D206" t="n">
         <v>1</v>
@@ -53459,7 +53459,7 @@
         </is>
       </c>
       <c r="C207" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D207" t="n">
         <v>1</v>
@@ -53488,7 +53488,7 @@
         </is>
       </c>
       <c r="C208" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D208" t="n">
         <v>1</v>
@@ -53517,7 +53517,7 @@
         </is>
       </c>
       <c r="C209" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D209" t="n">
         <v>1</v>
@@ -53546,7 +53546,7 @@
         </is>
       </c>
       <c r="C210" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D210" t="n">
         <v>1</v>
@@ -53575,7 +53575,7 @@
         </is>
       </c>
       <c r="C211" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D211" t="n">
         <v>1</v>
@@ -53604,7 +53604,7 @@
         </is>
       </c>
       <c r="C212" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D212" t="n">
         <v>1</v>
@@ -53633,7 +53633,7 @@
         </is>
       </c>
       <c r="C213" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D213" t="n">
         <v>1</v>
@@ -53662,7 +53662,7 @@
         </is>
       </c>
       <c r="C214" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D214" t="n">
         <v>1</v>
@@ -53682,7 +53682,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>marches/fx/USDCNY.csv</t>
+          <t>souverains/SUEDE_10A.csv</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -53691,7 +53691,7 @@
         </is>
       </c>
       <c r="C215" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D215" t="n">
         <v>1</v>
@@ -53700,7 +53700,7 @@
         <v>42</v>
       </c>
       <c r="F215" t="n">
-        <v>3903</v>
+        <v>9204</v>
       </c>
       <c r="G215" t="inlineStr">
         <is>
@@ -53711,7 +53711,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>marches/indices/DAX.csv</t>
+          <t>souverains/SUEDE_2A.csv</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -53720,7 +53720,7 @@
         </is>
       </c>
       <c r="C216" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D216" t="n">
         <v>1</v>
@@ -53729,7 +53729,7 @@
         <v>42</v>
       </c>
       <c r="F216" t="n">
-        <v>3801</v>
+        <v>9204</v>
       </c>
       <c r="G216" t="inlineStr">
         <is>
@@ -53740,7 +53740,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>marches/indices/EUROSTOXX50.csv</t>
+          <t>souverains/SUEDE_5A.csv</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -53749,7 +53749,7 @@
         </is>
       </c>
       <c r="C217" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D217" t="n">
         <v>1</v>
@@ -53758,7 +53758,7 @@
         <v>42</v>
       </c>
       <c r="F217" t="n">
-        <v>3758</v>
+        <v>9206</v>
       </c>
       <c r="G217" t="inlineStr">
         <is>
@@ -53769,7 +53769,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>marches/indices/FTSE100.csv</t>
+          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -53778,7 +53778,7 @@
         </is>
       </c>
       <c r="C218" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D218" t="n">
         <v>1</v>
@@ -53787,7 +53787,7 @@
         <v>42</v>
       </c>
       <c r="F218" t="n">
-        <v>3787</v>
+        <v>5641</v>
       </c>
       <c r="G218" t="inlineStr">
         <is>
@@ -53798,7 +53798,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>marches/indices/HANGSENG.csv</t>
+          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -53807,7 +53807,7 @@
         </is>
       </c>
       <c r="C219" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D219" t="n">
         <v>1</v>
@@ -53816,7 +53816,7 @@
         <v>42</v>
       </c>
       <c r="F219" t="n">
-        <v>3689</v>
+        <v>5641</v>
       </c>
       <c r="G219" t="inlineStr">
         <is>
@@ -53827,7 +53827,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>marches/indices/KOSPI.csv</t>
+          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -53836,7 +53836,7 @@
         </is>
       </c>
       <c r="C220" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D220" t="n">
         <v>1</v>
@@ -53845,7 +53845,7 @@
         <v>42</v>
       </c>
       <c r="F220" t="n">
-        <v>3680</v>
+        <v>5641</v>
       </c>
       <c r="G220" t="inlineStr">
         <is>
@@ -53856,7 +53856,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>marches/indices/NIKKEI225.csv</t>
+          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -53865,7 +53865,7 @@
         </is>
       </c>
       <c r="C221" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D221" t="n">
         <v>1</v>
@@ -53874,7 +53874,7 @@
         <v>42</v>
       </c>
       <c r="F221" t="n">
-        <v>3666</v>
+        <v>5641</v>
       </c>
       <c r="G221" t="inlineStr">
         <is>
@@ -53885,7 +53885,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_10A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -53894,7 +53894,7 @@
         </is>
       </c>
       <c r="C222" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D222" t="n">
         <v>1</v>
@@ -53903,7 +53903,7 @@
         <v>42</v>
       </c>
       <c r="F222" t="n">
-        <v>9204</v>
+        <v>5641</v>
       </c>
       <c r="G222" t="inlineStr">
         <is>
@@ -53914,7 +53914,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_2A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -53923,7 +53923,7 @@
         </is>
       </c>
       <c r="C223" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D223" t="n">
         <v>1</v>
@@ -53932,7 +53932,7 @@
         <v>42</v>
       </c>
       <c r="F223" t="n">
-        <v>9204</v>
+        <v>5641</v>
       </c>
       <c r="G223" t="inlineStr">
         <is>
@@ -53943,7 +53943,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>souverains/SUEDE_5A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
@@ -53952,7 +53952,7 @@
         </is>
       </c>
       <c r="C224" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D224" t="n">
         <v>1</v>
@@ -53961,7 +53961,7 @@
         <v>42</v>
       </c>
       <c r="F224" t="n">
-        <v>9206</v>
+        <v>5641</v>
       </c>
       <c r="G224" t="inlineStr">
         <is>
@@ -53972,7 +53972,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_10A.csv</t>
+          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
@@ -53981,7 +53981,7 @@
         </is>
       </c>
       <c r="C225" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D225" t="n">
         <v>1</v>
@@ -54001,7 +54001,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_1A.csv</t>
+          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -54010,7 +54010,7 @@
         </is>
       </c>
       <c r="C226" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D226" t="n">
         <v>1</v>
@@ -54030,7 +54030,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_20A.csv</t>
+          <t>tresor_us/dette_quotidienne.csv</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -54039,7 +54039,7 @@
         </is>
       </c>
       <c r="C227" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D227" t="n">
         <v>1</v>
@@ -54048,7 +54048,7 @@
         <v>42</v>
       </c>
       <c r="F227" t="n">
-        <v>5641</v>
+        <v>2000</v>
       </c>
       <c r="G227" t="inlineStr">
         <is>
@@ -54059,7 +54059,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_2A.csv</t>
+          <t>tresor_us/solde_tresorerie.csv</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -54068,7 +54068,7 @@
         </is>
       </c>
       <c r="C228" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D228" t="n">
         <v>1</v>
@@ -54077,7 +54077,7 @@
         <v>42</v>
       </c>
       <c r="F228" t="n">
-        <v>5641</v>
+        <v>500</v>
       </c>
       <c r="G228" t="inlineStr">
         <is>
@@ -54088,12 +54088,12 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_30A.csv</t>
+          <t>fred/ECBDFR.csv</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C229" t="n">
@@ -54106,7 +54106,7 @@
         <v>42</v>
       </c>
       <c r="F229" t="n">
-        <v>5641</v>
+        <v>3000</v>
       </c>
       <c r="G229" t="inlineStr">
         <is>
@@ -54117,12 +54117,12 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_3A.csv</t>
+          <t>fred/RRPONTSYD.csv</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C230" t="n">
@@ -54135,7 +54135,7 @@
         <v>42</v>
       </c>
       <c r="F230" t="n">
-        <v>5641</v>
+        <v>3000</v>
       </c>
       <c r="G230" t="inlineStr">
         <is>
@@ -54146,12 +54146,12 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_5A.csv</t>
+          <t>fred/T10YIE.csv</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C231" t="n">
@@ -54164,7 +54164,7 @@
         <v>42</v>
       </c>
       <c r="F231" t="n">
-        <v>5641</v>
+        <v>3000</v>
       </c>
       <c r="G231" t="inlineStr">
         <is>
@@ -54175,12 +54175,12 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_AAA_7A.csv</t>
+          <t>marches/indices/DAX.csv</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C232" t="n">
@@ -54193,7 +54193,7 @@
         <v>42</v>
       </c>
       <c r="F232" t="n">
-        <v>5641</v>
+        <v>3802</v>
       </c>
       <c r="G232" t="inlineStr">
         <is>
@@ -54204,12 +54204,12 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>souverains/ZONE_EURO_TOUS_10A.csv</t>
+          <t>marches/indices/EUROSTOXX50.csv</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C233" t="n">
@@ -54222,7 +54222,7 @@
         <v>42</v>
       </c>
       <c r="F233" t="n">
-        <v>5641</v>
+        <v>3759</v>
       </c>
       <c r="G233" t="inlineStr">
         <is>
@@ -54233,12 +54233,12 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>tresor_us/dette_quotidienne.csv</t>
+          <t>marches/indices/FTSE100.csv</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C234" t="n">
@@ -54251,7 +54251,7 @@
         <v>42</v>
       </c>
       <c r="F234" t="n">
-        <v>2000</v>
+        <v>3788</v>
       </c>
       <c r="G234" t="inlineStr">
         <is>
@@ -54262,12 +54262,12 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>tresor_us/solde_tresorerie.csv</t>
+          <t>marches/indices/HANGSENG.csv</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C235" t="n">
@@ -54280,7 +54280,7 @@
         <v>42</v>
       </c>
       <c r="F235" t="n">
-        <v>500</v>
+        <v>3690</v>
       </c>
       <c r="G235" t="inlineStr">
         <is>
@@ -54291,7 +54291,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>fred/ECBDFR.csv</t>
+          <t>marches/volatilite/GVZ.csv</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -54300,7 +54300,7 @@
         </is>
       </c>
       <c r="C236" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D236" t="n">
         <v>1</v>
@@ -54309,7 +54309,7 @@
         <v>42</v>
       </c>
       <c r="F236" t="n">
-        <v>3000</v>
+        <v>3770</v>
       </c>
       <c r="G236" t="inlineStr">
         <is>
@@ -54320,7 +54320,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>fred/RRPONTSYD.csv</t>
+          <t>marches/volatilite/MOVE.csv</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
@@ -54329,7 +54329,7 @@
         </is>
       </c>
       <c r="C237" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D237" t="n">
         <v>1</v>
@@ -54338,7 +54338,7 @@
         <v>42</v>
       </c>
       <c r="F237" t="n">
-        <v>3000</v>
+        <v>3689</v>
       </c>
       <c r="G237" t="inlineStr">
         <is>
@@ -54349,7 +54349,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>fred/T10YIE.csv</t>
+          <t>marches/volatilite/OVX.csv</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
@@ -54358,7 +54358,7 @@
         </is>
       </c>
       <c r="C238" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D238" t="n">
         <v>1</v>
@@ -54367,7 +54367,7 @@
         <v>42</v>
       </c>
       <c r="F238" t="n">
-        <v>3000</v>
+        <v>3770</v>
       </c>
       <c r="G238" t="inlineStr">
         <is>
@@ -54378,7 +54378,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>marches/fx/AUDJPY.csv</t>
+          <t>marches/volatilite/VVIX.csv</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
@@ -54387,7 +54387,7 @@
         </is>
       </c>
       <c r="C239" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D239" t="n">
         <v>1</v>
@@ -54396,7 +54396,7 @@
         <v>42</v>
       </c>
       <c r="F239" t="n">
-        <v>3908</v>
+        <v>3762</v>
       </c>
       <c r="G239" t="inlineStr">
         <is>
@@ -54407,7 +54407,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>marches/fx/AUDUSD.csv</t>
+          <t>marches/volatilite/VXN.csv</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
@@ -54416,7 +54416,7 @@
         </is>
       </c>
       <c r="C240" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D240" t="n">
         <v>1</v>
@@ -54425,7 +54425,7 @@
         <v>42</v>
       </c>
       <c r="F240" t="n">
-        <v>3904</v>
+        <v>3770</v>
       </c>
       <c r="G240" t="inlineStr">
         <is>
@@ -54436,7 +54436,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>marches/fx/DXY.csv</t>
+          <t>yfinance/SP500.csv</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
@@ -54445,7 +54445,7 @@
         </is>
       </c>
       <c r="C241" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D241" t="n">
         <v>1</v>
@@ -54454,7 +54454,7 @@
         <v>42</v>
       </c>
       <c r="F241" t="n">
-        <v>3772</v>
+        <v>7547</v>
       </c>
       <c r="G241" t="inlineStr">
         <is>
@@ -54465,7 +54465,7 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>marches/fx/EURCHF.csv</t>
+          <t>yfinance/VIX.csv</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
@@ -54474,7 +54474,7 @@
         </is>
       </c>
       <c r="C242" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D242" t="n">
         <v>1</v>
@@ -54483,7 +54483,7 @@
         <v>42</v>
       </c>
       <c r="F242" t="n">
-        <v>3905</v>
+        <v>7550</v>
       </c>
       <c r="G242" t="inlineStr">
         <is>
@@ -54494,7 +54494,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>marches/fx/EURGBP.csv</t>
+          <t>yfinance/XLB.csv</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
@@ -54503,7 +54503,7 @@
         </is>
       </c>
       <c r="C243" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D243" t="n">
         <v>1</v>
@@ -54512,7 +54512,7 @@
         <v>42</v>
       </c>
       <c r="F243" t="n">
-        <v>3907</v>
+        <v>501</v>
       </c>
       <c r="G243" t="inlineStr">
         <is>
@@ -54523,7 +54523,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>marches/fx/EURJPY.csv</t>
+          <t>yfinance/XLE.csv</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -54532,7 +54532,7 @@
         </is>
       </c>
       <c r="C244" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D244" t="n">
         <v>1</v>
@@ -54541,7 +54541,7 @@
         <v>42</v>
       </c>
       <c r="F244" t="n">
-        <v>3907</v>
+        <v>501</v>
       </c>
       <c r="G244" t="inlineStr">
         <is>
@@ -54552,7 +54552,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>marches/fx/EURUSD.csv</t>
+          <t>yfinance/XLF.csv</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -54561,7 +54561,7 @@
         </is>
       </c>
       <c r="C245" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D245" t="n">
         <v>1</v>
@@ -54570,7 +54570,7 @@
         <v>42</v>
       </c>
       <c r="F245" t="n">
-        <v>3904</v>
+        <v>501</v>
       </c>
       <c r="G245" t="inlineStr">
         <is>
@@ -54581,7 +54581,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>marches/fx/GBPUSD.csv</t>
+          <t>yfinance/XLI.csv</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -54590,7 +54590,7 @@
         </is>
       </c>
       <c r="C246" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D246" t="n">
         <v>1</v>
@@ -54599,7 +54599,7 @@
         <v>42</v>
       </c>
       <c r="F246" t="n">
-        <v>3905</v>
+        <v>501</v>
       </c>
       <c r="G246" t="inlineStr">
         <is>
@@ -54610,7 +54610,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>marches/fx/NZDUSD.csv</t>
+          <t>yfinance/XLK.csv</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
@@ -54619,7 +54619,7 @@
         </is>
       </c>
       <c r="C247" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D247" t="n">
         <v>1</v>
@@ -54628,7 +54628,7 @@
         <v>42</v>
       </c>
       <c r="F247" t="n">
-        <v>3905</v>
+        <v>501</v>
       </c>
       <c r="G247" t="inlineStr">
         <is>
@@ -54639,7 +54639,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>marches/fx/USDCAD.csv</t>
+          <t>yfinance/XLP.csv</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
@@ -54648,7 +54648,7 @@
         </is>
       </c>
       <c r="C248" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D248" t="n">
         <v>1</v>
@@ -54657,7 +54657,7 @@
         <v>42</v>
       </c>
       <c r="F248" t="n">
-        <v>3904</v>
+        <v>501</v>
       </c>
       <c r="G248" t="inlineStr">
         <is>
@@ -54668,7 +54668,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>marches/fx/USDCHF.csv</t>
+          <t>yfinance/XLRE.csv</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
@@ -54677,7 +54677,7 @@
         </is>
       </c>
       <c r="C249" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D249" t="n">
         <v>1</v>
@@ -54686,7 +54686,7 @@
         <v>42</v>
       </c>
       <c r="F249" t="n">
-        <v>3902</v>
+        <v>501</v>
       </c>
       <c r="G249" t="inlineStr">
         <is>
@@ -54697,7 +54697,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>marches/fx/USDJPY.csv</t>
+          <t>yfinance/XLU.csv</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
@@ -54706,7 +54706,7 @@
         </is>
       </c>
       <c r="C250" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D250" t="n">
         <v>1</v>
@@ -54715,7 +54715,7 @@
         <v>42</v>
       </c>
       <c r="F250" t="n">
-        <v>3905</v>
+        <v>501</v>
       </c>
       <c r="G250" t="inlineStr">
         <is>
@@ -54726,7 +54726,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>marches/fx/USDKRW.csv</t>
+          <t>yfinance/XLV.csv</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
@@ -54735,7 +54735,7 @@
         </is>
       </c>
       <c r="C251" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D251" t="n">
         <v>1</v>
@@ -54744,7 +54744,7 @@
         <v>42</v>
       </c>
       <c r="F251" t="n">
-        <v>3904</v>
+        <v>501</v>
       </c>
       <c r="G251" t="inlineStr">
         <is>
@@ -54755,7 +54755,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>marches/fx/USDNOK.csv</t>
+          <t>yfinance/XLY.csv</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
@@ -54764,7 +54764,7 @@
         </is>
       </c>
       <c r="C252" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D252" t="n">
         <v>1</v>
@@ -54773,7 +54773,7 @@
         <v>42</v>
       </c>
       <c r="F252" t="n">
-        <v>3905</v>
+        <v>501</v>
       </c>
       <c r="G252" t="inlineStr">
         <is>
@@ -54784,12 +54784,12 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>marches/fx/USDSEK.csv</t>
+          <t>marches/fx/AUDJPY.csv</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -54802,7 +54802,7 @@
         <v>42</v>
       </c>
       <c r="F253" t="n">
-        <v>3905</v>
+        <v>3908</v>
       </c>
       <c r="G253" t="inlineStr">
         <is>
@@ -54813,12 +54813,12 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>marches/matieres/BRENT.csv</t>
+          <t>marches/fx/AUDUSD.csv</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C254" t="n">
@@ -54831,7 +54831,7 @@
         <v>42</v>
       </c>
       <c r="F254" t="n">
-        <v>3751</v>
+        <v>3904</v>
       </c>
       <c r="G254" t="inlineStr">
         <is>
@@ -54842,12 +54842,12 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>marches/matieres/CUIVRE.csv</t>
+          <t>marches/fx/DXY.csv</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C255" t="n">
@@ -54860,7 +54860,7 @@
         <v>42</v>
       </c>
       <c r="F255" t="n">
-        <v>3771</v>
+        <v>3773</v>
       </c>
       <c r="G255" t="inlineStr">
         <is>
@@ -54871,12 +54871,12 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>marches/matieres/GAZ_HENRY_HUB.csv</t>
+          <t>marches/fx/EURCHF.csv</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C256" t="n">
@@ -54889,7 +54889,7 @@
         <v>42</v>
       </c>
       <c r="F256" t="n">
-        <v>3772</v>
+        <v>3905</v>
       </c>
       <c r="G256" t="inlineStr">
         <is>
@@ -54900,12 +54900,12 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>marches/matieres/OR.csv</t>
+          <t>marches/fx/EURGBP.csv</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -54918,7 +54918,7 @@
         <v>42</v>
       </c>
       <c r="F257" t="n">
-        <v>3771</v>
+        <v>3907</v>
       </c>
       <c r="G257" t="inlineStr">
         <is>
@@ -54929,12 +54929,12 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>marches/matieres/WTI.csv</t>
+          <t>marches/fx/EURJPY.csv</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -54947,7 +54947,7 @@
         <v>42</v>
       </c>
       <c r="F258" t="n">
-        <v>3771</v>
+        <v>3907</v>
       </c>
       <c r="G258" t="inlineStr">
         <is>
@@ -54958,12 +54958,12 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>marches/taux_futures/FED_FUNDS_FRONT.csv</t>
+          <t>marches/fx/EURUSD.csv</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C259" t="n">
@@ -54976,7 +54976,7 @@
         <v>42</v>
       </c>
       <c r="F259" t="n">
-        <v>3772</v>
+        <v>3904</v>
       </c>
       <c r="G259" t="inlineStr">
         <is>
@@ -54987,12 +54987,12 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>marches/volatilite/GVZ.csv</t>
+          <t>marches/fx/GBPUSD.csv</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C260" t="n">
@@ -55005,7 +55005,7 @@
         <v>42</v>
       </c>
       <c r="F260" t="n">
-        <v>3770</v>
+        <v>3905</v>
       </c>
       <c r="G260" t="inlineStr">
         <is>
@@ -55016,12 +55016,12 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>marches/volatilite/MOVE.csv</t>
+          <t>marches/fx/NZDUSD.csv</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C261" t="n">
@@ -55034,7 +55034,7 @@
         <v>42</v>
       </c>
       <c r="F261" t="n">
-        <v>3689</v>
+        <v>3905</v>
       </c>
       <c r="G261" t="inlineStr">
         <is>
@@ -55045,12 +55045,12 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>marches/volatilite/OVX.csv</t>
+          <t>marches/fx/USDCAD.csv</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -55063,7 +55063,7 @@
         <v>42</v>
       </c>
       <c r="F262" t="n">
-        <v>3770</v>
+        <v>3904</v>
       </c>
       <c r="G262" t="inlineStr">
         <is>
@@ -55074,12 +55074,12 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>marches/volatilite/VVIX.csv</t>
+          <t>marches/fx/USDCHF.csv</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C263" t="n">
@@ -55092,7 +55092,7 @@
         <v>42</v>
       </c>
       <c r="F263" t="n">
-        <v>3762</v>
+        <v>3902</v>
       </c>
       <c r="G263" t="inlineStr">
         <is>
@@ -55103,12 +55103,12 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>marches/volatilite/VXN.csv</t>
+          <t>marches/fx/USDCNY.csv</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C264" t="n">
@@ -55121,7 +55121,7 @@
         <v>42</v>
       </c>
       <c r="F264" t="n">
-        <v>3770</v>
+        <v>3904</v>
       </c>
       <c r="G264" t="inlineStr">
         <is>
@@ -55132,12 +55132,12 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>yfinance/SP500.csv</t>
+          <t>marches/fx/USDJPY.csv</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -55150,7 +55150,7 @@
         <v>42</v>
       </c>
       <c r="F265" t="n">
-        <v>7547</v>
+        <v>3905</v>
       </c>
       <c r="G265" t="inlineStr">
         <is>
@@ -55161,12 +55161,12 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>yfinance/VIX.csv</t>
+          <t>marches/fx/USDKRW.csv</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C266" t="n">
@@ -55179,7 +55179,7 @@
         <v>42</v>
       </c>
       <c r="F266" t="n">
-        <v>7550</v>
+        <v>3904</v>
       </c>
       <c r="G266" t="inlineStr">
         <is>
@@ -55190,12 +55190,12 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>yfinance/XLB.csv</t>
+          <t>marches/fx/USDNOK.csv</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C267" t="n">
@@ -55208,7 +55208,7 @@
         <v>42</v>
       </c>
       <c r="F267" t="n">
-        <v>501</v>
+        <v>3905</v>
       </c>
       <c r="G267" t="inlineStr">
         <is>
@@ -55219,12 +55219,12 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>yfinance/XLE.csv</t>
+          <t>marches/fx/USDSEK.csv</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -55237,7 +55237,7 @@
         <v>42</v>
       </c>
       <c r="F268" t="n">
-        <v>501</v>
+        <v>3905</v>
       </c>
       <c r="G268" t="inlineStr">
         <is>
@@ -55248,12 +55248,12 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>yfinance/XLF.csv</t>
+          <t>marches/indices/KOSPI.csv</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -55266,7 +55266,7 @@
         <v>42</v>
       </c>
       <c r="F269" t="n">
-        <v>501</v>
+        <v>3681</v>
       </c>
       <c r="G269" t="inlineStr">
         <is>
@@ -55277,12 +55277,12 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>yfinance/XLI.csv</t>
+          <t>marches/indices/NIKKEI225.csv</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -55295,7 +55295,7 @@
         <v>42</v>
       </c>
       <c r="F270" t="n">
-        <v>501</v>
+        <v>3667</v>
       </c>
       <c r="G270" t="inlineStr">
         <is>
@@ -55306,12 +55306,12 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>yfinance/XLK.csv</t>
+          <t>marches/matieres/BRENT.csv</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C271" t="n">
@@ -55324,7 +55324,7 @@
         <v>42</v>
       </c>
       <c r="F271" t="n">
-        <v>501</v>
+        <v>3751</v>
       </c>
       <c r="G271" t="inlineStr">
         <is>
@@ -55335,12 +55335,12 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>yfinance/XLP.csv</t>
+          <t>marches/matieres/CUIVRE.csv</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C272" t="n">
@@ -55353,7 +55353,7 @@
         <v>42</v>
       </c>
       <c r="F272" t="n">
-        <v>501</v>
+        <v>3771</v>
       </c>
       <c r="G272" t="inlineStr">
         <is>
@@ -55364,12 +55364,12 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>yfinance/XLRE.csv</t>
+          <t>marches/matieres/GAZ_HENRY_HUB.csv</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -55382,7 +55382,7 @@
         <v>42</v>
       </c>
       <c r="F273" t="n">
-        <v>501</v>
+        <v>3772</v>
       </c>
       <c r="G273" t="inlineStr">
         <is>
@@ -55393,12 +55393,12 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>yfinance/XLU.csv</t>
+          <t>marches/matieres/OR.csv</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C274" t="n">
@@ -55411,7 +55411,7 @@
         <v>42</v>
       </c>
       <c r="F274" t="n">
-        <v>501</v>
+        <v>3771</v>
       </c>
       <c r="G274" t="inlineStr">
         <is>
@@ -55422,12 +55422,12 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>yfinance/XLV.csv</t>
+          <t>marches/matieres/WTI.csv</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C275" t="n">
@@ -55440,7 +55440,7 @@
         <v>42</v>
       </c>
       <c r="F275" t="n">
-        <v>501</v>
+        <v>3771</v>
       </c>
       <c r="G275" t="inlineStr">
         <is>
@@ -55451,12 +55451,12 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>yfinance/XLY.csv</t>
+          <t>marches/taux_futures/FED_FUNDS_FRONT.csv</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C276" t="n">
@@ -55469,7 +55469,7 @@
         <v>42</v>
       </c>
       <c r="F276" t="n">
-        <v>501</v>
+        <v>3772</v>
       </c>
       <c r="G276" t="inlineStr">
         <is>
@@ -55489,7 +55489,7 @@
         </is>
       </c>
       <c r="C277" t="n">
-        <v>-6</v>
+        <v>-5</v>
       </c>
       <c r="D277" t="n">
         <v>2</v>
@@ -55518,7 +55518,7 @@
         </is>
       </c>
       <c r="C278" t="n">
-        <v>-433</v>
+        <v>-432</v>
       </c>
       <c r="D278" t="n">
         <v>42</v>
@@ -57136,17 +57136,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>6870.81</v>
+        <v>6831.65</v>
       </c>
       <c r="D2" t="n">
-        <v>-18.94</v>
+        <v>-10.68</v>
       </c>
       <c r="E2" t="n">
-        <v>100.24</v>
+        <v>97.68000000000001</v>
       </c>
     </row>
     <row r="3">
@@ -57157,44 +57157,44 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>65481.27</v>
+        <v>67947.91</v>
       </c>
       <c r="D3" t="n">
-        <v>-6.54</v>
+        <v>-1.14</v>
       </c>
       <c r="E3" t="n">
-        <v>45.37</v>
+        <v>52.52</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Zone euro (Euro Stoxx 50)</t>
+          <t>Etats-Unis (S&amp;P 500)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>6320.26</v>
+        <v>7651.54</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.12</v>
+        <v>2.25</v>
       </c>
       <c r="E4" t="n">
-        <v>14.77</v>
+        <v>14.4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Etats-Unis (S&amp;P 500)</t>
+          <t>Royaume-Uni (FTSE 100)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -57203,34 +57203,34 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>7651.54</v>
+        <v>10606</v>
       </c>
       <c r="D5" t="n">
-        <v>2.25</v>
+        <v>1.22</v>
       </c>
       <c r="E5" t="n">
-        <v>14.4</v>
+        <v>13.43</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Royaume-Uni (FTSE 100)</t>
+          <t>Zone euro (Euro Stoxx 50)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>10636.7</v>
+        <v>6269.02</v>
       </c>
       <c r="D6" t="n">
-        <v>1.33</v>
+        <v>-0.21</v>
       </c>
       <c r="E6" t="n">
-        <v>14.38</v>
+        <v>13.36</v>
       </c>
     </row>
     <row r="7">
@@ -57241,17 +57241,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>25399.21</v>
+        <v>25199.19</v>
       </c>
       <c r="D7" t="n">
-        <v>1.61</v>
+        <v>0.63</v>
       </c>
       <c r="E7" t="n">
-        <v>6.97</v>
+        <v>5.52</v>
       </c>
     </row>
     <row r="8">
@@ -57262,17 +57262,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>24523.57</v>
+        <v>24613.27</v>
       </c>
       <c r="D8" t="n">
-        <v>7.18</v>
+        <v>7.57</v>
       </c>
       <c r="E8" t="n">
-        <v>-7.89</v>
+        <v>-8.35</v>
       </c>
     </row>
   </sheetData>
@@ -59244,7 +59244,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -59633,6 +59633,3